<commit_message>
records: 2026-10-27 16:11 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -19,12 +19,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.00;[Red]-$#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.000000"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="170" formatCode="$#,##0.00;[Red]-$#,##0.00"/>
+    <numFmt numFmtId="171" formatCode="0.00%;[Red]-0.00%"/>
+    <numFmt numFmtId="172" formatCode="0.0"/>
+    <numFmt numFmtId="173" formatCode="0.0%"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -42,8 +47,13 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00627284"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0012805C"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -59,10 +69,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
@@ -97,29 +103,52 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="0012805C"/>
+        <sz val="10"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -190,6 +219,93 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA2" headerRowCount="1">
+  <autoFilter ref="A1:BA2"/>
+  <tableColumns count="53">
+    <tableColumn id="1" name="No"/>
+    <tableColumn id="2" name="Time Berlin"/>
+    <tableColumn id="3" name="Time New York"/>
+    <tableColumn id="4" name="Time UTC"/>
+    <tableColumn id="5" name="Side"/>
+    <tableColumn id="6" name="Symbol"/>
+    <tableColumn id="7" name="Company"/>
+    <tableColumn id="8" name="Exchange"/>
+    <tableColumn id="9" name="Status"/>
+    <tableColumn id="10" name="Qty filled"/>
+    <tableColumn id="11" name="Avg fill price $"/>
+    <tableColumn id="12" name="Fill value $"/>
+    <tableColumn id="13" name="Requested $"/>
+    <tableColumn id="14" name="Requested qty"/>
+    <tableColumn id="15" name="Rule"/>
+    <tableColumn id="16" name="Reason"/>
+    <tableColumn id="17" name="Greens (of 5)"/>
+    <tableColumn id="18" name="Time machine"/>
+    <tableColumn id="19" name="TM hit rate"/>
+    <tableColumn id="20" name="TM green days"/>
+    <tableColumn id="21" name="TM avg 5-day %"/>
+    <tableColumn id="22" name="Master switch 6-mo return %"/>
+    <tableColumn id="23" name="Agent rank"/>
+    <tableColumn id="24" name="1 Data real"/>
+    <tableColumn id="25" name="Source spread %"/>
+    <tableColumn id="26" name="2 Organic"/>
+    <tableColumn id="27" name="Organic score"/>
+    <tableColumn id="28" name="Organic flags"/>
+    <tableColumn id="29" name="3 Prediction"/>
+    <tableColumn id="30" name="Call"/>
+    <tableColumn id="31" name="Target $"/>
+    <tableColumn id="32" name="Range low $"/>
+    <tableColumn id="33" name="Range high $"/>
+    <tableColumn id="34" name="Call due"/>
+    <tableColumn id="35" name="Confidence"/>
+    <tableColumn id="36" name="4 News"/>
+    <tableColumn id="37" name="Headlines (72h)"/>
+    <tableColumn id="38" name="Top headline"/>
+    <tableColumn id="39" name="Price at decision $"/>
+    <tableColumn id="40" name="Move today %"/>
+    <tableColumn id="41" name="Account equity before $"/>
+    <tableColumn id="42" name="Cash before $"/>
+    <tableColumn id="43" name="Slot %"/>
+    <tableColumn id="44" name="Position qty before"/>
+    <tableColumn id="45" name="Avg entry before $"/>
+    <tableColumn id="46" name="P/L % before"/>
+    <tableColumn id="47" name="Account"/>
+    <tableColumn id="48" name="Order ID"/>
+    <tableColumn id="49" name="Client order ID"/>
+    <tableColumn id="50" name="Decided at (UTC)"/>
+    <tableColumn id="51" name="Filled at (UTC)"/>
+    <tableColumn id="52" name="Agent run (UTC)"/>
+    <tableColumn id="53" name="Error"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P2" headerRowCount="1">
+  <autoFilter ref="A1:P2"/>
+  <tableColumns count="16">
+    <tableColumn id="1" name="Symbol"/>
+    <tableColumn id="2" name="Company"/>
+    <tableColumn id="3" name="Bought (Berlin)"/>
+    <tableColumn id="4" name="Bought (New York)"/>
+    <tableColumn id="5" name="Buy price $"/>
+    <tableColumn id="6" name="Qty"/>
+    <tableColumn id="7" name="Cost $"/>
+    <tableColumn id="8" name="Sold (Berlin)"/>
+    <tableColumn id="9" name="Sold (New York)"/>
+    <tableColumn id="10" name="Sell price $"/>
+    <tableColumn id="11" name="Proceeds $"/>
+    <tableColumn id="12" name="P/L $"/>
+    <tableColumn id="13" name="P/L %"/>
+    <tableColumn id="14" name="Days held"/>
+    <tableColumn id="15" name="Exit rule"/>
+    <tableColumn id="16" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -502,7 +618,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46321.38127314814</v>
+        <v>46322.71640046296</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -522,7 +638,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46321.17293981482</v>
+        <v>46322.50806712963</v>
       </c>
     </row>
     <row r="4">
@@ -1034,15 +1150,195 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>No orders yet. Rows appear here as soon as the auto-trader places one.</t>
-        </is>
-      </c>
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="n">
+        <v>46322.71633101852</v>
+      </c>
+      <c r="C2" s="13" t="n">
+        <v>46322.50799768518</v>
+      </c>
+      <c r="D2" s="13" t="n">
+        <v>46322.67466435185</v>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific, Inc.</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J2" s="16" t="n">
+        <v>11.986804426</v>
+      </c>
+      <c r="K2" s="17" t="n">
+        <v>694.9299999999999</v>
+      </c>
+      <c r="L2" s="17">
+        <f>IF(AND(ISNUMBER(J2),ISNUMBER(K2)),J2*K2,"")</f>
+        <v/>
+      </c>
+      <c r="M2" s="17" t="n">
+        <v>8330</v>
+      </c>
+      <c r="N2" s="16" t="n"/>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P2" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $100,000.00 account</t>
+        </is>
+      </c>
+      <c r="Q2" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S2" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T2" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="U2" s="19" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="V2" s="19" t="n">
+        <v>-0.0173</v>
+      </c>
+      <c r="W2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y2" s="19" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Z2" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA2" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB2" s="15" t="n"/>
+      <c r="AC2" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD2" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE2" s="17" t="n">
+        <v>704.5304</v>
+      </c>
+      <c r="AF2" s="17" t="n">
+        <v>679.4169000000001</v>
+      </c>
+      <c r="AG2" s="17" t="n">
+        <v>729.644</v>
+      </c>
+      <c r="AH2" s="20" t="n">
+        <v>46329</v>
+      </c>
+      <c r="AI2" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ2" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL2" s="15" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific Experts to Host Webinar on Clario Endpoint Data Solutions</t>
+        </is>
+      </c>
+      <c r="AM2" s="17" t="n">
+        <v>694.485</v>
+      </c>
+      <c r="AN2" s="19" t="n">
+        <v>0.0141</v>
+      </c>
+      <c r="AO2" s="17" t="n">
+        <v>100000</v>
+      </c>
+      <c r="AP2" s="17" t="n">
+        <v>100000</v>
+      </c>
+      <c r="AQ2" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR2" s="16" t="n"/>
+      <c r="AS2" s="17" t="n"/>
+      <c r="AT2" s="19" t="n"/>
+      <c r="AU2" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV2" s="6" t="inlineStr">
+        <is>
+          <t>a17cede0-0466-4ec2-b2e1-ee5ddd1134cf</t>
+        </is>
+      </c>
+      <c r="AW2" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-TMO-1793117490105</t>
+        </is>
+      </c>
+      <c r="AX2" s="13" t="n">
+        <v>46322.67465277778</v>
+      </c>
+      <c r="AY2" s="13" t="n">
+        <v>46322.67466435185</v>
+      </c>
+      <c r="AZ2" s="13" t="n">
+        <v>46322.67446759259</v>
+      </c>
+      <c r="BA2" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1156,15 +1452,69 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>No filled buys yet.</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific, Inc.</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="n">
+        <v>46322.71633101852</v>
+      </c>
+      <c r="D2" s="21" t="n">
+        <v>46322.50799768518</v>
+      </c>
+      <c r="E2" s="17" t="n">
+        <v>694.9299999999999</v>
+      </c>
+      <c r="F2" s="16" t="n">
+        <v>11.986804426</v>
+      </c>
+      <c r="G2" s="17">
+        <f>E2*F2</f>
+        <v/>
+      </c>
+      <c r="H2" s="21" t="n"/>
+      <c r="I2" s="21" t="n"/>
+      <c r="J2" s="17" t="n"/>
+      <c r="K2" s="17">
+        <f>IF(ISNUMBER(J2),J2*F2,"")</f>
+        <v/>
+      </c>
+      <c r="L2" s="22">
+        <f>IF(ISNUMBER(J2),K2-G2,"")</f>
+        <v/>
+      </c>
+      <c r="M2" s="23">
+        <f>IF(ISNUMBER(J2),L2/G2,"")</f>
+        <v/>
+      </c>
+      <c r="N2" s="24">
+        <f>IF(ISNUMBER(H2),H2-C2,"")</f>
+        <v/>
+      </c>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="L2:M2">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1194,216 +1544,216 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>Master switch</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="25" t="inlineStr">
         <is>
           <t>Weekly time machine replays the last 6 months with these rules; if it would have lost money, no new buys</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>Buy</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>4 or 5 of 5 green, time machine and data-is-real green (vetoes), nothing red, not already held; funds/ETFs skipped</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Cash only</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>Never uses margin</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>No buys before close</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Last 60 minutes of the session: sells only</t>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Last 30 minutes of the session: sells only</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Daily loss guard</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>No new buys on a day the account is down 5% or more</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Exit: 3 of 5 green</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>Sell half, once (not again within 3 days)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>Exit: 2 or fewer of 5, or time machine red</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>Sell everything</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Sell line</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>5% below the highest price since buying, never lower than 5% under the buy price (bought 100, high 200: sells at 190). Also kept as a real Alpaca stop order that moves up with the price</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>Evening</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>In the last 30 minutes before the close, everything up less than +10% is sold; +10% or more stays overnight. No buys in the last 60 minutes</t>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Positions may be held overnight</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>Buy loop</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Each buy uses 8.33% of the cash available at that moment, repeated for every buy-ready stock (up to 40 stocks, orders of at least $5); never buys back a stock sold the same day</t>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>Each buy uses 8.33% of the cash available at that moment, repeated for every buy-ready stock (up to 12 stocks, orders of at least $5); never buys back a stock sold the same day</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>Bad day</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>Down 3% today and not 5 of 5 green: sell everything</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>Take profit</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>Off: winners keep running until the sell line or the close</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>Only positions the auto-trader bought (client order ID starts with tdagent-)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>Check 1 · Data is real</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>Price agrees across trade, quote, minute, hourly and daily bars; history has no broken bars or holes</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>Check 2 · Organic</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>No volume pump without news, no one-day jump doing the work, no gaps, no pump-and-fade, not thin</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>Check 3 · Prediction</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>5-trading-day momentum call with a volatility range; green only when it leans up</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>Check 4 · News</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>Headlines in the last 72 hours scored for high-impact words against today's move</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>Check 5 · Time machine</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="25" t="inlineStr">
         <is>
           <t>Replays the stock's past year: on days it looked green, did it rise over the next 5 trading days? Green at 55%+ hit rate and positive average</t>
         </is>

</xml_diff>

<commit_message>
records: 2026-10-27 18:05 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -222,8 +222,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA2" headerRowCount="1">
-  <autoFilter ref="A1:BA2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA3" headerRowCount="1">
+  <autoFilter ref="A1:BA3"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -284,8 +284,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P2" headerRowCount="1">
-  <autoFilter ref="A1:P2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P3" headerRowCount="1">
+  <autoFilter ref="A1:P3"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46322.71640046296</v>
+        <v>46322.7956712963</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46322.50806712963</v>
+        <v>46322.58733796296</v>
       </c>
     </row>
     <row r="4">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$2,"BUY")+COUNTIF(Orders!$E$2:$E$2,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$3,"BUY")+COUNTIF(Orders!$E$2:$E$3,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$2,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$3,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$2,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$3,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$2,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$3,"filled")</f>
         <v/>
       </c>
     </row>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$2,Orders!$E$2:$E$2,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$3,Orders!$E$2:$E$3,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$2,Orders!$E$2:$E$2,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$3,Orders!$E$2:$E$3,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$2,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$3,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$2,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$3,"Open")</f>
         <v/>
       </c>
     </row>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$2)</f>
+        <f>SUM('Round trips'!$L$2:$L$3)</f>
         <v/>
       </c>
     </row>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$2,"Closed",'Round trips'!$L$2:$L$2,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$3,"Closed",'Round trips'!$L$2:$L$3,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -824,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA2"/>
+  <dimension ref="A1:BA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1333,6 +1333,190 @@
       </c>
       <c r="BA2" s="6" t="n"/>
     </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="13" t="n">
+        <v>46322.79560185185</v>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>46322.58726851852</v>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>46322.75393518519</v>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="n">
+        <v>79.41675402600001</v>
+      </c>
+      <c r="K3" s="17" t="n">
+        <v>104.93</v>
+      </c>
+      <c r="L3" s="17">
+        <f>IF(AND(ISNUMBER(J3),ISNUMBER(K3)),J3*K3,"")</f>
+        <v/>
+      </c>
+      <c r="M3" s="17" t="n">
+        <v>8333.209999999999</v>
+      </c>
+      <c r="N3" s="16" t="n"/>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P3" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $100,038.60 account</t>
+        </is>
+      </c>
+      <c r="Q3" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S3" s="18" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="T3" s="12" t="n">
+        <v>92</v>
+      </c>
+      <c r="U3" s="19" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="V3" s="19" t="n">
+        <v>-0.0173</v>
+      </c>
+      <c r="W3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X3" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y3" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA3" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB3" s="15" t="n"/>
+      <c r="AC3" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD3" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE3" s="17" t="n">
+        <v>106.142</v>
+      </c>
+      <c r="AF3" s="17" t="n">
+        <v>103.062</v>
+      </c>
+      <c r="AG3" s="17" t="n">
+        <v>109.222</v>
+      </c>
+      <c r="AH3" s="20" t="n">
+        <v>46329</v>
+      </c>
+      <c r="AI3" s="18" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AJ3" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK3" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL3" s="15" t="inlineStr">
+        <is>
+          <t>Shell plc Announces Share Buyback Transaction</t>
+        </is>
+      </c>
+      <c r="AM3" s="17" t="n">
+        <v>104.91</v>
+      </c>
+      <c r="AN3" s="19" t="n">
+        <v>-0.0187</v>
+      </c>
+      <c r="AO3" s="17" t="n">
+        <v>100038.6</v>
+      </c>
+      <c r="AP3" s="17" t="n">
+        <v>91670.00999999999</v>
+      </c>
+      <c r="AQ3" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR3" s="16" t="n"/>
+      <c r="AS3" s="17" t="n"/>
+      <c r="AT3" s="19" t="n"/>
+      <c r="AU3" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV3" s="6" t="inlineStr">
+        <is>
+          <t>12db7300-b65a-4371-a182-4bcc07ceda77</t>
+        </is>
+      </c>
+      <c r="AW3" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-SHEL-1793124338749</t>
+        </is>
+      </c>
+      <c r="AX3" s="13" t="n">
+        <v>46322.75391203703</v>
+      </c>
+      <c r="AY3" s="13" t="n">
+        <v>46322.75393518519</v>
+      </c>
+      <c r="AZ3" s="13" t="n">
+        <v>46322.75368055556</v>
+      </c>
+      <c r="BA3" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -1348,7 +1532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1504,8 +1688,61 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="n">
+        <v>46322.79560185185</v>
+      </c>
+      <c r="D3" s="21" t="n">
+        <v>46322.58726851852</v>
+      </c>
+      <c r="E3" s="17" t="n">
+        <v>104.93</v>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>79.41675402600001</v>
+      </c>
+      <c r="G3" s="17">
+        <f>E3*F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="21" t="n"/>
+      <c r="I3" s="21" t="n"/>
+      <c r="J3" s="17" t="n"/>
+      <c r="K3" s="17">
+        <f>IF(ISNUMBER(J3),J3*F3,"")</f>
+        <v/>
+      </c>
+      <c r="L3" s="22">
+        <f>IF(ISNUMBER(J3),K3-G3,"")</f>
+        <v/>
+      </c>
+      <c r="M3" s="23">
+        <f>IF(ISNUMBER(J3),L3/G3,"")</f>
+        <v/>
+      </c>
+      <c r="N3" s="24">
+        <f>IF(ISNUMBER(H3),H3-C3,"")</f>
+        <v/>
+      </c>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M2">
+  <conditionalFormatting sqref="L2:M3">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-27 19:49 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="172" formatCode="0.0"/>
     <numFmt numFmtId="173" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +53,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="0012805C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C2362F"/>
       <sz val="10"/>
     </font>
     <font>
@@ -103,21 +109,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,6 +135,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -222,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA3" headerRowCount="1">
-  <autoFilter ref="A1:BA3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA5" headerRowCount="1">
+  <autoFilter ref="A1:BA5"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -618,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46322.7956712963</v>
+        <v>46322.86795138889</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -638,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46322.58733796296</v>
+        <v>46322.65961805556</v>
       </c>
     </row>
     <row r="4">
@@ -684,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$3,"BUY")+COUNTIF(Orders!$E$2:$E$3,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$5,"BUY")+COUNTIF(Orders!$E$2:$E$5,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -695,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$3,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$5,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -706,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$3,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$5,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -717,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$3,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$5,"filled")</f>
         <v/>
       </c>
     </row>
@@ -728,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$3,Orders!$E$2:$E$3,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$5,Orders!$E$2:$E$5,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -739,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$3,Orders!$E$2:$E$3,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$5,Orders!$E$2:$E$5,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -824,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA3"/>
+  <dimension ref="A1:BA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1517,6 +1524,382 @@
       </c>
       <c r="BA3" s="6" t="n"/>
     </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="n">
+        <v>46322.8678125</v>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>46322.65947916666</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>46322.82614583334</v>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="n">
+        <v>79.41675402600001</v>
+      </c>
+      <c r="K4" s="17" t="n">
+        <v>104.96</v>
+      </c>
+      <c r="L4" s="17">
+        <f>IF(AND(ISNUMBER(J4),ISNUMBER(K4)),J4*K4,"")</f>
+        <v/>
+      </c>
+      <c r="M4" s="17" t="n"/>
+      <c r="N4" s="16" t="n">
+        <v>79.41675402600001</v>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5%</t>
+        </is>
+      </c>
+      <c r="P4" s="15" t="inlineStr">
+        <is>
+          <t>Evening: +0.0% from the buy price (under +5%), sold 10 min before the close</t>
+        </is>
+      </c>
+      <c r="Q4" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S4" s="18" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="T4" s="12" t="n">
+        <v>92</v>
+      </c>
+      <c r="U4" s="19" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="V4" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W4" s="12" t="n"/>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y4" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z4" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA4" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB4" s="15" t="n"/>
+      <c r="AC4" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD4" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE4" s="17" t="n">
+        <v>106.1815</v>
+      </c>
+      <c r="AF4" s="17" t="n">
+        <v>103.1027</v>
+      </c>
+      <c r="AG4" s="17" t="n">
+        <v>109.2604</v>
+      </c>
+      <c r="AH4" s="20" t="n">
+        <v>46329</v>
+      </c>
+      <c r="AI4" s="18" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AJ4" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK4" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL4" s="15" t="inlineStr">
+        <is>
+          <t>'Washington discusses Russian deals for US oil majors in Ukraine peace talks' - Financial Times</t>
+        </is>
+      </c>
+      <c r="AM4" s="17" t="n">
+        <v>104.94</v>
+      </c>
+      <c r="AN4" s="19" t="n">
+        <v>-0.0183</v>
+      </c>
+      <c r="AO4" s="17" t="n">
+        <v>100056.57</v>
+      </c>
+      <c r="AP4" s="17" t="n">
+        <v>83336.81</v>
+      </c>
+      <c r="AQ4" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR4" s="16" t="n">
+        <v>79.41675402600001</v>
+      </c>
+      <c r="AS4" s="17" t="n">
+        <v>104.93</v>
+      </c>
+      <c r="AT4" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="AU4" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV4" s="6" t="inlineStr">
+        <is>
+          <t>be781221-5b78-4809-97c9-dde0425348d5</t>
+        </is>
+      </c>
+      <c r="AW4" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-SHEL-1793130578234</t>
+        </is>
+      </c>
+      <c r="AX4" s="13" t="n">
+        <v>46322.82613425926</v>
+      </c>
+      <c r="AY4" s="13" t="n">
+        <v>46322.82614583334</v>
+      </c>
+      <c r="AZ4" s="13" t="n">
+        <v>46322.8253587963</v>
+      </c>
+      <c r="BA4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>46322.86784722222</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>46322.65951388889</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>46322.82618055555</v>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="n">
+        <v>11.986804426</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <v>699.1666739999999</v>
+      </c>
+      <c r="L5" s="17">
+        <f>IF(AND(ISNUMBER(J5),ISNUMBER(K5)),J5*K5,"")</f>
+        <v/>
+      </c>
+      <c r="M5" s="17" t="n"/>
+      <c r="N5" s="16" t="n">
+        <v>11.986804426</v>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5%</t>
+        </is>
+      </c>
+      <c r="P5" s="15" t="inlineStr">
+        <is>
+          <t>Evening: +0.6% from the buy price (under +5%), sold 10 min before the close</t>
+        </is>
+      </c>
+      <c r="Q5" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S5" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T5" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="U5" s="19" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="V5" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W5" s="12" t="n"/>
+      <c r="X5" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y5" s="19" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="Z5" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA5" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB5" s="15" t="n"/>
+      <c r="AC5" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD5" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE5" s="17" t="n">
+        <v>710.0776</v>
+      </c>
+      <c r="AF5" s="17" t="n">
+        <v>684.5837</v>
+      </c>
+      <c r="AG5" s="17" t="n">
+        <v>735.5715</v>
+      </c>
+      <c r="AH5" s="20" t="n">
+        <v>46329</v>
+      </c>
+      <c r="AI5" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ5" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL5" s="15" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific Experts to Host Webinar on Clario Endpoint Data Solutions</t>
+        </is>
+      </c>
+      <c r="AM5" s="17" t="n">
+        <v>699.8</v>
+      </c>
+      <c r="AN5" s="19" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AO5" s="17" t="n">
+        <v>100056.57</v>
+      </c>
+      <c r="AP5" s="17" t="n">
+        <v>83336.81</v>
+      </c>
+      <c r="AQ5" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR5" s="16" t="n">
+        <v>11.986804426</v>
+      </c>
+      <c r="AS5" s="17" t="n">
+        <v>694.9299999999999</v>
+      </c>
+      <c r="AT5" s="19" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="AU5" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV5" s="6" t="inlineStr">
+        <is>
+          <t>3df9c111-1586-40fd-a37a-ab0a53ccf9d7</t>
+        </is>
+      </c>
+      <c r="AW5" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-TMO-1793130578875</t>
+        </is>
+      </c>
+      <c r="AX5" s="13" t="n">
+        <v>46322.82613425926</v>
+      </c>
+      <c r="AY5" s="13" t="n">
+        <v>46322.82618055555</v>
+      </c>
+      <c r="AZ5" s="13" t="n">
+        <v>46322.8253587963</v>
+      </c>
+      <c r="BA5" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -1646,10 +2029,10 @@
           <t>Thermo Fisher Scientific, Inc.</t>
         </is>
       </c>
-      <c r="C2" s="21" t="n">
+      <c r="C2" s="22" t="n">
         <v>46322.71633101852</v>
       </c>
-      <c r="D2" s="21" t="n">
+      <c r="D2" s="22" t="n">
         <v>46322.50799768518</v>
       </c>
       <c r="E2" s="17" t="n">
@@ -1662,29 +2045,39 @@
         <f>E2*F2</f>
         <v/>
       </c>
-      <c r="H2" s="21" t="n"/>
-      <c r="I2" s="21" t="n"/>
-      <c r="J2" s="17" t="n"/>
+      <c r="H2" s="22" t="n">
+        <v>46322.86784722222</v>
+      </c>
+      <c r="I2" s="22" t="n">
+        <v>46322.65951388889</v>
+      </c>
+      <c r="J2" s="17" t="n">
+        <v>699.1666739999999</v>
+      </c>
       <c r="K2" s="17">
         <f>IF(ISNUMBER(J2),J2*F2,"")</f>
         <v/>
       </c>
-      <c r="L2" s="22">
+      <c r="L2" s="23">
         <f>IF(ISNUMBER(J2),K2-G2,"")</f>
         <v/>
       </c>
-      <c r="M2" s="23">
+      <c r="M2" s="24">
         <f>IF(ISNUMBER(J2),L2/G2,"")</f>
         <v/>
       </c>
-      <c r="N2" s="24">
+      <c r="N2" s="25">
         <f>IF(ISNUMBER(H2),H2-C2,"")</f>
         <v/>
       </c>
-      <c r="O2" s="6" t="n"/>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5%</t>
+        </is>
+      </c>
       <c r="P2" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -1699,10 +2092,10 @@
           <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
         </is>
       </c>
-      <c r="C3" s="21" t="n">
+      <c r="C3" s="22" t="n">
         <v>46322.79560185185</v>
       </c>
-      <c r="D3" s="21" t="n">
+      <c r="D3" s="22" t="n">
         <v>46322.58726851852</v>
       </c>
       <c r="E3" s="17" t="n">
@@ -1715,29 +2108,39 @@
         <f>E3*F3</f>
         <v/>
       </c>
-      <c r="H3" s="21" t="n"/>
-      <c r="I3" s="21" t="n"/>
-      <c r="J3" s="17" t="n"/>
+      <c r="H3" s="22" t="n">
+        <v>46322.8678125</v>
+      </c>
+      <c r="I3" s="22" t="n">
+        <v>46322.65947916666</v>
+      </c>
+      <c r="J3" s="17" t="n">
+        <v>104.96</v>
+      </c>
       <c r="K3" s="17">
         <f>IF(ISNUMBER(J3),J3*F3,"")</f>
         <v/>
       </c>
-      <c r="L3" s="22">
+      <c r="L3" s="23">
         <f>IF(ISNUMBER(J3),K3-G3,"")</f>
         <v/>
       </c>
-      <c r="M3" s="23">
+      <c r="M3" s="24">
         <f>IF(ISNUMBER(J3),L3/G3,"")</f>
         <v/>
       </c>
-      <c r="N3" s="24">
+      <c r="N3" s="25">
         <f>IF(ISNUMBER(H3),H3-C3,"")</f>
         <v/>
       </c>
-      <c r="O3" s="6" t="n"/>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5%</t>
+        </is>
+      </c>
       <c r="P3" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -1781,216 +2184,216 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Master switch</t>
         </is>
       </c>
-      <c r="B2" s="25" t="inlineStr">
+      <c r="B2" s="26" t="inlineStr">
         <is>
           <t>Weekly time machine replays the last 6 months with these rules; if it would have lost money, no new buys</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Buy</t>
         </is>
       </c>
-      <c r="B3" s="25" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>4 or 5 of 5 green, time machine and data-is-real green (vetoes), nothing red, not already held; funds/ETFs skipped</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Cash only</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>Never uses margin</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>No buys before close</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Last 30 minutes of the session: sells only</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>Daily loss guard</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>No new buys on a day the account is down 5% or more</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Exit: 3 of 5 green</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Sell half, once (not again within 3 days)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Exit: 2 or fewer of 5, or time machine red</t>
         </is>
       </c>
-      <c r="B8" s="25" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Sell everything</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Sell line</t>
         </is>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>5% below the highest price since buying, never lower than 5% under the buy price (bought 100, high 200: sells at 190). Also kept as a real Alpaca stop order that moves up with the price</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Evening</t>
         </is>
       </c>
-      <c r="B10" s="25" t="inlineStr">
-        <is>
-          <t>Positions may be held overnight</t>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>In the last 30 minutes before the close, everything up less than +5% is sold; +5% or more stays overnight. No buys in the last 30 minutes</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>Buy loop</t>
         </is>
       </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>Each buy uses 8.33% of the cash available at that moment, repeated for every buy-ready stock (up to 12 stocks, orders of at least $5); never buys back a stock sold the same day</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Bad day</t>
         </is>
       </c>
-      <c r="B12" s="25" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Down 3% today and not 5 of 5 green: sell everything</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Take profit</t>
         </is>
       </c>
-      <c r="B13" s="25" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>Off: winners keep running until the sell line or the close</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B14" s="25" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Only positions the auto-trader bought (client order ID starts with tdagent-)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Check 1 · Data is real</t>
         </is>
       </c>
-      <c r="B15" s="25" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>Price agrees across trade, quote, minute, hourly and daily bars; history has no broken bars or holes</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Check 2 · Organic</t>
         </is>
       </c>
-      <c r="B16" s="25" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>No volume pump without news, no one-day jump doing the work, no gaps, no pump-and-fade, not thin</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>Check 3 · Prediction</t>
         </is>
       </c>
-      <c r="B17" s="25" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>5-trading-day momentum call with a volatility range; green only when it leans up</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>Check 4 · News</t>
         </is>
       </c>
-      <c r="B18" s="25" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>Headlines in the last 72 hours scored for high-impact words against today's move</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Check 5 · Time machine</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>Replays the stock's past year: on days it looked green, did it rise over the next 5 trading days? Green at 55%+ hit rate and positive average</t>
         </is>

</xml_diff>

<commit_message>
records: 2026-10-28 13:31 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA5" headerRowCount="1">
-  <autoFilter ref="A1:BA5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA17" headerRowCount="1">
+  <autoFilter ref="A1:BA17"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46322.86795138889</v>
+        <v>46323.6050925926</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46322.65961805556</v>
+        <v>46323.39675925926</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$5,"BUY")+COUNTIF(Orders!$E$2:$E$5,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$17,"BUY")+COUNTIF(Orders!$E$2:$E$17,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$5,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$17,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$5,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$17,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$5,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$17,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$5,Orders!$E$2:$E$5,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$17,Orders!$E$2:$E$17,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$5,Orders!$E$2:$E$5,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$17,Orders!$E$2:$E$17,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA5"/>
+  <dimension ref="A1:BA17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1900,6 +1900,2138 @@
       </c>
       <c r="BA5" s="6" t="n"/>
     </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>46323.60493055556</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>46323.39659722222</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>46323.56326388889</v>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific, Inc.</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="n"/>
+      <c r="K6" s="17" t="n"/>
+      <c r="L6" s="17">
+        <f>IF(AND(ISNUMBER(J6),ISNUMBER(K6)),J6*K6,"")</f>
+        <v/>
+      </c>
+      <c r="M6" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N6" s="16" t="n"/>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P6" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q6" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S6" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T6" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="U6" s="19" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="V6" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X6" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y6" s="19" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="Z6" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA6" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB6" s="15" t="n"/>
+      <c r="AC6" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD6" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE6" s="17" t="n">
+        <v>703.0821</v>
+      </c>
+      <c r="AF6" s="17" t="n">
+        <v>678.0519</v>
+      </c>
+      <c r="AG6" s="17" t="n">
+        <v>728.1123</v>
+      </c>
+      <c r="AH6" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI6" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ6" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL6" s="15" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific Experts to Host Webinar on Clario Endpoint Data Solutions</t>
+        </is>
+      </c>
+      <c r="AM6" s="17" t="n">
+        <v>692.41</v>
+      </c>
+      <c r="AN6" s="19" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AO6" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP6" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ6" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR6" s="16" t="n"/>
+      <c r="AS6" s="17" t="n"/>
+      <c r="AT6" s="19" t="n"/>
+      <c r="AU6" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV6" s="6" t="inlineStr">
+        <is>
+          <t>75ff6654-caa0-43af-a8e3-46fa207bc64a</t>
+        </is>
+      </c>
+      <c r="AW6" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-TMO-1793194262152</t>
+        </is>
+      </c>
+      <c r="AX6" s="13" t="n">
+        <v>46323.56321759259</v>
+      </c>
+      <c r="AY6" s="13" t="n"/>
+      <c r="AZ6" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>46323.60494212963</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>46323.3966087963</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>46323.56327546296</v>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Dynatrace, Inc.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="17" t="n"/>
+      <c r="L7" s="17">
+        <f>IF(AND(ISNUMBER(J7),ISNUMBER(K7)),J7*K7,"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N7" s="16" t="n"/>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P7" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #2, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q7" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S7" s="18" t="n">
+        <v>0.647</v>
+      </c>
+      <c r="T7" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="U7" s="19" t="n">
+        <v>0.0133</v>
+      </c>
+      <c r="V7" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W7" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="X7" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y7" s="19" t="n">
+        <v>0.0058</v>
+      </c>
+      <c r="Z7" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA7" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB7" s="15" t="n"/>
+      <c r="AC7" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD7" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE7" s="17" t="n">
+        <v>65.2238</v>
+      </c>
+      <c r="AF7" s="17" t="n">
+        <v>61.5643</v>
+      </c>
+      <c r="AG7" s="17" t="n">
+        <v>68.8832</v>
+      </c>
+      <c r="AH7" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI7" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ7" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK7" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL7" s="15" t="inlineStr">
+        <is>
+          <t>Analyst Raises Price Target for Dynatrace</t>
+        </is>
+      </c>
+      <c r="AM7" s="17" t="n">
+        <v>63.39</v>
+      </c>
+      <c r="AN7" s="19" t="n">
+        <v>-0.006500000000000001</v>
+      </c>
+      <c r="AO7" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP7" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ7" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR7" s="16" t="n"/>
+      <c r="AS7" s="17" t="n"/>
+      <c r="AT7" s="19" t="n"/>
+      <c r="AU7" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV7" s="6" t="inlineStr">
+        <is>
+          <t>ea46df9e-798f-47b6-8f79-15985b1f21c1</t>
+        </is>
+      </c>
+      <c r="AW7" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-DT-1793194262796</t>
+        </is>
+      </c>
+      <c r="AX7" s="13" t="n">
+        <v>46323.56321759259</v>
+      </c>
+      <c r="AY7" s="13" t="n"/>
+      <c r="AZ7" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>46323.6049537037</v>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>46323.39662037037</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>46323.56328703704</v>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>Monster Beverage Corporation</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="17" t="n"/>
+      <c r="L8" s="17">
+        <f>IF(AND(ISNUMBER(J8),ISNUMBER(K8)),J8*K8,"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N8" s="16" t="n"/>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P8" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #3, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q8" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S8" s="18" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="T8" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="U8" s="19" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="V8" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W8" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X8" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y8" s="19" t="n">
+        <v>0.0071</v>
+      </c>
+      <c r="Z8" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA8" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB8" s="15" t="n"/>
+      <c r="AC8" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD8" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE8" s="17" t="n">
+        <v>46.063</v>
+      </c>
+      <c r="AF8" s="17" t="n">
+        <v>44.4805</v>
+      </c>
+      <c r="AG8" s="17" t="n">
+        <v>47.6454</v>
+      </c>
+      <c r="AH8" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI8" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ8" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK8" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL8" s="15" t="inlineStr">
+        <is>
+          <t>JP Morgan Maintains Neutral on Monster Beverage, Lowers Price Target to $49</t>
+        </is>
+      </c>
+      <c r="AM8" s="17" t="n">
+        <v>45.11</v>
+      </c>
+      <c r="AN8" s="19" t="n">
+        <v>-0.0219</v>
+      </c>
+      <c r="AO8" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP8" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ8" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR8" s="16" t="n"/>
+      <c r="AS8" s="17" t="n"/>
+      <c r="AT8" s="19" t="n"/>
+      <c r="AU8" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV8" s="6" t="inlineStr">
+        <is>
+          <t>1618d695-4afd-42f8-b0f6-9dbbedd13f56</t>
+        </is>
+      </c>
+      <c r="AW8" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MNST-1793194263216</t>
+        </is>
+      </c>
+      <c r="AX8" s="13" t="n">
+        <v>46323.56322916667</v>
+      </c>
+      <c r="AY8" s="13" t="n"/>
+      <c r="AZ8" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>46323.60496527778</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>46323.39663194444</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>46323.56329861111</v>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>CBOE</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>Cboe Global Markets, Inc.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>BATS</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="n"/>
+      <c r="K9" s="17" t="n"/>
+      <c r="L9" s="17">
+        <f>IF(AND(ISNUMBER(J9),ISNUMBER(K9)),J9*K9,"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N9" s="16" t="n"/>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P9" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S9" s="18" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="T9" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="U9" s="19" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="V9" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W9" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X9" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA9" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB9" s="15" t="n"/>
+      <c r="AC9" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD9" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE9" s="17" t="n">
+        <v>331.8585</v>
+      </c>
+      <c r="AF9" s="17" t="n">
+        <v>314.9122</v>
+      </c>
+      <c r="AG9" s="17" t="n">
+        <v>348.8048</v>
+      </c>
+      <c r="AH9" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI9" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ9" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK9" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL9" s="15" t="inlineStr">
+        <is>
+          <t>JPMorgan Adjusts Price Target on Cboe Global Markets to $332 From $288</t>
+        </is>
+      </c>
+      <c r="AM9" s="17" t="n">
+        <v>325.08</v>
+      </c>
+      <c r="AN9" s="19" t="n">
+        <v>-0.0295</v>
+      </c>
+      <c r="AO9" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP9" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ9" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR9" s="16" t="n"/>
+      <c r="AS9" s="17" t="n"/>
+      <c r="AT9" s="19" t="n"/>
+      <c r="AU9" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV9" s="6" t="inlineStr">
+        <is>
+          <t>9bdcd091-8a94-4f6c-90f4-0dd5ee0bbaf3</t>
+        </is>
+      </c>
+      <c r="AW9" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-CBOE-1793194263728</t>
+        </is>
+      </c>
+      <c r="AX9" s="13" t="n">
+        <v>46323.56322916667</v>
+      </c>
+      <c r="AY9" s="13" t="n"/>
+      <c r="AZ9" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>46323.60496527778</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>46323.39663194444</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>46323.56329861111</v>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>McKesson Corporation</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J10" s="16" t="n"/>
+      <c r="K10" s="17" t="n"/>
+      <c r="L10" s="17">
+        <f>IF(AND(ISNUMBER(J10),ISNUMBER(K10)),J10*K10,"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N10" s="16" t="n"/>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P10" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #5, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q10" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S10" s="18" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="T10" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="U10" s="19" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="V10" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W10" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X10" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA10" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB10" s="15" t="n"/>
+      <c r="AC10" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD10" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE10" s="17" t="n">
+        <v>982.3085</v>
+      </c>
+      <c r="AF10" s="17" t="n">
+        <v>943.6373</v>
+      </c>
+      <c r="AG10" s="17" t="n">
+        <v>1020.9796</v>
+      </c>
+      <c r="AH10" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI10" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ10" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK10" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL10" s="15" t="inlineStr">
+        <is>
+          <t>Here's How Much $100 Invested In McKesson 5 Years Ago Would Be Worth Today</t>
+        </is>
+      </c>
+      <c r="AM10" s="17" t="n">
+        <v>966.84</v>
+      </c>
+      <c r="AN10" s="19" t="n">
+        <v>-0.0255</v>
+      </c>
+      <c r="AO10" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP10" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ10" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR10" s="16" t="n"/>
+      <c r="AS10" s="17" t="n"/>
+      <c r="AT10" s="19" t="n"/>
+      <c r="AU10" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV10" s="6" t="inlineStr">
+        <is>
+          <t>6189b904-77fc-4fcf-b41f-bde0ff4f39db</t>
+        </is>
+      </c>
+      <c r="AW10" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MCK-1793194264162</t>
+        </is>
+      </c>
+      <c r="AX10" s="13" t="n">
+        <v>46323.56324074074</v>
+      </c>
+      <c r="AY10" s="13" t="n"/>
+      <c r="AZ10" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>46323.60497685185</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>46323.39664351852</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>46323.56331018519</v>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="n"/>
+      <c r="K11" s="17" t="n"/>
+      <c r="L11" s="17">
+        <f>IF(AND(ISNUMBER(J11),ISNUMBER(K11)),J11*K11,"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N11" s="16" t="n"/>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P11" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #6, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q11" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S11" s="18" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="T11" s="12" t="n">
+        <v>91</v>
+      </c>
+      <c r="U11" s="19" t="n">
+        <v>0.0124</v>
+      </c>
+      <c r="V11" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W11" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="X11" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y11" s="19" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="Z11" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA11" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB11" s="15" t="n"/>
+      <c r="AC11" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD11" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE11" s="17" t="n">
+        <v>106.0087</v>
+      </c>
+      <c r="AF11" s="17" t="n">
+        <v>102.9244</v>
+      </c>
+      <c r="AG11" s="17" t="n">
+        <v>109.093</v>
+      </c>
+      <c r="AH11" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI11" s="18" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AJ11" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK11" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL11" s="15" t="inlineStr">
+        <is>
+          <t>'Washington discusses Russian deals for US oil majors in Ukraine peace talks' - Financial Times</t>
+        </is>
+      </c>
+      <c r="AM11" s="17" t="n">
+        <v>105.04</v>
+      </c>
+      <c r="AN11" s="19" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="AO11" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP11" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ11" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR11" s="16" t="n"/>
+      <c r="AS11" s="17" t="n"/>
+      <c r="AT11" s="19" t="n"/>
+      <c r="AU11" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV11" s="6" t="inlineStr">
+        <is>
+          <t>f2c34f6c-bb0c-4e2b-a829-02bd8a0f636f</t>
+        </is>
+      </c>
+      <c r="AW11" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-SHEL-1793194264666</t>
+        </is>
+      </c>
+      <c r="AX11" s="13" t="n">
+        <v>46323.56324074074</v>
+      </c>
+      <c r="AY11" s="13" t="n"/>
+      <c r="AZ11" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>46323.60498842593</v>
+      </c>
+      <c r="C12" s="13" t="n">
+        <v>46323.39665509259</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>46323.56332175926</v>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>Illumina, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="17" t="n"/>
+      <c r="L12" s="17">
+        <f>IF(AND(ISNUMBER(J12),ISNUMBER(K12)),J12*K12,"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N12" s="16" t="n"/>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P12" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #9, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q12" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S12" s="18" t="n">
+        <v>0.592</v>
+      </c>
+      <c r="T12" s="12" t="n">
+        <v>125</v>
+      </c>
+      <c r="U12" s="19" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="V12" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W12" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="X12" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y12" s="19" t="n">
+        <v>0.0029</v>
+      </c>
+      <c r="Z12" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA12" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB12" s="15" t="n"/>
+      <c r="AC12" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD12" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE12" s="17" t="n">
+        <v>287.5899</v>
+      </c>
+      <c r="AF12" s="17" t="n">
+        <v>267.1151</v>
+      </c>
+      <c r="AG12" s="17" t="n">
+        <v>308.0647</v>
+      </c>
+      <c r="AH12" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI12" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ12" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" s="15" t="n"/>
+      <c r="AM12" s="17" t="n">
+        <v>278.6</v>
+      </c>
+      <c r="AN12" s="19" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="AO12" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP12" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ12" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR12" s="16" t="n"/>
+      <c r="AS12" s="17" t="n"/>
+      <c r="AT12" s="19" t="n"/>
+      <c r="AU12" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV12" s="6" t="inlineStr">
+        <is>
+          <t>980f13dc-f907-4bd4-b53e-7799785ee61b</t>
+        </is>
+      </c>
+      <c r="AW12" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ILMN-1793194266066</t>
+        </is>
+      </c>
+      <c r="AX12" s="13" t="n">
+        <v>46323.56326388889</v>
+      </c>
+      <c r="AY12" s="13" t="n"/>
+      <c r="AZ12" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>46323.605</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>46323.39666666667</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>46323.56333333333</v>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>United Therapeutics Corporation Common Stock</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="n"/>
+      <c r="K13" s="17" t="n"/>
+      <c r="L13" s="17">
+        <f>IF(AND(ISNUMBER(J13),ISNUMBER(K13)),J13*K13,"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N13" s="16" t="n"/>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P13" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #10, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q13" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S13" s="18" t="n">
+        <v>0.569</v>
+      </c>
+      <c r="T13" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="U13" s="19" t="n">
+        <v>0.0118</v>
+      </c>
+      <c r="V13" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W13" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="X13" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA13" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB13" s="15" t="n"/>
+      <c r="AC13" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD13" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE13" s="17" t="n">
+        <v>604.2865</v>
+      </c>
+      <c r="AF13" s="17" t="n">
+        <v>571.9452</v>
+      </c>
+      <c r="AG13" s="17" t="n">
+        <v>636.6278</v>
+      </c>
+      <c r="AH13" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI13" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ13" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL13" s="15" t="n"/>
+      <c r="AM13" s="17" t="n">
+        <v>591.35</v>
+      </c>
+      <c r="AN13" s="19" t="n">
+        <v>-0.0023</v>
+      </c>
+      <c r="AO13" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP13" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ13" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR13" s="16" t="n"/>
+      <c r="AS13" s="17" t="n"/>
+      <c r="AT13" s="19" t="n"/>
+      <c r="AU13" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV13" s="6" t="inlineStr">
+        <is>
+          <t>4bf78c8b-c039-475a-999c-1bf4c352180c</t>
+        </is>
+      </c>
+      <c r="AW13" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-UTHR-1793194266530</t>
+        </is>
+      </c>
+      <c r="AX13" s="13" t="n">
+        <v>46323.56326388889</v>
+      </c>
+      <c r="AY13" s="13" t="n"/>
+      <c r="AZ13" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>46323.605</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>46323.39666666667</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>46323.56333333333</v>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>eBay Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="n"/>
+      <c r="K14" s="17" t="n"/>
+      <c r="L14" s="17">
+        <f>IF(AND(ISNUMBER(J14),ISNUMBER(K14)),J14*K14,"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N14" s="16" t="n"/>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P14" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #11, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q14" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S14" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T14" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="U14" s="19" t="n">
+        <v>0.005500000000000001</v>
+      </c>
+      <c r="V14" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W14" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="X14" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y14" s="19" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="Z14" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA14" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB14" s="15" t="n"/>
+      <c r="AC14" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD14" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE14" s="17" t="n">
+        <v>119.7698</v>
+      </c>
+      <c r="AF14" s="17" t="n">
+        <v>114.8704</v>
+      </c>
+      <c r="AG14" s="17" t="n">
+        <v>124.6691</v>
+      </c>
+      <c r="AH14" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI14" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ14" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK14" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL14" s="15" t="inlineStr">
+        <is>
+          <t>UBS Maintains Neutral on eBay, Raises Price Target to $131</t>
+        </is>
+      </c>
+      <c r="AM14" s="17" t="n">
+        <v>118.33</v>
+      </c>
+      <c r="AN14" s="19" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="AO14" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP14" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ14" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR14" s="16" t="n"/>
+      <c r="AS14" s="17" t="n"/>
+      <c r="AT14" s="19" t="n"/>
+      <c r="AU14" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV14" s="6" t="inlineStr">
+        <is>
+          <t>8449c305-1c64-40c9-a24f-a14b858d4888</t>
+        </is>
+      </c>
+      <c r="AW14" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EBAY-1793194267013</t>
+        </is>
+      </c>
+      <c r="AX14" s="13" t="n">
+        <v>46323.56327546296</v>
+      </c>
+      <c r="AY14" s="13" t="n"/>
+      <c r="AZ14" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>46323.60501157407</v>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>46323.39667824074</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>46323.56334490741</v>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>Occidental Petroleum Corporation</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="n"/>
+      <c r="K15" s="17" t="n"/>
+      <c r="L15" s="17">
+        <f>IF(AND(ISNUMBER(J15),ISNUMBER(K15)),J15*K15,"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N15" s="16" t="n"/>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P15" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #12, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q15" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R15" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S15" s="18" t="n">
+        <v>0.621</v>
+      </c>
+      <c r="T15" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="U15" s="19" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="V15" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W15" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="X15" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y15" s="19" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="Z15" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA15" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB15" s="15" t="n"/>
+      <c r="AC15" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD15" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE15" s="17" t="n">
+        <v>63.7925</v>
+      </c>
+      <c r="AF15" s="17" t="n">
+        <v>61.1362</v>
+      </c>
+      <c r="AG15" s="17" t="n">
+        <v>66.44889999999999</v>
+      </c>
+      <c r="AH15" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI15" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ15" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK15" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL15" s="15" t="inlineStr">
+        <is>
+          <t>Goldman Sachs Downgrades Occidental Petroleum to Neutral</t>
+        </is>
+      </c>
+      <c r="AM15" s="17" t="n">
+        <v>63.14</v>
+      </c>
+      <c r="AN15" s="19" t="n">
+        <v>-0.0209</v>
+      </c>
+      <c r="AO15" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP15" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ15" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR15" s="16" t="n"/>
+      <c r="AS15" s="17" t="n"/>
+      <c r="AT15" s="19" t="n"/>
+      <c r="AU15" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV15" s="6" t="inlineStr">
+        <is>
+          <t>e2f8f479-97ed-463a-aab1-2ca11da16008</t>
+        </is>
+      </c>
+      <c r="AW15" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-OXY-1793194267523</t>
+        </is>
+      </c>
+      <c r="AX15" s="13" t="n">
+        <v>46323.56327546296</v>
+      </c>
+      <c r="AY15" s="13" t="n"/>
+      <c r="AZ15" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>46323.60501157407</v>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>46323.39667824074</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>46323.56334490741</v>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>IQVIA Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="n"/>
+      <c r="K16" s="17" t="n"/>
+      <c r="L16" s="17">
+        <f>IF(AND(ISNUMBER(J16),ISNUMBER(K16)),J16*K16,"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N16" s="16" t="n"/>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P16" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #13, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q16" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S16" s="18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="T16" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="U16" s="19" t="n">
+        <v>0.0142</v>
+      </c>
+      <c r="V16" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W16" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="X16" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y16" s="19" t="n">
+        <v>0.004699999999999999</v>
+      </c>
+      <c r="Z16" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA16" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB16" s="15" t="n"/>
+      <c r="AC16" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD16" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE16" s="17" t="n">
+        <v>275.4603</v>
+      </c>
+      <c r="AF16" s="17" t="n">
+        <v>265.4096</v>
+      </c>
+      <c r="AG16" s="17" t="n">
+        <v>285.511</v>
+      </c>
+      <c r="AH16" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI16" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ16" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK16" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL16" s="15" t="inlineStr">
+        <is>
+          <t>IQVIA Hldgs Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM16" s="17" t="n">
+        <v>270.175</v>
+      </c>
+      <c r="AN16" s="19" t="n">
+        <v>-0.0092</v>
+      </c>
+      <c r="AO16" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP16" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ16" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR16" s="16" t="n"/>
+      <c r="AS16" s="17" t="n"/>
+      <c r="AT16" s="19" t="n"/>
+      <c r="AU16" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV16" s="6" t="inlineStr">
+        <is>
+          <t>dcb95512-fd40-4530-b67d-8e5ef4305ac4</t>
+        </is>
+      </c>
+      <c r="AW16" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-IQV-1793194268057</t>
+        </is>
+      </c>
+      <c r="AX16" s="13" t="n">
+        <v>46323.56328703704</v>
+      </c>
+      <c r="AY16" s="13" t="n"/>
+      <c r="AZ16" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>46323.60502314815</v>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>46323.39668981481</v>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>46323.56335648148</v>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>PBR.A</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>Petroleo Brasileiro S.A.-Petrobras</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="n"/>
+      <c r="K17" s="17" t="n"/>
+      <c r="L17" s="17">
+        <f>IF(AND(ISNUMBER(J17),ISNUMBER(K17)),J17*K17,"")</f>
+        <v/>
+      </c>
+      <c r="M17" s="17" t="n">
+        <v>8334.389999999999</v>
+      </c>
+      <c r="N17" s="16" t="n"/>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P17" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #14, 8.33% of the $100,052.80 account</t>
+        </is>
+      </c>
+      <c r="Q17" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R17" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S17" s="18" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="T17" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="U17" s="19" t="n">
+        <v>0.0247</v>
+      </c>
+      <c r="V17" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W17" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="X17" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y17" s="19" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="Z17" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AA17" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="AB17" s="15" t="inlineStr">
+        <is>
+          <t>One day (-15.4%) did 121% of the 10-day move. The trend rests on a single jump.; Price gapped 16.8% at an open in the last week.</t>
+        </is>
+      </c>
+      <c r="AC17" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD17" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE17" s="17" t="n">
+        <v>20.3103</v>
+      </c>
+      <c r="AF17" s="17" t="n">
+        <v>18.9221</v>
+      </c>
+      <c r="AG17" s="17" t="n">
+        <v>21.6984</v>
+      </c>
+      <c r="AH17" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI17" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ17" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK17" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL17" s="15" t="inlineStr">
+        <is>
+          <t>Halliburton Deploys ROCS Technology With Petrobras in Brazil</t>
+        </is>
+      </c>
+      <c r="AM17" s="17" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="AN17" s="19" t="n">
+        <v>-0.0075</v>
+      </c>
+      <c r="AO17" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AP17" s="17" t="n">
+        <v>100052.8</v>
+      </c>
+      <c r="AQ17" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR17" s="16" t="n"/>
+      <c r="AS17" s="17" t="n"/>
+      <c r="AT17" s="19" t="n"/>
+      <c r="AU17" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV17" s="6" t="inlineStr">
+        <is>
+          <t>d24a5b49-4f8b-4052-bbd2-144f6d025701</t>
+        </is>
+      </c>
+      <c r="AW17" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-PBR.A-1793194268661</t>
+        </is>
+      </c>
+      <c r="AX17" s="13" t="n">
+        <v>46323.56328703704</v>
+      </c>
+      <c r="AY17" s="13" t="n"/>
+      <c r="AZ17" s="13" t="n">
+        <v>46323.56269675926</v>
+      </c>
+      <c r="BA17" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
records: 2026-10-28 13:37 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA17" headerRowCount="1">
-  <autoFilter ref="A1:BA17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA19" headerRowCount="1">
+  <autoFilter ref="A1:BA19"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P3" headerRowCount="1">
-  <autoFilter ref="A1:P3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P17" headerRowCount="1">
+  <autoFilter ref="A1:P17"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.6050925926</v>
+        <v>46323.60902777778</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.39675925926</v>
+        <v>46323.40069444444</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$17,"BUY")+COUNTIF(Orders!$E$2:$E$17,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$19,"BUY")+COUNTIF(Orders!$E$2:$E$19,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$17,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$19,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$17,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$19,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$17,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$19,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$17,Orders!$E$2:$E$17,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$19,Orders!$E$2:$E$19,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$17,Orders!$E$2:$E$17,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$19,Orders!$E$2:$E$19,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$3,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$17,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$3,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$17,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$3)</f>
+        <f>SUM('Round trips'!$L$2:$L$17)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$3,"Closed",'Round trips'!$L$2:$L$3,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$17,"Closed",'Round trips'!$L$2:$L$17,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA17"/>
+  <dimension ref="A1:BA19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1905,13 +1905,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="13" t="n">
-        <v>46323.60493055556</v>
+        <v>46323.60681712963</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>46323.39659722222</v>
+        <v>46323.3984837963</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>46323.56326388889</v>
+        <v>46323.56515046296</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -1935,11 +1935,15 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="n">
+        <v>11.937064238</v>
+      </c>
+      <c r="K6" s="17" t="n">
+        <v>698.193445</v>
+      </c>
       <c r="L6" s="17">
         <f>IF(AND(ISNUMBER(J6),ISNUMBER(K6)),J6*K6,"")</f>
         <v/>
@@ -2072,7 +2076,9 @@
       <c r="AX6" s="13" t="n">
         <v>46323.56321759259</v>
       </c>
-      <c r="AY6" s="13" t="n"/>
+      <c r="AY6" s="13" t="n">
+        <v>46323.56515046296</v>
+      </c>
       <c r="AZ6" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -2083,13 +2089,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="13" t="n">
-        <v>46323.60494212963</v>
+        <v>46323.60652777777</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>46323.3966087963</v>
+        <v>46323.39819444445</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>46323.56327546296</v>
+        <v>46323.56486111111</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -2113,11 +2119,15 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>130.2953125</v>
+      </c>
+      <c r="K7" s="17" t="n">
+        <v>63.965309</v>
+      </c>
       <c r="L7" s="17">
         <f>IF(AND(ISNUMBER(J7),ISNUMBER(K7)),J7*K7,"")</f>
         <v/>
@@ -2250,7 +2260,9 @@
       <c r="AX7" s="13" t="n">
         <v>46323.56321759259</v>
       </c>
-      <c r="AY7" s="13" t="n"/>
+      <c r="AY7" s="13" t="n">
+        <v>46323.56486111111</v>
+      </c>
       <c r="AZ7" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -2261,13 +2273,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="13" t="n">
-        <v>46323.6049537037</v>
+        <v>46323.60728009259</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>46323.39662037037</v>
+        <v>46323.39894675926</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>46323.56328703704</v>
+        <v>46323.56561342593</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
@@ -2291,11 +2303,15 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J8" s="16" t="n"/>
-      <c r="K8" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="n">
+        <v>184.54038504</v>
+      </c>
+      <c r="K8" s="17" t="n">
+        <v>45.162906</v>
+      </c>
       <c r="L8" s="17">
         <f>IF(AND(ISNUMBER(J8),ISNUMBER(K8)),J8*K8,"")</f>
         <v/>
@@ -2428,7 +2444,9 @@
       <c r="AX8" s="13" t="n">
         <v>46323.56322916667</v>
       </c>
-      <c r="AY8" s="13" t="n"/>
+      <c r="AY8" s="13" t="n">
+        <v>46323.56561342593</v>
+      </c>
       <c r="AZ8" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -2439,13 +2457,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="13" t="n">
-        <v>46323.60496527778</v>
+        <v>46323.60716435185</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>46323.39663194444</v>
+        <v>46323.39883101852</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>46323.56329861111</v>
+        <v>46323.56549768519</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
@@ -2469,11 +2487,15 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J9" s="16" t="n"/>
-      <c r="K9" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="n">
+        <v>25.834717916</v>
+      </c>
+      <c r="K9" s="17" t="n">
+        <v>322.603871</v>
+      </c>
       <c r="L9" s="17">
         <f>IF(AND(ISNUMBER(J9),ISNUMBER(K9)),J9*K9,"")</f>
         <v/>
@@ -2606,7 +2628,9 @@
       <c r="AX9" s="13" t="n">
         <v>46323.56322916667</v>
       </c>
-      <c r="AY9" s="13" t="n"/>
+      <c r="AY9" s="13" t="n">
+        <v>46323.56549768519</v>
+      </c>
       <c r="AZ9" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -2617,13 +2641,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="13" t="n">
-        <v>46323.60496527778</v>
+        <v>46323.60681712963</v>
       </c>
       <c r="C10" s="13" t="n">
-        <v>46323.39663194444</v>
+        <v>46323.3984837963</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>46323.56329861111</v>
+        <v>46323.56515046296</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -2647,11 +2671,15 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J10" s="16" t="n"/>
-      <c r="K10" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J10" s="16" t="n">
+        <v>8.620135337000001</v>
+      </c>
+      <c r="K10" s="17" t="n">
+        <v>966.85025</v>
+      </c>
       <c r="L10" s="17">
         <f>IF(AND(ISNUMBER(J10),ISNUMBER(K10)),J10*K10,"")</f>
         <v/>
@@ -2784,7 +2812,9 @@
       <c r="AX10" s="13" t="n">
         <v>46323.56324074074</v>
       </c>
-      <c r="AY10" s="13" t="n"/>
+      <c r="AY10" s="13" t="n">
+        <v>46323.56515046296</v>
+      </c>
       <c r="AZ10" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -2795,13 +2825,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="13" t="n">
-        <v>46323.60497685185</v>
+        <v>46323.6061574074</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>46323.39664351852</v>
+        <v>46323.39782407408</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>46323.56331018519</v>
+        <v>46323.56449074074</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
@@ -2825,11 +2855,15 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J11" s="16" t="n"/>
-      <c r="K11" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="n">
+        <v>79.375047619</v>
+      </c>
+      <c r="K11" s="17" t="n">
+        <v>105</v>
+      </c>
       <c r="L11" s="17">
         <f>IF(AND(ISNUMBER(J11),ISNUMBER(K11)),J11*K11,"")</f>
         <v/>
@@ -2962,7 +2996,9 @@
       <c r="AX11" s="13" t="n">
         <v>46323.56324074074</v>
       </c>
-      <c r="AY11" s="13" t="n"/>
+      <c r="AY11" s="13" t="n">
+        <v>46323.56449074074</v>
+      </c>
       <c r="AZ11" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -2973,13 +3009,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="13" t="n">
-        <v>46323.60498842593</v>
+        <v>46323.60633101852</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>46323.39665509259</v>
+        <v>46323.39799768518</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>46323.56332175926</v>
+        <v>46323.56466435185</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -3003,11 +3039,15 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J12" s="16" t="n"/>
-      <c r="K12" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="n">
+        <v>29.659715302</v>
+      </c>
+      <c r="K12" s="17" t="n">
+        <v>281</v>
+      </c>
       <c r="L12" s="17">
         <f>IF(AND(ISNUMBER(J12),ISNUMBER(K12)),J12*K12,"")</f>
         <v/>
@@ -3136,7 +3176,9 @@
       <c r="AX12" s="13" t="n">
         <v>46323.56326388889</v>
       </c>
-      <c r="AY12" s="13" t="n"/>
+      <c r="AY12" s="13" t="n">
+        <v>46323.56466435185</v>
+      </c>
       <c r="AZ12" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -3147,13 +3189,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="13" t="n">
-        <v>46323.605</v>
+        <v>46323.60626157407</v>
       </c>
       <c r="C13" s="13" t="n">
-        <v>46323.39666666667</v>
+        <v>46323.39792824074</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>46323.56333333333</v>
+        <v>46323.56459490741</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
@@ -3177,11 +3219,15 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J13" s="16" t="n"/>
-      <c r="K13" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="n">
+        <v>14.223462352</v>
+      </c>
+      <c r="K13" s="17" t="n">
+        <v>585.96</v>
+      </c>
       <c r="L13" s="17">
         <f>IF(AND(ISNUMBER(J13),ISNUMBER(K13)),J13*K13,"")</f>
         <v/>
@@ -3310,7 +3356,9 @@
       <c r="AX13" s="13" t="n">
         <v>46323.56326388889</v>
       </c>
-      <c r="AY13" s="13" t="n"/>
+      <c r="AY13" s="13" t="n">
+        <v>46323.56459490741</v>
+      </c>
       <c r="AZ13" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -3321,13 +3369,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="13" t="n">
-        <v>46323.605</v>
+        <v>46323.60640046297</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>46323.39666666667</v>
+        <v>46323.39806712963</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>46323.56333333333</v>
+        <v>46323.56473379629</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
@@ -3351,11 +3399,15 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J14" s="16" t="n"/>
-      <c r="K14" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="n">
+        <v>70.13268309</v>
+      </c>
+      <c r="K14" s="17" t="n">
+        <v>118.837319</v>
+      </c>
       <c r="L14" s="17">
         <f>IF(AND(ISNUMBER(J14),ISNUMBER(K14)),J14*K14,"")</f>
         <v/>
@@ -3488,7 +3540,9 @@
       <c r="AX14" s="13" t="n">
         <v>46323.56327546296</v>
       </c>
-      <c r="AY14" s="13" t="n"/>
+      <c r="AY14" s="13" t="n">
+        <v>46323.56473379629</v>
+      </c>
       <c r="AZ14" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -3499,13 +3553,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="13" t="n">
-        <v>46323.60501157407</v>
+        <v>46323.60721064815</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>46323.39667824074</v>
+        <v>46323.39887731482</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>46323.56334490741</v>
+        <v>46323.56554398148</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
@@ -3529,11 +3583,15 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J15" s="16" t="n"/>
-      <c r="K15" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="n">
+        <v>132.295201779</v>
+      </c>
+      <c r="K15" s="17" t="n">
+        <v>62.998354</v>
+      </c>
       <c r="L15" s="17">
         <f>IF(AND(ISNUMBER(J15),ISNUMBER(K15)),J15*K15,"")</f>
         <v/>
@@ -3666,7 +3724,9 @@
       <c r="AX15" s="13" t="n">
         <v>46323.56327546296</v>
       </c>
-      <c r="AY15" s="13" t="n"/>
+      <c r="AY15" s="13" t="n">
+        <v>46323.56554398148</v>
+      </c>
       <c r="AZ15" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -3677,13 +3737,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="13" t="n">
-        <v>46323.60501157407</v>
+        <v>46323.60728009259</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>46323.39667824074</v>
+        <v>46323.39894675926</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>46323.56334490741</v>
+        <v>46323.56561342593</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
@@ -3707,11 +3767,15 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J16" s="16" t="n"/>
-      <c r="K16" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="n">
+        <v>30.359759869</v>
+      </c>
+      <c r="K16" s="17" t="n">
+        <v>274.520617</v>
+      </c>
       <c r="L16" s="17">
         <f>IF(AND(ISNUMBER(J16),ISNUMBER(K16)),J16*K16,"")</f>
         <v/>
@@ -3844,7 +3908,9 @@
       <c r="AX16" s="13" t="n">
         <v>46323.56328703704</v>
       </c>
-      <c r="AY16" s="13" t="n"/>
+      <c r="AY16" s="13" t="n">
+        <v>46323.56561342593</v>
+      </c>
       <c r="AZ16" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
@@ -3855,13 +3921,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="13" t="n">
-        <v>46323.60502314815</v>
+        <v>46323.60732638889</v>
       </c>
       <c r="C17" s="13" t="n">
-        <v>46323.39668981481</v>
+        <v>46323.39899305555</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>46323.56335648148</v>
+        <v>46323.56565972222</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -3885,11 +3951,15 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="J17" s="16" t="n"/>
-      <c r="K17" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="n">
+        <v>423.159067882</v>
+      </c>
+      <c r="K17" s="17" t="n">
+        <v>19.69562</v>
+      </c>
       <c r="L17" s="17">
         <f>IF(AND(ISNUMBER(J17),ISNUMBER(K17)),J17*K17,"")</f>
         <v/>
@@ -4026,11 +4096,393 @@
       <c r="AX17" s="13" t="n">
         <v>46323.56328703704</v>
       </c>
-      <c r="AY17" s="13" t="n"/>
+      <c r="AY17" s="13" t="n">
+        <v>46323.56565972222</v>
+      </c>
       <c r="AZ17" s="13" t="n">
         <v>46323.56269675926</v>
       </c>
       <c r="BA17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="13" t="n">
+        <v>46323.60892361111</v>
+      </c>
+      <c r="C18" s="13" t="n">
+        <v>46323.40059027778</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>46323.56725694444</v>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="n">
+        <v>15.179879934</v>
+      </c>
+      <c r="K18" s="17" t="n">
+        <v>273.44</v>
+      </c>
+      <c r="L18" s="17">
+        <f>IF(AND(ISNUMBER(J18),ISNUMBER(K18)),J18*K18,"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="17" t="n"/>
+      <c r="N18" s="16" t="n">
+        <v>15.179879934</v>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P18" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q18" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S18" s="18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="T18" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="U18" s="19" t="n">
+        <v>0.0142</v>
+      </c>
+      <c r="V18" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W18" s="12" t="n"/>
+      <c r="X18" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y18" s="19" t="n">
+        <v>0.0091</v>
+      </c>
+      <c r="Z18" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA18" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB18" s="15" t="n"/>
+      <c r="AC18" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD18" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE18" s="17" t="n">
+        <v>275.8908</v>
+      </c>
+      <c r="AF18" s="17" t="n">
+        <v>266.0138</v>
+      </c>
+      <c r="AG18" s="17" t="n">
+        <v>285.7679</v>
+      </c>
+      <c r="AH18" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI18" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ18" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK18" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL18" s="15" t="inlineStr">
+        <is>
+          <t>IQVIA Hldgs Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM18" s="17" t="n">
+        <v>271.94</v>
+      </c>
+      <c r="AN18" s="19" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="AO18" s="17" t="n">
+        <v>99990.35000000001</v>
+      </c>
+      <c r="AP18" s="17" t="n">
+        <v>40.24</v>
+      </c>
+      <c r="AQ18" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR18" s="16" t="n">
+        <v>30.359759869</v>
+      </c>
+      <c r="AS18" s="17" t="n">
+        <v>274.520617</v>
+      </c>
+      <c r="AT18" s="19" t="n">
+        <v>-0.0028</v>
+      </c>
+      <c r="AU18" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV18" s="6" t="inlineStr">
+        <is>
+          <t>23c6235d-dfef-4aeb-a7b4-d002f9b5f79f</t>
+        </is>
+      </c>
+      <c r="AW18" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-IQV-1793194607983</t>
+        </is>
+      </c>
+      <c r="AX18" s="13" t="n">
+        <v>46323.56721064815</v>
+      </c>
+      <c r="AY18" s="13" t="n">
+        <v>46323.56725694444</v>
+      </c>
+      <c r="AZ18" s="13" t="n">
+        <v>46323.56685185185</v>
+      </c>
+      <c r="BA18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="13" t="n">
+        <v>46323.60894675926</v>
+      </c>
+      <c r="C19" s="13" t="n">
+        <v>46323.40061342593</v>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>46323.56728009259</v>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>PBR.A</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>PBR.A</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="n">
+        <v>211.579533941</v>
+      </c>
+      <c r="K19" s="17" t="n">
+        <v>19.755625</v>
+      </c>
+      <c r="L19" s="17">
+        <f>IF(AND(ISNUMBER(J19),ISNUMBER(K19)),J19*K19,"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="17" t="n"/>
+      <c r="N19" s="16" t="n">
+        <v>211.579533941</v>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P19" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q19" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R19" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S19" s="18" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="T19" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="U19" s="19" t="n">
+        <v>0.0247</v>
+      </c>
+      <c r="V19" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W19" s="12" t="n"/>
+      <c r="X19" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y19" s="19" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="Z19" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AA19" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="AB19" s="15" t="inlineStr">
+        <is>
+          <t>One day (-15.4%) did 107% of the 10-day move. The trend rests on a single jump.; Price gapped 16.8% at an open in the last week.</t>
+        </is>
+      </c>
+      <c r="AC19" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD19" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE19" s="17" t="n">
+        <v>19.76</v>
+      </c>
+      <c r="AF19" s="17" t="n">
+        <v>18.3771</v>
+      </c>
+      <c r="AG19" s="17" t="n">
+        <v>21.1429</v>
+      </c>
+      <c r="AH19" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI19" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ19" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK19" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL19" s="15" t="inlineStr">
+        <is>
+          <t>Halliburton Deploys ROCS Technology With Petrobras in Brazil</t>
+        </is>
+      </c>
+      <c r="AM19" s="17" t="n">
+        <v>19.75</v>
+      </c>
+      <c r="AN19" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="AO19" s="17" t="n">
+        <v>99990.35000000001</v>
+      </c>
+      <c r="AP19" s="17" t="n">
+        <v>40.24</v>
+      </c>
+      <c r="AQ19" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR19" s="16" t="n">
+        <v>423.159067882</v>
+      </c>
+      <c r="AS19" s="17" t="n">
+        <v>19.69562</v>
+      </c>
+      <c r="AT19" s="19" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="AU19" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV19" s="6" t="inlineStr">
+        <is>
+          <t>e3451ca4-e963-4073-ad76-f95ca1253ccb</t>
+        </is>
+      </c>
+      <c r="AW19" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-PBR.A-1793194608171</t>
+        </is>
+      </c>
+      <c r="AX19" s="13" t="n">
+        <v>46323.56722222222</v>
+      </c>
+      <c r="AY19" s="13" t="n">
+        <v>46323.56728009259</v>
+      </c>
+      <c r="AZ19" s="13" t="n">
+        <v>46323.56685185185</v>
+      </c>
+      <c r="BA19" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4047,7 +4499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4276,8 +4728,770 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="n">
+        <v>46323.6061574074</v>
+      </c>
+      <c r="D4" s="22" t="n">
+        <v>46323.39782407408</v>
+      </c>
+      <c r="E4" s="17" t="n">
+        <v>105</v>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>79.375047619</v>
+      </c>
+      <c r="G4" s="17">
+        <f>E4*F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="22" t="n"/>
+      <c r="I4" s="22" t="n"/>
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="17">
+        <f>IF(ISNUMBER(J4),J4*F4,"")</f>
+        <v/>
+      </c>
+      <c r="L4" s="23">
+        <f>IF(ISNUMBER(J4),K4-G4,"")</f>
+        <v/>
+      </c>
+      <c r="M4" s="24">
+        <f>IF(ISNUMBER(J4),L4/G4,"")</f>
+        <v/>
+      </c>
+      <c r="N4" s="25">
+        <f>IF(ISNUMBER(H4),H4-C4,"")</f>
+        <v/>
+      </c>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>United Therapeutics Corporation Common Stock</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>46323.60626157407</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>46323.39792824074</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>585.96</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>14.223462352</v>
+      </c>
+      <c r="G5" s="17">
+        <f>E5*F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="22" t="n"/>
+      <c r="I5" s="22" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="17">
+        <f>IF(ISNUMBER(J5),J5*F5,"")</f>
+        <v/>
+      </c>
+      <c r="L5" s="23">
+        <f>IF(ISNUMBER(J5),K5-G5,"")</f>
+        <v/>
+      </c>
+      <c r="M5" s="24">
+        <f>IF(ISNUMBER(J5),L5/G5,"")</f>
+        <v/>
+      </c>
+      <c r="N5" s="25">
+        <f>IF(ISNUMBER(H5),H5-C5,"")</f>
+        <v/>
+      </c>
+      <c r="O5" s="6" t="n"/>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Illumina, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>46323.60633101852</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>46323.39799768518</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>281</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>29.659715302</v>
+      </c>
+      <c r="G6" s="17">
+        <f>E6*F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="22" t="n"/>
+      <c r="I6" s="22" t="n"/>
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="17">
+        <f>IF(ISNUMBER(J6),J6*F6,"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="23">
+        <f>IF(ISNUMBER(J6),K6-G6,"")</f>
+        <v/>
+      </c>
+      <c r="M6" s="24">
+        <f>IF(ISNUMBER(J6),L6/G6,"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="25">
+        <f>IF(ISNUMBER(H6),H6-C6,"")</f>
+        <v/>
+      </c>
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>eBay Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>46323.60640046297</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>46323.39806712963</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>118.837319</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>70.13268309</v>
+      </c>
+      <c r="G7" s="17">
+        <f>E7*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="22" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="17">
+        <f>IF(ISNUMBER(J7),J7*F7,"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="23">
+        <f>IF(ISNUMBER(J7),K7-G7,"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="24">
+        <f>IF(ISNUMBER(J7),L7/G7,"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="25">
+        <f>IF(ISNUMBER(H7),H7-C7,"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Dynatrace, Inc.</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>46323.60652777777</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>46323.39819444445</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>63.965309</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>130.2953125</v>
+      </c>
+      <c r="G8" s="17">
+        <f>E8*F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="22" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="17" t="n"/>
+      <c r="K8" s="17">
+        <f>IF(ISNUMBER(J8),J8*F8,"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="23">
+        <f>IF(ISNUMBER(J8),K8-G8,"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="24">
+        <f>IF(ISNUMBER(J8),L8/G8,"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="25">
+        <f>IF(ISNUMBER(H8),H8-C8,"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>McKesson Corporation</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>46323.60681712963</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>46323.3984837963</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>966.85025</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>8.620135337000001</v>
+      </c>
+      <c r="G9" s="17">
+        <f>E9*F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="22" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="17">
+        <f>IF(ISNUMBER(J9),J9*F9,"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="23">
+        <f>IF(ISNUMBER(J9),K9-G9,"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="24">
+        <f>IF(ISNUMBER(J9),L9/G9,"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="25">
+        <f>IF(ISNUMBER(H9),H9-C9,"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific, Inc.</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="n">
+        <v>46323.60681712963</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>46323.3984837963</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>698.193445</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>11.937064238</v>
+      </c>
+      <c r="G10" s="17">
+        <f>E10*F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="22" t="n"/>
+      <c r="I10" s="22" t="n"/>
+      <c r="J10" s="17" t="n"/>
+      <c r="K10" s="17">
+        <f>IF(ISNUMBER(J10),J10*F10,"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="23">
+        <f>IF(ISNUMBER(J10),K10-G10,"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="24">
+        <f>IF(ISNUMBER(J10),L10/G10,"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="25">
+        <f>IF(ISNUMBER(H10),H10-C10,"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>CBOE</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Cboe Global Markets, Inc.</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>46323.60716435185</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>46323.39883101852</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>322.603871</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>25.834717916</v>
+      </c>
+      <c r="G11" s="17">
+        <f>E11*F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="22" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="17">
+        <f>IF(ISNUMBER(J11),J11*F11,"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="23">
+        <f>IF(ISNUMBER(J11),K11-G11,"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="24">
+        <f>IF(ISNUMBER(J11),L11/G11,"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="25">
+        <f>IF(ISNUMBER(H11),H11-C11,"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Occidental Petroleum Corporation</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="n">
+        <v>46323.60721064815</v>
+      </c>
+      <c r="D12" s="22" t="n">
+        <v>46323.39887731482</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>62.998354</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>132.295201779</v>
+      </c>
+      <c r="G12" s="17">
+        <f>E12*F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="22" t="n"/>
+      <c r="I12" s="22" t="n"/>
+      <c r="J12" s="17" t="n"/>
+      <c r="K12" s="17">
+        <f>IF(ISNUMBER(J12),J12*F12,"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="23">
+        <f>IF(ISNUMBER(J12),K12-G12,"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="24">
+        <f>IF(ISNUMBER(J12),L12/G12,"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="25">
+        <f>IF(ISNUMBER(H12),H12-C12,"")</f>
+        <v/>
+      </c>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>IQVIA Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="n">
+        <v>46323.60728009259</v>
+      </c>
+      <c r="D13" s="22" t="n">
+        <v>46323.39894675926</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>274.520617</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>15.179879934</v>
+      </c>
+      <c r="G13" s="17">
+        <f>E13*F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="22" t="n">
+        <v>46323.60892361111</v>
+      </c>
+      <c r="I13" s="22" t="n">
+        <v>46323.40059027778</v>
+      </c>
+      <c r="J13" s="17" t="n">
+        <v>273.44</v>
+      </c>
+      <c r="K13" s="17">
+        <f>IF(ISNUMBER(J13),J13*F13,"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="23">
+        <f>IF(ISNUMBER(J13),K13-G13,"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="24">
+        <f>IF(ISNUMBER(J13),L13/G13,"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="25">
+        <f>IF(ISNUMBER(H13),H13-C13,"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>IQVIA Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="n">
+        <v>46323.60728009259</v>
+      </c>
+      <c r="D14" s="22" t="n">
+        <v>46323.39894675926</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>274.520617</v>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>15.179879935</v>
+      </c>
+      <c r="G14" s="17">
+        <f>E14*F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="22" t="n"/>
+      <c r="I14" s="22" t="n"/>
+      <c r="J14" s="17" t="n"/>
+      <c r="K14" s="17">
+        <f>IF(ISNUMBER(J14),J14*F14,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="23">
+        <f>IF(ISNUMBER(J14),K14-G14,"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="24">
+        <f>IF(ISNUMBER(J14),L14/G14,"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="25">
+        <f>IF(ISNUMBER(H14),H14-C14,"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Monster Beverage Corporation</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="n">
+        <v>46323.60728009259</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>46323.39894675926</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>45.162906</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>184.54038504</v>
+      </c>
+      <c r="G15" s="17">
+        <f>E15*F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="22" t="n"/>
+      <c r="I15" s="22" t="n"/>
+      <c r="J15" s="17" t="n"/>
+      <c r="K15" s="17">
+        <f>IF(ISNUMBER(J15),J15*F15,"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="23">
+        <f>IF(ISNUMBER(J15),K15-G15,"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="24">
+        <f>IF(ISNUMBER(J15),L15/G15,"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="25">
+        <f>IF(ISNUMBER(H15),H15-C15,"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="6" t="n"/>
+      <c r="P15" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>PBR.A</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Petroleo Brasileiro S.A.-Petrobras</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>46323.60732638889</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>46323.39899305555</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>19.69562</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>211.579533941</v>
+      </c>
+      <c r="G16" s="17">
+        <f>E16*F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="22" t="n">
+        <v>46323.60894675926</v>
+      </c>
+      <c r="I16" s="22" t="n">
+        <v>46323.40061342593</v>
+      </c>
+      <c r="J16" s="17" t="n">
+        <v>19.755625</v>
+      </c>
+      <c r="K16" s="17">
+        <f>IF(ISNUMBER(J16),J16*F16,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="23">
+        <f>IF(ISNUMBER(J16),K16-G16,"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="24">
+        <f>IF(ISNUMBER(J16),L16/G16,"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="25">
+        <f>IF(ISNUMBER(H16),H16-C16,"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P16" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>PBR.A</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Petroleo Brasileiro S.A.-Petrobras</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="n">
+        <v>46323.60732638889</v>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>46323.39899305555</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>19.69562</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>211.579533941</v>
+      </c>
+      <c r="G17" s="17">
+        <f>E17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="22" t="n"/>
+      <c r="I17" s="22" t="n"/>
+      <c r="J17" s="17" t="n"/>
+      <c r="K17" s="17">
+        <f>IF(ISNUMBER(J17),J17*F17,"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="23">
+        <f>IF(ISNUMBER(J17),K17-G17,"")</f>
+        <v/>
+      </c>
+      <c r="M17" s="24">
+        <f>IF(ISNUMBER(J17),L17/G17,"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="25">
+        <f>IF(ISNUMBER(H17),H17-C17,"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M3">
+  <conditionalFormatting sqref="L2:M17">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 14:52 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA19" headerRowCount="1">
-  <autoFilter ref="A1:BA19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA20" headerRowCount="1">
+  <autoFilter ref="A1:BA20"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P17" headerRowCount="1">
-  <autoFilter ref="A1:P17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P18" headerRowCount="1">
+  <autoFilter ref="A1:P18"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.60902777778</v>
+        <v>46323.6615625</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.40069444444</v>
+        <v>46323.45322916667</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$19,"BUY")+COUNTIF(Orders!$E$2:$E$19,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$20,"BUY")+COUNTIF(Orders!$E$2:$E$20,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$19,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$20,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$19,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$20,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$19,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$20,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$19,Orders!$E$2:$E$19,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$20,Orders!$E$2:$E$20,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$19,Orders!$E$2:$E$19,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$20,Orders!$E$2:$E$20,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$17,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$18,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$17,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$18,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$17)</f>
+        <f>SUM('Round trips'!$L$2:$L$18)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$17,"Closed",'Round trips'!$L$2:$L$17,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$18,"Closed",'Round trips'!$L$2:$L$18,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA19"/>
+  <dimension ref="A1:BA20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4484,6 +4484,194 @@
       </c>
       <c r="BA19" s="6" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="13" t="n">
+        <v>46323.66149305556</v>
+      </c>
+      <c r="C20" s="13" t="n">
+        <v>46323.45315972222</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>46323.61982638889</v>
+      </c>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J20" s="16" t="n">
+        <v>7.111731176</v>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v>588.24</v>
+      </c>
+      <c r="L20" s="17">
+        <f>IF(AND(ISNUMBER(J20),ISNUMBER(K20)),J20*K20,"")</f>
+        <v/>
+      </c>
+      <c r="M20" s="17" t="n"/>
+      <c r="N20" s="16" t="n">
+        <v>7.111731176</v>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P20" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q20" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R20" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S20" s="18" t="n">
+        <v>0.569</v>
+      </c>
+      <c r="T20" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="U20" s="19" t="n">
+        <v>0.0118</v>
+      </c>
+      <c r="V20" s="19" t="n">
+        <v>-0.1111</v>
+      </c>
+      <c r="W20" s="12" t="n"/>
+      <c r="X20" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y20" s="19" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+      <c r="Z20" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA20" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB20" s="15" t="n"/>
+      <c r="AC20" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD20" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE20" s="17" t="n">
+        <v>589.155</v>
+      </c>
+      <c r="AF20" s="17" t="n">
+        <v>556.9173</v>
+      </c>
+      <c r="AG20" s="17" t="n">
+        <v>621.3927</v>
+      </c>
+      <c r="AH20" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI20" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ20" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK20" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL20" s="15" t="inlineStr">
+        <is>
+          <t>$100 Invested In United Therapeutics 15 Years Ago Would Be Worth This Much Today</t>
+        </is>
+      </c>
+      <c r="AM20" s="17" t="n">
+        <v>589.155</v>
+      </c>
+      <c r="AN20" s="19" t="n">
+        <v>-0.0037</v>
+      </c>
+      <c r="AO20" s="17" t="n">
+        <v>100467.14</v>
+      </c>
+      <c r="AP20" s="17" t="n">
+        <v>8370.92</v>
+      </c>
+      <c r="AQ20" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR20" s="16" t="n">
+        <v>14.223462352</v>
+      </c>
+      <c r="AS20" s="17" t="n">
+        <v>585.96</v>
+      </c>
+      <c r="AT20" s="19" t="n">
+        <v>0.004699999999999999</v>
+      </c>
+      <c r="AU20" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV20" s="6" t="inlineStr">
+        <is>
+          <t>7bad1f9c-33ad-4b49-9f35-6a76bd48b748</t>
+        </is>
+      </c>
+      <c r="AW20" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-UTHR-1793199151204</t>
+        </is>
+      </c>
+      <c r="AX20" s="13" t="n">
+        <v>46323.61980324074</v>
+      </c>
+      <c r="AY20" s="13" t="n">
+        <v>46323.61982638889</v>
+      </c>
+      <c r="AZ20" s="13" t="n">
+        <v>46323.61961805556</v>
+      </c>
+      <c r="BA20" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -4499,7 +4687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4802,15 +4990,21 @@
         <v>585.96</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>14.223462352</v>
+        <v>7.111731176</v>
       </c>
       <c r="G5" s="17">
         <f>E5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="22" t="n"/>
-      <c r="I5" s="22" t="n"/>
-      <c r="J5" s="17" t="n"/>
+      <c r="H5" s="22" t="n">
+        <v>46323.66149305556</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>46323.45315972222</v>
+      </c>
+      <c r="J5" s="17" t="n">
+        <v>588.24</v>
+      </c>
       <c r="K5" s="17">
         <f>IF(ISNUMBER(J5),J5*F5,"")</f>
         <v/>
@@ -4827,35 +5021,39 @@
         <f>IF(ISNUMBER(H5),H5-C5,"")</f>
         <v/>
       </c>
-      <c r="O5" s="6" t="n"/>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>UTHR</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Illumina, Inc. Common Stock</t>
+          <t>United Therapeutics Corporation Common Stock</t>
         </is>
       </c>
       <c r="C6" s="22" t="n">
-        <v>46323.60633101852</v>
+        <v>46323.60626157407</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>46323.39799768518</v>
+        <v>46323.39792824074</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>281</v>
+        <v>585.96</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>29.659715302</v>
+        <v>7.111731176</v>
       </c>
       <c r="G6" s="17">
         <f>E6*F6</f>
@@ -4890,25 +5088,25 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>eBay Inc. Common Stock</t>
+          <t>Illumina, Inc. Common Stock</t>
         </is>
       </c>
       <c r="C7" s="22" t="n">
-        <v>46323.60640046297</v>
+        <v>46323.60633101852</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>46323.39806712963</v>
+        <v>46323.39799768518</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>118.837319</v>
+        <v>281</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>70.13268309</v>
+        <v>29.659715302</v>
       </c>
       <c r="G7" s="17">
         <f>E7*F7</f>
@@ -4943,25 +5141,25 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Dynatrace, Inc.</t>
+          <t>eBay Inc. Common Stock</t>
         </is>
       </c>
       <c r="C8" s="22" t="n">
-        <v>46323.60652777777</v>
+        <v>46323.60640046297</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>46323.39819444445</v>
+        <v>46323.39806712963</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>63.965309</v>
+        <v>118.837319</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>130.2953125</v>
+        <v>70.13268309</v>
       </c>
       <c r="G8" s="17">
         <f>E8*F8</f>
@@ -4996,25 +5194,25 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>MCK</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>McKesson Corporation</t>
+          <t>Dynatrace, Inc.</t>
         </is>
       </c>
       <c r="C9" s="22" t="n">
-        <v>46323.60681712963</v>
+        <v>46323.60652777777</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>46323.3984837963</v>
+        <v>46323.39819444445</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>966.85025</v>
+        <v>63.965309</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>8.620135337000001</v>
+        <v>130.2953125</v>
       </c>
       <c r="G9" s="17">
         <f>E9*F9</f>
@@ -5049,12 +5247,12 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>MCK</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Thermo Fisher Scientific, Inc.</t>
+          <t>McKesson Corporation</t>
         </is>
       </c>
       <c r="C10" s="22" t="n">
@@ -5064,10 +5262,10 @@
         <v>46323.3984837963</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>698.193445</v>
+        <v>966.85025</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>11.937064238</v>
+        <v>8.620135337000001</v>
       </c>
       <c r="G10" s="17">
         <f>E10*F10</f>
@@ -5102,25 +5300,25 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>CBOE</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Cboe Global Markets, Inc.</t>
+          <t>Thermo Fisher Scientific, Inc.</t>
         </is>
       </c>
       <c r="C11" s="22" t="n">
-        <v>46323.60716435185</v>
+        <v>46323.60681712963</v>
       </c>
       <c r="D11" s="22" t="n">
-        <v>46323.39883101852</v>
+        <v>46323.3984837963</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>322.603871</v>
+        <v>698.193445</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>25.834717916</v>
+        <v>11.937064238</v>
       </c>
       <c r="G11" s="17">
         <f>E11*F11</f>
@@ -5155,25 +5353,25 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>OXY</t>
+          <t>CBOE</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Occidental Petroleum Corporation</t>
+          <t>Cboe Global Markets, Inc.</t>
         </is>
       </c>
       <c r="C12" s="22" t="n">
-        <v>46323.60721064815</v>
+        <v>46323.60716435185</v>
       </c>
       <c r="D12" s="22" t="n">
-        <v>46323.39887731482</v>
+        <v>46323.39883101852</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>62.998354</v>
+        <v>322.603871</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>132.295201779</v>
+        <v>25.834717916</v>
       </c>
       <c r="G12" s="17">
         <f>E12*F12</f>
@@ -5208,39 +5406,33 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>IQV</t>
+          <t>OXY</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>IQVIA Holdings Inc.</t>
+          <t>Occidental Petroleum Corporation</t>
         </is>
       </c>
       <c r="C13" s="22" t="n">
-        <v>46323.60728009259</v>
+        <v>46323.60721064815</v>
       </c>
       <c r="D13" s="22" t="n">
-        <v>46323.39894675926</v>
+        <v>46323.39887731482</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>274.520617</v>
+        <v>62.998354</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>15.179879934</v>
+        <v>132.295201779</v>
       </c>
       <c r="G13" s="17">
         <f>E13*F13</f>
         <v/>
       </c>
-      <c r="H13" s="22" t="n">
-        <v>46323.60892361111</v>
-      </c>
-      <c r="I13" s="22" t="n">
-        <v>46323.40059027778</v>
-      </c>
-      <c r="J13" s="17" t="n">
-        <v>273.44</v>
-      </c>
+      <c r="H13" s="22" t="n"/>
+      <c r="I13" s="22" t="n"/>
+      <c r="J13" s="17" t="n"/>
       <c r="K13" s="17">
         <f>IF(ISNUMBER(J13),J13*F13,"")</f>
         <v/>
@@ -5257,14 +5449,10 @@
         <f>IF(ISNUMBER(H13),H13-C13,"")</f>
         <v/>
       </c>
-      <c r="O13" s="6" t="inlineStr">
-        <is>
-          <t>3 green: sell half</t>
-        </is>
-      </c>
+      <c r="O13" s="6" t="n"/>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5289,15 +5477,21 @@
         <v>274.520617</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>15.179879935</v>
+        <v>15.179879934</v>
       </c>
       <c r="G14" s="17">
         <f>E14*F14</f>
         <v/>
       </c>
-      <c r="H14" s="22" t="n"/>
-      <c r="I14" s="22" t="n"/>
-      <c r="J14" s="17" t="n"/>
+      <c r="H14" s="22" t="n">
+        <v>46323.60892361111</v>
+      </c>
+      <c r="I14" s="22" t="n">
+        <v>46323.40059027778</v>
+      </c>
+      <c r="J14" s="17" t="n">
+        <v>273.44</v>
+      </c>
       <c r="K14" s="17">
         <f>IF(ISNUMBER(J14),J14*F14,"")</f>
         <v/>
@@ -5314,22 +5508,26 @@
         <f>IF(ISNUMBER(H14),H14-C14,"")</f>
         <v/>
       </c>
-      <c r="O14" s="6" t="n"/>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>IQV</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Monster Beverage Corporation</t>
+          <t>IQVIA Holdings Inc.</t>
         </is>
       </c>
       <c r="C15" s="22" t="n">
@@ -5339,10 +5537,10 @@
         <v>46323.39894675926</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>45.162906</v>
+        <v>274.520617</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>184.54038504</v>
+        <v>15.179879935</v>
       </c>
       <c r="G15" s="17">
         <f>E15*F15</f>
@@ -5377,39 +5575,33 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>PBR.A</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Petroleo Brasileiro S.A.-Petrobras</t>
+          <t>Monster Beverage Corporation</t>
         </is>
       </c>
       <c r="C16" s="22" t="n">
-        <v>46323.60732638889</v>
+        <v>46323.60728009259</v>
       </c>
       <c r="D16" s="22" t="n">
-        <v>46323.39899305555</v>
+        <v>46323.39894675926</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>19.69562</v>
+        <v>45.162906</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>211.579533941</v>
+        <v>184.54038504</v>
       </c>
       <c r="G16" s="17">
         <f>E16*F16</f>
         <v/>
       </c>
-      <c r="H16" s="22" t="n">
-        <v>46323.60894675926</v>
-      </c>
-      <c r="I16" s="22" t="n">
-        <v>46323.40061342593</v>
-      </c>
-      <c r="J16" s="17" t="n">
-        <v>19.755625</v>
-      </c>
+      <c r="H16" s="22" t="n"/>
+      <c r="I16" s="22" t="n"/>
+      <c r="J16" s="17" t="n"/>
       <c r="K16" s="17">
         <f>IF(ISNUMBER(J16),J16*F16,"")</f>
         <v/>
@@ -5426,14 +5618,10 @@
         <f>IF(ISNUMBER(H16),H16-C16,"")</f>
         <v/>
       </c>
-      <c r="O16" s="6" t="inlineStr">
-        <is>
-          <t>3 green: sell half</t>
-        </is>
-      </c>
+      <c r="O16" s="6" t="n"/>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5464,9 +5652,15 @@
         <f>E17*F17</f>
         <v/>
       </c>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="22" t="n"/>
-      <c r="J17" s="17" t="n"/>
+      <c r="H17" s="22" t="n">
+        <v>46323.60894675926</v>
+      </c>
+      <c r="I17" s="22" t="n">
+        <v>46323.40061342593</v>
+      </c>
+      <c r="J17" s="17" t="n">
+        <v>19.755625</v>
+      </c>
       <c r="K17" s="17">
         <f>IF(ISNUMBER(J17),J17*F17,"")</f>
         <v/>
@@ -5483,15 +5677,72 @@
         <f>IF(ISNUMBER(H17),H17-C17,"")</f>
         <v/>
       </c>
-      <c r="O17" s="6" t="n"/>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>PBR.A</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Petroleo Brasileiro S.A.-Petrobras</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="n">
+        <v>46323.60732638889</v>
+      </c>
+      <c r="D18" s="22" t="n">
+        <v>46323.39899305555</v>
+      </c>
+      <c r="E18" s="17" t="n">
+        <v>19.69562</v>
+      </c>
+      <c r="F18" s="16" t="n">
+        <v>211.579533941</v>
+      </c>
+      <c r="G18" s="17">
+        <f>E18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="22" t="n"/>
+      <c r="I18" s="22" t="n"/>
+      <c r="J18" s="17" t="n"/>
+      <c r="K18" s="17">
+        <f>IF(ISNUMBER(J18),J18*F18,"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="23">
+        <f>IF(ISNUMBER(J18),K18-G18,"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="24">
+        <f>IF(ISNUMBER(J18),L18/G18,"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="25">
+        <f>IF(ISNUMBER(H18),H18-C18,"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M17">
+  <conditionalFormatting sqref="L2:M18">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 15:07 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA20" headerRowCount="1">
-  <autoFilter ref="A1:BA20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA32" headerRowCount="1">
+  <autoFilter ref="A1:BA32"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P18" headerRowCount="1">
-  <autoFilter ref="A1:P18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P30" headerRowCount="1">
+  <autoFilter ref="A1:P30"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.6615625</v>
+        <v>46323.67201388889</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.45322916667</v>
+        <v>46323.46368055556</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$20,"BUY")+COUNTIF(Orders!$E$2:$E$20,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$32,"BUY")+COUNTIF(Orders!$E$2:$E$32,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$20,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$32,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$20,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$32,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$20,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$32,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$20,Orders!$E$2:$E$20,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$32,Orders!$E$2:$E$32,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$20,Orders!$E$2:$E$20,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$32,Orders!$E$2:$E$32,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$18,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$18,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$30,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$18)</f>
+        <f>SUM('Round trips'!$L$2:$L$30)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$18,"Closed",'Round trips'!$L$2:$L$18,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$30,"Closed",'Round trips'!$L$2:$L$30,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA20"/>
+  <dimension ref="A1:BA32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4672,6 +4672,2198 @@
       </c>
       <c r="BA20" s="6" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="13" t="n">
+        <v>46323.67184027778</v>
+      </c>
+      <c r="C21" s="13" t="n">
+        <v>46323.46350694444</v>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>46323.63017361111</v>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Analog Devices, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="n">
+        <v>2.460611764</v>
+      </c>
+      <c r="K21" s="17" t="n">
+        <v>425</v>
+      </c>
+      <c r="L21" s="17">
+        <f>IF(AND(ISNUMBER(J21),ISNUMBER(K21)),J21*K21,"")</f>
+        <v/>
+      </c>
+      <c r="M21" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N21" s="16" t="n"/>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P21" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q21" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R21" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S21" s="18" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="T21" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="U21" s="19" t="n">
+        <v>0.0147</v>
+      </c>
+      <c r="V21" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W21" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X21" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA21" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB21" s="15" t="n"/>
+      <c r="AC21" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD21" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE21" s="17" t="n">
+        <v>431.932</v>
+      </c>
+      <c r="AF21" s="17" t="n">
+        <v>413.102</v>
+      </c>
+      <c r="AG21" s="17" t="n">
+        <v>450.762</v>
+      </c>
+      <c r="AH21" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI21" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ21" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK21" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL21" s="15" t="n"/>
+      <c r="AM21" s="17" t="n">
+        <v>424.4</v>
+      </c>
+      <c r="AN21" s="19" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="AO21" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP21" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ21" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR21" s="16" t="n"/>
+      <c r="AS21" s="17" t="n"/>
+      <c r="AT21" s="19" t="n"/>
+      <c r="AU21" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV21" s="6" t="inlineStr">
+        <is>
+          <t>e231ad14-a73b-476f-af0e-82110bbe24ec</t>
+        </is>
+      </c>
+      <c r="AW21" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ADI-1793200046969</t>
+        </is>
+      </c>
+      <c r="AX21" s="13" t="n">
+        <v>46323.63016203704</v>
+      </c>
+      <c r="AY21" s="13" t="n">
+        <v>46323.63017361111</v>
+      </c>
+      <c r="AZ21" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="13" t="n">
+        <v>46323.67185185185</v>
+      </c>
+      <c r="C22" s="13" t="n">
+        <v>46323.46351851852</v>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>46323.63018518518</v>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>Natera, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="n">
+        <v>2.434491107</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>429.56</v>
+      </c>
+      <c r="L22" s="17">
+        <f>IF(AND(ISNUMBER(J22),ISNUMBER(K22)),J22*K22,"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N22" s="16" t="n"/>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P22" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #2, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q22" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R22" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S22" s="18" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="T22" s="12" t="n">
+        <v>65</v>
+      </c>
+      <c r="U22" s="19" t="n">
+        <v>0.0284</v>
+      </c>
+      <c r="V22" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W22" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="X22" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y22" s="19" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="Z22" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA22" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB22" s="15" t="n"/>
+      <c r="AC22" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD22" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE22" s="17" t="n">
+        <v>442.7164</v>
+      </c>
+      <c r="AF22" s="17" t="n">
+        <v>409.2004</v>
+      </c>
+      <c r="AG22" s="17" t="n">
+        <v>476.2324</v>
+      </c>
+      <c r="AH22" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI22" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ22" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK22" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL22" s="15" t="inlineStr">
+        <is>
+          <t>BTIG Maintains Buy on Natera, Raises Price Target to $430</t>
+        </is>
+      </c>
+      <c r="AM22" s="17" t="n">
+        <v>429.31</v>
+      </c>
+      <c r="AN22" s="19" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AO22" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP22" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ22" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR22" s="16" t="n"/>
+      <c r="AS22" s="17" t="n"/>
+      <c r="AT22" s="19" t="n"/>
+      <c r="AU22" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV22" s="6" t="inlineStr">
+        <is>
+          <t>e246d111-60a8-4104-b741-c60e83ced992</t>
+        </is>
+      </c>
+      <c r="AW22" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-NTRA-1793200047226</t>
+        </is>
+      </c>
+      <c r="AX22" s="13" t="n">
+        <v>46323.63017361111</v>
+      </c>
+      <c r="AY22" s="13" t="n">
+        <v>46323.63018518518</v>
+      </c>
+      <c r="AZ22" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="13" t="n">
+        <v>46323.67184027778</v>
+      </c>
+      <c r="C23" s="13" t="n">
+        <v>46323.46350694444</v>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>46323.63017361111</v>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>LNG</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Cheniere Energy Inc</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="n">
+        <v>3.489356022</v>
+      </c>
+      <c r="K23" s="17" t="n">
+        <v>299.7</v>
+      </c>
+      <c r="L23" s="17">
+        <f>IF(AND(ISNUMBER(J23),ISNUMBER(K23)),J23*K23,"")</f>
+        <v/>
+      </c>
+      <c r="M23" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N23" s="16" t="n"/>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P23" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #3, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q23" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S23" s="18" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="T23" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="U23" s="19" t="n">
+        <v>0.0112</v>
+      </c>
+      <c r="V23" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W23" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X23" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA23" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB23" s="15" t="n"/>
+      <c r="AC23" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD23" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE23" s="17" t="n">
+        <v>304.4505</v>
+      </c>
+      <c r="AF23" s="17" t="n">
+        <v>292.3993</v>
+      </c>
+      <c r="AG23" s="17" t="n">
+        <v>316.5016</v>
+      </c>
+      <c r="AH23" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI23" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ23" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK23" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL23" s="15" t="n"/>
+      <c r="AM23" s="17" t="n">
+        <v>299.63</v>
+      </c>
+      <c r="AN23" s="19" t="n">
+        <v>-0.0003</v>
+      </c>
+      <c r="AO23" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP23" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ23" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR23" s="16" t="n"/>
+      <c r="AS23" s="17" t="n"/>
+      <c r="AT23" s="19" t="n"/>
+      <c r="AU23" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV23" s="6" t="inlineStr">
+        <is>
+          <t>ad27f149-a613-4f91-8db8-e8d8a78946b6</t>
+        </is>
+      </c>
+      <c r="AW23" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-LNG-1793200047525</t>
+        </is>
+      </c>
+      <c r="AX23" s="13" t="n">
+        <v>46323.63017361111</v>
+      </c>
+      <c r="AY23" s="13" t="n">
+        <v>46323.63017361111</v>
+      </c>
+      <c r="AZ23" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>46323.67185185185</v>
+      </c>
+      <c r="C24" s="13" t="n">
+        <v>46323.46351851852</v>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>46323.63018518518</v>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>Altria Group, Inc.</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="n">
+        <v>14.214489601</v>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v>73.56999999999999</v>
+      </c>
+      <c r="L24" s="17">
+        <f>IF(AND(ISNUMBER(J24),ISNUMBER(K24)),J24*K24,"")</f>
+        <v/>
+      </c>
+      <c r="M24" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N24" s="16" t="n"/>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P24" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q24" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R24" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S24" s="18" t="n">
+        <v>0.644</v>
+      </c>
+      <c r="T24" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="U24" s="19" t="n">
+        <v>0.0097</v>
+      </c>
+      <c r="V24" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W24" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X24" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y24" s="19" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="Z24" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA24" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB24" s="15" t="n"/>
+      <c r="AC24" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD24" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE24" s="17" t="n">
+        <v>74.5009</v>
+      </c>
+      <c r="AF24" s="17" t="n">
+        <v>72.1861</v>
+      </c>
+      <c r="AG24" s="17" t="n">
+        <v>76.8158</v>
+      </c>
+      <c r="AH24" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI24" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ24" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK24" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL24" s="15" t="n"/>
+      <c r="AM24" s="17" t="n">
+        <v>73.56</v>
+      </c>
+      <c r="AN24" s="19" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="AO24" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP24" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ24" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR24" s="16" t="n"/>
+      <c r="AS24" s="17" t="n"/>
+      <c r="AT24" s="19" t="n"/>
+      <c r="AU24" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV24" s="6" t="inlineStr">
+        <is>
+          <t>d54a6aee-45fb-4487-a477-f8cb923f7fd6</t>
+        </is>
+      </c>
+      <c r="AW24" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MO-1793200047792</t>
+        </is>
+      </c>
+      <c r="AX24" s="13" t="n">
+        <v>46323.63017361111</v>
+      </c>
+      <c r="AY24" s="13" t="n">
+        <v>46323.63018518518</v>
+      </c>
+      <c r="AZ24" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>46323.67186342592</v>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>46323.46353009259</v>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>The Kroger Co.</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="n">
+        <v>15.948757053</v>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v>65.56999999999999</v>
+      </c>
+      <c r="L25" s="17">
+        <f>IF(AND(ISNUMBER(J25),ISNUMBER(K25)),J25*K25,"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N25" s="16" t="n"/>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P25" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #5, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q25" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R25" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S25" s="18" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="T25" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="U25" s="19" t="n">
+        <v>0.0136</v>
+      </c>
+      <c r="V25" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W25" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X25" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y25" s="19" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="Z25" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA25" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB25" s="15" t="n"/>
+      <c r="AC25" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD25" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE25" s="17" t="n">
+        <v>66.62949999999999</v>
+      </c>
+      <c r="AF25" s="17" t="n">
+        <v>63.9933</v>
+      </c>
+      <c r="AG25" s="17" t="n">
+        <v>69.26560000000001</v>
+      </c>
+      <c r="AH25" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI25" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ25" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK25" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL25" s="15" t="inlineStr">
+        <is>
+          <t>Evercore Maintains Buy Rating on The Kroger Co.</t>
+        </is>
+      </c>
+      <c r="AM25" s="17" t="n">
+        <v>65.56</v>
+      </c>
+      <c r="AN25" s="19" t="n">
+        <v>-0.0043</v>
+      </c>
+      <c r="AO25" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP25" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ25" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR25" s="16" t="n"/>
+      <c r="AS25" s="17" t="n"/>
+      <c r="AT25" s="19" t="n"/>
+      <c r="AU25" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV25" s="6" t="inlineStr">
+        <is>
+          <t>c3da3c32-f2c1-4d43-a318-6418c1dfd3c8</t>
+        </is>
+      </c>
+      <c r="AW25" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-KR-1793200048071</t>
+        </is>
+      </c>
+      <c r="AX25" s="13" t="n">
+        <v>46323.63018518518</v>
+      </c>
+      <c r="AY25" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="AZ25" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="13" t="n">
+        <v>46323.67186342592</v>
+      </c>
+      <c r="C26" s="13" t="n">
+        <v>46323.46353009259</v>
+      </c>
+      <c r="D26" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Public Limited Company Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J26" s="16" t="n">
+        <v>3.263614517</v>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>320.43</v>
+      </c>
+      <c r="L26" s="17">
+        <f>IF(AND(ISNUMBER(J26),ISNUMBER(K26)),J26*K26,"")</f>
+        <v/>
+      </c>
+      <c r="M26" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N26" s="16" t="n"/>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P26" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #6, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q26" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R26" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S26" s="18" t="n">
+        <v>0.621</v>
+      </c>
+      <c r="T26" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U26" s="19" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="V26" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W26" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="X26" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y26" s="19" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Z26" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA26" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB26" s="15" t="n"/>
+      <c r="AC26" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD26" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE26" s="17" t="n">
+        <v>324.7385</v>
+      </c>
+      <c r="AF26" s="17" t="n">
+        <v>313.4173</v>
+      </c>
+      <c r="AG26" s="17" t="n">
+        <v>336.0597</v>
+      </c>
+      <c r="AH26" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI26" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ26" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK26" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL26" s="15" t="n"/>
+      <c r="AM26" s="17" t="n">
+        <v>320.21</v>
+      </c>
+      <c r="AN26" s="19" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="AO26" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP26" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ26" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR26" s="16" t="n"/>
+      <c r="AS26" s="17" t="n"/>
+      <c r="AT26" s="19" t="n"/>
+      <c r="AU26" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV26" s="6" t="inlineStr">
+        <is>
+          <t>5e449b92-c7e8-4ba7-84b2-04178ba9b5a4</t>
+        </is>
+      </c>
+      <c r="AW26" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-WTW-1793200048329</t>
+        </is>
+      </c>
+      <c r="AX26" s="13" t="n">
+        <v>46323.63018518518</v>
+      </c>
+      <c r="AY26" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="AZ26" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="13" t="n">
+        <v>46323.67186342592</v>
+      </c>
+      <c r="C27" s="13" t="n">
+        <v>46323.46353009259</v>
+      </c>
+      <c r="D27" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>ABBVIE INC.</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="n">
+        <v>3.63060686</v>
+      </c>
+      <c r="K27" s="17" t="n">
+        <v>288.04</v>
+      </c>
+      <c r="L27" s="17">
+        <f>IF(AND(ISNUMBER(J27),ISNUMBER(K27)),J27*K27,"")</f>
+        <v/>
+      </c>
+      <c r="M27" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N27" s="16" t="n"/>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P27" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #8, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q27" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R27" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S27" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T27" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U27" s="19" t="n">
+        <v>0.0177</v>
+      </c>
+      <c r="V27" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W27" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="X27" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y27" s="19" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Z27" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA27" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB27" s="15" t="n"/>
+      <c r="AC27" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD27" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE27" s="17" t="n">
+        <v>291.4779</v>
+      </c>
+      <c r="AF27" s="17" t="n">
+        <v>283.5332</v>
+      </c>
+      <c r="AG27" s="17" t="n">
+        <v>299.4226</v>
+      </c>
+      <c r="AH27" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI27" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ27" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK27" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL27" s="15" t="inlineStr">
+        <is>
+          <t>AbbVie Submits BLA for Etentamig to FDA for Multiple Myeloma</t>
+        </is>
+      </c>
+      <c r="AM27" s="17" t="n">
+        <v>288.3</v>
+      </c>
+      <c r="AN27" s="19" t="n">
+        <v>0.0067</v>
+      </c>
+      <c r="AO27" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP27" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ27" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR27" s="16" t="n"/>
+      <c r="AS27" s="17" t="n"/>
+      <c r="AT27" s="19" t="n"/>
+      <c r="AU27" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV27" s="6" t="inlineStr">
+        <is>
+          <t>8eb89be2-4ca4-45d4-910e-1f166d4d8478</t>
+        </is>
+      </c>
+      <c r="AW27" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ABBV-1793200048709</t>
+        </is>
+      </c>
+      <c r="AX27" s="13" t="n">
+        <v>46323.63018518518</v>
+      </c>
+      <c r="AY27" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="AZ27" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="13" t="n">
+        <v>46323.67188657408</v>
+      </c>
+      <c r="C28" s="13" t="n">
+        <v>46323.46355324074</v>
+      </c>
+      <c r="D28" s="13" t="n">
+        <v>46323.63021990741</v>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr">
+        <is>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J28" s="16" t="n">
+        <v>21.932885906</v>
+      </c>
+      <c r="K28" s="17" t="n">
+        <v>47.68</v>
+      </c>
+      <c r="L28" s="17">
+        <f>IF(AND(ISNUMBER(J28),ISNUMBER(K28)),J28*K28,"")</f>
+        <v/>
+      </c>
+      <c r="M28" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N28" s="16" t="n"/>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P28" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #11, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q28" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R28" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S28" s="18" t="n">
+        <v>0.662</v>
+      </c>
+      <c r="T28" s="12" t="n">
+        <v>77</v>
+      </c>
+      <c r="U28" s="19" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="V28" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W28" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="X28" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y28" s="19" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="Z28" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA28" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB28" s="15" t="n"/>
+      <c r="AC28" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD28" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE28" s="17" t="n">
+        <v>48.5643</v>
+      </c>
+      <c r="AF28" s="17" t="n">
+        <v>46.2786</v>
+      </c>
+      <c r="AG28" s="17" t="n">
+        <v>50.85</v>
+      </c>
+      <c r="AH28" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI28" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ28" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK28" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL28" s="15" t="inlineStr">
+        <is>
+          <t>Equinor Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM28" s="17" t="n">
+        <v>47.63</v>
+      </c>
+      <c r="AN28" s="19" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="AO28" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP28" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ28" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR28" s="16" t="n"/>
+      <c r="AS28" s="17" t="n"/>
+      <c r="AT28" s="19" t="n"/>
+      <c r="AU28" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV28" s="6" t="inlineStr">
+        <is>
+          <t>b2ebe048-4e00-46e3-ad7e-fd294b463157</t>
+        </is>
+      </c>
+      <c r="AW28" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EQNR-1793200049275</t>
+        </is>
+      </c>
+      <c r="AX28" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="AY28" s="13" t="n">
+        <v>46323.63021990741</v>
+      </c>
+      <c r="AZ28" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="13" t="n">
+        <v>46323.671875</v>
+      </c>
+      <c r="C29" s="13" t="n">
+        <v>46323.46354166666</v>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>46323.63020833334</v>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J29" s="16" t="n">
+        <v>3.676298952</v>
+      </c>
+      <c r="K29" s="17" t="n">
+        <v>284.46</v>
+      </c>
+      <c r="L29" s="17">
+        <f>IF(AND(ISNUMBER(J29),ISNUMBER(K29)),J29*K29,"")</f>
+        <v/>
+      </c>
+      <c r="M29" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N29" s="16" t="n"/>
+      <c r="O29" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P29" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #12, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q29" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R29" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S29" s="18" t="n">
+        <v>0.648</v>
+      </c>
+      <c r="T29" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="U29" s="19" t="n">
+        <v>0.0132</v>
+      </c>
+      <c r="V29" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W29" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="X29" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y29" s="19" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="Z29" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA29" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB29" s="15" t="n"/>
+      <c r="AC29" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD29" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE29" s="17" t="n">
+        <v>288.7555</v>
+      </c>
+      <c r="AF29" s="17" t="n">
+        <v>278.8917</v>
+      </c>
+      <c r="AG29" s="17" t="n">
+        <v>298.6194</v>
+      </c>
+      <c r="AH29" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI29" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ29" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK29" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL29" s="15" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing Q1 2027 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM29" s="17" t="n">
+        <v>284.29</v>
+      </c>
+      <c r="AN29" s="19" t="n">
+        <v>-0.0278</v>
+      </c>
+      <c r="AO29" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP29" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ29" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR29" s="16" t="n"/>
+      <c r="AS29" s="17" t="n"/>
+      <c r="AT29" s="19" t="n"/>
+      <c r="AU29" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV29" s="6" t="inlineStr">
+        <is>
+          <t>ebfbb0f0-7770-43ff-9da5-d7832ec8fefe</t>
+        </is>
+      </c>
+      <c r="AW29" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ADP-1793200049536</t>
+        </is>
+      </c>
+      <c r="AX29" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="AY29" s="13" t="n">
+        <v>46323.63020833334</v>
+      </c>
+      <c r="AZ29" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="13" t="n">
+        <v>46323.67188657408</v>
+      </c>
+      <c r="C30" s="13" t="n">
+        <v>46323.46355324074</v>
+      </c>
+      <c r="D30" s="13" t="n">
+        <v>46323.63021990741</v>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="G30" s="15" t="inlineStr">
+        <is>
+          <t>Cognizant Technology Solutions Corporation Class A Common Stock</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J30" s="16" t="n">
+        <v>15.713899323</v>
+      </c>
+      <c r="K30" s="17" t="n">
+        <v>66.55</v>
+      </c>
+      <c r="L30" s="17">
+        <f>IF(AND(ISNUMBER(J30),ISNUMBER(K30)),J30*K30,"")</f>
+        <v/>
+      </c>
+      <c r="M30" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N30" s="16" t="n"/>
+      <c r="O30" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P30" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #13, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q30" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R30" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S30" s="18" t="n">
+        <v>0.587</v>
+      </c>
+      <c r="T30" s="12" t="n">
+        <v>46</v>
+      </c>
+      <c r="U30" s="19" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="V30" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W30" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="X30" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y30" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z30" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA30" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB30" s="15" t="n"/>
+      <c r="AC30" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD30" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE30" s="17" t="n">
+        <v>68.1648</v>
+      </c>
+      <c r="AF30" s="17" t="n">
+        <v>64.25279999999999</v>
+      </c>
+      <c r="AG30" s="17" t="n">
+        <v>72.0767</v>
+      </c>
+      <c r="AH30" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI30" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ30" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK30" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL30" s="15" t="inlineStr">
+        <is>
+          <t>Morgan Stanley Downgrades Cognizant Technology Solutions to Neutral</t>
+        </is>
+      </c>
+      <c r="AM30" s="17" t="n">
+        <v>66.58</v>
+      </c>
+      <c r="AN30" s="19" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="AO30" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP30" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ30" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR30" s="16" t="n"/>
+      <c r="AS30" s="17" t="n"/>
+      <c r="AT30" s="19" t="n"/>
+      <c r="AU30" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV30" s="6" t="inlineStr">
+        <is>
+          <t>96d36240-c72a-4a79-8467-1c5b3b8d6462</t>
+        </is>
+      </c>
+      <c r="AW30" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-CTSH-1793200049798</t>
+        </is>
+      </c>
+      <c r="AX30" s="13" t="n">
+        <v>46323.63019675926</v>
+      </c>
+      <c r="AY30" s="13" t="n">
+        <v>46323.63021990741</v>
+      </c>
+      <c r="AZ30" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="13" t="n">
+        <v>46323.671875</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>46323.46354166666</v>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>46323.63020833334</v>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J31" s="16" t="n">
+        <v>1.704058088</v>
+      </c>
+      <c r="K31" s="17" t="n">
+        <v>613.688</v>
+      </c>
+      <c r="L31" s="17">
+        <f>IF(AND(ISNUMBER(J31),ISNUMBER(K31)),J31*K31,"")</f>
+        <v/>
+      </c>
+      <c r="M31" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N31" s="16" t="n"/>
+      <c r="O31" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P31" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #14, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q31" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R31" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S31" s="18" t="n">
+        <v>0.553</v>
+      </c>
+      <c r="T31" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="U31" s="19" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="V31" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W31" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="X31" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y31" s="19" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Z31" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA31" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB31" s="15" t="n"/>
+      <c r="AC31" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD31" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE31" s="17" t="n">
+        <v>620.3299</v>
+      </c>
+      <c r="AF31" s="17" t="n">
+        <v>604.5177</v>
+      </c>
+      <c r="AG31" s="17" t="n">
+        <v>636.1421</v>
+      </c>
+      <c r="AH31" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI31" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ31" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK31" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL31" s="15" t="inlineStr">
+        <is>
+          <t>Visa Earnings Prediction Market Preview: What Will Ryan McInerney Say?</t>
+        </is>
+      </c>
+      <c r="AM31" s="17" t="n">
+        <v>613.705</v>
+      </c>
+      <c r="AN31" s="19" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="AO31" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP31" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ31" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR31" s="16" t="n"/>
+      <c r="AS31" s="17" t="n"/>
+      <c r="AT31" s="19" t="n"/>
+      <c r="AU31" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV31" s="6" t="inlineStr">
+        <is>
+          <t>394e3ad3-8d54-4448-ba7c-fce04cf9d2f4</t>
+        </is>
+      </c>
+      <c r="AW31" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MA-1793200050051</t>
+        </is>
+      </c>
+      <c r="AX31" s="13" t="n">
+        <v>46323.63020833334</v>
+      </c>
+      <c r="AY31" s="13" t="n">
+        <v>46323.63020833334</v>
+      </c>
+      <c r="AZ31" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>46323.671875</v>
+      </c>
+      <c r="C32" s="13" t="n">
+        <v>46323.46354166666</v>
+      </c>
+      <c r="D32" s="13" t="n">
+        <v>46323.63020833334</v>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>CNC</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>Centene Corporation</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J32" s="16" t="n">
+        <v>15.180142255</v>
+      </c>
+      <c r="K32" s="17" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="L32" s="17">
+        <f>IF(AND(ISNUMBER(J32),ISNUMBER(K32)),J32*K32,"")</f>
+        <v/>
+      </c>
+      <c r="M32" s="17" t="n">
+        <v>1045.77</v>
+      </c>
+      <c r="N32" s="16" t="n"/>
+      <c r="O32" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P32" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #15, 8.33% of the $12,554.32 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q32" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R32" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S32" s="18" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="T32" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="U32" s="19" t="n">
+        <v>0.0126</v>
+      </c>
+      <c r="V32" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W32" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="X32" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y32" s="19" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="Z32" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA32" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB32" s="15" t="n"/>
+      <c r="AC32" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD32" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE32" s="17" t="n">
+        <v>70.1768</v>
+      </c>
+      <c r="AF32" s="17" t="n">
+        <v>66.9598</v>
+      </c>
+      <c r="AG32" s="17" t="n">
+        <v>73.3939</v>
+      </c>
+      <c r="AH32" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI32" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ32" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK32" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL32" s="15" t="inlineStr">
+        <is>
+          <t>Cantor Fitzgerald Upgrades Centene to Overweight and Raises Price Target to $79</t>
+        </is>
+      </c>
+      <c r="AM32" s="17" t="n">
+        <v>68.94</v>
+      </c>
+      <c r="AN32" s="19" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="AO32" s="17" t="n">
+        <v>100357.58</v>
+      </c>
+      <c r="AP32" s="17" t="n">
+        <v>12554.32</v>
+      </c>
+      <c r="AQ32" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR32" s="16" t="n"/>
+      <c r="AS32" s="17" t="n"/>
+      <c r="AT32" s="19" t="n"/>
+      <c r="AU32" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV32" s="6" t="inlineStr">
+        <is>
+          <t>545413f4-a3a5-4501-a6a3-27a435a4337f</t>
+        </is>
+      </c>
+      <c r="AW32" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-CNC-1793200050304</t>
+        </is>
+      </c>
+      <c r="AX32" s="13" t="n">
+        <v>46323.63020833334</v>
+      </c>
+      <c r="AY32" s="13" t="n">
+        <v>46323.63020833334</v>
+      </c>
+      <c r="AZ32" s="13" t="n">
+        <v>46323.62954861111</v>
+      </c>
+      <c r="BA32" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -4687,7 +6879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5741,8 +7933,644 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>LNG</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Cheniere Energy Inc</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="n">
+        <v>46323.67184027778</v>
+      </c>
+      <c r="D19" s="22" t="n">
+        <v>46323.46350694444</v>
+      </c>
+      <c r="E19" s="17" t="n">
+        <v>299.7</v>
+      </c>
+      <c r="F19" s="16" t="n">
+        <v>3.489356022</v>
+      </c>
+      <c r="G19" s="17">
+        <f>E19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="22" t="n"/>
+      <c r="I19" s="22" t="n"/>
+      <c r="J19" s="17" t="n"/>
+      <c r="K19" s="17">
+        <f>IF(ISNUMBER(J19),J19*F19,"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="23">
+        <f>IF(ISNUMBER(J19),K19-G19,"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="24">
+        <f>IF(ISNUMBER(J19),L19/G19,"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="25">
+        <f>IF(ISNUMBER(H19),H19-C19,"")</f>
+        <v/>
+      </c>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Analog Devices, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="n">
+        <v>46323.67184027778</v>
+      </c>
+      <c r="D20" s="22" t="n">
+        <v>46323.46350694444</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <v>425</v>
+      </c>
+      <c r="F20" s="16" t="n">
+        <v>2.460611764</v>
+      </c>
+      <c r="G20" s="17">
+        <f>E20*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="22" t="n"/>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="17" t="n"/>
+      <c r="K20" s="17">
+        <f>IF(ISNUMBER(J20),J20*F20,"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="23">
+        <f>IF(ISNUMBER(J20),K20-G20,"")</f>
+        <v/>
+      </c>
+      <c r="M20" s="24">
+        <f>IF(ISNUMBER(J20),L20/G20,"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="25">
+        <f>IF(ISNUMBER(H20),H20-C20,"")</f>
+        <v/>
+      </c>
+      <c r="O20" s="6" t="n"/>
+      <c r="P20" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Natera, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="n">
+        <v>46323.67185185185</v>
+      </c>
+      <c r="D21" s="22" t="n">
+        <v>46323.46351851852</v>
+      </c>
+      <c r="E21" s="17" t="n">
+        <v>429.56</v>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>2.434491107</v>
+      </c>
+      <c r="G21" s="17">
+        <f>E21*F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="22" t="n"/>
+      <c r="I21" s="22" t="n"/>
+      <c r="J21" s="17" t="n"/>
+      <c r="K21" s="17">
+        <f>IF(ISNUMBER(J21),J21*F21,"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="23">
+        <f>IF(ISNUMBER(J21),K21-G21,"")</f>
+        <v/>
+      </c>
+      <c r="M21" s="24">
+        <f>IF(ISNUMBER(J21),L21/G21,"")</f>
+        <v/>
+      </c>
+      <c r="N21" s="25">
+        <f>IF(ISNUMBER(H21),H21-C21,"")</f>
+        <v/>
+      </c>
+      <c r="O21" s="6" t="n"/>
+      <c r="P21" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Altria Group, Inc.</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="n">
+        <v>46323.67185185185</v>
+      </c>
+      <c r="D22" s="22" t="n">
+        <v>46323.46351851852</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>73.56999999999999</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>14.214489601</v>
+      </c>
+      <c r="G22" s="17">
+        <f>E22*F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="22" t="n"/>
+      <c r="I22" s="22" t="n"/>
+      <c r="J22" s="17" t="n"/>
+      <c r="K22" s="17">
+        <f>IF(ISNUMBER(J22),J22*F22,"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="23">
+        <f>IF(ISNUMBER(J22),K22-G22,"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="24">
+        <f>IF(ISNUMBER(J22),L22/G22,"")</f>
+        <v/>
+      </c>
+      <c r="N22" s="25">
+        <f>IF(ISNUMBER(H22),H22-C22,"")</f>
+        <v/>
+      </c>
+      <c r="O22" s="6" t="n"/>
+      <c r="P22" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Public Limited Company Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="n">
+        <v>46323.67186342592</v>
+      </c>
+      <c r="D23" s="22" t="n">
+        <v>46323.46353009259</v>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>320.43</v>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>3.263614517</v>
+      </c>
+      <c r="G23" s="17">
+        <f>E23*F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="22" t="n"/>
+      <c r="I23" s="22" t="n"/>
+      <c r="J23" s="17" t="n"/>
+      <c r="K23" s="17">
+        <f>IF(ISNUMBER(J23),J23*F23,"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="23">
+        <f>IF(ISNUMBER(J23),K23-G23,"")</f>
+        <v/>
+      </c>
+      <c r="M23" s="24">
+        <f>IF(ISNUMBER(J23),L23/G23,"")</f>
+        <v/>
+      </c>
+      <c r="N23" s="25">
+        <f>IF(ISNUMBER(H23),H23-C23,"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="6" t="n"/>
+      <c r="P23" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>The Kroger Co.</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>46323.67186342592</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>46323.46353009259</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>65.56999999999999</v>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>15.948757053</v>
+      </c>
+      <c r="G24" s="17">
+        <f>E24*F24</f>
+        <v/>
+      </c>
+      <c r="H24" s="22" t="n"/>
+      <c r="I24" s="22" t="n"/>
+      <c r="J24" s="17" t="n"/>
+      <c r="K24" s="17">
+        <f>IF(ISNUMBER(J24),J24*F24,"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="23">
+        <f>IF(ISNUMBER(J24),K24-G24,"")</f>
+        <v/>
+      </c>
+      <c r="M24" s="24">
+        <f>IF(ISNUMBER(J24),L24/G24,"")</f>
+        <v/>
+      </c>
+      <c r="N24" s="25">
+        <f>IF(ISNUMBER(H24),H24-C24,"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="6" t="n"/>
+      <c r="P24" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>ABBVIE INC.</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>46323.67186342592</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>46323.46353009259</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>288.04</v>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>3.63060686</v>
+      </c>
+      <c r="G25" s="17">
+        <f>E25*F25</f>
+        <v/>
+      </c>
+      <c r="H25" s="22" t="n"/>
+      <c r="I25" s="22" t="n"/>
+      <c r="J25" s="17" t="n"/>
+      <c r="K25" s="17">
+        <f>IF(ISNUMBER(J25),J25*F25,"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="23">
+        <f>IF(ISNUMBER(J25),K25-G25,"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="24">
+        <f>IF(ISNUMBER(J25),L25/G25,"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="25">
+        <f>IF(ISNUMBER(H25),H25-C25,"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="6" t="n"/>
+      <c r="P25" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>46323.671875</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <v>46323.46354166666</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>613.688</v>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>1.704058088</v>
+      </c>
+      <c r="G26" s="17">
+        <f>E26*F26</f>
+        <v/>
+      </c>
+      <c r="H26" s="22" t="n"/>
+      <c r="I26" s="22" t="n"/>
+      <c r="J26" s="17" t="n"/>
+      <c r="K26" s="17">
+        <f>IF(ISNUMBER(J26),J26*F26,"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="23">
+        <f>IF(ISNUMBER(J26),K26-G26,"")</f>
+        <v/>
+      </c>
+      <c r="M26" s="24">
+        <f>IF(ISNUMBER(J26),L26/G26,"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="25">
+        <f>IF(ISNUMBER(H26),H26-C26,"")</f>
+        <v/>
+      </c>
+      <c r="O26" s="6" t="n"/>
+      <c r="P26" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>46323.671875</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <v>46323.46354166666</v>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>284.46</v>
+      </c>
+      <c r="F27" s="16" t="n">
+        <v>3.676298952</v>
+      </c>
+      <c r="G27" s="17">
+        <f>E27*F27</f>
+        <v/>
+      </c>
+      <c r="H27" s="22" t="n"/>
+      <c r="I27" s="22" t="n"/>
+      <c r="J27" s="17" t="n"/>
+      <c r="K27" s="17">
+        <f>IF(ISNUMBER(J27),J27*F27,"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="23">
+        <f>IF(ISNUMBER(J27),K27-G27,"")</f>
+        <v/>
+      </c>
+      <c r="M27" s="24">
+        <f>IF(ISNUMBER(J27),L27/G27,"")</f>
+        <v/>
+      </c>
+      <c r="N27" s="25">
+        <f>IF(ISNUMBER(H27),H27-C27,"")</f>
+        <v/>
+      </c>
+      <c r="O27" s="6" t="n"/>
+      <c r="P27" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>CNC</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Centene Corporation</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>46323.671875</v>
+      </c>
+      <c r="D28" s="22" t="n">
+        <v>46323.46354166666</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="F28" s="16" t="n">
+        <v>15.180142255</v>
+      </c>
+      <c r="G28" s="17">
+        <f>E28*F28</f>
+        <v/>
+      </c>
+      <c r="H28" s="22" t="n"/>
+      <c r="I28" s="22" t="n"/>
+      <c r="J28" s="17" t="n"/>
+      <c r="K28" s="17">
+        <f>IF(ISNUMBER(J28),J28*F28,"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="23">
+        <f>IF(ISNUMBER(J28),K28-G28,"")</f>
+        <v/>
+      </c>
+      <c r="M28" s="24">
+        <f>IF(ISNUMBER(J28),L28/G28,"")</f>
+        <v/>
+      </c>
+      <c r="N28" s="25">
+        <f>IF(ISNUMBER(H28),H28-C28,"")</f>
+        <v/>
+      </c>
+      <c r="O28" s="6" t="n"/>
+      <c r="P28" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Cognizant Technology Solutions Corporation Class A Common Stock</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="n">
+        <v>46323.67188657408</v>
+      </c>
+      <c r="D29" s="22" t="n">
+        <v>46323.46355324074</v>
+      </c>
+      <c r="E29" s="17" t="n">
+        <v>66.55</v>
+      </c>
+      <c r="F29" s="16" t="n">
+        <v>15.713899323</v>
+      </c>
+      <c r="G29" s="17">
+        <f>E29*F29</f>
+        <v/>
+      </c>
+      <c r="H29" s="22" t="n"/>
+      <c r="I29" s="22" t="n"/>
+      <c r="J29" s="17" t="n"/>
+      <c r="K29" s="17">
+        <f>IF(ISNUMBER(J29),J29*F29,"")</f>
+        <v/>
+      </c>
+      <c r="L29" s="23">
+        <f>IF(ISNUMBER(J29),K29-G29,"")</f>
+        <v/>
+      </c>
+      <c r="M29" s="24">
+        <f>IF(ISNUMBER(J29),L29/G29,"")</f>
+        <v/>
+      </c>
+      <c r="N29" s="25">
+        <f>IF(ISNUMBER(H29),H29-C29,"")</f>
+        <v/>
+      </c>
+      <c r="O29" s="6" t="n"/>
+      <c r="P29" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="n">
+        <v>46323.67188657408</v>
+      </c>
+      <c r="D30" s="22" t="n">
+        <v>46323.46355324074</v>
+      </c>
+      <c r="E30" s="17" t="n">
+        <v>47.68</v>
+      </c>
+      <c r="F30" s="16" t="n">
+        <v>21.932885906</v>
+      </c>
+      <c r="G30" s="17">
+        <f>E30*F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="22" t="n"/>
+      <c r="I30" s="22" t="n"/>
+      <c r="J30" s="17" t="n"/>
+      <c r="K30" s="17">
+        <f>IF(ISNUMBER(J30),J30*F30,"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="23">
+        <f>IF(ISNUMBER(J30),K30-G30,"")</f>
+        <v/>
+      </c>
+      <c r="M30" s="24">
+        <f>IF(ISNUMBER(J30),L30/G30,"")</f>
+        <v/>
+      </c>
+      <c r="N30" s="25">
+        <f>IF(ISNUMBER(H30),H30-C30,"")</f>
+        <v/>
+      </c>
+      <c r="O30" s="6" t="n"/>
+      <c r="P30" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M18">
+  <conditionalFormatting sqref="L2:M30">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -5896,7 +8724,7 @@
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>Each buy uses 8.33% of the cash available at that moment, repeated for every buy-ready stock (up to 12 stocks, orders of at least $5); never buys back a stock sold the same day</t>
+          <t>Each buy uses 8.33% of the cash available at that moment, repeated for every buy-ready stock (up to 100 stocks, orders of at least $5); never buys back a stock sold the same day</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-28 15:09 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA32" headerRowCount="1">
-  <autoFilter ref="A1:BA32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA33" headerRowCount="1">
+  <autoFilter ref="A1:BA33"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.67201388889</v>
+        <v>46323.67351851852</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.46368055556</v>
+        <v>46323.46518518519</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$32,"BUY")+COUNTIF(Orders!$E$2:$E$32,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$33,"BUY")+COUNTIF(Orders!$E$2:$E$33,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$32,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$33,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$32,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$33,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$32,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$33,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$32,Orders!$E$2:$E$32,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$33,Orders!$E$2:$E$33,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$32,Orders!$E$2:$E$32,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$33,Orders!$E$2:$E$33,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA32"/>
+  <dimension ref="A1:BA33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6864,6 +6864,194 @@
       </c>
       <c r="BA32" s="6" t="n"/>
     </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="13" t="n">
+        <v>46323.67340277778</v>
+      </c>
+      <c r="C33" s="13" t="n">
+        <v>46323.46506944444</v>
+      </c>
+      <c r="D33" s="13" t="n">
+        <v>46323.63173611111</v>
+      </c>
+      <c r="E33" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J33" s="16" t="n">
+        <v>3.676298952</v>
+      </c>
+      <c r="K33" s="17" t="n">
+        <v>283.51</v>
+      </c>
+      <c r="L33" s="17">
+        <f>IF(AND(ISNUMBER(J33),ISNUMBER(K33)),J33*K33,"")</f>
+        <v/>
+      </c>
+      <c r="M33" s="17" t="n"/>
+      <c r="N33" s="16" t="n">
+        <v>3.676298952</v>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P33" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 3.1% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q33" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R33" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S33" s="18" t="n">
+        <v>0.648</v>
+      </c>
+      <c r="T33" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="U33" s="19" t="n">
+        <v>0.0132</v>
+      </c>
+      <c r="V33" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W33" s="12" t="n"/>
+      <c r="X33" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y33" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z33" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA33" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB33" s="15" t="n"/>
+      <c r="AC33" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD33" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE33" s="17" t="n">
+        <v>288.361</v>
+      </c>
+      <c r="AF33" s="17" t="n">
+        <v>278.4835</v>
+      </c>
+      <c r="AG33" s="17" t="n">
+        <v>298.2385</v>
+      </c>
+      <c r="AH33" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI33" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ33" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK33" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL33" s="15" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing Q1 2027 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM33" s="17" t="n">
+        <v>284.44</v>
+      </c>
+      <c r="AN33" s="19" t="n">
+        <v>-0.0291</v>
+      </c>
+      <c r="AO33" s="17" t="n">
+        <v>100436.88</v>
+      </c>
+      <c r="AP33" s="17" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="AQ33" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR33" s="16" t="n">
+        <v>3.676298952</v>
+      </c>
+      <c r="AS33" s="17" t="n">
+        <v>284.46</v>
+      </c>
+      <c r="AT33" s="19" t="n">
+        <v>-0.0017</v>
+      </c>
+      <c r="AU33" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV33" s="6" t="inlineStr">
+        <is>
+          <t>91487c54-b2fb-4b1a-a476-77ac1f697fc3</t>
+        </is>
+      </c>
+      <c r="AW33" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-ADP-1793200180561</t>
+        </is>
+      </c>
+      <c r="AX33" s="13" t="n">
+        <v>46323.63171296296</v>
+      </c>
+      <c r="AY33" s="13" t="n">
+        <v>46323.63173611111</v>
+      </c>
+      <c r="AZ33" s="13" t="n">
+        <v>46323.63150462963</v>
+      </c>
+      <c r="BA33" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -8384,9 +8572,15 @@
         <f>E27*F27</f>
         <v/>
       </c>
-      <c r="H27" s="22" t="n"/>
-      <c r="I27" s="22" t="n"/>
-      <c r="J27" s="17" t="n"/>
+      <c r="H27" s="22" t="n">
+        <v>46323.67340277778</v>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>46323.46506944444</v>
+      </c>
+      <c r="J27" s="17" t="n">
+        <v>283.51</v>
+      </c>
       <c r="K27" s="17">
         <f>IF(ISNUMBER(J27),J27*F27,"")</f>
         <v/>
@@ -8403,10 +8597,14 @@
         <f>IF(ISNUMBER(H27),H27-C27,"")</f>
         <v/>
       </c>
-      <c r="O27" s="6" t="n"/>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-28 15:16 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA33" headerRowCount="1">
-  <autoFilter ref="A1:BA33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA37" headerRowCount="1">
+  <autoFilter ref="A1:BA37"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P30" headerRowCount="1">
-  <autoFilter ref="A1:P30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P34" headerRowCount="1">
+  <autoFilter ref="A1:P34"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.67351851852</v>
+        <v>46323.67783564814</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.46518518519</v>
+        <v>46323.46950231482</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$33,"BUY")+COUNTIF(Orders!$E$2:$E$33,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$37,"BUY")+COUNTIF(Orders!$E$2:$E$37,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$33,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$37,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$33,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$37,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$33,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$37,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$33,Orders!$E$2:$E$33,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$37,Orders!$E$2:$E$37,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$33,Orders!$E$2:$E$33,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$37,Orders!$E$2:$E$37,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$34,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$30,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$34,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$30)</f>
+        <f>SUM('Round trips'!$L$2:$L$34)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$30,"Closed",'Round trips'!$L$2:$L$30,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$34,"Closed",'Round trips'!$L$2:$L$34,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA33"/>
+  <dimension ref="A1:BA37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7052,6 +7052,758 @@
       </c>
       <c r="BA33" s="6" t="n"/>
     </row>
+    <row r="34">
+      <c r="A34" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="13" t="n">
+        <v>46323.67767361111</v>
+      </c>
+      <c r="C34" s="13" t="n">
+        <v>46323.46934027778</v>
+      </c>
+      <c r="D34" s="13" t="n">
+        <v>46323.63600694444</v>
+      </c>
+      <c r="E34" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J34" s="16" t="n">
+        <v>0.852029044</v>
+      </c>
+      <c r="K34" s="17" t="n">
+        <v>614.554</v>
+      </c>
+      <c r="L34" s="17">
+        <f>IF(AND(ISNUMBER(J34),ISNUMBER(K34)),J34*K34,"")</f>
+        <v/>
+      </c>
+      <c r="M34" s="17" t="n"/>
+      <c r="N34" s="16" t="n">
+        <v>0.852029044</v>
+      </c>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P34" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q34" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R34" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S34" s="18" t="n">
+        <v>0.553</v>
+      </c>
+      <c r="T34" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="U34" s="19" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="V34" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W34" s="12" t="n"/>
+      <c r="X34" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y34" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z34" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA34" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB34" s="15" t="n"/>
+      <c r="AC34" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD34" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE34" s="17" t="n">
+        <v>614.625</v>
+      </c>
+      <c r="AF34" s="17" t="n">
+        <v>598.7848</v>
+      </c>
+      <c r="AG34" s="17" t="n">
+        <v>630.4652</v>
+      </c>
+      <c r="AH34" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI34" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ34" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK34" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL34" s="15" t="inlineStr">
+        <is>
+          <t>Visa Earnings Prediction Market Preview: What Will Ryan McInerney Say?</t>
+        </is>
+      </c>
+      <c r="AM34" s="17" t="n">
+        <v>614.625</v>
+      </c>
+      <c r="AN34" s="19" t="n">
+        <v>0.007800000000000001</v>
+      </c>
+      <c r="AO34" s="17" t="n">
+        <v>100369.37</v>
+      </c>
+      <c r="AP34" s="17" t="n">
+        <v>1047.47</v>
+      </c>
+      <c r="AQ34" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR34" s="16" t="n">
+        <v>1.704058088</v>
+      </c>
+      <c r="AS34" s="17" t="n">
+        <v>613.688</v>
+      </c>
+      <c r="AT34" s="19" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="AU34" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV34" s="6" t="inlineStr">
+        <is>
+          <t>2a80a5f5-7036-429a-a454-9494a1feec10</t>
+        </is>
+      </c>
+      <c r="AW34" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-MA-1793200550863</t>
+        </is>
+      </c>
+      <c r="AX34" s="13" t="n">
+        <v>46323.63599537037</v>
+      </c>
+      <c r="AY34" s="13" t="n">
+        <v>46323.63600694444</v>
+      </c>
+      <c r="AZ34" s="13" t="n">
+        <v>46323.63568287037</v>
+      </c>
+      <c r="BA34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="13" t="n">
+        <v>46323.67767361111</v>
+      </c>
+      <c r="C35" s="13" t="n">
+        <v>46323.46934027778</v>
+      </c>
+      <c r="D35" s="13" t="n">
+        <v>46323.63600694444</v>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>MARATHON PETROLEUM CORPORATION</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J35" s="16" t="n">
+        <v>0.19946772</v>
+      </c>
+      <c r="K35" s="17" t="n">
+        <v>437.364</v>
+      </c>
+      <c r="L35" s="17">
+        <f>IF(AND(ISNUMBER(J35),ISNUMBER(K35)),J35*K35,"")</f>
+        <v/>
+      </c>
+      <c r="M35" s="17" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="N35" s="16" t="n"/>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P35" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $1,047.47 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q35" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R35" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S35" s="18" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="T35" s="12" t="n">
+        <v>86</v>
+      </c>
+      <c r="U35" s="19" t="n">
+        <v>0.0246</v>
+      </c>
+      <c r="V35" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W35" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X35" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y35" s="19" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="Z35" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA35" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB35" s="15" t="inlineStr">
+        <is>
+          <t>One day (-7.4%) did 74% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC35" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD35" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE35" s="17" t="n">
+        <v>446.2446</v>
+      </c>
+      <c r="AF35" s="17" t="n">
+        <v>422.0831</v>
+      </c>
+      <c r="AG35" s="17" t="n">
+        <v>470.4061</v>
+      </c>
+      <c r="AH35" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI35" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ35" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK35" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL35" s="15" t="inlineStr">
+        <is>
+          <t>Refiner Stocks Suffer Worst Day Since the Tariff Shock: The Threat Is Not Cheaper Oil</t>
+        </is>
+      </c>
+      <c r="AM35" s="17" t="n">
+        <v>436.58</v>
+      </c>
+      <c r="AN35" s="19" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="AO35" s="17" t="n">
+        <v>100369.37</v>
+      </c>
+      <c r="AP35" s="17" t="n">
+        <v>1047.47</v>
+      </c>
+      <c r="AQ35" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR35" s="16" t="n"/>
+      <c r="AS35" s="17" t="n"/>
+      <c r="AT35" s="19" t="n"/>
+      <c r="AU35" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV35" s="6" t="inlineStr">
+        <is>
+          <t>795c1192-92f0-4087-a19e-e4a4afbb099c</t>
+        </is>
+      </c>
+      <c r="AW35" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MPC-1793200551740</t>
+        </is>
+      </c>
+      <c r="AX35" s="13" t="n">
+        <v>46323.63600694444</v>
+      </c>
+      <c r="AY35" s="13" t="n">
+        <v>46323.63600694444</v>
+      </c>
+      <c r="AZ35" s="13" t="n">
+        <v>46323.63568287037</v>
+      </c>
+      <c r="BA35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="13" t="n">
+        <v>46323.67768518518</v>
+      </c>
+      <c r="C36" s="13" t="n">
+        <v>46323.46935185185</v>
+      </c>
+      <c r="D36" s="13" t="n">
+        <v>46323.63601851852</v>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr">
+        <is>
+          <t>EQT CORP</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J36" s="16" t="n">
+        <v>1.562264961</v>
+      </c>
+      <c r="K36" s="17" t="n">
+        <v>55.842</v>
+      </c>
+      <c r="L36" s="17">
+        <f>IF(AND(ISNUMBER(J36),ISNUMBER(K36)),J36*K36,"")</f>
+        <v/>
+      </c>
+      <c r="M36" s="17" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="N36" s="16" t="n"/>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P36" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #6, 8.33% of the $1,047.47 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q36" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R36" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S36" s="18" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="T36" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U36" s="19" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="V36" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W36" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="X36" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y36" s="19" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="Z36" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA36" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="AB36" s="15" t="inlineStr">
+        <is>
+          <t>Price gapped 5.1% at an open in the last week.</t>
+        </is>
+      </c>
+      <c r="AC36" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD36" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE36" s="17" t="n">
+        <v>56.5868</v>
+      </c>
+      <c r="AF36" s="17" t="n">
+        <v>54.5198</v>
+      </c>
+      <c r="AG36" s="17" t="n">
+        <v>58.6539</v>
+      </c>
+      <c r="AH36" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI36" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ36" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK36" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL36" s="15" t="inlineStr">
+        <is>
+          <t>UBS Maintains Buy on EQT, Lowers Price Target to $75</t>
+        </is>
+      </c>
+      <c r="AM36" s="17" t="n">
+        <v>55.78</v>
+      </c>
+      <c r="AN36" s="19" t="n">
+        <v>-0.009399999999999999</v>
+      </c>
+      <c r="AO36" s="17" t="n">
+        <v>100369.37</v>
+      </c>
+      <c r="AP36" s="17" t="n">
+        <v>1047.47</v>
+      </c>
+      <c r="AQ36" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR36" s="16" t="n"/>
+      <c r="AS36" s="17" t="n"/>
+      <c r="AT36" s="19" t="n"/>
+      <c r="AU36" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV36" s="6" t="inlineStr">
+        <is>
+          <t>8dda163c-11b6-4647-b796-a4421efe2a2c</t>
+        </is>
+      </c>
+      <c r="AW36" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EQT-1793200552082</t>
+        </is>
+      </c>
+      <c r="AX36" s="13" t="n">
+        <v>46323.63601851852</v>
+      </c>
+      <c r="AY36" s="13" t="n">
+        <v>46323.63601851852</v>
+      </c>
+      <c r="AZ36" s="13" t="n">
+        <v>46323.63568287037</v>
+      </c>
+      <c r="BA36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="13" t="n">
+        <v>46323.67768518518</v>
+      </c>
+      <c r="C37" s="13" t="n">
+        <v>46323.46935185185</v>
+      </c>
+      <c r="D37" s="13" t="n">
+        <v>46323.63601851852</v>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>PSX</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr">
+        <is>
+          <t>PHILLIPS 66</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J37" s="16" t="n">
+        <v>0.323158986</v>
+      </c>
+      <c r="K37" s="17" t="n">
+        <v>269.96</v>
+      </c>
+      <c r="L37" s="17">
+        <f>IF(AND(ISNUMBER(J37),ISNUMBER(K37)),J37*K37,"")</f>
+        <v/>
+      </c>
+      <c r="M37" s="17" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="N37" s="16" t="n"/>
+      <c r="O37" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P37" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #7, 8.33% of the $1,047.47 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q37" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R37" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S37" s="18" t="n">
+        <v>0.569</v>
+      </c>
+      <c r="T37" s="12" t="n">
+        <v>72</v>
+      </c>
+      <c r="U37" s="19" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="V37" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W37" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="X37" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y37" s="19" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="Z37" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA37" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB37" s="15" t="inlineStr">
+        <is>
+          <t>One day (-7.0%) did 75% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC37" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD37" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE37" s="17" t="n">
+        <v>274.4826</v>
+      </c>
+      <c r="AF37" s="17" t="n">
+        <v>261.9386</v>
+      </c>
+      <c r="AG37" s="17" t="n">
+        <v>287.0267</v>
+      </c>
+      <c r="AH37" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI37" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ37" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK37" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL37" s="15" t="inlineStr">
+        <is>
+          <t>Refiner Stocks Suffer Worst Day Since the Tariff Shock: The Threat Is Not Cheaper Oil</t>
+        </is>
+      </c>
+      <c r="AM37" s="17" t="n">
+        <v>269.89</v>
+      </c>
+      <c r="AN37" s="19" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AO37" s="17" t="n">
+        <v>100369.37</v>
+      </c>
+      <c r="AP37" s="17" t="n">
+        <v>1047.47</v>
+      </c>
+      <c r="AQ37" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR37" s="16" t="n"/>
+      <c r="AS37" s="17" t="n"/>
+      <c r="AT37" s="19" t="n"/>
+      <c r="AU37" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV37" s="6" t="inlineStr">
+        <is>
+          <t>13fe6aef-0823-407e-9dae-d781ac0376cd</t>
+        </is>
+      </c>
+      <c r="AW37" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-PSX-1793200552421</t>
+        </is>
+      </c>
+      <c r="AX37" s="13" t="n">
+        <v>46323.63601851852</v>
+      </c>
+      <c r="AY37" s="13" t="n">
+        <v>46323.63601851852</v>
+      </c>
+      <c r="AZ37" s="13" t="n">
+        <v>46323.63568287037</v>
+      </c>
+      <c r="BA37" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -7067,7 +7819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8513,15 +9265,21 @@
         <v>613.688</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>1.704058088</v>
+        <v>0.852029044</v>
       </c>
       <c r="G26" s="17">
         <f>E26*F26</f>
         <v/>
       </c>
-      <c r="H26" s="22" t="n"/>
-      <c r="I26" s="22" t="n"/>
-      <c r="J26" s="17" t="n"/>
+      <c r="H26" s="22" t="n">
+        <v>46323.67767361111</v>
+      </c>
+      <c r="I26" s="22" t="n">
+        <v>46323.46934027778</v>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>614.554</v>
+      </c>
       <c r="K26" s="17">
         <f>IF(ISNUMBER(J26),J26*F26,"")</f>
         <v/>
@@ -8538,22 +9296,26 @@
         <f>IF(ISNUMBER(H26),H26-C26,"")</f>
         <v/>
       </c>
-      <c r="O26" s="6" t="n"/>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P26" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Automatic Data Processing, Inc. Common Stock</t>
+          <t>Mastercard Incorporated</t>
         </is>
       </c>
       <c r="C27" s="22" t="n">
@@ -8563,24 +9325,18 @@
         <v>46323.46354166666</v>
       </c>
       <c r="E27" s="17" t="n">
-        <v>284.46</v>
+        <v>613.688</v>
       </c>
       <c r="F27" s="16" t="n">
-        <v>3.676298952</v>
+        <v>0.852029044</v>
       </c>
       <c r="G27" s="17">
         <f>E27*F27</f>
         <v/>
       </c>
-      <c r="H27" s="22" t="n">
-        <v>46323.67340277778</v>
-      </c>
-      <c r="I27" s="22" t="n">
-        <v>46323.46506944444</v>
-      </c>
-      <c r="J27" s="17" t="n">
-        <v>283.51</v>
-      </c>
+      <c r="H27" s="22" t="n"/>
+      <c r="I27" s="22" t="n"/>
+      <c r="J27" s="17" t="n"/>
       <c r="K27" s="17">
         <f>IF(ISNUMBER(J27),J27*F27,"")</f>
         <v/>
@@ -8597,26 +9353,22 @@
         <f>IF(ISNUMBER(H27),H27-C27,"")</f>
         <v/>
       </c>
-      <c r="O27" s="6" t="inlineStr">
-        <is>
-          <t>bad day</t>
-        </is>
-      </c>
+      <c r="O27" s="6" t="n"/>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>CNC</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Centene Corporation</t>
+          <t>Automatic Data Processing, Inc. Common Stock</t>
         </is>
       </c>
       <c r="C28" s="22" t="n">
@@ -8626,18 +9378,24 @@
         <v>46323.46354166666</v>
       </c>
       <c r="E28" s="17" t="n">
-        <v>68.89</v>
+        <v>284.46</v>
       </c>
       <c r="F28" s="16" t="n">
-        <v>15.180142255</v>
+        <v>3.676298952</v>
       </c>
       <c r="G28" s="17">
         <f>E28*F28</f>
         <v/>
       </c>
-      <c r="H28" s="22" t="n"/>
-      <c r="I28" s="22" t="n"/>
-      <c r="J28" s="17" t="n"/>
+      <c r="H28" s="22" t="n">
+        <v>46323.67340277778</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <v>46323.46506944444</v>
+      </c>
+      <c r="J28" s="17" t="n">
+        <v>283.51</v>
+      </c>
       <c r="K28" s="17">
         <f>IF(ISNUMBER(J28),J28*F28,"")</f>
         <v/>
@@ -8654,35 +9412,39 @@
         <f>IF(ISNUMBER(H28),H28-C28,"")</f>
         <v/>
       </c>
-      <c r="O28" s="6" t="n"/>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>CNC</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Cognizant Technology Solutions Corporation Class A Common Stock</t>
+          <t>Centene Corporation</t>
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>46323.67188657408</v>
+        <v>46323.671875</v>
       </c>
       <c r="D29" s="22" t="n">
-        <v>46323.46355324074</v>
+        <v>46323.46354166666</v>
       </c>
       <c r="E29" s="17" t="n">
-        <v>66.55</v>
+        <v>68.89</v>
       </c>
       <c r="F29" s="16" t="n">
-        <v>15.713899323</v>
+        <v>15.180142255</v>
       </c>
       <c r="G29" s="17">
         <f>E29*F29</f>
@@ -8717,12 +9479,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>EQNR</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+          <t>Cognizant Technology Solutions Corporation Class A Common Stock</t>
         </is>
       </c>
       <c r="C30" s="22" t="n">
@@ -8732,10 +9494,10 @@
         <v>46323.46355324074</v>
       </c>
       <c r="E30" s="17" t="n">
-        <v>47.68</v>
+        <v>66.55</v>
       </c>
       <c r="F30" s="16" t="n">
-        <v>21.932885906</v>
+        <v>15.713899323</v>
       </c>
       <c r="G30" s="17">
         <f>E30*F30</f>
@@ -8767,8 +9529,220 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="n">
+        <v>46323.67188657408</v>
+      </c>
+      <c r="D31" s="22" t="n">
+        <v>46323.46355324074</v>
+      </c>
+      <c r="E31" s="17" t="n">
+        <v>47.68</v>
+      </c>
+      <c r="F31" s="16" t="n">
+        <v>21.932885906</v>
+      </c>
+      <c r="G31" s="17">
+        <f>E31*F31</f>
+        <v/>
+      </c>
+      <c r="H31" s="22" t="n"/>
+      <c r="I31" s="22" t="n"/>
+      <c r="J31" s="17" t="n"/>
+      <c r="K31" s="17">
+        <f>IF(ISNUMBER(J31),J31*F31,"")</f>
+        <v/>
+      </c>
+      <c r="L31" s="23">
+        <f>IF(ISNUMBER(J31),K31-G31,"")</f>
+        <v/>
+      </c>
+      <c r="M31" s="24">
+        <f>IF(ISNUMBER(J31),L31/G31,"")</f>
+        <v/>
+      </c>
+      <c r="N31" s="25">
+        <f>IF(ISNUMBER(H31),H31-C31,"")</f>
+        <v/>
+      </c>
+      <c r="O31" s="6" t="n"/>
+      <c r="P31" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>MARATHON PETROLEUM CORPORATION</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="n">
+        <v>46323.67767361111</v>
+      </c>
+      <c r="D32" s="22" t="n">
+        <v>46323.46934027778</v>
+      </c>
+      <c r="E32" s="17" t="n">
+        <v>437.364</v>
+      </c>
+      <c r="F32" s="16" t="n">
+        <v>0.19946772</v>
+      </c>
+      <c r="G32" s="17">
+        <f>E32*F32</f>
+        <v/>
+      </c>
+      <c r="H32" s="22" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="17" t="n"/>
+      <c r="K32" s="17">
+        <f>IF(ISNUMBER(J32),J32*F32,"")</f>
+        <v/>
+      </c>
+      <c r="L32" s="23">
+        <f>IF(ISNUMBER(J32),K32-G32,"")</f>
+        <v/>
+      </c>
+      <c r="M32" s="24">
+        <f>IF(ISNUMBER(J32),L32/G32,"")</f>
+        <v/>
+      </c>
+      <c r="N32" s="25">
+        <f>IF(ISNUMBER(H32),H32-C32,"")</f>
+        <v/>
+      </c>
+      <c r="O32" s="6" t="n"/>
+      <c r="P32" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>EQT CORP</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="n">
+        <v>46323.67768518518</v>
+      </c>
+      <c r="D33" s="22" t="n">
+        <v>46323.46935185185</v>
+      </c>
+      <c r="E33" s="17" t="n">
+        <v>55.842</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <v>1.562264961</v>
+      </c>
+      <c r="G33" s="17">
+        <f>E33*F33</f>
+        <v/>
+      </c>
+      <c r="H33" s="22" t="n"/>
+      <c r="I33" s="22" t="n"/>
+      <c r="J33" s="17" t="n"/>
+      <c r="K33" s="17">
+        <f>IF(ISNUMBER(J33),J33*F33,"")</f>
+        <v/>
+      </c>
+      <c r="L33" s="23">
+        <f>IF(ISNUMBER(J33),K33-G33,"")</f>
+        <v/>
+      </c>
+      <c r="M33" s="24">
+        <f>IF(ISNUMBER(J33),L33/G33,"")</f>
+        <v/>
+      </c>
+      <c r="N33" s="25">
+        <f>IF(ISNUMBER(H33),H33-C33,"")</f>
+        <v/>
+      </c>
+      <c r="O33" s="6" t="n"/>
+      <c r="P33" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>PSX</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>PHILLIPS 66</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="n">
+        <v>46323.67768518518</v>
+      </c>
+      <c r="D34" s="22" t="n">
+        <v>46323.46935185185</v>
+      </c>
+      <c r="E34" s="17" t="n">
+        <v>269.96</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>0.323158986</v>
+      </c>
+      <c r="G34" s="17">
+        <f>E34*F34</f>
+        <v/>
+      </c>
+      <c r="H34" s="22" t="n"/>
+      <c r="I34" s="22" t="n"/>
+      <c r="J34" s="17" t="n"/>
+      <c r="K34" s="17">
+        <f>IF(ISNUMBER(J34),J34*F34,"")</f>
+        <v/>
+      </c>
+      <c r="L34" s="23">
+        <f>IF(ISNUMBER(J34),K34-G34,"")</f>
+        <v/>
+      </c>
+      <c r="M34" s="24">
+        <f>IF(ISNUMBER(J34),L34/G34,"")</f>
+        <v/>
+      </c>
+      <c r="N34" s="25">
+        <f>IF(ISNUMBER(H34),H34-C34,"")</f>
+        <v/>
+      </c>
+      <c r="O34" s="6" t="n"/>
+      <c r="P34" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M30">
+  <conditionalFormatting sqref="L2:M34">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 15:32 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA37" headerRowCount="1">
-  <autoFilter ref="A1:BA37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA39" headerRowCount="1">
+  <autoFilter ref="A1:BA39"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P34" headerRowCount="1">
-  <autoFilter ref="A1:P34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P36" headerRowCount="1">
+  <autoFilter ref="A1:P36"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.67783564814</v>
+        <v>46323.68950231482</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.46950231482</v>
+        <v>46323.48116898148</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$37,"BUY")+COUNTIF(Orders!$E$2:$E$37,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$39,"BUY")+COUNTIF(Orders!$E$2:$E$39,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$37,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$39,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$37,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$39,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$37,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$39,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$37,Orders!$E$2:$E$37,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$39,Orders!$E$2:$E$39,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$37,Orders!$E$2:$E$37,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$39,Orders!$E$2:$E$39,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$34,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$36,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$34,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$36,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$34)</f>
+        <f>SUM('Round trips'!$L$2:$L$36)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$34,"Closed",'Round trips'!$L$2:$L$34,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$36,"Closed",'Round trips'!$L$2:$L$36,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA37"/>
+  <dimension ref="A1:BA39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7804,6 +7804,382 @@
       </c>
       <c r="BA37" s="6" t="n"/>
     </row>
+    <row r="38">
+      <c r="A38" s="12" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="13" t="n">
+        <v>46323.689375</v>
+      </c>
+      <c r="C38" s="13" t="n">
+        <v>46323.48104166667</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>46323.64770833333</v>
+      </c>
+      <c r="E38" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>CNC</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="inlineStr">
+        <is>
+          <t>CNC</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J38" s="16" t="n">
+        <v>7.590071127</v>
+      </c>
+      <c r="K38" s="17" t="n">
+        <v>69.01000000000001</v>
+      </c>
+      <c r="L38" s="17">
+        <f>IF(AND(ISNUMBER(J38),ISNUMBER(K38)),J38*K38,"")</f>
+        <v/>
+      </c>
+      <c r="M38" s="17" t="n"/>
+      <c r="N38" s="16" t="n">
+        <v>7.590071127</v>
+      </c>
+      <c r="O38" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P38" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q38" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R38" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S38" s="18" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="T38" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="U38" s="19" t="n">
+        <v>0.0126</v>
+      </c>
+      <c r="V38" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W38" s="12" t="n"/>
+      <c r="X38" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y38" s="19" t="n">
+        <v>0.009599999999999999</v>
+      </c>
+      <c r="Z38" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA38" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB38" s="15" t="n"/>
+      <c r="AC38" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD38" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE38" s="17" t="n">
+        <v>70.3807</v>
+      </c>
+      <c r="AF38" s="17" t="n">
+        <v>67.15389999999999</v>
+      </c>
+      <c r="AG38" s="17" t="n">
+        <v>73.60760000000001</v>
+      </c>
+      <c r="AH38" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI38" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ38" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK38" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL38" s="15" t="inlineStr">
+        <is>
+          <t>Cantor Fitzgerald Upgrades Centene to Overweight and Raises Price Target to $79</t>
+        </is>
+      </c>
+      <c r="AM38" s="17" t="n">
+        <v>69.09</v>
+      </c>
+      <c r="AN38" s="19" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="AO38" s="17" t="n">
+        <v>100387.39</v>
+      </c>
+      <c r="AP38" s="17" t="n">
+        <v>1309.37</v>
+      </c>
+      <c r="AQ38" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR38" s="16" t="n">
+        <v>15.180142255</v>
+      </c>
+      <c r="AS38" s="17" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="AT38" s="19" t="n">
+        <v>0.0021</v>
+      </c>
+      <c r="AU38" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV38" s="6" t="inlineStr">
+        <is>
+          <t>3b93b9ef-5e93-4cd1-a10b-1cea19899888</t>
+        </is>
+      </c>
+      <c r="AW38" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-CNC-1793201560611</t>
+        </is>
+      </c>
+      <c r="AX38" s="13" t="n">
+        <v>46323.64768518518</v>
+      </c>
+      <c r="AY38" s="13" t="n">
+        <v>46323.64770833333</v>
+      </c>
+      <c r="AZ38" s="13" t="n">
+        <v>46323.64743055555</v>
+      </c>
+      <c r="BA38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="13" t="n">
+        <v>46323.68936342592</v>
+      </c>
+      <c r="C39" s="13" t="n">
+        <v>46323.48103009259</v>
+      </c>
+      <c r="D39" s="13" t="n">
+        <v>46323.64769675926</v>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>DINO</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>HF Sinclair Corporation</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J39" s="16" t="n">
+        <v>0.973941309</v>
+      </c>
+      <c r="K39" s="17" t="n">
+        <v>111.978</v>
+      </c>
+      <c r="L39" s="17">
+        <f>IF(AND(ISNUMBER(J39),ISNUMBER(K39)),J39*K39,"")</f>
+        <v/>
+      </c>
+      <c r="M39" s="17" t="n">
+        <v>109.07</v>
+      </c>
+      <c r="N39" s="16" t="n"/>
+      <c r="O39" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P39" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $1,309.37 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q39" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R39" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S39" s="18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="T39" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="U39" s="19" t="n">
+        <v>0.0194</v>
+      </c>
+      <c r="V39" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W39" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X39" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y39" s="19" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="Z39" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA39" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB39" s="15" t="inlineStr">
+        <is>
+          <t>One day (-8.9%) did 73% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC39" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD39" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE39" s="17" t="n">
+        <v>114.8338</v>
+      </c>
+      <c r="AF39" s="17" t="n">
+        <v>108.2243</v>
+      </c>
+      <c r="AG39" s="17" t="n">
+        <v>121.4432</v>
+      </c>
+      <c r="AH39" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI39" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ39" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK39" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL39" s="15" t="inlineStr">
+        <is>
+          <t>HF Sinclair Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM39" s="17" t="n">
+        <v>112.31</v>
+      </c>
+      <c r="AN39" s="19" t="n">
+        <v>-0.0169</v>
+      </c>
+      <c r="AO39" s="17" t="n">
+        <v>100387.39</v>
+      </c>
+      <c r="AP39" s="17" t="n">
+        <v>1309.37</v>
+      </c>
+      <c r="AQ39" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR39" s="16" t="n"/>
+      <c r="AS39" s="17" t="n"/>
+      <c r="AT39" s="19" t="n"/>
+      <c r="AU39" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV39" s="6" t="inlineStr">
+        <is>
+          <t>f522894d-4a29-4dac-9deb-1e6b36780c89</t>
+        </is>
+      </c>
+      <c r="AW39" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-DINO-1793201561401</t>
+        </is>
+      </c>
+      <c r="AX39" s="13" t="n">
+        <v>46323.64769675926</v>
+      </c>
+      <c r="AY39" s="13" t="n">
+        <v>46323.64769675926</v>
+      </c>
+      <c r="AZ39" s="13" t="n">
+        <v>46323.64743055555</v>
+      </c>
+      <c r="BA39" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -7819,7 +8195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9444,15 +9820,21 @@
         <v>68.89</v>
       </c>
       <c r="F29" s="16" t="n">
-        <v>15.180142255</v>
+        <v>7.590071127</v>
       </c>
       <c r="G29" s="17">
         <f>E29*F29</f>
         <v/>
       </c>
-      <c r="H29" s="22" t="n"/>
-      <c r="I29" s="22" t="n"/>
-      <c r="J29" s="17" t="n"/>
+      <c r="H29" s="22" t="n">
+        <v>46323.689375</v>
+      </c>
+      <c r="I29" s="22" t="n">
+        <v>46323.48104166667</v>
+      </c>
+      <c r="J29" s="17" t="n">
+        <v>69.01000000000001</v>
+      </c>
       <c r="K29" s="17">
         <f>IF(ISNUMBER(J29),J29*F29,"")</f>
         <v/>
@@ -9469,35 +9851,39 @@
         <f>IF(ISNUMBER(H29),H29-C29,"")</f>
         <v/>
       </c>
-      <c r="O29" s="6" t="n"/>
+      <c r="O29" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>CNC</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Cognizant Technology Solutions Corporation Class A Common Stock</t>
+          <t>Centene Corporation</t>
         </is>
       </c>
       <c r="C30" s="22" t="n">
-        <v>46323.67188657408</v>
+        <v>46323.671875</v>
       </c>
       <c r="D30" s="22" t="n">
-        <v>46323.46355324074</v>
+        <v>46323.46354166666</v>
       </c>
       <c r="E30" s="17" t="n">
-        <v>66.55</v>
+        <v>68.89</v>
       </c>
       <c r="F30" s="16" t="n">
-        <v>15.713899323</v>
+        <v>7.590071128</v>
       </c>
       <c r="G30" s="17">
         <f>E30*F30</f>
@@ -9532,12 +9918,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>EQNR</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+          <t>Cognizant Technology Solutions Corporation Class A Common Stock</t>
         </is>
       </c>
       <c r="C31" s="22" t="n">
@@ -9547,10 +9933,10 @@
         <v>46323.46355324074</v>
       </c>
       <c r="E31" s="17" t="n">
-        <v>47.68</v>
+        <v>66.55</v>
       </c>
       <c r="F31" s="16" t="n">
-        <v>21.932885906</v>
+        <v>15.713899323</v>
       </c>
       <c r="G31" s="17">
         <f>E31*F31</f>
@@ -9585,25 +9971,25 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>EQNR</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>MARATHON PETROLEUM CORPORATION</t>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>46323.67767361111</v>
+        <v>46323.67188657408</v>
       </c>
       <c r="D32" s="22" t="n">
-        <v>46323.46934027778</v>
+        <v>46323.46355324074</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>437.364</v>
+        <v>47.68</v>
       </c>
       <c r="F32" s="16" t="n">
-        <v>0.19946772</v>
+        <v>21.932885906</v>
       </c>
       <c r="G32" s="17">
         <f>E32*F32</f>
@@ -9638,25 +10024,25 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>MPC</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>EQT CORP</t>
+          <t>MARATHON PETROLEUM CORPORATION</t>
         </is>
       </c>
       <c r="C33" s="22" t="n">
-        <v>46323.67768518518</v>
+        <v>46323.67767361111</v>
       </c>
       <c r="D33" s="22" t="n">
-        <v>46323.46935185185</v>
+        <v>46323.46934027778</v>
       </c>
       <c r="E33" s="17" t="n">
-        <v>55.842</v>
+        <v>437.364</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>1.562264961</v>
+        <v>0.19946772</v>
       </c>
       <c r="G33" s="17">
         <f>E33*F33</f>
@@ -9691,12 +10077,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>PHILLIPS 66</t>
+          <t>EQT CORP</t>
         </is>
       </c>
       <c r="C34" s="22" t="n">
@@ -9706,10 +10092,10 @@
         <v>46323.46935185185</v>
       </c>
       <c r="E34" s="17" t="n">
-        <v>269.96</v>
+        <v>55.842</v>
       </c>
       <c r="F34" s="16" t="n">
-        <v>0.323158986</v>
+        <v>1.562264961</v>
       </c>
       <c r="G34" s="17">
         <f>E34*F34</f>
@@ -9741,8 +10127,114 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>PSX</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>PHILLIPS 66</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="n">
+        <v>46323.67768518518</v>
+      </c>
+      <c r="D35" s="22" t="n">
+        <v>46323.46935185185</v>
+      </c>
+      <c r="E35" s="17" t="n">
+        <v>269.96</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>0.323158986</v>
+      </c>
+      <c r="G35" s="17">
+        <f>E35*F35</f>
+        <v/>
+      </c>
+      <c r="H35" s="22" t="n"/>
+      <c r="I35" s="22" t="n"/>
+      <c r="J35" s="17" t="n"/>
+      <c r="K35" s="17">
+        <f>IF(ISNUMBER(J35),J35*F35,"")</f>
+        <v/>
+      </c>
+      <c r="L35" s="23">
+        <f>IF(ISNUMBER(J35),K35-G35,"")</f>
+        <v/>
+      </c>
+      <c r="M35" s="24">
+        <f>IF(ISNUMBER(J35),L35/G35,"")</f>
+        <v/>
+      </c>
+      <c r="N35" s="25">
+        <f>IF(ISNUMBER(H35),H35-C35,"")</f>
+        <v/>
+      </c>
+      <c r="O35" s="6" t="n"/>
+      <c r="P35" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>DINO</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>HF Sinclair Corporation</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="n">
+        <v>46323.68936342592</v>
+      </c>
+      <c r="D36" s="22" t="n">
+        <v>46323.48103009259</v>
+      </c>
+      <c r="E36" s="17" t="n">
+        <v>111.978</v>
+      </c>
+      <c r="F36" s="16" t="n">
+        <v>0.973941309</v>
+      </c>
+      <c r="G36" s="17">
+        <f>E36*F36</f>
+        <v/>
+      </c>
+      <c r="H36" s="22" t="n"/>
+      <c r="I36" s="22" t="n"/>
+      <c r="J36" s="17" t="n"/>
+      <c r="K36" s="17">
+        <f>IF(ISNUMBER(J36),J36*F36,"")</f>
+        <v/>
+      </c>
+      <c r="L36" s="23">
+        <f>IF(ISNUMBER(J36),K36-G36,"")</f>
+        <v/>
+      </c>
+      <c r="M36" s="24">
+        <f>IF(ISNUMBER(J36),L36/G36,"")</f>
+        <v/>
+      </c>
+      <c r="N36" s="25">
+        <f>IF(ISNUMBER(H36),H36-C36,"")</f>
+        <v/>
+      </c>
+      <c r="O36" s="6" t="n"/>
+      <c r="P36" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M34">
+  <conditionalFormatting sqref="L2:M36">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 15:38 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA39" headerRowCount="1">
-  <autoFilter ref="A1:BA39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA40" headerRowCount="1">
+  <autoFilter ref="A1:BA40"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P36" headerRowCount="1">
-  <autoFilter ref="A1:P36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P37" headerRowCount="1">
+  <autoFilter ref="A1:P37"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.68950231482</v>
+        <v>46323.69357638889</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.48116898148</v>
+        <v>46323.48524305555</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$39,"BUY")+COUNTIF(Orders!$E$2:$E$39,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$40,"BUY")+COUNTIF(Orders!$E$2:$E$40,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$39,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$40,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$39,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$40,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$39,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$40,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$39,Orders!$E$2:$E$39,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$40,Orders!$E$2:$E$40,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$39,Orders!$E$2:$E$39,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$40,Orders!$E$2:$E$40,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$36,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$36,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$37,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$36)</f>
+        <f>SUM('Round trips'!$L$2:$L$37)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$36,"Closed",'Round trips'!$L$2:$L$36,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$37,"Closed",'Round trips'!$L$2:$L$37,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA39"/>
+  <dimension ref="A1:BA40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8180,6 +8180,198 @@
       </c>
       <c r="BA39" s="6" t="n"/>
     </row>
+    <row r="40">
+      <c r="A40" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="13" t="n">
+        <v>46323.69346064814</v>
+      </c>
+      <c r="C40" s="13" t="n">
+        <v>46323.48512731482</v>
+      </c>
+      <c r="D40" s="13" t="n">
+        <v>46323.65179398148</v>
+      </c>
+      <c r="E40" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>DINO</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>DINO</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J40" s="16" t="n">
+        <v>0.486970654</v>
+      </c>
+      <c r="K40" s="17" t="n">
+        <v>111.736</v>
+      </c>
+      <c r="L40" s="17">
+        <f>IF(AND(ISNUMBER(J40),ISNUMBER(K40)),J40*K40,"")</f>
+        <v/>
+      </c>
+      <c r="M40" s="17" t="n"/>
+      <c r="N40" s="16" t="n">
+        <v>0.486970654</v>
+      </c>
+      <c r="O40" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P40" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q40" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R40" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S40" s="18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="T40" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="U40" s="19" t="n">
+        <v>0.0194</v>
+      </c>
+      <c r="V40" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W40" s="12" t="n"/>
+      <c r="X40" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y40" s="19" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="Z40" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA40" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB40" s="15" t="inlineStr">
+        <is>
+          <t>One day (-8.9%) did 72% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC40" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD40" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE40" s="17" t="n">
+        <v>111.92</v>
+      </c>
+      <c r="AF40" s="17" t="n">
+        <v>105.318</v>
+      </c>
+      <c r="AG40" s="17" t="n">
+        <v>118.522</v>
+      </c>
+      <c r="AH40" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI40" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ40" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK40" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL40" s="15" t="inlineStr">
+        <is>
+          <t>HF Sinclair Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM40" s="17" t="n">
+        <v>111.92</v>
+      </c>
+      <c r="AN40" s="19" t="n">
+        <v>-0.0193</v>
+      </c>
+      <c r="AO40" s="17" t="n">
+        <v>100311.45</v>
+      </c>
+      <c r="AP40" s="17" t="n">
+        <v>1724.1</v>
+      </c>
+      <c r="AQ40" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR40" s="16" t="n">
+        <v>0.973941309</v>
+      </c>
+      <c r="AS40" s="17" t="n">
+        <v>111.978</v>
+      </c>
+      <c r="AT40" s="19" t="n">
+        <v>-0.0015</v>
+      </c>
+      <c r="AU40" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV40" s="6" t="inlineStr">
+        <is>
+          <t>b7e8fde4-772d-45c4-baa3-f36239fb4db9</t>
+        </is>
+      </c>
+      <c r="AW40" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-DINO-1793201915224</t>
+        </is>
+      </c>
+      <c r="AX40" s="13" t="n">
+        <v>46323.65179398148</v>
+      </c>
+      <c r="AY40" s="13" t="n">
+        <v>46323.65179398148</v>
+      </c>
+      <c r="AZ40" s="13" t="n">
+        <v>46323.65157407407</v>
+      </c>
+      <c r="BA40" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -8195,7 +8387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10201,15 +10393,21 @@
         <v>111.978</v>
       </c>
       <c r="F36" s="16" t="n">
-        <v>0.973941309</v>
+        <v>0.486970654</v>
       </c>
       <c r="G36" s="17">
         <f>E36*F36</f>
         <v/>
       </c>
-      <c r="H36" s="22" t="n"/>
-      <c r="I36" s="22" t="n"/>
-      <c r="J36" s="17" t="n"/>
+      <c r="H36" s="22" t="n">
+        <v>46323.69346064814</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>46323.48512731482</v>
+      </c>
+      <c r="J36" s="17" t="n">
+        <v>111.736</v>
+      </c>
       <c r="K36" s="17">
         <f>IF(ISNUMBER(J36),J36*F36,"")</f>
         <v/>
@@ -10226,15 +10424,72 @@
         <f>IF(ISNUMBER(H36),H36-C36,"")</f>
         <v/>
       </c>
-      <c r="O36" s="6" t="n"/>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P36" s="6" t="inlineStr">
         <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>DINO</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>HF Sinclair Corporation</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="n">
+        <v>46323.68936342592</v>
+      </c>
+      <c r="D37" s="22" t="n">
+        <v>46323.48103009259</v>
+      </c>
+      <c r="E37" s="17" t="n">
+        <v>111.978</v>
+      </c>
+      <c r="F37" s="16" t="n">
+        <v>0.486970655</v>
+      </c>
+      <c r="G37" s="17">
+        <f>E37*F37</f>
+        <v/>
+      </c>
+      <c r="H37" s="22" t="n"/>
+      <c r="I37" s="22" t="n"/>
+      <c r="J37" s="17" t="n"/>
+      <c r="K37" s="17">
+        <f>IF(ISNUMBER(J37),J37*F37,"")</f>
+        <v/>
+      </c>
+      <c r="L37" s="23">
+        <f>IF(ISNUMBER(J37),K37-G37,"")</f>
+        <v/>
+      </c>
+      <c r="M37" s="24">
+        <f>IF(ISNUMBER(J37),L37/G37,"")</f>
+        <v/>
+      </c>
+      <c r="N37" s="25">
+        <f>IF(ISNUMBER(H37),H37-C37,"")</f>
+        <v/>
+      </c>
+      <c r="O37" s="6" t="n"/>
+      <c r="P37" s="6" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M36">
+  <conditionalFormatting sqref="L2:M37">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 16:01 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA40" headerRowCount="1">
-  <autoFilter ref="A1:BA40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA41" headerRowCount="1">
+  <autoFilter ref="A1:BA41"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P37" headerRowCount="1">
-  <autoFilter ref="A1:P37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P38" headerRowCount="1">
+  <autoFilter ref="A1:P38"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.69357638889</v>
+        <v>46323.70961805555</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.48524305555</v>
+        <v>46323.50128472222</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$40,"BUY")+COUNTIF(Orders!$E$2:$E$40,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$41,"BUY")+COUNTIF(Orders!$E$2:$E$41,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$40,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$41,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$40,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$41,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$40,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$41,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$40,Orders!$E$2:$E$40,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$41,Orders!$E$2:$E$41,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$40,Orders!$E$2:$E$40,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$41,Orders!$E$2:$E$41,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$38,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$37,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$38,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$37)</f>
+        <f>SUM('Round trips'!$L$2:$L$38)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$37,"Closed",'Round trips'!$L$2:$L$37,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$38,"Closed",'Round trips'!$L$2:$L$38,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA40"/>
+  <dimension ref="A1:BA41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8372,6 +8372,190 @@
       </c>
       <c r="BA40" s="6" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="13" t="n">
+        <v>46323.70951388889</v>
+      </c>
+      <c r="C41" s="13" t="n">
+        <v>46323.50118055556</v>
+      </c>
+      <c r="D41" s="13" t="n">
+        <v>46323.66784722222</v>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>Eli Lilly &amp; Co.</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J41" s="16" t="n">
+        <v>0.114688452</v>
+      </c>
+      <c r="K41" s="17" t="n">
+        <v>1291.586</v>
+      </c>
+      <c r="L41" s="17">
+        <f>IF(AND(ISNUMBER(J41),ISNUMBER(K41)),J41*K41,"")</f>
+        <v/>
+      </c>
+      <c r="M41" s="17" t="n">
+        <v>148.14</v>
+      </c>
+      <c r="N41" s="16" t="n"/>
+      <c r="O41" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P41" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $1,778.51 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q41" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R41" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S41" s="18" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="T41" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="U41" s="19" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="V41" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W41" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X41" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y41" s="19" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Z41" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA41" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB41" s="15" t="n"/>
+      <c r="AC41" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD41" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE41" s="17" t="n">
+        <v>1312.6967</v>
+      </c>
+      <c r="AF41" s="17" t="n">
+        <v>1259.8799</v>
+      </c>
+      <c r="AG41" s="17" t="n">
+        <v>1365.5136</v>
+      </c>
+      <c r="AH41" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI41" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ41" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK41" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL41" s="15" t="inlineStr">
+        <is>
+          <t>Top Wall Street Forecasters Revamp Eli Lilly Expectations Ahead Of Q3 Earnings</t>
+        </is>
+      </c>
+      <c r="AM41" s="17" t="n">
+        <v>1291.56</v>
+      </c>
+      <c r="AN41" s="19" t="n">
+        <v>0.007800000000000001</v>
+      </c>
+      <c r="AO41" s="17" t="n">
+        <v>100276.25</v>
+      </c>
+      <c r="AP41" s="17" t="n">
+        <v>1778.51</v>
+      </c>
+      <c r="AQ41" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR41" s="16" t="n"/>
+      <c r="AS41" s="17" t="n"/>
+      <c r="AT41" s="19" t="n"/>
+      <c r="AU41" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV41" s="6" t="inlineStr">
+        <is>
+          <t>a897d815-b832-49ce-9b72-e2ae4abe5680</t>
+        </is>
+      </c>
+      <c r="AW41" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-LLY-1793203302691</t>
+        </is>
+      </c>
+      <c r="AX41" s="13" t="n">
+        <v>46323.66784722222</v>
+      </c>
+      <c r="AY41" s="13" t="n">
+        <v>46323.66784722222</v>
+      </c>
+      <c r="AZ41" s="13" t="n">
+        <v>46323.6675462963</v>
+      </c>
+      <c r="BA41" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -8387,7 +8571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10488,8 +10672,61 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Eli Lilly &amp; Co.</t>
+        </is>
+      </c>
+      <c r="C38" s="22" t="n">
+        <v>46323.70951388889</v>
+      </c>
+      <c r="D38" s="22" t="n">
+        <v>46323.50118055556</v>
+      </c>
+      <c r="E38" s="17" t="n">
+        <v>1291.586</v>
+      </c>
+      <c r="F38" s="16" t="n">
+        <v>0.114688452</v>
+      </c>
+      <c r="G38" s="17">
+        <f>E38*F38</f>
+        <v/>
+      </c>
+      <c r="H38" s="22" t="n"/>
+      <c r="I38" s="22" t="n"/>
+      <c r="J38" s="17" t="n"/>
+      <c r="K38" s="17">
+        <f>IF(ISNUMBER(J38),J38*F38,"")</f>
+        <v/>
+      </c>
+      <c r="L38" s="23">
+        <f>IF(ISNUMBER(J38),K38-G38,"")</f>
+        <v/>
+      </c>
+      <c r="M38" s="24">
+        <f>IF(ISNUMBER(J38),L38/G38,"")</f>
+        <v/>
+      </c>
+      <c r="N38" s="25">
+        <f>IF(ISNUMBER(H38),H38-C38,"")</f>
+        <v/>
+      </c>
+      <c r="O38" s="6" t="n"/>
+      <c r="P38" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M37">
+  <conditionalFormatting sqref="L2:M38">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 16:21 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA41" headerRowCount="1">
-  <autoFilter ref="A1:BA41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA42" headerRowCount="1">
+  <autoFilter ref="A1:BA42"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P38" headerRowCount="1">
-  <autoFilter ref="A1:P38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P39" headerRowCount="1">
+  <autoFilter ref="A1:P39"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.70961805555</v>
+        <v>46323.72351851852</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.50128472222</v>
+        <v>46323.51518518518</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$41,"BUY")+COUNTIF(Orders!$E$2:$E$41,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$42,"BUY")+COUNTIF(Orders!$E$2:$E$42,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$41,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$42,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$41,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$42,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$41,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$42,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$41,Orders!$E$2:$E$41,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$42,Orders!$E$2:$E$42,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$41,Orders!$E$2:$E$41,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$42,Orders!$E$2:$E$42,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$38,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$39,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$38,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$39,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$38)</f>
+        <f>SUM('Round trips'!$L$2:$L$39)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$38,"Closed",'Round trips'!$L$2:$L$38,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$39,"Closed",'Round trips'!$L$2:$L$39,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA41"/>
+  <dimension ref="A1:BA42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8556,6 +8556,190 @@
       </c>
       <c r="BA41" s="6" t="n"/>
     </row>
+    <row r="42">
+      <c r="A42" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="13" t="n">
+        <v>46323.72341435185</v>
+      </c>
+      <c r="C42" s="13" t="n">
+        <v>46323.51508101852</v>
+      </c>
+      <c r="D42" s="13" t="n">
+        <v>46323.68174768519</v>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J42" s="16" t="n">
+        <v>0.167361335</v>
+      </c>
+      <c r="K42" s="17" t="n">
+        <v>811.418</v>
+      </c>
+      <c r="L42" s="17">
+        <f>IF(AND(ISNUMBER(J42),ISNUMBER(K42)),J42*K42,"")</f>
+        <v/>
+      </c>
+      <c r="M42" s="17" t="n">
+        <v>135.81</v>
+      </c>
+      <c r="N42" s="16" t="n"/>
+      <c r="O42" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P42" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $1,630.38 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q42" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R42" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S42" s="18" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="T42" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U42" s="19" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="V42" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W42" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X42" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA42" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB42" s="15" t="n"/>
+      <c r="AC42" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD42" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE42" s="17" t="n">
+        <v>823.0616</v>
+      </c>
+      <c r="AF42" s="17" t="n">
+        <v>791.8951</v>
+      </c>
+      <c r="AG42" s="17" t="n">
+        <v>854.228</v>
+      </c>
+      <c r="AH42" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI42" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ42" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK42" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL42" s="15" t="inlineStr">
+        <is>
+          <t>Evercore ISI Adjusts Price Target on Regeneron Pharmaceuticals to $850 From $900</t>
+        </is>
+      </c>
+      <c r="AM42" s="17" t="n">
+        <v>810.595</v>
+      </c>
+      <c r="AN42" s="19" t="n">
+        <v>-0.0066</v>
+      </c>
+      <c r="AO42" s="17" t="n">
+        <v>100130.89</v>
+      </c>
+      <c r="AP42" s="17" t="n">
+        <v>1630.38</v>
+      </c>
+      <c r="AQ42" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR42" s="16" t="n"/>
+      <c r="AS42" s="17" t="n"/>
+      <c r="AT42" s="19" t="n"/>
+      <c r="AU42" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV42" s="6" t="inlineStr">
+        <is>
+          <t>dda46246-83f4-40ff-853e-79415343124a</t>
+        </is>
+      </c>
+      <c r="AW42" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-REGN-1793204503400</t>
+        </is>
+      </c>
+      <c r="AX42" s="13" t="n">
+        <v>46323.68174768519</v>
+      </c>
+      <c r="AY42" s="13" t="n">
+        <v>46323.68174768519</v>
+      </c>
+      <c r="AZ42" s="13" t="n">
+        <v>46323.68159722222</v>
+      </c>
+      <c r="BA42" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -8571,7 +8755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10725,8 +10909,61 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="n">
+        <v>46323.72341435185</v>
+      </c>
+      <c r="D39" s="22" t="n">
+        <v>46323.51508101852</v>
+      </c>
+      <c r="E39" s="17" t="n">
+        <v>811.418</v>
+      </c>
+      <c r="F39" s="16" t="n">
+        <v>0.167361335</v>
+      </c>
+      <c r="G39" s="17">
+        <f>E39*F39</f>
+        <v/>
+      </c>
+      <c r="H39" s="22" t="n"/>
+      <c r="I39" s="22" t="n"/>
+      <c r="J39" s="17" t="n"/>
+      <c r="K39" s="17">
+        <f>IF(ISNUMBER(J39),J39*F39,"")</f>
+        <v/>
+      </c>
+      <c r="L39" s="23">
+        <f>IF(ISNUMBER(J39),K39-G39,"")</f>
+        <v/>
+      </c>
+      <c r="M39" s="24">
+        <f>IF(ISNUMBER(J39),L39/G39,"")</f>
+        <v/>
+      </c>
+      <c r="N39" s="25">
+        <f>IF(ISNUMBER(H39),H39-C39,"")</f>
+        <v/>
+      </c>
+      <c r="O39" s="6" t="n"/>
+      <c r="P39" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M38">
+  <conditionalFormatting sqref="L2:M39">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 16:57 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA42" headerRowCount="1">
-  <autoFilter ref="A1:BA42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA44" headerRowCount="1">
+  <autoFilter ref="A1:BA44"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P39" headerRowCount="1">
-  <autoFilter ref="A1:P39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P41" headerRowCount="1">
+  <autoFilter ref="A1:P41"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.72351851852</v>
+        <v>46323.74844907408</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.51518518518</v>
+        <v>46323.54011574074</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$42,"BUY")+COUNTIF(Orders!$E$2:$E$42,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$44,"BUY")+COUNTIF(Orders!$E$2:$E$44,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$42,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$44,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$42,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$44,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$42,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$44,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$42,Orders!$E$2:$E$42,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$44,Orders!$E$2:$E$44,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$42,Orders!$E$2:$E$42,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$44,Orders!$E$2:$E$44,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$39,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$41,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$39,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$41,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$39)</f>
+        <f>SUM('Round trips'!$L$2:$L$41)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$39,"Closed",'Round trips'!$L$2:$L$39,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$41,"Closed",'Round trips'!$L$2:$L$41,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA42"/>
+  <dimension ref="A1:BA44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8740,6 +8740,382 @@
       </c>
       <c r="BA42" s="6" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="13" t="n">
+        <v>46323.74836805555</v>
+      </c>
+      <c r="C43" s="13" t="n">
+        <v>46323.54003472222</v>
+      </c>
+      <c r="D43" s="13" t="n">
+        <v>46323.70670138889</v>
+      </c>
+      <c r="E43" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J43" s="16" t="n">
+        <v>0.083680667</v>
+      </c>
+      <c r="K43" s="17" t="n">
+        <v>812.398</v>
+      </c>
+      <c r="L43" s="17">
+        <f>IF(AND(ISNUMBER(J43),ISNUMBER(K43)),J43*K43,"")</f>
+        <v/>
+      </c>
+      <c r="M43" s="17" t="n"/>
+      <c r="N43" s="16" t="n">
+        <v>0.083680667</v>
+      </c>
+      <c r="O43" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P43" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q43" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R43" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S43" s="18" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="T43" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U43" s="19" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="V43" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W43" s="12" t="n"/>
+      <c r="X43" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y43" s="19" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="Z43" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA43" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB43" s="15" t="n"/>
+      <c r="AC43" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD43" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE43" s="17" t="n">
+        <v>812.63</v>
+      </c>
+      <c r="AF43" s="17" t="n">
+        <v>781.4143</v>
+      </c>
+      <c r="AG43" s="17" t="n">
+        <v>843.8457</v>
+      </c>
+      <c r="AH43" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI43" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ43" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK43" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL43" s="15" t="inlineStr">
+        <is>
+          <t>Evercore ISI Adjusts Price Target on Regeneron Pharmaceuticals to $850 From $900</t>
+        </is>
+      </c>
+      <c r="AM43" s="17" t="n">
+        <v>812.63</v>
+      </c>
+      <c r="AN43" s="19" t="n">
+        <v>-0.004099999999999999</v>
+      </c>
+      <c r="AO43" s="17" t="n">
+        <v>100128.62</v>
+      </c>
+      <c r="AP43" s="17" t="n">
+        <v>1494.58</v>
+      </c>
+      <c r="AQ43" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR43" s="16" t="n">
+        <v>0.167361335</v>
+      </c>
+      <c r="AS43" s="17" t="n">
+        <v>811.418</v>
+      </c>
+      <c r="AT43" s="19" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="AU43" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV43" s="6" t="inlineStr">
+        <is>
+          <t>69cfbe81-3a03-4c37-bc49-4bd1b9359e83</t>
+        </is>
+      </c>
+      <c r="AW43" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-REGN-1793206659665</t>
+        </is>
+      </c>
+      <c r="AX43" s="13" t="n">
+        <v>46323.70670138889</v>
+      </c>
+      <c r="AY43" s="13" t="n">
+        <v>46323.70670138889</v>
+      </c>
+      <c r="AZ43" s="13" t="n">
+        <v>46323.7065625</v>
+      </c>
+      <c r="BA43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="13" t="n">
+        <v>46323.74836805555</v>
+      </c>
+      <c r="C44" s="13" t="n">
+        <v>46323.54003472222</v>
+      </c>
+      <c r="D44" s="13" t="n">
+        <v>46323.70670138889</v>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>The Southern Company</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J44" s="16" t="n">
+        <v>1.348382763</v>
+      </c>
+      <c r="K44" s="17" t="n">
+        <v>92.318</v>
+      </c>
+      <c r="L44" s="17">
+        <f>IF(AND(ISNUMBER(J44),ISNUMBER(K44)),J44*K44,"")</f>
+        <v/>
+      </c>
+      <c r="M44" s="17" t="n">
+        <v>124.49</v>
+      </c>
+      <c r="N44" s="16" t="n"/>
+      <c r="O44" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P44" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #5, 8.33% of the $1,494.58 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q44" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R44" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S44" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T44" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="U44" s="19" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="V44" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W44" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X44" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y44" s="19" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="Z44" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA44" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB44" s="15" t="inlineStr">
+        <is>
+          <t>One day (+3.8%) did 114% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC44" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD44" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE44" s="17" t="n">
+        <v>93.197</v>
+      </c>
+      <c r="AF44" s="17" t="n">
+        <v>91.0295</v>
+      </c>
+      <c r="AG44" s="17" t="n">
+        <v>95.3644</v>
+      </c>
+      <c r="AH44" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI44" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ44" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK44" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL44" s="15" t="inlineStr">
+        <is>
+          <t>RBC Capital Adjusts Southern Company Price Target</t>
+        </is>
+      </c>
+      <c r="AM44" s="17" t="n">
+        <v>92.33</v>
+      </c>
+      <c r="AN44" s="19" t="n">
+        <v>-0.0034</v>
+      </c>
+      <c r="AO44" s="17" t="n">
+        <v>100128.62</v>
+      </c>
+      <c r="AP44" s="17" t="n">
+        <v>1494.58</v>
+      </c>
+      <c r="AQ44" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR44" s="16" t="n"/>
+      <c r="AS44" s="17" t="n"/>
+      <c r="AT44" s="19" t="n"/>
+      <c r="AU44" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV44" s="6" t="inlineStr">
+        <is>
+          <t>84055f04-f1e8-4f84-b3d3-5c199cf649b6</t>
+        </is>
+      </c>
+      <c r="AW44" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-SO-1793206659765</t>
+        </is>
+      </c>
+      <c r="AX44" s="13" t="n">
+        <v>46323.70670138889</v>
+      </c>
+      <c r="AY44" s="13" t="n">
+        <v>46323.70670138889</v>
+      </c>
+      <c r="AZ44" s="13" t="n">
+        <v>46323.7065625</v>
+      </c>
+      <c r="BA44" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -8755,7 +9131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P39"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10930,15 +11306,21 @@
         <v>811.418</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>0.167361335</v>
+        <v>0.083680667</v>
       </c>
       <c r="G39" s="17">
         <f>E39*F39</f>
         <v/>
       </c>
-      <c r="H39" s="22" t="n"/>
-      <c r="I39" s="22" t="n"/>
-      <c r="J39" s="17" t="n"/>
+      <c r="H39" s="22" t="n">
+        <v>46323.74836805555</v>
+      </c>
+      <c r="I39" s="22" t="n">
+        <v>46323.54003472222</v>
+      </c>
+      <c r="J39" s="17" t="n">
+        <v>812.398</v>
+      </c>
       <c r="K39" s="17">
         <f>IF(ISNUMBER(J39),J39*F39,"")</f>
         <v/>
@@ -10955,15 +11337,125 @@
         <f>IF(ISNUMBER(H39),H39-C39,"")</f>
         <v/>
       </c>
-      <c r="O39" s="6" t="n"/>
+      <c r="O39" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P39" s="6" t="inlineStr">
         <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="n">
+        <v>46323.72341435185</v>
+      </c>
+      <c r="D40" s="22" t="n">
+        <v>46323.51508101852</v>
+      </c>
+      <c r="E40" s="17" t="n">
+        <v>811.418</v>
+      </c>
+      <c r="F40" s="16" t="n">
+        <v>0.083680668</v>
+      </c>
+      <c r="G40" s="17">
+        <f>E40*F40</f>
+        <v/>
+      </c>
+      <c r="H40" s="22" t="n"/>
+      <c r="I40" s="22" t="n"/>
+      <c r="J40" s="17" t="n"/>
+      <c r="K40" s="17">
+        <f>IF(ISNUMBER(J40),J40*F40,"")</f>
+        <v/>
+      </c>
+      <c r="L40" s="23">
+        <f>IF(ISNUMBER(J40),K40-G40,"")</f>
+        <v/>
+      </c>
+      <c r="M40" s="24">
+        <f>IF(ISNUMBER(J40),L40/G40,"")</f>
+        <v/>
+      </c>
+      <c r="N40" s="25">
+        <f>IF(ISNUMBER(H40),H40-C40,"")</f>
+        <v/>
+      </c>
+      <c r="O40" s="6" t="n"/>
+      <c r="P40" s="6" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>The Southern Company</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="n">
+        <v>46323.74836805555</v>
+      </c>
+      <c r="D41" s="22" t="n">
+        <v>46323.54003472222</v>
+      </c>
+      <c r="E41" s="17" t="n">
+        <v>92.318</v>
+      </c>
+      <c r="F41" s="16" t="n">
+        <v>1.348382763</v>
+      </c>
+      <c r="G41" s="17">
+        <f>E41*F41</f>
+        <v/>
+      </c>
+      <c r="H41" s="22" t="n"/>
+      <c r="I41" s="22" t="n"/>
+      <c r="J41" s="17" t="n"/>
+      <c r="K41" s="17">
+        <f>IF(ISNUMBER(J41),J41*F41,"")</f>
+        <v/>
+      </c>
+      <c r="L41" s="23">
+        <f>IF(ISNUMBER(J41),K41-G41,"")</f>
+        <v/>
+      </c>
+      <c r="M41" s="24">
+        <f>IF(ISNUMBER(J41),L41/G41,"")</f>
+        <v/>
+      </c>
+      <c r="N41" s="25">
+        <f>IF(ISNUMBER(H41),H41-C41,"")</f>
+        <v/>
+      </c>
+      <c r="O41" s="6" t="n"/>
+      <c r="P41" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M39">
+  <conditionalFormatting sqref="L2:M41">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 17:26 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA44" headerRowCount="1">
-  <autoFilter ref="A1:BA44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA45" headerRowCount="1">
+  <autoFilter ref="A1:BA45"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.74844907408</v>
+        <v>46323.76866898148</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.54011574074</v>
+        <v>46323.56033564815</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$44,"BUY")+COUNTIF(Orders!$E$2:$E$44,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$45,"BUY")+COUNTIF(Orders!$E$2:$E$45,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$44,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$45,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$44,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$45,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$44,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$45,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$44,Orders!$E$2:$E$44,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$45,Orders!$E$2:$E$45,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$44,Orders!$E$2:$E$44,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$45,Orders!$E$2:$E$45,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA44"/>
+  <dimension ref="A1:BA45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9116,6 +9116,194 @@
       </c>
       <c r="BA44" s="6" t="n"/>
     </row>
+    <row r="45">
+      <c r="A45" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="13" t="n">
+        <v>46323.76857638889</v>
+      </c>
+      <c r="C45" s="13" t="n">
+        <v>46323.56024305556</v>
+      </c>
+      <c r="D45" s="13" t="n">
+        <v>46323.72690972222</v>
+      </c>
+      <c r="E45" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>CNC</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="inlineStr">
+        <is>
+          <t>CNC</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J45" s="16" t="n">
+        <v>7.590071128</v>
+      </c>
+      <c r="K45" s="17" t="n">
+        <v>67.72</v>
+      </c>
+      <c r="L45" s="17">
+        <f>IF(AND(ISNUMBER(J45),ISNUMBER(K45)),J45*K45,"")</f>
+        <v/>
+      </c>
+      <c r="M45" s="17" t="n"/>
+      <c r="N45" s="16" t="n">
+        <v>7.590071128</v>
+      </c>
+      <c r="O45" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
+      <c r="P45" s="15" t="inlineStr">
+        <is>
+          <t>Only 2 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="R45" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S45" s="18" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="T45" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="U45" s="19" t="n">
+        <v>0.0126</v>
+      </c>
+      <c r="V45" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W45" s="12" t="n"/>
+      <c r="X45" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y45" s="19" t="n">
+        <v>0.0083</v>
+      </c>
+      <c r="Z45" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA45" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB45" s="15" t="n"/>
+      <c r="AC45" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD45" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE45" s="17" t="n">
+        <v>67.675</v>
+      </c>
+      <c r="AF45" s="17" t="n">
+        <v>64.496</v>
+      </c>
+      <c r="AG45" s="17" t="n">
+        <v>70.854</v>
+      </c>
+      <c r="AH45" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI45" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ45" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK45" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL45" s="15" t="inlineStr">
+        <is>
+          <t>Cantor Fitzgerald Upgrades Centene to Overweight and Raises Price Target to $79</t>
+        </is>
+      </c>
+      <c r="AM45" s="17" t="n">
+        <v>67.675</v>
+      </c>
+      <c r="AN45" s="19" t="n">
+        <v>-0.0164</v>
+      </c>
+      <c r="AO45" s="17" t="n">
+        <v>100241.95</v>
+      </c>
+      <c r="AP45" s="17" t="n">
+        <v>1438.08</v>
+      </c>
+      <c r="AQ45" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR45" s="16" t="n">
+        <v>7.590071128</v>
+      </c>
+      <c r="AS45" s="17" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="AT45" s="19" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="AU45" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV45" s="6" t="inlineStr">
+        <is>
+          <t>7ff433f1-3689-4c21-b29e-7b59fcb42089</t>
+        </is>
+      </c>
+      <c r="AW45" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-CNC-1793208403624</t>
+        </is>
+      </c>
+      <c r="AX45" s="13" t="n">
+        <v>46323.72688657408</v>
+      </c>
+      <c r="AY45" s="13" t="n">
+        <v>46323.72690972222</v>
+      </c>
+      <c r="AZ45" s="13" t="n">
+        <v>46323.72672453704</v>
+      </c>
+      <c r="BA45" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -10825,9 +11013,15 @@
         <f>E30*F30</f>
         <v/>
       </c>
-      <c r="H30" s="22" t="n"/>
-      <c r="I30" s="22" t="n"/>
-      <c r="J30" s="17" t="n"/>
+      <c r="H30" s="22" t="n">
+        <v>46323.76857638889</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>46323.56024305556</v>
+      </c>
+      <c r="J30" s="17" t="n">
+        <v>67.72</v>
+      </c>
       <c r="K30" s="17">
         <f>IF(ISNUMBER(J30),J30*F30,"")</f>
         <v/>
@@ -10844,10 +11038,14 @@
         <f>IF(ISNUMBER(H30),H30-C30,"")</f>
         <v/>
       </c>
-      <c r="O30" s="6" t="n"/>
+      <c r="O30" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-28 18:49 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA45" headerRowCount="1">
-  <autoFilter ref="A1:BA45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA46" headerRowCount="1">
+  <autoFilter ref="A1:BA46"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P41" headerRowCount="1">
-  <autoFilter ref="A1:P41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P42" headerRowCount="1">
+  <autoFilter ref="A1:P42"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.76866898148</v>
+        <v>46323.82621527778</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.56033564815</v>
+        <v>46323.61788194445</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$45,"BUY")+COUNTIF(Orders!$E$2:$E$45,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$46,"BUY")+COUNTIF(Orders!$E$2:$E$46,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$45,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$46,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$45,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$46,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$45,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$46,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$45,Orders!$E$2:$E$45,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$46,Orders!$E$2:$E$46,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$45,Orders!$E$2:$E$45,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$46,Orders!$E$2:$E$46,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$41,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$42,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$41,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$42,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$41)</f>
+        <f>SUM('Round trips'!$L$2:$L$42)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$41,"Closed",'Round trips'!$L$2:$L$41,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$42,"Closed",'Round trips'!$L$2:$L$42,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA45"/>
+  <dimension ref="A1:BA46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9304,6 +9304,194 @@
       </c>
       <c r="BA45" s="6" t="n"/>
     </row>
+    <row r="46">
+      <c r="A46" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="13" t="n">
+        <v>46323.82612268518</v>
+      </c>
+      <c r="C46" s="13" t="n">
+        <v>46323.61778935185</v>
+      </c>
+      <c r="D46" s="13" t="n">
+        <v>46323.78445601852</v>
+      </c>
+      <c r="E46" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J46" s="16" t="n">
+        <v>0.057344226</v>
+      </c>
+      <c r="K46" s="17" t="n">
+        <v>1291.566</v>
+      </c>
+      <c r="L46" s="17">
+        <f>IF(AND(ISNUMBER(J46),ISNUMBER(K46)),J46*K46,"")</f>
+        <v/>
+      </c>
+      <c r="M46" s="17" t="n"/>
+      <c r="N46" s="16" t="n">
+        <v>0.057344226</v>
+      </c>
+      <c r="O46" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P46" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R46" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S46" s="18" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="T46" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="U46" s="19" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="V46" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W46" s="12" t="n"/>
+      <c r="X46" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y46" s="19" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="Z46" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA46" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB46" s="15" t="n"/>
+      <c r="AC46" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD46" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE46" s="17" t="n">
+        <v>1313.054</v>
+      </c>
+      <c r="AF46" s="17" t="n">
+        <v>1260.219</v>
+      </c>
+      <c r="AG46" s="17" t="n">
+        <v>1365.889</v>
+      </c>
+      <c r="AH46" s="20" t="n">
+        <v>46330</v>
+      </c>
+      <c r="AI46" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ46" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK46" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL46" s="15" t="inlineStr">
+        <is>
+          <t>Top Wall Street Forecasters Revamp Eli Lilly Expectations Ahead Of Q3 Earnings</t>
+        </is>
+      </c>
+      <c r="AM46" s="17" t="n">
+        <v>1291.92</v>
+      </c>
+      <c r="AN46" s="19" t="n">
+        <v>0.008100000000000001</v>
+      </c>
+      <c r="AO46" s="17" t="n">
+        <v>100349.98</v>
+      </c>
+      <c r="AP46" s="17" t="n">
+        <v>1952.08</v>
+      </c>
+      <c r="AQ46" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR46" s="16" t="n">
+        <v>0.114688452</v>
+      </c>
+      <c r="AS46" s="17" t="n">
+        <v>1291.586</v>
+      </c>
+      <c r="AT46" s="19" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="AU46" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV46" s="6" t="inlineStr">
+        <is>
+          <t>f363e653-14b2-4970-9a58-3eb3ffaf679d</t>
+        </is>
+      </c>
+      <c r="AW46" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-LLY-1793213377714</t>
+        </is>
+      </c>
+      <c r="AX46" s="13" t="n">
+        <v>46323.78445601852</v>
+      </c>
+      <c r="AY46" s="13" t="n">
+        <v>46323.78445601852</v>
+      </c>
+      <c r="AZ46" s="13" t="n">
+        <v>46323.78435185185</v>
+      </c>
+      <c r="BA46" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -9319,7 +9507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11451,15 +11639,21 @@
         <v>1291.586</v>
       </c>
       <c r="F38" s="16" t="n">
-        <v>0.114688452</v>
+        <v>0.057344226</v>
       </c>
       <c r="G38" s="17">
         <f>E38*F38</f>
         <v/>
       </c>
-      <c r="H38" s="22" t="n"/>
-      <c r="I38" s="22" t="n"/>
-      <c r="J38" s="17" t="n"/>
+      <c r="H38" s="22" t="n">
+        <v>46323.82612268518</v>
+      </c>
+      <c r="I38" s="22" t="n">
+        <v>46323.61778935185</v>
+      </c>
+      <c r="J38" s="17" t="n">
+        <v>1291.566</v>
+      </c>
       <c r="K38" s="17">
         <f>IF(ISNUMBER(J38),J38*F38,"")</f>
         <v/>
@@ -11476,49 +11670,47 @@
         <f>IF(ISNUMBER(H38),H38-C38,"")</f>
         <v/>
       </c>
-      <c r="O38" s="6" t="n"/>
+      <c r="O38" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+          <t>Eli Lilly &amp; Co.</t>
         </is>
       </c>
       <c r="C39" s="22" t="n">
-        <v>46323.72341435185</v>
+        <v>46323.70951388889</v>
       </c>
       <c r="D39" s="22" t="n">
-        <v>46323.51508101852</v>
+        <v>46323.50118055556</v>
       </c>
       <c r="E39" s="17" t="n">
-        <v>811.418</v>
+        <v>1291.586</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>0.083680667</v>
+        <v>0.057344226</v>
       </c>
       <c r="G39" s="17">
         <f>E39*F39</f>
         <v/>
       </c>
-      <c r="H39" s="22" t="n">
-        <v>46323.74836805555</v>
-      </c>
-      <c r="I39" s="22" t="n">
-        <v>46323.54003472222</v>
-      </c>
-      <c r="J39" s="17" t="n">
-        <v>812.398</v>
-      </c>
+      <c r="H39" s="22" t="n"/>
+      <c r="I39" s="22" t="n"/>
+      <c r="J39" s="17" t="n"/>
       <c r="K39" s="17">
         <f>IF(ISNUMBER(J39),J39*F39,"")</f>
         <v/>
@@ -11535,14 +11727,10 @@
         <f>IF(ISNUMBER(H39),H39-C39,"")</f>
         <v/>
       </c>
-      <c r="O39" s="6" t="inlineStr">
-        <is>
-          <t>3 green: sell half</t>
-        </is>
-      </c>
+      <c r="O39" s="6" t="n"/>
       <c r="P39" s="6" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -11567,15 +11755,21 @@
         <v>811.418</v>
       </c>
       <c r="F40" s="16" t="n">
-        <v>0.083680668</v>
+        <v>0.083680667</v>
       </c>
       <c r="G40" s="17">
         <f>E40*F40</f>
         <v/>
       </c>
-      <c r="H40" s="22" t="n"/>
-      <c r="I40" s="22" t="n"/>
-      <c r="J40" s="17" t="n"/>
+      <c r="H40" s="22" t="n">
+        <v>46323.74836805555</v>
+      </c>
+      <c r="I40" s="22" t="n">
+        <v>46323.54003472222</v>
+      </c>
+      <c r="J40" s="17" t="n">
+        <v>812.398</v>
+      </c>
       <c r="K40" s="17">
         <f>IF(ISNUMBER(J40),J40*F40,"")</f>
         <v/>
@@ -11592,35 +11786,39 @@
         <f>IF(ISNUMBER(H40),H40-C40,"")</f>
         <v/>
       </c>
-      <c r="O40" s="6" t="n"/>
+      <c r="O40" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>The Southern Company</t>
+          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
         </is>
       </c>
       <c r="C41" s="22" t="n">
-        <v>46323.74836805555</v>
+        <v>46323.72341435185</v>
       </c>
       <c r="D41" s="22" t="n">
-        <v>46323.54003472222</v>
+        <v>46323.51508101852</v>
       </c>
       <c r="E41" s="17" t="n">
-        <v>92.318</v>
+        <v>811.418</v>
       </c>
       <c r="F41" s="16" t="n">
-        <v>1.348382763</v>
+        <v>0.083680668</v>
       </c>
       <c r="G41" s="17">
         <f>E41*F41</f>
@@ -11652,8 +11850,61 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>The Southern Company</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="n">
+        <v>46323.74836805555</v>
+      </c>
+      <c r="D42" s="22" t="n">
+        <v>46323.54003472222</v>
+      </c>
+      <c r="E42" s="17" t="n">
+        <v>92.318</v>
+      </c>
+      <c r="F42" s="16" t="n">
+        <v>1.348382763</v>
+      </c>
+      <c r="G42" s="17">
+        <f>E42*F42</f>
+        <v/>
+      </c>
+      <c r="H42" s="22" t="n"/>
+      <c r="I42" s="22" t="n"/>
+      <c r="J42" s="17" t="n"/>
+      <c r="K42" s="17">
+        <f>IF(ISNUMBER(J42),J42*F42,"")</f>
+        <v/>
+      </c>
+      <c r="L42" s="23">
+        <f>IF(ISNUMBER(J42),K42-G42,"")</f>
+        <v/>
+      </c>
+      <c r="M42" s="24">
+        <f>IF(ISNUMBER(J42),L42/G42,"")</f>
+        <v/>
+      </c>
+      <c r="N42" s="25">
+        <f>IF(ISNUMBER(H42),H42-C42,"")</f>
+        <v/>
+      </c>
+      <c r="O42" s="6" t="n"/>
+      <c r="P42" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M41">
+  <conditionalFormatting sqref="L2:M42">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-28 19:31 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA46" headerRowCount="1">
-  <autoFilter ref="A1:BA46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA75" headerRowCount="1">
+  <autoFilter ref="A1:BA75"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.82621527778</v>
+        <v>46323.85530092593</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.61788194445</v>
+        <v>46323.64696759259</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$46,"BUY")+COUNTIF(Orders!$E$2:$E$46,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$75,"BUY")+COUNTIF(Orders!$E$2:$E$75,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$46,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$75,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$46,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$75,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$46,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$75,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$46,Orders!$E$2:$E$46,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$75,Orders!$E$2:$E$75,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$46,Orders!$E$2:$E$46,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$75,Orders!$E$2:$E$75,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA46"/>
+  <dimension ref="A1:BA75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9492,6 +9492,3138 @@
       </c>
       <c r="BA46" s="6" t="n"/>
     </row>
+    <row r="47">
+      <c r="A47" s="12" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="13" t="n">
+        <v>46323.85436342593</v>
+      </c>
+      <c r="C47" s="13" t="n">
+        <v>46323.64603009259</v>
+      </c>
+      <c r="D47" s="13" t="n">
+        <v>46323.81269675926</v>
+      </c>
+      <c r="E47" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="n"/>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J47" s="16" t="n">
+        <v>3.63060686</v>
+      </c>
+      <c r="K47" s="17" t="n">
+        <v>286.66</v>
+      </c>
+      <c r="L47" s="17">
+        <f>IF(AND(ISNUMBER(J47),ISNUMBER(K47)),J47*K47,"")</f>
+        <v/>
+      </c>
+      <c r="M47" s="17" t="n"/>
+      <c r="N47" s="16" t="n">
+        <v>3.63060686</v>
+      </c>
+      <c r="O47" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P47" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q47" s="12" t="n"/>
+      <c r="R47" s="6" t="n"/>
+      <c r="S47" s="18" t="n"/>
+      <c r="T47" s="12" t="n"/>
+      <c r="U47" s="19" t="n"/>
+      <c r="V47" s="19" t="n"/>
+      <c r="W47" s="12" t="n"/>
+      <c r="X47" s="6" t="n"/>
+      <c r="Y47" s="19" t="n"/>
+      <c r="Z47" s="6" t="n"/>
+      <c r="AA47" s="12" t="n"/>
+      <c r="AB47" s="15" t="n"/>
+      <c r="AC47" s="6" t="n"/>
+      <c r="AD47" s="6" t="n"/>
+      <c r="AE47" s="17" t="n"/>
+      <c r="AF47" s="17" t="n"/>
+      <c r="AG47" s="17" t="n"/>
+      <c r="AH47" s="20" t="n"/>
+      <c r="AI47" s="18" t="n"/>
+      <c r="AJ47" s="6" t="n"/>
+      <c r="AK47" s="12" t="n"/>
+      <c r="AL47" s="15" t="n"/>
+      <c r="AM47" s="17" t="n"/>
+      <c r="AN47" s="19" t="n"/>
+      <c r="AO47" s="17" t="n"/>
+      <c r="AP47" s="17" t="n"/>
+      <c r="AQ47" s="19" t="n"/>
+      <c r="AR47" s="16" t="n"/>
+      <c r="AS47" s="17" t="n"/>
+      <c r="AT47" s="19" t="n"/>
+      <c r="AU47" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV47" s="6" t="inlineStr">
+        <is>
+          <t>ecdb68eb-fd99-4135-a88a-1eec26aaa8a3</t>
+        </is>
+      </c>
+      <c r="AW47" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ABBV-1793215815607</t>
+        </is>
+      </c>
+      <c r="AX47" s="13" t="n">
+        <v>46323.81267361111</v>
+      </c>
+      <c r="AY47" s="13" t="n">
+        <v>46323.81269675926</v>
+      </c>
+      <c r="AZ47" s="13" t="n"/>
+      <c r="BA47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="13" t="n">
+        <v>46323.854375</v>
+      </c>
+      <c r="C48" s="13" t="n">
+        <v>46323.64604166667</v>
+      </c>
+      <c r="D48" s="13" t="n">
+        <v>46323.81270833333</v>
+      </c>
+      <c r="E48" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="G48" s="15" t="n"/>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J48" s="16" t="n">
+        <v>2.460611764</v>
+      </c>
+      <c r="K48" s="17" t="n">
+        <v>426.02</v>
+      </c>
+      <c r="L48" s="17">
+        <f>IF(AND(ISNUMBER(J48),ISNUMBER(K48)),J48*K48,"")</f>
+        <v/>
+      </c>
+      <c r="M48" s="17" t="n"/>
+      <c r="N48" s="16" t="n">
+        <v>2.460611764</v>
+      </c>
+      <c r="O48" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P48" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q48" s="12" t="n"/>
+      <c r="R48" s="6" t="n"/>
+      <c r="S48" s="18" t="n"/>
+      <c r="T48" s="12" t="n"/>
+      <c r="U48" s="19" t="n"/>
+      <c r="V48" s="19" t="n"/>
+      <c r="W48" s="12" t="n"/>
+      <c r="X48" s="6" t="n"/>
+      <c r="Y48" s="19" t="n"/>
+      <c r="Z48" s="6" t="n"/>
+      <c r="AA48" s="12" t="n"/>
+      <c r="AB48" s="15" t="n"/>
+      <c r="AC48" s="6" t="n"/>
+      <c r="AD48" s="6" t="n"/>
+      <c r="AE48" s="17" t="n"/>
+      <c r="AF48" s="17" t="n"/>
+      <c r="AG48" s="17" t="n"/>
+      <c r="AH48" s="20" t="n"/>
+      <c r="AI48" s="18" t="n"/>
+      <c r="AJ48" s="6" t="n"/>
+      <c r="AK48" s="12" t="n"/>
+      <c r="AL48" s="15" t="n"/>
+      <c r="AM48" s="17" t="n"/>
+      <c r="AN48" s="19" t="n"/>
+      <c r="AO48" s="17" t="n"/>
+      <c r="AP48" s="17" t="n"/>
+      <c r="AQ48" s="19" t="n"/>
+      <c r="AR48" s="16" t="n"/>
+      <c r="AS48" s="17" t="n"/>
+      <c r="AT48" s="19" t="n"/>
+      <c r="AU48" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV48" s="6" t="inlineStr">
+        <is>
+          <t>c9c245bf-f10e-4860-8dbd-030c02ab0556</t>
+        </is>
+      </c>
+      <c r="AW48" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ADI-1793215816980</t>
+        </is>
+      </c>
+      <c r="AX48" s="13" t="n">
+        <v>46323.81269675926</v>
+      </c>
+      <c r="AY48" s="13" t="n">
+        <v>46323.81270833333</v>
+      </c>
+      <c r="AZ48" s="13" t="n"/>
+      <c r="BA48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="13" t="n">
+        <v>46323.85439814815</v>
+      </c>
+      <c r="C49" s="13" t="n">
+        <v>46323.64606481481</v>
+      </c>
+      <c r="D49" s="13" t="n">
+        <v>46323.81273148148</v>
+      </c>
+      <c r="E49" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>CBOE</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="n"/>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J49" s="16" t="n">
+        <v>25.834717916</v>
+      </c>
+      <c r="K49" s="17" t="n">
+        <v>322.32659</v>
+      </c>
+      <c r="L49" s="17">
+        <f>IF(AND(ISNUMBER(J49),ISNUMBER(K49)),J49*K49,"")</f>
+        <v/>
+      </c>
+      <c r="M49" s="17" t="n"/>
+      <c r="N49" s="16" t="n">
+        <v>25.834717916</v>
+      </c>
+      <c r="O49" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P49" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q49" s="12" t="n"/>
+      <c r="R49" s="6" t="n"/>
+      <c r="S49" s="18" t="n"/>
+      <c r="T49" s="12" t="n"/>
+      <c r="U49" s="19" t="n"/>
+      <c r="V49" s="19" t="n"/>
+      <c r="W49" s="12" t="n"/>
+      <c r="X49" s="6" t="n"/>
+      <c r="Y49" s="19" t="n"/>
+      <c r="Z49" s="6" t="n"/>
+      <c r="AA49" s="12" t="n"/>
+      <c r="AB49" s="15" t="n"/>
+      <c r="AC49" s="6" t="n"/>
+      <c r="AD49" s="6" t="n"/>
+      <c r="AE49" s="17" t="n"/>
+      <c r="AF49" s="17" t="n"/>
+      <c r="AG49" s="17" t="n"/>
+      <c r="AH49" s="20" t="n"/>
+      <c r="AI49" s="18" t="n"/>
+      <c r="AJ49" s="6" t="n"/>
+      <c r="AK49" s="12" t="n"/>
+      <c r="AL49" s="15" t="n"/>
+      <c r="AM49" s="17" t="n"/>
+      <c r="AN49" s="19" t="n"/>
+      <c r="AO49" s="17" t="n"/>
+      <c r="AP49" s="17" t="n"/>
+      <c r="AQ49" s="19" t="n"/>
+      <c r="AR49" s="16" t="n"/>
+      <c r="AS49" s="17" t="n"/>
+      <c r="AT49" s="19" t="n"/>
+      <c r="AU49" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV49" s="6" t="inlineStr">
+        <is>
+          <t>348491cc-58de-42d7-8c1f-65813f0e1722</t>
+        </is>
+      </c>
+      <c r="AW49" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-CBOE-1793215818325</t>
+        </is>
+      </c>
+      <c r="AX49" s="13" t="n">
+        <v>46323.81270833333</v>
+      </c>
+      <c r="AY49" s="13" t="n">
+        <v>46323.81273148148</v>
+      </c>
+      <c r="AZ49" s="13" t="n"/>
+      <c r="BA49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="13" t="n">
+        <v>46323.8544212963</v>
+      </c>
+      <c r="C50" s="13" t="n">
+        <v>46323.64608796296</v>
+      </c>
+      <c r="D50" s="13" t="n">
+        <v>46323.81275462963</v>
+      </c>
+      <c r="E50" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="G50" s="15" t="n"/>
+      <c r="H50" s="6" t="n"/>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J50" s="16" t="n">
+        <v>15.713899323</v>
+      </c>
+      <c r="K50" s="17" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="L50" s="17">
+        <f>IF(AND(ISNUMBER(J50),ISNUMBER(K50)),J50*K50,"")</f>
+        <v/>
+      </c>
+      <c r="M50" s="17" t="n"/>
+      <c r="N50" s="16" t="n">
+        <v>15.713899323</v>
+      </c>
+      <c r="O50" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P50" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q50" s="12" t="n"/>
+      <c r="R50" s="6" t="n"/>
+      <c r="S50" s="18" t="n"/>
+      <c r="T50" s="12" t="n"/>
+      <c r="U50" s="19" t="n"/>
+      <c r="V50" s="19" t="n"/>
+      <c r="W50" s="12" t="n"/>
+      <c r="X50" s="6" t="n"/>
+      <c r="Y50" s="19" t="n"/>
+      <c r="Z50" s="6" t="n"/>
+      <c r="AA50" s="12" t="n"/>
+      <c r="AB50" s="15" t="n"/>
+      <c r="AC50" s="6" t="n"/>
+      <c r="AD50" s="6" t="n"/>
+      <c r="AE50" s="17" t="n"/>
+      <c r="AF50" s="17" t="n"/>
+      <c r="AG50" s="17" t="n"/>
+      <c r="AH50" s="20" t="n"/>
+      <c r="AI50" s="18" t="n"/>
+      <c r="AJ50" s="6" t="n"/>
+      <c r="AK50" s="12" t="n"/>
+      <c r="AL50" s="15" t="n"/>
+      <c r="AM50" s="17" t="n"/>
+      <c r="AN50" s="19" t="n"/>
+      <c r="AO50" s="17" t="n"/>
+      <c r="AP50" s="17" t="n"/>
+      <c r="AQ50" s="19" t="n"/>
+      <c r="AR50" s="16" t="n"/>
+      <c r="AS50" s="17" t="n"/>
+      <c r="AT50" s="19" t="n"/>
+      <c r="AU50" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV50" s="6" t="inlineStr">
+        <is>
+          <t>2325c275-144c-4627-9a2a-204c654b3f61</t>
+        </is>
+      </c>
+      <c r="AW50" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-CTSH-1793215819690</t>
+        </is>
+      </c>
+      <c r="AX50" s="13" t="n">
+        <v>46323.81271990741</v>
+      </c>
+      <c r="AY50" s="13" t="n">
+        <v>46323.81275462963</v>
+      </c>
+      <c r="AZ50" s="13" t="n"/>
+      <c r="BA50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="13" t="n">
+        <v>46323.85440972223</v>
+      </c>
+      <c r="C51" s="13" t="n">
+        <v>46323.64607638889</v>
+      </c>
+      <c r="D51" s="13" t="n">
+        <v>46323.81274305555</v>
+      </c>
+      <c r="E51" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>DINO</t>
+        </is>
+      </c>
+      <c r="G51" s="15" t="n"/>
+      <c r="H51" s="6" t="n"/>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J51" s="16" t="n">
+        <v>0.486970655</v>
+      </c>
+      <c r="K51" s="17" t="n">
+        <v>113.556</v>
+      </c>
+      <c r="L51" s="17">
+        <f>IF(AND(ISNUMBER(J51),ISNUMBER(K51)),J51*K51,"")</f>
+        <v/>
+      </c>
+      <c r="M51" s="17" t="n"/>
+      <c r="N51" s="16" t="n">
+        <v>0.486970655</v>
+      </c>
+      <c r="O51" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P51" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q51" s="12" t="n"/>
+      <c r="R51" s="6" t="n"/>
+      <c r="S51" s="18" t="n"/>
+      <c r="T51" s="12" t="n"/>
+      <c r="U51" s="19" t="n"/>
+      <c r="V51" s="19" t="n"/>
+      <c r="W51" s="12" t="n"/>
+      <c r="X51" s="6" t="n"/>
+      <c r="Y51" s="19" t="n"/>
+      <c r="Z51" s="6" t="n"/>
+      <c r="AA51" s="12" t="n"/>
+      <c r="AB51" s="15" t="n"/>
+      <c r="AC51" s="6" t="n"/>
+      <c r="AD51" s="6" t="n"/>
+      <c r="AE51" s="17" t="n"/>
+      <c r="AF51" s="17" t="n"/>
+      <c r="AG51" s="17" t="n"/>
+      <c r="AH51" s="20" t="n"/>
+      <c r="AI51" s="18" t="n"/>
+      <c r="AJ51" s="6" t="n"/>
+      <c r="AK51" s="12" t="n"/>
+      <c r="AL51" s="15" t="n"/>
+      <c r="AM51" s="17" t="n"/>
+      <c r="AN51" s="19" t="n"/>
+      <c r="AO51" s="17" t="n"/>
+      <c r="AP51" s="17" t="n"/>
+      <c r="AQ51" s="19" t="n"/>
+      <c r="AR51" s="16" t="n"/>
+      <c r="AS51" s="17" t="n"/>
+      <c r="AT51" s="19" t="n"/>
+      <c r="AU51" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV51" s="6" t="inlineStr">
+        <is>
+          <t>bbf19542-ad5d-4daf-99e4-e0780f5cba3c</t>
+        </is>
+      </c>
+      <c r="AW51" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-DINO-1793215821053</t>
+        </is>
+      </c>
+      <c r="AX51" s="13" t="n">
+        <v>46323.81274305555</v>
+      </c>
+      <c r="AY51" s="13" t="n">
+        <v>46323.81274305555</v>
+      </c>
+      <c r="AZ51" s="13" t="n"/>
+      <c r="BA51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="13" t="n">
+        <v>46323.85445601852</v>
+      </c>
+      <c r="C52" s="13" t="n">
+        <v>46323.64612268518</v>
+      </c>
+      <c r="D52" s="13" t="n">
+        <v>46323.81278935185</v>
+      </c>
+      <c r="E52" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="G52" s="15" t="n"/>
+      <c r="H52" s="6" t="n"/>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J52" s="16" t="n">
+        <v>130.2953125</v>
+      </c>
+      <c r="K52" s="17" t="n">
+        <v>62.591634</v>
+      </c>
+      <c r="L52" s="17">
+        <f>IF(AND(ISNUMBER(J52),ISNUMBER(K52)),J52*K52,"")</f>
+        <v/>
+      </c>
+      <c r="M52" s="17" t="n"/>
+      <c r="N52" s="16" t="n">
+        <v>130.2953125</v>
+      </c>
+      <c r="O52" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P52" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q52" s="12" t="n"/>
+      <c r="R52" s="6" t="n"/>
+      <c r="S52" s="18" t="n"/>
+      <c r="T52" s="12" t="n"/>
+      <c r="U52" s="19" t="n"/>
+      <c r="V52" s="19" t="n"/>
+      <c r="W52" s="12" t="n"/>
+      <c r="X52" s="6" t="n"/>
+      <c r="Y52" s="19" t="n"/>
+      <c r="Z52" s="6" t="n"/>
+      <c r="AA52" s="12" t="n"/>
+      <c r="AB52" s="15" t="n"/>
+      <c r="AC52" s="6" t="n"/>
+      <c r="AD52" s="6" t="n"/>
+      <c r="AE52" s="17" t="n"/>
+      <c r="AF52" s="17" t="n"/>
+      <c r="AG52" s="17" t="n"/>
+      <c r="AH52" s="20" t="n"/>
+      <c r="AI52" s="18" t="n"/>
+      <c r="AJ52" s="6" t="n"/>
+      <c r="AK52" s="12" t="n"/>
+      <c r="AL52" s="15" t="n"/>
+      <c r="AM52" s="17" t="n"/>
+      <c r="AN52" s="19" t="n"/>
+      <c r="AO52" s="17" t="n"/>
+      <c r="AP52" s="17" t="n"/>
+      <c r="AQ52" s="19" t="n"/>
+      <c r="AR52" s="16" t="n"/>
+      <c r="AS52" s="17" t="n"/>
+      <c r="AT52" s="19" t="n"/>
+      <c r="AU52" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV52" s="6" t="inlineStr">
+        <is>
+          <t>99c08b19-1d7a-4a5a-bb13-20150fde7167</t>
+        </is>
+      </c>
+      <c r="AW52" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-DT-1793215822409</t>
+        </is>
+      </c>
+      <c r="AX52" s="13" t="n">
+        <v>46323.81275462963</v>
+      </c>
+      <c r="AY52" s="13" t="n">
+        <v>46323.81278935185</v>
+      </c>
+      <c r="AZ52" s="13" t="n"/>
+      <c r="BA52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="13" t="n">
+        <v>46323.85445601852</v>
+      </c>
+      <c r="C53" s="13" t="n">
+        <v>46323.64612268518</v>
+      </c>
+      <c r="D53" s="13" t="n">
+        <v>46323.81278935185</v>
+      </c>
+      <c r="E53" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="G53" s="15" t="n"/>
+      <c r="H53" s="6" t="n"/>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J53" s="16" t="n">
+        <v>70.13268309</v>
+      </c>
+      <c r="K53" s="17" t="n">
+        <v>117.477719</v>
+      </c>
+      <c r="L53" s="17">
+        <f>IF(AND(ISNUMBER(J53),ISNUMBER(K53)),J53*K53,"")</f>
+        <v/>
+      </c>
+      <c r="M53" s="17" t="n"/>
+      <c r="N53" s="16" t="n">
+        <v>70.13268309</v>
+      </c>
+      <c r="O53" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P53" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q53" s="12" t="n"/>
+      <c r="R53" s="6" t="n"/>
+      <c r="S53" s="18" t="n"/>
+      <c r="T53" s="12" t="n"/>
+      <c r="U53" s="19" t="n"/>
+      <c r="V53" s="19" t="n"/>
+      <c r="W53" s="12" t="n"/>
+      <c r="X53" s="6" t="n"/>
+      <c r="Y53" s="19" t="n"/>
+      <c r="Z53" s="6" t="n"/>
+      <c r="AA53" s="12" t="n"/>
+      <c r="AB53" s="15" t="n"/>
+      <c r="AC53" s="6" t="n"/>
+      <c r="AD53" s="6" t="n"/>
+      <c r="AE53" s="17" t="n"/>
+      <c r="AF53" s="17" t="n"/>
+      <c r="AG53" s="17" t="n"/>
+      <c r="AH53" s="20" t="n"/>
+      <c r="AI53" s="18" t="n"/>
+      <c r="AJ53" s="6" t="n"/>
+      <c r="AK53" s="12" t="n"/>
+      <c r="AL53" s="15" t="n"/>
+      <c r="AM53" s="17" t="n"/>
+      <c r="AN53" s="19" t="n"/>
+      <c r="AO53" s="17" t="n"/>
+      <c r="AP53" s="17" t="n"/>
+      <c r="AQ53" s="19" t="n"/>
+      <c r="AR53" s="16" t="n"/>
+      <c r="AS53" s="17" t="n"/>
+      <c r="AT53" s="19" t="n"/>
+      <c r="AU53" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV53" s="6" t="inlineStr">
+        <is>
+          <t>7e3b9a25-df34-45b9-87d0-39f00f5b6161</t>
+        </is>
+      </c>
+      <c r="AW53" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-EBAY-1793215823758</t>
+        </is>
+      </c>
+      <c r="AX53" s="13" t="n">
+        <v>46323.8127662037</v>
+      </c>
+      <c r="AY53" s="13" t="n">
+        <v>46323.81278935185</v>
+      </c>
+      <c r="AZ53" s="13" t="n"/>
+      <c r="BA53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="13" t="n">
+        <v>46323.8544675926</v>
+      </c>
+      <c r="C54" s="13" t="n">
+        <v>46323.64613425926</v>
+      </c>
+      <c r="D54" s="13" t="n">
+        <v>46323.81280092592</v>
+      </c>
+      <c r="E54" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="G54" s="15" t="n"/>
+      <c r="H54" s="6" t="n"/>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J54" s="16" t="n">
+        <v>21.932885906</v>
+      </c>
+      <c r="K54" s="17" t="n">
+        <v>47.68</v>
+      </c>
+      <c r="L54" s="17">
+        <f>IF(AND(ISNUMBER(J54),ISNUMBER(K54)),J54*K54,"")</f>
+        <v/>
+      </c>
+      <c r="M54" s="17" t="n"/>
+      <c r="N54" s="16" t="n">
+        <v>21.932885906</v>
+      </c>
+      <c r="O54" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P54" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q54" s="12" t="n"/>
+      <c r="R54" s="6" t="n"/>
+      <c r="S54" s="18" t="n"/>
+      <c r="T54" s="12" t="n"/>
+      <c r="U54" s="19" t="n"/>
+      <c r="V54" s="19" t="n"/>
+      <c r="W54" s="12" t="n"/>
+      <c r="X54" s="6" t="n"/>
+      <c r="Y54" s="19" t="n"/>
+      <c r="Z54" s="6" t="n"/>
+      <c r="AA54" s="12" t="n"/>
+      <c r="AB54" s="15" t="n"/>
+      <c r="AC54" s="6" t="n"/>
+      <c r="AD54" s="6" t="n"/>
+      <c r="AE54" s="17" t="n"/>
+      <c r="AF54" s="17" t="n"/>
+      <c r="AG54" s="17" t="n"/>
+      <c r="AH54" s="20" t="n"/>
+      <c r="AI54" s="18" t="n"/>
+      <c r="AJ54" s="6" t="n"/>
+      <c r="AK54" s="12" t="n"/>
+      <c r="AL54" s="15" t="n"/>
+      <c r="AM54" s="17" t="n"/>
+      <c r="AN54" s="19" t="n"/>
+      <c r="AO54" s="17" t="n"/>
+      <c r="AP54" s="17" t="n"/>
+      <c r="AQ54" s="19" t="n"/>
+      <c r="AR54" s="16" t="n"/>
+      <c r="AS54" s="17" t="n"/>
+      <c r="AT54" s="19" t="n"/>
+      <c r="AU54" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV54" s="6" t="inlineStr">
+        <is>
+          <t>5706b4df-35d3-4d73-921f-dfffda2590f2</t>
+        </is>
+      </c>
+      <c r="AW54" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-EQNR-1793215825105</t>
+        </is>
+      </c>
+      <c r="AX54" s="13" t="n">
+        <v>46323.81278935185</v>
+      </c>
+      <c r="AY54" s="13" t="n">
+        <v>46323.81280092592</v>
+      </c>
+      <c r="AZ54" s="13" t="n"/>
+      <c r="BA54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="13" t="n">
+        <v>46323.85447916666</v>
+      </c>
+      <c r="C55" s="13" t="n">
+        <v>46323.64614583334</v>
+      </c>
+      <c r="D55" s="13" t="n">
+        <v>46323.8128125</v>
+      </c>
+      <c r="E55" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="n"/>
+      <c r="H55" s="6" t="n"/>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J55" s="16" t="n">
+        <v>1.562264961</v>
+      </c>
+      <c r="K55" s="17" t="n">
+        <v>56.34</v>
+      </c>
+      <c r="L55" s="17">
+        <f>IF(AND(ISNUMBER(J55),ISNUMBER(K55)),J55*K55,"")</f>
+        <v/>
+      </c>
+      <c r="M55" s="17" t="n"/>
+      <c r="N55" s="16" t="n">
+        <v>1.562264961</v>
+      </c>
+      <c r="O55" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P55" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q55" s="12" t="n"/>
+      <c r="R55" s="6" t="n"/>
+      <c r="S55" s="18" t="n"/>
+      <c r="T55" s="12" t="n"/>
+      <c r="U55" s="19" t="n"/>
+      <c r="V55" s="19" t="n"/>
+      <c r="W55" s="12" t="n"/>
+      <c r="X55" s="6" t="n"/>
+      <c r="Y55" s="19" t="n"/>
+      <c r="Z55" s="6" t="n"/>
+      <c r="AA55" s="12" t="n"/>
+      <c r="AB55" s="15" t="n"/>
+      <c r="AC55" s="6" t="n"/>
+      <c r="AD55" s="6" t="n"/>
+      <c r="AE55" s="17" t="n"/>
+      <c r="AF55" s="17" t="n"/>
+      <c r="AG55" s="17" t="n"/>
+      <c r="AH55" s="20" t="n"/>
+      <c r="AI55" s="18" t="n"/>
+      <c r="AJ55" s="6" t="n"/>
+      <c r="AK55" s="12" t="n"/>
+      <c r="AL55" s="15" t="n"/>
+      <c r="AM55" s="17" t="n"/>
+      <c r="AN55" s="19" t="n"/>
+      <c r="AO55" s="17" t="n"/>
+      <c r="AP55" s="17" t="n"/>
+      <c r="AQ55" s="19" t="n"/>
+      <c r="AR55" s="16" t="n"/>
+      <c r="AS55" s="17" t="n"/>
+      <c r="AT55" s="19" t="n"/>
+      <c r="AU55" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV55" s="6" t="inlineStr">
+        <is>
+          <t>bb32325f-f3dd-462d-9764-ab7b61e177e6</t>
+        </is>
+      </c>
+      <c r="AW55" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-EQT-1793215826520</t>
+        </is>
+      </c>
+      <c r="AX55" s="13" t="n">
+        <v>46323.81280092592</v>
+      </c>
+      <c r="AY55" s="13" t="n">
+        <v>46323.8128125</v>
+      </c>
+      <c r="AZ55" s="13" t="n"/>
+      <c r="BA55" s="6" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="13" t="n">
+        <v>46323.85449074074</v>
+      </c>
+      <c r="C56" s="13" t="n">
+        <v>46323.64615740741</v>
+      </c>
+      <c r="D56" s="13" t="n">
+        <v>46323.81282407408</v>
+      </c>
+      <c r="E56" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="G56" s="15" t="n"/>
+      <c r="H56" s="6" t="n"/>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J56" s="16" t="n">
+        <v>29.659715302</v>
+      </c>
+      <c r="K56" s="17" t="n">
+        <v>288.51</v>
+      </c>
+      <c r="L56" s="17">
+        <f>IF(AND(ISNUMBER(J56),ISNUMBER(K56)),J56*K56,"")</f>
+        <v/>
+      </c>
+      <c r="M56" s="17" t="n"/>
+      <c r="N56" s="16" t="n">
+        <v>29.659715302</v>
+      </c>
+      <c r="O56" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P56" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q56" s="12" t="n"/>
+      <c r="R56" s="6" t="n"/>
+      <c r="S56" s="18" t="n"/>
+      <c r="T56" s="12" t="n"/>
+      <c r="U56" s="19" t="n"/>
+      <c r="V56" s="19" t="n"/>
+      <c r="W56" s="12" t="n"/>
+      <c r="X56" s="6" t="n"/>
+      <c r="Y56" s="19" t="n"/>
+      <c r="Z56" s="6" t="n"/>
+      <c r="AA56" s="12" t="n"/>
+      <c r="AB56" s="15" t="n"/>
+      <c r="AC56" s="6" t="n"/>
+      <c r="AD56" s="6" t="n"/>
+      <c r="AE56" s="17" t="n"/>
+      <c r="AF56" s="17" t="n"/>
+      <c r="AG56" s="17" t="n"/>
+      <c r="AH56" s="20" t="n"/>
+      <c r="AI56" s="18" t="n"/>
+      <c r="AJ56" s="6" t="n"/>
+      <c r="AK56" s="12" t="n"/>
+      <c r="AL56" s="15" t="n"/>
+      <c r="AM56" s="17" t="n"/>
+      <c r="AN56" s="19" t="n"/>
+      <c r="AO56" s="17" t="n"/>
+      <c r="AP56" s="17" t="n"/>
+      <c r="AQ56" s="19" t="n"/>
+      <c r="AR56" s="16" t="n"/>
+      <c r="AS56" s="17" t="n"/>
+      <c r="AT56" s="19" t="n"/>
+      <c r="AU56" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV56" s="6" t="inlineStr">
+        <is>
+          <t>ec00043f-733c-4dec-be1d-d537a299dd76</t>
+        </is>
+      </c>
+      <c r="AW56" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ILMN-1793215827864</t>
+        </is>
+      </c>
+      <c r="AX56" s="13" t="n">
+        <v>46323.81282407408</v>
+      </c>
+      <c r="AY56" s="13" t="n">
+        <v>46323.81282407408</v>
+      </c>
+      <c r="AZ56" s="13" t="n"/>
+      <c r="BA56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="13" t="n">
+        <v>46323.85454861111</v>
+      </c>
+      <c r="C57" s="13" t="n">
+        <v>46323.64621527777</v>
+      </c>
+      <c r="D57" s="13" t="n">
+        <v>46323.81288194445</v>
+      </c>
+      <c r="E57" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="G57" s="15" t="n"/>
+      <c r="H57" s="6" t="n"/>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J57" s="16" t="n">
+        <v>15.179879935</v>
+      </c>
+      <c r="K57" s="17" t="n">
+        <v>276.99</v>
+      </c>
+      <c r="L57" s="17">
+        <f>IF(AND(ISNUMBER(J57),ISNUMBER(K57)),J57*K57,"")</f>
+        <v/>
+      </c>
+      <c r="M57" s="17" t="n"/>
+      <c r="N57" s="16" t="n">
+        <v>15.179879935</v>
+      </c>
+      <c r="O57" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P57" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q57" s="12" t="n"/>
+      <c r="R57" s="6" t="n"/>
+      <c r="S57" s="18" t="n"/>
+      <c r="T57" s="12" t="n"/>
+      <c r="U57" s="19" t="n"/>
+      <c r="V57" s="19" t="n"/>
+      <c r="W57" s="12" t="n"/>
+      <c r="X57" s="6" t="n"/>
+      <c r="Y57" s="19" t="n"/>
+      <c r="Z57" s="6" t="n"/>
+      <c r="AA57" s="12" t="n"/>
+      <c r="AB57" s="15" t="n"/>
+      <c r="AC57" s="6" t="n"/>
+      <c r="AD57" s="6" t="n"/>
+      <c r="AE57" s="17" t="n"/>
+      <c r="AF57" s="17" t="n"/>
+      <c r="AG57" s="17" t="n"/>
+      <c r="AH57" s="20" t="n"/>
+      <c r="AI57" s="18" t="n"/>
+      <c r="AJ57" s="6" t="n"/>
+      <c r="AK57" s="12" t="n"/>
+      <c r="AL57" s="15" t="n"/>
+      <c r="AM57" s="17" t="n"/>
+      <c r="AN57" s="19" t="n"/>
+      <c r="AO57" s="17" t="n"/>
+      <c r="AP57" s="17" t="n"/>
+      <c r="AQ57" s="19" t="n"/>
+      <c r="AR57" s="16" t="n"/>
+      <c r="AS57" s="17" t="n"/>
+      <c r="AT57" s="19" t="n"/>
+      <c r="AU57" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV57" s="6" t="inlineStr">
+        <is>
+          <t>b8de6178-d62b-48bd-b758-40dc1a541577</t>
+        </is>
+      </c>
+      <c r="AW57" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-IQV-1793215829241</t>
+        </is>
+      </c>
+      <c r="AX57" s="13" t="n">
+        <v>46323.81283564815</v>
+      </c>
+      <c r="AY57" s="13" t="n">
+        <v>46323.81288194445</v>
+      </c>
+      <c r="AZ57" s="13" t="n"/>
+      <c r="BA57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="13" t="n">
+        <v>46323.85454861111</v>
+      </c>
+      <c r="C58" s="13" t="n">
+        <v>46323.64621527777</v>
+      </c>
+      <c r="D58" s="13" t="n">
+        <v>46323.81288194445</v>
+      </c>
+      <c r="E58" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="G58" s="15" t="n"/>
+      <c r="H58" s="6" t="n"/>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J58" s="16" t="n">
+        <v>15.948757053</v>
+      </c>
+      <c r="K58" s="17" t="n">
+        <v>65.22</v>
+      </c>
+      <c r="L58" s="17">
+        <f>IF(AND(ISNUMBER(J58),ISNUMBER(K58)),J58*K58,"")</f>
+        <v/>
+      </c>
+      <c r="M58" s="17" t="n"/>
+      <c r="N58" s="16" t="n">
+        <v>15.948757053</v>
+      </c>
+      <c r="O58" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P58" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q58" s="12" t="n"/>
+      <c r="R58" s="6" t="n"/>
+      <c r="S58" s="18" t="n"/>
+      <c r="T58" s="12" t="n"/>
+      <c r="U58" s="19" t="n"/>
+      <c r="V58" s="19" t="n"/>
+      <c r="W58" s="12" t="n"/>
+      <c r="X58" s="6" t="n"/>
+      <c r="Y58" s="19" t="n"/>
+      <c r="Z58" s="6" t="n"/>
+      <c r="AA58" s="12" t="n"/>
+      <c r="AB58" s="15" t="n"/>
+      <c r="AC58" s="6" t="n"/>
+      <c r="AD58" s="6" t="n"/>
+      <c r="AE58" s="17" t="n"/>
+      <c r="AF58" s="17" t="n"/>
+      <c r="AG58" s="17" t="n"/>
+      <c r="AH58" s="20" t="n"/>
+      <c r="AI58" s="18" t="n"/>
+      <c r="AJ58" s="6" t="n"/>
+      <c r="AK58" s="12" t="n"/>
+      <c r="AL58" s="15" t="n"/>
+      <c r="AM58" s="17" t="n"/>
+      <c r="AN58" s="19" t="n"/>
+      <c r="AO58" s="17" t="n"/>
+      <c r="AP58" s="17" t="n"/>
+      <c r="AQ58" s="19" t="n"/>
+      <c r="AR58" s="16" t="n"/>
+      <c r="AS58" s="17" t="n"/>
+      <c r="AT58" s="19" t="n"/>
+      <c r="AU58" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV58" s="6" t="inlineStr">
+        <is>
+          <t>ee9ae1f0-579c-4aa0-a2c4-6f9e252ed5eb</t>
+        </is>
+      </c>
+      <c r="AW58" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-KR-1793215830670</t>
+        </is>
+      </c>
+      <c r="AX58" s="13" t="n">
+        <v>46323.81284722222</v>
+      </c>
+      <c r="AY58" s="13" t="n">
+        <v>46323.81288194445</v>
+      </c>
+      <c r="AZ58" s="13" t="n"/>
+      <c r="BA58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="13" t="n">
+        <v>46323.85453703703</v>
+      </c>
+      <c r="C59" s="13" t="n">
+        <v>46323.64620370371</v>
+      </c>
+      <c r="D59" s="13" t="n">
+        <v>46323.81287037037</v>
+      </c>
+      <c r="E59" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="G59" s="15" t="n"/>
+      <c r="H59" s="6" t="n"/>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J59" s="16" t="n">
+        <v>0.057344226</v>
+      </c>
+      <c r="K59" s="17" t="n">
+        <v>1295.462</v>
+      </c>
+      <c r="L59" s="17">
+        <f>IF(AND(ISNUMBER(J59),ISNUMBER(K59)),J59*K59,"")</f>
+        <v/>
+      </c>
+      <c r="M59" s="17" t="n"/>
+      <c r="N59" s="16" t="n">
+        <v>0.057344226</v>
+      </c>
+      <c r="O59" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P59" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q59" s="12" t="n"/>
+      <c r="R59" s="6" t="n"/>
+      <c r="S59" s="18" t="n"/>
+      <c r="T59" s="12" t="n"/>
+      <c r="U59" s="19" t="n"/>
+      <c r="V59" s="19" t="n"/>
+      <c r="W59" s="12" t="n"/>
+      <c r="X59" s="6" t="n"/>
+      <c r="Y59" s="19" t="n"/>
+      <c r="Z59" s="6" t="n"/>
+      <c r="AA59" s="12" t="n"/>
+      <c r="AB59" s="15" t="n"/>
+      <c r="AC59" s="6" t="n"/>
+      <c r="AD59" s="6" t="n"/>
+      <c r="AE59" s="17" t="n"/>
+      <c r="AF59" s="17" t="n"/>
+      <c r="AG59" s="17" t="n"/>
+      <c r="AH59" s="20" t="n"/>
+      <c r="AI59" s="18" t="n"/>
+      <c r="AJ59" s="6" t="n"/>
+      <c r="AK59" s="12" t="n"/>
+      <c r="AL59" s="15" t="n"/>
+      <c r="AM59" s="17" t="n"/>
+      <c r="AN59" s="19" t="n"/>
+      <c r="AO59" s="17" t="n"/>
+      <c r="AP59" s="17" t="n"/>
+      <c r="AQ59" s="19" t="n"/>
+      <c r="AR59" s="16" t="n"/>
+      <c r="AS59" s="17" t="n"/>
+      <c r="AT59" s="19" t="n"/>
+      <c r="AU59" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV59" s="6" t="inlineStr">
+        <is>
+          <t>6821bf60-59eb-4195-a107-b43395f1d9bf</t>
+        </is>
+      </c>
+      <c r="AW59" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-LLY-1793215832015</t>
+        </is>
+      </c>
+      <c r="AX59" s="13" t="n">
+        <v>46323.81287037037</v>
+      </c>
+      <c r="AY59" s="13" t="n">
+        <v>46323.81287037037</v>
+      </c>
+      <c r="AZ59" s="13" t="n"/>
+      <c r="BA59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="13" t="n">
+        <v>46323.85457175926</v>
+      </c>
+      <c r="C60" s="13" t="n">
+        <v>46323.64623842593</v>
+      </c>
+      <c r="D60" s="13" t="n">
+        <v>46323.81290509259</v>
+      </c>
+      <c r="E60" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>LNG</t>
+        </is>
+      </c>
+      <c r="G60" s="15" t="n"/>
+      <c r="H60" s="6" t="n"/>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J60" s="16" t="n">
+        <v>3.489356022</v>
+      </c>
+      <c r="K60" s="17" t="n">
+        <v>297.565854</v>
+      </c>
+      <c r="L60" s="17">
+        <f>IF(AND(ISNUMBER(J60),ISNUMBER(K60)),J60*K60,"")</f>
+        <v/>
+      </c>
+      <c r="M60" s="17" t="n"/>
+      <c r="N60" s="16" t="n">
+        <v>3.489356022</v>
+      </c>
+      <c r="O60" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P60" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q60" s="12" t="n"/>
+      <c r="R60" s="6" t="n"/>
+      <c r="S60" s="18" t="n"/>
+      <c r="T60" s="12" t="n"/>
+      <c r="U60" s="19" t="n"/>
+      <c r="V60" s="19" t="n"/>
+      <c r="W60" s="12" t="n"/>
+      <c r="X60" s="6" t="n"/>
+      <c r="Y60" s="19" t="n"/>
+      <c r="Z60" s="6" t="n"/>
+      <c r="AA60" s="12" t="n"/>
+      <c r="AB60" s="15" t="n"/>
+      <c r="AC60" s="6" t="n"/>
+      <c r="AD60" s="6" t="n"/>
+      <c r="AE60" s="17" t="n"/>
+      <c r="AF60" s="17" t="n"/>
+      <c r="AG60" s="17" t="n"/>
+      <c r="AH60" s="20" t="n"/>
+      <c r="AI60" s="18" t="n"/>
+      <c r="AJ60" s="6" t="n"/>
+      <c r="AK60" s="12" t="n"/>
+      <c r="AL60" s="15" t="n"/>
+      <c r="AM60" s="17" t="n"/>
+      <c r="AN60" s="19" t="n"/>
+      <c r="AO60" s="17" t="n"/>
+      <c r="AP60" s="17" t="n"/>
+      <c r="AQ60" s="19" t="n"/>
+      <c r="AR60" s="16" t="n"/>
+      <c r="AS60" s="17" t="n"/>
+      <c r="AT60" s="19" t="n"/>
+      <c r="AU60" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV60" s="6" t="inlineStr">
+        <is>
+          <t>f6446b61-0fb1-4a55-af62-bfdd09ad3c3e</t>
+        </is>
+      </c>
+      <c r="AW60" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-LNG-1793215833366</t>
+        </is>
+      </c>
+      <c r="AX60" s="13" t="n">
+        <v>46323.81288194445</v>
+      </c>
+      <c r="AY60" s="13" t="n">
+        <v>46323.81290509259</v>
+      </c>
+      <c r="AZ60" s="13" t="n"/>
+      <c r="BA60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="13" t="n">
+        <v>46323.85456018519</v>
+      </c>
+      <c r="C61" s="13" t="n">
+        <v>46323.64622685185</v>
+      </c>
+      <c r="D61" s="13" t="n">
+        <v>46323.81289351852</v>
+      </c>
+      <c r="E61" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="n"/>
+      <c r="H61" s="6" t="n"/>
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J61" s="16" t="n">
+        <v>0.852029044</v>
+      </c>
+      <c r="K61" s="17" t="n">
+        <v>612.568</v>
+      </c>
+      <c r="L61" s="17">
+        <f>IF(AND(ISNUMBER(J61),ISNUMBER(K61)),J61*K61,"")</f>
+        <v/>
+      </c>
+      <c r="M61" s="17" t="n"/>
+      <c r="N61" s="16" t="n">
+        <v>0.852029044</v>
+      </c>
+      <c r="O61" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P61" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q61" s="12" t="n"/>
+      <c r="R61" s="6" t="n"/>
+      <c r="S61" s="18" t="n"/>
+      <c r="T61" s="12" t="n"/>
+      <c r="U61" s="19" t="n"/>
+      <c r="V61" s="19" t="n"/>
+      <c r="W61" s="12" t="n"/>
+      <c r="X61" s="6" t="n"/>
+      <c r="Y61" s="19" t="n"/>
+      <c r="Z61" s="6" t="n"/>
+      <c r="AA61" s="12" t="n"/>
+      <c r="AB61" s="15" t="n"/>
+      <c r="AC61" s="6" t="n"/>
+      <c r="AD61" s="6" t="n"/>
+      <c r="AE61" s="17" t="n"/>
+      <c r="AF61" s="17" t="n"/>
+      <c r="AG61" s="17" t="n"/>
+      <c r="AH61" s="20" t="n"/>
+      <c r="AI61" s="18" t="n"/>
+      <c r="AJ61" s="6" t="n"/>
+      <c r="AK61" s="12" t="n"/>
+      <c r="AL61" s="15" t="n"/>
+      <c r="AM61" s="17" t="n"/>
+      <c r="AN61" s="19" t="n"/>
+      <c r="AO61" s="17" t="n"/>
+      <c r="AP61" s="17" t="n"/>
+      <c r="AQ61" s="19" t="n"/>
+      <c r="AR61" s="16" t="n"/>
+      <c r="AS61" s="17" t="n"/>
+      <c r="AT61" s="19" t="n"/>
+      <c r="AU61" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV61" s="6" t="inlineStr">
+        <is>
+          <t>c2f75328-b02e-4fd9-a6d3-34f8f02b82df</t>
+        </is>
+      </c>
+      <c r="AW61" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MA-1793215834729</t>
+        </is>
+      </c>
+      <c r="AX61" s="13" t="n">
+        <v>46323.81289351852</v>
+      </c>
+      <c r="AY61" s="13" t="n">
+        <v>46323.81289351852</v>
+      </c>
+      <c r="AZ61" s="13" t="n"/>
+      <c r="BA61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="13" t="n">
+        <v>46323.85459490741</v>
+      </c>
+      <c r="C62" s="13" t="n">
+        <v>46323.64626157407</v>
+      </c>
+      <c r="D62" s="13" t="n">
+        <v>46323.81292824074</v>
+      </c>
+      <c r="E62" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="n"/>
+      <c r="H62" s="6" t="n"/>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J62" s="16" t="n">
+        <v>8.620135337000001</v>
+      </c>
+      <c r="K62" s="17" t="n">
+        <v>959.34</v>
+      </c>
+      <c r="L62" s="17">
+        <f>IF(AND(ISNUMBER(J62),ISNUMBER(K62)),J62*K62,"")</f>
+        <v/>
+      </c>
+      <c r="M62" s="17" t="n"/>
+      <c r="N62" s="16" t="n">
+        <v>8.620135337000001</v>
+      </c>
+      <c r="O62" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P62" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q62" s="12" t="n"/>
+      <c r="R62" s="6" t="n"/>
+      <c r="S62" s="18" t="n"/>
+      <c r="T62" s="12" t="n"/>
+      <c r="U62" s="19" t="n"/>
+      <c r="V62" s="19" t="n"/>
+      <c r="W62" s="12" t="n"/>
+      <c r="X62" s="6" t="n"/>
+      <c r="Y62" s="19" t="n"/>
+      <c r="Z62" s="6" t="n"/>
+      <c r="AA62" s="12" t="n"/>
+      <c r="AB62" s="15" t="n"/>
+      <c r="AC62" s="6" t="n"/>
+      <c r="AD62" s="6" t="n"/>
+      <c r="AE62" s="17" t="n"/>
+      <c r="AF62" s="17" t="n"/>
+      <c r="AG62" s="17" t="n"/>
+      <c r="AH62" s="20" t="n"/>
+      <c r="AI62" s="18" t="n"/>
+      <c r="AJ62" s="6" t="n"/>
+      <c r="AK62" s="12" t="n"/>
+      <c r="AL62" s="15" t="n"/>
+      <c r="AM62" s="17" t="n"/>
+      <c r="AN62" s="19" t="n"/>
+      <c r="AO62" s="17" t="n"/>
+      <c r="AP62" s="17" t="n"/>
+      <c r="AQ62" s="19" t="n"/>
+      <c r="AR62" s="16" t="n"/>
+      <c r="AS62" s="17" t="n"/>
+      <c r="AT62" s="19" t="n"/>
+      <c r="AU62" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV62" s="6" t="inlineStr">
+        <is>
+          <t>1cbaf7af-df8c-49b5-a02a-0b94c3695da5</t>
+        </is>
+      </c>
+      <c r="AW62" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MCK-1793215836074</t>
+        </is>
+      </c>
+      <c r="AX62" s="13" t="n">
+        <v>46323.81291666667</v>
+      </c>
+      <c r="AY62" s="13" t="n">
+        <v>46323.81292824074</v>
+      </c>
+      <c r="AZ62" s="13" t="n"/>
+      <c r="BA62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="13" t="n">
+        <v>46323.8546412037</v>
+      </c>
+      <c r="C63" s="13" t="n">
+        <v>46323.64630787037</v>
+      </c>
+      <c r="D63" s="13" t="n">
+        <v>46323.81297453704</v>
+      </c>
+      <c r="E63" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="n"/>
+      <c r="H63" s="6" t="n"/>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J63" s="16" t="n">
+        <v>184.54038504</v>
+      </c>
+      <c r="K63" s="17" t="n">
+        <v>45.67</v>
+      </c>
+      <c r="L63" s="17">
+        <f>IF(AND(ISNUMBER(J63),ISNUMBER(K63)),J63*K63,"")</f>
+        <v/>
+      </c>
+      <c r="M63" s="17" t="n"/>
+      <c r="N63" s="16" t="n">
+        <v>184.54038504</v>
+      </c>
+      <c r="O63" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P63" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q63" s="12" t="n"/>
+      <c r="R63" s="6" t="n"/>
+      <c r="S63" s="18" t="n"/>
+      <c r="T63" s="12" t="n"/>
+      <c r="U63" s="19" t="n"/>
+      <c r="V63" s="19" t="n"/>
+      <c r="W63" s="12" t="n"/>
+      <c r="X63" s="6" t="n"/>
+      <c r="Y63" s="19" t="n"/>
+      <c r="Z63" s="6" t="n"/>
+      <c r="AA63" s="12" t="n"/>
+      <c r="AB63" s="15" t="n"/>
+      <c r="AC63" s="6" t="n"/>
+      <c r="AD63" s="6" t="n"/>
+      <c r="AE63" s="17" t="n"/>
+      <c r="AF63" s="17" t="n"/>
+      <c r="AG63" s="17" t="n"/>
+      <c r="AH63" s="20" t="n"/>
+      <c r="AI63" s="18" t="n"/>
+      <c r="AJ63" s="6" t="n"/>
+      <c r="AK63" s="12" t="n"/>
+      <c r="AL63" s="15" t="n"/>
+      <c r="AM63" s="17" t="n"/>
+      <c r="AN63" s="19" t="n"/>
+      <c r="AO63" s="17" t="n"/>
+      <c r="AP63" s="17" t="n"/>
+      <c r="AQ63" s="19" t="n"/>
+      <c r="AR63" s="16" t="n"/>
+      <c r="AS63" s="17" t="n"/>
+      <c r="AT63" s="19" t="n"/>
+      <c r="AU63" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV63" s="6" t="inlineStr">
+        <is>
+          <t>4738e0cb-2c25-4745-9f69-03c405f631f5</t>
+        </is>
+      </c>
+      <c r="AW63" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MNST-1793215837443</t>
+        </is>
+      </c>
+      <c r="AX63" s="13" t="n">
+        <v>46323.81292824074</v>
+      </c>
+      <c r="AY63" s="13" t="n">
+        <v>46323.81297453704</v>
+      </c>
+      <c r="AZ63" s="13" t="n"/>
+      <c r="BA63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="13" t="n">
+        <v>46323.85461805556</v>
+      </c>
+      <c r="C64" s="13" t="n">
+        <v>46323.64628472222</v>
+      </c>
+      <c r="D64" s="13" t="n">
+        <v>46323.81295138889</v>
+      </c>
+      <c r="E64" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="n"/>
+      <c r="H64" s="6" t="n"/>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J64" s="16" t="n">
+        <v>14.214489601</v>
+      </c>
+      <c r="K64" s="17" t="n">
+        <v>73.23</v>
+      </c>
+      <c r="L64" s="17">
+        <f>IF(AND(ISNUMBER(J64),ISNUMBER(K64)),J64*K64,"")</f>
+        <v/>
+      </c>
+      <c r="M64" s="17" t="n"/>
+      <c r="N64" s="16" t="n">
+        <v>14.214489601</v>
+      </c>
+      <c r="O64" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P64" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q64" s="12" t="n"/>
+      <c r="R64" s="6" t="n"/>
+      <c r="S64" s="18" t="n"/>
+      <c r="T64" s="12" t="n"/>
+      <c r="U64" s="19" t="n"/>
+      <c r="V64" s="19" t="n"/>
+      <c r="W64" s="12" t="n"/>
+      <c r="X64" s="6" t="n"/>
+      <c r="Y64" s="19" t="n"/>
+      <c r="Z64" s="6" t="n"/>
+      <c r="AA64" s="12" t="n"/>
+      <c r="AB64" s="15" t="n"/>
+      <c r="AC64" s="6" t="n"/>
+      <c r="AD64" s="6" t="n"/>
+      <c r="AE64" s="17" t="n"/>
+      <c r="AF64" s="17" t="n"/>
+      <c r="AG64" s="17" t="n"/>
+      <c r="AH64" s="20" t="n"/>
+      <c r="AI64" s="18" t="n"/>
+      <c r="AJ64" s="6" t="n"/>
+      <c r="AK64" s="12" t="n"/>
+      <c r="AL64" s="15" t="n"/>
+      <c r="AM64" s="17" t="n"/>
+      <c r="AN64" s="19" t="n"/>
+      <c r="AO64" s="17" t="n"/>
+      <c r="AP64" s="17" t="n"/>
+      <c r="AQ64" s="19" t="n"/>
+      <c r="AR64" s="16" t="n"/>
+      <c r="AS64" s="17" t="n"/>
+      <c r="AT64" s="19" t="n"/>
+      <c r="AU64" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV64" s="6" t="inlineStr">
+        <is>
+          <t>c3ad0775-b864-4e0e-a442-53a048adc811</t>
+        </is>
+      </c>
+      <c r="AW64" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MO-1793215838801</t>
+        </is>
+      </c>
+      <c r="AX64" s="13" t="n">
+        <v>46323.81293981482</v>
+      </c>
+      <c r="AY64" s="13" t="n">
+        <v>46323.81295138889</v>
+      </c>
+      <c r="AZ64" s="13" t="n"/>
+      <c r="BA64" s="6" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="13" t="n">
+        <v>46323.85462962963</v>
+      </c>
+      <c r="C65" s="13" t="n">
+        <v>46323.6462962963</v>
+      </c>
+      <c r="D65" s="13" t="n">
+        <v>46323.81296296296</v>
+      </c>
+      <c r="E65" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="n"/>
+      <c r="H65" s="6" t="n"/>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J65" s="16" t="n">
+        <v>0.19946772</v>
+      </c>
+      <c r="K65" s="17" t="n">
+        <v>442.04</v>
+      </c>
+      <c r="L65" s="17">
+        <f>IF(AND(ISNUMBER(J65),ISNUMBER(K65)),J65*K65,"")</f>
+        <v/>
+      </c>
+      <c r="M65" s="17" t="n"/>
+      <c r="N65" s="16" t="n">
+        <v>0.19946772</v>
+      </c>
+      <c r="O65" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P65" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q65" s="12" t="n"/>
+      <c r="R65" s="6" t="n"/>
+      <c r="S65" s="18" t="n"/>
+      <c r="T65" s="12" t="n"/>
+      <c r="U65" s="19" t="n"/>
+      <c r="V65" s="19" t="n"/>
+      <c r="W65" s="12" t="n"/>
+      <c r="X65" s="6" t="n"/>
+      <c r="Y65" s="19" t="n"/>
+      <c r="Z65" s="6" t="n"/>
+      <c r="AA65" s="12" t="n"/>
+      <c r="AB65" s="15" t="n"/>
+      <c r="AC65" s="6" t="n"/>
+      <c r="AD65" s="6" t="n"/>
+      <c r="AE65" s="17" t="n"/>
+      <c r="AF65" s="17" t="n"/>
+      <c r="AG65" s="17" t="n"/>
+      <c r="AH65" s="20" t="n"/>
+      <c r="AI65" s="18" t="n"/>
+      <c r="AJ65" s="6" t="n"/>
+      <c r="AK65" s="12" t="n"/>
+      <c r="AL65" s="15" t="n"/>
+      <c r="AM65" s="17" t="n"/>
+      <c r="AN65" s="19" t="n"/>
+      <c r="AO65" s="17" t="n"/>
+      <c r="AP65" s="17" t="n"/>
+      <c r="AQ65" s="19" t="n"/>
+      <c r="AR65" s="16" t="n"/>
+      <c r="AS65" s="17" t="n"/>
+      <c r="AT65" s="19" t="n"/>
+      <c r="AU65" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV65" s="6" t="inlineStr">
+        <is>
+          <t>1f0db5c0-bbf7-4a79-adad-ddc5fe2a6212</t>
+        </is>
+      </c>
+      <c r="AW65" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MPC-1793215840170</t>
+        </is>
+      </c>
+      <c r="AX65" s="13" t="n">
+        <v>46323.81296296296</v>
+      </c>
+      <c r="AY65" s="13" t="n">
+        <v>46323.81296296296</v>
+      </c>
+      <c r="AZ65" s="13" t="n"/>
+      <c r="BA65" s="6" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="13" t="n">
+        <v>46323.85466435185</v>
+      </c>
+      <c r="C66" s="13" t="n">
+        <v>46323.64633101852</v>
+      </c>
+      <c r="D66" s="13" t="n">
+        <v>46323.81299768519</v>
+      </c>
+      <c r="E66" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="G66" s="15" t="n"/>
+      <c r="H66" s="6" t="n"/>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J66" s="16" t="n">
+        <v>2.434491107</v>
+      </c>
+      <c r="K66" s="17" t="n">
+        <v>427.12</v>
+      </c>
+      <c r="L66" s="17">
+        <f>IF(AND(ISNUMBER(J66),ISNUMBER(K66)),J66*K66,"")</f>
+        <v/>
+      </c>
+      <c r="M66" s="17" t="n"/>
+      <c r="N66" s="16" t="n">
+        <v>2.434491107</v>
+      </c>
+      <c r="O66" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P66" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q66" s="12" t="n"/>
+      <c r="R66" s="6" t="n"/>
+      <c r="S66" s="18" t="n"/>
+      <c r="T66" s="12" t="n"/>
+      <c r="U66" s="19" t="n"/>
+      <c r="V66" s="19" t="n"/>
+      <c r="W66" s="12" t="n"/>
+      <c r="X66" s="6" t="n"/>
+      <c r="Y66" s="19" t="n"/>
+      <c r="Z66" s="6" t="n"/>
+      <c r="AA66" s="12" t="n"/>
+      <c r="AB66" s="15" t="n"/>
+      <c r="AC66" s="6" t="n"/>
+      <c r="AD66" s="6" t="n"/>
+      <c r="AE66" s="17" t="n"/>
+      <c r="AF66" s="17" t="n"/>
+      <c r="AG66" s="17" t="n"/>
+      <c r="AH66" s="20" t="n"/>
+      <c r="AI66" s="18" t="n"/>
+      <c r="AJ66" s="6" t="n"/>
+      <c r="AK66" s="12" t="n"/>
+      <c r="AL66" s="15" t="n"/>
+      <c r="AM66" s="17" t="n"/>
+      <c r="AN66" s="19" t="n"/>
+      <c r="AO66" s="17" t="n"/>
+      <c r="AP66" s="17" t="n"/>
+      <c r="AQ66" s="19" t="n"/>
+      <c r="AR66" s="16" t="n"/>
+      <c r="AS66" s="17" t="n"/>
+      <c r="AT66" s="19" t="n"/>
+      <c r="AU66" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV66" s="6" t="inlineStr">
+        <is>
+          <t>296a097e-6f40-4873-b358-c3ec6cb2e91d</t>
+        </is>
+      </c>
+      <c r="AW66" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-NTRA-1793215841512</t>
+        </is>
+      </c>
+      <c r="AX66" s="13" t="n">
+        <v>46323.81297453704</v>
+      </c>
+      <c r="AY66" s="13" t="n">
+        <v>46323.81299768519</v>
+      </c>
+      <c r="AZ66" s="13" t="n"/>
+      <c r="BA66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="13" t="n">
+        <v>46323.85467592593</v>
+      </c>
+      <c r="C67" s="13" t="n">
+        <v>46323.64634259259</v>
+      </c>
+      <c r="D67" s="13" t="n">
+        <v>46323.81300925926</v>
+      </c>
+      <c r="E67" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="G67" s="15" t="n"/>
+      <c r="H67" s="6" t="n"/>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J67" s="16" t="n">
+        <v>132.295201779</v>
+      </c>
+      <c r="K67" s="17" t="n">
+        <v>63.186349</v>
+      </c>
+      <c r="L67" s="17">
+        <f>IF(AND(ISNUMBER(J67),ISNUMBER(K67)),J67*K67,"")</f>
+        <v/>
+      </c>
+      <c r="M67" s="17" t="n"/>
+      <c r="N67" s="16" t="n">
+        <v>132.295201779</v>
+      </c>
+      <c r="O67" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P67" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q67" s="12" t="n"/>
+      <c r="R67" s="6" t="n"/>
+      <c r="S67" s="18" t="n"/>
+      <c r="T67" s="12" t="n"/>
+      <c r="U67" s="19" t="n"/>
+      <c r="V67" s="19" t="n"/>
+      <c r="W67" s="12" t="n"/>
+      <c r="X67" s="6" t="n"/>
+      <c r="Y67" s="19" t="n"/>
+      <c r="Z67" s="6" t="n"/>
+      <c r="AA67" s="12" t="n"/>
+      <c r="AB67" s="15" t="n"/>
+      <c r="AC67" s="6" t="n"/>
+      <c r="AD67" s="6" t="n"/>
+      <c r="AE67" s="17" t="n"/>
+      <c r="AF67" s="17" t="n"/>
+      <c r="AG67" s="17" t="n"/>
+      <c r="AH67" s="20" t="n"/>
+      <c r="AI67" s="18" t="n"/>
+      <c r="AJ67" s="6" t="n"/>
+      <c r="AK67" s="12" t="n"/>
+      <c r="AL67" s="15" t="n"/>
+      <c r="AM67" s="17" t="n"/>
+      <c r="AN67" s="19" t="n"/>
+      <c r="AO67" s="17" t="n"/>
+      <c r="AP67" s="17" t="n"/>
+      <c r="AQ67" s="19" t="n"/>
+      <c r="AR67" s="16" t="n"/>
+      <c r="AS67" s="17" t="n"/>
+      <c r="AT67" s="19" t="n"/>
+      <c r="AU67" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV67" s="6" t="inlineStr">
+        <is>
+          <t>e7f04beb-2d54-4819-b1af-8900d56301f5</t>
+        </is>
+      </c>
+      <c r="AW67" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-OXY-1793215842873</t>
+        </is>
+      </c>
+      <c r="AX67" s="13" t="n">
+        <v>46323.81299768519</v>
+      </c>
+      <c r="AY67" s="13" t="n">
+        <v>46323.81300925926</v>
+      </c>
+      <c r="AZ67" s="13" t="n"/>
+      <c r="BA67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="13" t="n">
+        <v>46323.85472222222</v>
+      </c>
+      <c r="C68" s="13" t="n">
+        <v>46323.64638888889</v>
+      </c>
+      <c r="D68" s="13" t="n">
+        <v>46323.81305555555</v>
+      </c>
+      <c r="E68" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>PBR.A</t>
+        </is>
+      </c>
+      <c r="G68" s="15" t="n"/>
+      <c r="H68" s="6" t="n"/>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J68" s="16" t="n">
+        <v>211.579533941</v>
+      </c>
+      <c r="K68" s="17" t="n">
+        <v>19.779925</v>
+      </c>
+      <c r="L68" s="17">
+        <f>IF(AND(ISNUMBER(J68),ISNUMBER(K68)),J68*K68,"")</f>
+        <v/>
+      </c>
+      <c r="M68" s="17" t="n"/>
+      <c r="N68" s="16" t="n">
+        <v>211.579533941</v>
+      </c>
+      <c r="O68" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P68" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q68" s="12" t="n"/>
+      <c r="R68" s="6" t="n"/>
+      <c r="S68" s="18" t="n"/>
+      <c r="T68" s="12" t="n"/>
+      <c r="U68" s="19" t="n"/>
+      <c r="V68" s="19" t="n"/>
+      <c r="W68" s="12" t="n"/>
+      <c r="X68" s="6" t="n"/>
+      <c r="Y68" s="19" t="n"/>
+      <c r="Z68" s="6" t="n"/>
+      <c r="AA68" s="12" t="n"/>
+      <c r="AB68" s="15" t="n"/>
+      <c r="AC68" s="6" t="n"/>
+      <c r="AD68" s="6" t="n"/>
+      <c r="AE68" s="17" t="n"/>
+      <c r="AF68" s="17" t="n"/>
+      <c r="AG68" s="17" t="n"/>
+      <c r="AH68" s="20" t="n"/>
+      <c r="AI68" s="18" t="n"/>
+      <c r="AJ68" s="6" t="n"/>
+      <c r="AK68" s="12" t="n"/>
+      <c r="AL68" s="15" t="n"/>
+      <c r="AM68" s="17" t="n"/>
+      <c r="AN68" s="19" t="n"/>
+      <c r="AO68" s="17" t="n"/>
+      <c r="AP68" s="17" t="n"/>
+      <c r="AQ68" s="19" t="n"/>
+      <c r="AR68" s="16" t="n"/>
+      <c r="AS68" s="17" t="n"/>
+      <c r="AT68" s="19" t="n"/>
+      <c r="AU68" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV68" s="6" t="inlineStr">
+        <is>
+          <t>59c7a439-754b-4dab-ac2c-45cf18aea1e0</t>
+        </is>
+      </c>
+      <c r="AW68" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-PBR.A-1793215844413</t>
+        </is>
+      </c>
+      <c r="AX68" s="13" t="n">
+        <v>46323.81300925926</v>
+      </c>
+      <c r="AY68" s="13" t="n">
+        <v>46323.81305555555</v>
+      </c>
+      <c r="AZ68" s="13" t="n"/>
+      <c r="BA68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="13" t="n">
+        <v>46323.8546875</v>
+      </c>
+      <c r="C69" s="13" t="n">
+        <v>46323.64635416667</v>
+      </c>
+      <c r="D69" s="13" t="n">
+        <v>46323.81302083333</v>
+      </c>
+      <c r="E69" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>PSX</t>
+        </is>
+      </c>
+      <c r="G69" s="15" t="n"/>
+      <c r="H69" s="6" t="n"/>
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J69" s="16" t="n">
+        <v>0.323158986</v>
+      </c>
+      <c r="K69" s="17" t="n">
+        <v>273.476</v>
+      </c>
+      <c r="L69" s="17">
+        <f>IF(AND(ISNUMBER(J69),ISNUMBER(K69)),J69*K69,"")</f>
+        <v/>
+      </c>
+      <c r="M69" s="17" t="n"/>
+      <c r="N69" s="16" t="n">
+        <v>0.323158986</v>
+      </c>
+      <c r="O69" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P69" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q69" s="12" t="n"/>
+      <c r="R69" s="6" t="n"/>
+      <c r="S69" s="18" t="n"/>
+      <c r="T69" s="12" t="n"/>
+      <c r="U69" s="19" t="n"/>
+      <c r="V69" s="19" t="n"/>
+      <c r="W69" s="12" t="n"/>
+      <c r="X69" s="6" t="n"/>
+      <c r="Y69" s="19" t="n"/>
+      <c r="Z69" s="6" t="n"/>
+      <c r="AA69" s="12" t="n"/>
+      <c r="AB69" s="15" t="n"/>
+      <c r="AC69" s="6" t="n"/>
+      <c r="AD69" s="6" t="n"/>
+      <c r="AE69" s="17" t="n"/>
+      <c r="AF69" s="17" t="n"/>
+      <c r="AG69" s="17" t="n"/>
+      <c r="AH69" s="20" t="n"/>
+      <c r="AI69" s="18" t="n"/>
+      <c r="AJ69" s="6" t="n"/>
+      <c r="AK69" s="12" t="n"/>
+      <c r="AL69" s="15" t="n"/>
+      <c r="AM69" s="17" t="n"/>
+      <c r="AN69" s="19" t="n"/>
+      <c r="AO69" s="17" t="n"/>
+      <c r="AP69" s="17" t="n"/>
+      <c r="AQ69" s="19" t="n"/>
+      <c r="AR69" s="16" t="n"/>
+      <c r="AS69" s="17" t="n"/>
+      <c r="AT69" s="19" t="n"/>
+      <c r="AU69" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV69" s="6" t="inlineStr">
+        <is>
+          <t>9d75ff07-7e08-4f59-be02-9900eaae6063</t>
+        </is>
+      </c>
+      <c r="AW69" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-PSX-1793215845765</t>
+        </is>
+      </c>
+      <c r="AX69" s="13" t="n">
+        <v>46323.81302083333</v>
+      </c>
+      <c r="AY69" s="13" t="n">
+        <v>46323.81302083333</v>
+      </c>
+      <c r="AZ69" s="13" t="n"/>
+      <c r="BA69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="13" t="n">
+        <v>46323.85471064815</v>
+      </c>
+      <c r="C70" s="13" t="n">
+        <v>46323.64637731481</v>
+      </c>
+      <c r="D70" s="13" t="n">
+        <v>46323.81304398148</v>
+      </c>
+      <c r="E70" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="n"/>
+      <c r="H70" s="6" t="n"/>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J70" s="16" t="n">
+        <v>0.083680668</v>
+      </c>
+      <c r="K70" s="17" t="n">
+        <v>810.48</v>
+      </c>
+      <c r="L70" s="17">
+        <f>IF(AND(ISNUMBER(J70),ISNUMBER(K70)),J70*K70,"")</f>
+        <v/>
+      </c>
+      <c r="M70" s="17" t="n"/>
+      <c r="N70" s="16" t="n">
+        <v>0.083680668</v>
+      </c>
+      <c r="O70" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P70" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q70" s="12" t="n"/>
+      <c r="R70" s="6" t="n"/>
+      <c r="S70" s="18" t="n"/>
+      <c r="T70" s="12" t="n"/>
+      <c r="U70" s="19" t="n"/>
+      <c r="V70" s="19" t="n"/>
+      <c r="W70" s="12" t="n"/>
+      <c r="X70" s="6" t="n"/>
+      <c r="Y70" s="19" t="n"/>
+      <c r="Z70" s="6" t="n"/>
+      <c r="AA70" s="12" t="n"/>
+      <c r="AB70" s="15" t="n"/>
+      <c r="AC70" s="6" t="n"/>
+      <c r="AD70" s="6" t="n"/>
+      <c r="AE70" s="17" t="n"/>
+      <c r="AF70" s="17" t="n"/>
+      <c r="AG70" s="17" t="n"/>
+      <c r="AH70" s="20" t="n"/>
+      <c r="AI70" s="18" t="n"/>
+      <c r="AJ70" s="6" t="n"/>
+      <c r="AK70" s="12" t="n"/>
+      <c r="AL70" s="15" t="n"/>
+      <c r="AM70" s="17" t="n"/>
+      <c r="AN70" s="19" t="n"/>
+      <c r="AO70" s="17" t="n"/>
+      <c r="AP70" s="17" t="n"/>
+      <c r="AQ70" s="19" t="n"/>
+      <c r="AR70" s="16" t="n"/>
+      <c r="AS70" s="17" t="n"/>
+      <c r="AT70" s="19" t="n"/>
+      <c r="AU70" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV70" s="6" t="inlineStr">
+        <is>
+          <t>f7ccdc37-ea56-4dcf-b793-2e2d754c5388</t>
+        </is>
+      </c>
+      <c r="AW70" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-REGN-1793215847104</t>
+        </is>
+      </c>
+      <c r="AX70" s="13" t="n">
+        <v>46323.81304398148</v>
+      </c>
+      <c r="AY70" s="13" t="n">
+        <v>46323.81304398148</v>
+      </c>
+      <c r="AZ70" s="13" t="n"/>
+      <c r="BA70" s="6" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="13" t="n">
+        <v>46323.85476851852</v>
+      </c>
+      <c r="C71" s="13" t="n">
+        <v>46323.64643518518</v>
+      </c>
+      <c r="D71" s="13" t="n">
+        <v>46323.81310185185</v>
+      </c>
+      <c r="E71" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="G71" s="15" t="n"/>
+      <c r="H71" s="6" t="n"/>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J71" s="16" t="n">
+        <v>79.375047619</v>
+      </c>
+      <c r="K71" s="17" t="n">
+        <v>105.486426</v>
+      </c>
+      <c r="L71" s="17">
+        <f>IF(AND(ISNUMBER(J71),ISNUMBER(K71)),J71*K71,"")</f>
+        <v/>
+      </c>
+      <c r="M71" s="17" t="n"/>
+      <c r="N71" s="16" t="n">
+        <v>79.375047619</v>
+      </c>
+      <c r="O71" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P71" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q71" s="12" t="n"/>
+      <c r="R71" s="6" t="n"/>
+      <c r="S71" s="18" t="n"/>
+      <c r="T71" s="12" t="n"/>
+      <c r="U71" s="19" t="n"/>
+      <c r="V71" s="19" t="n"/>
+      <c r="W71" s="12" t="n"/>
+      <c r="X71" s="6" t="n"/>
+      <c r="Y71" s="19" t="n"/>
+      <c r="Z71" s="6" t="n"/>
+      <c r="AA71" s="12" t="n"/>
+      <c r="AB71" s="15" t="n"/>
+      <c r="AC71" s="6" t="n"/>
+      <c r="AD71" s="6" t="n"/>
+      <c r="AE71" s="17" t="n"/>
+      <c r="AF71" s="17" t="n"/>
+      <c r="AG71" s="17" t="n"/>
+      <c r="AH71" s="20" t="n"/>
+      <c r="AI71" s="18" t="n"/>
+      <c r="AJ71" s="6" t="n"/>
+      <c r="AK71" s="12" t="n"/>
+      <c r="AL71" s="15" t="n"/>
+      <c r="AM71" s="17" t="n"/>
+      <c r="AN71" s="19" t="n"/>
+      <c r="AO71" s="17" t="n"/>
+      <c r="AP71" s="17" t="n"/>
+      <c r="AQ71" s="19" t="n"/>
+      <c r="AR71" s="16" t="n"/>
+      <c r="AS71" s="17" t="n"/>
+      <c r="AT71" s="19" t="n"/>
+      <c r="AU71" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV71" s="6" t="inlineStr">
+        <is>
+          <t>4f273e09-685f-45ff-8b93-5289151b596c</t>
+        </is>
+      </c>
+      <c r="AW71" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-SHEL-1793215848475</t>
+        </is>
+      </c>
+      <c r="AX71" s="13" t="n">
+        <v>46323.81305555555</v>
+      </c>
+      <c r="AY71" s="13" t="n">
+        <v>46323.81310185185</v>
+      </c>
+      <c r="AZ71" s="13" t="n"/>
+      <c r="BA71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="13" t="n">
+        <v>46323.85474537037</v>
+      </c>
+      <c r="C72" s="13" t="n">
+        <v>46323.64641203704</v>
+      </c>
+      <c r="D72" s="13" t="n">
+        <v>46323.8130787037</v>
+      </c>
+      <c r="E72" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="n"/>
+      <c r="H72" s="6" t="n"/>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J72" s="16" t="n">
+        <v>1.348382763</v>
+      </c>
+      <c r="K72" s="17" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="L72" s="17">
+        <f>IF(AND(ISNUMBER(J72),ISNUMBER(K72)),J72*K72,"")</f>
+        <v/>
+      </c>
+      <c r="M72" s="17" t="n"/>
+      <c r="N72" s="16" t="n">
+        <v>1.348382763</v>
+      </c>
+      <c r="O72" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P72" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q72" s="12" t="n"/>
+      <c r="R72" s="6" t="n"/>
+      <c r="S72" s="18" t="n"/>
+      <c r="T72" s="12" t="n"/>
+      <c r="U72" s="19" t="n"/>
+      <c r="V72" s="19" t="n"/>
+      <c r="W72" s="12" t="n"/>
+      <c r="X72" s="6" t="n"/>
+      <c r="Y72" s="19" t="n"/>
+      <c r="Z72" s="6" t="n"/>
+      <c r="AA72" s="12" t="n"/>
+      <c r="AB72" s="15" t="n"/>
+      <c r="AC72" s="6" t="n"/>
+      <c r="AD72" s="6" t="n"/>
+      <c r="AE72" s="17" t="n"/>
+      <c r="AF72" s="17" t="n"/>
+      <c r="AG72" s="17" t="n"/>
+      <c r="AH72" s="20" t="n"/>
+      <c r="AI72" s="18" t="n"/>
+      <c r="AJ72" s="6" t="n"/>
+      <c r="AK72" s="12" t="n"/>
+      <c r="AL72" s="15" t="n"/>
+      <c r="AM72" s="17" t="n"/>
+      <c r="AN72" s="19" t="n"/>
+      <c r="AO72" s="17" t="n"/>
+      <c r="AP72" s="17" t="n"/>
+      <c r="AQ72" s="19" t="n"/>
+      <c r="AR72" s="16" t="n"/>
+      <c r="AS72" s="17" t="n"/>
+      <c r="AT72" s="19" t="n"/>
+      <c r="AU72" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV72" s="6" t="inlineStr">
+        <is>
+          <t>e928c244-9f2a-49be-9037-96375011a7e7</t>
+        </is>
+      </c>
+      <c r="AW72" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-SO-1793215849828</t>
+        </is>
+      </c>
+      <c r="AX72" s="13" t="n">
+        <v>46323.81306712963</v>
+      </c>
+      <c r="AY72" s="13" t="n">
+        <v>46323.8130787037</v>
+      </c>
+      <c r="AZ72" s="13" t="n"/>
+      <c r="BA72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="13" t="n">
+        <v>46323.85476851852</v>
+      </c>
+      <c r="C73" s="13" t="n">
+        <v>46323.64643518518</v>
+      </c>
+      <c r="D73" s="13" t="n">
+        <v>46323.81310185185</v>
+      </c>
+      <c r="E73" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="G73" s="15" t="n"/>
+      <c r="H73" s="6" t="n"/>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J73" s="16" t="n">
+        <v>11.937064238</v>
+      </c>
+      <c r="K73" s="17" t="n">
+        <v>705.6</v>
+      </c>
+      <c r="L73" s="17">
+        <f>IF(AND(ISNUMBER(J73),ISNUMBER(K73)),J73*K73,"")</f>
+        <v/>
+      </c>
+      <c r="M73" s="17" t="n"/>
+      <c r="N73" s="16" t="n">
+        <v>11.937064238</v>
+      </c>
+      <c r="O73" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P73" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q73" s="12" t="n"/>
+      <c r="R73" s="6" t="n"/>
+      <c r="S73" s="18" t="n"/>
+      <c r="T73" s="12" t="n"/>
+      <c r="U73" s="19" t="n"/>
+      <c r="V73" s="19" t="n"/>
+      <c r="W73" s="12" t="n"/>
+      <c r="X73" s="6" t="n"/>
+      <c r="Y73" s="19" t="n"/>
+      <c r="Z73" s="6" t="n"/>
+      <c r="AA73" s="12" t="n"/>
+      <c r="AB73" s="15" t="n"/>
+      <c r="AC73" s="6" t="n"/>
+      <c r="AD73" s="6" t="n"/>
+      <c r="AE73" s="17" t="n"/>
+      <c r="AF73" s="17" t="n"/>
+      <c r="AG73" s="17" t="n"/>
+      <c r="AH73" s="20" t="n"/>
+      <c r="AI73" s="18" t="n"/>
+      <c r="AJ73" s="6" t="n"/>
+      <c r="AK73" s="12" t="n"/>
+      <c r="AL73" s="15" t="n"/>
+      <c r="AM73" s="17" t="n"/>
+      <c r="AN73" s="19" t="n"/>
+      <c r="AO73" s="17" t="n"/>
+      <c r="AP73" s="17" t="n"/>
+      <c r="AQ73" s="19" t="n"/>
+      <c r="AR73" s="16" t="n"/>
+      <c r="AS73" s="17" t="n"/>
+      <c r="AT73" s="19" t="n"/>
+      <c r="AU73" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV73" s="6" t="inlineStr">
+        <is>
+          <t>d0b9b04c-efbc-45ee-a684-634fe792ccb0</t>
+        </is>
+      </c>
+      <c r="AW73" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-TMO-1793215851174</t>
+        </is>
+      </c>
+      <c r="AX73" s="13" t="n">
+        <v>46323.81309027778</v>
+      </c>
+      <c r="AY73" s="13" t="n">
+        <v>46323.81310185185</v>
+      </c>
+      <c r="AZ73" s="13" t="n"/>
+      <c r="BA73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="13" t="n">
+        <v>46323.8547800926</v>
+      </c>
+      <c r="C74" s="13" t="n">
+        <v>46323.64644675926</v>
+      </c>
+      <c r="D74" s="13" t="n">
+        <v>46323.81311342592</v>
+      </c>
+      <c r="E74" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+      <c r="G74" s="15" t="n"/>
+      <c r="H74" s="6" t="n"/>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J74" s="16" t="n">
+        <v>7.111731176</v>
+      </c>
+      <c r="K74" s="17" t="n">
+        <v>584.76</v>
+      </c>
+      <c r="L74" s="17">
+        <f>IF(AND(ISNUMBER(J74),ISNUMBER(K74)),J74*K74,"")</f>
+        <v/>
+      </c>
+      <c r="M74" s="17" t="n"/>
+      <c r="N74" s="16" t="n">
+        <v>7.111731176</v>
+      </c>
+      <c r="O74" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P74" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q74" s="12" t="n"/>
+      <c r="R74" s="6" t="n"/>
+      <c r="S74" s="18" t="n"/>
+      <c r="T74" s="12" t="n"/>
+      <c r="U74" s="19" t="n"/>
+      <c r="V74" s="19" t="n"/>
+      <c r="W74" s="12" t="n"/>
+      <c r="X74" s="6" t="n"/>
+      <c r="Y74" s="19" t="n"/>
+      <c r="Z74" s="6" t="n"/>
+      <c r="AA74" s="12" t="n"/>
+      <c r="AB74" s="15" t="n"/>
+      <c r="AC74" s="6" t="n"/>
+      <c r="AD74" s="6" t="n"/>
+      <c r="AE74" s="17" t="n"/>
+      <c r="AF74" s="17" t="n"/>
+      <c r="AG74" s="17" t="n"/>
+      <c r="AH74" s="20" t="n"/>
+      <c r="AI74" s="18" t="n"/>
+      <c r="AJ74" s="6" t="n"/>
+      <c r="AK74" s="12" t="n"/>
+      <c r="AL74" s="15" t="n"/>
+      <c r="AM74" s="17" t="n"/>
+      <c r="AN74" s="19" t="n"/>
+      <c r="AO74" s="17" t="n"/>
+      <c r="AP74" s="17" t="n"/>
+      <c r="AQ74" s="19" t="n"/>
+      <c r="AR74" s="16" t="n"/>
+      <c r="AS74" s="17" t="n"/>
+      <c r="AT74" s="19" t="n"/>
+      <c r="AU74" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV74" s="6" t="inlineStr">
+        <is>
+          <t>8b0a7b04-ea32-44e6-b0fb-6e7acef961bf</t>
+        </is>
+      </c>
+      <c r="AW74" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-UTHR-1793215852531</t>
+        </is>
+      </c>
+      <c r="AX74" s="13" t="n">
+        <v>46323.81310185185</v>
+      </c>
+      <c r="AY74" s="13" t="n">
+        <v>46323.81311342592</v>
+      </c>
+      <c r="AZ74" s="13" t="n"/>
+      <c r="BA74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="13" t="n">
+        <v>46323.85480324074</v>
+      </c>
+      <c r="C75" s="13" t="n">
+        <v>46323.64646990741</v>
+      </c>
+      <c r="D75" s="13" t="n">
+        <v>46323.81313657408</v>
+      </c>
+      <c r="E75" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="G75" s="15" t="n"/>
+      <c r="H75" s="6" t="n"/>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J75" s="16" t="n">
+        <v>3.263614517</v>
+      </c>
+      <c r="K75" s="17" t="n">
+        <v>321.15</v>
+      </c>
+      <c r="L75" s="17">
+        <f>IF(AND(ISNUMBER(J75),ISNUMBER(K75)),J75*K75,"")</f>
+        <v/>
+      </c>
+      <c r="M75" s="17" t="n"/>
+      <c r="N75" s="16" t="n">
+        <v>3.263614517</v>
+      </c>
+      <c r="O75" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P75" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q75" s="12" t="n"/>
+      <c r="R75" s="6" t="n"/>
+      <c r="S75" s="18" t="n"/>
+      <c r="T75" s="12" t="n"/>
+      <c r="U75" s="19" t="n"/>
+      <c r="V75" s="19" t="n"/>
+      <c r="W75" s="12" t="n"/>
+      <c r="X75" s="6" t="n"/>
+      <c r="Y75" s="19" t="n"/>
+      <c r="Z75" s="6" t="n"/>
+      <c r="AA75" s="12" t="n"/>
+      <c r="AB75" s="15" t="n"/>
+      <c r="AC75" s="6" t="n"/>
+      <c r="AD75" s="6" t="n"/>
+      <c r="AE75" s="17" t="n"/>
+      <c r="AF75" s="17" t="n"/>
+      <c r="AG75" s="17" t="n"/>
+      <c r="AH75" s="20" t="n"/>
+      <c r="AI75" s="18" t="n"/>
+      <c r="AJ75" s="6" t="n"/>
+      <c r="AK75" s="12" t="n"/>
+      <c r="AL75" s="15" t="n"/>
+      <c r="AM75" s="17" t="n"/>
+      <c r="AN75" s="19" t="n"/>
+      <c r="AO75" s="17" t="n"/>
+      <c r="AP75" s="17" t="n"/>
+      <c r="AQ75" s="19" t="n"/>
+      <c r="AR75" s="16" t="n"/>
+      <c r="AS75" s="17" t="n"/>
+      <c r="AT75" s="19" t="n"/>
+      <c r="AU75" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV75" s="6" t="inlineStr">
+        <is>
+          <t>a1e562c0-783e-46a1-a0d1-7da042b5b3c8</t>
+        </is>
+      </c>
+      <c r="AW75" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-WTW-1793215853872</t>
+        </is>
+      </c>
+      <c r="AX75" s="13" t="n">
+        <v>46323.813125</v>
+      </c>
+      <c r="AY75" s="13" t="n">
+        <v>46323.81313657408</v>
+      </c>
+      <c r="AZ75" s="13" t="n"/>
+      <c r="BA75" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -9763,9 +12895,15 @@
         <f>E4*F4</f>
         <v/>
       </c>
-      <c r="H4" s="22" t="n"/>
-      <c r="I4" s="22" t="n"/>
-      <c r="J4" s="17" t="n"/>
+      <c r="H4" s="22" t="n">
+        <v>46323.85476851852</v>
+      </c>
+      <c r="I4" s="22" t="n">
+        <v>46323.64643518518</v>
+      </c>
+      <c r="J4" s="17" t="n">
+        <v>105.486426</v>
+      </c>
       <c r="K4" s="17">
         <f>IF(ISNUMBER(J4),J4*F4,"")</f>
         <v/>
@@ -9782,10 +12920,14 @@
         <f>IF(ISNUMBER(H4),H4-C4,"")</f>
         <v/>
       </c>
-      <c r="O4" s="6" t="n"/>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P4" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9879,9 +13021,15 @@
         <f>E6*F6</f>
         <v/>
       </c>
-      <c r="H6" s="22" t="n"/>
-      <c r="I6" s="22" t="n"/>
-      <c r="J6" s="17" t="n"/>
+      <c r="H6" s="22" t="n">
+        <v>46323.8547800926</v>
+      </c>
+      <c r="I6" s="22" t="n">
+        <v>46323.64644675926</v>
+      </c>
+      <c r="J6" s="17" t="n">
+        <v>584.76</v>
+      </c>
       <c r="K6" s="17">
         <f>IF(ISNUMBER(J6),J6*F6,"")</f>
         <v/>
@@ -9898,10 +13046,14 @@
         <f>IF(ISNUMBER(H6),H6-C6,"")</f>
         <v/>
       </c>
-      <c r="O6" s="6" t="n"/>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9932,9 +13084,15 @@
         <f>E7*F7</f>
         <v/>
       </c>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="17" t="n"/>
+      <c r="H7" s="22" t="n">
+        <v>46323.85449074074</v>
+      </c>
+      <c r="I7" s="22" t="n">
+        <v>46323.64615740741</v>
+      </c>
+      <c r="J7" s="17" t="n">
+        <v>288.51</v>
+      </c>
       <c r="K7" s="17">
         <f>IF(ISNUMBER(J7),J7*F7,"")</f>
         <v/>
@@ -9951,10 +13109,14 @@
         <f>IF(ISNUMBER(H7),H7-C7,"")</f>
         <v/>
       </c>
-      <c r="O7" s="6" t="n"/>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9985,9 +13147,15 @@
         <f>E8*F8</f>
         <v/>
       </c>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="22" t="n"/>
-      <c r="J8" s="17" t="n"/>
+      <c r="H8" s="22" t="n">
+        <v>46323.85445601852</v>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>46323.64612268518</v>
+      </c>
+      <c r="J8" s="17" t="n">
+        <v>117.477719</v>
+      </c>
       <c r="K8" s="17">
         <f>IF(ISNUMBER(J8),J8*F8,"")</f>
         <v/>
@@ -10004,10 +13172,14 @@
         <f>IF(ISNUMBER(H8),H8-C8,"")</f>
         <v/>
       </c>
-      <c r="O8" s="6" t="n"/>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10038,9 +13210,15 @@
         <f>E9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="22" t="n"/>
-      <c r="I9" s="22" t="n"/>
-      <c r="J9" s="17" t="n"/>
+      <c r="H9" s="22" t="n">
+        <v>46323.85445601852</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>46323.64612268518</v>
+      </c>
+      <c r="J9" s="17" t="n">
+        <v>62.591634</v>
+      </c>
       <c r="K9" s="17">
         <f>IF(ISNUMBER(J9),J9*F9,"")</f>
         <v/>
@@ -10057,10 +13235,14 @@
         <f>IF(ISNUMBER(H9),H9-C9,"")</f>
         <v/>
       </c>
-      <c r="O9" s="6" t="n"/>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10091,9 +13273,15 @@
         <f>E10*F10</f>
         <v/>
       </c>
-      <c r="H10" s="22" t="n"/>
-      <c r="I10" s="22" t="n"/>
-      <c r="J10" s="17" t="n"/>
+      <c r="H10" s="22" t="n">
+        <v>46323.85459490741</v>
+      </c>
+      <c r="I10" s="22" t="n">
+        <v>46323.64626157407</v>
+      </c>
+      <c r="J10" s="17" t="n">
+        <v>959.34</v>
+      </c>
       <c r="K10" s="17">
         <f>IF(ISNUMBER(J10),J10*F10,"")</f>
         <v/>
@@ -10110,10 +13298,14 @@
         <f>IF(ISNUMBER(H10),H10-C10,"")</f>
         <v/>
       </c>
-      <c r="O10" s="6" t="n"/>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10144,9 +13336,15 @@
         <f>E11*F11</f>
         <v/>
       </c>
-      <c r="H11" s="22" t="n"/>
-      <c r="I11" s="22" t="n"/>
-      <c r="J11" s="17" t="n"/>
+      <c r="H11" s="22" t="n">
+        <v>46323.85476851852</v>
+      </c>
+      <c r="I11" s="22" t="n">
+        <v>46323.64643518518</v>
+      </c>
+      <c r="J11" s="17" t="n">
+        <v>705.6</v>
+      </c>
       <c r="K11" s="17">
         <f>IF(ISNUMBER(J11),J11*F11,"")</f>
         <v/>
@@ -10163,10 +13361,14 @@
         <f>IF(ISNUMBER(H11),H11-C11,"")</f>
         <v/>
       </c>
-      <c r="O11" s="6" t="n"/>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10197,9 +13399,15 @@
         <f>E12*F12</f>
         <v/>
       </c>
-      <c r="H12" s="22" t="n"/>
-      <c r="I12" s="22" t="n"/>
-      <c r="J12" s="17" t="n"/>
+      <c r="H12" s="22" t="n">
+        <v>46323.85439814815</v>
+      </c>
+      <c r="I12" s="22" t="n">
+        <v>46323.64606481481</v>
+      </c>
+      <c r="J12" s="17" t="n">
+        <v>322.32659</v>
+      </c>
       <c r="K12" s="17">
         <f>IF(ISNUMBER(J12),J12*F12,"")</f>
         <v/>
@@ -10216,10 +13424,14 @@
         <f>IF(ISNUMBER(H12),H12-C12,"")</f>
         <v/>
       </c>
-      <c r="O12" s="6" t="n"/>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10250,9 +13462,15 @@
         <f>E13*F13</f>
         <v/>
       </c>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="22" t="n"/>
-      <c r="J13" s="17" t="n"/>
+      <c r="H13" s="22" t="n">
+        <v>46323.85467592593</v>
+      </c>
+      <c r="I13" s="22" t="n">
+        <v>46323.64634259259</v>
+      </c>
+      <c r="J13" s="17" t="n">
+        <v>63.186349</v>
+      </c>
       <c r="K13" s="17">
         <f>IF(ISNUMBER(J13),J13*F13,"")</f>
         <v/>
@@ -10269,10 +13487,14 @@
         <f>IF(ISNUMBER(H13),H13-C13,"")</f>
         <v/>
       </c>
-      <c r="O13" s="6" t="n"/>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10366,9 +13588,15 @@
         <f>E15*F15</f>
         <v/>
       </c>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="22" t="n"/>
-      <c r="J15" s="17" t="n"/>
+      <c r="H15" s="22" t="n">
+        <v>46323.85454861111</v>
+      </c>
+      <c r="I15" s="22" t="n">
+        <v>46323.64621527777</v>
+      </c>
+      <c r="J15" s="17" t="n">
+        <v>276.99</v>
+      </c>
       <c r="K15" s="17">
         <f>IF(ISNUMBER(J15),J15*F15,"")</f>
         <v/>
@@ -10385,10 +13613,14 @@
         <f>IF(ISNUMBER(H15),H15-C15,"")</f>
         <v/>
       </c>
-      <c r="O15" s="6" t="n"/>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10419,9 +13651,15 @@
         <f>E16*F16</f>
         <v/>
       </c>
-      <c r="H16" s="22" t="n"/>
-      <c r="I16" s="22" t="n"/>
-      <c r="J16" s="17" t="n"/>
+      <c r="H16" s="22" t="n">
+        <v>46323.8546412037</v>
+      </c>
+      <c r="I16" s="22" t="n">
+        <v>46323.64630787037</v>
+      </c>
+      <c r="J16" s="17" t="n">
+        <v>45.67</v>
+      </c>
       <c r="K16" s="17">
         <f>IF(ISNUMBER(J16),J16*F16,"")</f>
         <v/>
@@ -10438,10 +13676,14 @@
         <f>IF(ISNUMBER(H16),H16-C16,"")</f>
         <v/>
       </c>
-      <c r="O16" s="6" t="n"/>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10535,9 +13777,15 @@
         <f>E18*F18</f>
         <v/>
       </c>
-      <c r="H18" s="22" t="n"/>
-      <c r="I18" s="22" t="n"/>
-      <c r="J18" s="17" t="n"/>
+      <c r="H18" s="22" t="n">
+        <v>46323.85472222222</v>
+      </c>
+      <c r="I18" s="22" t="n">
+        <v>46323.64638888889</v>
+      </c>
+      <c r="J18" s="17" t="n">
+        <v>19.779925</v>
+      </c>
       <c r="K18" s="17">
         <f>IF(ISNUMBER(J18),J18*F18,"")</f>
         <v/>
@@ -10554,10 +13802,14 @@
         <f>IF(ISNUMBER(H18),H18-C18,"")</f>
         <v/>
       </c>
-      <c r="O18" s="6" t="n"/>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10588,9 +13840,15 @@
         <f>E19*F19</f>
         <v/>
       </c>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="22" t="n"/>
-      <c r="J19" s="17" t="n"/>
+      <c r="H19" s="22" t="n">
+        <v>46323.85457175926</v>
+      </c>
+      <c r="I19" s="22" t="n">
+        <v>46323.64623842593</v>
+      </c>
+      <c r="J19" s="17" t="n">
+        <v>297.565854</v>
+      </c>
       <c r="K19" s="17">
         <f>IF(ISNUMBER(J19),J19*F19,"")</f>
         <v/>
@@ -10607,10 +13865,14 @@
         <f>IF(ISNUMBER(H19),H19-C19,"")</f>
         <v/>
       </c>
-      <c r="O19" s="6" t="n"/>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10641,9 +13903,15 @@
         <f>E20*F20</f>
         <v/>
       </c>
-      <c r="H20" s="22" t="n"/>
-      <c r="I20" s="22" t="n"/>
-      <c r="J20" s="17" t="n"/>
+      <c r="H20" s="22" t="n">
+        <v>46323.854375</v>
+      </c>
+      <c r="I20" s="22" t="n">
+        <v>46323.64604166667</v>
+      </c>
+      <c r="J20" s="17" t="n">
+        <v>426.02</v>
+      </c>
       <c r="K20" s="17">
         <f>IF(ISNUMBER(J20),J20*F20,"")</f>
         <v/>
@@ -10660,10 +13928,14 @@
         <f>IF(ISNUMBER(H20),H20-C20,"")</f>
         <v/>
       </c>
-      <c r="O20" s="6" t="n"/>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P20" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10694,9 +13966,15 @@
         <f>E21*F21</f>
         <v/>
       </c>
-      <c r="H21" s="22" t="n"/>
-      <c r="I21" s="22" t="n"/>
-      <c r="J21" s="17" t="n"/>
+      <c r="H21" s="22" t="n">
+        <v>46323.85466435185</v>
+      </c>
+      <c r="I21" s="22" t="n">
+        <v>46323.64633101852</v>
+      </c>
+      <c r="J21" s="17" t="n">
+        <v>427.12</v>
+      </c>
       <c r="K21" s="17">
         <f>IF(ISNUMBER(J21),J21*F21,"")</f>
         <v/>
@@ -10713,10 +13991,14 @@
         <f>IF(ISNUMBER(H21),H21-C21,"")</f>
         <v/>
       </c>
-      <c r="O21" s="6" t="n"/>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10747,9 +14029,15 @@
         <f>E22*F22</f>
         <v/>
       </c>
-      <c r="H22" s="22" t="n"/>
-      <c r="I22" s="22" t="n"/>
-      <c r="J22" s="17" t="n"/>
+      <c r="H22" s="22" t="n">
+        <v>46323.85461805556</v>
+      </c>
+      <c r="I22" s="22" t="n">
+        <v>46323.64628472222</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>73.23</v>
+      </c>
       <c r="K22" s="17">
         <f>IF(ISNUMBER(J22),J22*F22,"")</f>
         <v/>
@@ -10766,10 +14054,14 @@
         <f>IF(ISNUMBER(H22),H22-C22,"")</f>
         <v/>
       </c>
-      <c r="O22" s="6" t="n"/>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P22" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10800,9 +14092,15 @@
         <f>E23*F23</f>
         <v/>
       </c>
-      <c r="H23" s="22" t="n"/>
-      <c r="I23" s="22" t="n"/>
-      <c r="J23" s="17" t="n"/>
+      <c r="H23" s="22" t="n">
+        <v>46323.85480324074</v>
+      </c>
+      <c r="I23" s="22" t="n">
+        <v>46323.64646990741</v>
+      </c>
+      <c r="J23" s="17" t="n">
+        <v>321.15</v>
+      </c>
       <c r="K23" s="17">
         <f>IF(ISNUMBER(J23),J23*F23,"")</f>
         <v/>
@@ -10819,10 +14117,14 @@
         <f>IF(ISNUMBER(H23),H23-C23,"")</f>
         <v/>
       </c>
-      <c r="O23" s="6" t="n"/>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P23" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10853,9 +14155,15 @@
         <f>E24*F24</f>
         <v/>
       </c>
-      <c r="H24" s="22" t="n"/>
-      <c r="I24" s="22" t="n"/>
-      <c r="J24" s="17" t="n"/>
+      <c r="H24" s="22" t="n">
+        <v>46323.85454861111</v>
+      </c>
+      <c r="I24" s="22" t="n">
+        <v>46323.64621527777</v>
+      </c>
+      <c r="J24" s="17" t="n">
+        <v>65.22</v>
+      </c>
       <c r="K24" s="17">
         <f>IF(ISNUMBER(J24),J24*F24,"")</f>
         <v/>
@@ -10872,10 +14180,14 @@
         <f>IF(ISNUMBER(H24),H24-C24,"")</f>
         <v/>
       </c>
-      <c r="O24" s="6" t="n"/>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10906,9 +14218,15 @@
         <f>E25*F25</f>
         <v/>
       </c>
-      <c r="H25" s="22" t="n"/>
-      <c r="I25" s="22" t="n"/>
-      <c r="J25" s="17" t="n"/>
+      <c r="H25" s="22" t="n">
+        <v>46323.85436342593</v>
+      </c>
+      <c r="I25" s="22" t="n">
+        <v>46323.64603009259</v>
+      </c>
+      <c r="J25" s="17" t="n">
+        <v>286.66</v>
+      </c>
       <c r="K25" s="17">
         <f>IF(ISNUMBER(J25),J25*F25,"")</f>
         <v/>
@@ -10925,10 +14243,14 @@
         <f>IF(ISNUMBER(H25),H25-C25,"")</f>
         <v/>
       </c>
-      <c r="O25" s="6" t="n"/>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11022,9 +14344,15 @@
         <f>E27*F27</f>
         <v/>
       </c>
-      <c r="H27" s="22" t="n"/>
-      <c r="I27" s="22" t="n"/>
-      <c r="J27" s="17" t="n"/>
+      <c r="H27" s="22" t="n">
+        <v>46323.85456018519</v>
+      </c>
+      <c r="I27" s="22" t="n">
+        <v>46323.64622685185</v>
+      </c>
+      <c r="J27" s="17" t="n">
+        <v>612.568</v>
+      </c>
       <c r="K27" s="17">
         <f>IF(ISNUMBER(J27),J27*F27,"")</f>
         <v/>
@@ -11041,10 +14369,14 @@
         <f>IF(ISNUMBER(H27),H27-C27,"")</f>
         <v/>
       </c>
-      <c r="O27" s="6" t="n"/>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11264,9 +14596,15 @@
         <f>E31*F31</f>
         <v/>
       </c>
-      <c r="H31" s="22" t="n"/>
-      <c r="I31" s="22" t="n"/>
-      <c r="J31" s="17" t="n"/>
+      <c r="H31" s="22" t="n">
+        <v>46323.8544212963</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>46323.64608796296</v>
+      </c>
+      <c r="J31" s="17" t="n">
+        <v>66.09999999999999</v>
+      </c>
       <c r="K31" s="17">
         <f>IF(ISNUMBER(J31),J31*F31,"")</f>
         <v/>
@@ -11283,10 +14621,14 @@
         <f>IF(ISNUMBER(H31),H31-C31,"")</f>
         <v/>
       </c>
-      <c r="O31" s="6" t="n"/>
+      <c r="O31" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P31" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11317,9 +14659,15 @@
         <f>E32*F32</f>
         <v/>
       </c>
-      <c r="H32" s="22" t="n"/>
-      <c r="I32" s="22" t="n"/>
-      <c r="J32" s="17" t="n"/>
+      <c r="H32" s="22" t="n">
+        <v>46323.8544675926</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>46323.64613425926</v>
+      </c>
+      <c r="J32" s="17" t="n">
+        <v>47.68</v>
+      </c>
       <c r="K32" s="17">
         <f>IF(ISNUMBER(J32),J32*F32,"")</f>
         <v/>
@@ -11336,10 +14684,14 @@
         <f>IF(ISNUMBER(H32),H32-C32,"")</f>
         <v/>
       </c>
-      <c r="O32" s="6" t="n"/>
+      <c r="O32" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11370,9 +14722,15 @@
         <f>E33*F33</f>
         <v/>
       </c>
-      <c r="H33" s="22" t="n"/>
-      <c r="I33" s="22" t="n"/>
-      <c r="J33" s="17" t="n"/>
+      <c r="H33" s="22" t="n">
+        <v>46323.85462962963</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>46323.6462962963</v>
+      </c>
+      <c r="J33" s="17" t="n">
+        <v>442.04</v>
+      </c>
       <c r="K33" s="17">
         <f>IF(ISNUMBER(J33),J33*F33,"")</f>
         <v/>
@@ -11389,10 +14747,14 @@
         <f>IF(ISNUMBER(H33),H33-C33,"")</f>
         <v/>
       </c>
-      <c r="O33" s="6" t="n"/>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P33" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11423,9 +14785,15 @@
         <f>E34*F34</f>
         <v/>
       </c>
-      <c r="H34" s="22" t="n"/>
-      <c r="I34" s="22" t="n"/>
-      <c r="J34" s="17" t="n"/>
+      <c r="H34" s="22" t="n">
+        <v>46323.85447916666</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>46323.64614583334</v>
+      </c>
+      <c r="J34" s="17" t="n">
+        <v>56.34</v>
+      </c>
       <c r="K34" s="17">
         <f>IF(ISNUMBER(J34),J34*F34,"")</f>
         <v/>
@@ -11442,10 +14810,14 @@
         <f>IF(ISNUMBER(H34),H34-C34,"")</f>
         <v/>
       </c>
-      <c r="O34" s="6" t="n"/>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11476,9 +14848,15 @@
         <f>E35*F35</f>
         <v/>
       </c>
-      <c r="H35" s="22" t="n"/>
-      <c r="I35" s="22" t="n"/>
-      <c r="J35" s="17" t="n"/>
+      <c r="H35" s="22" t="n">
+        <v>46323.8546875</v>
+      </c>
+      <c r="I35" s="22" t="n">
+        <v>46323.64635416667</v>
+      </c>
+      <c r="J35" s="17" t="n">
+        <v>273.476</v>
+      </c>
       <c r="K35" s="17">
         <f>IF(ISNUMBER(J35),J35*F35,"")</f>
         <v/>
@@ -11495,10 +14873,14 @@
         <f>IF(ISNUMBER(H35),H35-C35,"")</f>
         <v/>
       </c>
-      <c r="O35" s="6" t="n"/>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P35" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11592,9 +14974,15 @@
         <f>E37*F37</f>
         <v/>
       </c>
-      <c r="H37" s="22" t="n"/>
-      <c r="I37" s="22" t="n"/>
-      <c r="J37" s="17" t="n"/>
+      <c r="H37" s="22" t="n">
+        <v>46323.85440972223</v>
+      </c>
+      <c r="I37" s="22" t="n">
+        <v>46323.64607638889</v>
+      </c>
+      <c r="J37" s="17" t="n">
+        <v>113.556</v>
+      </c>
       <c r="K37" s="17">
         <f>IF(ISNUMBER(J37),J37*F37,"")</f>
         <v/>
@@ -11611,10 +14999,14 @@
         <f>IF(ISNUMBER(H37),H37-C37,"")</f>
         <v/>
       </c>
-      <c r="O37" s="6" t="n"/>
+      <c r="O37" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P37" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11708,9 +15100,15 @@
         <f>E39*F39</f>
         <v/>
       </c>
-      <c r="H39" s="22" t="n"/>
-      <c r="I39" s="22" t="n"/>
-      <c r="J39" s="17" t="n"/>
+      <c r="H39" s="22" t="n">
+        <v>46323.85453703703</v>
+      </c>
+      <c r="I39" s="22" t="n">
+        <v>46323.64620370371</v>
+      </c>
+      <c r="J39" s="17" t="n">
+        <v>1295.462</v>
+      </c>
       <c r="K39" s="17">
         <f>IF(ISNUMBER(J39),J39*F39,"")</f>
         <v/>
@@ -11727,10 +15125,14 @@
         <f>IF(ISNUMBER(H39),H39-C39,"")</f>
         <v/>
       </c>
-      <c r="O39" s="6" t="n"/>
+      <c r="O39" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P39" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11824,9 +15226,15 @@
         <f>E41*F41</f>
         <v/>
       </c>
-      <c r="H41" s="22" t="n"/>
-      <c r="I41" s="22" t="n"/>
-      <c r="J41" s="17" t="n"/>
+      <c r="H41" s="22" t="n">
+        <v>46323.85471064815</v>
+      </c>
+      <c r="I41" s="22" t="n">
+        <v>46323.64637731481</v>
+      </c>
+      <c r="J41" s="17" t="n">
+        <v>810.48</v>
+      </c>
       <c r="K41" s="17">
         <f>IF(ISNUMBER(J41),J41*F41,"")</f>
         <v/>
@@ -11843,10 +15251,14 @@
         <f>IF(ISNUMBER(H41),H41-C41,"")</f>
         <v/>
       </c>
-      <c r="O41" s="6" t="n"/>
+      <c r="O41" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P41" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11877,9 +15289,15 @@
         <f>E42*F42</f>
         <v/>
       </c>
-      <c r="H42" s="22" t="n"/>
-      <c r="I42" s="22" t="n"/>
-      <c r="J42" s="17" t="n"/>
+      <c r="H42" s="22" t="n">
+        <v>46323.85474537037</v>
+      </c>
+      <c r="I42" s="22" t="n">
+        <v>46323.64641203704</v>
+      </c>
+      <c r="J42" s="17" t="n">
+        <v>91.59999999999999</v>
+      </c>
       <c r="K42" s="17">
         <f>IF(ISNUMBER(J42),J42*F42,"")</f>
         <v/>
@@ -11896,10 +15314,14 @@
         <f>IF(ISNUMBER(H42),H42-C42,"")</f>
         <v/>
       </c>
-      <c r="O42" s="6" t="n"/>
+      <c r="O42" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P42" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-29 13:30 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA75" headerRowCount="1">
-  <autoFilter ref="A1:BA75"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA87" headerRowCount="1">
+  <autoFilter ref="A1:BA87"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46323.85530092593</v>
+        <v>46324.60480324074</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46323.64696759259</v>
+        <v>46324.39646990741</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$75,"BUY")+COUNTIF(Orders!$E$2:$E$75,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$87,"BUY")+COUNTIF(Orders!$E$2:$E$87,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$75,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$87,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$75,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$87,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$75,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$87,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$75,Orders!$E$2:$E$75,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$87,Orders!$E$2:$E$87,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$75,Orders!$E$2:$E$75,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$87,Orders!$E$2:$E$87,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA75"/>
+  <dimension ref="A1:BA87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12624,6 +12624,2138 @@
       <c r="AZ75" s="13" t="n"/>
       <c r="BA75" s="6" t="n"/>
     </row>
+    <row r="76">
+      <c r="A76" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="13" t="n">
+        <v>46324.60471064815</v>
+      </c>
+      <c r="C76" s="13" t="n">
+        <v>46324.39637731481</v>
+      </c>
+      <c r="D76" s="13" t="n">
+        <v>46324.56304398148</v>
+      </c>
+      <c r="E76" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>Analog Devices, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J76" s="16" t="n"/>
+      <c r="K76" s="17" t="n"/>
+      <c r="L76" s="17">
+        <f>IF(AND(ISNUMBER(J76),ISNUMBER(K76)),J76*K76,"")</f>
+        <v/>
+      </c>
+      <c r="M76" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N76" s="16" t="n"/>
+      <c r="O76" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P76" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q76" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R76" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S76" s="18" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="T76" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="U76" s="19" t="n">
+        <v>0.0147</v>
+      </c>
+      <c r="V76" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W76" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X76" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y76" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z76" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA76" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB76" s="15" t="n"/>
+      <c r="AC76" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD76" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE76" s="17" t="n">
+        <v>435.9943</v>
+      </c>
+      <c r="AF76" s="17" t="n">
+        <v>416.9835</v>
+      </c>
+      <c r="AG76" s="17" t="n">
+        <v>455.0052</v>
+      </c>
+      <c r="AH76" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI76" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ76" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK76" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL76" s="15" t="inlineStr">
+        <is>
+          <t>Analog Devices Adopts ChipAgents AI Platform for Semiconductor Design</t>
+        </is>
+      </c>
+      <c r="AM76" s="17" t="n">
+        <v>428.5</v>
+      </c>
+      <c r="AN76" s="19" t="n">
+        <v>0.0074</v>
+      </c>
+      <c r="AO76" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP76" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ76" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR76" s="16" t="n"/>
+      <c r="AS76" s="17" t="n"/>
+      <c r="AT76" s="19" t="n"/>
+      <c r="AU76" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV76" s="6" t="inlineStr">
+        <is>
+          <t>945e18ba-dacb-4f18-8f6d-b6d52b27a5b1</t>
+        </is>
+      </c>
+      <c r="AW76" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ADI-1793280647910</t>
+        </is>
+      </c>
+      <c r="AX76" s="13" t="n">
+        <v>46324.56304398148</v>
+      </c>
+      <c r="AY76" s="13" t="n"/>
+      <c r="AZ76" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA76" s="6" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="13" t="n">
+        <v>46324.60471064815</v>
+      </c>
+      <c r="C77" s="13" t="n">
+        <v>46324.39637731481</v>
+      </c>
+      <c r="D77" s="13" t="n">
+        <v>46324.56304398148</v>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="G77" s="15" t="inlineStr">
+        <is>
+          <t>Natera, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J77" s="16" t="n"/>
+      <c r="K77" s="17" t="n"/>
+      <c r="L77" s="17">
+        <f>IF(AND(ISNUMBER(J77),ISNUMBER(K77)),J77*K77,"")</f>
+        <v/>
+      </c>
+      <c r="M77" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N77" s="16" t="n"/>
+      <c r="O77" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P77" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #2, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q77" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R77" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S77" s="18" t="n">
+        <v>0.697</v>
+      </c>
+      <c r="T77" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="U77" s="19" t="n">
+        <v>0.0283</v>
+      </c>
+      <c r="V77" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W77" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="X77" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y77" s="19" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="Z77" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA77" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB77" s="15" t="n"/>
+      <c r="AC77" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD77" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE77" s="17" t="n">
+        <v>437.523</v>
+      </c>
+      <c r="AF77" s="17" t="n">
+        <v>404.5655</v>
+      </c>
+      <c r="AG77" s="17" t="n">
+        <v>470.4804</v>
+      </c>
+      <c r="AH77" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI77" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ77" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK77" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL77" s="15" t="inlineStr">
+        <is>
+          <t>BTIG Maintains Buy on Natera, Raises Price Target to $430</t>
+        </is>
+      </c>
+      <c r="AM77" s="17" t="n">
+        <v>422.38</v>
+      </c>
+      <c r="AN77" s="19" t="n">
+        <v>0.0329</v>
+      </c>
+      <c r="AO77" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP77" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ77" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR77" s="16" t="n"/>
+      <c r="AS77" s="17" t="n"/>
+      <c r="AT77" s="19" t="n"/>
+      <c r="AU77" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV77" s="6" t="inlineStr">
+        <is>
+          <t>f905344b-0702-4074-925b-69965f045190</t>
+        </is>
+      </c>
+      <c r="AW77" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-NTRA-1793280647961</t>
+        </is>
+      </c>
+      <c r="AX77" s="13" t="n">
+        <v>46324.56304398148</v>
+      </c>
+      <c r="AY77" s="13" t="n"/>
+      <c r="AZ77" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA77" s="6" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C78" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D78" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E78" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="G78" s="15" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific, Inc.</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J78" s="16" t="n"/>
+      <c r="K78" s="17" t="n"/>
+      <c r="L78" s="17">
+        <f>IF(AND(ISNUMBER(J78),ISNUMBER(K78)),J78*K78,"")</f>
+        <v/>
+      </c>
+      <c r="M78" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N78" s="16" t="n"/>
+      <c r="O78" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P78" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #3, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q78" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R78" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S78" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T78" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="U78" s="19" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="V78" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W78" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X78" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y78" s="19" t="n">
+        <v>0.0034</v>
+      </c>
+      <c r="Z78" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA78" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB78" s="15" t="n"/>
+      <c r="AC78" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD78" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE78" s="17" t="n">
+        <v>714.9629</v>
+      </c>
+      <c r="AF78" s="17" t="n">
+        <v>689.6806</v>
+      </c>
+      <c r="AG78" s="17" t="n">
+        <v>740.2453</v>
+      </c>
+      <c r="AH78" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI78" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ78" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK78" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL78" s="15" t="inlineStr">
+        <is>
+          <t>Evercore ISI Adjusts Thermo Fisher Scientific Price Target</t>
+        </is>
+      </c>
+      <c r="AM78" s="17" t="n">
+        <v>702.4400000000001</v>
+      </c>
+      <c r="AN78" s="19" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="AO78" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP78" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ78" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR78" s="16" t="n"/>
+      <c r="AS78" s="17" t="n"/>
+      <c r="AT78" s="19" t="n"/>
+      <c r="AU78" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV78" s="6" t="inlineStr">
+        <is>
+          <t>20e9d99f-3228-44b0-99cc-7e07dc593677</t>
+        </is>
+      </c>
+      <c r="AW78" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-TMO-1793280648003</t>
+        </is>
+      </c>
+      <c r="AX78" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY78" s="13" t="n"/>
+      <c r="AZ78" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA78" s="6" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C79" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D79" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E79" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="G79" s="15" t="inlineStr">
+        <is>
+          <t>Occidental Petroleum Corporation</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J79" s="16" t="n"/>
+      <c r="K79" s="17" t="n"/>
+      <c r="L79" s="17">
+        <f>IF(AND(ISNUMBER(J79),ISNUMBER(K79)),J79*K79,"")</f>
+        <v/>
+      </c>
+      <c r="M79" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N79" s="16" t="n"/>
+      <c r="O79" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P79" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q79" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R79" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S79" s="18" t="n">
+        <v>0.621</v>
+      </c>
+      <c r="T79" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="U79" s="19" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="V79" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W79" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X79" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y79" s="19" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="Z79" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA79" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB79" s="15" t="n"/>
+      <c r="AC79" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD79" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE79" s="17" t="n">
+        <v>63.9326</v>
+      </c>
+      <c r="AF79" s="17" t="n">
+        <v>61.2761</v>
+      </c>
+      <c r="AG79" s="17" t="n">
+        <v>66.5891</v>
+      </c>
+      <c r="AH79" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI79" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ79" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK79" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL79" s="15" t="n"/>
+      <c r="AM79" s="17" t="n">
+        <v>63.27</v>
+      </c>
+      <c r="AN79" s="19" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="AO79" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP79" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ79" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR79" s="16" t="n"/>
+      <c r="AS79" s="17" t="n"/>
+      <c r="AT79" s="19" t="n"/>
+      <c r="AU79" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV79" s="6" t="inlineStr">
+        <is>
+          <t>8be935fc-0d73-4a10-9b3e-154f3b63f820</t>
+        </is>
+      </c>
+      <c r="AW79" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-OXY-1793280648055</t>
+        </is>
+      </c>
+      <c r="AX79" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY79" s="13" t="n"/>
+      <c r="AZ79" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA79" s="6" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C80" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D80" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E80" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="G80" s="15" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Public Limited Company Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J80" s="16" t="n"/>
+      <c r="K80" s="17" t="n"/>
+      <c r="L80" s="17">
+        <f>IF(AND(ISNUMBER(J80),ISNUMBER(K80)),J80*K80,"")</f>
+        <v/>
+      </c>
+      <c r="M80" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N80" s="16" t="n"/>
+      <c r="O80" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P80" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #5, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q80" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R80" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S80" s="18" t="n">
+        <v>0.621</v>
+      </c>
+      <c r="T80" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U80" s="19" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="V80" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W80" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X80" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y80" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA80" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB80" s="15" t="n"/>
+      <c r="AC80" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD80" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE80" s="17" t="n">
+        <v>326.195</v>
+      </c>
+      <c r="AF80" s="17" t="n">
+        <v>314.8075</v>
+      </c>
+      <c r="AG80" s="17" t="n">
+        <v>337.5825</v>
+      </c>
+      <c r="AH80" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI80" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ80" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK80" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL80" s="15" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Q3 Adj. EPS $3.63 Beats $3.59 Estimate, Sales $2.460B Beat $2.455B Estimate</t>
+        </is>
+      </c>
+      <c r="AM80" s="17" t="n">
+        <v>321.64</v>
+      </c>
+      <c r="AN80" s="19" t="n">
+        <v>0.0061</v>
+      </c>
+      <c r="AO80" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP80" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ80" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR80" s="16" t="n"/>
+      <c r="AS80" s="17" t="n"/>
+      <c r="AT80" s="19" t="n"/>
+      <c r="AU80" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV80" s="6" t="inlineStr">
+        <is>
+          <t>76d68fb4-073e-48a2-a54a-417213babaf1</t>
+        </is>
+      </c>
+      <c r="AW80" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-WTW-1793280648101</t>
+        </is>
+      </c>
+      <c r="AX80" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY80" s="13" t="n"/>
+      <c r="AZ80" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA80" s="6" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C81" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D81" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E81" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>McKesson Corporation</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J81" s="16" t="n"/>
+      <c r="K81" s="17" t="n"/>
+      <c r="L81" s="17">
+        <f>IF(AND(ISNUMBER(J81),ISNUMBER(K81)),J81*K81,"")</f>
+        <v/>
+      </c>
+      <c r="M81" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N81" s="16" t="n"/>
+      <c r="O81" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P81" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #6, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q81" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R81" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S81" s="18" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="T81" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="U81" s="19" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="V81" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W81" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="X81" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y81" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA81" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB81" s="15" t="n"/>
+      <c r="AC81" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD81" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE81" s="17" t="n">
+        <v>976.5787</v>
+      </c>
+      <c r="AF81" s="17" t="n">
+        <v>938.082</v>
+      </c>
+      <c r="AG81" s="17" t="n">
+        <v>1015.0753</v>
+      </c>
+      <c r="AH81" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI81" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ81" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK81" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL81" s="15" t="n"/>
+      <c r="AM81" s="17" t="n">
+        <v>961.1799999999999</v>
+      </c>
+      <c r="AN81" s="19" t="n">
+        <v>-0.0059</v>
+      </c>
+      <c r="AO81" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP81" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ81" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR81" s="16" t="n"/>
+      <c r="AS81" s="17" t="n"/>
+      <c r="AT81" s="19" t="n"/>
+      <c r="AU81" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV81" s="6" t="inlineStr">
+        <is>
+          <t>40624c33-d43b-482d-b12f-30fb41c490bd</t>
+        </is>
+      </c>
+      <c r="AW81" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MCK-1793280648174</t>
+        </is>
+      </c>
+      <c r="AX81" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY81" s="13" t="n"/>
+      <c r="AZ81" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA81" s="6" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C82" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D82" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E82" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="G82" s="15" t="inlineStr">
+        <is>
+          <t>Intuitive Surgical, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J82" s="16" t="n"/>
+      <c r="K82" s="17" t="n"/>
+      <c r="L82" s="17">
+        <f>IF(AND(ISNUMBER(J82),ISNUMBER(K82)),J82*K82,"")</f>
+        <v/>
+      </c>
+      <c r="M82" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N82" s="16" t="n"/>
+      <c r="O82" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P82" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #9, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q82" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R82" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S82" s="18" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="T82" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U82" s="19" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="V82" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W82" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="X82" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y82" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z82" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA82" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB82" s="15" t="n"/>
+      <c r="AC82" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD82" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE82" s="17" t="n">
+        <v>451.3904</v>
+      </c>
+      <c r="AF82" s="17" t="n">
+        <v>433.3894</v>
+      </c>
+      <c r="AG82" s="17" t="n">
+        <v>469.3914</v>
+      </c>
+      <c r="AH82" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI82" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ82" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK82" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL82" s="15" t="inlineStr">
+        <is>
+          <t>Evercore ISI Adjusts Intuitive Surgical Price Target to $375 From $385</t>
+        </is>
+      </c>
+      <c r="AM82" s="17" t="n">
+        <v>444.19</v>
+      </c>
+      <c r="AN82" s="19" t="n">
+        <v>-0.0039</v>
+      </c>
+      <c r="AO82" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP82" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ82" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR82" s="16" t="n"/>
+      <c r="AS82" s="17" t="n"/>
+      <c r="AT82" s="19" t="n"/>
+      <c r="AU82" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV82" s="6" t="inlineStr">
+        <is>
+          <t>d6ce49ed-c1b3-489d-93c3-851dba2e9981</t>
+        </is>
+      </c>
+      <c r="AW82" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ISRG-1793280648289</t>
+        </is>
+      </c>
+      <c r="AX82" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY82" s="13" t="n"/>
+      <c r="AZ82" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA82" s="6" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="12" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C83" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D83" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E83" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="G83" s="15" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J83" s="16" t="n"/>
+      <c r="K83" s="17" t="n"/>
+      <c r="L83" s="17">
+        <f>IF(AND(ISNUMBER(J83),ISNUMBER(K83)),J83*K83,"")</f>
+        <v/>
+      </c>
+      <c r="M83" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N83" s="16" t="n"/>
+      <c r="O83" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P83" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #10, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q83" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R83" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S83" s="18" t="n">
+        <v>0.648</v>
+      </c>
+      <c r="T83" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="U83" s="19" t="n">
+        <v>0.0132</v>
+      </c>
+      <c r="V83" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W83" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="X83" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y83" s="19" t="n">
+        <v>0.0064</v>
+      </c>
+      <c r="Z83" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA83" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB83" s="15" t="n"/>
+      <c r="AC83" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD83" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE83" s="17" t="n">
+        <v>289.3086</v>
+      </c>
+      <c r="AF83" s="17" t="n">
+        <v>279.4621</v>
+      </c>
+      <c r="AG83" s="17" t="n">
+        <v>299.1552</v>
+      </c>
+      <c r="AH83" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI83" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ83" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK83" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL83" s="15" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing Q1 2027 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM83" s="17" t="n">
+        <v>287.21</v>
+      </c>
+      <c r="AN83" s="19" t="n">
+        <v>-0.0258</v>
+      </c>
+      <c r="AO83" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP83" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ83" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR83" s="16" t="n"/>
+      <c r="AS83" s="17" t="n"/>
+      <c r="AT83" s="19" t="n"/>
+      <c r="AU83" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV83" s="6" t="inlineStr">
+        <is>
+          <t>8a1d5db1-bd96-4ec4-8cf7-90f3d674ae95</t>
+        </is>
+      </c>
+      <c r="AW83" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ADP-1793280648342</t>
+        </is>
+      </c>
+      <c r="AX83" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY83" s="13" t="n"/>
+      <c r="AZ83" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA83" s="6" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C84" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D84" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E84" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="G84" s="15" t="inlineStr">
+        <is>
+          <t>IQVIA Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J84" s="16" t="n"/>
+      <c r="K84" s="17" t="n"/>
+      <c r="L84" s="17">
+        <f>IF(AND(ISNUMBER(J84),ISNUMBER(K84)),J84*K84,"")</f>
+        <v/>
+      </c>
+      <c r="M84" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N84" s="16" t="n"/>
+      <c r="O84" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P84" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #11, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q84" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R84" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S84" s="18" t="n">
+        <v>0.608</v>
+      </c>
+      <c r="T84" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="U84" s="19" t="n">
+        <v>0.0149</v>
+      </c>
+      <c r="V84" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W84" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="X84" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y84" s="19" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="Z84" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA84" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB84" s="15" t="n"/>
+      <c r="AC84" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD84" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE84" s="17" t="n">
+        <v>283.0364</v>
+      </c>
+      <c r="AF84" s="17" t="n">
+        <v>272.7205</v>
+      </c>
+      <c r="AG84" s="17" t="n">
+        <v>293.3523</v>
+      </c>
+      <c r="AH84" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI84" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ84" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK84" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL84" s="15" t="inlineStr">
+        <is>
+          <t>JP Morgan Maintains Overweight on IQVIA Holdings, Raises Price Target to $325</t>
+        </is>
+      </c>
+      <c r="AM84" s="17" t="n">
+        <v>278.7</v>
+      </c>
+      <c r="AN84" s="19" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="AO84" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP84" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ84" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR84" s="16" t="n"/>
+      <c r="AS84" s="17" t="n"/>
+      <c r="AT84" s="19" t="n"/>
+      <c r="AU84" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV84" s="6" t="inlineStr">
+        <is>
+          <t>f2ead90d-b916-49fe-9325-a63c56fae54a</t>
+        </is>
+      </c>
+      <c r="AW84" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-IQV-1793280648394</t>
+        </is>
+      </c>
+      <c r="AX84" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY84" s="13" t="n"/>
+      <c r="AZ84" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA84" s="6" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C85" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D85" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E85" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="G85" s="15" t="inlineStr">
+        <is>
+          <t>Eli Lilly &amp; Co.</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J85" s="16" t="n"/>
+      <c r="K85" s="17" t="n"/>
+      <c r="L85" s="17">
+        <f>IF(AND(ISNUMBER(J85),ISNUMBER(K85)),J85*K85,"")</f>
+        <v/>
+      </c>
+      <c r="M85" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N85" s="16" t="n"/>
+      <c r="O85" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P85" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #12, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q85" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R85" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S85" s="18" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="T85" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="U85" s="19" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="V85" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W85" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="X85" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y85" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z85" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA85" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB85" s="15" t="n"/>
+      <c r="AC85" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD85" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE85" s="17" t="n">
+        <v>1311.7784</v>
+      </c>
+      <c r="AF85" s="17" t="n">
+        <v>1259.0074</v>
+      </c>
+      <c r="AG85" s="17" t="n">
+        <v>1364.5494</v>
+      </c>
+      <c r="AH85" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI85" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ85" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK85" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL85" s="15" t="inlineStr">
+        <is>
+          <t>Eli Lilly Lowers FY2026 Adj EPS Guidance from $35.50-$36.50 to $35.00-$36.00 vs $34.04 Est; Raises FY2026 Sales Guidance from $85.000B-$87.000B to $91.000B-$92.000B vs $88.848B Est</t>
+        </is>
+      </c>
+      <c r="AM85" s="17" t="n">
+        <v>1290.67</v>
+      </c>
+      <c r="AN85" s="19" t="n">
+        <v>0.0071</v>
+      </c>
+      <c r="AO85" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP85" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ85" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR85" s="16" t="n"/>
+      <c r="AS85" s="17" t="n"/>
+      <c r="AT85" s="19" t="n"/>
+      <c r="AU85" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV85" s="6" t="inlineStr">
+        <is>
+          <t>c6b04753-7485-469f-8d38-d301e8e7b741</t>
+        </is>
+      </c>
+      <c r="AW85" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-LLY-1793280648448</t>
+        </is>
+      </c>
+      <c r="AX85" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY85" s="13" t="n"/>
+      <c r="AZ85" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA85" s="6" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C86" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D86" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E86" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="G86" s="15" t="inlineStr">
+        <is>
+          <t>MARATHON PETROLEUM CORPORATION</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J86" s="16" t="n"/>
+      <c r="K86" s="17" t="n"/>
+      <c r="L86" s="17">
+        <f>IF(AND(ISNUMBER(J86),ISNUMBER(K86)),J86*K86,"")</f>
+        <v/>
+      </c>
+      <c r="M86" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N86" s="16" t="n"/>
+      <c r="O86" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P86" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #13, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q86" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R86" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S86" s="18" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="T86" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="U86" s="19" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="V86" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W86" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="X86" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y86" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z86" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA86" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB86" s="15" t="inlineStr">
+        <is>
+          <t>One day (-7.4%) did 81% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC86" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD86" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE86" s="17" t="n">
+        <v>450.3744</v>
+      </c>
+      <c r="AF86" s="17" t="n">
+        <v>425.9885</v>
+      </c>
+      <c r="AG86" s="17" t="n">
+        <v>474.7603</v>
+      </c>
+      <c r="AH86" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI86" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ86" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK86" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL86" s="15" t="inlineStr">
+        <is>
+          <t>Reported Earlier, Marathon Petroleum Raises Quarterly Dividend 10% To $1.10 Per Share From $1.00, Payable Dec. 10, 2026, To Shareholders Of Record As Of Nov. 18</t>
+        </is>
+      </c>
+      <c r="AM86" s="17" t="n">
+        <v>440.62</v>
+      </c>
+      <c r="AN86" s="19" t="n">
+        <v>0.0108</v>
+      </c>
+      <c r="AO86" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP86" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ86" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR86" s="16" t="n"/>
+      <c r="AS86" s="17" t="n"/>
+      <c r="AT86" s="19" t="n"/>
+      <c r="AU86" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV86" s="6" t="inlineStr">
+        <is>
+          <t>290918e4-4d4f-4c2f-af48-d921cb97a8b1</t>
+        </is>
+      </c>
+      <c r="AW86" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MPC-1793280648508</t>
+        </is>
+      </c>
+      <c r="AX86" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY86" s="13" t="n"/>
+      <c r="AZ86" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA86" s="6" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="12" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="13" t="n">
+        <v>46324.60472222222</v>
+      </c>
+      <c r="C87" s="13" t="n">
+        <v>46324.39638888889</v>
+      </c>
+      <c r="D87" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="E87" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G87" s="15" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J87" s="16" t="n"/>
+      <c r="K87" s="17" t="n"/>
+      <c r="L87" s="17">
+        <f>IF(AND(ISNUMBER(J87),ISNUMBER(K87)),J87*K87,"")</f>
+        <v/>
+      </c>
+      <c r="M87" s="17" t="n">
+        <v>8345.969999999999</v>
+      </c>
+      <c r="N87" s="16" t="n"/>
+      <c r="O87" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P87" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #14, 8.33% of the $100,191.79 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q87" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R87" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S87" s="18" t="n">
+        <v>0.553</v>
+      </c>
+      <c r="T87" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="U87" s="19" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="V87" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W87" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="X87" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y87" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z87" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA87" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB87" s="15" t="n"/>
+      <c r="AC87" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD87" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE87" s="17" t="n">
+        <v>617.0697</v>
+      </c>
+      <c r="AF87" s="17" t="n">
+        <v>601.3704</v>
+      </c>
+      <c r="AG87" s="17" t="n">
+        <v>632.769</v>
+      </c>
+      <c r="AH87" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI87" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ87" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK87" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL87" s="15" t="inlineStr">
+        <is>
+          <t>Msatercard CEO Says While There Continues To Be Economic And Geopolitical Uncertainty, Consumers Continue To Spend</t>
+        </is>
+      </c>
+      <c r="AM87" s="17" t="n">
+        <v>610.79</v>
+      </c>
+      <c r="AN87" s="19" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="AO87" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AP87" s="17" t="n">
+        <v>100191.79</v>
+      </c>
+      <c r="AQ87" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR87" s="16" t="n"/>
+      <c r="AS87" s="17" t="n"/>
+      <c r="AT87" s="19" t="n"/>
+      <c r="AU87" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV87" s="6" t="inlineStr">
+        <is>
+          <t>456ab71a-6843-4001-b9a0-e1c7c379c39f</t>
+        </is>
+      </c>
+      <c r="AW87" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MA-1793280648546</t>
+        </is>
+      </c>
+      <c r="AX87" s="13" t="n">
+        <v>46324.56305555555</v>
+      </c>
+      <c r="AY87" s="13" t="n"/>
+      <c r="AZ87" s="13" t="n">
+        <v>46324.56267361111</v>
+      </c>
+      <c r="BA87" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
records: 2026-10-29 13:37 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P42" headerRowCount="1">
-  <autoFilter ref="A1:P42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P54" headerRowCount="1">
+  <autoFilter ref="A1:P54"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.60480324074</v>
+        <v>46324.60924768518</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.39646990741</v>
+        <v>46324.40091435185</v>
       </c>
     </row>
     <row r="4">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$42,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$42,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$54,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$42)</f>
+        <f>SUM('Round trips'!$L$2:$L$54)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$42,"Closed",'Round trips'!$L$2:$L$42,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$54,"Closed",'Round trips'!$L$2:$L$54,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -12629,13 +12629,13 @@
         <v>75</v>
       </c>
       <c r="B76" s="13" t="n">
-        <v>46324.60471064815</v>
+        <v>46324.6062962963</v>
       </c>
       <c r="C76" s="13" t="n">
-        <v>46324.39637731481</v>
+        <v>46324.39796296296</v>
       </c>
       <c r="D76" s="13" t="n">
-        <v>46324.56304398148</v>
+        <v>46324.56462962963</v>
       </c>
       <c r="E76" s="14" t="inlineStr">
         <is>
@@ -12659,11 +12659,15 @@
       </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J76" s="16" t="n"/>
-      <c r="K76" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J76" s="16" t="n">
+        <v>19.536817436</v>
+      </c>
+      <c r="K76" s="17" t="n">
+        <v>427.19138</v>
+      </c>
       <c r="L76" s="17">
         <f>IF(AND(ISNUMBER(J76),ISNUMBER(K76)),J76*K76,"")</f>
         <v/>
@@ -12796,7 +12800,9 @@
       <c r="AX76" s="13" t="n">
         <v>46324.56304398148</v>
       </c>
-      <c r="AY76" s="13" t="n"/>
+      <c r="AY76" s="13" t="n">
+        <v>46324.56462962963</v>
+      </c>
       <c r="AZ76" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -12807,13 +12813,13 @@
         <v>76</v>
       </c>
       <c r="B77" s="13" t="n">
-        <v>46324.60471064815</v>
+        <v>46324.60716435185</v>
       </c>
       <c r="C77" s="13" t="n">
-        <v>46324.39637731481</v>
+        <v>46324.39883101852</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>46324.56304398148</v>
+        <v>46324.56549768519</v>
       </c>
       <c r="E77" s="14" t="inlineStr">
         <is>
@@ -12837,11 +12843,15 @@
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J77" s="16" t="n"/>
-      <c r="K77" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J77" s="16" t="n">
+        <v>19.644723215</v>
+      </c>
+      <c r="K77" s="17" t="n">
+        <v>424.844876</v>
+      </c>
       <c r="L77" s="17">
         <f>IF(AND(ISNUMBER(J77),ISNUMBER(K77)),J77*K77,"")</f>
         <v/>
@@ -12974,7 +12984,9 @@
       <c r="AX77" s="13" t="n">
         <v>46324.56304398148</v>
       </c>
-      <c r="AY77" s="13" t="n"/>
+      <c r="AY77" s="13" t="n">
+        <v>46324.56549768519</v>
+      </c>
       <c r="AZ77" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -12985,13 +12997,13 @@
         <v>77</v>
       </c>
       <c r="B78" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60688657407</v>
       </c>
       <c r="C78" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39855324074</v>
       </c>
       <c r="D78" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56521990741</v>
       </c>
       <c r="E78" s="14" t="inlineStr">
         <is>
@@ -13015,11 +13027,15 @@
       </c>
       <c r="I78" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J78" s="16" t="n"/>
-      <c r="K78" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J78" s="16" t="n">
+        <v>11.851651941</v>
+      </c>
+      <c r="K78" s="17" t="n">
+        <v>704.202253</v>
+      </c>
       <c r="L78" s="17">
         <f>IF(AND(ISNUMBER(J78),ISNUMBER(K78)),J78*K78,"")</f>
         <v/>
@@ -13152,7 +13168,9 @@
       <c r="AX78" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY78" s="13" t="n"/>
+      <c r="AY78" s="13" t="n">
+        <v>46324.56521990741</v>
+      </c>
       <c r="AZ78" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -13163,13 +13181,13 @@
         <v>78</v>
       </c>
       <c r="B79" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60554398148</v>
       </c>
       <c r="C79" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39721064815</v>
       </c>
       <c r="D79" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56387731482</v>
       </c>
       <c r="E79" s="14" t="inlineStr">
         <is>
@@ -13193,11 +13211,15 @@
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J79" s="16" t="n"/>
-      <c r="K79" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J79" s="16" t="n">
+        <v>132.370499603</v>
+      </c>
+      <c r="K79" s="17" t="n">
+        <v>63.05</v>
+      </c>
       <c r="L79" s="17">
         <f>IF(AND(ISNUMBER(J79),ISNUMBER(K79)),J79*K79,"")</f>
         <v/>
@@ -13326,7 +13348,9 @@
       <c r="AX79" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY79" s="13" t="n"/>
+      <c r="AY79" s="13" t="n">
+        <v>46324.56387731482</v>
+      </c>
       <c r="AZ79" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -13337,13 +13361,13 @@
         <v>79</v>
       </c>
       <c r="B80" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60677083334</v>
       </c>
       <c r="C80" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.3984375</v>
       </c>
       <c r="D80" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56510416666</v>
       </c>
       <c r="E80" s="14" t="inlineStr">
         <is>
@@ -13367,11 +13391,15 @@
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J80" s="16" t="n"/>
-      <c r="K80" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J80" s="16" t="n">
+        <v>26.078334421</v>
+      </c>
+      <c r="K80" s="17" t="n">
+        <v>320.034243</v>
+      </c>
       <c r="L80" s="17">
         <f>IF(AND(ISNUMBER(J80),ISNUMBER(K80)),J80*K80,"")</f>
         <v/>
@@ -13504,7 +13532,9 @@
       <c r="AX80" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY80" s="13" t="n"/>
+      <c r="AY80" s="13" t="n">
+        <v>46324.56510416666</v>
+      </c>
       <c r="AZ80" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -13515,13 +13545,13 @@
         <v>80</v>
       </c>
       <c r="B81" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60704861111</v>
       </c>
       <c r="C81" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39871527778</v>
       </c>
       <c r="D81" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56538194444</v>
       </c>
       <c r="E81" s="14" t="inlineStr">
         <is>
@@ -13545,11 +13575,15 @@
       </c>
       <c r="I81" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J81" s="16" t="n"/>
-      <c r="K81" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J81" s="16" t="n">
+        <v>8.556874402</v>
+      </c>
+      <c r="K81" s="17" t="n">
+        <v>975.351467</v>
+      </c>
       <c r="L81" s="17">
         <f>IF(AND(ISNUMBER(J81),ISNUMBER(K81)),J81*K81,"")</f>
         <v/>
@@ -13678,7 +13712,9 @@
       <c r="AX81" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY81" s="13" t="n"/>
+      <c r="AY81" s="13" t="n">
+        <v>46324.56538194444</v>
+      </c>
       <c r="AZ81" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -13689,13 +13725,13 @@
         <v>81</v>
       </c>
       <c r="B82" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60655092593</v>
       </c>
       <c r="C82" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39821759259</v>
       </c>
       <c r="D82" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56488425926</v>
       </c>
       <c r="E82" s="14" t="inlineStr">
         <is>
@@ -13719,11 +13755,15 @@
       </c>
       <c r="I82" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J82" s="16" t="n"/>
-      <c r="K82" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J82" s="16" t="n">
+        <v>18.645716072</v>
+      </c>
+      <c r="K82" s="17" t="n">
+        <v>447.607374</v>
+      </c>
       <c r="L82" s="17">
         <f>IF(AND(ISNUMBER(J82),ISNUMBER(K82)),J82*K82,"")</f>
         <v/>
@@ -13856,7 +13896,9 @@
       <c r="AX82" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY82" s="13" t="n"/>
+      <c r="AY82" s="13" t="n">
+        <v>46324.56488425926</v>
+      </c>
       <c r="AZ82" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -13867,13 +13909,13 @@
         <v>82</v>
       </c>
       <c r="B83" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60613425926</v>
       </c>
       <c r="C83" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39780092592</v>
       </c>
       <c r="D83" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56446759259</v>
       </c>
       <c r="E83" s="14" t="inlineStr">
         <is>
@@ -13897,11 +13939,15 @@
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J83" s="16" t="n"/>
-      <c r="K83" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J83" s="16" t="n">
+        <v>28.879753624</v>
+      </c>
+      <c r="K83" s="17" t="n">
+        <v>288.99</v>
+      </c>
       <c r="L83" s="17">
         <f>IF(AND(ISNUMBER(J83),ISNUMBER(K83)),J83*K83,"")</f>
         <v/>
@@ -14034,7 +14080,9 @@
       <c r="AX83" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY83" s="13" t="n"/>
+      <c r="AY83" s="13" t="n">
+        <v>46324.56446759259</v>
+      </c>
       <c r="AZ83" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -14045,13 +14093,13 @@
         <v>83</v>
       </c>
       <c r="B84" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60626157407</v>
       </c>
       <c r="C84" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39792824074</v>
       </c>
       <c r="D84" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56459490741</v>
       </c>
       <c r="E84" s="14" t="inlineStr">
         <is>
@@ -14075,11 +14123,15 @@
       </c>
       <c r="I84" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J84" s="16" t="n"/>
-      <c r="K84" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J84" s="16" t="n">
+        <v>30.075531531</v>
+      </c>
+      <c r="K84" s="17" t="n">
+        <v>277.5</v>
+      </c>
       <c r="L84" s="17">
         <f>IF(AND(ISNUMBER(J84),ISNUMBER(K84)),J84*K84,"")</f>
         <v/>
@@ -14212,7 +14264,9 @@
       <c r="AX84" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY84" s="13" t="n"/>
+      <c r="AY84" s="13" t="n">
+        <v>46324.56459490741</v>
+      </c>
       <c r="AZ84" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -14223,13 +14277,13 @@
         <v>84</v>
       </c>
       <c r="B85" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60625</v>
       </c>
       <c r="C85" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39791666667</v>
       </c>
       <c r="D85" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56458333333</v>
       </c>
       <c r="E85" s="14" t="inlineStr">
         <is>
@@ -14253,11 +14307,15 @@
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J85" s="16" t="n"/>
-      <c r="K85" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J85" s="16" t="n">
+        <v>6.035195373</v>
+      </c>
+      <c r="K85" s="17" t="n">
+        <v>1382.881495</v>
+      </c>
       <c r="L85" s="17">
         <f>IF(AND(ISNUMBER(J85),ISNUMBER(K85)),J85*K85,"")</f>
         <v/>
@@ -14390,7 +14448,9 @@
       <c r="AX85" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY85" s="13" t="n"/>
+      <c r="AY85" s="13" t="n">
+        <v>46324.56458333333</v>
+      </c>
       <c r="AZ85" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -14401,13 +14461,13 @@
         <v>85</v>
       </c>
       <c r="B86" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60640046297</v>
       </c>
       <c r="C86" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39806712963</v>
       </c>
       <c r="D86" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56473379629</v>
       </c>
       <c r="E86" s="14" t="inlineStr">
         <is>
@@ -14431,11 +14491,15 @@
       </c>
       <c r="I86" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J86" s="16" t="n"/>
-      <c r="K86" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J86" s="16" t="n">
+        <v>18.846467973</v>
+      </c>
+      <c r="K86" s="17" t="n">
+        <v>442.839476</v>
+      </c>
       <c r="L86" s="17">
         <f>IF(AND(ISNUMBER(J86),ISNUMBER(K86)),J86*K86,"")</f>
         <v/>
@@ -14572,7 +14636,9 @@
       <c r="AX86" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY86" s="13" t="n"/>
+      <c r="AY86" s="13" t="n">
+        <v>46324.56473379629</v>
+      </c>
       <c r="AZ86" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -14583,13 +14649,13 @@
         <v>86</v>
       </c>
       <c r="B87" s="13" t="n">
-        <v>46324.60472222222</v>
+        <v>46324.60722222222</v>
       </c>
       <c r="C87" s="13" t="n">
-        <v>46324.39638888889</v>
+        <v>46324.39888888889</v>
       </c>
       <c r="D87" s="13" t="n">
-        <v>46324.56305555555</v>
+        <v>46324.56555555556</v>
       </c>
       <c r="E87" s="14" t="inlineStr">
         <is>
@@ -14613,11 +14679,15 @@
       </c>
       <c r="I87" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J87" s="16" t="n"/>
-      <c r="K87" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J87" s="16" t="n">
+        <v>13.053417297</v>
+      </c>
+      <c r="K87" s="17" t="n">
+        <v>639.369739</v>
+      </c>
       <c r="L87" s="17">
         <f>IF(AND(ISNUMBER(J87),ISNUMBER(K87)),J87*K87,"")</f>
         <v/>
@@ -14750,7 +14820,9 @@
       <c r="AX87" s="13" t="n">
         <v>46324.56305555555</v>
       </c>
-      <c r="AY87" s="13" t="n"/>
+      <c r="AY87" s="13" t="n">
+        <v>46324.56555555556</v>
+      </c>
       <c r="AZ87" s="13" t="n">
         <v>46324.56267361111</v>
       </c>
@@ -14771,7 +14843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -17457,8 +17529,644 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Occidental Petroleum Corporation</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="n">
+        <v>46324.60554398148</v>
+      </c>
+      <c r="D43" s="22" t="n">
+        <v>46324.39721064815</v>
+      </c>
+      <c r="E43" s="17" t="n">
+        <v>63.05</v>
+      </c>
+      <c r="F43" s="16" t="n">
+        <v>132.370499603</v>
+      </c>
+      <c r="G43" s="17">
+        <f>E43*F43</f>
+        <v/>
+      </c>
+      <c r="H43" s="22" t="n"/>
+      <c r="I43" s="22" t="n"/>
+      <c r="J43" s="17" t="n"/>
+      <c r="K43" s="17">
+        <f>IF(ISNUMBER(J43),J43*F43,"")</f>
+        <v/>
+      </c>
+      <c r="L43" s="23">
+        <f>IF(ISNUMBER(J43),K43-G43,"")</f>
+        <v/>
+      </c>
+      <c r="M43" s="24">
+        <f>IF(ISNUMBER(J43),L43/G43,"")</f>
+        <v/>
+      </c>
+      <c r="N43" s="25">
+        <f>IF(ISNUMBER(H43),H43-C43,"")</f>
+        <v/>
+      </c>
+      <c r="O43" s="6" t="n"/>
+      <c r="P43" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="n">
+        <v>46324.60613425926</v>
+      </c>
+      <c r="D44" s="22" t="n">
+        <v>46324.39780092592</v>
+      </c>
+      <c r="E44" s="17" t="n">
+        <v>288.99</v>
+      </c>
+      <c r="F44" s="16" t="n">
+        <v>28.879753624</v>
+      </c>
+      <c r="G44" s="17">
+        <f>E44*F44</f>
+        <v/>
+      </c>
+      <c r="H44" s="22" t="n"/>
+      <c r="I44" s="22" t="n"/>
+      <c r="J44" s="17" t="n"/>
+      <c r="K44" s="17">
+        <f>IF(ISNUMBER(J44),J44*F44,"")</f>
+        <v/>
+      </c>
+      <c r="L44" s="23">
+        <f>IF(ISNUMBER(J44),K44-G44,"")</f>
+        <v/>
+      </c>
+      <c r="M44" s="24">
+        <f>IF(ISNUMBER(J44),L44/G44,"")</f>
+        <v/>
+      </c>
+      <c r="N44" s="25">
+        <f>IF(ISNUMBER(H44),H44-C44,"")</f>
+        <v/>
+      </c>
+      <c r="O44" s="6" t="n"/>
+      <c r="P44" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Eli Lilly &amp; Co.</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="n">
+        <v>46324.60625</v>
+      </c>
+      <c r="D45" s="22" t="n">
+        <v>46324.39791666667</v>
+      </c>
+      <c r="E45" s="17" t="n">
+        <v>1382.881495</v>
+      </c>
+      <c r="F45" s="16" t="n">
+        <v>6.035195373</v>
+      </c>
+      <c r="G45" s="17">
+        <f>E45*F45</f>
+        <v/>
+      </c>
+      <c r="H45" s="22" t="n"/>
+      <c r="I45" s="22" t="n"/>
+      <c r="J45" s="17" t="n"/>
+      <c r="K45" s="17">
+        <f>IF(ISNUMBER(J45),J45*F45,"")</f>
+        <v/>
+      </c>
+      <c r="L45" s="23">
+        <f>IF(ISNUMBER(J45),K45-G45,"")</f>
+        <v/>
+      </c>
+      <c r="M45" s="24">
+        <f>IF(ISNUMBER(J45),L45/G45,"")</f>
+        <v/>
+      </c>
+      <c r="N45" s="25">
+        <f>IF(ISNUMBER(H45),H45-C45,"")</f>
+        <v/>
+      </c>
+      <c r="O45" s="6" t="n"/>
+      <c r="P45" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>IQVIA Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="n">
+        <v>46324.60626157407</v>
+      </c>
+      <c r="D46" s="22" t="n">
+        <v>46324.39792824074</v>
+      </c>
+      <c r="E46" s="17" t="n">
+        <v>277.5</v>
+      </c>
+      <c r="F46" s="16" t="n">
+        <v>30.075531531</v>
+      </c>
+      <c r="G46" s="17">
+        <f>E46*F46</f>
+        <v/>
+      </c>
+      <c r="H46" s="22" t="n"/>
+      <c r="I46" s="22" t="n"/>
+      <c r="J46" s="17" t="n"/>
+      <c r="K46" s="17">
+        <f>IF(ISNUMBER(J46),J46*F46,"")</f>
+        <v/>
+      </c>
+      <c r="L46" s="23">
+        <f>IF(ISNUMBER(J46),K46-G46,"")</f>
+        <v/>
+      </c>
+      <c r="M46" s="24">
+        <f>IF(ISNUMBER(J46),L46/G46,"")</f>
+        <v/>
+      </c>
+      <c r="N46" s="25">
+        <f>IF(ISNUMBER(H46),H46-C46,"")</f>
+        <v/>
+      </c>
+      <c r="O46" s="6" t="n"/>
+      <c r="P46" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Analog Devices, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="n">
+        <v>46324.6062962963</v>
+      </c>
+      <c r="D47" s="22" t="n">
+        <v>46324.39796296296</v>
+      </c>
+      <c r="E47" s="17" t="n">
+        <v>427.19138</v>
+      </c>
+      <c r="F47" s="16" t="n">
+        <v>19.536817436</v>
+      </c>
+      <c r="G47" s="17">
+        <f>E47*F47</f>
+        <v/>
+      </c>
+      <c r="H47" s="22" t="n"/>
+      <c r="I47" s="22" t="n"/>
+      <c r="J47" s="17" t="n"/>
+      <c r="K47" s="17">
+        <f>IF(ISNUMBER(J47),J47*F47,"")</f>
+        <v/>
+      </c>
+      <c r="L47" s="23">
+        <f>IF(ISNUMBER(J47),K47-G47,"")</f>
+        <v/>
+      </c>
+      <c r="M47" s="24">
+        <f>IF(ISNUMBER(J47),L47/G47,"")</f>
+        <v/>
+      </c>
+      <c r="N47" s="25">
+        <f>IF(ISNUMBER(H47),H47-C47,"")</f>
+        <v/>
+      </c>
+      <c r="O47" s="6" t="n"/>
+      <c r="P47" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>MARATHON PETROLEUM CORPORATION</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="n">
+        <v>46324.60640046297</v>
+      </c>
+      <c r="D48" s="22" t="n">
+        <v>46324.39806712963</v>
+      </c>
+      <c r="E48" s="17" t="n">
+        <v>442.839476</v>
+      </c>
+      <c r="F48" s="16" t="n">
+        <v>18.846467973</v>
+      </c>
+      <c r="G48" s="17">
+        <f>E48*F48</f>
+        <v/>
+      </c>
+      <c r="H48" s="22" t="n"/>
+      <c r="I48" s="22" t="n"/>
+      <c r="J48" s="17" t="n"/>
+      <c r="K48" s="17">
+        <f>IF(ISNUMBER(J48),J48*F48,"")</f>
+        <v/>
+      </c>
+      <c r="L48" s="23">
+        <f>IF(ISNUMBER(J48),K48-G48,"")</f>
+        <v/>
+      </c>
+      <c r="M48" s="24">
+        <f>IF(ISNUMBER(J48),L48/G48,"")</f>
+        <v/>
+      </c>
+      <c r="N48" s="25">
+        <f>IF(ISNUMBER(H48),H48-C48,"")</f>
+        <v/>
+      </c>
+      <c r="O48" s="6" t="n"/>
+      <c r="P48" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Intuitive Surgical, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="n">
+        <v>46324.60655092593</v>
+      </c>
+      <c r="D49" s="22" t="n">
+        <v>46324.39821759259</v>
+      </c>
+      <c r="E49" s="17" t="n">
+        <v>447.607374</v>
+      </c>
+      <c r="F49" s="16" t="n">
+        <v>18.645716072</v>
+      </c>
+      <c r="G49" s="17">
+        <f>E49*F49</f>
+        <v/>
+      </c>
+      <c r="H49" s="22" t="n"/>
+      <c r="I49" s="22" t="n"/>
+      <c r="J49" s="17" t="n"/>
+      <c r="K49" s="17">
+        <f>IF(ISNUMBER(J49),J49*F49,"")</f>
+        <v/>
+      </c>
+      <c r="L49" s="23">
+        <f>IF(ISNUMBER(J49),K49-G49,"")</f>
+        <v/>
+      </c>
+      <c r="M49" s="24">
+        <f>IF(ISNUMBER(J49),L49/G49,"")</f>
+        <v/>
+      </c>
+      <c r="N49" s="25">
+        <f>IF(ISNUMBER(H49),H49-C49,"")</f>
+        <v/>
+      </c>
+      <c r="O49" s="6" t="n"/>
+      <c r="P49" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Public Limited Company Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="n">
+        <v>46324.60677083334</v>
+      </c>
+      <c r="D50" s="22" t="n">
+        <v>46324.3984375</v>
+      </c>
+      <c r="E50" s="17" t="n">
+        <v>320.034243</v>
+      </c>
+      <c r="F50" s="16" t="n">
+        <v>26.078334421</v>
+      </c>
+      <c r="G50" s="17">
+        <f>E50*F50</f>
+        <v/>
+      </c>
+      <c r="H50" s="22" t="n"/>
+      <c r="I50" s="22" t="n"/>
+      <c r="J50" s="17" t="n"/>
+      <c r="K50" s="17">
+        <f>IF(ISNUMBER(J50),J50*F50,"")</f>
+        <v/>
+      </c>
+      <c r="L50" s="23">
+        <f>IF(ISNUMBER(J50),K50-G50,"")</f>
+        <v/>
+      </c>
+      <c r="M50" s="24">
+        <f>IF(ISNUMBER(J50),L50/G50,"")</f>
+        <v/>
+      </c>
+      <c r="N50" s="25">
+        <f>IF(ISNUMBER(H50),H50-C50,"")</f>
+        <v/>
+      </c>
+      <c r="O50" s="6" t="n"/>
+      <c r="P50" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific, Inc.</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="n">
+        <v>46324.60688657407</v>
+      </c>
+      <c r="D51" s="22" t="n">
+        <v>46324.39855324074</v>
+      </c>
+      <c r="E51" s="17" t="n">
+        <v>704.202253</v>
+      </c>
+      <c r="F51" s="16" t="n">
+        <v>11.851651941</v>
+      </c>
+      <c r="G51" s="17">
+        <f>E51*F51</f>
+        <v/>
+      </c>
+      <c r="H51" s="22" t="n"/>
+      <c r="I51" s="22" t="n"/>
+      <c r="J51" s="17" t="n"/>
+      <c r="K51" s="17">
+        <f>IF(ISNUMBER(J51),J51*F51,"")</f>
+        <v/>
+      </c>
+      <c r="L51" s="23">
+        <f>IF(ISNUMBER(J51),K51-G51,"")</f>
+        <v/>
+      </c>
+      <c r="M51" s="24">
+        <f>IF(ISNUMBER(J51),L51/G51,"")</f>
+        <v/>
+      </c>
+      <c r="N51" s="25">
+        <f>IF(ISNUMBER(H51),H51-C51,"")</f>
+        <v/>
+      </c>
+      <c r="O51" s="6" t="n"/>
+      <c r="P51" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>McKesson Corporation</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="n">
+        <v>46324.60704861111</v>
+      </c>
+      <c r="D52" s="22" t="n">
+        <v>46324.39871527778</v>
+      </c>
+      <c r="E52" s="17" t="n">
+        <v>975.351467</v>
+      </c>
+      <c r="F52" s="16" t="n">
+        <v>8.556874402</v>
+      </c>
+      <c r="G52" s="17">
+        <f>E52*F52</f>
+        <v/>
+      </c>
+      <c r="H52" s="22" t="n"/>
+      <c r="I52" s="22" t="n"/>
+      <c r="J52" s="17" t="n"/>
+      <c r="K52" s="17">
+        <f>IF(ISNUMBER(J52),J52*F52,"")</f>
+        <v/>
+      </c>
+      <c r="L52" s="23">
+        <f>IF(ISNUMBER(J52),K52-G52,"")</f>
+        <v/>
+      </c>
+      <c r="M52" s="24">
+        <f>IF(ISNUMBER(J52),L52/G52,"")</f>
+        <v/>
+      </c>
+      <c r="N52" s="25">
+        <f>IF(ISNUMBER(H52),H52-C52,"")</f>
+        <v/>
+      </c>
+      <c r="O52" s="6" t="n"/>
+      <c r="P52" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Natera, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="n">
+        <v>46324.60716435185</v>
+      </c>
+      <c r="D53" s="22" t="n">
+        <v>46324.39883101852</v>
+      </c>
+      <c r="E53" s="17" t="n">
+        <v>424.844876</v>
+      </c>
+      <c r="F53" s="16" t="n">
+        <v>19.644723215</v>
+      </c>
+      <c r="G53" s="17">
+        <f>E53*F53</f>
+        <v/>
+      </c>
+      <c r="H53" s="22" t="n"/>
+      <c r="I53" s="22" t="n"/>
+      <c r="J53" s="17" t="n"/>
+      <c r="K53" s="17">
+        <f>IF(ISNUMBER(J53),J53*F53,"")</f>
+        <v/>
+      </c>
+      <c r="L53" s="23">
+        <f>IF(ISNUMBER(J53),K53-G53,"")</f>
+        <v/>
+      </c>
+      <c r="M53" s="24">
+        <f>IF(ISNUMBER(J53),L53/G53,"")</f>
+        <v/>
+      </c>
+      <c r="N53" s="25">
+        <f>IF(ISNUMBER(H53),H53-C53,"")</f>
+        <v/>
+      </c>
+      <c r="O53" s="6" t="n"/>
+      <c r="P53" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="C54" s="22" t="n">
+        <v>46324.60722222222</v>
+      </c>
+      <c r="D54" s="22" t="n">
+        <v>46324.39888888889</v>
+      </c>
+      <c r="E54" s="17" t="n">
+        <v>639.369739</v>
+      </c>
+      <c r="F54" s="16" t="n">
+        <v>13.053417297</v>
+      </c>
+      <c r="G54" s="17">
+        <f>E54*F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="22" t="n"/>
+      <c r="I54" s="22" t="n"/>
+      <c r="J54" s="17" t="n"/>
+      <c r="K54" s="17">
+        <f>IF(ISNUMBER(J54),J54*F54,"")</f>
+        <v/>
+      </c>
+      <c r="L54" s="23">
+        <f>IF(ISNUMBER(J54),K54-G54,"")</f>
+        <v/>
+      </c>
+      <c r="M54" s="24">
+        <f>IF(ISNUMBER(J54),L54/G54,"")</f>
+        <v/>
+      </c>
+      <c r="N54" s="25">
+        <f>IF(ISNUMBER(H54),H54-C54,"")</f>
+        <v/>
+      </c>
+      <c r="O54" s="6" t="n"/>
+      <c r="P54" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M42">
+  <conditionalFormatting sqref="L2:M54">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 15:11 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA87" headerRowCount="1">
-  <autoFilter ref="A1:BA87"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA88" headerRowCount="1">
+  <autoFilter ref="A1:BA88"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.60924768518</v>
+        <v>46324.67479166666</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.40091435185</v>
+        <v>46324.46645833334</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$87,"BUY")+COUNTIF(Orders!$E$2:$E$87,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$88,"BUY")+COUNTIF(Orders!$E$2:$E$88,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$87,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$88,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$87,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$88,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$87,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$88,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$87,Orders!$E$2:$E$87,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$88,Orders!$E$2:$E$88,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$87,Orders!$E$2:$E$87,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$88,Orders!$E$2:$E$88,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA87"/>
+  <dimension ref="A1:BA88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14828,6 +14828,194 @@
       </c>
       <c r="BA87" s="6" t="n"/>
     </row>
+    <row r="88">
+      <c r="A88" s="12" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="13" t="n">
+        <v>46324.6747337963</v>
+      </c>
+      <c r="C88" s="13" t="n">
+        <v>46324.46640046296</v>
+      </c>
+      <c r="D88" s="13" t="n">
+        <v>46324.63306712963</v>
+      </c>
+      <c r="E88" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="G88" s="15" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J88" s="16" t="n">
+        <v>18.846467973</v>
+      </c>
+      <c r="K88" s="17" t="n">
+        <v>421.33</v>
+      </c>
+      <c r="L88" s="17">
+        <f>IF(AND(ISNUMBER(J88),ISNUMBER(K88)),J88*K88,"")</f>
+        <v/>
+      </c>
+      <c r="M88" s="17" t="n"/>
+      <c r="N88" s="16" t="n">
+        <v>18.846467973</v>
+      </c>
+      <c r="O88" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P88" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 4.3% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q88" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R88" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S88" s="18" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="T88" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="U88" s="19" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="V88" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W88" s="12" t="n"/>
+      <c r="X88" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y88" s="19" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="Z88" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA88" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB88" s="15" t="n"/>
+      <c r="AC88" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD88" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE88" s="17" t="n">
+        <v>431.5162</v>
+      </c>
+      <c r="AF88" s="17" t="n">
+        <v>408.3508</v>
+      </c>
+      <c r="AG88" s="17" t="n">
+        <v>454.6815</v>
+      </c>
+      <c r="AH88" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI88" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ88" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK88" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL88" s="15" t="inlineStr">
+        <is>
+          <t>Reported Earlier, Marathon Petroleum Raises Quarterly Dividend 10% To $1.10 Per Share From $1.00, Payable Dec. 10, 2026, To Shareholders Of Record As Of Nov. 18</t>
+        </is>
+      </c>
+      <c r="AM88" s="17" t="n">
+        <v>422.25</v>
+      </c>
+      <c r="AN88" s="19" t="n">
+        <v>-0.0417</v>
+      </c>
+      <c r="AO88" s="17" t="n">
+        <v>99315.96000000001</v>
+      </c>
+      <c r="AP88" s="17" t="n">
+        <v>40.27</v>
+      </c>
+      <c r="AQ88" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR88" s="16" t="n">
+        <v>18.846467973</v>
+      </c>
+      <c r="AS88" s="17" t="n">
+        <v>442.839476</v>
+      </c>
+      <c r="AT88" s="19" t="n">
+        <v>-0.0476</v>
+      </c>
+      <c r="AU88" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV88" s="6" t="inlineStr">
+        <is>
+          <t>ffdb00ef-b2db-4f38-8488-0fe2b35782a8</t>
+        </is>
+      </c>
+      <c r="AW88" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-MPC-1793286695996</t>
+        </is>
+      </c>
+      <c r="AX88" s="13" t="n">
+        <v>46324.63304398148</v>
+      </c>
+      <c r="AY88" s="13" t="n">
+        <v>46324.63306712963</v>
+      </c>
+      <c r="AZ88" s="13" t="n">
+        <v>46324.63278935185</v>
+      </c>
+      <c r="BA88" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -17821,9 +18009,15 @@
         <f>E48*F48</f>
         <v/>
       </c>
-      <c r="H48" s="22" t="n"/>
-      <c r="I48" s="22" t="n"/>
-      <c r="J48" s="17" t="n"/>
+      <c r="H48" s="22" t="n">
+        <v>46324.6747337963</v>
+      </c>
+      <c r="I48" s="22" t="n">
+        <v>46324.46640046296</v>
+      </c>
+      <c r="J48" s="17" t="n">
+        <v>421.33</v>
+      </c>
       <c r="K48" s="17">
         <f>IF(ISNUMBER(J48),J48*F48,"")</f>
         <v/>
@@ -17840,10 +18034,14 @@
         <f>IF(ISNUMBER(H48),H48-C48,"")</f>
         <v/>
       </c>
-      <c r="O48" s="6" t="n"/>
+      <c r="O48" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P48" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-29 15:17 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA88" headerRowCount="1">
-  <autoFilter ref="A1:BA88"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA100" headerRowCount="1">
+  <autoFilter ref="A1:BA100"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P54" headerRowCount="1">
-  <autoFilter ref="A1:P54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P66" headerRowCount="1">
+  <autoFilter ref="A1:P66"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.67479166666</v>
+        <v>46324.67849537037</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.46645833334</v>
+        <v>46324.47016203704</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$88,"BUY")+COUNTIF(Orders!$E$2:$E$88,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$100,"BUY")+COUNTIF(Orders!$E$2:$E$100,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$88,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$100,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$88,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$100,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$88,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$100,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$88,Orders!$E$2:$E$88,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$100,Orders!$E$2:$E$100,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$88,Orders!$E$2:$E$88,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$100,Orders!$E$2:$E$100,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$54,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$66,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$54,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$66,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$54)</f>
+        <f>SUM('Round trips'!$L$2:$L$66)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$54,"Closed",'Round trips'!$L$2:$L$54,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$66,"Closed",'Round trips'!$L$2:$L$66,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA88"/>
+  <dimension ref="A1:BA100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -15016,6 +15016,2214 @@
       </c>
       <c r="BA88" s="6" t="n"/>
     </row>
+    <row r="89">
+      <c r="A89" s="12" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="13" t="n">
+        <v>46324.67833333334</v>
+      </c>
+      <c r="C89" s="13" t="n">
+        <v>46324.47</v>
+      </c>
+      <c r="D89" s="13" t="n">
+        <v>46324.63666666667</v>
+      </c>
+      <c r="E89" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="G89" s="15" t="inlineStr">
+        <is>
+          <t>Veeva Systems Inc.</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J89" s="16" t="n">
+        <v>2.132719514</v>
+      </c>
+      <c r="K89" s="17" t="n">
+        <v>311.71</v>
+      </c>
+      <c r="L89" s="17">
+        <f>IF(AND(ISNUMBER(J89),ISNUMBER(K89)),J89*K89,"")</f>
+        <v/>
+      </c>
+      <c r="M89" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N89" s="16" t="n"/>
+      <c r="O89" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P89" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q89" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R89" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S89" s="18" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="T89" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="U89" s="19" t="n">
+        <v>0.0567</v>
+      </c>
+      <c r="V89" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W89" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X89" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y89" s="19" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="Z89" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA89" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB89" s="15" t="n"/>
+      <c r="AC89" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD89" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE89" s="17" t="n">
+        <v>319.9537</v>
+      </c>
+      <c r="AF89" s="17" t="n">
+        <v>300.332</v>
+      </c>
+      <c r="AG89" s="17" t="n">
+        <v>339.5754</v>
+      </c>
+      <c r="AH89" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI89" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ89" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK89" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL89" s="15" t="inlineStr">
+        <is>
+          <t>Mizuho Adjusts Price Target on Veeva Systems</t>
+        </is>
+      </c>
+      <c r="AM89" s="17" t="n">
+        <v>311.6</v>
+      </c>
+      <c r="AN89" s="19" t="n">
+        <v>-0.0183</v>
+      </c>
+      <c r="AO89" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP89" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ89" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR89" s="16" t="n"/>
+      <c r="AS89" s="17" t="n"/>
+      <c r="AT89" s="19" t="n"/>
+      <c r="AU89" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV89" s="6" t="inlineStr">
+        <is>
+          <t>432ddb49-7fbc-49b5-9550-5546f03e0680</t>
+        </is>
+      </c>
+      <c r="AW89" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-VEEV-1793287007828</t>
+        </is>
+      </c>
+      <c r="AX89" s="13" t="n">
+        <v>46324.6366550926</v>
+      </c>
+      <c r="AY89" s="13" t="n">
+        <v>46324.63666666667</v>
+      </c>
+      <c r="AZ89" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA89" s="6" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="13" t="n">
+        <v>46324.67834490741</v>
+      </c>
+      <c r="C90" s="13" t="n">
+        <v>46324.47001157407</v>
+      </c>
+      <c r="D90" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="E90" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="G90" s="15" t="inlineStr">
+        <is>
+          <t>Avantor, Inc.</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I90" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J90" s="16" t="n">
+        <v>40.314736203</v>
+      </c>
+      <c r="K90" s="17" t="n">
+        <v>16.49</v>
+      </c>
+      <c r="L90" s="17">
+        <f>IF(AND(ISNUMBER(J90),ISNUMBER(K90)),J90*K90,"")</f>
+        <v/>
+      </c>
+      <c r="M90" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N90" s="16" t="n"/>
+      <c r="O90" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P90" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #2, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q90" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R90" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S90" s="18" t="n">
+        <v>0.823</v>
+      </c>
+      <c r="T90" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="U90" s="19" t="n">
+        <v>0.0453</v>
+      </c>
+      <c r="V90" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W90" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="X90" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y90" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z90" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA90" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB90" s="15" t="n"/>
+      <c r="AC90" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD90" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE90" s="17" t="n">
+        <v>16.739</v>
+      </c>
+      <c r="AF90" s="17" t="n">
+        <v>16.0789</v>
+      </c>
+      <c r="AG90" s="17" t="n">
+        <v>17.3992</v>
+      </c>
+      <c r="AH90" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI90" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ90" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK90" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL90" s="15" t="inlineStr">
+        <is>
+          <t>Barclays Maintains Underweight on Avantor, Raises Price Target to $16</t>
+        </is>
+      </c>
+      <c r="AM90" s="17" t="n">
+        <v>16.47</v>
+      </c>
+      <c r="AN90" s="19" t="n">
+        <v>-0.0123</v>
+      </c>
+      <c r="AO90" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP90" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ90" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR90" s="16" t="n"/>
+      <c r="AS90" s="17" t="n"/>
+      <c r="AT90" s="19" t="n"/>
+      <c r="AU90" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV90" s="6" t="inlineStr">
+        <is>
+          <t>2846835a-3061-47df-84bc-c57549c0d863</t>
+        </is>
+      </c>
+      <c r="AW90" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-AVTR-1793287008089</t>
+        </is>
+      </c>
+      <c r="AX90" s="13" t="n">
+        <v>46324.63666666667</v>
+      </c>
+      <c r="AY90" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="AZ90" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA90" s="6" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="13" t="n">
+        <v>46324.67834490741</v>
+      </c>
+      <c r="C91" s="13" t="n">
+        <v>46324.47001157407</v>
+      </c>
+      <c r="D91" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="E91" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="G91" s="15" t="inlineStr">
+        <is>
+          <t>ABBVIE INC.</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I91" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J91" s="16" t="n">
+        <v>2.290483737</v>
+      </c>
+      <c r="K91" s="17" t="n">
+        <v>290.24</v>
+      </c>
+      <c r="L91" s="17">
+        <f>IF(AND(ISNUMBER(J91),ISNUMBER(K91)),J91*K91,"")</f>
+        <v/>
+      </c>
+      <c r="M91" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N91" s="16" t="n"/>
+      <c r="O91" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P91" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #3, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q91" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R91" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S91" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T91" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U91" s="19" t="n">
+        <v>0.0177</v>
+      </c>
+      <c r="V91" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W91" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X91" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y91" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z91" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA91" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB91" s="15" t="n"/>
+      <c r="AC91" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD91" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE91" s="17" t="n">
+        <v>293.3377</v>
+      </c>
+      <c r="AF91" s="17" t="n">
+        <v>285.3184</v>
+      </c>
+      <c r="AG91" s="17" t="n">
+        <v>301.3571</v>
+      </c>
+      <c r="AH91" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI91" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ91" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK91" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL91" s="15" t="inlineStr">
+        <is>
+          <t>Steve Jobs' Son Says GLP-1 Weight Loss Drugs Could Be Among Most Important Medicines Ever, With Potential Impact on Cancer</t>
+        </is>
+      </c>
+      <c r="AM91" s="17" t="n">
+        <v>290.1</v>
+      </c>
+      <c r="AN91" s="19" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="AO91" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP91" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ91" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR91" s="16" t="n"/>
+      <c r="AS91" s="17" t="n"/>
+      <c r="AT91" s="19" t="n"/>
+      <c r="AU91" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV91" s="6" t="inlineStr">
+        <is>
+          <t>6e3e1966-fed1-4e2c-8f60-4d6a94ba2b8f</t>
+        </is>
+      </c>
+      <c r="AW91" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ABBV-1793287008370</t>
+        </is>
+      </c>
+      <c r="AX91" s="13" t="n">
+        <v>46324.63666666667</v>
+      </c>
+      <c r="AY91" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="AZ91" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA91" s="6" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="12" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="13" t="n">
+        <v>46324.67834490741</v>
+      </c>
+      <c r="C92" s="13" t="n">
+        <v>46324.47001157407</v>
+      </c>
+      <c r="D92" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="E92" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="G92" s="15" t="inlineStr">
+        <is>
+          <t>ExxonMobil Holdings Corporation</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J92" s="16" t="n">
+        <v>3.658320493</v>
+      </c>
+      <c r="K92" s="17" t="n">
+        <v>181.72</v>
+      </c>
+      <c r="L92" s="17">
+        <f>IF(AND(ISNUMBER(J92),ISNUMBER(K92)),J92*K92,"")</f>
+        <v/>
+      </c>
+      <c r="M92" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N92" s="16" t="n"/>
+      <c r="O92" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P92" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q92" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R92" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S92" s="18" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="T92" s="12" t="n">
+        <v>93</v>
+      </c>
+      <c r="U92" s="19" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="V92" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W92" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X92" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y92" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z92" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA92" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB92" s="15" t="n"/>
+      <c r="AC92" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD92" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE92" s="17" t="n">
+        <v>184.0513</v>
+      </c>
+      <c r="AF92" s="17" t="n">
+        <v>177.9106</v>
+      </c>
+      <c r="AG92" s="17" t="n">
+        <v>190.1919</v>
+      </c>
+      <c r="AH92" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI92" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ92" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK92" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL92" s="15" t="inlineStr">
+        <is>
+          <t>Top 3 Energy Stocks You May Want To Dump In Q4</t>
+        </is>
+      </c>
+      <c r="AM92" s="17" t="n">
+        <v>181.595</v>
+      </c>
+      <c r="AN92" s="19" t="n">
+        <v>-0.0027</v>
+      </c>
+      <c r="AO92" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP92" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ92" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR92" s="16" t="n"/>
+      <c r="AS92" s="17" t="n"/>
+      <c r="AT92" s="19" t="n"/>
+      <c r="AU92" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV92" s="6" t="inlineStr">
+        <is>
+          <t>894141b0-8346-46b3-a49c-bbf0dbf99138</t>
+        </is>
+      </c>
+      <c r="AW92" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-XOM-1793287008620</t>
+        </is>
+      </c>
+      <c r="AX92" s="13" t="n">
+        <v>46324.63666666667</v>
+      </c>
+      <c r="AY92" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="AZ92" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA92" s="6" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="12" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="13" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="C93" s="13" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="D93" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="E93" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="G93" s="15" t="inlineStr">
+        <is>
+          <t>Dynatrace, Inc.</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I93" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J93" s="16" t="n">
+        <v>10.943045267</v>
+      </c>
+      <c r="K93" s="17" t="n">
+        <v>60.75</v>
+      </c>
+      <c r="L93" s="17">
+        <f>IF(AND(ISNUMBER(J93),ISNUMBER(K93)),J93*K93,"")</f>
+        <v/>
+      </c>
+      <c r="M93" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N93" s="16" t="n"/>
+      <c r="O93" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P93" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #5, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q93" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R93" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S93" s="18" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="T93" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="U93" s="19" t="n">
+        <v>0.0125</v>
+      </c>
+      <c r="V93" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W93" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X93" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y93" s="19" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="Z93" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA93" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB93" s="15" t="n"/>
+      <c r="AC93" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD93" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE93" s="17" t="n">
+        <v>62.0102</v>
+      </c>
+      <c r="AF93" s="17" t="n">
+        <v>59.0097</v>
+      </c>
+      <c r="AG93" s="17" t="n">
+        <v>65.0106</v>
+      </c>
+      <c r="AH93" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI93" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ93" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK93" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL93" s="15" t="inlineStr">
+        <is>
+          <t>Rosenblatt Maintains Buy on Dynatrace, Raises Price Target to $70</t>
+        </is>
+      </c>
+      <c r="AM93" s="17" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="AN93" s="19" t="n">
+        <v>-0.0329</v>
+      </c>
+      <c r="AO93" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP93" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ93" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR93" s="16" t="n"/>
+      <c r="AS93" s="17" t="n"/>
+      <c r="AT93" s="19" t="n"/>
+      <c r="AU93" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV93" s="6" t="inlineStr">
+        <is>
+          <t>80a8cba4-7fd6-4ee7-9cb9-d4b67e28d726</t>
+        </is>
+      </c>
+      <c r="AW93" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-DT-1793287008877</t>
+        </is>
+      </c>
+      <c r="AX93" s="13" t="n">
+        <v>46324.63666666667</v>
+      </c>
+      <c r="AY93" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AZ93" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA93" s="6" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="13" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="C94" s="13" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="D94" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="E94" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F94" s="6" t="inlineStr">
+        <is>
+          <t>DUK</t>
+        </is>
+      </c>
+      <c r="G94" s="15" t="inlineStr">
+        <is>
+          <t>Duke Energy Corporation</t>
+        </is>
+      </c>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J94" s="16" t="n">
+        <v>5.287020836</v>
+      </c>
+      <c r="K94" s="17" t="n">
+        <v>125.74</v>
+      </c>
+      <c r="L94" s="17">
+        <f>IF(AND(ISNUMBER(J94),ISNUMBER(K94)),J94*K94,"")</f>
+        <v/>
+      </c>
+      <c r="M94" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N94" s="16" t="n"/>
+      <c r="O94" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P94" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #6, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q94" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R94" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S94" s="18" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="T94" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="U94" s="19" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="V94" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W94" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="X94" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y94" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z94" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA94" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB94" s="15" t="n"/>
+      <c r="AC94" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD94" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE94" s="17" t="n">
+        <v>126.9377</v>
+      </c>
+      <c r="AF94" s="17" t="n">
+        <v>123.8434</v>
+      </c>
+      <c r="AG94" s="17" t="n">
+        <v>130.032</v>
+      </c>
+      <c r="AH94" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI94" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ94" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK94" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL94" s="15" t="inlineStr">
+        <is>
+          <t>Duke Energy Updates Emergency Planning Zones for Brunswick Nuclear Plant</t>
+        </is>
+      </c>
+      <c r="AM94" s="17" t="n">
+        <v>125.7</v>
+      </c>
+      <c r="AN94" s="19" t="n">
+        <v>0.0167</v>
+      </c>
+      <c r="AO94" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP94" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ94" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR94" s="16" t="n"/>
+      <c r="AS94" s="17" t="n"/>
+      <c r="AT94" s="19" t="n"/>
+      <c r="AU94" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV94" s="6" t="inlineStr">
+        <is>
+          <t>584d2887-04f8-4615-a1fa-d901e34e2f86</t>
+        </is>
+      </c>
+      <c r="AW94" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-DUK-1793287009163</t>
+        </is>
+      </c>
+      <c r="AX94" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="AY94" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AZ94" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA94" s="6" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="12" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="13" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="C95" s="13" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="D95" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="E95" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="G95" s="15" t="inlineStr">
+        <is>
+          <t>The Kroger Co.</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I95" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J95" s="16" t="n">
+        <v>10.152565668</v>
+      </c>
+      <c r="K95" s="17" t="n">
+        <v>65.48</v>
+      </c>
+      <c r="L95" s="17">
+        <f>IF(AND(ISNUMBER(J95),ISNUMBER(K95)),J95*K95,"")</f>
+        <v/>
+      </c>
+      <c r="M95" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N95" s="16" t="n"/>
+      <c r="O95" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P95" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #7, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q95" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R95" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S95" s="18" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="T95" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U95" s="19" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="V95" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W95" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="X95" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y95" s="19" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="Z95" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA95" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB95" s="15" t="n"/>
+      <c r="AC95" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD95" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE95" s="17" t="n">
+        <v>66.5149</v>
+      </c>
+      <c r="AF95" s="17" t="n">
+        <v>63.9026</v>
+      </c>
+      <c r="AG95" s="17" t="n">
+        <v>69.12730000000001</v>
+      </c>
+      <c r="AH95" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI95" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ95" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK95" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL95" s="15" t="inlineStr">
+        <is>
+          <t>Kroger Announces High Critical Ratings for Exclusive Wine Portfolio</t>
+        </is>
+      </c>
+      <c r="AM95" s="17" t="n">
+        <v>65.47</v>
+      </c>
+      <c r="AN95" s="19" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="AO95" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP95" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ95" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR95" s="16" t="n"/>
+      <c r="AS95" s="17" t="n"/>
+      <c r="AT95" s="19" t="n"/>
+      <c r="AU95" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV95" s="6" t="inlineStr">
+        <is>
+          <t>aeb6105c-3950-4bf5-801f-10b147dce0b5</t>
+        </is>
+      </c>
+      <c r="AW95" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-KR-1793287009428</t>
+        </is>
+      </c>
+      <c r="AX95" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="AY95" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AZ95" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA95" s="6" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="13" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="C96" s="13" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="D96" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="E96" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="G96" s="15" t="inlineStr">
+        <is>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+        </is>
+      </c>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I96" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J96" s="16" t="n">
+        <v>6.184668341</v>
+      </c>
+      <c r="K96" s="17" t="n">
+        <v>107.49</v>
+      </c>
+      <c r="L96" s="17">
+        <f>IF(AND(ISNUMBER(J96),ISNUMBER(K96)),J96*K96,"")</f>
+        <v/>
+      </c>
+      <c r="M96" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N96" s="16" t="n"/>
+      <c r="O96" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P96" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #8, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q96" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R96" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S96" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T96" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="U96" s="19" t="n">
+        <v>0.0127</v>
+      </c>
+      <c r="V96" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W96" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="X96" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y96" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z96" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA96" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB96" s="15" t="n"/>
+      <c r="AC96" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD96" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE96" s="17" t="n">
+        <v>108.6361</v>
+      </c>
+      <c r="AF96" s="17" t="n">
+        <v>105.5708</v>
+      </c>
+      <c r="AG96" s="17" t="n">
+        <v>111.7015</v>
+      </c>
+      <c r="AH96" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI96" s="18" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AJ96" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK96" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL96" s="15" t="inlineStr">
+        <is>
+          <t>Shell Q3 Earnings Reach Highest Level Since 2022 Amid Middle-East Turmoil</t>
+        </is>
+      </c>
+      <c r="AM96" s="17" t="n">
+        <v>107.405</v>
+      </c>
+      <c r="AN96" s="19" t="n">
+        <v>0.0219</v>
+      </c>
+      <c r="AO96" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP96" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ96" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR96" s="16" t="n"/>
+      <c r="AS96" s="17" t="n"/>
+      <c r="AT96" s="19" t="n"/>
+      <c r="AU96" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV96" s="6" t="inlineStr">
+        <is>
+          <t>aa029f26-64e4-4ab1-b405-70dc8dc432cc</t>
+        </is>
+      </c>
+      <c r="AW96" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-SHEL-1793287009677</t>
+        </is>
+      </c>
+      <c r="AX96" s="13" t="n">
+        <v>46324.63667824074</v>
+      </c>
+      <c r="AY96" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AZ96" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA96" s="6" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="12" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="13" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="C97" s="13" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="D97" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="E97" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="G97" s="15" t="inlineStr">
+        <is>
+          <t>Illumina, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H97" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J97" s="16" t="n">
+        <v>2.303818963</v>
+      </c>
+      <c r="K97" s="17" t="n">
+        <v>288.56</v>
+      </c>
+      <c r="L97" s="17">
+        <f>IF(AND(ISNUMBER(J97),ISNUMBER(K97)),J97*K97,"")</f>
+        <v/>
+      </c>
+      <c r="M97" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N97" s="16" t="n"/>
+      <c r="O97" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P97" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #10, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q97" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R97" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S97" s="18" t="n">
+        <v>0.595</v>
+      </c>
+      <c r="T97" s="12" t="n">
+        <v>126</v>
+      </c>
+      <c r="U97" s="19" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="V97" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W97" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="X97" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y97" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z97" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA97" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB97" s="15" t="n"/>
+      <c r="AC97" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD97" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE97" s="17" t="n">
+        <v>296.6903</v>
+      </c>
+      <c r="AF97" s="17" t="n">
+        <v>275.5645</v>
+      </c>
+      <c r="AG97" s="17" t="n">
+        <v>317.8161</v>
+      </c>
+      <c r="AH97" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI97" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ97" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK97" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL97" s="15" t="inlineStr">
+        <is>
+          <t>Amazon, Eli Lilly On Deck Thursday As AWS Growth, Drug Demand Face Test</t>
+        </is>
+      </c>
+      <c r="AM97" s="17" t="n">
+        <v>288.24</v>
+      </c>
+      <c r="AN97" s="19" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="AO97" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP97" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ97" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR97" s="16" t="n"/>
+      <c r="AS97" s="17" t="n"/>
+      <c r="AT97" s="19" t="n"/>
+      <c r="AU97" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV97" s="6" t="inlineStr">
+        <is>
+          <t>31d91322-0a25-4696-abe1-71b5cad5972d</t>
+        </is>
+      </c>
+      <c r="AW97" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ILMN-1793287010075</t>
+        </is>
+      </c>
+      <c r="AX97" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AY97" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AZ97" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA97" s="6" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="12" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="13" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="C98" s="13" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="D98" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="E98" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="G98" s="15" t="inlineStr">
+        <is>
+          <t>Accenture PLC</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J98" s="16" t="n">
+        <v>2.726336942</v>
+      </c>
+      <c r="K98" s="17" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="L98" s="17">
+        <f>IF(AND(ISNUMBER(J98),ISNUMBER(K98)),J98*K98,"")</f>
+        <v/>
+      </c>
+      <c r="M98" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N98" s="16" t="n"/>
+      <c r="O98" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P98" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #12, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q98" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R98" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S98" s="18" t="n">
+        <v>0.551</v>
+      </c>
+      <c r="T98" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="U98" s="19" t="n">
+        <v>0.0072</v>
+      </c>
+      <c r="V98" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W98" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="X98" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y98" s="19" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="Z98" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA98" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB98" s="15" t="n"/>
+      <c r="AC98" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD98" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE98" s="17" t="n">
+        <v>250.9857</v>
+      </c>
+      <c r="AF98" s="17" t="n">
+        <v>232.234</v>
+      </c>
+      <c r="AG98" s="17" t="n">
+        <v>269.7373</v>
+      </c>
+      <c r="AH98" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI98" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ98" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK98" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL98" s="15" t="inlineStr">
+        <is>
+          <t>Accenture Recognized in 2026 Guidewire PartnerConnect Excellence Awards</t>
+        </is>
+      </c>
+      <c r="AM98" s="17" t="n">
+        <v>243.485</v>
+      </c>
+      <c r="AN98" s="19" t="n">
+        <v>-0.0015</v>
+      </c>
+      <c r="AO98" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP98" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ98" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR98" s="16" t="n"/>
+      <c r="AS98" s="17" t="n"/>
+      <c r="AT98" s="19" t="n"/>
+      <c r="AU98" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV98" s="6" t="inlineStr">
+        <is>
+          <t>10044009-32c9-4f22-a20f-9acdfdd2b100</t>
+        </is>
+      </c>
+      <c r="AW98" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ACN-1793287010453</t>
+        </is>
+      </c>
+      <c r="AX98" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AY98" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AZ98" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA98" s="6" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="12" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="13" t="n">
+        <v>46324.67839120371</v>
+      </c>
+      <c r="C99" s="13" t="n">
+        <v>46324.47005787037</v>
+      </c>
+      <c r="D99" s="13" t="n">
+        <v>46324.63672453703</v>
+      </c>
+      <c r="E99" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="G99" s="15" t="inlineStr">
+        <is>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J99" s="16" t="n">
+        <v>14.117434699</v>
+      </c>
+      <c r="K99" s="17" t="n">
+        <v>47.09</v>
+      </c>
+      <c r="L99" s="17">
+        <f>IF(AND(ISNUMBER(J99),ISNUMBER(K99)),J99*K99,"")</f>
+        <v/>
+      </c>
+      <c r="M99" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N99" s="16" t="n"/>
+      <c r="O99" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P99" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #13, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q99" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R99" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S99" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T99" s="12" t="n">
+        <v>78</v>
+      </c>
+      <c r="U99" s="19" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="V99" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W99" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="X99" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y99" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z99" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA99" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB99" s="15" t="n"/>
+      <c r="AC99" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD99" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE99" s="17" t="n">
+        <v>47.9373</v>
+      </c>
+      <c r="AF99" s="17" t="n">
+        <v>45.7066</v>
+      </c>
+      <c r="AG99" s="17" t="n">
+        <v>50.1679</v>
+      </c>
+      <c r="AH99" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI99" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ99" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK99" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL99" s="15" t="inlineStr">
+        <is>
+          <t>Equinor Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM99" s="17" t="n">
+        <v>47.04</v>
+      </c>
+      <c r="AN99" s="19" t="n">
+        <v>-0.0129</v>
+      </c>
+      <c r="AO99" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP99" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ99" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR99" s="16" t="n"/>
+      <c r="AS99" s="17" t="n"/>
+      <c r="AT99" s="19" t="n"/>
+      <c r="AU99" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV99" s="6" t="inlineStr">
+        <is>
+          <t>e5e7881d-f385-4d1d-8fa7-1603b6afc37d</t>
+        </is>
+      </c>
+      <c r="AW99" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EQNR-1793287010714</t>
+        </is>
+      </c>
+      <c r="AX99" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AY99" s="13" t="n">
+        <v>46324.63672453703</v>
+      </c>
+      <c r="AZ99" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA99" s="6" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="12" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="13" t="n">
+        <v>46324.67836805555</v>
+      </c>
+      <c r="C100" s="13" t="n">
+        <v>46324.47003472222</v>
+      </c>
+      <c r="D100" s="13" t="n">
+        <v>46324.63670138889</v>
+      </c>
+      <c r="E100" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="G100" s="15" t="inlineStr">
+        <is>
+          <t>Linde plc Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J100" s="16" t="n">
+        <v>1.325708929</v>
+      </c>
+      <c r="K100" s="17" t="n">
+        <v>501.46</v>
+      </c>
+      <c r="L100" s="17">
+        <f>IF(AND(ISNUMBER(J100),ISNUMBER(K100)),J100*K100,"")</f>
+        <v/>
+      </c>
+      <c r="M100" s="17" t="n">
+        <v>664.8</v>
+      </c>
+      <c r="N100" s="16" t="n"/>
+      <c r="O100" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P100" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #14, 8.33% of the $7,980.85 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q100" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R100" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S100" s="18" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="T100" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="U100" s="19" t="n">
+        <v>0.0104</v>
+      </c>
+      <c r="V100" s="19" t="n">
+        <v>-0.1395</v>
+      </c>
+      <c r="W100" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="X100" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y100" s="19" t="n">
+        <v>0.0031</v>
+      </c>
+      <c r="Z100" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA100" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB100" s="15" t="n"/>
+      <c r="AC100" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD100" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE100" s="17" t="n">
+        <v>505.5059</v>
+      </c>
+      <c r="AF100" s="17" t="n">
+        <v>495.3912</v>
+      </c>
+      <c r="AG100" s="17" t="n">
+        <v>515.6206</v>
+      </c>
+      <c r="AH100" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI100" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ100" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK100" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL100" s="15" t="inlineStr">
+        <is>
+          <t>Linde Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM100" s="17" t="n">
+        <v>501.46</v>
+      </c>
+      <c r="AN100" s="19" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="AO100" s="17" t="n">
+        <v>99368.08</v>
+      </c>
+      <c r="AP100" s="17" t="n">
+        <v>7980.85</v>
+      </c>
+      <c r="AQ100" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR100" s="16" t="n"/>
+      <c r="AS100" s="17" t="n"/>
+      <c r="AT100" s="19" t="n"/>
+      <c r="AU100" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV100" s="6" t="inlineStr">
+        <is>
+          <t>6378bfbf-8394-4536-9bf4-aabfe70b3e4f</t>
+        </is>
+      </c>
+      <c r="AW100" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-LIN-1793287010962</t>
+        </is>
+      </c>
+      <c r="AX100" s="13" t="n">
+        <v>46324.63668981481</v>
+      </c>
+      <c r="AY100" s="13" t="n">
+        <v>46324.63670138889</v>
+      </c>
+      <c r="AZ100" s="13" t="n">
+        <v>46324.63631944444</v>
+      </c>
+      <c r="BA100" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -15031,7 +17239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -18363,8 +20571,644 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Veeva Systems Inc.</t>
+        </is>
+      </c>
+      <c r="C55" s="22" t="n">
+        <v>46324.67833333334</v>
+      </c>
+      <c r="D55" s="22" t="n">
+        <v>46324.47</v>
+      </c>
+      <c r="E55" s="17" t="n">
+        <v>311.71</v>
+      </c>
+      <c r="F55" s="16" t="n">
+        <v>2.132719514</v>
+      </c>
+      <c r="G55" s="17">
+        <f>E55*F55</f>
+        <v/>
+      </c>
+      <c r="H55" s="22" t="n"/>
+      <c r="I55" s="22" t="n"/>
+      <c r="J55" s="17" t="n"/>
+      <c r="K55" s="17">
+        <f>IF(ISNUMBER(J55),J55*F55,"")</f>
+        <v/>
+      </c>
+      <c r="L55" s="23">
+        <f>IF(ISNUMBER(J55),K55-G55,"")</f>
+        <v/>
+      </c>
+      <c r="M55" s="24">
+        <f>IF(ISNUMBER(J55),L55/G55,"")</f>
+        <v/>
+      </c>
+      <c r="N55" s="25">
+        <f>IF(ISNUMBER(H55),H55-C55,"")</f>
+        <v/>
+      </c>
+      <c r="O55" s="6" t="n"/>
+      <c r="P55" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>ABBVIE INC.</t>
+        </is>
+      </c>
+      <c r="C56" s="22" t="n">
+        <v>46324.67834490741</v>
+      </c>
+      <c r="D56" s="22" t="n">
+        <v>46324.47001157407</v>
+      </c>
+      <c r="E56" s="17" t="n">
+        <v>290.24</v>
+      </c>
+      <c r="F56" s="16" t="n">
+        <v>2.290483737</v>
+      </c>
+      <c r="G56" s="17">
+        <f>E56*F56</f>
+        <v/>
+      </c>
+      <c r="H56" s="22" t="n"/>
+      <c r="I56" s="22" t="n"/>
+      <c r="J56" s="17" t="n"/>
+      <c r="K56" s="17">
+        <f>IF(ISNUMBER(J56),J56*F56,"")</f>
+        <v/>
+      </c>
+      <c r="L56" s="23">
+        <f>IF(ISNUMBER(J56),K56-G56,"")</f>
+        <v/>
+      </c>
+      <c r="M56" s="24">
+        <f>IF(ISNUMBER(J56),L56/G56,"")</f>
+        <v/>
+      </c>
+      <c r="N56" s="25">
+        <f>IF(ISNUMBER(H56),H56-C56,"")</f>
+        <v/>
+      </c>
+      <c r="O56" s="6" t="n"/>
+      <c r="P56" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>Avantor, Inc.</t>
+        </is>
+      </c>
+      <c r="C57" s="22" t="n">
+        <v>46324.67834490741</v>
+      </c>
+      <c r="D57" s="22" t="n">
+        <v>46324.47001157407</v>
+      </c>
+      <c r="E57" s="17" t="n">
+        <v>16.49</v>
+      </c>
+      <c r="F57" s="16" t="n">
+        <v>40.314736203</v>
+      </c>
+      <c r="G57" s="17">
+        <f>E57*F57</f>
+        <v/>
+      </c>
+      <c r="H57" s="22" t="n"/>
+      <c r="I57" s="22" t="n"/>
+      <c r="J57" s="17" t="n"/>
+      <c r="K57" s="17">
+        <f>IF(ISNUMBER(J57),J57*F57,"")</f>
+        <v/>
+      </c>
+      <c r="L57" s="23">
+        <f>IF(ISNUMBER(J57),K57-G57,"")</f>
+        <v/>
+      </c>
+      <c r="M57" s="24">
+        <f>IF(ISNUMBER(J57),L57/G57,"")</f>
+        <v/>
+      </c>
+      <c r="N57" s="25">
+        <f>IF(ISNUMBER(H57),H57-C57,"")</f>
+        <v/>
+      </c>
+      <c r="O57" s="6" t="n"/>
+      <c r="P57" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>ExxonMobil Holdings Corporation</t>
+        </is>
+      </c>
+      <c r="C58" s="22" t="n">
+        <v>46324.67834490741</v>
+      </c>
+      <c r="D58" s="22" t="n">
+        <v>46324.47001157407</v>
+      </c>
+      <c r="E58" s="17" t="n">
+        <v>181.72</v>
+      </c>
+      <c r="F58" s="16" t="n">
+        <v>3.658320493</v>
+      </c>
+      <c r="G58" s="17">
+        <f>E58*F58</f>
+        <v/>
+      </c>
+      <c r="H58" s="22" t="n"/>
+      <c r="I58" s="22" t="n"/>
+      <c r="J58" s="17" t="n"/>
+      <c r="K58" s="17">
+        <f>IF(ISNUMBER(J58),J58*F58,"")</f>
+        <v/>
+      </c>
+      <c r="L58" s="23">
+        <f>IF(ISNUMBER(J58),K58-G58,"")</f>
+        <v/>
+      </c>
+      <c r="M58" s="24">
+        <f>IF(ISNUMBER(J58),L58/G58,"")</f>
+        <v/>
+      </c>
+      <c r="N58" s="25">
+        <f>IF(ISNUMBER(H58),H58-C58,"")</f>
+        <v/>
+      </c>
+      <c r="O58" s="6" t="n"/>
+      <c r="P58" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+        </is>
+      </c>
+      <c r="C59" s="22" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="D59" s="22" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="E59" s="17" t="n">
+        <v>107.49</v>
+      </c>
+      <c r="F59" s="16" t="n">
+        <v>6.184668341</v>
+      </c>
+      <c r="G59" s="17">
+        <f>E59*F59</f>
+        <v/>
+      </c>
+      <c r="H59" s="22" t="n"/>
+      <c r="I59" s="22" t="n"/>
+      <c r="J59" s="17" t="n"/>
+      <c r="K59" s="17">
+        <f>IF(ISNUMBER(J59),J59*F59,"")</f>
+        <v/>
+      </c>
+      <c r="L59" s="23">
+        <f>IF(ISNUMBER(J59),K59-G59,"")</f>
+        <v/>
+      </c>
+      <c r="M59" s="24">
+        <f>IF(ISNUMBER(J59),L59/G59,"")</f>
+        <v/>
+      </c>
+      <c r="N59" s="25">
+        <f>IF(ISNUMBER(H59),H59-C59,"")</f>
+        <v/>
+      </c>
+      <c r="O59" s="6" t="n"/>
+      <c r="P59" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>DUK</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Duke Energy Corporation</t>
+        </is>
+      </c>
+      <c r="C60" s="22" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="D60" s="22" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="E60" s="17" t="n">
+        <v>125.74</v>
+      </c>
+      <c r="F60" s="16" t="n">
+        <v>5.287020836</v>
+      </c>
+      <c r="G60" s="17">
+        <f>E60*F60</f>
+        <v/>
+      </c>
+      <c r="H60" s="22" t="n"/>
+      <c r="I60" s="22" t="n"/>
+      <c r="J60" s="17" t="n"/>
+      <c r="K60" s="17">
+        <f>IF(ISNUMBER(J60),J60*F60,"")</f>
+        <v/>
+      </c>
+      <c r="L60" s="23">
+        <f>IF(ISNUMBER(J60),K60-G60,"")</f>
+        <v/>
+      </c>
+      <c r="M60" s="24">
+        <f>IF(ISNUMBER(J60),L60/G60,"")</f>
+        <v/>
+      </c>
+      <c r="N60" s="25">
+        <f>IF(ISNUMBER(H60),H60-C60,"")</f>
+        <v/>
+      </c>
+      <c r="O60" s="6" t="n"/>
+      <c r="P60" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>Dynatrace, Inc.</t>
+        </is>
+      </c>
+      <c r="C61" s="22" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="D61" s="22" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="E61" s="17" t="n">
+        <v>60.75</v>
+      </c>
+      <c r="F61" s="16" t="n">
+        <v>10.943045267</v>
+      </c>
+      <c r="G61" s="17">
+        <f>E61*F61</f>
+        <v/>
+      </c>
+      <c r="H61" s="22" t="n"/>
+      <c r="I61" s="22" t="n"/>
+      <c r="J61" s="17" t="n"/>
+      <c r="K61" s="17">
+        <f>IF(ISNUMBER(J61),J61*F61,"")</f>
+        <v/>
+      </c>
+      <c r="L61" s="23">
+        <f>IF(ISNUMBER(J61),K61-G61,"")</f>
+        <v/>
+      </c>
+      <c r="M61" s="24">
+        <f>IF(ISNUMBER(J61),L61/G61,"")</f>
+        <v/>
+      </c>
+      <c r="N61" s="25">
+        <f>IF(ISNUMBER(H61),H61-C61,"")</f>
+        <v/>
+      </c>
+      <c r="O61" s="6" t="n"/>
+      <c r="P61" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>The Kroger Co.</t>
+        </is>
+      </c>
+      <c r="C62" s="22" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="D62" s="22" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="E62" s="17" t="n">
+        <v>65.48</v>
+      </c>
+      <c r="F62" s="16" t="n">
+        <v>10.152565668</v>
+      </c>
+      <c r="G62" s="17">
+        <f>E62*F62</f>
+        <v/>
+      </c>
+      <c r="H62" s="22" t="n"/>
+      <c r="I62" s="22" t="n"/>
+      <c r="J62" s="17" t="n"/>
+      <c r="K62" s="17">
+        <f>IF(ISNUMBER(J62),J62*F62,"")</f>
+        <v/>
+      </c>
+      <c r="L62" s="23">
+        <f>IF(ISNUMBER(J62),K62-G62,"")</f>
+        <v/>
+      </c>
+      <c r="M62" s="24">
+        <f>IF(ISNUMBER(J62),L62/G62,"")</f>
+        <v/>
+      </c>
+      <c r="N62" s="25">
+        <f>IF(ISNUMBER(H62),H62-C62,"")</f>
+        <v/>
+      </c>
+      <c r="O62" s="6" t="n"/>
+      <c r="P62" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Accenture PLC</t>
+        </is>
+      </c>
+      <c r="C63" s="22" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="D63" s="22" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="E63" s="17" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="F63" s="16" t="n">
+        <v>2.726336942</v>
+      </c>
+      <c r="G63" s="17">
+        <f>E63*F63</f>
+        <v/>
+      </c>
+      <c r="H63" s="22" t="n"/>
+      <c r="I63" s="22" t="n"/>
+      <c r="J63" s="17" t="n"/>
+      <c r="K63" s="17">
+        <f>IF(ISNUMBER(J63),J63*F63,"")</f>
+        <v/>
+      </c>
+      <c r="L63" s="23">
+        <f>IF(ISNUMBER(J63),K63-G63,"")</f>
+        <v/>
+      </c>
+      <c r="M63" s="24">
+        <f>IF(ISNUMBER(J63),L63/G63,"")</f>
+        <v/>
+      </c>
+      <c r="N63" s="25">
+        <f>IF(ISNUMBER(H63),H63-C63,"")</f>
+        <v/>
+      </c>
+      <c r="O63" s="6" t="n"/>
+      <c r="P63" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Illumina, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C64" s="22" t="n">
+        <v>46324.67835648148</v>
+      </c>
+      <c r="D64" s="22" t="n">
+        <v>46324.47002314815</v>
+      </c>
+      <c r="E64" s="17" t="n">
+        <v>288.56</v>
+      </c>
+      <c r="F64" s="16" t="n">
+        <v>2.303818963</v>
+      </c>
+      <c r="G64" s="17">
+        <f>E64*F64</f>
+        <v/>
+      </c>
+      <c r="H64" s="22" t="n"/>
+      <c r="I64" s="22" t="n"/>
+      <c r="J64" s="17" t="n"/>
+      <c r="K64" s="17">
+        <f>IF(ISNUMBER(J64),J64*F64,"")</f>
+        <v/>
+      </c>
+      <c r="L64" s="23">
+        <f>IF(ISNUMBER(J64),K64-G64,"")</f>
+        <v/>
+      </c>
+      <c r="M64" s="24">
+        <f>IF(ISNUMBER(J64),L64/G64,"")</f>
+        <v/>
+      </c>
+      <c r="N64" s="25">
+        <f>IF(ISNUMBER(H64),H64-C64,"")</f>
+        <v/>
+      </c>
+      <c r="O64" s="6" t="n"/>
+      <c r="P64" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Linde plc Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="C65" s="22" t="n">
+        <v>46324.67836805555</v>
+      </c>
+      <c r="D65" s="22" t="n">
+        <v>46324.47003472222</v>
+      </c>
+      <c r="E65" s="17" t="n">
+        <v>501.46</v>
+      </c>
+      <c r="F65" s="16" t="n">
+        <v>1.325708929</v>
+      </c>
+      <c r="G65" s="17">
+        <f>E65*F65</f>
+        <v/>
+      </c>
+      <c r="H65" s="22" t="n"/>
+      <c r="I65" s="22" t="n"/>
+      <c r="J65" s="17" t="n"/>
+      <c r="K65" s="17">
+        <f>IF(ISNUMBER(J65),J65*F65,"")</f>
+        <v/>
+      </c>
+      <c r="L65" s="23">
+        <f>IF(ISNUMBER(J65),K65-G65,"")</f>
+        <v/>
+      </c>
+      <c r="M65" s="24">
+        <f>IF(ISNUMBER(J65),L65/G65,"")</f>
+        <v/>
+      </c>
+      <c r="N65" s="25">
+        <f>IF(ISNUMBER(H65),H65-C65,"")</f>
+        <v/>
+      </c>
+      <c r="O65" s="6" t="n"/>
+      <c r="P65" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+        </is>
+      </c>
+      <c r="C66" s="22" t="n">
+        <v>46324.67839120371</v>
+      </c>
+      <c r="D66" s="22" t="n">
+        <v>46324.47005787037</v>
+      </c>
+      <c r="E66" s="17" t="n">
+        <v>47.09</v>
+      </c>
+      <c r="F66" s="16" t="n">
+        <v>14.117434699</v>
+      </c>
+      <c r="G66" s="17">
+        <f>E66*F66</f>
+        <v/>
+      </c>
+      <c r="H66" s="22" t="n"/>
+      <c r="I66" s="22" t="n"/>
+      <c r="J66" s="17" t="n"/>
+      <c r="K66" s="17">
+        <f>IF(ISNUMBER(J66),J66*F66,"")</f>
+        <v/>
+      </c>
+      <c r="L66" s="23">
+        <f>IF(ISNUMBER(J66),K66-G66,"")</f>
+        <v/>
+      </c>
+      <c r="M66" s="24">
+        <f>IF(ISNUMBER(J66),L66/G66,"")</f>
+        <v/>
+      </c>
+      <c r="N66" s="25">
+        <f>IF(ISNUMBER(H66),H66-C66,"")</f>
+        <v/>
+      </c>
+      <c r="O66" s="6" t="n"/>
+      <c r="P66" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M54">
+  <conditionalFormatting sqref="L2:M66">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 15:26 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA100" headerRowCount="1">
-  <autoFilter ref="A1:BA100"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA102" headerRowCount="1">
+  <autoFilter ref="A1:BA102"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.67849537037</v>
+        <v>46324.68532407407</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.47016203704</v>
+        <v>46324.47699074074</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$100,"BUY")+COUNTIF(Orders!$E$2:$E$100,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$102,"BUY")+COUNTIF(Orders!$E$2:$E$102,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$100,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$102,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$100,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$102,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$100,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$102,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$100,Orders!$E$2:$E$100,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$102,Orders!$E$2:$E$102,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$100,Orders!$E$2:$E$100,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$102,Orders!$E$2:$E$102,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA100"/>
+  <dimension ref="A1:BA102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17224,6 +17224,382 @@
       </c>
       <c r="BA100" s="6" t="n"/>
     </row>
+    <row r="101">
+      <c r="A101" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="13" t="n">
+        <v>46324.68523148148</v>
+      </c>
+      <c r="C101" s="13" t="n">
+        <v>46324.47689814815</v>
+      </c>
+      <c r="D101" s="13" t="n">
+        <v>46324.64356481482</v>
+      </c>
+      <c r="E101" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="G101" s="15" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="H101" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J101" s="16" t="n">
+        <v>6.035195373</v>
+      </c>
+      <c r="K101" s="17" t="n">
+        <v>1370.33</v>
+      </c>
+      <c r="L101" s="17">
+        <f>IF(AND(ISNUMBER(J101),ISNUMBER(K101)),J101*K101,"")</f>
+        <v/>
+      </c>
+      <c r="M101" s="17" t="n"/>
+      <c r="N101" s="16" t="n">
+        <v>6.035195373</v>
+      </c>
+      <c r="O101" s="6" t="inlineStr">
+        <is>
+          <t>trailing stop</t>
+        </is>
+      </c>
+      <c r="P101" s="15" t="inlineStr">
+        <is>
+          <t>High risk sell line (1%): highest $1,398.38, fell 2.0% to $1,371.12 (line $1,384.40), -0.9% from the buy price</t>
+        </is>
+      </c>
+      <c r="Q101" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R101" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S101" s="18" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="T101" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="U101" s="19" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="V101" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W101" s="12" t="n"/>
+      <c r="X101" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y101" s="19" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="Z101" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA101" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB101" s="15" t="n"/>
+      <c r="AC101" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD101" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE101" s="17" t="n">
+        <v>1372.57</v>
+      </c>
+      <c r="AF101" s="17" t="n">
+        <v>1314.0104</v>
+      </c>
+      <c r="AG101" s="17" t="n">
+        <v>1431.1296</v>
+      </c>
+      <c r="AH101" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI101" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ101" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AK101" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL101" s="15" t="inlineStr">
+        <is>
+          <t>Eli Lilly Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM101" s="17" t="n">
+        <v>1372.57</v>
+      </c>
+      <c r="AN101" s="19" t="n">
+        <v>0.0635</v>
+      </c>
+      <c r="AO101" s="17" t="n">
+        <v>99412.24000000001</v>
+      </c>
+      <c r="AP101" s="17" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="AQ101" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR101" s="16" t="n">
+        <v>6.035195373</v>
+      </c>
+      <c r="AS101" s="17" t="n">
+        <v>1382.881495</v>
+      </c>
+      <c r="AT101" s="19" t="n">
+        <v>-0.008500000000000001</v>
+      </c>
+      <c r="AU101" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV101" s="6" t="inlineStr">
+        <is>
+          <t>5d4ca2e7-bc86-484f-9f55-e93b264f00d5</t>
+        </is>
+      </c>
+      <c r="AW101" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-LLY-1793287603579</t>
+        </is>
+      </c>
+      <c r="AX101" s="13" t="n">
+        <v>46324.64355324074</v>
+      </c>
+      <c r="AY101" s="13" t="n">
+        <v>46324.64356481482</v>
+      </c>
+      <c r="AZ101" s="13" t="n">
+        <v>46324.64244212963</v>
+      </c>
+      <c r="BA101" s="6" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="12" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="13" t="n">
+        <v>46324.68523148148</v>
+      </c>
+      <c r="C102" s="13" t="n">
+        <v>46324.47689814815</v>
+      </c>
+      <c r="D102" s="13" t="n">
+        <v>46324.64356481482</v>
+      </c>
+      <c r="E102" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="G102" s="15" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J102" s="16" t="n">
+        <v>26.078334421</v>
+      </c>
+      <c r="K102" s="17" t="n">
+        <v>313.76</v>
+      </c>
+      <c r="L102" s="17">
+        <f>IF(AND(ISNUMBER(J102),ISNUMBER(K102)),J102*K102,"")</f>
+        <v/>
+      </c>
+      <c r="M102" s="17" t="n"/>
+      <c r="N102" s="16" t="n">
+        <v>26.078334421</v>
+      </c>
+      <c r="O102" s="6" t="inlineStr">
+        <is>
+          <t>trailing stop</t>
+        </is>
+      </c>
+      <c r="P102" s="15" t="inlineStr">
+        <is>
+          <t>High risk sell line (1%): highest $325.01, fell 3.4% to $314.04 (line $321.76), -1.9% from the buy price</t>
+        </is>
+      </c>
+      <c r="Q102" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R102" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S102" s="18" t="n">
+        <v>0.621</v>
+      </c>
+      <c r="T102" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U102" s="19" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="V102" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W102" s="12" t="n"/>
+      <c r="X102" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y102" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z102" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA102" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB102" s="15" t="n"/>
+      <c r="AC102" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD102" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE102" s="17" t="n">
+        <v>318.7003</v>
+      </c>
+      <c r="AF102" s="17" t="n">
+        <v>307.3995</v>
+      </c>
+      <c r="AG102" s="17" t="n">
+        <v>330.0012</v>
+      </c>
+      <c r="AH102" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI102" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ102" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK102" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL102" s="15" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM102" s="17" t="n">
+        <v>314.18</v>
+      </c>
+      <c r="AN102" s="19" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="AO102" s="17" t="n">
+        <v>99412.24000000001</v>
+      </c>
+      <c r="AP102" s="17" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="AQ102" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR102" s="16" t="n">
+        <v>26.078334421</v>
+      </c>
+      <c r="AS102" s="17" t="n">
+        <v>320.034243</v>
+      </c>
+      <c r="AT102" s="19" t="n">
+        <v>-0.0187</v>
+      </c>
+      <c r="AU102" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV102" s="6" t="inlineStr">
+        <is>
+          <t>7f4b08a7-ccda-4caa-ad4f-79824ad160e8</t>
+        </is>
+      </c>
+      <c r="AW102" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-WTW-1793287604105</t>
+        </is>
+      </c>
+      <c r="AX102" s="13" t="n">
+        <v>46324.64356481482</v>
+      </c>
+      <c r="AY102" s="13" t="n">
+        <v>46324.64356481482</v>
+      </c>
+      <c r="AZ102" s="13" t="n">
+        <v>46324.64244212963</v>
+      </c>
+      <c r="BA102" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -20058,9 +20434,15 @@
         <f>E45*F45</f>
         <v/>
       </c>
-      <c r="H45" s="22" t="n"/>
-      <c r="I45" s="22" t="n"/>
-      <c r="J45" s="17" t="n"/>
+      <c r="H45" s="22" t="n">
+        <v>46324.68523148148</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>46324.47689814815</v>
+      </c>
+      <c r="J45" s="17" t="n">
+        <v>1370.33</v>
+      </c>
       <c r="K45" s="17">
         <f>IF(ISNUMBER(J45),J45*F45,"")</f>
         <v/>
@@ -20077,10 +20459,14 @@
         <f>IF(ISNUMBER(H45),H45-C45,"")</f>
         <v/>
       </c>
-      <c r="O45" s="6" t="n"/>
+      <c r="O45" s="6" t="inlineStr">
+        <is>
+          <t>trailing stop</t>
+        </is>
+      </c>
       <c r="P45" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -20333,9 +20719,15 @@
         <f>E50*F50</f>
         <v/>
       </c>
-      <c r="H50" s="22" t="n"/>
-      <c r="I50" s="22" t="n"/>
-      <c r="J50" s="17" t="n"/>
+      <c r="H50" s="22" t="n">
+        <v>46324.68523148148</v>
+      </c>
+      <c r="I50" s="22" t="n">
+        <v>46324.47689814815</v>
+      </c>
+      <c r="J50" s="17" t="n">
+        <v>313.76</v>
+      </c>
       <c r="K50" s="17">
         <f>IF(ISNUMBER(J50),J50*F50,"")</f>
         <v/>
@@ -20352,10 +20744,14 @@
         <f>IF(ISNUMBER(H50),H50-C50,"")</f>
         <v/>
       </c>
-      <c r="O50" s="6" t="n"/>
+      <c r="O50" s="6" t="inlineStr">
+        <is>
+          <t>trailing stop</t>
+        </is>
+      </c>
       <c r="P50" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-29 15:33 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA102" headerRowCount="1">
-  <autoFilter ref="A1:BA102"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA104" headerRowCount="1">
+  <autoFilter ref="A1:BA104"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P66" headerRowCount="1">
-  <autoFilter ref="A1:P66"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P68" headerRowCount="1">
+  <autoFilter ref="A1:P68"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.68532407407</v>
+        <v>46324.69009259259</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.47699074074</v>
+        <v>46324.48175925926</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$102,"BUY")+COUNTIF(Orders!$E$2:$E$102,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$104,"BUY")+COUNTIF(Orders!$E$2:$E$104,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$102,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$104,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$102,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$104,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$102,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$104,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$102,Orders!$E$2:$E$102,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$104,Orders!$E$2:$E$104,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$102,Orders!$E$2:$E$102,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$104,Orders!$E$2:$E$104,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$66,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$68,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$66,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$68,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$66)</f>
+        <f>SUM('Round trips'!$L$2:$L$68)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$66,"Closed",'Round trips'!$L$2:$L$66,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$68,"Closed",'Round trips'!$L$2:$L$68,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA102"/>
+  <dimension ref="A1:BA104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17600,6 +17600,378 @@
       </c>
       <c r="BA102" s="6" t="n"/>
     </row>
+    <row r="103">
+      <c r="A103" s="12" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="13" t="n">
+        <v>46324.68998842593</v>
+      </c>
+      <c r="C103" s="13" t="n">
+        <v>46324.48165509259</v>
+      </c>
+      <c r="D103" s="13" t="n">
+        <v>46324.64832175926</v>
+      </c>
+      <c r="E103" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F103" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="G103" s="15" t="inlineStr">
+        <is>
+          <t>The Southern Company</t>
+        </is>
+      </c>
+      <c r="H103" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I103" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J103" s="16" t="n">
+        <v>14.744111003</v>
+      </c>
+      <c r="K103" s="17" t="n">
+        <v>92.97</v>
+      </c>
+      <c r="L103" s="17">
+        <f>IF(AND(ISNUMBER(J103),ISNUMBER(K103)),J103*K103,"")</f>
+        <v/>
+      </c>
+      <c r="M103" s="17" t="n">
+        <v>1370.77</v>
+      </c>
+      <c r="N103" s="16" t="n"/>
+      <c r="O103" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P103" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $16,455.92 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q103" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R103" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S103" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T103" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="U103" s="19" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="V103" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W103" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X103" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y103" s="19" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="Z103" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA103" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB103" s="15" t="inlineStr">
+        <is>
+          <t>One day (+3.8%) did 89% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC103" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD103" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE103" s="17" t="n">
+        <v>93.8866</v>
+      </c>
+      <c r="AF103" s="17" t="n">
+        <v>91.645</v>
+      </c>
+      <c r="AG103" s="17" t="n">
+        <v>96.1283</v>
+      </c>
+      <c r="AH103" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI103" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ103" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK103" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL103" s="15" t="n"/>
+      <c r="AM103" s="17" t="n">
+        <v>92.98999999999999</v>
+      </c>
+      <c r="AN103" s="19" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="AO103" s="17" t="n">
+        <v>99419.13</v>
+      </c>
+      <c r="AP103" s="17" t="n">
+        <v>16455.92</v>
+      </c>
+      <c r="AQ103" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR103" s="16" t="n"/>
+      <c r="AS103" s="17" t="n"/>
+      <c r="AT103" s="19" t="n"/>
+      <c r="AU103" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV103" s="6" t="inlineStr">
+        <is>
+          <t>8e339eed-87fb-4c60-bd50-cbc4d5c766d1</t>
+        </is>
+      </c>
+      <c r="AW103" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-SO-1793288015546</t>
+        </is>
+      </c>
+      <c r="AX103" s="13" t="n">
+        <v>46324.64832175926</v>
+      </c>
+      <c r="AY103" s="13" t="n">
+        <v>46324.64832175926</v>
+      </c>
+      <c r="AZ103" s="13" t="n">
+        <v>46324.64809027778</v>
+      </c>
+      <c r="BA103" s="6" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="12" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="13" t="n">
+        <v>46324.69001157407</v>
+      </c>
+      <c r="C104" s="13" t="n">
+        <v>46324.48167824074</v>
+      </c>
+      <c r="D104" s="13" t="n">
+        <v>46324.64834490741</v>
+      </c>
+      <c r="E104" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F104" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="G104" s="15" t="inlineStr">
+        <is>
+          <t>EQT CORP</t>
+        </is>
+      </c>
+      <c r="H104" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I104" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J104" s="16" t="n">
+        <v>24.950127411</v>
+      </c>
+      <c r="K104" s="17" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="L104" s="17">
+        <f>IF(AND(ISNUMBER(J104),ISNUMBER(K104)),J104*K104,"")</f>
+        <v/>
+      </c>
+      <c r="M104" s="17" t="n">
+        <v>1370.77</v>
+      </c>
+      <c r="N104" s="16" t="n"/>
+      <c r="O104" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P104" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $16,455.92 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q104" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R104" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S104" s="18" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="T104" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U104" s="19" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="V104" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W104" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X104" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y104" s="19" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="Z104" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA104" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="AB104" s="15" t="inlineStr">
+        <is>
+          <t>Price gapped 5.1% at an open in the last week.</t>
+        </is>
+      </c>
+      <c r="AC104" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD104" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE104" s="17" t="n">
+        <v>55.7426</v>
+      </c>
+      <c r="AF104" s="17" t="n">
+        <v>53.7237</v>
+      </c>
+      <c r="AG104" s="17" t="n">
+        <v>57.7615</v>
+      </c>
+      <c r="AH104" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI104" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ104" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK104" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL104" s="15" t="inlineStr">
+        <is>
+          <t>UBS Maintains Buy on EQT, Lowers Price Target to $75</t>
+        </is>
+      </c>
+      <c r="AM104" s="17" t="n">
+        <v>54.935</v>
+      </c>
+      <c r="AN104" s="19" t="n">
+        <v>-0.023</v>
+      </c>
+      <c r="AO104" s="17" t="n">
+        <v>99419.13</v>
+      </c>
+      <c r="AP104" s="17" t="n">
+        <v>16455.92</v>
+      </c>
+      <c r="AQ104" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR104" s="16" t="n"/>
+      <c r="AS104" s="17" t="n"/>
+      <c r="AT104" s="19" t="n"/>
+      <c r="AU104" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV104" s="6" t="inlineStr">
+        <is>
+          <t>c8464e45-bd19-4274-bffc-d557838e3703</t>
+        </is>
+      </c>
+      <c r="AW104" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EQT-1793288015588</t>
+        </is>
+      </c>
+      <c r="AX104" s="13" t="n">
+        <v>46324.64832175926</v>
+      </c>
+      <c r="AY104" s="13" t="n">
+        <v>46324.64834490741</v>
+      </c>
+      <c r="AZ104" s="13" t="n">
+        <v>46324.64809027778</v>
+      </c>
+      <c r="BA104" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -17615,7 +17987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P66"/>
+  <dimension ref="A1:P68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -21603,8 +21975,114 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>The Southern Company</t>
+        </is>
+      </c>
+      <c r="C67" s="22" t="n">
+        <v>46324.68998842593</v>
+      </c>
+      <c r="D67" s="22" t="n">
+        <v>46324.48165509259</v>
+      </c>
+      <c r="E67" s="17" t="n">
+        <v>92.97</v>
+      </c>
+      <c r="F67" s="16" t="n">
+        <v>14.744111003</v>
+      </c>
+      <c r="G67" s="17">
+        <f>E67*F67</f>
+        <v/>
+      </c>
+      <c r="H67" s="22" t="n"/>
+      <c r="I67" s="22" t="n"/>
+      <c r="J67" s="17" t="n"/>
+      <c r="K67" s="17">
+        <f>IF(ISNUMBER(J67),J67*F67,"")</f>
+        <v/>
+      </c>
+      <c r="L67" s="23">
+        <f>IF(ISNUMBER(J67),K67-G67,"")</f>
+        <v/>
+      </c>
+      <c r="M67" s="24">
+        <f>IF(ISNUMBER(J67),L67/G67,"")</f>
+        <v/>
+      </c>
+      <c r="N67" s="25">
+        <f>IF(ISNUMBER(H67),H67-C67,"")</f>
+        <v/>
+      </c>
+      <c r="O67" s="6" t="n"/>
+      <c r="P67" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>EQT CORP</t>
+        </is>
+      </c>
+      <c r="C68" s="22" t="n">
+        <v>46324.69001157407</v>
+      </c>
+      <c r="D68" s="22" t="n">
+        <v>46324.48167824074</v>
+      </c>
+      <c r="E68" s="17" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="F68" s="16" t="n">
+        <v>24.950127411</v>
+      </c>
+      <c r="G68" s="17">
+        <f>E68*F68</f>
+        <v/>
+      </c>
+      <c r="H68" s="22" t="n"/>
+      <c r="I68" s="22" t="n"/>
+      <c r="J68" s="17" t="n"/>
+      <c r="K68" s="17">
+        <f>IF(ISNUMBER(J68),J68*F68,"")</f>
+        <v/>
+      </c>
+      <c r="L68" s="23">
+        <f>IF(ISNUMBER(J68),K68-G68,"")</f>
+        <v/>
+      </c>
+      <c r="M68" s="24">
+        <f>IF(ISNUMBER(J68),L68/G68,"")</f>
+        <v/>
+      </c>
+      <c r="N68" s="25">
+        <f>IF(ISNUMBER(H68),H68-C68,"")</f>
+        <v/>
+      </c>
+      <c r="O68" s="6" t="n"/>
+      <c r="P68" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M66">
+  <conditionalFormatting sqref="L2:M68">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 16:03 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA104" headerRowCount="1">
-  <autoFilter ref="A1:BA104"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA105" headerRowCount="1">
+  <autoFilter ref="A1:BA105"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P68" headerRowCount="1">
-  <autoFilter ref="A1:P68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P69" headerRowCount="1">
+  <autoFilter ref="A1:P69"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.69009259259</v>
+        <v>46324.71086805555</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.48175925926</v>
+        <v>46324.50253472223</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$104,"BUY")+COUNTIF(Orders!$E$2:$E$104,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$105,"BUY")+COUNTIF(Orders!$E$2:$E$105,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$104,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$105,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$104,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$105,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$104,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$105,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$104,Orders!$E$2:$E$104,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$105,Orders!$E$2:$E$105,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$104,Orders!$E$2:$E$104,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$105,Orders!$E$2:$E$105,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$68,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$69,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$68,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$69,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$68)</f>
+        <f>SUM('Round trips'!$L$2:$L$69)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$68,"Closed",'Round trips'!$L$2:$L$68,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$69,"Closed",'Round trips'!$L$2:$L$69,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA104"/>
+  <dimension ref="A1:BA105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17972,6 +17972,194 @@
       </c>
       <c r="BA104" s="6" t="n"/>
     </row>
+    <row r="105">
+      <c r="A105" s="12" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="13" t="n">
+        <v>46324.71079861111</v>
+      </c>
+      <c r="C105" s="13" t="n">
+        <v>46324.50246527778</v>
+      </c>
+      <c r="D105" s="13" t="n">
+        <v>46324.66913194444</v>
+      </c>
+      <c r="E105" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F105" s="6" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="G105" s="15" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="H105" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I105" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J105" s="16" t="n">
+        <v>1.829160246</v>
+      </c>
+      <c r="K105" s="17" t="n">
+        <v>182.01</v>
+      </c>
+      <c r="L105" s="17">
+        <f>IF(AND(ISNUMBER(J105),ISNUMBER(K105)),J105*K105,"")</f>
+        <v/>
+      </c>
+      <c r="M105" s="17" t="n"/>
+      <c r="N105" s="16" t="n">
+        <v>1.829160246</v>
+      </c>
+      <c r="O105" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P105" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q105" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R105" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S105" s="18" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="T105" s="12" t="n">
+        <v>93</v>
+      </c>
+      <c r="U105" s="19" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="V105" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W105" s="12" t="n"/>
+      <c r="X105" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y105" s="19" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="Z105" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA105" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB105" s="15" t="n"/>
+      <c r="AC105" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD105" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE105" s="17" t="n">
+        <v>182.12</v>
+      </c>
+      <c r="AF105" s="17" t="n">
+        <v>175.9674</v>
+      </c>
+      <c r="AG105" s="17" t="n">
+        <v>188.2726</v>
+      </c>
+      <c r="AH105" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI105" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ105" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK105" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL105" s="15" t="inlineStr">
+        <is>
+          <t>Exxon Mobil and Citgo Petroleum Acquire Venezuelan Crude Oil Shipment</t>
+        </is>
+      </c>
+      <c r="AM105" s="17" t="n">
+        <v>182.07</v>
+      </c>
+      <c r="AN105" s="19" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="AO105" s="17" t="n">
+        <v>99360.92</v>
+      </c>
+      <c r="AP105" s="17" t="n">
+        <v>13714.4</v>
+      </c>
+      <c r="AQ105" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR105" s="16" t="n">
+        <v>3.658320493</v>
+      </c>
+      <c r="AS105" s="17" t="n">
+        <v>181.72</v>
+      </c>
+      <c r="AT105" s="19" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="AU105" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV105" s="6" t="inlineStr">
+        <is>
+          <t>d1779449-01e2-4e2c-ab7c-32190e1cec52</t>
+        </is>
+      </c>
+      <c r="AW105" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-XOM-1793289812720</t>
+        </is>
+      </c>
+      <c r="AX105" s="13" t="n">
+        <v>46324.66912037037</v>
+      </c>
+      <c r="AY105" s="13" t="n">
+        <v>46324.66913194444</v>
+      </c>
+      <c r="AZ105" s="13" t="n">
+        <v>46324.66893518518</v>
+      </c>
+      <c r="BA105" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -17987,7 +18175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P68"/>
+  <dimension ref="A1:P69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -21519,15 +21707,21 @@
         <v>181.72</v>
       </c>
       <c r="F58" s="16" t="n">
-        <v>3.658320493</v>
+        <v>1.829160246</v>
       </c>
       <c r="G58" s="17">
         <f>E58*F58</f>
         <v/>
       </c>
-      <c r="H58" s="22" t="n"/>
-      <c r="I58" s="22" t="n"/>
-      <c r="J58" s="17" t="n"/>
+      <c r="H58" s="22" t="n">
+        <v>46324.71079861111</v>
+      </c>
+      <c r="I58" s="22" t="n">
+        <v>46324.50246527778</v>
+      </c>
+      <c r="J58" s="17" t="n">
+        <v>182.01</v>
+      </c>
       <c r="K58" s="17">
         <f>IF(ISNUMBER(J58),J58*F58,"")</f>
         <v/>
@@ -21544,35 +21738,39 @@
         <f>IF(ISNUMBER(H58),H58-C58,"")</f>
         <v/>
       </c>
-      <c r="O58" s="6" t="n"/>
+      <c r="O58" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P58" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>SHEL</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+          <t>ExxonMobil Holdings Corporation</t>
         </is>
       </c>
       <c r="C59" s="22" t="n">
-        <v>46324.67835648148</v>
+        <v>46324.67834490741</v>
       </c>
       <c r="D59" s="22" t="n">
-        <v>46324.47002314815</v>
+        <v>46324.47001157407</v>
       </c>
       <c r="E59" s="17" t="n">
-        <v>107.49</v>
+        <v>181.72</v>
       </c>
       <c r="F59" s="16" t="n">
-        <v>6.184668341</v>
+        <v>1.829160247</v>
       </c>
       <c r="G59" s="17">
         <f>E59*F59</f>
@@ -21607,12 +21805,12 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>SHEL</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Duke Energy Corporation</t>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
         </is>
       </c>
       <c r="C60" s="22" t="n">
@@ -21622,10 +21820,10 @@
         <v>46324.47002314815</v>
       </c>
       <c r="E60" s="17" t="n">
-        <v>125.74</v>
+        <v>107.49</v>
       </c>
       <c r="F60" s="16" t="n">
-        <v>5.287020836</v>
+        <v>6.184668341</v>
       </c>
       <c r="G60" s="17">
         <f>E60*F60</f>
@@ -21660,12 +21858,12 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>Dynatrace, Inc.</t>
+          <t>Duke Energy Corporation</t>
         </is>
       </c>
       <c r="C61" s="22" t="n">
@@ -21675,10 +21873,10 @@
         <v>46324.47002314815</v>
       </c>
       <c r="E61" s="17" t="n">
-        <v>60.75</v>
+        <v>125.74</v>
       </c>
       <c r="F61" s="16" t="n">
-        <v>10.943045267</v>
+        <v>5.287020836</v>
       </c>
       <c r="G61" s="17">
         <f>E61*F61</f>
@@ -21713,12 +21911,12 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>The Kroger Co.</t>
+          <t>Dynatrace, Inc.</t>
         </is>
       </c>
       <c r="C62" s="22" t="n">
@@ -21728,10 +21926,10 @@
         <v>46324.47002314815</v>
       </c>
       <c r="E62" s="17" t="n">
-        <v>65.48</v>
+        <v>60.75</v>
       </c>
       <c r="F62" s="16" t="n">
-        <v>10.152565668</v>
+        <v>10.943045267</v>
       </c>
       <c r="G62" s="17">
         <f>E62*F62</f>
@@ -21766,12 +21964,12 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Accenture PLC</t>
+          <t>The Kroger Co.</t>
         </is>
       </c>
       <c r="C63" s="22" t="n">
@@ -21781,10 +21979,10 @@
         <v>46324.47002314815</v>
       </c>
       <c r="E63" s="17" t="n">
-        <v>243.84</v>
+        <v>65.48</v>
       </c>
       <c r="F63" s="16" t="n">
-        <v>2.726336942</v>
+        <v>10.152565668</v>
       </c>
       <c r="G63" s="17">
         <f>E63*F63</f>
@@ -21819,12 +22017,12 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Illumina, Inc. Common Stock</t>
+          <t>Accenture PLC</t>
         </is>
       </c>
       <c r="C64" s="22" t="n">
@@ -21834,10 +22032,10 @@
         <v>46324.47002314815</v>
       </c>
       <c r="E64" s="17" t="n">
-        <v>288.56</v>
+        <v>243.84</v>
       </c>
       <c r="F64" s="16" t="n">
-        <v>2.303818963</v>
+        <v>2.726336942</v>
       </c>
       <c r="G64" s="17">
         <f>E64*F64</f>
@@ -21872,25 +22070,25 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Linde plc Ordinary Shares</t>
+          <t>Illumina, Inc. Common Stock</t>
         </is>
       </c>
       <c r="C65" s="22" t="n">
-        <v>46324.67836805555</v>
+        <v>46324.67835648148</v>
       </c>
       <c r="D65" s="22" t="n">
-        <v>46324.47003472222</v>
+        <v>46324.47002314815</v>
       </c>
       <c r="E65" s="17" t="n">
-        <v>501.46</v>
+        <v>288.56</v>
       </c>
       <c r="F65" s="16" t="n">
-        <v>1.325708929</v>
+        <v>2.303818963</v>
       </c>
       <c r="G65" s="17">
         <f>E65*F65</f>
@@ -21925,25 +22123,25 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EQNR</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+          <t>Linde plc Ordinary Shares</t>
         </is>
       </c>
       <c r="C66" s="22" t="n">
-        <v>46324.67839120371</v>
+        <v>46324.67836805555</v>
       </c>
       <c r="D66" s="22" t="n">
-        <v>46324.47005787037</v>
+        <v>46324.47003472222</v>
       </c>
       <c r="E66" s="17" t="n">
-        <v>47.09</v>
+        <v>501.46</v>
       </c>
       <c r="F66" s="16" t="n">
-        <v>14.117434699</v>
+        <v>1.325708929</v>
       </c>
       <c r="G66" s="17">
         <f>E66*F66</f>
@@ -21978,25 +22176,25 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>EQNR</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>The Southern Company</t>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
         </is>
       </c>
       <c r="C67" s="22" t="n">
-        <v>46324.68998842593</v>
+        <v>46324.67839120371</v>
       </c>
       <c r="D67" s="22" t="n">
-        <v>46324.48165509259</v>
+        <v>46324.47005787037</v>
       </c>
       <c r="E67" s="17" t="n">
-        <v>92.97</v>
+        <v>47.09</v>
       </c>
       <c r="F67" s="16" t="n">
-        <v>14.744111003</v>
+        <v>14.117434699</v>
       </c>
       <c r="G67" s="17">
         <f>E67*F67</f>
@@ -22031,25 +22229,25 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>EQT CORP</t>
+          <t>The Southern Company</t>
         </is>
       </c>
       <c r="C68" s="22" t="n">
-        <v>46324.69001157407</v>
+        <v>46324.68998842593</v>
       </c>
       <c r="D68" s="22" t="n">
-        <v>46324.48167824074</v>
+        <v>46324.48165509259</v>
       </c>
       <c r="E68" s="17" t="n">
-        <v>54.94</v>
+        <v>92.97</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>24.950127411</v>
+        <v>14.744111003</v>
       </c>
       <c r="G68" s="17">
         <f>E68*F68</f>
@@ -22081,8 +22279,61 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>EQT CORP</t>
+        </is>
+      </c>
+      <c r="C69" s="22" t="n">
+        <v>46324.69001157407</v>
+      </c>
+      <c r="D69" s="22" t="n">
+        <v>46324.48167824074</v>
+      </c>
+      <c r="E69" s="17" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="F69" s="16" t="n">
+        <v>24.950127411</v>
+      </c>
+      <c r="G69" s="17">
+        <f>E69*F69</f>
+        <v/>
+      </c>
+      <c r="H69" s="22" t="n"/>
+      <c r="I69" s="22" t="n"/>
+      <c r="J69" s="17" t="n"/>
+      <c r="K69" s="17">
+        <f>IF(ISNUMBER(J69),J69*F69,"")</f>
+        <v/>
+      </c>
+      <c r="L69" s="23">
+        <f>IF(ISNUMBER(J69),K69-G69,"")</f>
+        <v/>
+      </c>
+      <c r="M69" s="24">
+        <f>IF(ISNUMBER(J69),L69/G69,"")</f>
+        <v/>
+      </c>
+      <c r="N69" s="25">
+        <f>IF(ISNUMBER(H69),H69-C69,"")</f>
+        <v/>
+      </c>
+      <c r="O69" s="6" t="n"/>
+      <c r="P69" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M68">
+  <conditionalFormatting sqref="L2:M69">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 16:09 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA105" headerRowCount="1">
-  <autoFilter ref="A1:BA105"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA106" headerRowCount="1">
+  <autoFilter ref="A1:BA106"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P69" headerRowCount="1">
-  <autoFilter ref="A1:P69"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P70" headerRowCount="1">
+  <autoFilter ref="A1:P70"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.71086805555</v>
+        <v>46324.71497685185</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.50253472223</v>
+        <v>46324.50664351852</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$105,"BUY")+COUNTIF(Orders!$E$2:$E$105,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$106,"BUY")+COUNTIF(Orders!$E$2:$E$106,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$105,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$106,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$105,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$106,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$105,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$106,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$105,Orders!$E$2:$E$105,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$106,Orders!$E$2:$E$106,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$105,Orders!$E$2:$E$105,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$106,Orders!$E$2:$E$106,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$69,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$70,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$69,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$70,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$69)</f>
+        <f>SUM('Round trips'!$L$2:$L$70)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$69,"Closed",'Round trips'!$L$2:$L$69,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$70,"Closed",'Round trips'!$L$2:$L$70,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA105"/>
+  <dimension ref="A1:BA106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18160,6 +18160,190 @@
       </c>
       <c r="BA105" s="6" t="n"/>
     </row>
+    <row r="106">
+      <c r="A106" s="12" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="13" t="n">
+        <v>46324.7149074074</v>
+      </c>
+      <c r="C106" s="13" t="n">
+        <v>46324.50657407408</v>
+      </c>
+      <c r="D106" s="13" t="n">
+        <v>46324.67324074074</v>
+      </c>
+      <c r="E106" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F106" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="G106" s="15" t="inlineStr">
+        <is>
+          <t>eBay Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I106" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J106" s="16" t="n">
+        <v>9.638632618999999</v>
+      </c>
+      <c r="K106" s="17" t="n">
+        <v>121.4</v>
+      </c>
+      <c r="L106" s="17">
+        <f>IF(AND(ISNUMBER(J106),ISNUMBER(K106)),J106*K106,"")</f>
+        <v/>
+      </c>
+      <c r="M106" s="17" t="n">
+        <v>1170.14</v>
+      </c>
+      <c r="N106" s="16" t="n"/>
+      <c r="O106" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P106" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #3, 8.33% of the $14,047.33 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q106" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R106" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S106" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T106" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="U106" s="19" t="n">
+        <v>0.005500000000000001</v>
+      </c>
+      <c r="V106" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W106" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X106" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y106" s="19" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="Z106" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA106" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB106" s="15" t="n"/>
+      <c r="AC106" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD106" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE106" s="17" t="n">
+        <v>123.4909</v>
+      </c>
+      <c r="AF106" s="17" t="n">
+        <v>118.4136</v>
+      </c>
+      <c r="AG106" s="17" t="n">
+        <v>128.5682</v>
+      </c>
+      <c r="AH106" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI106" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ106" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK106" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL106" s="15" t="inlineStr">
+        <is>
+          <t>eBay Stock Nears 52-Week High on 2027 Growth Outlook</t>
+        </is>
+      </c>
+      <c r="AM106" s="17" t="n">
+        <v>121.46</v>
+      </c>
+      <c r="AN106" s="19" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="AO106" s="17" t="n">
+        <v>99391.81</v>
+      </c>
+      <c r="AP106" s="17" t="n">
+        <v>14047.33</v>
+      </c>
+      <c r="AQ106" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR106" s="16" t="n"/>
+      <c r="AS106" s="17" t="n"/>
+      <c r="AT106" s="19" t="n"/>
+      <c r="AU106" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV106" s="6" t="inlineStr">
+        <is>
+          <t>8f3a9ec6-8716-4391-8ca4-3f77ebea3507</t>
+        </is>
+      </c>
+      <c r="AW106" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EBAY-1793290168000</t>
+        </is>
+      </c>
+      <c r="AX106" s="13" t="n">
+        <v>46324.67324074074</v>
+      </c>
+      <c r="AY106" s="13" t="n">
+        <v>46324.67324074074</v>
+      </c>
+      <c r="AZ106" s="13" t="n">
+        <v>46324.67306712963</v>
+      </c>
+      <c r="BA106" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -18175,7 +18359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P69"/>
+  <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -22332,8 +22516,61 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>eBay Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C70" s="22" t="n">
+        <v>46324.7149074074</v>
+      </c>
+      <c r="D70" s="22" t="n">
+        <v>46324.50657407408</v>
+      </c>
+      <c r="E70" s="17" t="n">
+        <v>121.4</v>
+      </c>
+      <c r="F70" s="16" t="n">
+        <v>9.638632618999999</v>
+      </c>
+      <c r="G70" s="17">
+        <f>E70*F70</f>
+        <v/>
+      </c>
+      <c r="H70" s="22" t="n"/>
+      <c r="I70" s="22" t="n"/>
+      <c r="J70" s="17" t="n"/>
+      <c r="K70" s="17">
+        <f>IF(ISNUMBER(J70),J70*F70,"")</f>
+        <v/>
+      </c>
+      <c r="L70" s="23">
+        <f>IF(ISNUMBER(J70),K70-G70,"")</f>
+        <v/>
+      </c>
+      <c r="M70" s="24">
+        <f>IF(ISNUMBER(J70),L70/G70,"")</f>
+        <v/>
+      </c>
+      <c r="N70" s="25">
+        <f>IF(ISNUMBER(H70),H70-C70,"")</f>
+        <v/>
+      </c>
+      <c r="O70" s="6" t="n"/>
+      <c r="P70" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M69">
+  <conditionalFormatting sqref="L2:M70">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 17:06 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA106" headerRowCount="1">
-  <autoFilter ref="A1:BA106"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA107" headerRowCount="1">
+  <autoFilter ref="A1:BA107"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P70" headerRowCount="1">
-  <autoFilter ref="A1:P70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P71" headerRowCount="1">
+  <autoFilter ref="A1:P71"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.71497685185</v>
+        <v>46324.75469907407</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.50664351852</v>
+        <v>46324.54636574074</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$106,"BUY")+COUNTIF(Orders!$E$2:$E$106,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$107,"BUY")+COUNTIF(Orders!$E$2:$E$107,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$106,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$107,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$106,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$107,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$106,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$107,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$106,Orders!$E$2:$E$106,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$107,Orders!$E$2:$E$107,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$106,Orders!$E$2:$E$106,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$107,Orders!$E$2:$E$107,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$70,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$71,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$70,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$71,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$70)</f>
+        <f>SUM('Round trips'!$L$2:$L$71)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$70,"Closed",'Round trips'!$L$2:$L$70,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$71,"Closed",'Round trips'!$L$2:$L$71,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA106"/>
+  <dimension ref="A1:BA107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18344,6 +18344,194 @@
       </c>
       <c r="BA106" s="6" t="n"/>
     </row>
+    <row r="107">
+      <c r="A107" s="12" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="13" t="n">
+        <v>46324.75462962963</v>
+      </c>
+      <c r="C107" s="13" t="n">
+        <v>46324.5462962963</v>
+      </c>
+      <c r="D107" s="13" t="n">
+        <v>46324.71296296296</v>
+      </c>
+      <c r="E107" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F107" s="6" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="G107" s="15" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J107" s="16" t="n">
+        <v>1.363168471</v>
+      </c>
+      <c r="K107" s="17" t="n">
+        <v>245.55</v>
+      </c>
+      <c r="L107" s="17">
+        <f>IF(AND(ISNUMBER(J107),ISNUMBER(K107)),J107*K107,"")</f>
+        <v/>
+      </c>
+      <c r="M107" s="17" t="n"/>
+      <c r="N107" s="16" t="n">
+        <v>1.363168471</v>
+      </c>
+      <c r="O107" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P107" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q107" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R107" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S107" s="18" t="n">
+        <v>0.551</v>
+      </c>
+      <c r="T107" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="U107" s="19" t="n">
+        <v>0.0072</v>
+      </c>
+      <c r="V107" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W107" s="12" t="n"/>
+      <c r="X107" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y107" s="19" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="Z107" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA107" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB107" s="15" t="n"/>
+      <c r="AC107" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD107" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE107" s="17" t="n">
+        <v>245.24</v>
+      </c>
+      <c r="AF107" s="17" t="n">
+        <v>226.362</v>
+      </c>
+      <c r="AG107" s="17" t="n">
+        <v>264.118</v>
+      </c>
+      <c r="AH107" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI107" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ107" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK107" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL107" s="15" t="inlineStr">
+        <is>
+          <t>Accenture Recognized in 2026 Guidewire PartnerConnect Excellence Awards</t>
+        </is>
+      </c>
+      <c r="AM107" s="17" t="n">
+        <v>245.585</v>
+      </c>
+      <c r="AN107" s="19" t="n">
+        <v>0.005699999999999999</v>
+      </c>
+      <c r="AO107" s="17" t="n">
+        <v>99521.99000000001</v>
+      </c>
+      <c r="AP107" s="17" t="n">
+        <v>12877.2</v>
+      </c>
+      <c r="AQ107" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR107" s="16" t="n">
+        <v>2.726336942</v>
+      </c>
+      <c r="AS107" s="17" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="AT107" s="19" t="n">
+        <v>0.0072</v>
+      </c>
+      <c r="AU107" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV107" s="6" t="inlineStr">
+        <is>
+          <t>54ffb774-a2a5-48dc-bed4-428649caa4b4</t>
+        </is>
+      </c>
+      <c r="AW107" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-ACN-1793293599550</t>
+        </is>
+      </c>
+      <c r="AX107" s="13" t="n">
+        <v>46324.71295138889</v>
+      </c>
+      <c r="AY107" s="13" t="n">
+        <v>46324.71296296296</v>
+      </c>
+      <c r="AZ107" s="13" t="n">
+        <v>46324.71270833333</v>
+      </c>
+      <c r="BA107" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -18359,7 +18547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -22219,15 +22407,21 @@
         <v>243.84</v>
       </c>
       <c r="F64" s="16" t="n">
-        <v>2.726336942</v>
+        <v>1.363168471</v>
       </c>
       <c r="G64" s="17">
         <f>E64*F64</f>
         <v/>
       </c>
-      <c r="H64" s="22" t="n"/>
-      <c r="I64" s="22" t="n"/>
-      <c r="J64" s="17" t="n"/>
+      <c r="H64" s="22" t="n">
+        <v>46324.75462962963</v>
+      </c>
+      <c r="I64" s="22" t="n">
+        <v>46324.5462962963</v>
+      </c>
+      <c r="J64" s="17" t="n">
+        <v>245.55</v>
+      </c>
       <c r="K64" s="17">
         <f>IF(ISNUMBER(J64),J64*F64,"")</f>
         <v/>
@@ -22244,22 +22438,26 @@
         <f>IF(ISNUMBER(H64),H64-C64,"")</f>
         <v/>
       </c>
-      <c r="O64" s="6" t="n"/>
+      <c r="O64" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P64" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Illumina, Inc. Common Stock</t>
+          <t>Accenture PLC</t>
         </is>
       </c>
       <c r="C65" s="22" t="n">
@@ -22269,10 +22467,10 @@
         <v>46324.47002314815</v>
       </c>
       <c r="E65" s="17" t="n">
-        <v>288.56</v>
+        <v>243.84</v>
       </c>
       <c r="F65" s="16" t="n">
-        <v>2.303818963</v>
+        <v>1.363168471</v>
       </c>
       <c r="G65" s="17">
         <f>E65*F65</f>
@@ -22307,25 +22505,25 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Linde plc Ordinary Shares</t>
+          <t>Illumina, Inc. Common Stock</t>
         </is>
       </c>
       <c r="C66" s="22" t="n">
-        <v>46324.67836805555</v>
+        <v>46324.67835648148</v>
       </c>
       <c r="D66" s="22" t="n">
-        <v>46324.47003472222</v>
+        <v>46324.47002314815</v>
       </c>
       <c r="E66" s="17" t="n">
-        <v>501.46</v>
+        <v>288.56</v>
       </c>
       <c r="F66" s="16" t="n">
-        <v>1.325708929</v>
+        <v>2.303818963</v>
       </c>
       <c r="G66" s="17">
         <f>E66*F66</f>
@@ -22360,25 +22558,25 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EQNR</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+          <t>Linde plc Ordinary Shares</t>
         </is>
       </c>
       <c r="C67" s="22" t="n">
-        <v>46324.67839120371</v>
+        <v>46324.67836805555</v>
       </c>
       <c r="D67" s="22" t="n">
-        <v>46324.47005787037</v>
+        <v>46324.47003472222</v>
       </c>
       <c r="E67" s="17" t="n">
-        <v>47.09</v>
+        <v>501.46</v>
       </c>
       <c r="F67" s="16" t="n">
-        <v>14.117434699</v>
+        <v>1.325708929</v>
       </c>
       <c r="G67" s="17">
         <f>E67*F67</f>
@@ -22413,25 +22611,25 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>EQNR</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>The Southern Company</t>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
         </is>
       </c>
       <c r="C68" s="22" t="n">
-        <v>46324.68998842593</v>
+        <v>46324.67839120371</v>
       </c>
       <c r="D68" s="22" t="n">
-        <v>46324.48165509259</v>
+        <v>46324.47005787037</v>
       </c>
       <c r="E68" s="17" t="n">
-        <v>92.97</v>
+        <v>47.09</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>14.744111003</v>
+        <v>14.117434699</v>
       </c>
       <c r="G68" s="17">
         <f>E68*F68</f>
@@ -22466,25 +22664,25 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>EQT CORP</t>
+          <t>The Southern Company</t>
         </is>
       </c>
       <c r="C69" s="22" t="n">
-        <v>46324.69001157407</v>
+        <v>46324.68998842593</v>
       </c>
       <c r="D69" s="22" t="n">
-        <v>46324.48167824074</v>
+        <v>46324.48165509259</v>
       </c>
       <c r="E69" s="17" t="n">
-        <v>54.94</v>
+        <v>92.97</v>
       </c>
       <c r="F69" s="16" t="n">
-        <v>24.950127411</v>
+        <v>14.744111003</v>
       </c>
       <c r="G69" s="17">
         <f>E69*F69</f>
@@ -22519,25 +22717,25 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>eBay Inc. Common Stock</t>
+          <t>EQT CORP</t>
         </is>
       </c>
       <c r="C70" s="22" t="n">
-        <v>46324.7149074074</v>
+        <v>46324.69001157407</v>
       </c>
       <c r="D70" s="22" t="n">
-        <v>46324.50657407408</v>
+        <v>46324.48167824074</v>
       </c>
       <c r="E70" s="17" t="n">
-        <v>121.4</v>
+        <v>54.94</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>9.638632618999999</v>
+        <v>24.950127411</v>
       </c>
       <c r="G70" s="17">
         <f>E70*F70</f>
@@ -22569,8 +22767,61 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>eBay Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C71" s="22" t="n">
+        <v>46324.7149074074</v>
+      </c>
+      <c r="D71" s="22" t="n">
+        <v>46324.50657407408</v>
+      </c>
+      <c r="E71" s="17" t="n">
+        <v>121.4</v>
+      </c>
+      <c r="F71" s="16" t="n">
+        <v>9.638632618999999</v>
+      </c>
+      <c r="G71" s="17">
+        <f>E71*F71</f>
+        <v/>
+      </c>
+      <c r="H71" s="22" t="n"/>
+      <c r="I71" s="22" t="n"/>
+      <c r="J71" s="17" t="n"/>
+      <c r="K71" s="17">
+        <f>IF(ISNUMBER(J71),J71*F71,"")</f>
+        <v/>
+      </c>
+      <c r="L71" s="23">
+        <f>IF(ISNUMBER(J71),K71-G71,"")</f>
+        <v/>
+      </c>
+      <c r="M71" s="24">
+        <f>IF(ISNUMBER(J71),L71/G71,"")</f>
+        <v/>
+      </c>
+      <c r="N71" s="25">
+        <f>IF(ISNUMBER(H71),H71-C71,"")</f>
+        <v/>
+      </c>
+      <c r="O71" s="6" t="n"/>
+      <c r="P71" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M70">
+  <conditionalFormatting sqref="L2:M71">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 17:13 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA107" headerRowCount="1">
-  <autoFilter ref="A1:BA107"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA108" headerRowCount="1">
+  <autoFilter ref="A1:BA108"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.75469907407</v>
+        <v>46324.7590162037</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.54636574074</v>
+        <v>46324.55068287037</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$107,"BUY")+COUNTIF(Orders!$E$2:$E$107,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$108,"BUY")+COUNTIF(Orders!$E$2:$E$108,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$107,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$108,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$107,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$108,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$107,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$108,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$107,Orders!$E$2:$E$107,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$108,Orders!$E$2:$E$108,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$107,Orders!$E$2:$E$107,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$108,Orders!$E$2:$E$108,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA107"/>
+  <dimension ref="A1:BA108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18532,6 +18532,198 @@
       </c>
       <c r="BA107" s="6" t="n"/>
     </row>
+    <row r="108">
+      <c r="A108" s="12" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="13" t="n">
+        <v>46324.75886574074</v>
+      </c>
+      <c r="C108" s="13" t="n">
+        <v>46324.5505324074</v>
+      </c>
+      <c r="D108" s="13" t="n">
+        <v>46324.71719907408</v>
+      </c>
+      <c r="E108" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="G108" s="15" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I108" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J108" s="16" t="n">
+        <v>24.950127411</v>
+      </c>
+      <c r="K108" s="17" t="n">
+        <v>54.75</v>
+      </c>
+      <c r="L108" s="17">
+        <f>IF(AND(ISNUMBER(J108),ISNUMBER(K108)),J108*K108,"")</f>
+        <v/>
+      </c>
+      <c r="M108" s="17" t="n"/>
+      <c r="N108" s="16" t="n">
+        <v>24.950127411</v>
+      </c>
+      <c r="O108" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
+      <c r="P108" s="15" t="inlineStr">
+        <is>
+          <t>Only 2 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q108" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="R108" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S108" s="18" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="T108" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U108" s="19" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="V108" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W108" s="12" t="n"/>
+      <c r="X108" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y108" s="19" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="Z108" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AA108" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="AB108" s="15" t="inlineStr">
+        <is>
+          <t>Price gapped 5.1% at an open in the last week.; Rose 4.1% then gave back most of it within hours. Looks like pump-and-fade.</t>
+        </is>
+      </c>
+      <c r="AC108" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD108" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE108" s="17" t="n">
+        <v>55.5938</v>
+      </c>
+      <c r="AF108" s="17" t="n">
+        <v>53.5719</v>
+      </c>
+      <c r="AG108" s="17" t="n">
+        <v>57.6156</v>
+      </c>
+      <c r="AH108" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI108" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ108" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK108" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL108" s="15" t="inlineStr">
+        <is>
+          <t>UBS Maintains Buy on EQT, Lowers Price Target to $75</t>
+        </is>
+      </c>
+      <c r="AM108" s="17" t="n">
+        <v>54.785</v>
+      </c>
+      <c r="AN108" s="19" t="n">
+        <v>-0.0257</v>
+      </c>
+      <c r="AO108" s="17" t="n">
+        <v>99498.22</v>
+      </c>
+      <c r="AP108" s="17" t="n">
+        <v>13211.93</v>
+      </c>
+      <c r="AQ108" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR108" s="16" t="n">
+        <v>24.950127411</v>
+      </c>
+      <c r="AS108" s="17" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="AT108" s="19" t="n">
+        <v>-0.0033</v>
+      </c>
+      <c r="AU108" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV108" s="6" t="inlineStr">
+        <is>
+          <t>3539abf7-dadc-480f-b7ab-2912f7545db5</t>
+        </is>
+      </c>
+      <c r="AW108" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-EQT-1793293964775</t>
+        </is>
+      </c>
+      <c r="AX108" s="13" t="n">
+        <v>46324.71717592593</v>
+      </c>
+      <c r="AY108" s="13" t="n">
+        <v>46324.71719907408</v>
+      </c>
+      <c r="AZ108" s="13" t="n">
+        <v>46324.71689814814</v>
+      </c>
+      <c r="BA108" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -22741,9 +22933,15 @@
         <f>E70*F70</f>
         <v/>
       </c>
-      <c r="H70" s="22" t="n"/>
-      <c r="I70" s="22" t="n"/>
-      <c r="J70" s="17" t="n"/>
+      <c r="H70" s="22" t="n">
+        <v>46324.75886574074</v>
+      </c>
+      <c r="I70" s="22" t="n">
+        <v>46324.5505324074</v>
+      </c>
+      <c r="J70" s="17" t="n">
+        <v>54.75</v>
+      </c>
       <c r="K70" s="17">
         <f>IF(ISNUMBER(J70),J70*F70,"")</f>
         <v/>
@@ -22760,10 +22958,14 @@
         <f>IF(ISNUMBER(H70),H70-C70,"")</f>
         <v/>
       </c>
-      <c r="O70" s="6" t="n"/>
+      <c r="O70" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
       <c r="P70" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-29 17:31 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA108" headerRowCount="1">
-  <autoFilter ref="A1:BA108"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA109" headerRowCount="1">
+  <autoFilter ref="A1:BA109"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.7590162037</v>
+        <v>46324.77162037037</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.55068287037</v>
+        <v>46324.56328703704</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$108,"BUY")+COUNTIF(Orders!$E$2:$E$108,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$109,"BUY")+COUNTIF(Orders!$E$2:$E$109,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$108,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$109,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$108,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$109,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$108,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$109,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$108,Orders!$E$2:$E$108,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$109,Orders!$E$2:$E$109,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$108,Orders!$E$2:$E$108,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$109,Orders!$E$2:$E$109,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA108"/>
+  <dimension ref="A1:BA109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18724,6 +18724,114 @@
       </c>
       <c r="BA108" s="6" t="n"/>
     </row>
+    <row r="109">
+      <c r="A109" s="12" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="13" t="n">
+        <v>46324.76877314815</v>
+      </c>
+      <c r="C109" s="13" t="n">
+        <v>46324.56043981481</v>
+      </c>
+      <c r="D109" s="13" t="n">
+        <v>46324.72710648148</v>
+      </c>
+      <c r="E109" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="G109" s="15" t="n"/>
+      <c r="H109" s="6" t="n"/>
+      <c r="I109" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J109" s="16" t="n">
+        <v>2.303818963</v>
+      </c>
+      <c r="K109" s="17" t="n">
+        <v>289.14</v>
+      </c>
+      <c r="L109" s="17">
+        <f>IF(AND(ISNUMBER(J109),ISNUMBER(K109)),J109*K109,"")</f>
+        <v/>
+      </c>
+      <c r="M109" s="17" t="n"/>
+      <c r="N109" s="16" t="n">
+        <v>2.303818963</v>
+      </c>
+      <c r="O109" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
+      <c r="P109" s="15" t="inlineStr">
+        <is>
+          <t>Alpaca stop order triggered at 289.95 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q109" s="12" t="n"/>
+      <c r="R109" s="6" t="n"/>
+      <c r="S109" s="18" t="n"/>
+      <c r="T109" s="12" t="n"/>
+      <c r="U109" s="19" t="n"/>
+      <c r="V109" s="19" t="n"/>
+      <c r="W109" s="12" t="n"/>
+      <c r="X109" s="6" t="n"/>
+      <c r="Y109" s="19" t="n"/>
+      <c r="Z109" s="6" t="n"/>
+      <c r="AA109" s="12" t="n"/>
+      <c r="AB109" s="15" t="n"/>
+      <c r="AC109" s="6" t="n"/>
+      <c r="AD109" s="6" t="n"/>
+      <c r="AE109" s="17" t="n"/>
+      <c r="AF109" s="17" t="n"/>
+      <c r="AG109" s="17" t="n"/>
+      <c r="AH109" s="20" t="n"/>
+      <c r="AI109" s="18" t="n"/>
+      <c r="AJ109" s="6" t="n"/>
+      <c r="AK109" s="12" t="n"/>
+      <c r="AL109" s="15" t="n"/>
+      <c r="AM109" s="17" t="n"/>
+      <c r="AN109" s="19" t="n"/>
+      <c r="AO109" s="17" t="n"/>
+      <c r="AP109" s="17" t="n"/>
+      <c r="AQ109" s="19" t="n"/>
+      <c r="AR109" s="16" t="n"/>
+      <c r="AS109" s="17" t="n"/>
+      <c r="AT109" s="19" t="n"/>
+      <c r="AU109" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV109" s="6" t="inlineStr">
+        <is>
+          <t>ce4efa09-f361-4d52-9ef0-72a2d170660d</t>
+        </is>
+      </c>
+      <c r="AW109" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-stop-ILMN-1793293969433</t>
+        </is>
+      </c>
+      <c r="AX109" s="13" t="n">
+        <v>46324.7172337963</v>
+      </c>
+      <c r="AY109" s="13" t="n">
+        <v>46324.72710648148</v>
+      </c>
+      <c r="AZ109" s="13" t="n"/>
+      <c r="BA109" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -22721,9 +22829,15 @@
         <f>E66*F66</f>
         <v/>
       </c>
-      <c r="H66" s="22" t="n"/>
-      <c r="I66" s="22" t="n"/>
-      <c r="J66" s="17" t="n"/>
+      <c r="H66" s="22" t="n">
+        <v>46324.76877314815</v>
+      </c>
+      <c r="I66" s="22" t="n">
+        <v>46324.56043981481</v>
+      </c>
+      <c r="J66" s="17" t="n">
+        <v>289.14</v>
+      </c>
       <c r="K66" s="17">
         <f>IF(ISNUMBER(J66),J66*F66,"")</f>
         <v/>
@@ -22740,10 +22854,14 @@
         <f>IF(ISNUMBER(H66),H66-C66,"")</f>
         <v/>
       </c>
-      <c r="O66" s="6" t="n"/>
+      <c r="O66" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P66" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-29 17:36 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA109" headerRowCount="1">
-  <autoFilter ref="A1:BA109"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA110" headerRowCount="1">
+  <autoFilter ref="A1:BA110"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P71" headerRowCount="1">
-  <autoFilter ref="A1:P71"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P72" headerRowCount="1">
+  <autoFilter ref="A1:P72"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.77162037037</v>
+        <v>46324.77552083333</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.56328703704</v>
+        <v>46324.5671875</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$109,"BUY")+COUNTIF(Orders!$E$2:$E$109,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$110,"BUY")+COUNTIF(Orders!$E$2:$E$110,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$109,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$110,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$109,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$110,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$109,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$110,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$109,Orders!$E$2:$E$109,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$110,Orders!$E$2:$E$110,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$109,Orders!$E$2:$E$109,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$110,Orders!$E$2:$E$110,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$71,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$72,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$71,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$72,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$71)</f>
+        <f>SUM('Round trips'!$L$2:$L$72)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$71,"Closed",'Round trips'!$L$2:$L$71,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$72,"Closed",'Round trips'!$L$2:$L$72,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA109"/>
+  <dimension ref="A1:BA110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18832,6 +18832,190 @@
       <c r="AZ109" s="13" t="n"/>
       <c r="BA109" s="6" t="n"/>
     </row>
+    <row r="110">
+      <c r="A110" s="12" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="13" t="n">
+        <v>46324.77543981482</v>
+      </c>
+      <c r="C110" s="13" t="n">
+        <v>46324.56710648148</v>
+      </c>
+      <c r="D110" s="13" t="n">
+        <v>46324.73377314815</v>
+      </c>
+      <c r="E110" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="G110" s="15" t="inlineStr">
+        <is>
+          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J110" s="16" t="n">
+        <v>1.562144008</v>
+      </c>
+      <c r="K110" s="17" t="n">
+        <v>812.87</v>
+      </c>
+      <c r="L110" s="17">
+        <f>IF(AND(ISNUMBER(J110),ISNUMBER(K110)),J110*K110,"")</f>
+        <v/>
+      </c>
+      <c r="M110" s="17" t="n">
+        <v>1269.83</v>
+      </c>
+      <c r="N110" s="16" t="n"/>
+      <c r="O110" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P110" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $15,244.08 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q110" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R110" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S110" s="18" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="T110" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U110" s="19" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="V110" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W110" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X110" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y110" s="19" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="Z110" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA110" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB110" s="15" t="n"/>
+      <c r="AC110" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD110" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE110" s="17" t="n">
+        <v>824.77</v>
+      </c>
+      <c r="AF110" s="17" t="n">
+        <v>793.6451</v>
+      </c>
+      <c r="AG110" s="17" t="n">
+        <v>855.8949</v>
+      </c>
+      <c r="AH110" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI110" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ110" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK110" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL110" s="15" t="inlineStr">
+        <is>
+          <t>Canaccord Genuity Maintains Buy on Regeneron Pharmaceuticals, Raises Price Target to $922</t>
+        </is>
+      </c>
+      <c r="AM110" s="17" t="n">
+        <v>812.3200000000001</v>
+      </c>
+      <c r="AN110" s="19" t="n">
+        <v>-0.0016</v>
+      </c>
+      <c r="AO110" s="17" t="n">
+        <v>99345.75</v>
+      </c>
+      <c r="AP110" s="17" t="n">
+        <v>15244.08</v>
+      </c>
+      <c r="AQ110" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR110" s="16" t="n"/>
+      <c r="AS110" s="17" t="n"/>
+      <c r="AT110" s="19" t="n"/>
+      <c r="AU110" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV110" s="6" t="inlineStr">
+        <is>
+          <t>1f5a23ed-afbf-4216-8e41-ba5eccfed86a</t>
+        </is>
+      </c>
+      <c r="AW110" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-REGN-1793295398213</t>
+        </is>
+      </c>
+      <c r="AX110" s="13" t="n">
+        <v>46324.73377314815</v>
+      </c>
+      <c r="AY110" s="13" t="n">
+        <v>46324.73377314815</v>
+      </c>
+      <c r="AZ110" s="13" t="n">
+        <v>46324.73350694445</v>
+      </c>
+      <c r="BA110" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -18847,7 +19031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P71"/>
+  <dimension ref="A1:P72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -23140,8 +23324,61 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C72" s="22" t="n">
+        <v>46324.77543981482</v>
+      </c>
+      <c r="D72" s="22" t="n">
+        <v>46324.56710648148</v>
+      </c>
+      <c r="E72" s="17" t="n">
+        <v>812.87</v>
+      </c>
+      <c r="F72" s="16" t="n">
+        <v>1.562144008</v>
+      </c>
+      <c r="G72" s="17">
+        <f>E72*F72</f>
+        <v/>
+      </c>
+      <c r="H72" s="22" t="n"/>
+      <c r="I72" s="22" t="n"/>
+      <c r="J72" s="17" t="n"/>
+      <c r="K72" s="17">
+        <f>IF(ISNUMBER(J72),J72*F72,"")</f>
+        <v/>
+      </c>
+      <c r="L72" s="23">
+        <f>IF(ISNUMBER(J72),K72-G72,"")</f>
+        <v/>
+      </c>
+      <c r="M72" s="24">
+        <f>IF(ISNUMBER(J72),L72/G72,"")</f>
+        <v/>
+      </c>
+      <c r="N72" s="25">
+        <f>IF(ISNUMBER(H72),H72-C72,"")</f>
+        <v/>
+      </c>
+      <c r="O72" s="6" t="n"/>
+      <c r="P72" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M71">
+  <conditionalFormatting sqref="L2:M72">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 18:01 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA110" headerRowCount="1">
-  <autoFilter ref="A1:BA110"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA112" headerRowCount="1">
+  <autoFilter ref="A1:BA112"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.77552083333</v>
+        <v>46324.7925462963</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.5671875</v>
+        <v>46324.58421296296</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$110,"BUY")+COUNTIF(Orders!$E$2:$E$110,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$112,"BUY")+COUNTIF(Orders!$E$2:$E$112,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$110,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$112,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$110,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$112,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$110,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$112,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$110,Orders!$E$2:$E$110,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$112,Orders!$E$2:$E$112,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$110,Orders!$E$2:$E$110,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$112,Orders!$E$2:$E$112,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA110"/>
+  <dimension ref="A1:BA112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18349,13 +18349,13 @@
         <v>106</v>
       </c>
       <c r="B107" s="13" t="n">
-        <v>46324.75462962963</v>
+        <v>46324.78903935185</v>
       </c>
       <c r="C107" s="13" t="n">
-        <v>46324.5462962963</v>
+        <v>46324.58070601852</v>
       </c>
       <c r="D107" s="13" t="n">
-        <v>46324.71296296296</v>
+        <v>46324.74737268518</v>
       </c>
       <c r="E107" s="21" t="inlineStr">
         <is>
@@ -18364,29 +18364,21 @@
       </c>
       <c r="F107" s="6" t="inlineStr">
         <is>
-          <t>ACN</t>
-        </is>
-      </c>
-      <c r="G107" s="15" t="inlineStr">
-        <is>
-          <t>ACN</t>
-        </is>
-      </c>
-      <c r="H107" s="6" t="inlineStr">
-        <is>
-          <t>NYSE</t>
-        </is>
-      </c>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="G107" s="15" t="n"/>
+      <c r="H107" s="6" t="n"/>
       <c r="I107" s="6" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
       <c r="J107" s="16" t="n">
-        <v>1.363168471</v>
+        <v>40.314736203</v>
       </c>
       <c r="K107" s="17" t="n">
-        <v>245.55</v>
+        <v>16.54</v>
       </c>
       <c r="L107" s="17">
         <f>IF(AND(ISNUMBER(J107),ISNUMBER(K107)),J107*K107,"")</f>
@@ -18394,118 +18386,48 @@
       </c>
       <c r="M107" s="17" t="n"/>
       <c r="N107" s="16" t="n">
-        <v>1.363168471</v>
+        <v>40.314736203</v>
       </c>
       <c r="O107" s="6" t="inlineStr">
         <is>
-          <t>3 green: sell half</t>
+          <t>stop-loss (Alpaca order)</t>
         </is>
       </c>
       <c r="P107" s="15" t="inlineStr">
         <is>
-          <t>3 of 5 green: start selling (half)</t>
-        </is>
-      </c>
-      <c r="Q107" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="R107" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="S107" s="18" t="n">
-        <v>0.551</v>
-      </c>
-      <c r="T107" s="12" t="n">
-        <v>49</v>
-      </c>
-      <c r="U107" s="19" t="n">
-        <v>0.0072</v>
-      </c>
-      <c r="V107" s="19" t="n">
-        <v>0.2893</v>
-      </c>
+          <t>Alpaca stop order triggered at 16.55 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q107" s="12" t="n"/>
+      <c r="R107" s="6" t="n"/>
+      <c r="S107" s="18" t="n"/>
+      <c r="T107" s="12" t="n"/>
+      <c r="U107" s="19" t="n"/>
+      <c r="V107" s="19" t="n"/>
       <c r="W107" s="12" t="n"/>
-      <c r="X107" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y107" s="19" t="n">
-        <v>0.0014</v>
-      </c>
-      <c r="Z107" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AA107" s="12" t="n">
-        <v>100</v>
-      </c>
+      <c r="X107" s="6" t="n"/>
+      <c r="Y107" s="19" t="n"/>
+      <c r="Z107" s="6" t="n"/>
+      <c r="AA107" s="12" t="n"/>
       <c r="AB107" s="15" t="n"/>
-      <c r="AC107" s="6" t="inlineStr">
-        <is>
-          <t>watch</t>
-        </is>
-      </c>
-      <c r="AD107" s="6" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="AE107" s="17" t="n">
-        <v>245.24</v>
-      </c>
-      <c r="AF107" s="17" t="n">
-        <v>226.362</v>
-      </c>
-      <c r="AG107" s="17" t="n">
-        <v>264.118</v>
-      </c>
-      <c r="AH107" s="20" t="n">
-        <v>46331</v>
-      </c>
-      <c r="AI107" s="18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AJ107" s="6" t="inlineStr">
-        <is>
-          <t>watch</t>
-        </is>
-      </c>
-      <c r="AK107" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL107" s="15" t="inlineStr">
-        <is>
-          <t>Accenture Recognized in 2026 Guidewire PartnerConnect Excellence Awards</t>
-        </is>
-      </c>
-      <c r="AM107" s="17" t="n">
-        <v>245.585</v>
-      </c>
-      <c r="AN107" s="19" t="n">
-        <v>0.005699999999999999</v>
-      </c>
-      <c r="AO107" s="17" t="n">
-        <v>99521.99000000001</v>
-      </c>
-      <c r="AP107" s="17" t="n">
-        <v>12877.2</v>
-      </c>
-      <c r="AQ107" s="19" t="n">
-        <v>0.0833</v>
-      </c>
-      <c r="AR107" s="16" t="n">
-        <v>2.726336942</v>
-      </c>
-      <c r="AS107" s="17" t="n">
-        <v>243.84</v>
-      </c>
-      <c r="AT107" s="19" t="n">
-        <v>0.0072</v>
-      </c>
+      <c r="AC107" s="6" t="n"/>
+      <c r="AD107" s="6" t="n"/>
+      <c r="AE107" s="17" t="n"/>
+      <c r="AF107" s="17" t="n"/>
+      <c r="AG107" s="17" t="n"/>
+      <c r="AH107" s="20" t="n"/>
+      <c r="AI107" s="18" t="n"/>
+      <c r="AJ107" s="6" t="n"/>
+      <c r="AK107" s="12" t="n"/>
+      <c r="AL107" s="15" t="n"/>
+      <c r="AM107" s="17" t="n"/>
+      <c r="AN107" s="19" t="n"/>
+      <c r="AO107" s="17" t="n"/>
+      <c r="AP107" s="17" t="n"/>
+      <c r="AQ107" s="19" t="n"/>
+      <c r="AR107" s="16" t="n"/>
+      <c r="AS107" s="17" t="n"/>
+      <c r="AT107" s="19" t="n"/>
       <c r="AU107" s="6" t="inlineStr">
         <is>
           <t>paper</t>
@@ -18513,23 +18435,21 @@
       </c>
       <c r="AV107" s="6" t="inlineStr">
         <is>
-          <t>54ffb774-a2a5-48dc-bed4-428649caa4b4</t>
+          <t>c5898ad1-8ed5-4f96-859c-f303e2b03686</t>
         </is>
       </c>
       <c r="AW107" s="6" t="inlineStr">
         <is>
-          <t>tdagent-sell-ACN-1793293599550</t>
+          <t>tdagent-stop-AVTR-1793291808809</t>
         </is>
       </c>
       <c r="AX107" s="13" t="n">
-        <v>46324.71295138889</v>
+        <v>46324.69222222222</v>
       </c>
       <c r="AY107" s="13" t="n">
-        <v>46324.71296296296</v>
-      </c>
-      <c r="AZ107" s="13" t="n">
-        <v>46324.71270833333</v>
-      </c>
+        <v>46324.74737268518</v>
+      </c>
+      <c r="AZ107" s="13" t="n"/>
       <c r="BA107" s="6" t="n"/>
     </row>
     <row r="108">
@@ -18537,13 +18457,13 @@
         <v>107</v>
       </c>
       <c r="B108" s="13" t="n">
-        <v>46324.75886574074</v>
+        <v>46324.75462962963</v>
       </c>
       <c r="C108" s="13" t="n">
-        <v>46324.5505324074</v>
+        <v>46324.5462962963</v>
       </c>
       <c r="D108" s="13" t="n">
-        <v>46324.71719907408</v>
+        <v>46324.71296296296</v>
       </c>
       <c r="E108" s="21" t="inlineStr">
         <is>
@@ -18552,12 +18472,12 @@
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="G108" s="15" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="H108" s="6" t="inlineStr">
@@ -18571,10 +18491,10 @@
         </is>
       </c>
       <c r="J108" s="16" t="n">
-        <v>24.950127411</v>
+        <v>1.363168471</v>
       </c>
       <c r="K108" s="17" t="n">
-        <v>54.75</v>
+        <v>245.55</v>
       </c>
       <c r="L108" s="17">
         <f>IF(AND(ISNUMBER(J108),ISNUMBER(K108)),J108*K108,"")</f>
@@ -18582,20 +18502,20 @@
       </c>
       <c r="M108" s="17" t="n"/>
       <c r="N108" s="16" t="n">
-        <v>24.950127411</v>
+        <v>1.363168471</v>
       </c>
       <c r="O108" s="6" t="inlineStr">
         <is>
-          <t>2 or fewer green</t>
+          <t>3 green: sell half</t>
         </is>
       </c>
       <c r="P108" s="15" t="inlineStr">
         <is>
-          <t>Only 2 of 5 green</t>
+          <t>3 of 5 green: start selling (half)</t>
         </is>
       </c>
       <c r="Q108" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R108" s="6" t="inlineStr">
         <is>
@@ -18603,13 +18523,13 @@
         </is>
       </c>
       <c r="S108" s="18" t="n">
-        <v>0.552</v>
+        <v>0.551</v>
       </c>
       <c r="T108" s="12" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="U108" s="19" t="n">
-        <v>0.0017</v>
+        <v>0.0072</v>
       </c>
       <c r="V108" s="19" t="n">
         <v>0.2893</v>
@@ -18625,17 +18545,13 @@
       </c>
       <c r="Z108" s="6" t="inlineStr">
         <is>
-          <t>alert</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AA108" s="12" t="n">
-        <v>60</v>
-      </c>
-      <c r="AB108" s="15" t="inlineStr">
-        <is>
-          <t>Price gapped 5.1% at an open in the last week.; Rose 4.1% then gave back most of it within hours. Looks like pump-and-fade.</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="AB108" s="15" t="n"/>
       <c r="AC108" s="6" t="inlineStr">
         <is>
           <t>watch</t>
@@ -18643,23 +18559,23 @@
       </c>
       <c r="AD108" s="6" t="inlineStr">
         <is>
-          <t>up</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="AE108" s="17" t="n">
-        <v>55.5938</v>
+        <v>245.24</v>
       </c>
       <c r="AF108" s="17" t="n">
-        <v>53.5719</v>
+        <v>226.362</v>
       </c>
       <c r="AG108" s="17" t="n">
-        <v>57.6156</v>
+        <v>264.118</v>
       </c>
       <c r="AH108" s="20" t="n">
         <v>46331</v>
       </c>
       <c r="AI108" s="18" t="n">
-        <v>0.54</v>
+        <v>0.5</v>
       </c>
       <c r="AJ108" s="6" t="inlineStr">
         <is>
@@ -18671,32 +18587,32 @@
       </c>
       <c r="AL108" s="15" t="inlineStr">
         <is>
-          <t>UBS Maintains Buy on EQT, Lowers Price Target to $75</t>
+          <t>Accenture Recognized in 2026 Guidewire PartnerConnect Excellence Awards</t>
         </is>
       </c>
       <c r="AM108" s="17" t="n">
-        <v>54.785</v>
+        <v>245.585</v>
       </c>
       <c r="AN108" s="19" t="n">
-        <v>-0.0257</v>
+        <v>0.005699999999999999</v>
       </c>
       <c r="AO108" s="17" t="n">
-        <v>99498.22</v>
+        <v>99521.99000000001</v>
       </c>
       <c r="AP108" s="17" t="n">
-        <v>13211.93</v>
+        <v>12877.2</v>
       </c>
       <c r="AQ108" s="19" t="n">
         <v>0.0833</v>
       </c>
       <c r="AR108" s="16" t="n">
-        <v>24.950127411</v>
+        <v>2.726336942</v>
       </c>
       <c r="AS108" s="17" t="n">
-        <v>54.94</v>
+        <v>243.84</v>
       </c>
       <c r="AT108" s="19" t="n">
-        <v>-0.0033</v>
+        <v>0.0072</v>
       </c>
       <c r="AU108" s="6" t="inlineStr">
         <is>
@@ -18705,22 +18621,22 @@
       </c>
       <c r="AV108" s="6" t="inlineStr">
         <is>
-          <t>3539abf7-dadc-480f-b7ab-2912f7545db5</t>
+          <t>54ffb774-a2a5-48dc-bed4-428649caa4b4</t>
         </is>
       </c>
       <c r="AW108" s="6" t="inlineStr">
         <is>
-          <t>tdagent-sell-EQT-1793293964775</t>
+          <t>tdagent-sell-ACN-1793293599550</t>
         </is>
       </c>
       <c r="AX108" s="13" t="n">
-        <v>46324.71717592593</v>
+        <v>46324.71295138889</v>
       </c>
       <c r="AY108" s="13" t="n">
-        <v>46324.71719907408</v>
+        <v>46324.71296296296</v>
       </c>
       <c r="AZ108" s="13" t="n">
-        <v>46324.71689814814</v>
+        <v>46324.71270833333</v>
       </c>
       <c r="BA108" s="6" t="n"/>
     </row>
@@ -18729,13 +18645,13 @@
         <v>108</v>
       </c>
       <c r="B109" s="13" t="n">
-        <v>46324.76877314815</v>
+        <v>46324.75886574074</v>
       </c>
       <c r="C109" s="13" t="n">
-        <v>46324.56043981481</v>
+        <v>46324.5505324074</v>
       </c>
       <c r="D109" s="13" t="n">
-        <v>46324.72710648148</v>
+        <v>46324.71719907408</v>
       </c>
       <c r="E109" s="21" t="inlineStr">
         <is>
@@ -18744,21 +18660,29 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>ILMN</t>
-        </is>
-      </c>
-      <c r="G109" s="15" t="n"/>
-      <c r="H109" s="6" t="n"/>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="G109" s="15" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
       <c r="I109" s="6" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
       <c r="J109" s="16" t="n">
-        <v>2.303818963</v>
+        <v>24.950127411</v>
       </c>
       <c r="K109" s="17" t="n">
-        <v>289.14</v>
+        <v>54.75</v>
       </c>
       <c r="L109" s="17">
         <f>IF(AND(ISNUMBER(J109),ISNUMBER(K109)),J109*K109,"")</f>
@@ -18766,48 +18690,122 @@
       </c>
       <c r="M109" s="17" t="n"/>
       <c r="N109" s="16" t="n">
-        <v>2.303818963</v>
+        <v>24.950127411</v>
       </c>
       <c r="O109" s="6" t="inlineStr">
         <is>
-          <t>stop-loss (Alpaca order)</t>
+          <t>2 or fewer green</t>
         </is>
       </c>
       <c r="P109" s="15" t="inlineStr">
         <is>
-          <t>Alpaca stop order triggered at 289.95 (the stock's sell line)</t>
-        </is>
-      </c>
-      <c r="Q109" s="12" t="n"/>
-      <c r="R109" s="6" t="n"/>
-      <c r="S109" s="18" t="n"/>
-      <c r="T109" s="12" t="n"/>
-      <c r="U109" s="19" t="n"/>
-      <c r="V109" s="19" t="n"/>
+          <t>Only 2 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q109" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="R109" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S109" s="18" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="T109" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U109" s="19" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="V109" s="19" t="n">
+        <v>0.2893</v>
+      </c>
       <c r="W109" s="12" t="n"/>
-      <c r="X109" s="6" t="n"/>
-      <c r="Y109" s="19" t="n"/>
-      <c r="Z109" s="6" t="n"/>
-      <c r="AA109" s="12" t="n"/>
-      <c r="AB109" s="15" t="n"/>
-      <c r="AC109" s="6" t="n"/>
-      <c r="AD109" s="6" t="n"/>
-      <c r="AE109" s="17" t="n"/>
-      <c r="AF109" s="17" t="n"/>
-      <c r="AG109" s="17" t="n"/>
-      <c r="AH109" s="20" t="n"/>
-      <c r="AI109" s="18" t="n"/>
-      <c r="AJ109" s="6" t="n"/>
-      <c r="AK109" s="12" t="n"/>
-      <c r="AL109" s="15" t="n"/>
-      <c r="AM109" s="17" t="n"/>
-      <c r="AN109" s="19" t="n"/>
-      <c r="AO109" s="17" t="n"/>
-      <c r="AP109" s="17" t="n"/>
-      <c r="AQ109" s="19" t="n"/>
-      <c r="AR109" s="16" t="n"/>
-      <c r="AS109" s="17" t="n"/>
-      <c r="AT109" s="19" t="n"/>
+      <c r="X109" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y109" s="19" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="Z109" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AA109" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="AB109" s="15" t="inlineStr">
+        <is>
+          <t>Price gapped 5.1% at an open in the last week.; Rose 4.1% then gave back most of it within hours. Looks like pump-and-fade.</t>
+        </is>
+      </c>
+      <c r="AC109" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD109" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE109" s="17" t="n">
+        <v>55.5938</v>
+      </c>
+      <c r="AF109" s="17" t="n">
+        <v>53.5719</v>
+      </c>
+      <c r="AG109" s="17" t="n">
+        <v>57.6156</v>
+      </c>
+      <c r="AH109" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI109" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ109" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK109" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL109" s="15" t="inlineStr">
+        <is>
+          <t>UBS Maintains Buy on EQT, Lowers Price Target to $75</t>
+        </is>
+      </c>
+      <c r="AM109" s="17" t="n">
+        <v>54.785</v>
+      </c>
+      <c r="AN109" s="19" t="n">
+        <v>-0.0257</v>
+      </c>
+      <c r="AO109" s="17" t="n">
+        <v>99498.22</v>
+      </c>
+      <c r="AP109" s="17" t="n">
+        <v>13211.93</v>
+      </c>
+      <c r="AQ109" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR109" s="16" t="n">
+        <v>24.950127411</v>
+      </c>
+      <c r="AS109" s="17" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="AT109" s="19" t="n">
+        <v>-0.0033</v>
+      </c>
       <c r="AU109" s="6" t="inlineStr">
         <is>
           <t>paper</t>
@@ -18815,21 +18813,23 @@
       </c>
       <c r="AV109" s="6" t="inlineStr">
         <is>
-          <t>ce4efa09-f361-4d52-9ef0-72a2d170660d</t>
+          <t>3539abf7-dadc-480f-b7ab-2912f7545db5</t>
         </is>
       </c>
       <c r="AW109" s="6" t="inlineStr">
         <is>
-          <t>tdagent-stop-ILMN-1793293969433</t>
+          <t>tdagent-sell-EQT-1793293964775</t>
         </is>
       </c>
       <c r="AX109" s="13" t="n">
-        <v>46324.7172337963</v>
+        <v>46324.71717592593</v>
       </c>
       <c r="AY109" s="13" t="n">
-        <v>46324.72710648148</v>
-      </c>
-      <c r="AZ109" s="13" t="n"/>
+        <v>46324.71719907408</v>
+      </c>
+      <c r="AZ109" s="13" t="n">
+        <v>46324.71689814814</v>
+      </c>
       <c r="BA109" s="6" t="n"/>
     </row>
     <row r="110">
@@ -18837,156 +18837,82 @@
         <v>109</v>
       </c>
       <c r="B110" s="13" t="n">
-        <v>46324.77543981482</v>
+        <v>46324.76877314815</v>
       </c>
       <c r="C110" s="13" t="n">
-        <v>46324.56710648148</v>
+        <v>46324.56043981481</v>
       </c>
       <c r="D110" s="13" t="n">
-        <v>46324.73377314815</v>
-      </c>
-      <c r="E110" s="14" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>46324.72710648148</v>
+      </c>
+      <c r="E110" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F110" s="6" t="inlineStr">
         <is>
-          <t>REGN</t>
-        </is>
-      </c>
-      <c r="G110" s="15" t="inlineStr">
-        <is>
-          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
-        </is>
-      </c>
-      <c r="H110" s="6" t="inlineStr">
-        <is>
-          <t>NASDAQ</t>
-        </is>
-      </c>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="G110" s="15" t="n"/>
+      <c r="H110" s="6" t="n"/>
       <c r="I110" s="6" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
       <c r="J110" s="16" t="n">
-        <v>1.562144008</v>
+        <v>2.303818963</v>
       </c>
       <c r="K110" s="17" t="n">
-        <v>812.87</v>
+        <v>289.14</v>
       </c>
       <c r="L110" s="17">
         <f>IF(AND(ISNUMBER(J110),ISNUMBER(K110)),J110*K110,"")</f>
         <v/>
       </c>
-      <c r="M110" s="17" t="n">
-        <v>1269.83</v>
-      </c>
-      <c r="N110" s="16" t="n"/>
+      <c r="M110" s="17" t="n"/>
+      <c r="N110" s="16" t="n">
+        <v>2.303818963</v>
+      </c>
       <c r="O110" s="6" t="inlineStr">
         <is>
-          <t>4+/5 green</t>
+          <t>stop-loss (Alpaca order)</t>
         </is>
       </c>
       <c r="P110" s="15" t="inlineStr">
         <is>
-          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $15,244.08 free cash split 12 ways</t>
-        </is>
-      </c>
-      <c r="Q110" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="R110" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="S110" s="18" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="T110" s="12" t="n">
-        <v>39</v>
-      </c>
-      <c r="U110" s="19" t="n">
-        <v>0.0069</v>
-      </c>
-      <c r="V110" s="19" t="n">
-        <v>0.2893</v>
-      </c>
-      <c r="W110" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="X110" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y110" s="19" t="n">
-        <v>0.0018</v>
-      </c>
-      <c r="Z110" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AA110" s="12" t="n">
-        <v>100</v>
-      </c>
+          <t>Alpaca stop order triggered at 289.95 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q110" s="12" t="n"/>
+      <c r="R110" s="6" t="n"/>
+      <c r="S110" s="18" t="n"/>
+      <c r="T110" s="12" t="n"/>
+      <c r="U110" s="19" t="n"/>
+      <c r="V110" s="19" t="n"/>
+      <c r="W110" s="12" t="n"/>
+      <c r="X110" s="6" t="n"/>
+      <c r="Y110" s="19" t="n"/>
+      <c r="Z110" s="6" t="n"/>
+      <c r="AA110" s="12" t="n"/>
       <c r="AB110" s="15" t="n"/>
-      <c r="AC110" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AD110" s="6" t="inlineStr">
-        <is>
-          <t>up</t>
-        </is>
-      </c>
-      <c r="AE110" s="17" t="n">
-        <v>824.77</v>
-      </c>
-      <c r="AF110" s="17" t="n">
-        <v>793.6451</v>
-      </c>
-      <c r="AG110" s="17" t="n">
-        <v>855.8949</v>
-      </c>
-      <c r="AH110" s="20" t="n">
-        <v>46331</v>
-      </c>
-      <c r="AI110" s="18" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="AJ110" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AK110" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL110" s="15" t="inlineStr">
-        <is>
-          <t>Canaccord Genuity Maintains Buy on Regeneron Pharmaceuticals, Raises Price Target to $922</t>
-        </is>
-      </c>
-      <c r="AM110" s="17" t="n">
-        <v>812.3200000000001</v>
-      </c>
-      <c r="AN110" s="19" t="n">
-        <v>-0.0016</v>
-      </c>
-      <c r="AO110" s="17" t="n">
-        <v>99345.75</v>
-      </c>
-      <c r="AP110" s="17" t="n">
-        <v>15244.08</v>
-      </c>
-      <c r="AQ110" s="19" t="n">
-        <v>0.0833</v>
-      </c>
+      <c r="AC110" s="6" t="n"/>
+      <c r="AD110" s="6" t="n"/>
+      <c r="AE110" s="17" t="n"/>
+      <c r="AF110" s="17" t="n"/>
+      <c r="AG110" s="17" t="n"/>
+      <c r="AH110" s="20" t="n"/>
+      <c r="AI110" s="18" t="n"/>
+      <c r="AJ110" s="6" t="n"/>
+      <c r="AK110" s="12" t="n"/>
+      <c r="AL110" s="15" t="n"/>
+      <c r="AM110" s="17" t="n"/>
+      <c r="AN110" s="19" t="n"/>
+      <c r="AO110" s="17" t="n"/>
+      <c r="AP110" s="17" t="n"/>
+      <c r="AQ110" s="19" t="n"/>
       <c r="AR110" s="16" t="n"/>
       <c r="AS110" s="17" t="n"/>
       <c r="AT110" s="19" t="n"/>
@@ -18997,24 +18923,314 @@
       </c>
       <c r="AV110" s="6" t="inlineStr">
         <is>
+          <t>ce4efa09-f361-4d52-9ef0-72a2d170660d</t>
+        </is>
+      </c>
+      <c r="AW110" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-stop-ILMN-1793293969433</t>
+        </is>
+      </c>
+      <c r="AX110" s="13" t="n">
+        <v>46324.7172337963</v>
+      </c>
+      <c r="AY110" s="13" t="n">
+        <v>46324.72710648148</v>
+      </c>
+      <c r="AZ110" s="13" t="n"/>
+      <c r="BA110" s="6" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="12" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="13" t="n">
+        <v>46324.78953703704</v>
+      </c>
+      <c r="C111" s="13" t="n">
+        <v>46324.5812037037</v>
+      </c>
+      <c r="D111" s="13" t="n">
+        <v>46324.74787037037</v>
+      </c>
+      <c r="E111" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="G111" s="15" t="n"/>
+      <c r="H111" s="6" t="n"/>
+      <c r="I111" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J111" s="16" t="n">
+        <v>11.851651941</v>
+      </c>
+      <c r="K111" s="17" t="n">
+        <v>704.25</v>
+      </c>
+      <c r="L111" s="17">
+        <f>IF(AND(ISNUMBER(J111),ISNUMBER(K111)),J111*K111,"")</f>
+        <v/>
+      </c>
+      <c r="M111" s="17" t="n"/>
+      <c r="N111" s="16" t="n">
+        <v>11.851651941</v>
+      </c>
+      <c r="O111" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
+      <c r="P111" s="15" t="inlineStr">
+        <is>
+          <t>Alpaca stop order triggered at 704.35 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q111" s="12" t="n"/>
+      <c r="R111" s="6" t="n"/>
+      <c r="S111" s="18" t="n"/>
+      <c r="T111" s="12" t="n"/>
+      <c r="U111" s="19" t="n"/>
+      <c r="V111" s="19" t="n"/>
+      <c r="W111" s="12" t="n"/>
+      <c r="X111" s="6" t="n"/>
+      <c r="Y111" s="19" t="n"/>
+      <c r="Z111" s="6" t="n"/>
+      <c r="AA111" s="12" t="n"/>
+      <c r="AB111" s="15" t="n"/>
+      <c r="AC111" s="6" t="n"/>
+      <c r="AD111" s="6" t="n"/>
+      <c r="AE111" s="17" t="n"/>
+      <c r="AF111" s="17" t="n"/>
+      <c r="AG111" s="17" t="n"/>
+      <c r="AH111" s="20" t="n"/>
+      <c r="AI111" s="18" t="n"/>
+      <c r="AJ111" s="6" t="n"/>
+      <c r="AK111" s="12" t="n"/>
+      <c r="AL111" s="15" t="n"/>
+      <c r="AM111" s="17" t="n"/>
+      <c r="AN111" s="19" t="n"/>
+      <c r="AO111" s="17" t="n"/>
+      <c r="AP111" s="17" t="n"/>
+      <c r="AQ111" s="19" t="n"/>
+      <c r="AR111" s="16" t="n"/>
+      <c r="AS111" s="17" t="n"/>
+      <c r="AT111" s="19" t="n"/>
+      <c r="AU111" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV111" s="6" t="inlineStr">
+        <is>
+          <t>40c48aa1-abe9-44e0-9690-d876391f8eb9</t>
+        </is>
+      </c>
+      <c r="AW111" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-stop-TMO-1793293970703</t>
+        </is>
+      </c>
+      <c r="AX111" s="13" t="n">
+        <v>46324.71724537037</v>
+      </c>
+      <c r="AY111" s="13" t="n">
+        <v>46324.74787037037</v>
+      </c>
+      <c r="AZ111" s="13" t="n"/>
+      <c r="BA111" s="6" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="12" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="13" t="n">
+        <v>46324.77543981482</v>
+      </c>
+      <c r="C112" s="13" t="n">
+        <v>46324.56710648148</v>
+      </c>
+      <c r="D112" s="13" t="n">
+        <v>46324.73377314815</v>
+      </c>
+      <c r="E112" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="G112" s="15" t="inlineStr">
+        <is>
+          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I112" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J112" s="16" t="n">
+        <v>1.562144008</v>
+      </c>
+      <c r="K112" s="17" t="n">
+        <v>812.87</v>
+      </c>
+      <c r="L112" s="17">
+        <f>IF(AND(ISNUMBER(J112),ISNUMBER(K112)),J112*K112,"")</f>
+        <v/>
+      </c>
+      <c r="M112" s="17" t="n">
+        <v>1269.83</v>
+      </c>
+      <c r="N112" s="16" t="n"/>
+      <c r="O112" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P112" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $15,244.08 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q112" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R112" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S112" s="18" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="T112" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U112" s="19" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="V112" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W112" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X112" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y112" s="19" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="Z112" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA112" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB112" s="15" t="n"/>
+      <c r="AC112" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD112" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE112" s="17" t="n">
+        <v>824.77</v>
+      </c>
+      <c r="AF112" s="17" t="n">
+        <v>793.6451</v>
+      </c>
+      <c r="AG112" s="17" t="n">
+        <v>855.8949</v>
+      </c>
+      <c r="AH112" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI112" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ112" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK112" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL112" s="15" t="inlineStr">
+        <is>
+          <t>Canaccord Genuity Maintains Buy on Regeneron Pharmaceuticals, Raises Price Target to $922</t>
+        </is>
+      </c>
+      <c r="AM112" s="17" t="n">
+        <v>812.3200000000001</v>
+      </c>
+      <c r="AN112" s="19" t="n">
+        <v>-0.0016</v>
+      </c>
+      <c r="AO112" s="17" t="n">
+        <v>99345.75</v>
+      </c>
+      <c r="AP112" s="17" t="n">
+        <v>15244.08</v>
+      </c>
+      <c r="AQ112" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR112" s="16" t="n"/>
+      <c r="AS112" s="17" t="n"/>
+      <c r="AT112" s="19" t="n"/>
+      <c r="AU112" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV112" s="6" t="inlineStr">
+        <is>
           <t>1f5a23ed-afbf-4216-8e41-ba5eccfed86a</t>
         </is>
       </c>
-      <c r="AW110" s="6" t="inlineStr">
+      <c r="AW112" s="6" t="inlineStr">
         <is>
           <t>tdagent-buy-REGN-1793295398213</t>
         </is>
       </c>
-      <c r="AX110" s="13" t="n">
+      <c r="AX112" s="13" t="n">
         <v>46324.73377314815</v>
       </c>
-      <c r="AY110" s="13" t="n">
+      <c r="AY112" s="13" t="n">
         <v>46324.73377314815</v>
       </c>
-      <c r="AZ110" s="13" t="n">
+      <c r="AZ112" s="13" t="n">
         <v>46324.73350694445</v>
       </c>
-      <c r="BA110" s="6" t="n"/>
+      <c r="BA112" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22198,9 +22414,15 @@
         <f>E51*F51</f>
         <v/>
       </c>
-      <c r="H51" s="22" t="n"/>
-      <c r="I51" s="22" t="n"/>
-      <c r="J51" s="17" t="n"/>
+      <c r="H51" s="22" t="n">
+        <v>46324.78953703704</v>
+      </c>
+      <c r="I51" s="22" t="n">
+        <v>46324.5812037037</v>
+      </c>
+      <c r="J51" s="17" t="n">
+        <v>704.25</v>
+      </c>
       <c r="K51" s="17">
         <f>IF(ISNUMBER(J51),J51*F51,"")</f>
         <v/>
@@ -22217,10 +22439,14 @@
         <f>IF(ISNUMBER(H51),H51-C51,"")</f>
         <v/>
       </c>
-      <c r="O51" s="6" t="n"/>
+      <c r="O51" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P51" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -22516,9 +22742,15 @@
         <f>E57*F57</f>
         <v/>
       </c>
-      <c r="H57" s="22" t="n"/>
-      <c r="I57" s="22" t="n"/>
-      <c r="J57" s="17" t="n"/>
+      <c r="H57" s="22" t="n">
+        <v>46324.78903935185</v>
+      </c>
+      <c r="I57" s="22" t="n">
+        <v>46324.58070601852</v>
+      </c>
+      <c r="J57" s="17" t="n">
+        <v>16.54</v>
+      </c>
       <c r="K57" s="17">
         <f>IF(ISNUMBER(J57),J57*F57,"")</f>
         <v/>
@@ -22535,10 +22767,14 @@
         <f>IF(ISNUMBER(H57),H57-C57,"")</f>
         <v/>
       </c>
-      <c r="O57" s="6" t="n"/>
+      <c r="O57" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P57" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-29 18:28 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA112" headerRowCount="1">
-  <autoFilter ref="A1:BA112"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA113" headerRowCount="1">
+  <autoFilter ref="A1:BA113"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P72" headerRowCount="1">
-  <autoFilter ref="A1:P72"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P73" headerRowCount="1">
+  <autoFilter ref="A1:P73"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.7925462963</v>
+        <v>46324.81164351852</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.58421296296</v>
+        <v>46324.60331018519</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$112,"BUY")+COUNTIF(Orders!$E$2:$E$112,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$113,"BUY")+COUNTIF(Orders!$E$2:$E$113,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$112,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$113,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$112,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$113,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$112,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$113,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$112,Orders!$E$2:$E$112,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$113,Orders!$E$2:$E$113,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$112,Orders!$E$2:$E$112,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$113,Orders!$E$2:$E$113,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$72,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$73,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$72,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$73,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$72)</f>
+        <f>SUM('Round trips'!$L$2:$L$73)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$72,"Closed",'Round trips'!$L$2:$L$72,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$73,"Closed",'Round trips'!$L$2:$L$73,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA112"/>
+  <dimension ref="A1:BA113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -19232,6 +19232,194 @@
       </c>
       <c r="BA112" s="6" t="n"/>
     </row>
+    <row r="113">
+      <c r="A113" s="12" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="13" t="n">
+        <v>46324.81153935185</v>
+      </c>
+      <c r="C113" s="13" t="n">
+        <v>46324.60320601852</v>
+      </c>
+      <c r="D113" s="13" t="n">
+        <v>46324.76987268519</v>
+      </c>
+      <c r="E113" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="G113" s="15" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="H113" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I113" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J113" s="16" t="n">
+        <v>0.662854464</v>
+      </c>
+      <c r="K113" s="17" t="n">
+        <v>502.818</v>
+      </c>
+      <c r="L113" s="17">
+        <f>IF(AND(ISNUMBER(J113),ISNUMBER(K113)),J113*K113,"")</f>
+        <v/>
+      </c>
+      <c r="M113" s="17" t="n"/>
+      <c r="N113" s="16" t="n">
+        <v>0.662854464</v>
+      </c>
+      <c r="O113" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
+      <c r="P113" s="15" t="inlineStr">
+        <is>
+          <t>3 of 5 green: start selling (half)</t>
+        </is>
+      </c>
+      <c r="Q113" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R113" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S113" s="18" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="T113" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="U113" s="19" t="n">
+        <v>0.0104</v>
+      </c>
+      <c r="V113" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W113" s="12" t="n"/>
+      <c r="X113" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y113" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z113" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA113" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB113" s="15" t="n"/>
+      <c r="AC113" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD113" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE113" s="17" t="n">
+        <v>502.76</v>
+      </c>
+      <c r="AF113" s="17" t="n">
+        <v>492.6839</v>
+      </c>
+      <c r="AG113" s="17" t="n">
+        <v>512.8361</v>
+      </c>
+      <c r="AH113" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI113" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ113" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK113" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL113" s="15" t="inlineStr">
+        <is>
+          <t>Linde Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM113" s="17" t="n">
+        <v>502.905</v>
+      </c>
+      <c r="AN113" s="19" t="n">
+        <v>-0.0104</v>
+      </c>
+      <c r="AO113" s="17" t="n">
+        <v>99432.78</v>
+      </c>
+      <c r="AP113" s="17" t="n">
+        <v>22987.6</v>
+      </c>
+      <c r="AQ113" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR113" s="16" t="n">
+        <v>1.325708929</v>
+      </c>
+      <c r="AS113" s="17" t="n">
+        <v>501.46</v>
+      </c>
+      <c r="AT113" s="19" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="AU113" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV113" s="6" t="inlineStr">
+        <is>
+          <t>b675bf9c-d103-4e06-b118-e159543a194b</t>
+        </is>
+      </c>
+      <c r="AW113" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-LIN-1793298517331</t>
+        </is>
+      </c>
+      <c r="AX113" s="13" t="n">
+        <v>46324.76987268519</v>
+      </c>
+      <c r="AY113" s="13" t="n">
+        <v>46324.76987268519</v>
+      </c>
+      <c r="AZ113" s="13" t="n">
+        <v>46324.7696412037</v>
+      </c>
+      <c r="BA113" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -19247,7 +19435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P72"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -23306,15 +23494,21 @@
         <v>501.46</v>
       </c>
       <c r="F67" s="16" t="n">
-        <v>1.325708929</v>
+        <v>0.662854464</v>
       </c>
       <c r="G67" s="17">
         <f>E67*F67</f>
         <v/>
       </c>
-      <c r="H67" s="22" t="n"/>
-      <c r="I67" s="22" t="n"/>
-      <c r="J67" s="17" t="n"/>
+      <c r="H67" s="22" t="n">
+        <v>46324.81153935185</v>
+      </c>
+      <c r="I67" s="22" t="n">
+        <v>46324.60320601852</v>
+      </c>
+      <c r="J67" s="17" t="n">
+        <v>502.818</v>
+      </c>
       <c r="K67" s="17">
         <f>IF(ISNUMBER(J67),J67*F67,"")</f>
         <v/>
@@ -23331,35 +23525,39 @@
         <f>IF(ISNUMBER(H67),H67-C67,"")</f>
         <v/>
       </c>
-      <c r="O67" s="6" t="n"/>
+      <c r="O67" s="6" t="inlineStr">
+        <is>
+          <t>3 green: sell half</t>
+        </is>
+      </c>
       <c r="P67" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EQNR</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+          <t>Linde plc Ordinary Shares</t>
         </is>
       </c>
       <c r="C68" s="22" t="n">
-        <v>46324.67839120371</v>
+        <v>46324.67836805555</v>
       </c>
       <c r="D68" s="22" t="n">
-        <v>46324.47005787037</v>
+        <v>46324.47003472222</v>
       </c>
       <c r="E68" s="17" t="n">
-        <v>47.09</v>
+        <v>501.46</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>14.117434699</v>
+        <v>0.6628544649999999</v>
       </c>
       <c r="G68" s="17">
         <f>E68*F68</f>
@@ -23394,25 +23592,25 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>EQNR</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>The Southern Company</t>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
         </is>
       </c>
       <c r="C69" s="22" t="n">
-        <v>46324.68998842593</v>
+        <v>46324.67839120371</v>
       </c>
       <c r="D69" s="22" t="n">
-        <v>46324.48165509259</v>
+        <v>46324.47005787037</v>
       </c>
       <c r="E69" s="17" t="n">
-        <v>92.97</v>
+        <v>47.09</v>
       </c>
       <c r="F69" s="16" t="n">
-        <v>14.744111003</v>
+        <v>14.117434699</v>
       </c>
       <c r="G69" s="17">
         <f>E69*F69</f>
@@ -23447,39 +23645,33 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EQT CORP</t>
+          <t>The Southern Company</t>
         </is>
       </c>
       <c r="C70" s="22" t="n">
-        <v>46324.69001157407</v>
+        <v>46324.68998842593</v>
       </c>
       <c r="D70" s="22" t="n">
-        <v>46324.48167824074</v>
+        <v>46324.48165509259</v>
       </c>
       <c r="E70" s="17" t="n">
-        <v>54.94</v>
+        <v>92.97</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>24.950127411</v>
+        <v>14.744111003</v>
       </c>
       <c r="G70" s="17">
         <f>E70*F70</f>
         <v/>
       </c>
-      <c r="H70" s="22" t="n">
-        <v>46324.75886574074</v>
-      </c>
-      <c r="I70" s="22" t="n">
-        <v>46324.5505324074</v>
-      </c>
-      <c r="J70" s="17" t="n">
-        <v>54.75</v>
-      </c>
+      <c r="H70" s="22" t="n"/>
+      <c r="I70" s="22" t="n"/>
+      <c r="J70" s="17" t="n"/>
       <c r="K70" s="17">
         <f>IF(ISNUMBER(J70),J70*F70,"")</f>
         <v/>
@@ -23496,47 +23688,49 @@
         <f>IF(ISNUMBER(H70),H70-C70,"")</f>
         <v/>
       </c>
-      <c r="O70" s="6" t="inlineStr">
-        <is>
-          <t>2 or fewer green</t>
-        </is>
-      </c>
+      <c r="O70" s="6" t="n"/>
       <c r="P70" s="6" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>eBay Inc. Common Stock</t>
+          <t>EQT CORP</t>
         </is>
       </c>
       <c r="C71" s="22" t="n">
-        <v>46324.7149074074</v>
+        <v>46324.69001157407</v>
       </c>
       <c r="D71" s="22" t="n">
-        <v>46324.50657407408</v>
+        <v>46324.48167824074</v>
       </c>
       <c r="E71" s="17" t="n">
-        <v>121.4</v>
+        <v>54.94</v>
       </c>
       <c r="F71" s="16" t="n">
-        <v>9.638632618999999</v>
+        <v>24.950127411</v>
       </c>
       <c r="G71" s="17">
         <f>E71*F71</f>
         <v/>
       </c>
-      <c r="H71" s="22" t="n"/>
-      <c r="I71" s="22" t="n"/>
-      <c r="J71" s="17" t="n"/>
+      <c r="H71" s="22" t="n">
+        <v>46324.75886574074</v>
+      </c>
+      <c r="I71" s="22" t="n">
+        <v>46324.5505324074</v>
+      </c>
+      <c r="J71" s="17" t="n">
+        <v>54.75</v>
+      </c>
       <c r="K71" s="17">
         <f>IF(ISNUMBER(J71),J71*F71,"")</f>
         <v/>
@@ -23553,35 +23747,39 @@
         <f>IF(ISNUMBER(H71),H71-C71,"")</f>
         <v/>
       </c>
-      <c r="O71" s="6" t="n"/>
+      <c r="O71" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
       <c r="P71" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+          <t>eBay Inc. Common Stock</t>
         </is>
       </c>
       <c r="C72" s="22" t="n">
-        <v>46324.77543981482</v>
+        <v>46324.7149074074</v>
       </c>
       <c r="D72" s="22" t="n">
-        <v>46324.56710648148</v>
+        <v>46324.50657407408</v>
       </c>
       <c r="E72" s="17" t="n">
-        <v>812.87</v>
+        <v>121.4</v>
       </c>
       <c r="F72" s="16" t="n">
-        <v>1.562144008</v>
+        <v>9.638632618999999</v>
       </c>
       <c r="G72" s="17">
         <f>E72*F72</f>
@@ -23613,8 +23811,61 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Regeneron Pharmaceuticals, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C73" s="22" t="n">
+        <v>46324.77543981482</v>
+      </c>
+      <c r="D73" s="22" t="n">
+        <v>46324.56710648148</v>
+      </c>
+      <c r="E73" s="17" t="n">
+        <v>812.87</v>
+      </c>
+      <c r="F73" s="16" t="n">
+        <v>1.562144008</v>
+      </c>
+      <c r="G73" s="17">
+        <f>E73*F73</f>
+        <v/>
+      </c>
+      <c r="H73" s="22" t="n"/>
+      <c r="I73" s="22" t="n"/>
+      <c r="J73" s="17" t="n"/>
+      <c r="K73" s="17">
+        <f>IF(ISNUMBER(J73),J73*F73,"")</f>
+        <v/>
+      </c>
+      <c r="L73" s="23">
+        <f>IF(ISNUMBER(J73),K73-G73,"")</f>
+        <v/>
+      </c>
+      <c r="M73" s="24">
+        <f>IF(ISNUMBER(J73),L73/G73,"")</f>
+        <v/>
+      </c>
+      <c r="N73" s="25">
+        <f>IF(ISNUMBER(H73),H73-C73,"")</f>
+        <v/>
+      </c>
+      <c r="O73" s="6" t="n"/>
+      <c r="P73" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M72">
+  <conditionalFormatting sqref="L2:M73">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 19:08 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA113" headerRowCount="1">
-  <autoFilter ref="A1:BA113"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA114" headerRowCount="1">
+  <autoFilter ref="A1:BA114"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P73" headerRowCount="1">
-  <autoFilter ref="A1:P73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P74" headerRowCount="1">
+  <autoFilter ref="A1:P74"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.81164351852</v>
+        <v>46324.83895833333</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.60331018519</v>
+        <v>46324.630625</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$113,"BUY")+COUNTIF(Orders!$E$2:$E$113,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$114,"BUY")+COUNTIF(Orders!$E$2:$E$114,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$113,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$114,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$113,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$114,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$113,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$114,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$113,Orders!$E$2:$E$113,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$114,Orders!$E$2:$E$114,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$113,Orders!$E$2:$E$113,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$114,Orders!$E$2:$E$114,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$73,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$74,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$73,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$74,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$73)</f>
+        <f>SUM('Round trips'!$L$2:$L$74)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$73,"Closed",'Round trips'!$L$2:$L$73,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$74,"Closed",'Round trips'!$L$2:$L$74,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA113"/>
+  <dimension ref="A1:BA114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -19420,6 +19420,190 @@
       </c>
       <c r="BA113" s="6" t="n"/>
     </row>
+    <row r="114">
+      <c r="A114" s="12" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="13" t="n">
+        <v>46324.83886574074</v>
+      </c>
+      <c r="C114" s="13" t="n">
+        <v>46324.63053240741</v>
+      </c>
+      <c r="D114" s="13" t="n">
+        <v>46324.79719907408</v>
+      </c>
+      <c r="E114" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="G114" s="15" t="inlineStr">
+        <is>
+          <t>Monster Beverage Corporation</t>
+        </is>
+      </c>
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I114" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J114" s="16" t="n">
+        <v>41.930066911</v>
+      </c>
+      <c r="K114" s="17" t="n">
+        <v>46.33</v>
+      </c>
+      <c r="L114" s="17">
+        <f>IF(AND(ISNUMBER(J114),ISNUMBER(K114)),J114*K114,"")</f>
+        <v/>
+      </c>
+      <c r="M114" s="17" t="n">
+        <v>1942.63</v>
+      </c>
+      <c r="N114" s="16" t="n"/>
+      <c r="O114" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P114" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $23,320.90 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q114" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R114" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S114" s="18" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="T114" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="U114" s="19" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="V114" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W114" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X114" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y114" s="19" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="Z114" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA114" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB114" s="15" t="n"/>
+      <c r="AC114" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD114" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE114" s="17" t="n">
+        <v>46.9591</v>
+      </c>
+      <c r="AF114" s="17" t="n">
+        <v>45.3364</v>
+      </c>
+      <c r="AG114" s="17" t="n">
+        <v>48.5818</v>
+      </c>
+      <c r="AH114" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI114" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ114" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK114" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL114" s="15" t="inlineStr">
+        <is>
+          <t>Monster Beverage Corporation Announces Third Quarter 2026 Earnings Release Date</t>
+        </is>
+      </c>
+      <c r="AM114" s="17" t="n">
+        <v>46.32</v>
+      </c>
+      <c r="AN114" s="19" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="AO114" s="17" t="n">
+        <v>99455.06</v>
+      </c>
+      <c r="AP114" s="17" t="n">
+        <v>23320.9</v>
+      </c>
+      <c r="AQ114" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR114" s="16" t="n"/>
+      <c r="AS114" s="17" t="n"/>
+      <c r="AT114" s="19" t="n"/>
+      <c r="AU114" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV114" s="6" t="inlineStr">
+        <is>
+          <t>3e9a5e35-8f69-42ac-88d5-32689c3ef2c2</t>
+        </is>
+      </c>
+      <c r="AW114" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MNST-1793300877596</t>
+        </is>
+      </c>
+      <c r="AX114" s="13" t="n">
+        <v>46324.7971875</v>
+      </c>
+      <c r="AY114" s="13" t="n">
+        <v>46324.79719907408</v>
+      </c>
+      <c r="AZ114" s="13" t="n">
+        <v>46324.79684027778</v>
+      </c>
+      <c r="BA114" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -19435,7 +19619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P73"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -23864,8 +24048,61 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Monster Beverage Corporation</t>
+        </is>
+      </c>
+      <c r="C74" s="22" t="n">
+        <v>46324.83886574074</v>
+      </c>
+      <c r="D74" s="22" t="n">
+        <v>46324.63053240741</v>
+      </c>
+      <c r="E74" s="17" t="n">
+        <v>46.33</v>
+      </c>
+      <c r="F74" s="16" t="n">
+        <v>41.930066911</v>
+      </c>
+      <c r="G74" s="17">
+        <f>E74*F74</f>
+        <v/>
+      </c>
+      <c r="H74" s="22" t="n"/>
+      <c r="I74" s="22" t="n"/>
+      <c r="J74" s="17" t="n"/>
+      <c r="K74" s="17">
+        <f>IF(ISNUMBER(J74),J74*F74,"")</f>
+        <v/>
+      </c>
+      <c r="L74" s="23">
+        <f>IF(ISNUMBER(J74),K74-G74,"")</f>
+        <v/>
+      </c>
+      <c r="M74" s="24">
+        <f>IF(ISNUMBER(J74),L74/G74,"")</f>
+        <v/>
+      </c>
+      <c r="N74" s="25">
+        <f>IF(ISNUMBER(H74),H74-C74,"")</f>
+        <v/>
+      </c>
+      <c r="O74" s="6" t="n"/>
+      <c r="P74" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M73">
+  <conditionalFormatting sqref="L2:M74">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-29 19:20 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA114" headerRowCount="1">
-  <autoFilter ref="A1:BA114"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA115" headerRowCount="1">
+  <autoFilter ref="A1:BA115"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.83895833333</v>
+        <v>46324.84730324074</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.630625</v>
+        <v>46324.63896990741</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$114,"BUY")+COUNTIF(Orders!$E$2:$E$114,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$115,"BUY")+COUNTIF(Orders!$E$2:$E$115,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$114,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$115,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$114,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$115,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$114,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$115,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$114,Orders!$E$2:$E$114,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$115,Orders!$E$2:$E$115,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$114,Orders!$E$2:$E$114,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$115,Orders!$E$2:$E$115,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA114"/>
+  <dimension ref="A1:BA115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -19604,6 +19604,194 @@
       </c>
       <c r="BA114" s="6" t="n"/>
     </row>
+    <row r="115">
+      <c r="A115" s="12" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="13" t="n">
+        <v>46324.84719907407</v>
+      </c>
+      <c r="C115" s="13" t="n">
+        <v>46324.63886574074</v>
+      </c>
+      <c r="D115" s="13" t="n">
+        <v>46324.80553240741</v>
+      </c>
+      <c r="E115" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="G115" s="15" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="H115" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I115" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J115" s="16" t="n">
+        <v>1.829160247</v>
+      </c>
+      <c r="K115" s="17" t="n">
+        <v>182.77</v>
+      </c>
+      <c r="L115" s="17">
+        <f>IF(AND(ISNUMBER(J115),ISNUMBER(K115)),J115*K115,"")</f>
+        <v/>
+      </c>
+      <c r="M115" s="17" t="n"/>
+      <c r="N115" s="16" t="n">
+        <v>1.829160247</v>
+      </c>
+      <c r="O115" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
+      <c r="P115" s="15" t="inlineStr">
+        <is>
+          <t>Only 2 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q115" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="R115" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S115" s="18" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="T115" s="12" t="n">
+        <v>93</v>
+      </c>
+      <c r="U115" s="19" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="V115" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W115" s="12" t="n"/>
+      <c r="X115" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y115" s="19" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="Z115" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA115" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB115" s="15" t="n"/>
+      <c r="AC115" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD115" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE115" s="17" t="n">
+        <v>182.76</v>
+      </c>
+      <c r="AF115" s="17" t="n">
+        <v>176.5879</v>
+      </c>
+      <c r="AG115" s="17" t="n">
+        <v>188.9321</v>
+      </c>
+      <c r="AH115" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI115" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ115" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK115" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL115" s="15" t="inlineStr">
+        <is>
+          <t>Exxon Mobil and Citgo Petroleum Acquire Venezuelan Crude Oil Shipment</t>
+        </is>
+      </c>
+      <c r="AM115" s="17" t="n">
+        <v>182.76</v>
+      </c>
+      <c r="AN115" s="19" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="AO115" s="17" t="n">
+        <v>99423.74000000001</v>
+      </c>
+      <c r="AP115" s="17" t="n">
+        <v>21378.28</v>
+      </c>
+      <c r="AQ115" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR115" s="16" t="n">
+        <v>1.829160247</v>
+      </c>
+      <c r="AS115" s="17" t="n">
+        <v>181.72</v>
+      </c>
+      <c r="AT115" s="19" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="AU115" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV115" s="6" t="inlineStr">
+        <is>
+          <t>c5433a9a-d16b-46fa-9feb-760487f14491</t>
+        </is>
+      </c>
+      <c r="AW115" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-XOM-1793301597035</t>
+        </is>
+      </c>
+      <c r="AX115" s="13" t="n">
+        <v>46324.80552083333</v>
+      </c>
+      <c r="AY115" s="13" t="n">
+        <v>46324.80553240741</v>
+      </c>
+      <c r="AZ115" s="13" t="n">
+        <v>46324.80516203704</v>
+      </c>
+      <c r="BA115" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -23240,9 +23428,15 @@
         <f>E59*F59</f>
         <v/>
       </c>
-      <c r="H59" s="22" t="n"/>
-      <c r="I59" s="22" t="n"/>
-      <c r="J59" s="17" t="n"/>
+      <c r="H59" s="22" t="n">
+        <v>46324.84719907407</v>
+      </c>
+      <c r="I59" s="22" t="n">
+        <v>46324.63886574074</v>
+      </c>
+      <c r="J59" s="17" t="n">
+        <v>182.77</v>
+      </c>
       <c r="K59" s="17">
         <f>IF(ISNUMBER(J59),J59*F59,"")</f>
         <v/>
@@ -23259,10 +23453,14 @@
         <f>IF(ISNUMBER(H59),H59-C59,"")</f>
         <v/>
       </c>
-      <c r="O59" s="6" t="n"/>
+      <c r="O59" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
       <c r="P59" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-29 19:31 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA115" headerRowCount="1">
-  <autoFilter ref="A1:BA115"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA136" headerRowCount="1">
+  <autoFilter ref="A1:BA136"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.84730324074</v>
+        <v>46324.85512731481</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.63896990741</v>
+        <v>46324.64679398148</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$115,"BUY")+COUNTIF(Orders!$E$2:$E$115,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$136,"BUY")+COUNTIF(Orders!$E$2:$E$136,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$115,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$136,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$115,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$136,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$115,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$136,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$115,Orders!$E$2:$E$115,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$136,Orders!$E$2:$E$136,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$115,Orders!$E$2:$E$115,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$136,Orders!$E$2:$E$136,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA115"/>
+  <dimension ref="A1:BA136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -19425,156 +19425,82 @@
         <v>113</v>
       </c>
       <c r="B114" s="13" t="n">
-        <v>46324.83886574074</v>
+        <v>46324.85206018519</v>
       </c>
       <c r="C114" s="13" t="n">
-        <v>46324.63053240741</v>
+        <v>46324.64372685185</v>
       </c>
       <c r="D114" s="13" t="n">
-        <v>46324.79719907408</v>
-      </c>
-      <c r="E114" s="14" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>46324.81039351852</v>
+      </c>
+      <c r="E114" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F114" s="6" t="inlineStr">
         <is>
-          <t>MNST</t>
-        </is>
-      </c>
-      <c r="G114" s="15" t="inlineStr">
-        <is>
-          <t>Monster Beverage Corporation</t>
-        </is>
-      </c>
-      <c r="H114" s="6" t="inlineStr">
-        <is>
-          <t>NASDAQ</t>
-        </is>
-      </c>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="G114" s="15" t="n"/>
+      <c r="H114" s="6" t="n"/>
       <c r="I114" s="6" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
       <c r="J114" s="16" t="n">
-        <v>41.930066911</v>
+        <v>9.638632618999999</v>
       </c>
       <c r="K114" s="17" t="n">
-        <v>46.33</v>
+        <v>122.25</v>
       </c>
       <c r="L114" s="17">
         <f>IF(AND(ISNUMBER(J114),ISNUMBER(K114)),J114*K114,"")</f>
         <v/>
       </c>
-      <c r="M114" s="17" t="n">
-        <v>1942.63</v>
-      </c>
-      <c r="N114" s="16" t="n"/>
+      <c r="M114" s="17" t="n"/>
+      <c r="N114" s="16" t="n">
+        <v>9.638632618999999</v>
+      </c>
       <c r="O114" s="6" t="inlineStr">
         <is>
-          <t>4+/5 green</t>
+          <t>stop-loss (Alpaca order)</t>
         </is>
       </c>
       <c r="P114" s="15" t="inlineStr">
         <is>
-          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $23,320.90 free cash split 12 ways</t>
-        </is>
-      </c>
-      <c r="Q114" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="R114" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="S114" s="18" t="n">
-        <v>0.652</v>
-      </c>
-      <c r="T114" s="12" t="n">
-        <v>89</v>
-      </c>
-      <c r="U114" s="19" t="n">
-        <v>0.0089</v>
-      </c>
-      <c r="V114" s="19" t="n">
-        <v>0.2893</v>
-      </c>
-      <c r="W114" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="X114" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y114" s="19" t="n">
-        <v>0.0002</v>
-      </c>
-      <c r="Z114" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AA114" s="12" t="n">
-        <v>100</v>
-      </c>
+          <t>Alpaca stop order triggered at 122.34 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q114" s="12" t="n"/>
+      <c r="R114" s="6" t="n"/>
+      <c r="S114" s="18" t="n"/>
+      <c r="T114" s="12" t="n"/>
+      <c r="U114" s="19" t="n"/>
+      <c r="V114" s="19" t="n"/>
+      <c r="W114" s="12" t="n"/>
+      <c r="X114" s="6" t="n"/>
+      <c r="Y114" s="19" t="n"/>
+      <c r="Z114" s="6" t="n"/>
+      <c r="AA114" s="12" t="n"/>
       <c r="AB114" s="15" t="n"/>
-      <c r="AC114" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AD114" s="6" t="inlineStr">
-        <is>
-          <t>up</t>
-        </is>
-      </c>
-      <c r="AE114" s="17" t="n">
-        <v>46.9591</v>
-      </c>
-      <c r="AF114" s="17" t="n">
-        <v>45.3364</v>
-      </c>
-      <c r="AG114" s="17" t="n">
-        <v>48.5818</v>
-      </c>
-      <c r="AH114" s="20" t="n">
-        <v>46331</v>
-      </c>
-      <c r="AI114" s="18" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="AJ114" s="6" t="inlineStr">
-        <is>
-          <t>watch</t>
-        </is>
-      </c>
-      <c r="AK114" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL114" s="15" t="inlineStr">
-        <is>
-          <t>Monster Beverage Corporation Announces Third Quarter 2026 Earnings Release Date</t>
-        </is>
-      </c>
-      <c r="AM114" s="17" t="n">
-        <v>46.32</v>
-      </c>
-      <c r="AN114" s="19" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="AO114" s="17" t="n">
-        <v>99455.06</v>
-      </c>
-      <c r="AP114" s="17" t="n">
-        <v>23320.9</v>
-      </c>
-      <c r="AQ114" s="19" t="n">
-        <v>0.0833</v>
-      </c>
+      <c r="AC114" s="6" t="n"/>
+      <c r="AD114" s="6" t="n"/>
+      <c r="AE114" s="17" t="n"/>
+      <c r="AF114" s="17" t="n"/>
+      <c r="AG114" s="17" t="n"/>
+      <c r="AH114" s="20" t="n"/>
+      <c r="AI114" s="18" t="n"/>
+      <c r="AJ114" s="6" t="n"/>
+      <c r="AK114" s="12" t="n"/>
+      <c r="AL114" s="15" t="n"/>
+      <c r="AM114" s="17" t="n"/>
+      <c r="AN114" s="19" t="n"/>
+      <c r="AO114" s="17" t="n"/>
+      <c r="AP114" s="17" t="n"/>
+      <c r="AQ114" s="19" t="n"/>
       <c r="AR114" s="16" t="n"/>
       <c r="AS114" s="17" t="n"/>
       <c r="AT114" s="19" t="n"/>
@@ -19585,23 +19511,21 @@
       </c>
       <c r="AV114" s="6" t="inlineStr">
         <is>
-          <t>3e9a5e35-8f69-42ac-88d5-32689c3ef2c2</t>
+          <t>2a1a9111-8f6b-42f5-b73a-345167f1962b</t>
         </is>
       </c>
       <c r="AW114" s="6" t="inlineStr">
         <is>
-          <t>tdagent-buy-MNST-1793300877596</t>
+          <t>tdagent-stop-EBAY-1793300832914</t>
         </is>
       </c>
       <c r="AX114" s="13" t="n">
-        <v>46324.7971875</v>
+        <v>46324.79666666667</v>
       </c>
       <c r="AY114" s="13" t="n">
-        <v>46324.79719907408</v>
-      </c>
-      <c r="AZ114" s="13" t="n">
-        <v>46324.79684027778</v>
-      </c>
+        <v>46324.81039351852</v>
+      </c>
+      <c r="AZ114" s="13" t="n"/>
       <c r="BA114" s="6" t="n"/>
     </row>
     <row r="115">
@@ -19609,32 +19533,32 @@
         <v>114</v>
       </c>
       <c r="B115" s="13" t="n">
-        <v>46324.84719907407</v>
+        <v>46324.83886574074</v>
       </c>
       <c r="C115" s="13" t="n">
-        <v>46324.63886574074</v>
+        <v>46324.63053240741</v>
       </c>
       <c r="D115" s="13" t="n">
-        <v>46324.80553240741</v>
-      </c>
-      <c r="E115" s="21" t="inlineStr">
-        <is>
-          <t>SELL</t>
+        <v>46324.79719907408</v>
+      </c>
+      <c r="E115" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F115" s="6" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="G115" s="15" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>Monster Beverage Corporation</t>
         </is>
       </c>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="I115" s="6" t="inlineStr">
@@ -19643,31 +19567,31 @@
         </is>
       </c>
       <c r="J115" s="16" t="n">
-        <v>1.829160247</v>
+        <v>41.930066911</v>
       </c>
       <c r="K115" s="17" t="n">
-        <v>182.77</v>
+        <v>46.33</v>
       </c>
       <c r="L115" s="17">
         <f>IF(AND(ISNUMBER(J115),ISNUMBER(K115)),J115*K115,"")</f>
         <v/>
       </c>
-      <c r="M115" s="17" t="n"/>
-      <c r="N115" s="16" t="n">
-        <v>1.829160247</v>
-      </c>
+      <c r="M115" s="17" t="n">
+        <v>1942.63</v>
+      </c>
+      <c r="N115" s="16" t="n"/>
       <c r="O115" s="6" t="inlineStr">
         <is>
-          <t>2 or fewer green</t>
+          <t>4+/5 green</t>
         </is>
       </c>
       <c r="P115" s="15" t="inlineStr">
         <is>
-          <t>Only 2 of 5 green</t>
+          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $23,320.90 free cash split 12 ways</t>
         </is>
       </c>
       <c r="Q115" s="12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R115" s="6" t="inlineStr">
         <is>
@@ -19675,25 +19599,27 @@
         </is>
       </c>
       <c r="S115" s="18" t="n">
-        <v>0.624</v>
+        <v>0.652</v>
       </c>
       <c r="T115" s="12" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="U115" s="19" t="n">
-        <v>0.0119</v>
+        <v>0.0089</v>
       </c>
       <c r="V115" s="19" t="n">
         <v>0.2893</v>
       </c>
-      <c r="W115" s="12" t="n"/>
+      <c r="W115" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="X115" s="6" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="Y115" s="19" t="n">
-        <v>0.008</v>
+        <v>0.0002</v>
       </c>
       <c r="Z115" s="6" t="inlineStr">
         <is>
@@ -19706,28 +19632,28 @@
       <c r="AB115" s="15" t="n"/>
       <c r="AC115" s="6" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AD115" s="6" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>up</t>
         </is>
       </c>
       <c r="AE115" s="17" t="n">
-        <v>182.76</v>
+        <v>46.9591</v>
       </c>
       <c r="AF115" s="17" t="n">
-        <v>176.5879</v>
+        <v>45.3364</v>
       </c>
       <c r="AG115" s="17" t="n">
-        <v>188.9321</v>
+        <v>48.5818</v>
       </c>
       <c r="AH115" s="20" t="n">
         <v>46331</v>
       </c>
       <c r="AI115" s="18" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="AJ115" s="6" t="inlineStr">
         <is>
@@ -19735,62 +19661,2404 @@
         </is>
       </c>
       <c r="AK115" s="12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AL115" s="15" t="inlineStr">
         <is>
-          <t>Exxon Mobil and Citgo Petroleum Acquire Venezuelan Crude Oil Shipment</t>
+          <t>Monster Beverage Corporation Announces Third Quarter 2026 Earnings Release Date</t>
         </is>
       </c>
       <c r="AM115" s="17" t="n">
-        <v>182.76</v>
+        <v>46.32</v>
       </c>
       <c r="AN115" s="19" t="n">
-        <v>0.0037</v>
+        <v>0.014</v>
       </c>
       <c r="AO115" s="17" t="n">
-        <v>99423.74000000001</v>
+        <v>99455.06</v>
       </c>
       <c r="AP115" s="17" t="n">
-        <v>21378.28</v>
+        <v>23320.9</v>
       </c>
       <c r="AQ115" s="19" t="n">
         <v>0.0833</v>
       </c>
-      <c r="AR115" s="16" t="n">
+      <c r="AR115" s="16" t="n"/>
+      <c r="AS115" s="17" t="n"/>
+      <c r="AT115" s="19" t="n"/>
+      <c r="AU115" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV115" s="6" t="inlineStr">
+        <is>
+          <t>3e9a5e35-8f69-42ac-88d5-32689c3ef2c2</t>
+        </is>
+      </c>
+      <c r="AW115" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MNST-1793300877596</t>
+        </is>
+      </c>
+      <c r="AX115" s="13" t="n">
+        <v>46324.7971875</v>
+      </c>
+      <c r="AY115" s="13" t="n">
+        <v>46324.79719907408</v>
+      </c>
+      <c r="AZ115" s="13" t="n">
+        <v>46324.79684027778</v>
+      </c>
+      <c r="BA115" s="6" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="12" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="13" t="n">
+        <v>46324.84719907407</v>
+      </c>
+      <c r="C116" s="13" t="n">
+        <v>46324.63886574074</v>
+      </c>
+      <c r="D116" s="13" t="n">
+        <v>46324.80553240741</v>
+      </c>
+      <c r="E116" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F116" s="6" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="G116" s="15" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I116" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J116" s="16" t="n">
         <v>1.829160247</v>
       </c>
-      <c r="AS115" s="17" t="n">
+      <c r="K116" s="17" t="n">
+        <v>182.77</v>
+      </c>
+      <c r="L116" s="17">
+        <f>IF(AND(ISNUMBER(J116),ISNUMBER(K116)),J116*K116,"")</f>
+        <v/>
+      </c>
+      <c r="M116" s="17" t="n"/>
+      <c r="N116" s="16" t="n">
+        <v>1.829160247</v>
+      </c>
+      <c r="O116" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
+      <c r="P116" s="15" t="inlineStr">
+        <is>
+          <t>Only 2 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q116" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="R116" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S116" s="18" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="T116" s="12" t="n">
+        <v>93</v>
+      </c>
+      <c r="U116" s="19" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="V116" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W116" s="12" t="n"/>
+      <c r="X116" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y116" s="19" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="Z116" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA116" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB116" s="15" t="n"/>
+      <c r="AC116" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD116" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE116" s="17" t="n">
+        <v>182.76</v>
+      </c>
+      <c r="AF116" s="17" t="n">
+        <v>176.5879</v>
+      </c>
+      <c r="AG116" s="17" t="n">
+        <v>188.9321</v>
+      </c>
+      <c r="AH116" s="20" t="n">
+        <v>46331</v>
+      </c>
+      <c r="AI116" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ116" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK116" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL116" s="15" t="inlineStr">
+        <is>
+          <t>Exxon Mobil and Citgo Petroleum Acquire Venezuelan Crude Oil Shipment</t>
+        </is>
+      </c>
+      <c r="AM116" s="17" t="n">
+        <v>182.76</v>
+      </c>
+      <c r="AN116" s="19" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="AO116" s="17" t="n">
+        <v>99423.74000000001</v>
+      </c>
+      <c r="AP116" s="17" t="n">
+        <v>21378.28</v>
+      </c>
+      <c r="AQ116" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR116" s="16" t="n">
+        <v>1.829160247</v>
+      </c>
+      <c r="AS116" s="17" t="n">
         <v>181.72</v>
       </c>
-      <c r="AT115" s="19" t="n">
+      <c r="AT116" s="19" t="n">
         <v>0.0059</v>
       </c>
-      <c r="AU115" s="6" t="inlineStr">
+      <c r="AU116" s="6" t="inlineStr">
         <is>
           <t>paper</t>
         </is>
       </c>
-      <c r="AV115" s="6" t="inlineStr">
+      <c r="AV116" s="6" t="inlineStr">
         <is>
           <t>c5433a9a-d16b-46fa-9feb-760487f14491</t>
         </is>
       </c>
-      <c r="AW115" s="6" t="inlineStr">
+      <c r="AW116" s="6" t="inlineStr">
         <is>
           <t>tdagent-sell-XOM-1793301597035</t>
         </is>
       </c>
-      <c r="AX115" s="13" t="n">
+      <c r="AX116" s="13" t="n">
         <v>46324.80552083333</v>
       </c>
-      <c r="AY115" s="13" t="n">
+      <c r="AY116" s="13" t="n">
         <v>46324.80553240741</v>
       </c>
-      <c r="AZ115" s="13" t="n">
+      <c r="AZ116" s="13" t="n">
         <v>46324.80516203704</v>
       </c>
-      <c r="BA115" s="6" t="n"/>
+      <c r="BA116" s="6" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="12" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="13" t="n">
+        <v>46324.8543287037</v>
+      </c>
+      <c r="C117" s="13" t="n">
+        <v>46324.64599537037</v>
+      </c>
+      <c r="D117" s="13" t="n">
+        <v>46324.81266203704</v>
+      </c>
+      <c r="E117" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="G117" s="15" t="n"/>
+      <c r="H117" s="6" t="n"/>
+      <c r="I117" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J117" s="16" t="n">
+        <v>2.290483737</v>
+      </c>
+      <c r="K117" s="17" t="n">
+        <v>289.706195</v>
+      </c>
+      <c r="L117" s="17">
+        <f>IF(AND(ISNUMBER(J117),ISNUMBER(K117)),J117*K117,"")</f>
+        <v/>
+      </c>
+      <c r="M117" s="17" t="n"/>
+      <c r="N117" s="16" t="n">
+        <v>2.290483737</v>
+      </c>
+      <c r="O117" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P117" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q117" s="12" t="n"/>
+      <c r="R117" s="6" t="n"/>
+      <c r="S117" s="18" t="n"/>
+      <c r="T117" s="12" t="n"/>
+      <c r="U117" s="19" t="n"/>
+      <c r="V117" s="19" t="n"/>
+      <c r="W117" s="12" t="n"/>
+      <c r="X117" s="6" t="n"/>
+      <c r="Y117" s="19" t="n"/>
+      <c r="Z117" s="6" t="n"/>
+      <c r="AA117" s="12" t="n"/>
+      <c r="AB117" s="15" t="n"/>
+      <c r="AC117" s="6" t="n"/>
+      <c r="AD117" s="6" t="n"/>
+      <c r="AE117" s="17" t="n"/>
+      <c r="AF117" s="17" t="n"/>
+      <c r="AG117" s="17" t="n"/>
+      <c r="AH117" s="20" t="n"/>
+      <c r="AI117" s="18" t="n"/>
+      <c r="AJ117" s="6" t="n"/>
+      <c r="AK117" s="12" t="n"/>
+      <c r="AL117" s="15" t="n"/>
+      <c r="AM117" s="17" t="n"/>
+      <c r="AN117" s="19" t="n"/>
+      <c r="AO117" s="17" t="n"/>
+      <c r="AP117" s="17" t="n"/>
+      <c r="AQ117" s="19" t="n"/>
+      <c r="AR117" s="16" t="n"/>
+      <c r="AS117" s="17" t="n"/>
+      <c r="AT117" s="19" t="n"/>
+      <c r="AU117" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV117" s="6" t="inlineStr">
+        <is>
+          <t>5c44e124-3b8e-49c8-8288-d302ffa068d2</t>
+        </is>
+      </c>
+      <c r="AW117" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ABBV-1793302212504</t>
+        </is>
+      </c>
+      <c r="AX117" s="13" t="n">
+        <v>46324.81263888889</v>
+      </c>
+      <c r="AY117" s="13" t="n">
+        <v>46324.81266203704</v>
+      </c>
+      <c r="AZ117" s="13" t="n"/>
+      <c r="BA117" s="6" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="12" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="13" t="n">
+        <v>46324.85434027778</v>
+      </c>
+      <c r="C118" s="13" t="n">
+        <v>46324.64600694444</v>
+      </c>
+      <c r="D118" s="13" t="n">
+        <v>46324.81267361111</v>
+      </c>
+      <c r="E118" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F118" s="6" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="G118" s="15" t="n"/>
+      <c r="H118" s="6" t="n"/>
+      <c r="I118" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J118" s="16" t="n">
+        <v>1.363168471</v>
+      </c>
+      <c r="K118" s="17" t="n">
+        <v>245.64</v>
+      </c>
+      <c r="L118" s="17">
+        <f>IF(AND(ISNUMBER(J118),ISNUMBER(K118)),J118*K118,"")</f>
+        <v/>
+      </c>
+      <c r="M118" s="17" t="n"/>
+      <c r="N118" s="16" t="n">
+        <v>1.363168471</v>
+      </c>
+      <c r="O118" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P118" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q118" s="12" t="n"/>
+      <c r="R118" s="6" t="n"/>
+      <c r="S118" s="18" t="n"/>
+      <c r="T118" s="12" t="n"/>
+      <c r="U118" s="19" t="n"/>
+      <c r="V118" s="19" t="n"/>
+      <c r="W118" s="12" t="n"/>
+      <c r="X118" s="6" t="n"/>
+      <c r="Y118" s="19" t="n"/>
+      <c r="Z118" s="6" t="n"/>
+      <c r="AA118" s="12" t="n"/>
+      <c r="AB118" s="15" t="n"/>
+      <c r="AC118" s="6" t="n"/>
+      <c r="AD118" s="6" t="n"/>
+      <c r="AE118" s="17" t="n"/>
+      <c r="AF118" s="17" t="n"/>
+      <c r="AG118" s="17" t="n"/>
+      <c r="AH118" s="20" t="n"/>
+      <c r="AI118" s="18" t="n"/>
+      <c r="AJ118" s="6" t="n"/>
+      <c r="AK118" s="12" t="n"/>
+      <c r="AL118" s="15" t="n"/>
+      <c r="AM118" s="17" t="n"/>
+      <c r="AN118" s="19" t="n"/>
+      <c r="AO118" s="17" t="n"/>
+      <c r="AP118" s="17" t="n"/>
+      <c r="AQ118" s="19" t="n"/>
+      <c r="AR118" s="16" t="n"/>
+      <c r="AS118" s="17" t="n"/>
+      <c r="AT118" s="19" t="n"/>
+      <c r="AU118" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV118" s="6" t="inlineStr">
+        <is>
+          <t>e708708c-b448-43a6-ae40-8b7efa5b803b</t>
+        </is>
+      </c>
+      <c r="AW118" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ACN-1793302213623</t>
+        </is>
+      </c>
+      <c r="AX118" s="13" t="n">
+        <v>46324.81265046296</v>
+      </c>
+      <c r="AY118" s="13" t="n">
+        <v>46324.81267361111</v>
+      </c>
+      <c r="AZ118" s="13" t="n"/>
+      <c r="BA118" s="6" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="12" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="13" t="n">
+        <v>46324.85439814815</v>
+      </c>
+      <c r="C119" s="13" t="n">
+        <v>46324.64606481481</v>
+      </c>
+      <c r="D119" s="13" t="n">
+        <v>46324.81273148148</v>
+      </c>
+      <c r="E119" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="G119" s="15" t="n"/>
+      <c r="H119" s="6" t="n"/>
+      <c r="I119" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J119" s="16" t="n">
+        <v>19.536817436</v>
+      </c>
+      <c r="K119" s="17" t="n">
+        <v>431.109505</v>
+      </c>
+      <c r="L119" s="17">
+        <f>IF(AND(ISNUMBER(J119),ISNUMBER(K119)),J119*K119,"")</f>
+        <v/>
+      </c>
+      <c r="M119" s="17" t="n"/>
+      <c r="N119" s="16" t="n">
+        <v>19.536817436</v>
+      </c>
+      <c r="O119" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P119" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q119" s="12" t="n"/>
+      <c r="R119" s="6" t="n"/>
+      <c r="S119" s="18" t="n"/>
+      <c r="T119" s="12" t="n"/>
+      <c r="U119" s="19" t="n"/>
+      <c r="V119" s="19" t="n"/>
+      <c r="W119" s="12" t="n"/>
+      <c r="X119" s="6" t="n"/>
+      <c r="Y119" s="19" t="n"/>
+      <c r="Z119" s="6" t="n"/>
+      <c r="AA119" s="12" t="n"/>
+      <c r="AB119" s="15" t="n"/>
+      <c r="AC119" s="6" t="n"/>
+      <c r="AD119" s="6" t="n"/>
+      <c r="AE119" s="17" t="n"/>
+      <c r="AF119" s="17" t="n"/>
+      <c r="AG119" s="17" t="n"/>
+      <c r="AH119" s="20" t="n"/>
+      <c r="AI119" s="18" t="n"/>
+      <c r="AJ119" s="6" t="n"/>
+      <c r="AK119" s="12" t="n"/>
+      <c r="AL119" s="15" t="n"/>
+      <c r="AM119" s="17" t="n"/>
+      <c r="AN119" s="19" t="n"/>
+      <c r="AO119" s="17" t="n"/>
+      <c r="AP119" s="17" t="n"/>
+      <c r="AQ119" s="19" t="n"/>
+      <c r="AR119" s="16" t="n"/>
+      <c r="AS119" s="17" t="n"/>
+      <c r="AT119" s="19" t="n"/>
+      <c r="AU119" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV119" s="6" t="inlineStr">
+        <is>
+          <t>91005add-93e1-43d8-a728-f2cf72ff6f9e</t>
+        </is>
+      </c>
+      <c r="AW119" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ADI-1793302214716</t>
+        </is>
+      </c>
+      <c r="AX119" s="13" t="n">
+        <v>46324.81266203704</v>
+      </c>
+      <c r="AY119" s="13" t="n">
+        <v>46324.81273148148</v>
+      </c>
+      <c r="AZ119" s="13" t="n"/>
+      <c r="BA119" s="6" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="12" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="13" t="n">
+        <v>46324.8544212963</v>
+      </c>
+      <c r="C120" s="13" t="n">
+        <v>46324.64608796296</v>
+      </c>
+      <c r="D120" s="13" t="n">
+        <v>46324.81275462963</v>
+      </c>
+      <c r="E120" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F120" s="6" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="G120" s="15" t="n"/>
+      <c r="H120" s="6" t="n"/>
+      <c r="I120" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J120" s="16" t="n">
+        <v>28.879753624</v>
+      </c>
+      <c r="K120" s="17" t="n">
+        <v>285.89</v>
+      </c>
+      <c r="L120" s="17">
+        <f>IF(AND(ISNUMBER(J120),ISNUMBER(K120)),J120*K120,"")</f>
+        <v/>
+      </c>
+      <c r="M120" s="17" t="n"/>
+      <c r="N120" s="16" t="n">
+        <v>28.879753624</v>
+      </c>
+      <c r="O120" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P120" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q120" s="12" t="n"/>
+      <c r="R120" s="6" t="n"/>
+      <c r="S120" s="18" t="n"/>
+      <c r="T120" s="12" t="n"/>
+      <c r="U120" s="19" t="n"/>
+      <c r="V120" s="19" t="n"/>
+      <c r="W120" s="12" t="n"/>
+      <c r="X120" s="6" t="n"/>
+      <c r="Y120" s="19" t="n"/>
+      <c r="Z120" s="6" t="n"/>
+      <c r="AA120" s="12" t="n"/>
+      <c r="AB120" s="15" t="n"/>
+      <c r="AC120" s="6" t="n"/>
+      <c r="AD120" s="6" t="n"/>
+      <c r="AE120" s="17" t="n"/>
+      <c r="AF120" s="17" t="n"/>
+      <c r="AG120" s="17" t="n"/>
+      <c r="AH120" s="20" t="n"/>
+      <c r="AI120" s="18" t="n"/>
+      <c r="AJ120" s="6" t="n"/>
+      <c r="AK120" s="12" t="n"/>
+      <c r="AL120" s="15" t="n"/>
+      <c r="AM120" s="17" t="n"/>
+      <c r="AN120" s="19" t="n"/>
+      <c r="AO120" s="17" t="n"/>
+      <c r="AP120" s="17" t="n"/>
+      <c r="AQ120" s="19" t="n"/>
+      <c r="AR120" s="16" t="n"/>
+      <c r="AS120" s="17" t="n"/>
+      <c r="AT120" s="19" t="n"/>
+      <c r="AU120" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV120" s="6" t="inlineStr">
+        <is>
+          <t>47489b81-e334-43f3-84f4-044d35788923</t>
+        </is>
+      </c>
+      <c r="AW120" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ADP-1793302215802</t>
+        </is>
+      </c>
+      <c r="AX120" s="13" t="n">
+        <v>46324.81267361111</v>
+      </c>
+      <c r="AY120" s="13" t="n">
+        <v>46324.81275462963</v>
+      </c>
+      <c r="AZ120" s="13" t="n"/>
+      <c r="BA120" s="6" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="12" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="13" t="n">
+        <v>46324.85438657407</v>
+      </c>
+      <c r="C121" s="13" t="n">
+        <v>46324.64605324074</v>
+      </c>
+      <c r="D121" s="13" t="n">
+        <v>46324.81271990741</v>
+      </c>
+      <c r="E121" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="G121" s="15" t="n"/>
+      <c r="H121" s="6" t="n"/>
+      <c r="I121" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J121" s="16" t="n">
+        <v>10.943045267</v>
+      </c>
+      <c r="K121" s="17" t="n">
+        <v>60.63</v>
+      </c>
+      <c r="L121" s="17">
+        <f>IF(AND(ISNUMBER(J121),ISNUMBER(K121)),J121*K121,"")</f>
+        <v/>
+      </c>
+      <c r="M121" s="17" t="n"/>
+      <c r="N121" s="16" t="n">
+        <v>10.943045267</v>
+      </c>
+      <c r="O121" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P121" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q121" s="12" t="n"/>
+      <c r="R121" s="6" t="n"/>
+      <c r="S121" s="18" t="n"/>
+      <c r="T121" s="12" t="n"/>
+      <c r="U121" s="19" t="n"/>
+      <c r="V121" s="19" t="n"/>
+      <c r="W121" s="12" t="n"/>
+      <c r="X121" s="6" t="n"/>
+      <c r="Y121" s="19" t="n"/>
+      <c r="Z121" s="6" t="n"/>
+      <c r="AA121" s="12" t="n"/>
+      <c r="AB121" s="15" t="n"/>
+      <c r="AC121" s="6" t="n"/>
+      <c r="AD121" s="6" t="n"/>
+      <c r="AE121" s="17" t="n"/>
+      <c r="AF121" s="17" t="n"/>
+      <c r="AG121" s="17" t="n"/>
+      <c r="AH121" s="20" t="n"/>
+      <c r="AI121" s="18" t="n"/>
+      <c r="AJ121" s="6" t="n"/>
+      <c r="AK121" s="12" t="n"/>
+      <c r="AL121" s="15" t="n"/>
+      <c r="AM121" s="17" t="n"/>
+      <c r="AN121" s="19" t="n"/>
+      <c r="AO121" s="17" t="n"/>
+      <c r="AP121" s="17" t="n"/>
+      <c r="AQ121" s="19" t="n"/>
+      <c r="AR121" s="16" t="n"/>
+      <c r="AS121" s="17" t="n"/>
+      <c r="AT121" s="19" t="n"/>
+      <c r="AU121" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV121" s="6" t="inlineStr">
+        <is>
+          <t>70826b79-984c-44eb-99b9-5aa87a6349f8</t>
+        </is>
+      </c>
+      <c r="AW121" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-DT-1793302216891</t>
+        </is>
+      </c>
+      <c r="AX121" s="13" t="n">
+        <v>46324.81268518518</v>
+      </c>
+      <c r="AY121" s="13" t="n">
+        <v>46324.81271990741</v>
+      </c>
+      <c r="AZ121" s="13" t="n"/>
+      <c r="BA121" s="6" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="13" t="n">
+        <v>46324.85438657407</v>
+      </c>
+      <c r="C122" s="13" t="n">
+        <v>46324.64605324074</v>
+      </c>
+      <c r="D122" s="13" t="n">
+        <v>46324.81271990741</v>
+      </c>
+      <c r="E122" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>DUK</t>
+        </is>
+      </c>
+      <c r="G122" s="15" t="n"/>
+      <c r="H122" s="6" t="n"/>
+      <c r="I122" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J122" s="16" t="n">
+        <v>5.287020836</v>
+      </c>
+      <c r="K122" s="17" t="n">
+        <v>125.812435</v>
+      </c>
+      <c r="L122" s="17">
+        <f>IF(AND(ISNUMBER(J122),ISNUMBER(K122)),J122*K122,"")</f>
+        <v/>
+      </c>
+      <c r="M122" s="17" t="n"/>
+      <c r="N122" s="16" t="n">
+        <v>5.287020836</v>
+      </c>
+      <c r="O122" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P122" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q122" s="12" t="n"/>
+      <c r="R122" s="6" t="n"/>
+      <c r="S122" s="18" t="n"/>
+      <c r="T122" s="12" t="n"/>
+      <c r="U122" s="19" t="n"/>
+      <c r="V122" s="19" t="n"/>
+      <c r="W122" s="12" t="n"/>
+      <c r="X122" s="6" t="n"/>
+      <c r="Y122" s="19" t="n"/>
+      <c r="Z122" s="6" t="n"/>
+      <c r="AA122" s="12" t="n"/>
+      <c r="AB122" s="15" t="n"/>
+      <c r="AC122" s="6" t="n"/>
+      <c r="AD122" s="6" t="n"/>
+      <c r="AE122" s="17" t="n"/>
+      <c r="AF122" s="17" t="n"/>
+      <c r="AG122" s="17" t="n"/>
+      <c r="AH122" s="20" t="n"/>
+      <c r="AI122" s="18" t="n"/>
+      <c r="AJ122" s="6" t="n"/>
+      <c r="AK122" s="12" t="n"/>
+      <c r="AL122" s="15" t="n"/>
+      <c r="AM122" s="17" t="n"/>
+      <c r="AN122" s="19" t="n"/>
+      <c r="AO122" s="17" t="n"/>
+      <c r="AP122" s="17" t="n"/>
+      <c r="AQ122" s="19" t="n"/>
+      <c r="AR122" s="16" t="n"/>
+      <c r="AS122" s="17" t="n"/>
+      <c r="AT122" s="19" t="n"/>
+      <c r="AU122" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV122" s="6" t="inlineStr">
+        <is>
+          <t>348f6363-619c-4aa1-b358-aaa2b12b49b2</t>
+        </is>
+      </c>
+      <c r="AW122" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-DUK-1793302218019</t>
+        </is>
+      </c>
+      <c r="AX122" s="13" t="n">
+        <v>46324.81270833333</v>
+      </c>
+      <c r="AY122" s="13" t="n">
+        <v>46324.81271990741</v>
+      </c>
+      <c r="AZ122" s="13" t="n"/>
+      <c r="BA122" s="6" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="12" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="13" t="n">
+        <v>46324.85438657407</v>
+      </c>
+      <c r="C123" s="13" t="n">
+        <v>46324.64605324074</v>
+      </c>
+      <c r="D123" s="13" t="n">
+        <v>46324.81271990741</v>
+      </c>
+      <c r="E123" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="G123" s="15" t="n"/>
+      <c r="H123" s="6" t="n"/>
+      <c r="I123" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J123" s="16" t="n">
+        <v>14.117434699</v>
+      </c>
+      <c r="K123" s="17" t="n">
+        <v>47.39</v>
+      </c>
+      <c r="L123" s="17">
+        <f>IF(AND(ISNUMBER(J123),ISNUMBER(K123)),J123*K123,"")</f>
+        <v/>
+      </c>
+      <c r="M123" s="17" t="n"/>
+      <c r="N123" s="16" t="n">
+        <v>14.117434699</v>
+      </c>
+      <c r="O123" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P123" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q123" s="12" t="n"/>
+      <c r="R123" s="6" t="n"/>
+      <c r="S123" s="18" t="n"/>
+      <c r="T123" s="12" t="n"/>
+      <c r="U123" s="19" t="n"/>
+      <c r="V123" s="19" t="n"/>
+      <c r="W123" s="12" t="n"/>
+      <c r="X123" s="6" t="n"/>
+      <c r="Y123" s="19" t="n"/>
+      <c r="Z123" s="6" t="n"/>
+      <c r="AA123" s="12" t="n"/>
+      <c r="AB123" s="15" t="n"/>
+      <c r="AC123" s="6" t="n"/>
+      <c r="AD123" s="6" t="n"/>
+      <c r="AE123" s="17" t="n"/>
+      <c r="AF123" s="17" t="n"/>
+      <c r="AG123" s="17" t="n"/>
+      <c r="AH123" s="20" t="n"/>
+      <c r="AI123" s="18" t="n"/>
+      <c r="AJ123" s="6" t="n"/>
+      <c r="AK123" s="12" t="n"/>
+      <c r="AL123" s="15" t="n"/>
+      <c r="AM123" s="17" t="n"/>
+      <c r="AN123" s="19" t="n"/>
+      <c r="AO123" s="17" t="n"/>
+      <c r="AP123" s="17" t="n"/>
+      <c r="AQ123" s="19" t="n"/>
+      <c r="AR123" s="16" t="n"/>
+      <c r="AS123" s="17" t="n"/>
+      <c r="AT123" s="19" t="n"/>
+      <c r="AU123" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV123" s="6" t="inlineStr">
+        <is>
+          <t>6ad8f539-215e-4c7d-a884-078aac8ed06e</t>
+        </is>
+      </c>
+      <c r="AW123" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-EQNR-1793302219116</t>
+        </is>
+      </c>
+      <c r="AX123" s="13" t="n">
+        <v>46324.81271990741</v>
+      </c>
+      <c r="AY123" s="13" t="n">
+        <v>46324.81271990741</v>
+      </c>
+      <c r="AZ123" s="13" t="n"/>
+      <c r="BA123" s="6" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="12" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="13" t="n">
+        <v>46324.85445601852</v>
+      </c>
+      <c r="C124" s="13" t="n">
+        <v>46324.64612268518</v>
+      </c>
+      <c r="D124" s="13" t="n">
+        <v>46324.81278935185</v>
+      </c>
+      <c r="E124" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="G124" s="15" t="n"/>
+      <c r="H124" s="6" t="n"/>
+      <c r="I124" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J124" s="16" t="n">
+        <v>30.075531531</v>
+      </c>
+      <c r="K124" s="17" t="n">
+        <v>273.44</v>
+      </c>
+      <c r="L124" s="17">
+        <f>IF(AND(ISNUMBER(J124),ISNUMBER(K124)),J124*K124,"")</f>
+        <v/>
+      </c>
+      <c r="M124" s="17" t="n"/>
+      <c r="N124" s="16" t="n">
+        <v>30.075531531</v>
+      </c>
+      <c r="O124" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P124" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q124" s="12" t="n"/>
+      <c r="R124" s="6" t="n"/>
+      <c r="S124" s="18" t="n"/>
+      <c r="T124" s="12" t="n"/>
+      <c r="U124" s="19" t="n"/>
+      <c r="V124" s="19" t="n"/>
+      <c r="W124" s="12" t="n"/>
+      <c r="X124" s="6" t="n"/>
+      <c r="Y124" s="19" t="n"/>
+      <c r="Z124" s="6" t="n"/>
+      <c r="AA124" s="12" t="n"/>
+      <c r="AB124" s="15" t="n"/>
+      <c r="AC124" s="6" t="n"/>
+      <c r="AD124" s="6" t="n"/>
+      <c r="AE124" s="17" t="n"/>
+      <c r="AF124" s="17" t="n"/>
+      <c r="AG124" s="17" t="n"/>
+      <c r="AH124" s="20" t="n"/>
+      <c r="AI124" s="18" t="n"/>
+      <c r="AJ124" s="6" t="n"/>
+      <c r="AK124" s="12" t="n"/>
+      <c r="AL124" s="15" t="n"/>
+      <c r="AM124" s="17" t="n"/>
+      <c r="AN124" s="19" t="n"/>
+      <c r="AO124" s="17" t="n"/>
+      <c r="AP124" s="17" t="n"/>
+      <c r="AQ124" s="19" t="n"/>
+      <c r="AR124" s="16" t="n"/>
+      <c r="AS124" s="17" t="n"/>
+      <c r="AT124" s="19" t="n"/>
+      <c r="AU124" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV124" s="6" t="inlineStr">
+        <is>
+          <t>f5de0c37-168f-4a39-a590-8f5f3a72ee8e</t>
+        </is>
+      </c>
+      <c r="AW124" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-IQV-1793302220210</t>
+        </is>
+      </c>
+      <c r="AX124" s="13" t="n">
+        <v>46324.81273148148</v>
+      </c>
+      <c r="AY124" s="13" t="n">
+        <v>46324.81278935185</v>
+      </c>
+      <c r="AZ124" s="13" t="n"/>
+      <c r="BA124" s="6" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="12" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="13" t="n">
+        <v>46324.8544212963</v>
+      </c>
+      <c r="C125" s="13" t="n">
+        <v>46324.64608796296</v>
+      </c>
+      <c r="D125" s="13" t="n">
+        <v>46324.81275462963</v>
+      </c>
+      <c r="E125" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="G125" s="15" t="n"/>
+      <c r="H125" s="6" t="n"/>
+      <c r="I125" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J125" s="16" t="n">
+        <v>18.645716072</v>
+      </c>
+      <c r="K125" s="17" t="n">
+        <v>447.605811</v>
+      </c>
+      <c r="L125" s="17">
+        <f>IF(AND(ISNUMBER(J125),ISNUMBER(K125)),J125*K125,"")</f>
+        <v/>
+      </c>
+      <c r="M125" s="17" t="n"/>
+      <c r="N125" s="16" t="n">
+        <v>18.645716072</v>
+      </c>
+      <c r="O125" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P125" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q125" s="12" t="n"/>
+      <c r="R125" s="6" t="n"/>
+      <c r="S125" s="18" t="n"/>
+      <c r="T125" s="12" t="n"/>
+      <c r="U125" s="19" t="n"/>
+      <c r="V125" s="19" t="n"/>
+      <c r="W125" s="12" t="n"/>
+      <c r="X125" s="6" t="n"/>
+      <c r="Y125" s="19" t="n"/>
+      <c r="Z125" s="6" t="n"/>
+      <c r="AA125" s="12" t="n"/>
+      <c r="AB125" s="15" t="n"/>
+      <c r="AC125" s="6" t="n"/>
+      <c r="AD125" s="6" t="n"/>
+      <c r="AE125" s="17" t="n"/>
+      <c r="AF125" s="17" t="n"/>
+      <c r="AG125" s="17" t="n"/>
+      <c r="AH125" s="20" t="n"/>
+      <c r="AI125" s="18" t="n"/>
+      <c r="AJ125" s="6" t="n"/>
+      <c r="AK125" s="12" t="n"/>
+      <c r="AL125" s="15" t="n"/>
+      <c r="AM125" s="17" t="n"/>
+      <c r="AN125" s="19" t="n"/>
+      <c r="AO125" s="17" t="n"/>
+      <c r="AP125" s="17" t="n"/>
+      <c r="AQ125" s="19" t="n"/>
+      <c r="AR125" s="16" t="n"/>
+      <c r="AS125" s="17" t="n"/>
+      <c r="AT125" s="19" t="n"/>
+      <c r="AU125" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV125" s="6" t="inlineStr">
+        <is>
+          <t>791db3a1-fc31-49d0-a38c-66748711cab6</t>
+        </is>
+      </c>
+      <c r="AW125" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ISRG-1793302221336</t>
+        </is>
+      </c>
+      <c r="AX125" s="13" t="n">
+        <v>46324.81274305555</v>
+      </c>
+      <c r="AY125" s="13" t="n">
+        <v>46324.81275462963</v>
+      </c>
+      <c r="AZ125" s="13" t="n"/>
+      <c r="BA125" s="6" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="12" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="13" t="n">
+        <v>46324.85443287037</v>
+      </c>
+      <c r="C126" s="13" t="n">
+        <v>46324.64609953704</v>
+      </c>
+      <c r="D126" s="13" t="n">
+        <v>46324.8127662037</v>
+      </c>
+      <c r="E126" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="G126" s="15" t="n"/>
+      <c r="H126" s="6" t="n"/>
+      <c r="I126" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J126" s="16" t="n">
+        <v>10.152565668</v>
+      </c>
+      <c r="K126" s="17" t="n">
+        <v>65.98</v>
+      </c>
+      <c r="L126" s="17">
+        <f>IF(AND(ISNUMBER(J126),ISNUMBER(K126)),J126*K126,"")</f>
+        <v/>
+      </c>
+      <c r="M126" s="17" t="n"/>
+      <c r="N126" s="16" t="n">
+        <v>10.152565668</v>
+      </c>
+      <c r="O126" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P126" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q126" s="12" t="n"/>
+      <c r="R126" s="6" t="n"/>
+      <c r="S126" s="18" t="n"/>
+      <c r="T126" s="12" t="n"/>
+      <c r="U126" s="19" t="n"/>
+      <c r="V126" s="19" t="n"/>
+      <c r="W126" s="12" t="n"/>
+      <c r="X126" s="6" t="n"/>
+      <c r="Y126" s="19" t="n"/>
+      <c r="Z126" s="6" t="n"/>
+      <c r="AA126" s="12" t="n"/>
+      <c r="AB126" s="15" t="n"/>
+      <c r="AC126" s="6" t="n"/>
+      <c r="AD126" s="6" t="n"/>
+      <c r="AE126" s="17" t="n"/>
+      <c r="AF126" s="17" t="n"/>
+      <c r="AG126" s="17" t="n"/>
+      <c r="AH126" s="20" t="n"/>
+      <c r="AI126" s="18" t="n"/>
+      <c r="AJ126" s="6" t="n"/>
+      <c r="AK126" s="12" t="n"/>
+      <c r="AL126" s="15" t="n"/>
+      <c r="AM126" s="17" t="n"/>
+      <c r="AN126" s="19" t="n"/>
+      <c r="AO126" s="17" t="n"/>
+      <c r="AP126" s="17" t="n"/>
+      <c r="AQ126" s="19" t="n"/>
+      <c r="AR126" s="16" t="n"/>
+      <c r="AS126" s="17" t="n"/>
+      <c r="AT126" s="19" t="n"/>
+      <c r="AU126" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV126" s="6" t="inlineStr">
+        <is>
+          <t>12ae221a-1a89-4f87-8f12-4aa502131b8b</t>
+        </is>
+      </c>
+      <c r="AW126" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-KR-1793302222404</t>
+        </is>
+      </c>
+      <c r="AX126" s="13" t="n">
+        <v>46324.81275462963</v>
+      </c>
+      <c r="AY126" s="13" t="n">
+        <v>46324.8127662037</v>
+      </c>
+      <c r="AZ126" s="13" t="n"/>
+      <c r="BA126" s="6" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="12" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="13" t="n">
+        <v>46324.85443287037</v>
+      </c>
+      <c r="C127" s="13" t="n">
+        <v>46324.64609953704</v>
+      </c>
+      <c r="D127" s="13" t="n">
+        <v>46324.8127662037</v>
+      </c>
+      <c r="E127" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="G127" s="15" t="n"/>
+      <c r="H127" s="6" t="n"/>
+      <c r="I127" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J127" s="16" t="n">
+        <v>0.662854465</v>
+      </c>
+      <c r="K127" s="17" t="n">
+        <v>502.036</v>
+      </c>
+      <c r="L127" s="17">
+        <f>IF(AND(ISNUMBER(J127),ISNUMBER(K127)),J127*K127,"")</f>
+        <v/>
+      </c>
+      <c r="M127" s="17" t="n"/>
+      <c r="N127" s="16" t="n">
+        <v>0.662854465</v>
+      </c>
+      <c r="O127" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P127" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q127" s="12" t="n"/>
+      <c r="R127" s="6" t="n"/>
+      <c r="S127" s="18" t="n"/>
+      <c r="T127" s="12" t="n"/>
+      <c r="U127" s="19" t="n"/>
+      <c r="V127" s="19" t="n"/>
+      <c r="W127" s="12" t="n"/>
+      <c r="X127" s="6" t="n"/>
+      <c r="Y127" s="19" t="n"/>
+      <c r="Z127" s="6" t="n"/>
+      <c r="AA127" s="12" t="n"/>
+      <c r="AB127" s="15" t="n"/>
+      <c r="AC127" s="6" t="n"/>
+      <c r="AD127" s="6" t="n"/>
+      <c r="AE127" s="17" t="n"/>
+      <c r="AF127" s="17" t="n"/>
+      <c r="AG127" s="17" t="n"/>
+      <c r="AH127" s="20" t="n"/>
+      <c r="AI127" s="18" t="n"/>
+      <c r="AJ127" s="6" t="n"/>
+      <c r="AK127" s="12" t="n"/>
+      <c r="AL127" s="15" t="n"/>
+      <c r="AM127" s="17" t="n"/>
+      <c r="AN127" s="19" t="n"/>
+      <c r="AO127" s="17" t="n"/>
+      <c r="AP127" s="17" t="n"/>
+      <c r="AQ127" s="19" t="n"/>
+      <c r="AR127" s="16" t="n"/>
+      <c r="AS127" s="17" t="n"/>
+      <c r="AT127" s="19" t="n"/>
+      <c r="AU127" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV127" s="6" t="inlineStr">
+        <is>
+          <t>8b50e38b-e426-4498-90ee-f675c33ee23f</t>
+        </is>
+      </c>
+      <c r="AW127" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-LIN-1793302223485</t>
+        </is>
+      </c>
+      <c r="AX127" s="13" t="n">
+        <v>46324.8127662037</v>
+      </c>
+      <c r="AY127" s="13" t="n">
+        <v>46324.8127662037</v>
+      </c>
+      <c r="AZ127" s="13" t="n"/>
+      <c r="BA127" s="6" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="12" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="13" t="n">
+        <v>46324.85445601852</v>
+      </c>
+      <c r="C128" s="13" t="n">
+        <v>46324.64612268518</v>
+      </c>
+      <c r="D128" s="13" t="n">
+        <v>46324.81278935185</v>
+      </c>
+      <c r="E128" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G128" s="15" t="n"/>
+      <c r="H128" s="6" t="n"/>
+      <c r="I128" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J128" s="16" t="n">
+        <v>13.053417297</v>
+      </c>
+      <c r="K128" s="17" t="n">
+        <v>637</v>
+      </c>
+      <c r="L128" s="17">
+        <f>IF(AND(ISNUMBER(J128),ISNUMBER(K128)),J128*K128,"")</f>
+        <v/>
+      </c>
+      <c r="M128" s="17" t="n"/>
+      <c r="N128" s="16" t="n">
+        <v>13.053417297</v>
+      </c>
+      <c r="O128" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P128" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q128" s="12" t="n"/>
+      <c r="R128" s="6" t="n"/>
+      <c r="S128" s="18" t="n"/>
+      <c r="T128" s="12" t="n"/>
+      <c r="U128" s="19" t="n"/>
+      <c r="V128" s="19" t="n"/>
+      <c r="W128" s="12" t="n"/>
+      <c r="X128" s="6" t="n"/>
+      <c r="Y128" s="19" t="n"/>
+      <c r="Z128" s="6" t="n"/>
+      <c r="AA128" s="12" t="n"/>
+      <c r="AB128" s="15" t="n"/>
+      <c r="AC128" s="6" t="n"/>
+      <c r="AD128" s="6" t="n"/>
+      <c r="AE128" s="17" t="n"/>
+      <c r="AF128" s="17" t="n"/>
+      <c r="AG128" s="17" t="n"/>
+      <c r="AH128" s="20" t="n"/>
+      <c r="AI128" s="18" t="n"/>
+      <c r="AJ128" s="6" t="n"/>
+      <c r="AK128" s="12" t="n"/>
+      <c r="AL128" s="15" t="n"/>
+      <c r="AM128" s="17" t="n"/>
+      <c r="AN128" s="19" t="n"/>
+      <c r="AO128" s="17" t="n"/>
+      <c r="AP128" s="17" t="n"/>
+      <c r="AQ128" s="19" t="n"/>
+      <c r="AR128" s="16" t="n"/>
+      <c r="AS128" s="17" t="n"/>
+      <c r="AT128" s="19" t="n"/>
+      <c r="AU128" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV128" s="6" t="inlineStr">
+        <is>
+          <t>1b141de1-e91d-41ba-99de-554f42f3eb60</t>
+        </is>
+      </c>
+      <c r="AW128" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MA-1793302224558</t>
+        </is>
+      </c>
+      <c r="AX128" s="13" t="n">
+        <v>46324.81277777778</v>
+      </c>
+      <c r="AY128" s="13" t="n">
+        <v>46324.81278935185</v>
+      </c>
+      <c r="AZ128" s="13" t="n"/>
+      <c r="BA128" s="6" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="12" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="13" t="n">
+        <v>46324.85450231482</v>
+      </c>
+      <c r="C129" s="13" t="n">
+        <v>46324.64616898148</v>
+      </c>
+      <c r="D129" s="13" t="n">
+        <v>46324.81283564815</v>
+      </c>
+      <c r="E129" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="G129" s="15" t="n"/>
+      <c r="H129" s="6" t="n"/>
+      <c r="I129" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J129" s="16" t="n">
+        <v>8.556874402</v>
+      </c>
+      <c r="K129" s="17" t="n">
+        <v>972.61</v>
+      </c>
+      <c r="L129" s="17">
+        <f>IF(AND(ISNUMBER(J129),ISNUMBER(K129)),J129*K129,"")</f>
+        <v/>
+      </c>
+      <c r="M129" s="17" t="n"/>
+      <c r="N129" s="16" t="n">
+        <v>8.556874402</v>
+      </c>
+      <c r="O129" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P129" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q129" s="12" t="n"/>
+      <c r="R129" s="6" t="n"/>
+      <c r="S129" s="18" t="n"/>
+      <c r="T129" s="12" t="n"/>
+      <c r="U129" s="19" t="n"/>
+      <c r="V129" s="19" t="n"/>
+      <c r="W129" s="12" t="n"/>
+      <c r="X129" s="6" t="n"/>
+      <c r="Y129" s="19" t="n"/>
+      <c r="Z129" s="6" t="n"/>
+      <c r="AA129" s="12" t="n"/>
+      <c r="AB129" s="15" t="n"/>
+      <c r="AC129" s="6" t="n"/>
+      <c r="AD129" s="6" t="n"/>
+      <c r="AE129" s="17" t="n"/>
+      <c r="AF129" s="17" t="n"/>
+      <c r="AG129" s="17" t="n"/>
+      <c r="AH129" s="20" t="n"/>
+      <c r="AI129" s="18" t="n"/>
+      <c r="AJ129" s="6" t="n"/>
+      <c r="AK129" s="12" t="n"/>
+      <c r="AL129" s="15" t="n"/>
+      <c r="AM129" s="17" t="n"/>
+      <c r="AN129" s="19" t="n"/>
+      <c r="AO129" s="17" t="n"/>
+      <c r="AP129" s="17" t="n"/>
+      <c r="AQ129" s="19" t="n"/>
+      <c r="AR129" s="16" t="n"/>
+      <c r="AS129" s="17" t="n"/>
+      <c r="AT129" s="19" t="n"/>
+      <c r="AU129" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV129" s="6" t="inlineStr">
+        <is>
+          <t>58882f88-fc2f-4f06-a730-ccd4bc3689f0</t>
+        </is>
+      </c>
+      <c r="AW129" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MCK-1793302225650</t>
+        </is>
+      </c>
+      <c r="AX129" s="13" t="n">
+        <v>46324.81278935185</v>
+      </c>
+      <c r="AY129" s="13" t="n">
+        <v>46324.81283564815</v>
+      </c>
+      <c r="AZ129" s="13" t="n"/>
+      <c r="BA129" s="6" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="12" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="13" t="n">
+        <v>46324.85450231482</v>
+      </c>
+      <c r="C130" s="13" t="n">
+        <v>46324.64616898148</v>
+      </c>
+      <c r="D130" s="13" t="n">
+        <v>46324.81283564815</v>
+      </c>
+      <c r="E130" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="G130" s="15" t="n"/>
+      <c r="H130" s="6" t="n"/>
+      <c r="I130" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J130" s="16" t="n">
+        <v>41.930066911</v>
+      </c>
+      <c r="K130" s="17" t="n">
+        <v>46.32</v>
+      </c>
+      <c r="L130" s="17">
+        <f>IF(AND(ISNUMBER(J130),ISNUMBER(K130)),J130*K130,"")</f>
+        <v/>
+      </c>
+      <c r="M130" s="17" t="n"/>
+      <c r="N130" s="16" t="n">
+        <v>41.930066911</v>
+      </c>
+      <c r="O130" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P130" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q130" s="12" t="n"/>
+      <c r="R130" s="6" t="n"/>
+      <c r="S130" s="18" t="n"/>
+      <c r="T130" s="12" t="n"/>
+      <c r="U130" s="19" t="n"/>
+      <c r="V130" s="19" t="n"/>
+      <c r="W130" s="12" t="n"/>
+      <c r="X130" s="6" t="n"/>
+      <c r="Y130" s="19" t="n"/>
+      <c r="Z130" s="6" t="n"/>
+      <c r="AA130" s="12" t="n"/>
+      <c r="AB130" s="15" t="n"/>
+      <c r="AC130" s="6" t="n"/>
+      <c r="AD130" s="6" t="n"/>
+      <c r="AE130" s="17" t="n"/>
+      <c r="AF130" s="17" t="n"/>
+      <c r="AG130" s="17" t="n"/>
+      <c r="AH130" s="20" t="n"/>
+      <c r="AI130" s="18" t="n"/>
+      <c r="AJ130" s="6" t="n"/>
+      <c r="AK130" s="12" t="n"/>
+      <c r="AL130" s="15" t="n"/>
+      <c r="AM130" s="17" t="n"/>
+      <c r="AN130" s="19" t="n"/>
+      <c r="AO130" s="17" t="n"/>
+      <c r="AP130" s="17" t="n"/>
+      <c r="AQ130" s="19" t="n"/>
+      <c r="AR130" s="16" t="n"/>
+      <c r="AS130" s="17" t="n"/>
+      <c r="AT130" s="19" t="n"/>
+      <c r="AU130" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV130" s="6" t="inlineStr">
+        <is>
+          <t>5d595309-9547-4900-8434-57839c5a42d9</t>
+        </is>
+      </c>
+      <c r="AW130" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MNST-1793302226953</t>
+        </is>
+      </c>
+      <c r="AX130" s="13" t="n">
+        <v>46324.8128125</v>
+      </c>
+      <c r="AY130" s="13" t="n">
+        <v>46324.81283564815</v>
+      </c>
+      <c r="AZ130" s="13" t="n"/>
+      <c r="BA130" s="6" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="13" t="n">
+        <v>46324.85451388889</v>
+      </c>
+      <c r="C131" s="13" t="n">
+        <v>46324.64618055556</v>
+      </c>
+      <c r="D131" s="13" t="n">
+        <v>46324.81284722222</v>
+      </c>
+      <c r="E131" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="G131" s="15" t="n"/>
+      <c r="H131" s="6" t="n"/>
+      <c r="I131" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J131" s="16" t="n">
+        <v>19.644723215</v>
+      </c>
+      <c r="K131" s="17" t="n">
+        <v>430.31</v>
+      </c>
+      <c r="L131" s="17">
+        <f>IF(AND(ISNUMBER(J131),ISNUMBER(K131)),J131*K131,"")</f>
+        <v/>
+      </c>
+      <c r="M131" s="17" t="n"/>
+      <c r="N131" s="16" t="n">
+        <v>19.644723215</v>
+      </c>
+      <c r="O131" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P131" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q131" s="12" t="n"/>
+      <c r="R131" s="6" t="n"/>
+      <c r="S131" s="18" t="n"/>
+      <c r="T131" s="12" t="n"/>
+      <c r="U131" s="19" t="n"/>
+      <c r="V131" s="19" t="n"/>
+      <c r="W131" s="12" t="n"/>
+      <c r="X131" s="6" t="n"/>
+      <c r="Y131" s="19" t="n"/>
+      <c r="Z131" s="6" t="n"/>
+      <c r="AA131" s="12" t="n"/>
+      <c r="AB131" s="15" t="n"/>
+      <c r="AC131" s="6" t="n"/>
+      <c r="AD131" s="6" t="n"/>
+      <c r="AE131" s="17" t="n"/>
+      <c r="AF131" s="17" t="n"/>
+      <c r="AG131" s="17" t="n"/>
+      <c r="AH131" s="20" t="n"/>
+      <c r="AI131" s="18" t="n"/>
+      <c r="AJ131" s="6" t="n"/>
+      <c r="AK131" s="12" t="n"/>
+      <c r="AL131" s="15" t="n"/>
+      <c r="AM131" s="17" t="n"/>
+      <c r="AN131" s="19" t="n"/>
+      <c r="AO131" s="17" t="n"/>
+      <c r="AP131" s="17" t="n"/>
+      <c r="AQ131" s="19" t="n"/>
+      <c r="AR131" s="16" t="n"/>
+      <c r="AS131" s="17" t="n"/>
+      <c r="AT131" s="19" t="n"/>
+      <c r="AU131" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV131" s="6" t="inlineStr">
+        <is>
+          <t>2525d2a0-c046-4536-be04-c49f21c0f9ed</t>
+        </is>
+      </c>
+      <c r="AW131" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-NTRA-1793302228020</t>
+        </is>
+      </c>
+      <c r="AX131" s="13" t="n">
+        <v>46324.81282407408</v>
+      </c>
+      <c r="AY131" s="13" t="n">
+        <v>46324.81284722222</v>
+      </c>
+      <c r="AZ131" s="13" t="n"/>
+      <c r="BA131" s="6" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="12" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="13" t="n">
+        <v>46324.85458333333</v>
+      </c>
+      <c r="C132" s="13" t="n">
+        <v>46324.64625</v>
+      </c>
+      <c r="D132" s="13" t="n">
+        <v>46324.81291666667</v>
+      </c>
+      <c r="E132" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F132" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="G132" s="15" t="n"/>
+      <c r="H132" s="6" t="n"/>
+      <c r="I132" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J132" s="16" t="n">
+        <v>132.370499603</v>
+      </c>
+      <c r="K132" s="17" t="n">
+        <v>62.615865</v>
+      </c>
+      <c r="L132" s="17">
+        <f>IF(AND(ISNUMBER(J132),ISNUMBER(K132)),J132*K132,"")</f>
+        <v/>
+      </c>
+      <c r="M132" s="17" t="n"/>
+      <c r="N132" s="16" t="n">
+        <v>132.370499603</v>
+      </c>
+      <c r="O132" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P132" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q132" s="12" t="n"/>
+      <c r="R132" s="6" t="n"/>
+      <c r="S132" s="18" t="n"/>
+      <c r="T132" s="12" t="n"/>
+      <c r="U132" s="19" t="n"/>
+      <c r="V132" s="19" t="n"/>
+      <c r="W132" s="12" t="n"/>
+      <c r="X132" s="6" t="n"/>
+      <c r="Y132" s="19" t="n"/>
+      <c r="Z132" s="6" t="n"/>
+      <c r="AA132" s="12" t="n"/>
+      <c r="AB132" s="15" t="n"/>
+      <c r="AC132" s="6" t="n"/>
+      <c r="AD132" s="6" t="n"/>
+      <c r="AE132" s="17" t="n"/>
+      <c r="AF132" s="17" t="n"/>
+      <c r="AG132" s="17" t="n"/>
+      <c r="AH132" s="20" t="n"/>
+      <c r="AI132" s="18" t="n"/>
+      <c r="AJ132" s="6" t="n"/>
+      <c r="AK132" s="12" t="n"/>
+      <c r="AL132" s="15" t="n"/>
+      <c r="AM132" s="17" t="n"/>
+      <c r="AN132" s="19" t="n"/>
+      <c r="AO132" s="17" t="n"/>
+      <c r="AP132" s="17" t="n"/>
+      <c r="AQ132" s="19" t="n"/>
+      <c r="AR132" s="16" t="n"/>
+      <c r="AS132" s="17" t="n"/>
+      <c r="AT132" s="19" t="n"/>
+      <c r="AU132" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV132" s="6" t="inlineStr">
+        <is>
+          <t>779bd3ce-6645-42cc-a2d7-b0d5a4c8285c</t>
+        </is>
+      </c>
+      <c r="AW132" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-OXY-1793302229102</t>
+        </is>
+      </c>
+      <c r="AX132" s="13" t="n">
+        <v>46324.81283564815</v>
+      </c>
+      <c r="AY132" s="13" t="n">
+        <v>46324.81291666667</v>
+      </c>
+      <c r="AZ132" s="13" t="n"/>
+      <c r="BA132" s="6" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="12" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="13" t="n">
+        <v>46324.85451388889</v>
+      </c>
+      <c r="C133" s="13" t="n">
+        <v>46324.64618055556</v>
+      </c>
+      <c r="D133" s="13" t="n">
+        <v>46324.81284722222</v>
+      </c>
+      <c r="E133" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F133" s="6" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+      <c r="G133" s="15" t="n"/>
+      <c r="H133" s="6" t="n"/>
+      <c r="I133" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J133" s="16" t="n">
+        <v>1.562144008</v>
+      </c>
+      <c r="K133" s="17" t="n">
+        <v>814.27</v>
+      </c>
+      <c r="L133" s="17">
+        <f>IF(AND(ISNUMBER(J133),ISNUMBER(K133)),J133*K133,"")</f>
+        <v/>
+      </c>
+      <c r="M133" s="17" t="n"/>
+      <c r="N133" s="16" t="n">
+        <v>1.562144008</v>
+      </c>
+      <c r="O133" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P133" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q133" s="12" t="n"/>
+      <c r="R133" s="6" t="n"/>
+      <c r="S133" s="18" t="n"/>
+      <c r="T133" s="12" t="n"/>
+      <c r="U133" s="19" t="n"/>
+      <c r="V133" s="19" t="n"/>
+      <c r="W133" s="12" t="n"/>
+      <c r="X133" s="6" t="n"/>
+      <c r="Y133" s="19" t="n"/>
+      <c r="Z133" s="6" t="n"/>
+      <c r="AA133" s="12" t="n"/>
+      <c r="AB133" s="15" t="n"/>
+      <c r="AC133" s="6" t="n"/>
+      <c r="AD133" s="6" t="n"/>
+      <c r="AE133" s="17" t="n"/>
+      <c r="AF133" s="17" t="n"/>
+      <c r="AG133" s="17" t="n"/>
+      <c r="AH133" s="20" t="n"/>
+      <c r="AI133" s="18" t="n"/>
+      <c r="AJ133" s="6" t="n"/>
+      <c r="AK133" s="12" t="n"/>
+      <c r="AL133" s="15" t="n"/>
+      <c r="AM133" s="17" t="n"/>
+      <c r="AN133" s="19" t="n"/>
+      <c r="AO133" s="17" t="n"/>
+      <c r="AP133" s="17" t="n"/>
+      <c r="AQ133" s="19" t="n"/>
+      <c r="AR133" s="16" t="n"/>
+      <c r="AS133" s="17" t="n"/>
+      <c r="AT133" s="19" t="n"/>
+      <c r="AU133" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV133" s="6" t="inlineStr">
+        <is>
+          <t>ac545554-f080-4159-afde-cb853b451a45</t>
+        </is>
+      </c>
+      <c r="AW133" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-REGN-1793302230168</t>
+        </is>
+      </c>
+      <c r="AX133" s="13" t="n">
+        <v>46324.81284722222</v>
+      </c>
+      <c r="AY133" s="13" t="n">
+        <v>46324.81284722222</v>
+      </c>
+      <c r="AZ133" s="13" t="n"/>
+      <c r="BA133" s="6" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="12" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="13" t="n">
+        <v>46324.85454861111</v>
+      </c>
+      <c r="C134" s="13" t="n">
+        <v>46324.64621527777</v>
+      </c>
+      <c r="D134" s="13" t="n">
+        <v>46324.81288194445</v>
+      </c>
+      <c r="E134" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F134" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="G134" s="15" t="n"/>
+      <c r="H134" s="6" t="n"/>
+      <c r="I134" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J134" s="16" t="n">
+        <v>6.184668341</v>
+      </c>
+      <c r="K134" s="17" t="n">
+        <v>107.668085</v>
+      </c>
+      <c r="L134" s="17">
+        <f>IF(AND(ISNUMBER(J134),ISNUMBER(K134)),J134*K134,"")</f>
+        <v/>
+      </c>
+      <c r="M134" s="17" t="n"/>
+      <c r="N134" s="16" t="n">
+        <v>6.184668341</v>
+      </c>
+      <c r="O134" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P134" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q134" s="12" t="n"/>
+      <c r="R134" s="6" t="n"/>
+      <c r="S134" s="18" t="n"/>
+      <c r="T134" s="12" t="n"/>
+      <c r="U134" s="19" t="n"/>
+      <c r="V134" s="19" t="n"/>
+      <c r="W134" s="12" t="n"/>
+      <c r="X134" s="6" t="n"/>
+      <c r="Y134" s="19" t="n"/>
+      <c r="Z134" s="6" t="n"/>
+      <c r="AA134" s="12" t="n"/>
+      <c r="AB134" s="15" t="n"/>
+      <c r="AC134" s="6" t="n"/>
+      <c r="AD134" s="6" t="n"/>
+      <c r="AE134" s="17" t="n"/>
+      <c r="AF134" s="17" t="n"/>
+      <c r="AG134" s="17" t="n"/>
+      <c r="AH134" s="20" t="n"/>
+      <c r="AI134" s="18" t="n"/>
+      <c r="AJ134" s="6" t="n"/>
+      <c r="AK134" s="12" t="n"/>
+      <c r="AL134" s="15" t="n"/>
+      <c r="AM134" s="17" t="n"/>
+      <c r="AN134" s="19" t="n"/>
+      <c r="AO134" s="17" t="n"/>
+      <c r="AP134" s="17" t="n"/>
+      <c r="AQ134" s="19" t="n"/>
+      <c r="AR134" s="16" t="n"/>
+      <c r="AS134" s="17" t="n"/>
+      <c r="AT134" s="19" t="n"/>
+      <c r="AU134" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV134" s="6" t="inlineStr">
+        <is>
+          <t>b4c64afe-002e-437a-b3a1-f77a11dfc1d9</t>
+        </is>
+      </c>
+      <c r="AW134" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-SHEL-1793302231236</t>
+        </is>
+      </c>
+      <c r="AX134" s="13" t="n">
+        <v>46324.81285879629</v>
+      </c>
+      <c r="AY134" s="13" t="n">
+        <v>46324.81288194445</v>
+      </c>
+      <c r="AZ134" s="13" t="n"/>
+      <c r="BA134" s="6" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="12" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="13" t="n">
+        <v>46324.85454861111</v>
+      </c>
+      <c r="C135" s="13" t="n">
+        <v>46324.64621527777</v>
+      </c>
+      <c r="D135" s="13" t="n">
+        <v>46324.81288194445</v>
+      </c>
+      <c r="E135" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="G135" s="15" t="n"/>
+      <c r="H135" s="6" t="n"/>
+      <c r="I135" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J135" s="16" t="n">
+        <v>14.744111003</v>
+      </c>
+      <c r="K135" s="17" t="n">
+        <v>93.03</v>
+      </c>
+      <c r="L135" s="17">
+        <f>IF(AND(ISNUMBER(J135),ISNUMBER(K135)),J135*K135,"")</f>
+        <v/>
+      </c>
+      <c r="M135" s="17" t="n"/>
+      <c r="N135" s="16" t="n">
+        <v>14.744111003</v>
+      </c>
+      <c r="O135" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P135" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q135" s="12" t="n"/>
+      <c r="R135" s="6" t="n"/>
+      <c r="S135" s="18" t="n"/>
+      <c r="T135" s="12" t="n"/>
+      <c r="U135" s="19" t="n"/>
+      <c r="V135" s="19" t="n"/>
+      <c r="W135" s="12" t="n"/>
+      <c r="X135" s="6" t="n"/>
+      <c r="Y135" s="19" t="n"/>
+      <c r="Z135" s="6" t="n"/>
+      <c r="AA135" s="12" t="n"/>
+      <c r="AB135" s="15" t="n"/>
+      <c r="AC135" s="6" t="n"/>
+      <c r="AD135" s="6" t="n"/>
+      <c r="AE135" s="17" t="n"/>
+      <c r="AF135" s="17" t="n"/>
+      <c r="AG135" s="17" t="n"/>
+      <c r="AH135" s="20" t="n"/>
+      <c r="AI135" s="18" t="n"/>
+      <c r="AJ135" s="6" t="n"/>
+      <c r="AK135" s="12" t="n"/>
+      <c r="AL135" s="15" t="n"/>
+      <c r="AM135" s="17" t="n"/>
+      <c r="AN135" s="19" t="n"/>
+      <c r="AO135" s="17" t="n"/>
+      <c r="AP135" s="17" t="n"/>
+      <c r="AQ135" s="19" t="n"/>
+      <c r="AR135" s="16" t="n"/>
+      <c r="AS135" s="17" t="n"/>
+      <c r="AT135" s="19" t="n"/>
+      <c r="AU135" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV135" s="6" t="inlineStr">
+        <is>
+          <t>5beca5e0-06a3-4be1-a5d9-c97a5e140c7d</t>
+        </is>
+      </c>
+      <c r="AW135" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-SO-1793302232319</t>
+        </is>
+      </c>
+      <c r="AX135" s="13" t="n">
+        <v>46324.81287037037</v>
+      </c>
+      <c r="AY135" s="13" t="n">
+        <v>46324.81288194445</v>
+      </c>
+      <c r="AZ135" s="13" t="n"/>
+      <c r="BA135" s="6" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="12" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="13" t="n">
+        <v>46324.85456018519</v>
+      </c>
+      <c r="C136" s="13" t="n">
+        <v>46324.64622685185</v>
+      </c>
+      <c r="D136" s="13" t="n">
+        <v>46324.81289351852</v>
+      </c>
+      <c r="E136" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F136" s="6" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="G136" s="15" t="n"/>
+      <c r="H136" s="6" t="n"/>
+      <c r="I136" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J136" s="16" t="n">
+        <v>2.132719514</v>
+      </c>
+      <c r="K136" s="17" t="n">
+        <v>310.44</v>
+      </c>
+      <c r="L136" s="17">
+        <f>IF(AND(ISNUMBER(J136),ISNUMBER(K136)),J136*K136,"")</f>
+        <v/>
+      </c>
+      <c r="M136" s="17" t="n"/>
+      <c r="N136" s="16" t="n">
+        <v>2.132719514</v>
+      </c>
+      <c r="O136" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P136" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q136" s="12" t="n"/>
+      <c r="R136" s="6" t="n"/>
+      <c r="S136" s="18" t="n"/>
+      <c r="T136" s="12" t="n"/>
+      <c r="U136" s="19" t="n"/>
+      <c r="V136" s="19" t="n"/>
+      <c r="W136" s="12" t="n"/>
+      <c r="X136" s="6" t="n"/>
+      <c r="Y136" s="19" t="n"/>
+      <c r="Z136" s="6" t="n"/>
+      <c r="AA136" s="12" t="n"/>
+      <c r="AB136" s="15" t="n"/>
+      <c r="AC136" s="6" t="n"/>
+      <c r="AD136" s="6" t="n"/>
+      <c r="AE136" s="17" t="n"/>
+      <c r="AF136" s="17" t="n"/>
+      <c r="AG136" s="17" t="n"/>
+      <c r="AH136" s="20" t="n"/>
+      <c r="AI136" s="18" t="n"/>
+      <c r="AJ136" s="6" t="n"/>
+      <c r="AK136" s="12" t="n"/>
+      <c r="AL136" s="15" t="n"/>
+      <c r="AM136" s="17" t="n"/>
+      <c r="AN136" s="19" t="n"/>
+      <c r="AO136" s="17" t="n"/>
+      <c r="AP136" s="17" t="n"/>
+      <c r="AQ136" s="19" t="n"/>
+      <c r="AR136" s="16" t="n"/>
+      <c r="AS136" s="17" t="n"/>
+      <c r="AT136" s="19" t="n"/>
+      <c r="AU136" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV136" s="6" t="inlineStr">
+        <is>
+          <t>d1f32e1f-3a83-4042-8079-a7edc3e38000</t>
+        </is>
+      </c>
+      <c r="AW136" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-VEEV-1793302233394</t>
+        </is>
+      </c>
+      <c r="AX136" s="13" t="n">
+        <v>46324.81288194445</v>
+      </c>
+      <c r="AY136" s="13" t="n">
+        <v>46324.81289351852</v>
+      </c>
+      <c r="AZ136" s="13" t="n"/>
+      <c r="BA136" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22520,9 +24788,15 @@
         <f>E43*F43</f>
         <v/>
       </c>
-      <c r="H43" s="22" t="n"/>
-      <c r="I43" s="22" t="n"/>
-      <c r="J43" s="17" t="n"/>
+      <c r="H43" s="22" t="n">
+        <v>46324.85458333333</v>
+      </c>
+      <c r="I43" s="22" t="n">
+        <v>46324.64625</v>
+      </c>
+      <c r="J43" s="17" t="n">
+        <v>62.615865</v>
+      </c>
       <c r="K43" s="17">
         <f>IF(ISNUMBER(J43),J43*F43,"")</f>
         <v/>
@@ -22539,10 +24813,14 @@
         <f>IF(ISNUMBER(H43),H43-C43,"")</f>
         <v/>
       </c>
-      <c r="O43" s="6" t="n"/>
+      <c r="O43" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P43" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -22573,9 +24851,15 @@
         <f>E44*F44</f>
         <v/>
       </c>
-      <c r="H44" s="22" t="n"/>
-      <c r="I44" s="22" t="n"/>
-      <c r="J44" s="17" t="n"/>
+      <c r="H44" s="22" t="n">
+        <v>46324.8544212963</v>
+      </c>
+      <c r="I44" s="22" t="n">
+        <v>46324.64608796296</v>
+      </c>
+      <c r="J44" s="17" t="n">
+        <v>285.89</v>
+      </c>
       <c r="K44" s="17">
         <f>IF(ISNUMBER(J44),J44*F44,"")</f>
         <v/>
@@ -22592,10 +24876,14 @@
         <f>IF(ISNUMBER(H44),H44-C44,"")</f>
         <v/>
       </c>
-      <c r="O44" s="6" t="n"/>
+      <c r="O44" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P44" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -22689,9 +24977,15 @@
         <f>E46*F46</f>
         <v/>
       </c>
-      <c r="H46" s="22" t="n"/>
-      <c r="I46" s="22" t="n"/>
-      <c r="J46" s="17" t="n"/>
+      <c r="H46" s="22" t="n">
+        <v>46324.85445601852</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>46324.64612268518</v>
+      </c>
+      <c r="J46" s="17" t="n">
+        <v>273.44</v>
+      </c>
       <c r="K46" s="17">
         <f>IF(ISNUMBER(J46),J46*F46,"")</f>
         <v/>
@@ -22708,10 +25002,14 @@
         <f>IF(ISNUMBER(H46),H46-C46,"")</f>
         <v/>
       </c>
-      <c r="O46" s="6" t="n"/>
+      <c r="O46" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P46" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -22742,9 +25040,15 @@
         <f>E47*F47</f>
         <v/>
       </c>
-      <c r="H47" s="22" t="n"/>
-      <c r="I47" s="22" t="n"/>
-      <c r="J47" s="17" t="n"/>
+      <c r="H47" s="22" t="n">
+        <v>46324.85439814815</v>
+      </c>
+      <c r="I47" s="22" t="n">
+        <v>46324.64606481481</v>
+      </c>
+      <c r="J47" s="17" t="n">
+        <v>431.109505</v>
+      </c>
       <c r="K47" s="17">
         <f>IF(ISNUMBER(J47),J47*F47,"")</f>
         <v/>
@@ -22761,10 +25065,14 @@
         <f>IF(ISNUMBER(H47),H47-C47,"")</f>
         <v/>
       </c>
-      <c r="O47" s="6" t="n"/>
+      <c r="O47" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P47" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -22858,9 +25166,15 @@
         <f>E49*F49</f>
         <v/>
       </c>
-      <c r="H49" s="22" t="n"/>
-      <c r="I49" s="22" t="n"/>
-      <c r="J49" s="17" t="n"/>
+      <c r="H49" s="22" t="n">
+        <v>46324.8544212963</v>
+      </c>
+      <c r="I49" s="22" t="n">
+        <v>46324.64608796296</v>
+      </c>
+      <c r="J49" s="17" t="n">
+        <v>447.605811</v>
+      </c>
       <c r="K49" s="17">
         <f>IF(ISNUMBER(J49),J49*F49,"")</f>
         <v/>
@@ -22877,10 +25191,14 @@
         <f>IF(ISNUMBER(H49),H49-C49,"")</f>
         <v/>
       </c>
-      <c r="O49" s="6" t="n"/>
+      <c r="O49" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P49" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23037,9 +25355,15 @@
         <f>E52*F52</f>
         <v/>
       </c>
-      <c r="H52" s="22" t="n"/>
-      <c r="I52" s="22" t="n"/>
-      <c r="J52" s="17" t="n"/>
+      <c r="H52" s="22" t="n">
+        <v>46324.85450231482</v>
+      </c>
+      <c r="I52" s="22" t="n">
+        <v>46324.64616898148</v>
+      </c>
+      <c r="J52" s="17" t="n">
+        <v>972.61</v>
+      </c>
       <c r="K52" s="17">
         <f>IF(ISNUMBER(J52),J52*F52,"")</f>
         <v/>
@@ -23056,10 +25380,14 @@
         <f>IF(ISNUMBER(H52),H52-C52,"")</f>
         <v/>
       </c>
-      <c r="O52" s="6" t="n"/>
+      <c r="O52" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P52" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23090,9 +25418,15 @@
         <f>E53*F53</f>
         <v/>
       </c>
-      <c r="H53" s="22" t="n"/>
-      <c r="I53" s="22" t="n"/>
-      <c r="J53" s="17" t="n"/>
+      <c r="H53" s="22" t="n">
+        <v>46324.85451388889</v>
+      </c>
+      <c r="I53" s="22" t="n">
+        <v>46324.64618055556</v>
+      </c>
+      <c r="J53" s="17" t="n">
+        <v>430.31</v>
+      </c>
       <c r="K53" s="17">
         <f>IF(ISNUMBER(J53),J53*F53,"")</f>
         <v/>
@@ -23109,10 +25443,14 @@
         <f>IF(ISNUMBER(H53),H53-C53,"")</f>
         <v/>
       </c>
-      <c r="O53" s="6" t="n"/>
+      <c r="O53" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P53" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23143,9 +25481,15 @@
         <f>E54*F54</f>
         <v/>
       </c>
-      <c r="H54" s="22" t="n"/>
-      <c r="I54" s="22" t="n"/>
-      <c r="J54" s="17" t="n"/>
+      <c r="H54" s="22" t="n">
+        <v>46324.85445601852</v>
+      </c>
+      <c r="I54" s="22" t="n">
+        <v>46324.64612268518</v>
+      </c>
+      <c r="J54" s="17" t="n">
+        <v>637</v>
+      </c>
       <c r="K54" s="17">
         <f>IF(ISNUMBER(J54),J54*F54,"")</f>
         <v/>
@@ -23162,10 +25506,14 @@
         <f>IF(ISNUMBER(H54),H54-C54,"")</f>
         <v/>
       </c>
-      <c r="O54" s="6" t="n"/>
+      <c r="O54" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P54" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23196,9 +25544,15 @@
         <f>E55*F55</f>
         <v/>
       </c>
-      <c r="H55" s="22" t="n"/>
-      <c r="I55" s="22" t="n"/>
-      <c r="J55" s="17" t="n"/>
+      <c r="H55" s="22" t="n">
+        <v>46324.85456018519</v>
+      </c>
+      <c r="I55" s="22" t="n">
+        <v>46324.64622685185</v>
+      </c>
+      <c r="J55" s="17" t="n">
+        <v>310.44</v>
+      </c>
       <c r="K55" s="17">
         <f>IF(ISNUMBER(J55),J55*F55,"")</f>
         <v/>
@@ -23215,10 +25569,14 @@
         <f>IF(ISNUMBER(H55),H55-C55,"")</f>
         <v/>
       </c>
-      <c r="O55" s="6" t="n"/>
+      <c r="O55" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P55" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23249,9 +25607,15 @@
         <f>E56*F56</f>
         <v/>
       </c>
-      <c r="H56" s="22" t="n"/>
-      <c r="I56" s="22" t="n"/>
-      <c r="J56" s="17" t="n"/>
+      <c r="H56" s="22" t="n">
+        <v>46324.8543287037</v>
+      </c>
+      <c r="I56" s="22" t="n">
+        <v>46324.64599537037</v>
+      </c>
+      <c r="J56" s="17" t="n">
+        <v>289.706195</v>
+      </c>
       <c r="K56" s="17">
         <f>IF(ISNUMBER(J56),J56*F56,"")</f>
         <v/>
@@ -23268,10 +25632,14 @@
         <f>IF(ISNUMBER(H56),H56-C56,"")</f>
         <v/>
       </c>
-      <c r="O56" s="6" t="n"/>
+      <c r="O56" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P56" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23491,9 +25859,15 @@
         <f>E60*F60</f>
         <v/>
       </c>
-      <c r="H60" s="22" t="n"/>
-      <c r="I60" s="22" t="n"/>
-      <c r="J60" s="17" t="n"/>
+      <c r="H60" s="22" t="n">
+        <v>46324.85454861111</v>
+      </c>
+      <c r="I60" s="22" t="n">
+        <v>46324.64621527777</v>
+      </c>
+      <c r="J60" s="17" t="n">
+        <v>107.668085</v>
+      </c>
       <c r="K60" s="17">
         <f>IF(ISNUMBER(J60),J60*F60,"")</f>
         <v/>
@@ -23510,10 +25884,14 @@
         <f>IF(ISNUMBER(H60),H60-C60,"")</f>
         <v/>
       </c>
-      <c r="O60" s="6" t="n"/>
+      <c r="O60" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P60" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23544,9 +25922,15 @@
         <f>E61*F61</f>
         <v/>
       </c>
-      <c r="H61" s="22" t="n"/>
-      <c r="I61" s="22" t="n"/>
-      <c r="J61" s="17" t="n"/>
+      <c r="H61" s="22" t="n">
+        <v>46324.85438657407</v>
+      </c>
+      <c r="I61" s="22" t="n">
+        <v>46324.64605324074</v>
+      </c>
+      <c r="J61" s="17" t="n">
+        <v>125.812435</v>
+      </c>
       <c r="K61" s="17">
         <f>IF(ISNUMBER(J61),J61*F61,"")</f>
         <v/>
@@ -23563,10 +25947,14 @@
         <f>IF(ISNUMBER(H61),H61-C61,"")</f>
         <v/>
       </c>
-      <c r="O61" s="6" t="n"/>
+      <c r="O61" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P61" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23597,9 +25985,15 @@
         <f>E62*F62</f>
         <v/>
       </c>
-      <c r="H62" s="22" t="n"/>
-      <c r="I62" s="22" t="n"/>
-      <c r="J62" s="17" t="n"/>
+      <c r="H62" s="22" t="n">
+        <v>46324.85438657407</v>
+      </c>
+      <c r="I62" s="22" t="n">
+        <v>46324.64605324074</v>
+      </c>
+      <c r="J62" s="17" t="n">
+        <v>60.63</v>
+      </c>
       <c r="K62" s="17">
         <f>IF(ISNUMBER(J62),J62*F62,"")</f>
         <v/>
@@ -23616,10 +26010,14 @@
         <f>IF(ISNUMBER(H62),H62-C62,"")</f>
         <v/>
       </c>
-      <c r="O62" s="6" t="n"/>
+      <c r="O62" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P62" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23650,9 +26048,15 @@
         <f>E63*F63</f>
         <v/>
       </c>
-      <c r="H63" s="22" t="n"/>
-      <c r="I63" s="22" t="n"/>
-      <c r="J63" s="17" t="n"/>
+      <c r="H63" s="22" t="n">
+        <v>46324.85443287037</v>
+      </c>
+      <c r="I63" s="22" t="n">
+        <v>46324.64609953704</v>
+      </c>
+      <c r="J63" s="17" t="n">
+        <v>65.98</v>
+      </c>
       <c r="K63" s="17">
         <f>IF(ISNUMBER(J63),J63*F63,"")</f>
         <v/>
@@ -23669,10 +26073,14 @@
         <f>IF(ISNUMBER(H63),H63-C63,"")</f>
         <v/>
       </c>
-      <c r="O63" s="6" t="n"/>
+      <c r="O63" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P63" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23766,9 +26174,15 @@
         <f>E65*F65</f>
         <v/>
       </c>
-      <c r="H65" s="22" t="n"/>
-      <c r="I65" s="22" t="n"/>
-      <c r="J65" s="17" t="n"/>
+      <c r="H65" s="22" t="n">
+        <v>46324.85434027778</v>
+      </c>
+      <c r="I65" s="22" t="n">
+        <v>46324.64600694444</v>
+      </c>
+      <c r="J65" s="17" t="n">
+        <v>245.64</v>
+      </c>
       <c r="K65" s="17">
         <f>IF(ISNUMBER(J65),J65*F65,"")</f>
         <v/>
@@ -23785,10 +26199,14 @@
         <f>IF(ISNUMBER(H65),H65-C65,"")</f>
         <v/>
       </c>
-      <c r="O65" s="6" t="n"/>
+      <c r="O65" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P65" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23945,9 +26363,15 @@
         <f>E68*F68</f>
         <v/>
       </c>
-      <c r="H68" s="22" t="n"/>
-      <c r="I68" s="22" t="n"/>
-      <c r="J68" s="17" t="n"/>
+      <c r="H68" s="22" t="n">
+        <v>46324.85443287037</v>
+      </c>
+      <c r="I68" s="22" t="n">
+        <v>46324.64609953704</v>
+      </c>
+      <c r="J68" s="17" t="n">
+        <v>502.036</v>
+      </c>
       <c r="K68" s="17">
         <f>IF(ISNUMBER(J68),J68*F68,"")</f>
         <v/>
@@ -23964,10 +26388,14 @@
         <f>IF(ISNUMBER(H68),H68-C68,"")</f>
         <v/>
       </c>
-      <c r="O68" s="6" t="n"/>
+      <c r="O68" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P68" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -23998,9 +26426,15 @@
         <f>E69*F69</f>
         <v/>
       </c>
-      <c r="H69" s="22" t="n"/>
-      <c r="I69" s="22" t="n"/>
-      <c r="J69" s="17" t="n"/>
+      <c r="H69" s="22" t="n">
+        <v>46324.85438657407</v>
+      </c>
+      <c r="I69" s="22" t="n">
+        <v>46324.64605324074</v>
+      </c>
+      <c r="J69" s="17" t="n">
+        <v>47.39</v>
+      </c>
       <c r="K69" s="17">
         <f>IF(ISNUMBER(J69),J69*F69,"")</f>
         <v/>
@@ -24017,10 +26451,14 @@
         <f>IF(ISNUMBER(H69),H69-C69,"")</f>
         <v/>
       </c>
-      <c r="O69" s="6" t="n"/>
+      <c r="O69" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P69" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -24051,9 +26489,15 @@
         <f>E70*F70</f>
         <v/>
       </c>
-      <c r="H70" s="22" t="n"/>
-      <c r="I70" s="22" t="n"/>
-      <c r="J70" s="17" t="n"/>
+      <c r="H70" s="22" t="n">
+        <v>46324.85454861111</v>
+      </c>
+      <c r="I70" s="22" t="n">
+        <v>46324.64621527777</v>
+      </c>
+      <c r="J70" s="17" t="n">
+        <v>93.03</v>
+      </c>
       <c r="K70" s="17">
         <f>IF(ISNUMBER(J70),J70*F70,"")</f>
         <v/>
@@ -24070,10 +26514,14 @@
         <f>IF(ISNUMBER(H70),H70-C70,"")</f>
         <v/>
       </c>
-      <c r="O70" s="6" t="n"/>
+      <c r="O70" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P70" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -24167,9 +26615,15 @@
         <f>E72*F72</f>
         <v/>
       </c>
-      <c r="H72" s="22" t="n"/>
-      <c r="I72" s="22" t="n"/>
-      <c r="J72" s="17" t="n"/>
+      <c r="H72" s="22" t="n">
+        <v>46324.85206018519</v>
+      </c>
+      <c r="I72" s="22" t="n">
+        <v>46324.64372685185</v>
+      </c>
+      <c r="J72" s="17" t="n">
+        <v>122.25</v>
+      </c>
       <c r="K72" s="17">
         <f>IF(ISNUMBER(J72),J72*F72,"")</f>
         <v/>
@@ -24186,10 +26640,14 @@
         <f>IF(ISNUMBER(H72),H72-C72,"")</f>
         <v/>
       </c>
-      <c r="O72" s="6" t="n"/>
+      <c r="O72" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P72" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -24220,9 +26678,15 @@
         <f>E73*F73</f>
         <v/>
       </c>
-      <c r="H73" s="22" t="n"/>
-      <c r="I73" s="22" t="n"/>
-      <c r="J73" s="17" t="n"/>
+      <c r="H73" s="22" t="n">
+        <v>46324.85451388889</v>
+      </c>
+      <c r="I73" s="22" t="n">
+        <v>46324.64618055556</v>
+      </c>
+      <c r="J73" s="17" t="n">
+        <v>814.27</v>
+      </c>
       <c r="K73" s="17">
         <f>IF(ISNUMBER(J73),J73*F73,"")</f>
         <v/>
@@ -24239,10 +26703,14 @@
         <f>IF(ISNUMBER(H73),H73-C73,"")</f>
         <v/>
       </c>
-      <c r="O73" s="6" t="n"/>
+      <c r="O73" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P73" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -24273,9 +26741,15 @@
         <f>E74*F74</f>
         <v/>
       </c>
-      <c r="H74" s="22" t="n"/>
-      <c r="I74" s="22" t="n"/>
-      <c r="J74" s="17" t="n"/>
+      <c r="H74" s="22" t="n">
+        <v>46324.85450231482</v>
+      </c>
+      <c r="I74" s="22" t="n">
+        <v>46324.64616898148</v>
+      </c>
+      <c r="J74" s="17" t="n">
+        <v>46.32</v>
+      </c>
       <c r="K74" s="17">
         <f>IF(ISNUMBER(J74),J74*F74,"")</f>
         <v/>
@@ -24292,10 +26766,14 @@
         <f>IF(ISNUMBER(H74),H74-C74,"")</f>
         <v/>
       </c>
-      <c r="O74" s="6" t="n"/>
+      <c r="O74" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P74" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-30 13:31 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA136" headerRowCount="1">
-  <autoFilter ref="A1:BA136"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA147" headerRowCount="1">
+  <autoFilter ref="A1:BA147"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46324.85512731481</v>
+        <v>46325.60520833333</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46324.64679398148</v>
+        <v>46325.396875</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$136,"BUY")+COUNTIF(Orders!$E$2:$E$136,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$147,"BUY")+COUNTIF(Orders!$E$2:$E$147,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$136,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$147,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$136,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$147,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$136,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$147,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$136,Orders!$E$2:$E$136,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$147,Orders!$E$2:$E$147,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$136,Orders!$E$2:$E$136,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$147,Orders!$E$2:$E$147,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA136"/>
+  <dimension ref="A1:BA147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -22060,6 +22060,1968 @@
       <c r="AZ136" s="13" t="n"/>
       <c r="BA136" s="6" t="n"/>
     </row>
+    <row r="137">
+      <c r="A137" s="12" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C137" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D137" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E137" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F137" s="6" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="G137" s="15" t="inlineStr">
+        <is>
+          <t>Veeva Systems Inc.</t>
+        </is>
+      </c>
+      <c r="H137" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I137" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J137" s="16" t="n"/>
+      <c r="K137" s="17" t="n"/>
+      <c r="L137" s="17">
+        <f>IF(AND(ISNUMBER(J137),ISNUMBER(K137)),J137*K137,"")</f>
+        <v/>
+      </c>
+      <c r="M137" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N137" s="16" t="n"/>
+      <c r="O137" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P137" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q137" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R137" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S137" s="18" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="T137" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="U137" s="19" t="n">
+        <v>0.0567</v>
+      </c>
+      <c r="V137" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W137" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X137" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y137" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z137" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA137" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB137" s="15" t="n"/>
+      <c r="AC137" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD137" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE137" s="17" t="n">
+        <v>318.1494</v>
+      </c>
+      <c r="AF137" s="17" t="n">
+        <v>298.5759</v>
+      </c>
+      <c r="AG137" s="17" t="n">
+        <v>337.7229</v>
+      </c>
+      <c r="AH137" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI137" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ137" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK137" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL137" s="15" t="inlineStr">
+        <is>
+          <t>Mizuho Adjusts Price Target on Veeva Systems</t>
+        </is>
+      </c>
+      <c r="AM137" s="17" t="n">
+        <v>310.32</v>
+      </c>
+      <c r="AN137" s="19" t="n">
+        <v>-0.0239</v>
+      </c>
+      <c r="AO137" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP137" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ137" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR137" s="16" t="n"/>
+      <c r="AS137" s="17" t="n"/>
+      <c r="AT137" s="19" t="n"/>
+      <c r="AU137" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV137" s="6" t="inlineStr">
+        <is>
+          <t>f91d62b7-8568-4f9e-be71-796e63d65117</t>
+        </is>
+      </c>
+      <c r="AW137" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-VEEV-1793367081183</t>
+        </is>
+      </c>
+      <c r="AX137" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY137" s="13" t="n"/>
+      <c r="AZ137" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA137" s="6" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="12" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C138" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D138" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E138" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F138" s="6" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="G138" s="15" t="inlineStr">
+        <is>
+          <t>Avantor, Inc.</t>
+        </is>
+      </c>
+      <c r="H138" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I138" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J138" s="16" t="n"/>
+      <c r="K138" s="17" t="n"/>
+      <c r="L138" s="17">
+        <f>IF(AND(ISNUMBER(J138),ISNUMBER(K138)),J138*K138,"")</f>
+        <v/>
+      </c>
+      <c r="M138" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N138" s="16" t="n"/>
+      <c r="O138" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P138" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #2, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q138" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R138" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S138" s="18" t="n">
+        <v>0.823</v>
+      </c>
+      <c r="T138" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="U138" s="19" t="n">
+        <v>0.0453</v>
+      </c>
+      <c r="V138" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W138" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="X138" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y138" s="19" t="n">
+        <v>0.004500000000000001</v>
+      </c>
+      <c r="Z138" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA138" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB138" s="15" t="n"/>
+      <c r="AC138" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD138" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE138" s="17" t="n">
+        <v>16.9406</v>
+      </c>
+      <c r="AF138" s="17" t="n">
+        <v>16.2766</v>
+      </c>
+      <c r="AG138" s="17" t="n">
+        <v>17.6045</v>
+      </c>
+      <c r="AH138" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI138" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ138" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK138" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL138" s="15" t="inlineStr">
+        <is>
+          <t>Incyte To Rally More Than 23%? Here Are 10 Top Analyst Forecasts For Friday</t>
+        </is>
+      </c>
+      <c r="AM138" s="17" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="AN138" s="19" t="n">
+        <v>-0.0003</v>
+      </c>
+      <c r="AO138" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP138" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ138" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR138" s="16" t="n"/>
+      <c r="AS138" s="17" t="n"/>
+      <c r="AT138" s="19" t="n"/>
+      <c r="AU138" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV138" s="6" t="inlineStr">
+        <is>
+          <t>ccc52b9b-563a-44f9-b2bf-27ec4616476d</t>
+        </is>
+      </c>
+      <c r="AW138" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-AVTR-1793367081262</t>
+        </is>
+      </c>
+      <c r="AX138" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY138" s="13" t="n"/>
+      <c r="AZ138" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA138" s="6" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="12" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C139" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D139" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E139" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F139" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="G139" s="15" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific, Inc.</t>
+        </is>
+      </c>
+      <c r="H139" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I139" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J139" s="16" t="n"/>
+      <c r="K139" s="17" t="n"/>
+      <c r="L139" s="17">
+        <f>IF(AND(ISNUMBER(J139),ISNUMBER(K139)),J139*K139,"")</f>
+        <v/>
+      </c>
+      <c r="M139" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N139" s="16" t="n"/>
+      <c r="O139" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P139" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #3, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q139" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R139" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S139" s="18" t="n">
+        <v>0.671</v>
+      </c>
+      <c r="T139" s="12" t="n">
+        <v>82</v>
+      </c>
+      <c r="U139" s="19" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="V139" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W139" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X139" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y139" s="19" t="n">
+        <v>0.0031</v>
+      </c>
+      <c r="Z139" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA139" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB139" s="15" t="n"/>
+      <c r="AC139" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD139" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE139" s="17" t="n">
+        <v>719.5843</v>
+      </c>
+      <c r="AF139" s="17" t="n">
+        <v>694.4236</v>
+      </c>
+      <c r="AG139" s="17" t="n">
+        <v>744.7449</v>
+      </c>
+      <c r="AH139" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI139" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ139" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK139" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL139" s="15" t="n"/>
+      <c r="AM139" s="17" t="n">
+        <v>709.52</v>
+      </c>
+      <c r="AN139" s="19" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="AO139" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP139" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ139" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR139" s="16" t="n"/>
+      <c r="AS139" s="17" t="n"/>
+      <c r="AT139" s="19" t="n"/>
+      <c r="AU139" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV139" s="6" t="inlineStr">
+        <is>
+          <t>c7a24925-a6d8-46bd-8523-07cdb34887bb</t>
+        </is>
+      </c>
+      <c r="AW139" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-TMO-1793367081364</t>
+        </is>
+      </c>
+      <c r="AX139" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY139" s="13" t="n"/>
+      <c r="AZ139" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA139" s="6" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="12" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C140" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D140" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E140" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F140" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="G140" s="15" t="inlineStr">
+        <is>
+          <t>McKesson Corporation</t>
+        </is>
+      </c>
+      <c r="H140" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I140" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J140" s="16" t="n"/>
+      <c r="K140" s="17" t="n"/>
+      <c r="L140" s="17">
+        <f>IF(AND(ISNUMBER(J140),ISNUMBER(K140)),J140*K140,"")</f>
+        <v/>
+      </c>
+      <c r="M140" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N140" s="16" t="n"/>
+      <c r="O140" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P140" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #5, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q140" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R140" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S140" s="18" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="T140" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="U140" s="19" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="V140" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W140" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X140" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y140" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z140" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA140" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB140" s="15" t="n"/>
+      <c r="AC140" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD140" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE140" s="17" t="n">
+        <v>995.9461</v>
+      </c>
+      <c r="AF140" s="17" t="n">
+        <v>959.4058</v>
+      </c>
+      <c r="AG140" s="17" t="n">
+        <v>1032.4865</v>
+      </c>
+      <c r="AH140" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI140" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ140" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK140" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL140" s="15" t="n"/>
+      <c r="AM140" s="17" t="n">
+        <v>981.33</v>
+      </c>
+      <c r="AN140" s="19" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="AO140" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP140" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ140" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR140" s="16" t="n"/>
+      <c r="AS140" s="17" t="n"/>
+      <c r="AT140" s="19" t="n"/>
+      <c r="AU140" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV140" s="6" t="inlineStr">
+        <is>
+          <t>c9d18008-3091-4eaa-b62d-1e1b97e85236</t>
+        </is>
+      </c>
+      <c r="AW140" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MCK-1793367081495</t>
+        </is>
+      </c>
+      <c r="AX140" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY140" s="13" t="n"/>
+      <c r="AZ140" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA140" s="6" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="12" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C141" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D141" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E141" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F141" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="G141" s="15" t="inlineStr">
+        <is>
+          <t>IQVIA Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="H141" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I141" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J141" s="16" t="n"/>
+      <c r="K141" s="17" t="n"/>
+      <c r="L141" s="17">
+        <f>IF(AND(ISNUMBER(J141),ISNUMBER(K141)),J141*K141,"")</f>
+        <v/>
+      </c>
+      <c r="M141" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N141" s="16" t="n"/>
+      <c r="O141" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P141" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #6, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q141" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R141" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S141" s="18" t="n">
+        <v>0.608</v>
+      </c>
+      <c r="T141" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="U141" s="19" t="n">
+        <v>0.0149</v>
+      </c>
+      <c r="V141" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W141" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="X141" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y141" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z141" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA141" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB141" s="15" t="n"/>
+      <c r="AC141" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD141" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE141" s="17" t="n">
+        <v>278.6477</v>
+      </c>
+      <c r="AF141" s="17" t="n">
+        <v>268.7034</v>
+      </c>
+      <c r="AG141" s="17" t="n">
+        <v>288.592</v>
+      </c>
+      <c r="AH141" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI141" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ141" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK141" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL141" s="15" t="inlineStr">
+        <is>
+          <t>TD Cowen Maintains Buy on IQVIA Holdings, Raises Price Target to $307</t>
+        </is>
+      </c>
+      <c r="AM141" s="17" t="n">
+        <v>274.67</v>
+      </c>
+      <c r="AN141" s="19" t="n">
+        <v>-0.0152</v>
+      </c>
+      <c r="AO141" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP141" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ141" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR141" s="16" t="n"/>
+      <c r="AS141" s="17" t="n"/>
+      <c r="AT141" s="19" t="n"/>
+      <c r="AU141" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV141" s="6" t="inlineStr">
+        <is>
+          <t>8b58392b-214c-48a0-9d1f-677ea8856dba</t>
+        </is>
+      </c>
+      <c r="AW141" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-IQV-1793367081570</t>
+        </is>
+      </c>
+      <c r="AX141" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY141" s="13" t="n"/>
+      <c r="AZ141" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA141" s="6" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="12" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C142" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D142" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E142" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F142" s="6" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="G142" s="15" t="inlineStr">
+        <is>
+          <t>Intuitive Surgical, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H142" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I142" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J142" s="16" t="n"/>
+      <c r="K142" s="17" t="n"/>
+      <c r="L142" s="17">
+        <f>IF(AND(ISNUMBER(J142),ISNUMBER(K142)),J142*K142,"")</f>
+        <v/>
+      </c>
+      <c r="M142" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N142" s="16" t="n"/>
+      <c r="O142" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P142" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #7, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q142" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R142" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S142" s="18" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="T142" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U142" s="19" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="V142" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W142" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="X142" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y142" s="19" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="Z142" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA142" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB142" s="15" t="n"/>
+      <c r="AC142" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD142" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE142" s="17" t="n">
+        <v>456.004</v>
+      </c>
+      <c r="AF142" s="17" t="n">
+        <v>437.9065</v>
+      </c>
+      <c r="AG142" s="17" t="n">
+        <v>474.1015</v>
+      </c>
+      <c r="AH142" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI142" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ142" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK142" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL142" s="15" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals Adopts Intuitive's Da Vinci 5 Surgical System</t>
+        </is>
+      </c>
+      <c r="AM142" s="17" t="n">
+        <v>449.52</v>
+      </c>
+      <c r="AN142" s="19" t="n">
+        <v>0.0103</v>
+      </c>
+      <c r="AO142" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP142" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ142" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR142" s="16" t="n"/>
+      <c r="AS142" s="17" t="n"/>
+      <c r="AT142" s="19" t="n"/>
+      <c r="AU142" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV142" s="6" t="inlineStr">
+        <is>
+          <t>2cf2a5c5-e672-4191-af35-c681b6b1185e</t>
+        </is>
+      </c>
+      <c r="AW142" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ISRG-1793367081690</t>
+        </is>
+      </c>
+      <c r="AX142" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY142" s="13" t="n"/>
+      <c r="AZ142" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA142" s="6" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="12" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C143" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D143" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E143" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F143" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="G143" s="15" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Public Limited Company Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="H143" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I143" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J143" s="16" t="n"/>
+      <c r="K143" s="17" t="n"/>
+      <c r="L143" s="17">
+        <f>IF(AND(ISNUMBER(J143),ISNUMBER(K143)),J143*K143,"")</f>
+        <v/>
+      </c>
+      <c r="M143" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N143" s="16" t="n"/>
+      <c r="O143" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P143" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #8, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q143" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R143" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S143" s="18" t="n">
+        <v>0.621</v>
+      </c>
+      <c r="T143" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U143" s="19" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="V143" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W143" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="X143" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y143" s="19" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="Z143" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA143" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB143" s="15" t="n"/>
+      <c r="AC143" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD143" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE143" s="17" t="n">
+        <v>325.3718</v>
+      </c>
+      <c r="AF143" s="17" t="n">
+        <v>314.0173</v>
+      </c>
+      <c r="AG143" s="17" t="n">
+        <v>336.7264</v>
+      </c>
+      <c r="AH143" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI143" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ143" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK143" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL143" s="15" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM143" s="17" t="n">
+        <v>322.725</v>
+      </c>
+      <c r="AN143" s="19" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="AO143" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP143" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ143" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR143" s="16" t="n"/>
+      <c r="AS143" s="17" t="n"/>
+      <c r="AT143" s="19" t="n"/>
+      <c r="AU143" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV143" s="6" t="inlineStr">
+        <is>
+          <t>4080f48b-6805-43bd-a8b5-cdcfa33ccf8e</t>
+        </is>
+      </c>
+      <c r="AW143" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-WTW-1793367081759</t>
+        </is>
+      </c>
+      <c r="AX143" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY143" s="13" t="n"/>
+      <c r="AZ143" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA143" s="6" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="12" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C144" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D144" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E144" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F144" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="G144" s="15" t="inlineStr">
+        <is>
+          <t>MARATHON PETROLEUM CORPORATION</t>
+        </is>
+      </c>
+      <c r="H144" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I144" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J144" s="16" t="n"/>
+      <c r="K144" s="17" t="n"/>
+      <c r="L144" s="17">
+        <f>IF(AND(ISNUMBER(J144),ISNUMBER(K144)),J144*K144,"")</f>
+        <v/>
+      </c>
+      <c r="M144" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N144" s="16" t="n"/>
+      <c r="O144" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P144" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #9, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q144" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R144" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S144" s="18" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="T144" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="U144" s="19" t="n">
+        <v>0.0249</v>
+      </c>
+      <c r="V144" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W144" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="X144" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y144" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z144" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA144" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB144" s="15" t="inlineStr">
+        <is>
+          <t>One day (-7.4%) did 80% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC144" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD144" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE144" s="17" t="n">
+        <v>441.7857</v>
+      </c>
+      <c r="AF144" s="17" t="n">
+        <v>418.6214</v>
+      </c>
+      <c r="AG144" s="17" t="n">
+        <v>464.95</v>
+      </c>
+      <c r="AH144" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI144" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ144" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK144" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL144" s="15" t="inlineStr">
+        <is>
+          <t>Reported Earlier, Marathon Petroleum Raises Quarterly Dividend 10% To $1.10 Per Share From $1.00, Payable Dec. 10, 2026, To Shareholders Of Record As Of Nov. 18</t>
+        </is>
+      </c>
+      <c r="AM144" s="17" t="n">
+        <v>432.52</v>
+      </c>
+      <c r="AN144" s="19" t="n">
+        <v>-0.0184</v>
+      </c>
+      <c r="AO144" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP144" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ144" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR144" s="16" t="n"/>
+      <c r="AS144" s="17" t="n"/>
+      <c r="AT144" s="19" t="n"/>
+      <c r="AU144" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV144" s="6" t="inlineStr">
+        <is>
+          <t>90c35321-ddbd-467a-bdd7-1f209883669a</t>
+        </is>
+      </c>
+      <c r="AW144" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MPC-1793367081834</t>
+        </is>
+      </c>
+      <c r="AX144" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY144" s="13" t="n"/>
+      <c r="AZ144" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA144" s="6" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="12" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="13" t="n">
+        <v>46325.60510416667</v>
+      </c>
+      <c r="C145" s="13" t="n">
+        <v>46325.39677083334</v>
+      </c>
+      <c r="D145" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="E145" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F145" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="G145" s="15" t="inlineStr">
+        <is>
+          <t>eBay Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H145" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I145" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J145" s="16" t="n"/>
+      <c r="K145" s="17" t="n"/>
+      <c r="L145" s="17">
+        <f>IF(AND(ISNUMBER(J145),ISNUMBER(K145)),J145*K145,"")</f>
+        <v/>
+      </c>
+      <c r="M145" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N145" s="16" t="n"/>
+      <c r="O145" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P145" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #10, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q145" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R145" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S145" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T145" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="U145" s="19" t="n">
+        <v>0.005500000000000001</v>
+      </c>
+      <c r="V145" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W145" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="X145" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y145" s="19" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="Z145" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA145" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB145" s="15" t="n"/>
+      <c r="AC145" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD145" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE145" s="17" t="n">
+        <v>123.3662</v>
+      </c>
+      <c r="AF145" s="17" t="n">
+        <v>118.3007</v>
+      </c>
+      <c r="AG145" s="17" t="n">
+        <v>128.4317</v>
+      </c>
+      <c r="AH145" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI145" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ145" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK145" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL145" s="15" t="inlineStr">
+        <is>
+          <t>Susquehanna Maintains Neutral on eBay, Raises Price Target to $125</t>
+        </is>
+      </c>
+      <c r="AM145" s="17" t="n">
+        <v>121.45</v>
+      </c>
+      <c r="AN145" s="19" t="n">
+        <v>0.0288</v>
+      </c>
+      <c r="AO145" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP145" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ145" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR145" s="16" t="n"/>
+      <c r="AS145" s="17" t="n"/>
+      <c r="AT145" s="19" t="n"/>
+      <c r="AU145" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV145" s="6" t="inlineStr">
+        <is>
+          <t>bf9079fb-f332-4a9e-8e61-0ea1e7f0299f</t>
+        </is>
+      </c>
+      <c r="AW145" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EBAY-1793367081920</t>
+        </is>
+      </c>
+      <c r="AX145" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY145" s="13" t="n"/>
+      <c r="AZ145" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA145" s="6" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="13" t="n">
+        <v>46325.60511574074</v>
+      </c>
+      <c r="C146" s="13" t="n">
+        <v>46325.39678240741</v>
+      </c>
+      <c r="D146" s="13" t="n">
+        <v>46325.56344907408</v>
+      </c>
+      <c r="E146" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F146" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="G146" s="15" t="inlineStr">
+        <is>
+          <t>EQT CORP</t>
+        </is>
+      </c>
+      <c r="H146" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I146" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J146" s="16" t="n"/>
+      <c r="K146" s="17" t="n"/>
+      <c r="L146" s="17">
+        <f>IF(AND(ISNUMBER(J146),ISNUMBER(K146)),J146*K146,"")</f>
+        <v/>
+      </c>
+      <c r="M146" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N146" s="16" t="n"/>
+      <c r="O146" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P146" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #11, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q146" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R146" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S146" s="18" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="T146" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U146" s="19" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="V146" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W146" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="X146" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y146" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z146" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA146" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="AB146" s="15" t="inlineStr">
+        <is>
+          <t>Price gapped 5.1% at an open in the last week.</t>
+        </is>
+      </c>
+      <c r="AC146" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD146" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE146" s="17" t="n">
+        <v>55.3612</v>
+      </c>
+      <c r="AF146" s="17" t="n">
+        <v>53.3331</v>
+      </c>
+      <c r="AG146" s="17" t="n">
+        <v>57.3893</v>
+      </c>
+      <c r="AH146" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI146" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ146" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK146" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL146" s="15" t="inlineStr">
+        <is>
+          <t>UBS Maintains Buy on EQT, Lowers Price Target to $74</t>
+        </is>
+      </c>
+      <c r="AM146" s="17" t="n">
+        <v>54.555</v>
+      </c>
+      <c r="AN146" s="19" t="n">
+        <v>-0.0299</v>
+      </c>
+      <c r="AO146" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP146" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ146" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR146" s="16" t="n"/>
+      <c r="AS146" s="17" t="n"/>
+      <c r="AT146" s="19" t="n"/>
+      <c r="AU146" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV146" s="6" t="inlineStr">
+        <is>
+          <t>9194868d-072a-4e4b-9802-c5706295191a</t>
+        </is>
+      </c>
+      <c r="AW146" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EQT-1793367081985</t>
+        </is>
+      </c>
+      <c r="AX146" s="13" t="n">
+        <v>46325.5634375</v>
+      </c>
+      <c r="AY146" s="13" t="n"/>
+      <c r="AZ146" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA146" s="6" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="12" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="13" t="n">
+        <v>46325.60511574074</v>
+      </c>
+      <c r="C147" s="13" t="n">
+        <v>46325.39678240741</v>
+      </c>
+      <c r="D147" s="13" t="n">
+        <v>46325.56344907408</v>
+      </c>
+      <c r="E147" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F147" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="G147" s="15" t="inlineStr">
+        <is>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+        </is>
+      </c>
+      <c r="H147" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I147" s="6" t="inlineStr">
+        <is>
+          <t>pending_new</t>
+        </is>
+      </c>
+      <c r="J147" s="16" t="n"/>
+      <c r="K147" s="17" t="n"/>
+      <c r="L147" s="17">
+        <f>IF(AND(ISNUMBER(J147),ISNUMBER(K147)),J147*K147,"")</f>
+        <v/>
+      </c>
+      <c r="M147" s="17" t="n">
+        <v>8282.450000000001</v>
+      </c>
+      <c r="N147" s="16" t="n"/>
+      <c r="O147" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P147" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #12, 8.33% of the $99,429.18 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q147" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R147" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S147" s="18" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="T147" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="U147" s="19" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="V147" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W147" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="X147" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y147" s="19" t="n">
+        <v>0.0072</v>
+      </c>
+      <c r="Z147" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA147" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB147" s="15" t="inlineStr">
+        <is>
+          <t>One day (+3.0%) did 76% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC147" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD147" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE147" s="17" t="n">
+        <v>108.9052</v>
+      </c>
+      <c r="AF147" s="17" t="n">
+        <v>105.8173</v>
+      </c>
+      <c r="AG147" s="17" t="n">
+        <v>111.993</v>
+      </c>
+      <c r="AH147" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI147" s="18" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AJ147" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK147" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL147" s="15" t="inlineStr">
+        <is>
+          <t>Shell Q3 Earnings Reach Highest Level Since 2022 Amid Middle-East Turmoil</t>
+        </is>
+      </c>
+      <c r="AM147" s="17" t="n">
+        <v>108.45</v>
+      </c>
+      <c r="AN147" s="19" t="n">
+        <v>0.0244</v>
+      </c>
+      <c r="AO147" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AP147" s="17" t="n">
+        <v>99429.17999999999</v>
+      </c>
+      <c r="AQ147" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR147" s="16" t="n"/>
+      <c r="AS147" s="17" t="n"/>
+      <c r="AT147" s="19" t="n"/>
+      <c r="AU147" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV147" s="6" t="inlineStr">
+        <is>
+          <t>de9144d0-8cb1-416e-a57b-fbb5f6a89c52</t>
+        </is>
+      </c>
+      <c r="AW147" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-SHEL-1793367082064</t>
+        </is>
+      </c>
+      <c r="AX147" s="13" t="n">
+        <v>46325.56344907408</v>
+      </c>
+      <c r="AY147" s="13" t="n"/>
+      <c r="AZ147" s="13" t="n">
+        <v>46325.5627662037</v>
+      </c>
+      <c r="BA147" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
records: 2026-10-30 13:37 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA147" headerRowCount="1">
-  <autoFilter ref="A1:BA147"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA160" headerRowCount="1">
+  <autoFilter ref="A1:BA160"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P74" headerRowCount="1">
-  <autoFilter ref="A1:P74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P97" headerRowCount="1">
+  <autoFilter ref="A1:P97"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.60520833333</v>
+        <v>46325.60930555555</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.396875</v>
+        <v>46325.40097222223</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$147,"BUY")+COUNTIF(Orders!$E$2:$E$147,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$160,"BUY")+COUNTIF(Orders!$E$2:$E$160,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$147,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$160,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$147,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$160,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$147,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$160,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$147,Orders!$E$2:$E$147,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$160,Orders!$E$2:$E$160,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$147,Orders!$E$2:$E$147,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$160,Orders!$E$2:$E$160,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$74,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$97,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$74,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$97,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$74)</f>
+        <f>SUM('Round trips'!$L$2:$L$97)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$74,"Closed",'Round trips'!$L$2:$L$74,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$97,"Closed",'Round trips'!$L$2:$L$97,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA147"/>
+  <dimension ref="A1:BA160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -22065,13 +22065,13 @@
         <v>136</v>
       </c>
       <c r="B137" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.60730324074</v>
       </c>
       <c r="C137" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.39896990741</v>
       </c>
       <c r="D137" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56563657407</v>
       </c>
       <c r="E137" s="14" t="inlineStr">
         <is>
@@ -22095,11 +22095,15 @@
       </c>
       <c r="I137" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J137" s="16" t="n"/>
-      <c r="K137" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J137" s="16" t="n">
+        <v>26.419297124</v>
+      </c>
+      <c r="K137" s="17" t="n">
+        <v>313.499635</v>
+      </c>
       <c r="L137" s="17">
         <f>IF(AND(ISNUMBER(J137),ISNUMBER(K137)),J137*K137,"")</f>
         <v/>
@@ -22232,7 +22236,9 @@
       <c r="AX137" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY137" s="13" t="n"/>
+      <c r="AY137" s="13" t="n">
+        <v>46325.56563657407</v>
+      </c>
       <c r="AZ137" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -22243,13 +22249,13 @@
         <v>137</v>
       </c>
       <c r="B138" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.60703703704</v>
       </c>
       <c r="C138" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.3987037037</v>
       </c>
       <c r="D138" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56537037037</v>
       </c>
       <c r="E138" s="14" t="inlineStr">
         <is>
@@ -22273,11 +22279,15 @@
       </c>
       <c r="I138" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J138" s="16" t="n"/>
-      <c r="K138" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J138" s="16" t="n">
+        <v>506</v>
+      </c>
+      <c r="K138" s="17" t="n">
+        <v>16.368458</v>
+      </c>
       <c r="L138" s="17">
         <f>IF(AND(ISNUMBER(J138),ISNUMBER(K138)),J138*K138,"")</f>
         <v/>
@@ -22410,7 +22420,9 @@
       <c r="AX138" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY138" s="13" t="n"/>
+      <c r="AY138" s="13" t="n">
+        <v>46325.56537037037</v>
+      </c>
       <c r="AZ138" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -22421,13 +22433,13 @@
         <v>138</v>
       </c>
       <c r="B139" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.6065162037</v>
       </c>
       <c r="C139" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.39818287037</v>
       </c>
       <c r="D139" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56484953704</v>
       </c>
       <c r="E139" s="14" t="inlineStr">
         <is>
@@ -22451,11 +22463,15 @@
       </c>
       <c r="I139" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J139" s="16" t="n"/>
-      <c r="K139" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J139" s="16" t="n">
+        <v>11.642778824</v>
+      </c>
+      <c r="K139" s="17" t="n">
+        <v>711.38</v>
+      </c>
       <c r="L139" s="17">
         <f>IF(AND(ISNUMBER(J139),ISNUMBER(K139)),J139*K139,"")</f>
         <v/>
@@ -22584,7 +22600,9 @@
       <c r="AX139" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY139" s="13" t="n"/>
+      <c r="AY139" s="13" t="n">
+        <v>46325.56484953704</v>
+      </c>
       <c r="AZ139" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -22595,13 +22613,13 @@
         <v>139</v>
       </c>
       <c r="B140" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.60611111111</v>
       </c>
       <c r="C140" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.39777777778</v>
       </c>
       <c r="D140" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56444444445</v>
       </c>
       <c r="E140" s="14" t="inlineStr">
         <is>
@@ -22625,11 +22643,15 @@
       </c>
       <c r="I140" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J140" s="16" t="n"/>
-      <c r="K140" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J140" s="16" t="n">
+        <v>8.201734928</v>
+      </c>
+      <c r="K140" s="17" t="n">
+        <v>1009.84</v>
+      </c>
       <c r="L140" s="17">
         <f>IF(AND(ISNUMBER(J140),ISNUMBER(K140)),J140*K140,"")</f>
         <v/>
@@ -22758,7 +22780,9 @@
       <c r="AX140" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY140" s="13" t="n"/>
+      <c r="AY140" s="13" t="n">
+        <v>46325.56444444445</v>
+      </c>
       <c r="AZ140" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -22769,13 +22793,13 @@
         <v>140</v>
       </c>
       <c r="B141" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.60637731481</v>
       </c>
       <c r="C141" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.39804398148</v>
       </c>
       <c r="D141" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56471064815</v>
       </c>
       <c r="E141" s="14" t="inlineStr">
         <is>
@@ -22799,11 +22823,15 @@
       </c>
       <c r="I141" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J141" s="16" t="n"/>
-      <c r="K141" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J141" s="16" t="n">
+        <v>30.574919709</v>
+      </c>
+      <c r="K141" s="17" t="n">
+        <v>270.89</v>
+      </c>
       <c r="L141" s="17">
         <f>IF(AND(ISNUMBER(J141),ISNUMBER(K141)),J141*K141,"")</f>
         <v/>
@@ -22936,7 +22964,9 @@
       <c r="AX141" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY141" s="13" t="n"/>
+      <c r="AY141" s="13" t="n">
+        <v>46325.56471064815</v>
+      </c>
       <c r="AZ141" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -22947,13 +22977,13 @@
         <v>141</v>
       </c>
       <c r="B142" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.60603009259</v>
       </c>
       <c r="C142" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.39769675926</v>
       </c>
       <c r="D142" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56436342592</v>
       </c>
       <c r="E142" s="14" t="inlineStr">
         <is>
@@ -22977,11 +23007,15 @@
       </c>
       <c r="I142" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J142" s="16" t="n"/>
-      <c r="K142" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J142" s="16" t="n">
+        <v>18.497085557</v>
+      </c>
+      <c r="K142" s="17" t="n">
+        <v>447.77</v>
+      </c>
       <c r="L142" s="17">
         <f>IF(AND(ISNUMBER(J142),ISNUMBER(K142)),J142*K142,"")</f>
         <v/>
@@ -23114,7 +23148,9 @@
       <c r="AX142" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY142" s="13" t="n"/>
+      <c r="AY142" s="13" t="n">
+        <v>46325.56436342592</v>
+      </c>
       <c r="AZ142" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -23125,13 +23161,13 @@
         <v>142</v>
       </c>
       <c r="B143" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.60714120371</v>
       </c>
       <c r="C143" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.39880787037</v>
       </c>
       <c r="D143" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56547453703</v>
       </c>
       <c r="E143" s="14" t="inlineStr">
         <is>
@@ -23155,11 +23191,15 @@
       </c>
       <c r="I143" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J143" s="16" t="n"/>
-      <c r="K143" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J143" s="16" t="n">
+        <v>25.40677088</v>
+      </c>
+      <c r="K143" s="17" t="n">
+        <v>325.993415</v>
+      </c>
       <c r="L143" s="17">
         <f>IF(AND(ISNUMBER(J143),ISNUMBER(K143)),J143*K143,"")</f>
         <v/>
@@ -23292,7 +23332,9 @@
       <c r="AX143" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY143" s="13" t="n"/>
+      <c r="AY143" s="13" t="n">
+        <v>46325.56547453703</v>
+      </c>
       <c r="AZ143" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -23303,13 +23345,13 @@
         <v>143</v>
       </c>
       <c r="B144" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.60696759259</v>
       </c>
       <c r="C144" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.39863425926</v>
       </c>
       <c r="D144" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56530092593</v>
       </c>
       <c r="E144" s="14" t="inlineStr">
         <is>
@@ -23333,11 +23375,15 @@
       </c>
       <c r="I144" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J144" s="16" t="n"/>
-      <c r="K144" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J144" s="16" t="n">
+        <v>18.738552036</v>
+      </c>
+      <c r="K144" s="17" t="n">
+        <v>442</v>
+      </c>
       <c r="L144" s="17">
         <f>IF(AND(ISNUMBER(J144),ISNUMBER(K144)),J144*K144,"")</f>
         <v/>
@@ -23474,7 +23520,9 @@
       <c r="AX144" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY144" s="13" t="n"/>
+      <c r="AY144" s="13" t="n">
+        <v>46325.56530092593</v>
+      </c>
       <c r="AZ144" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -23485,13 +23533,13 @@
         <v>144</v>
       </c>
       <c r="B145" s="13" t="n">
-        <v>46325.60510416667</v>
+        <v>46325.60626157407</v>
       </c>
       <c r="C145" s="13" t="n">
-        <v>46325.39677083334</v>
+        <v>46325.39792824074</v>
       </c>
       <c r="D145" s="13" t="n">
-        <v>46325.5634375</v>
+        <v>46325.56459490741</v>
       </c>
       <c r="E145" s="14" t="inlineStr">
         <is>
@@ -23515,11 +23563,15 @@
       </c>
       <c r="I145" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J145" s="16" t="n"/>
-      <c r="K145" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J145" s="16" t="n">
+        <v>68.49520344</v>
+      </c>
+      <c r="K145" s="17" t="n">
+        <v>120.92</v>
+      </c>
       <c r="L145" s="17">
         <f>IF(AND(ISNUMBER(J145),ISNUMBER(K145)),J145*K145,"")</f>
         <v/>
@@ -23652,7 +23704,9 @@
       <c r="AX145" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY145" s="13" t="n"/>
+      <c r="AY145" s="13" t="n">
+        <v>46325.56459490741</v>
+      </c>
       <c r="AZ145" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -23663,13 +23717,13 @@
         <v>145</v>
       </c>
       <c r="B146" s="13" t="n">
-        <v>46325.60511574074</v>
+        <v>46325.60633101852</v>
       </c>
       <c r="C146" s="13" t="n">
-        <v>46325.39678240741</v>
+        <v>46325.39799768518</v>
       </c>
       <c r="D146" s="13" t="n">
-        <v>46325.56344907408</v>
+        <v>46325.56466435185</v>
       </c>
       <c r="E146" s="14" t="inlineStr">
         <is>
@@ -23693,11 +23747,15 @@
       </c>
       <c r="I146" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J146" s="16" t="n"/>
-      <c r="K146" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J146" s="16" t="n">
+        <v>150.343801052</v>
+      </c>
+      <c r="K146" s="17" t="n">
+        <v>55.09</v>
+      </c>
       <c r="L146" s="17">
         <f>IF(AND(ISNUMBER(J146),ISNUMBER(K146)),J146*K146,"")</f>
         <v/>
@@ -23834,7 +23892,9 @@
       <c r="AX146" s="13" t="n">
         <v>46325.5634375</v>
       </c>
-      <c r="AY146" s="13" t="n"/>
+      <c r="AY146" s="13" t="n">
+        <v>46325.56466435185</v>
+      </c>
       <c r="AZ146" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
@@ -23845,13 +23905,13 @@
         <v>146</v>
       </c>
       <c r="B147" s="13" t="n">
-        <v>46325.60511574074</v>
+        <v>46325.60664351852</v>
       </c>
       <c r="C147" s="13" t="n">
-        <v>46325.39678240741</v>
+        <v>46325.39831018518</v>
       </c>
       <c r="D147" s="13" t="n">
-        <v>46325.56344907408</v>
+        <v>46325.56497685185</v>
       </c>
       <c r="E147" s="14" t="inlineStr">
         <is>
@@ -23875,11 +23935,15 @@
       </c>
       <c r="I147" s="6" t="inlineStr">
         <is>
-          <t>pending_new</t>
-        </is>
-      </c>
-      <c r="J147" s="16" t="n"/>
-      <c r="K147" s="17" t="n"/>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J147" s="16" t="n">
+        <v>76.12460944599999</v>
+      </c>
+      <c r="K147" s="17" t="n">
+        <v>108.801084</v>
+      </c>
       <c r="L147" s="17">
         <f>IF(AND(ISNUMBER(J147),ISNUMBER(K147)),J147*K147,"")</f>
         <v/>
@@ -24016,11 +24080,2413 @@
       <c r="AX147" s="13" t="n">
         <v>46325.56344907408</v>
       </c>
-      <c r="AY147" s="13" t="n"/>
+      <c r="AY147" s="13" t="n">
+        <v>46325.56497685185</v>
+      </c>
       <c r="AZ147" s="13" t="n">
         <v>46325.5627662037</v>
       </c>
       <c r="BA147" s="6" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="13" t="n">
+        <v>46325.6091087963</v>
+      </c>
+      <c r="C148" s="13" t="n">
+        <v>46325.40077546296</v>
+      </c>
+      <c r="D148" s="13" t="n">
+        <v>46325.56744212963</v>
+      </c>
+      <c r="E148" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F148" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="G148" s="15" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="H148" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I148" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J148" s="16" t="n">
+        <v>30.574919709</v>
+      </c>
+      <c r="K148" s="17" t="n">
+        <v>270.36</v>
+      </c>
+      <c r="L148" s="17">
+        <f>IF(AND(ISNUMBER(J148),ISNUMBER(K148)),J148*K148,"")</f>
+        <v/>
+      </c>
+      <c r="M148" s="17" t="n"/>
+      <c r="N148" s="16" t="n">
+        <v>30.574919709</v>
+      </c>
+      <c r="O148" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
+      <c r="P148" s="15" t="inlineStr">
+        <is>
+          <t>Only 1 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q148" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="R148" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S148" s="18" t="n">
+        <v>0.608</v>
+      </c>
+      <c r="T148" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="U148" s="19" t="n">
+        <v>0.0149</v>
+      </c>
+      <c r="V148" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W148" s="12" t="n"/>
+      <c r="X148" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y148" s="19" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="Z148" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AA148" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="AB148" s="15" t="inlineStr">
+        <is>
+          <t>Rose 3.4% then gave back most of it within hours. Looks like pump-and-fade.</t>
+        </is>
+      </c>
+      <c r="AC148" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD148" s="6" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="AE148" s="17" t="n">
+        <v>269.445</v>
+      </c>
+      <c r="AF148" s="17" t="n">
+        <v>259.6489</v>
+      </c>
+      <c r="AG148" s="17" t="n">
+        <v>279.2411</v>
+      </c>
+      <c r="AH148" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI148" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ148" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK148" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL148" s="15" t="inlineStr">
+        <is>
+          <t>TD Cowen Maintains Buy on IQVIA Holdings, Raises Price Target to $307</t>
+        </is>
+      </c>
+      <c r="AM148" s="17" t="n">
+        <v>269.445</v>
+      </c>
+      <c r="AN148" s="19" t="n">
+        <v>-0.019</v>
+      </c>
+      <c r="AO148" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP148" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ148" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR148" s="16" t="n">
+        <v>30.574919709</v>
+      </c>
+      <c r="AS148" s="17" t="n">
+        <v>270.89</v>
+      </c>
+      <c r="AT148" s="19" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="AU148" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV148" s="6" t="inlineStr">
+        <is>
+          <t>37b862e6-6e57-487a-ac6f-930b1731f235</t>
+        </is>
+      </c>
+      <c r="AW148" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-IQV-1793367425337</t>
+        </is>
+      </c>
+      <c r="AX148" s="13" t="n">
+        <v>46325.56741898148</v>
+      </c>
+      <c r="AY148" s="13" t="n">
+        <v>46325.56744212963</v>
+      </c>
+      <c r="AZ148" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA148" s="6" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="12" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="13" t="n">
+        <v>46325.60908564815</v>
+      </c>
+      <c r="C149" s="13" t="n">
+        <v>46325.40075231482</v>
+      </c>
+      <c r="D149" s="13" t="n">
+        <v>46325.56741898148</v>
+      </c>
+      <c r="E149" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F149" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="G149" s="15" t="inlineStr">
+        <is>
+          <t>Analog Devices, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H149" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I149" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J149" s="16" t="n">
+        <v>1.637432978</v>
+      </c>
+      <c r="K149" s="17" t="n">
+        <v>423.37</v>
+      </c>
+      <c r="L149" s="17">
+        <f>IF(AND(ISNUMBER(J149),ISNUMBER(K149)),J149*K149,"")</f>
+        <v/>
+      </c>
+      <c r="M149" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N149" s="16" t="n"/>
+      <c r="O149" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P149" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q149" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R149" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S149" s="18" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="T149" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="U149" s="19" t="n">
+        <v>0.0147</v>
+      </c>
+      <c r="V149" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W149" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X149" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y149" s="19" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="Z149" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA149" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB149" s="15" t="n"/>
+      <c r="AC149" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD149" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE149" s="17" t="n">
+        <v>430.0826</v>
+      </c>
+      <c r="AF149" s="17" t="n">
+        <v>411.051</v>
+      </c>
+      <c r="AG149" s="17" t="n">
+        <v>449.1142</v>
+      </c>
+      <c r="AH149" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI149" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ149" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK149" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL149" s="15" t="inlineStr">
+        <is>
+          <t>If You Invested $1000 In Analog Devices Stock 5 Years Ago, You Would Have This Much Today</t>
+        </is>
+      </c>
+      <c r="AM149" s="17" t="n">
+        <v>422.58</v>
+      </c>
+      <c r="AN149" s="19" t="n">
+        <v>-0.0248</v>
+      </c>
+      <c r="AO149" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP149" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ149" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR149" s="16" t="n"/>
+      <c r="AS149" s="17" t="n"/>
+      <c r="AT149" s="19" t="n"/>
+      <c r="AU149" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV149" s="6" t="inlineStr">
+        <is>
+          <t>1d4e579a-c77c-4eee-9733-1b9a79afe2c7</t>
+        </is>
+      </c>
+      <c r="AW149" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ADI-1793367425725</t>
+        </is>
+      </c>
+      <c r="AX149" s="13" t="n">
+        <v>46325.56741898148</v>
+      </c>
+      <c r="AY149" s="13" t="n">
+        <v>46325.56741898148</v>
+      </c>
+      <c r="AZ149" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA149" s="6" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="12" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="13" t="n">
+        <v>46325.60914351852</v>
+      </c>
+      <c r="C150" s="13" t="n">
+        <v>46325.40081018519</v>
+      </c>
+      <c r="D150" s="13" t="n">
+        <v>46325.56747685185</v>
+      </c>
+      <c r="E150" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F150" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="G150" s="15" t="inlineStr">
+        <is>
+          <t>Occidental Petroleum Corporation</t>
+        </is>
+      </c>
+      <c r="H150" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I150" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J150" s="16" t="n">
+        <v>10.872647427</v>
+      </c>
+      <c r="K150" s="17" t="n">
+        <v>63.76</v>
+      </c>
+      <c r="L150" s="17">
+        <f>IF(AND(ISNUMBER(J150),ISNUMBER(K150)),J150*K150,"")</f>
+        <v/>
+      </c>
+      <c r="M150" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N150" s="16" t="n"/>
+      <c r="O150" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P150" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #3, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q150" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R150" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S150" s="18" t="n">
+        <v>0.621</v>
+      </c>
+      <c r="T150" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="U150" s="19" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="V150" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W150" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X150" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y150" s="19" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="Z150" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA150" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB150" s="15" t="n"/>
+      <c r="AC150" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD150" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE150" s="17" t="n">
+        <v>64.5534</v>
+      </c>
+      <c r="AF150" s="17" t="n">
+        <v>62.0074</v>
+      </c>
+      <c r="AG150" s="17" t="n">
+        <v>67.0994</v>
+      </c>
+      <c r="AH150" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI150" s="18" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AJ150" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK150" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL150" s="15" t="n"/>
+      <c r="AM150" s="17" t="n">
+        <v>63.49</v>
+      </c>
+      <c r="AN150" s="19" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="AO150" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP150" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ150" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR150" s="16" t="n"/>
+      <c r="AS150" s="17" t="n"/>
+      <c r="AT150" s="19" t="n"/>
+      <c r="AU150" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV150" s="6" t="inlineStr">
+        <is>
+          <t>64ee67ad-aa68-41d6-af90-78737e29bde2</t>
+        </is>
+      </c>
+      <c r="AW150" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-OXY-1793367426265</t>
+        </is>
+      </c>
+      <c r="AX150" s="13" t="n">
+        <v>46325.56743055556</v>
+      </c>
+      <c r="AY150" s="13" t="n">
+        <v>46325.56747685185</v>
+      </c>
+      <c r="AZ150" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA150" s="6" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="13" t="n">
+        <v>46325.60912037037</v>
+      </c>
+      <c r="C151" s="13" t="n">
+        <v>46325.40078703704</v>
+      </c>
+      <c r="D151" s="13" t="n">
+        <v>46325.5674537037</v>
+      </c>
+      <c r="E151" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F151" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="G151" s="15" t="inlineStr">
+        <is>
+          <t>ABBVIE INC.</t>
+        </is>
+      </c>
+      <c r="H151" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I151" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J151" s="16" t="n">
+        <v>2.342106152</v>
+      </c>
+      <c r="K151" s="17" t="n">
+        <v>295.99</v>
+      </c>
+      <c r="L151" s="17">
+        <f>IF(AND(ISNUMBER(J151),ISNUMBER(K151)),J151*K151,"")</f>
+        <v/>
+      </c>
+      <c r="M151" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N151" s="16" t="n"/>
+      <c r="O151" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P151" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #4, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q151" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R151" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S151" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T151" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U151" s="19" t="n">
+        <v>0.0177</v>
+      </c>
+      <c r="V151" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W151" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X151" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y151" s="19" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="Z151" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA151" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB151" s="15" t="n"/>
+      <c r="AC151" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD151" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE151" s="17" t="n">
+        <v>297.3239</v>
+      </c>
+      <c r="AF151" s="17" t="n">
+        <v>289.2142</v>
+      </c>
+      <c r="AG151" s="17" t="n">
+        <v>305.4336</v>
+      </c>
+      <c r="AH151" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI151" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ151" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK151" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL151" s="15" t="inlineStr">
+        <is>
+          <t>AbbVie Raises FY2026 Adj EPS Guidance from $13.76-$13.96 to $13.95-$13.99 vs $13.93 Est</t>
+        </is>
+      </c>
+      <c r="AM151" s="17" t="n">
+        <v>294.46</v>
+      </c>
+      <c r="AN151" s="19" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="AO151" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP151" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ151" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR151" s="16" t="n"/>
+      <c r="AS151" s="17" t="n"/>
+      <c r="AT151" s="19" t="n"/>
+      <c r="AU151" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV151" s="6" t="inlineStr">
+        <is>
+          <t>dbc17052-8288-418e-be59-a06cc90f2b99</t>
+        </is>
+      </c>
+      <c r="AW151" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ABBV-1793367426625</t>
+        </is>
+      </c>
+      <c r="AX151" s="13" t="n">
+        <v>46325.56743055556</v>
+      </c>
+      <c r="AY151" s="13" t="n">
+        <v>46325.5674537037</v>
+      </c>
+      <c r="AZ151" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA151" s="6" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="12" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="13" t="n">
+        <v>46325.60915509259</v>
+      </c>
+      <c r="C152" s="13" t="n">
+        <v>46325.40082175926</v>
+      </c>
+      <c r="D152" s="13" t="n">
+        <v>46325.56748842593</v>
+      </c>
+      <c r="E152" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F152" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="G152" s="15" t="inlineStr">
+        <is>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+        </is>
+      </c>
+      <c r="H152" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I152" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J152" s="16" t="n">
+        <v>14.229932252</v>
+      </c>
+      <c r="K152" s="17" t="n">
+        <v>48.717028</v>
+      </c>
+      <c r="L152" s="17">
+        <f>IF(AND(ISNUMBER(J152),ISNUMBER(K152)),J152*K152,"")</f>
+        <v/>
+      </c>
+      <c r="M152" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N152" s="16" t="n"/>
+      <c r="O152" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P152" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #7, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q152" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R152" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S152" s="18" t="n">
+        <v>0.671</v>
+      </c>
+      <c r="T152" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="U152" s="19" t="n">
+        <v>0.0139</v>
+      </c>
+      <c r="V152" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W152" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="X152" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y152" s="19" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="Z152" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA152" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB152" s="15" t="n"/>
+      <c r="AC152" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD152" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE152" s="17" t="n">
+        <v>49.4953</v>
+      </c>
+      <c r="AF152" s="17" t="n">
+        <v>47.2321</v>
+      </c>
+      <c r="AG152" s="17" t="n">
+        <v>51.7584</v>
+      </c>
+      <c r="AH152" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI152" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ152" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK152" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL152" s="15" t="inlineStr">
+        <is>
+          <t>Equinor Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM152" s="17" t="n">
+        <v>48.56</v>
+      </c>
+      <c r="AN152" s="19" t="n">
+        <v>0.0208</v>
+      </c>
+      <c r="AO152" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP152" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ152" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR152" s="16" t="n"/>
+      <c r="AS152" s="17" t="n"/>
+      <c r="AT152" s="19" t="n"/>
+      <c r="AU152" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV152" s="6" t="inlineStr">
+        <is>
+          <t>1288753f-a95c-42cc-a3bf-c3902fb74c53</t>
+        </is>
+      </c>
+      <c r="AW152" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-EQNR-1793367427388</t>
+        </is>
+      </c>
+      <c r="AX152" s="13" t="n">
+        <v>46325.56744212963</v>
+      </c>
+      <c r="AY152" s="13" t="n">
+        <v>46325.56748842593</v>
+      </c>
+      <c r="AZ152" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA152" s="6" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="12" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="13" t="n">
+        <v>46325.60915509259</v>
+      </c>
+      <c r="C153" s="13" t="n">
+        <v>46325.40082175926</v>
+      </c>
+      <c r="D153" s="13" t="n">
+        <v>46325.56748842593</v>
+      </c>
+      <c r="E153" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F153" s="6" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="G153" s="15" t="inlineStr">
+        <is>
+          <t>SharkNinja, Inc.</t>
+        </is>
+      </c>
+      <c r="H153" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I153" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J153" s="16" t="n">
+        <v>3.304762358</v>
+      </c>
+      <c r="K153" s="17" t="n">
+        <v>209.77</v>
+      </c>
+      <c r="L153" s="17">
+        <f>IF(AND(ISNUMBER(J153),ISNUMBER(K153)),J153*K153,"")</f>
+        <v/>
+      </c>
+      <c r="M153" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N153" s="16" t="n"/>
+      <c r="O153" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P153" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #8, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q153" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R153" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S153" s="18" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="T153" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="U153" s="19" t="n">
+        <v>0.0143</v>
+      </c>
+      <c r="V153" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W153" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="X153" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y153" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z153" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA153" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB153" s="15" t="n"/>
+      <c r="AC153" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD153" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE153" s="17" t="n">
+        <v>213.3553</v>
+      </c>
+      <c r="AF153" s="17" t="n">
+        <v>202.3295</v>
+      </c>
+      <c r="AG153" s="17" t="n">
+        <v>224.3812</v>
+      </c>
+      <c r="AH153" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI153" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ153" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK153" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL153" s="15" t="inlineStr">
+        <is>
+          <t>Piper Sandler Raises SharkNinja Price Target to $234</t>
+        </is>
+      </c>
+      <c r="AM153" s="17" t="n">
+        <v>208.945</v>
+      </c>
+      <c r="AN153" s="19" t="n">
+        <v>-0.0021</v>
+      </c>
+      <c r="AO153" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP153" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ153" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR153" s="16" t="n"/>
+      <c r="AS153" s="17" t="n"/>
+      <c r="AT153" s="19" t="n"/>
+      <c r="AU153" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV153" s="6" t="inlineStr">
+        <is>
+          <t>7d290955-f67e-4ab2-bbed-7e18b5f58b35</t>
+        </is>
+      </c>
+      <c r="AW153" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-SN-1793367427758</t>
+        </is>
+      </c>
+      <c r="AX153" s="13" t="n">
+        <v>46325.56744212963</v>
+      </c>
+      <c r="AY153" s="13" t="n">
+        <v>46325.56748842593</v>
+      </c>
+      <c r="AZ153" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA153" s="6" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="12" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="13" t="n">
+        <v>46325.60914351852</v>
+      </c>
+      <c r="C154" s="13" t="n">
+        <v>46325.40081018519</v>
+      </c>
+      <c r="D154" s="13" t="n">
+        <v>46325.56747685185</v>
+      </c>
+      <c r="E154" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F154" s="6" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="G154" s="15" t="inlineStr">
+        <is>
+          <t>Intercontinental Exchange  Inc.</t>
+        </is>
+      </c>
+      <c r="H154" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I154" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J154" s="16" t="n">
+        <v>4.145924286</v>
+      </c>
+      <c r="K154" s="17" t="n">
+        <v>167.21</v>
+      </c>
+      <c r="L154" s="17">
+        <f>IF(AND(ISNUMBER(J154),ISNUMBER(K154)),J154*K154,"")</f>
+        <v/>
+      </c>
+      <c r="M154" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N154" s="16" t="n"/>
+      <c r="O154" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P154" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #9, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q154" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R154" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S154" s="18" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="T154" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="U154" s="19" t="n">
+        <v>0.0083</v>
+      </c>
+      <c r="V154" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W154" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="X154" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y154" s="19" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="Z154" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA154" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB154" s="15" t="n"/>
+      <c r="AC154" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD154" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE154" s="17" t="n">
+        <v>169.0806</v>
+      </c>
+      <c r="AF154" s="17" t="n">
+        <v>163.504</v>
+      </c>
+      <c r="AG154" s="17" t="n">
+        <v>174.6573</v>
+      </c>
+      <c r="AH154" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI154" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ154" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK154" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL154" s="15" t="inlineStr">
+        <is>
+          <t>Intercontinental Exchange Updates Timeline for MarketAxess Acquisition</t>
+        </is>
+      </c>
+      <c r="AM154" s="17" t="n">
+        <v>166.85</v>
+      </c>
+      <c r="AN154" s="19" t="n">
+        <v>0.0238</v>
+      </c>
+      <c r="AO154" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP154" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ154" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR154" s="16" t="n"/>
+      <c r="AS154" s="17" t="n"/>
+      <c r="AT154" s="19" t="n"/>
+      <c r="AU154" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV154" s="6" t="inlineStr">
+        <is>
+          <t>3900e1dd-02f8-49fa-abc8-e385dff5a3a5</t>
+        </is>
+      </c>
+      <c r="AW154" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ICE-1793367428109</t>
+        </is>
+      </c>
+      <c r="AX154" s="13" t="n">
+        <v>46325.5674537037</v>
+      </c>
+      <c r="AY154" s="13" t="n">
+        <v>46325.56747685185</v>
+      </c>
+      <c r="AZ154" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA154" s="6" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="12" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="13" t="n">
+        <v>46325.60915509259</v>
+      </c>
+      <c r="C155" s="13" t="n">
+        <v>46325.40082175926</v>
+      </c>
+      <c r="D155" s="13" t="n">
+        <v>46325.56748842593</v>
+      </c>
+      <c r="E155" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F155" s="6" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="G155" s="15" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H155" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I155" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J155" s="16" t="n">
+        <v>2.362539617</v>
+      </c>
+      <c r="K155" s="17" t="n">
+        <v>293.43</v>
+      </c>
+      <c r="L155" s="17">
+        <f>IF(AND(ISNUMBER(J155),ISNUMBER(K155)),J155*K155,"")</f>
+        <v/>
+      </c>
+      <c r="M155" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N155" s="16" t="n"/>
+      <c r="O155" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P155" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #10, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q155" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R155" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S155" s="18" t="n">
+        <v>0.648</v>
+      </c>
+      <c r="T155" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="U155" s="19" t="n">
+        <v>0.0132</v>
+      </c>
+      <c r="V155" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W155" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="X155" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y155" s="19" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Z155" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA155" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB155" s="15" t="n"/>
+      <c r="AC155" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD155" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE155" s="17" t="n">
+        <v>296.5587</v>
+      </c>
+      <c r="AF155" s="17" t="n">
+        <v>286.3619</v>
+      </c>
+      <c r="AG155" s="17" t="n">
+        <v>306.7556</v>
+      </c>
+      <c r="AH155" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI155" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ155" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK155" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL155" s="15" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing Q1 2027 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM155" s="17" t="n">
+        <v>292.61</v>
+      </c>
+      <c r="AN155" s="19" t="n">
+        <v>0.0223</v>
+      </c>
+      <c r="AO155" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP155" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ155" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR155" s="16" t="n"/>
+      <c r="AS155" s="17" t="n"/>
+      <c r="AT155" s="19" t="n"/>
+      <c r="AU155" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV155" s="6" t="inlineStr">
+        <is>
+          <t>295fd24e-6551-4219-a27c-1173fa9d0833</t>
+        </is>
+      </c>
+      <c r="AW155" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ADP-1793367428507</t>
+        </is>
+      </c>
+      <c r="AX155" s="13" t="n">
+        <v>46325.5674537037</v>
+      </c>
+      <c r="AY155" s="13" t="n">
+        <v>46325.56748842593</v>
+      </c>
+      <c r="AZ155" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA155" s="6" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="12" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="13" t="n">
+        <v>46325.60915509259</v>
+      </c>
+      <c r="C156" s="13" t="n">
+        <v>46325.40082175926</v>
+      </c>
+      <c r="D156" s="13" t="n">
+        <v>46325.56748842593</v>
+      </c>
+      <c r="E156" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F156" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="G156" s="15" t="inlineStr">
+        <is>
+          <t>Monster Beverage Corporation</t>
+        </is>
+      </c>
+      <c r="H156" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I156" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J156" s="16" t="n">
+        <v>14.687288135</v>
+      </c>
+      <c r="K156" s="17" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="L156" s="17">
+        <f>IF(AND(ISNUMBER(J156),ISNUMBER(K156)),J156*K156,"")</f>
+        <v/>
+      </c>
+      <c r="M156" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N156" s="16" t="n"/>
+      <c r="O156" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P156" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #11, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q156" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R156" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S156" s="18" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="T156" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="U156" s="19" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="V156" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W156" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="X156" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y156" s="19" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="Z156" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA156" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB156" s="15" t="n"/>
+      <c r="AC156" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD156" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE156" s="17" t="n">
+        <v>47.9107</v>
+      </c>
+      <c r="AF156" s="17" t="n">
+        <v>46.234</v>
+      </c>
+      <c r="AG156" s="17" t="n">
+        <v>49.5873</v>
+      </c>
+      <c r="AH156" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI156" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ156" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK156" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL156" s="15" t="inlineStr">
+        <is>
+          <t>Monster Beverage Corporation Announces Third Quarter 2026 Earnings Release Date</t>
+        </is>
+      </c>
+      <c r="AM156" s="17" t="n">
+        <v>47.24</v>
+      </c>
+      <c r="AN156" s="19" t="n">
+        <v>0.0189</v>
+      </c>
+      <c r="AO156" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP156" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ156" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR156" s="16" t="n"/>
+      <c r="AS156" s="17" t="n"/>
+      <c r="AT156" s="19" t="n"/>
+      <c r="AU156" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV156" s="6" t="inlineStr">
+        <is>
+          <t>e6c7e054-2150-45fb-b223-75931e03dd36</t>
+        </is>
+      </c>
+      <c r="AW156" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MNST-1793367428855</t>
+        </is>
+      </c>
+      <c r="AX156" s="13" t="n">
+        <v>46325.5674537037</v>
+      </c>
+      <c r="AY156" s="13" t="n">
+        <v>46325.56748842593</v>
+      </c>
+      <c r="AZ156" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA156" s="6" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="12" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="13" t="n">
+        <v>46325.60916666667</v>
+      </c>
+      <c r="C157" s="13" t="n">
+        <v>46325.40083333333</v>
+      </c>
+      <c r="D157" s="13" t="n">
+        <v>46325.5675</v>
+      </c>
+      <c r="E157" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F157" s="6" t="inlineStr">
+        <is>
+          <t>CBOE</t>
+        </is>
+      </c>
+      <c r="G157" s="15" t="inlineStr">
+        <is>
+          <t>Cboe Global Markets, Inc.</t>
+        </is>
+      </c>
+      <c r="H157" s="6" t="inlineStr">
+        <is>
+          <t>BATS</t>
+        </is>
+      </c>
+      <c r="I157" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J157" s="16" t="n">
+        <v>2.096661021</v>
+      </c>
+      <c r="K157" s="17" t="n">
+        <v>330.64</v>
+      </c>
+      <c r="L157" s="17">
+        <f>IF(AND(ISNUMBER(J157),ISNUMBER(K157)),J157*K157,"")</f>
+        <v/>
+      </c>
+      <c r="M157" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N157" s="16" t="n"/>
+      <c r="O157" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P157" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #12, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q157" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R157" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S157" s="18" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="T157" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="U157" s="19" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="V157" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W157" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="X157" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y157" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z157" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA157" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB157" s="15" t="n"/>
+      <c r="AC157" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD157" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE157" s="17" t="n">
+        <v>334.9048</v>
+      </c>
+      <c r="AF157" s="17" t="n">
+        <v>317.5679</v>
+      </c>
+      <c r="AG157" s="17" t="n">
+        <v>352.2417</v>
+      </c>
+      <c r="AH157" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI157" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ157" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK157" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL157" s="15" t="inlineStr">
+        <is>
+          <t>Cboe Global Markets Q3 Adj. EPS $3.63 Beats $3.43 Estimate, Sales $712.200M Beat $706.412M Estimate</t>
+        </is>
+      </c>
+      <c r="AM157" s="17" t="n">
+        <v>327.97</v>
+      </c>
+      <c r="AN157" s="19" t="n">
+        <v>0.0451</v>
+      </c>
+      <c r="AO157" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP157" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ157" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR157" s="16" t="n"/>
+      <c r="AS157" s="17" t="n"/>
+      <c r="AT157" s="19" t="n"/>
+      <c r="AU157" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV157" s="6" t="inlineStr">
+        <is>
+          <t>33c92f83-68a7-456c-ad64-2a5682129dda</t>
+        </is>
+      </c>
+      <c r="AW157" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-CBOE-1793367429323</t>
+        </is>
+      </c>
+      <c r="AX157" s="13" t="n">
+        <v>46325.56746527777</v>
+      </c>
+      <c r="AY157" s="13" t="n">
+        <v>46325.5675</v>
+      </c>
+      <c r="AZ157" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA157" s="6" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="12" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="13" t="n">
+        <v>46325.60917824074</v>
+      </c>
+      <c r="C158" s="13" t="n">
+        <v>46325.40084490741</v>
+      </c>
+      <c r="D158" s="13" t="n">
+        <v>46325.56751157407</v>
+      </c>
+      <c r="E158" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F158" s="6" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="G158" s="15" t="inlineStr">
+        <is>
+          <t>Cognizant Technology Solutions Corporation Class A Common Stock</t>
+        </is>
+      </c>
+      <c r="H158" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I158" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J158" s="16" t="n">
+        <v>10.809917355</v>
+      </c>
+      <c r="K158" s="17" t="n">
+        <v>64.13</v>
+      </c>
+      <c r="L158" s="17">
+        <f>IF(AND(ISNUMBER(J158),ISNUMBER(K158)),J158*K158,"")</f>
+        <v/>
+      </c>
+      <c r="M158" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N158" s="16" t="n"/>
+      <c r="O158" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P158" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #13, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q158" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R158" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S158" s="18" t="n">
+        <v>0.587</v>
+      </c>
+      <c r="T158" s="12" t="n">
+        <v>46</v>
+      </c>
+      <c r="U158" s="19" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="V158" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W158" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="X158" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y158" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z158" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA158" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB158" s="15" t="n"/>
+      <c r="AC158" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD158" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE158" s="17" t="n">
+        <v>65.95740000000001</v>
+      </c>
+      <c r="AF158" s="17" t="n">
+        <v>62.0015</v>
+      </c>
+      <c r="AG158" s="17" t="n">
+        <v>69.9132</v>
+      </c>
+      <c r="AH158" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI158" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ158" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK158" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL158" s="15" t="inlineStr">
+        <is>
+          <t>Cognizant Tech Solns Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM158" s="17" t="n">
+        <v>64.375</v>
+      </c>
+      <c r="AN158" s="19" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="AO158" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP158" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ158" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR158" s="16" t="n"/>
+      <c r="AS158" s="17" t="n"/>
+      <c r="AT158" s="19" t="n"/>
+      <c r="AU158" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV158" s="6" t="inlineStr">
+        <is>
+          <t>bc151369-b0e4-4f81-980e-7311df152c15</t>
+        </is>
+      </c>
+      <c r="AW158" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-CTSH-1793367429719</t>
+        </is>
+      </c>
+      <c r="AX158" s="13" t="n">
+        <v>46325.56746527777</v>
+      </c>
+      <c r="AY158" s="13" t="n">
+        <v>46325.56751157407</v>
+      </c>
+      <c r="AZ158" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA158" s="6" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="13" t="n">
+        <v>46325.60917824074</v>
+      </c>
+      <c r="C159" s="13" t="n">
+        <v>46325.40084490741</v>
+      </c>
+      <c r="D159" s="13" t="n">
+        <v>46325.56751157407</v>
+      </c>
+      <c r="E159" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F159" s="6" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="G159" s="15" t="inlineStr">
+        <is>
+          <t>Zscaler, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H159" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I159" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J159" s="16" t="n">
+        <v>2.823788187</v>
+      </c>
+      <c r="K159" s="17" t="n">
+        <v>245.5</v>
+      </c>
+      <c r="L159" s="17">
+        <f>IF(AND(ISNUMBER(J159),ISNUMBER(K159)),J159*K159,"")</f>
+        <v/>
+      </c>
+      <c r="M159" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N159" s="16" t="n"/>
+      <c r="O159" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P159" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #14, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q159" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R159" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S159" s="18" t="n">
+        <v>0.5580000000000001</v>
+      </c>
+      <c r="T159" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="U159" s="19" t="n">
+        <v>0.0164</v>
+      </c>
+      <c r="V159" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W159" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="X159" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y159" s="19" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="Z159" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA159" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB159" s="15" t="n"/>
+      <c r="AC159" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD159" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE159" s="17" t="n">
+        <v>254.0979</v>
+      </c>
+      <c r="AF159" s="17" t="n">
+        <v>231.0406</v>
+      </c>
+      <c r="AG159" s="17" t="n">
+        <v>277.1553</v>
+      </c>
+      <c r="AH159" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI159" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ159" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK159" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL159" s="15" t="inlineStr">
+        <is>
+          <t>ServiceNow Posts Downbeat Q3 Earnings, Joins Sprouts Farmers Market, Alphabet And Other Big Stocks Moving Lower In Thursday’s Pre-Market Session</t>
+        </is>
+      </c>
+      <c r="AM159" s="17" t="n">
+        <v>245.28</v>
+      </c>
+      <c r="AN159" s="19" t="n">
+        <v>-0.0115</v>
+      </c>
+      <c r="AO159" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP159" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ159" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR159" s="16" t="n"/>
+      <c r="AS159" s="17" t="n"/>
+      <c r="AT159" s="19" t="n"/>
+      <c r="AU159" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV159" s="6" t="inlineStr">
+        <is>
+          <t>221087d9-06fa-499f-a134-d0ef36ce31fd</t>
+        </is>
+      </c>
+      <c r="AW159" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ZS-1793367430074</t>
+        </is>
+      </c>
+      <c r="AX159" s="13" t="n">
+        <v>46325.56747685185</v>
+      </c>
+      <c r="AY159" s="13" t="n">
+        <v>46325.56751157407</v>
+      </c>
+      <c r="AZ159" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA159" s="6" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="12" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" s="13" t="n">
+        <v>46325.60918981482</v>
+      </c>
+      <c r="C160" s="13" t="n">
+        <v>46325.40085648148</v>
+      </c>
+      <c r="D160" s="13" t="n">
+        <v>46325.56752314815</v>
+      </c>
+      <c r="E160" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F160" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="G160" s="15" t="inlineStr">
+        <is>
+          <t>The Kroger Co.</t>
+        </is>
+      </c>
+      <c r="H160" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I160" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J160" s="16" t="n">
+        <v>10.24745011</v>
+      </c>
+      <c r="K160" s="17" t="n">
+        <v>67.65000000000001</v>
+      </c>
+      <c r="L160" s="17">
+        <f>IF(AND(ISNUMBER(J160),ISNUMBER(K160)),J160*K160,"")</f>
+        <v/>
+      </c>
+      <c r="M160" s="17" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="N160" s="16" t="n"/>
+      <c r="O160" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P160" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #15, 8.33% of the $8,322.34 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q160" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R160" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S160" s="18" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="T160" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="U160" s="19" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="V160" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W160" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="X160" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y160" s="19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="Z160" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA160" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB160" s="15" t="inlineStr">
+        <is>
+          <t>One day (+5.8%) did 92% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC160" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD160" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE160" s="17" t="n">
+        <v>68.7871</v>
+      </c>
+      <c r="AF160" s="17" t="n">
+        <v>66.0444</v>
+      </c>
+      <c r="AG160" s="17" t="n">
+        <v>71.52979999999999</v>
+      </c>
+      <c r="AH160" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI160" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ160" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK160" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL160" s="15" t="inlineStr">
+        <is>
+          <t>Evergreen Family Wines Expands Alki Chardonnay Distribution to Kroger Stores</t>
+        </is>
+      </c>
+      <c r="AM160" s="17" t="n">
+        <v>67.68000000000001</v>
+      </c>
+      <c r="AN160" s="19" t="n">
+        <v>0.0265</v>
+      </c>
+      <c r="AO160" s="17" t="n">
+        <v>99570.17</v>
+      </c>
+      <c r="AP160" s="17" t="n">
+        <v>8322.34</v>
+      </c>
+      <c r="AQ160" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR160" s="16" t="n"/>
+      <c r="AS160" s="17" t="n"/>
+      <c r="AT160" s="19" t="n"/>
+      <c r="AU160" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV160" s="6" t="inlineStr">
+        <is>
+          <t>b5262411-61fa-4e52-9fac-cdd5c66efca6</t>
+        </is>
+      </c>
+      <c r="AW160" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-KR-1793367430438</t>
+        </is>
+      </c>
+      <c r="AX160" s="13" t="n">
+        <v>46325.56747685185</v>
+      </c>
+      <c r="AY160" s="13" t="n">
+        <v>46325.56752314815</v>
+      </c>
+      <c r="AZ160" s="13" t="n">
+        <v>46325.56684027778</v>
+      </c>
+      <c r="BA160" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24037,7 +26503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P74"/>
+  <dimension ref="A1:P97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -28739,8 +31205,1237 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Intuitive Surgical, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C75" s="22" t="n">
+        <v>46325.60603009259</v>
+      </c>
+      <c r="D75" s="22" t="n">
+        <v>46325.39769675926</v>
+      </c>
+      <c r="E75" s="17" t="n">
+        <v>447.77</v>
+      </c>
+      <c r="F75" s="16" t="n">
+        <v>18.497085557</v>
+      </c>
+      <c r="G75" s="17">
+        <f>E75*F75</f>
+        <v/>
+      </c>
+      <c r="H75" s="22" t="n"/>
+      <c r="I75" s="22" t="n"/>
+      <c r="J75" s="17" t="n"/>
+      <c r="K75" s="17">
+        <f>IF(ISNUMBER(J75),J75*F75,"")</f>
+        <v/>
+      </c>
+      <c r="L75" s="23">
+        <f>IF(ISNUMBER(J75),K75-G75,"")</f>
+        <v/>
+      </c>
+      <c r="M75" s="24">
+        <f>IF(ISNUMBER(J75),L75/G75,"")</f>
+        <v/>
+      </c>
+      <c r="N75" s="25">
+        <f>IF(ISNUMBER(H75),H75-C75,"")</f>
+        <v/>
+      </c>
+      <c r="O75" s="6" t="n"/>
+      <c r="P75" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>McKesson Corporation</t>
+        </is>
+      </c>
+      <c r="C76" s="22" t="n">
+        <v>46325.60611111111</v>
+      </c>
+      <c r="D76" s="22" t="n">
+        <v>46325.39777777778</v>
+      </c>
+      <c r="E76" s="17" t="n">
+        <v>1009.84</v>
+      </c>
+      <c r="F76" s="16" t="n">
+        <v>8.201734928</v>
+      </c>
+      <c r="G76" s="17">
+        <f>E76*F76</f>
+        <v/>
+      </c>
+      <c r="H76" s="22" t="n"/>
+      <c r="I76" s="22" t="n"/>
+      <c r="J76" s="17" t="n"/>
+      <c r="K76" s="17">
+        <f>IF(ISNUMBER(J76),J76*F76,"")</f>
+        <v/>
+      </c>
+      <c r="L76" s="23">
+        <f>IF(ISNUMBER(J76),K76-G76,"")</f>
+        <v/>
+      </c>
+      <c r="M76" s="24">
+        <f>IF(ISNUMBER(J76),L76/G76,"")</f>
+        <v/>
+      </c>
+      <c r="N76" s="25">
+        <f>IF(ISNUMBER(H76),H76-C76,"")</f>
+        <v/>
+      </c>
+      <c r="O76" s="6" t="n"/>
+      <c r="P76" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>eBay Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C77" s="22" t="n">
+        <v>46325.60626157407</v>
+      </c>
+      <c r="D77" s="22" t="n">
+        <v>46325.39792824074</v>
+      </c>
+      <c r="E77" s="17" t="n">
+        <v>120.92</v>
+      </c>
+      <c r="F77" s="16" t="n">
+        <v>68.49520344</v>
+      </c>
+      <c r="G77" s="17">
+        <f>E77*F77</f>
+        <v/>
+      </c>
+      <c r="H77" s="22" t="n"/>
+      <c r="I77" s="22" t="n"/>
+      <c r="J77" s="17" t="n"/>
+      <c r="K77" s="17">
+        <f>IF(ISNUMBER(J77),J77*F77,"")</f>
+        <v/>
+      </c>
+      <c r="L77" s="23">
+        <f>IF(ISNUMBER(J77),K77-G77,"")</f>
+        <v/>
+      </c>
+      <c r="M77" s="24">
+        <f>IF(ISNUMBER(J77),L77/G77,"")</f>
+        <v/>
+      </c>
+      <c r="N77" s="25">
+        <f>IF(ISNUMBER(H77),H77-C77,"")</f>
+        <v/>
+      </c>
+      <c r="O77" s="6" t="n"/>
+      <c r="P77" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>EQT CORP</t>
+        </is>
+      </c>
+      <c r="C78" s="22" t="n">
+        <v>46325.60633101852</v>
+      </c>
+      <c r="D78" s="22" t="n">
+        <v>46325.39799768518</v>
+      </c>
+      <c r="E78" s="17" t="n">
+        <v>55.09</v>
+      </c>
+      <c r="F78" s="16" t="n">
+        <v>150.343801052</v>
+      </c>
+      <c r="G78" s="17">
+        <f>E78*F78</f>
+        <v/>
+      </c>
+      <c r="H78" s="22" t="n"/>
+      <c r="I78" s="22" t="n"/>
+      <c r="J78" s="17" t="n"/>
+      <c r="K78" s="17">
+        <f>IF(ISNUMBER(J78),J78*F78,"")</f>
+        <v/>
+      </c>
+      <c r="L78" s="23">
+        <f>IF(ISNUMBER(J78),K78-G78,"")</f>
+        <v/>
+      </c>
+      <c r="M78" s="24">
+        <f>IF(ISNUMBER(J78),L78/G78,"")</f>
+        <v/>
+      </c>
+      <c r="N78" s="25">
+        <f>IF(ISNUMBER(H78),H78-C78,"")</f>
+        <v/>
+      </c>
+      <c r="O78" s="6" t="n"/>
+      <c r="P78" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>IQVIA Holdings Inc.</t>
+        </is>
+      </c>
+      <c r="C79" s="22" t="n">
+        <v>46325.60637731481</v>
+      </c>
+      <c r="D79" s="22" t="n">
+        <v>46325.39804398148</v>
+      </c>
+      <c r="E79" s="17" t="n">
+        <v>270.89</v>
+      </c>
+      <c r="F79" s="16" t="n">
+        <v>30.574919709</v>
+      </c>
+      <c r="G79" s="17">
+        <f>E79*F79</f>
+        <v/>
+      </c>
+      <c r="H79" s="22" t="n">
+        <v>46325.6091087963</v>
+      </c>
+      <c r="I79" s="22" t="n">
+        <v>46325.40077546296</v>
+      </c>
+      <c r="J79" s="17" t="n">
+        <v>270.36</v>
+      </c>
+      <c r="K79" s="17">
+        <f>IF(ISNUMBER(J79),J79*F79,"")</f>
+        <v/>
+      </c>
+      <c r="L79" s="23">
+        <f>IF(ISNUMBER(J79),K79-G79,"")</f>
+        <v/>
+      </c>
+      <c r="M79" s="24">
+        <f>IF(ISNUMBER(J79),L79/G79,"")</f>
+        <v/>
+      </c>
+      <c r="N79" s="25">
+        <f>IF(ISNUMBER(H79),H79-C79,"")</f>
+        <v/>
+      </c>
+      <c r="O79" s="6" t="inlineStr">
+        <is>
+          <t>2 or fewer green</t>
+        </is>
+      </c>
+      <c r="P79" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific, Inc.</t>
+        </is>
+      </c>
+      <c r="C80" s="22" t="n">
+        <v>46325.6065162037</v>
+      </c>
+      <c r="D80" s="22" t="n">
+        <v>46325.39818287037</v>
+      </c>
+      <c r="E80" s="17" t="n">
+        <v>711.38</v>
+      </c>
+      <c r="F80" s="16" t="n">
+        <v>11.642778824</v>
+      </c>
+      <c r="G80" s="17">
+        <f>E80*F80</f>
+        <v/>
+      </c>
+      <c r="H80" s="22" t="n"/>
+      <c r="I80" s="22" t="n"/>
+      <c r="J80" s="17" t="n"/>
+      <c r="K80" s="17">
+        <f>IF(ISNUMBER(J80),J80*F80,"")</f>
+        <v/>
+      </c>
+      <c r="L80" s="23">
+        <f>IF(ISNUMBER(J80),K80-G80,"")</f>
+        <v/>
+      </c>
+      <c r="M80" s="24">
+        <f>IF(ISNUMBER(J80),L80/G80,"")</f>
+        <v/>
+      </c>
+      <c r="N80" s="25">
+        <f>IF(ISNUMBER(H80),H80-C80,"")</f>
+        <v/>
+      </c>
+      <c r="O80" s="6" t="n"/>
+      <c r="P80" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>Shell plc American Depositary Shares (Each represents two Ordinary shares)</t>
+        </is>
+      </c>
+      <c r="C81" s="22" t="n">
+        <v>46325.60664351852</v>
+      </c>
+      <c r="D81" s="22" t="n">
+        <v>46325.39831018518</v>
+      </c>
+      <c r="E81" s="17" t="n">
+        <v>108.801084</v>
+      </c>
+      <c r="F81" s="16" t="n">
+        <v>76.12460944599999</v>
+      </c>
+      <c r="G81" s="17">
+        <f>E81*F81</f>
+        <v/>
+      </c>
+      <c r="H81" s="22" t="n"/>
+      <c r="I81" s="22" t="n"/>
+      <c r="J81" s="17" t="n"/>
+      <c r="K81" s="17">
+        <f>IF(ISNUMBER(J81),J81*F81,"")</f>
+        <v/>
+      </c>
+      <c r="L81" s="23">
+        <f>IF(ISNUMBER(J81),K81-G81,"")</f>
+        <v/>
+      </c>
+      <c r="M81" s="24">
+        <f>IF(ISNUMBER(J81),L81/G81,"")</f>
+        <v/>
+      </c>
+      <c r="N81" s="25">
+        <f>IF(ISNUMBER(H81),H81-C81,"")</f>
+        <v/>
+      </c>
+      <c r="O81" s="6" t="n"/>
+      <c r="P81" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>MARATHON PETROLEUM CORPORATION</t>
+        </is>
+      </c>
+      <c r="C82" s="22" t="n">
+        <v>46325.60696759259</v>
+      </c>
+      <c r="D82" s="22" t="n">
+        <v>46325.39863425926</v>
+      </c>
+      <c r="E82" s="17" t="n">
+        <v>442</v>
+      </c>
+      <c r="F82" s="16" t="n">
+        <v>18.738552036</v>
+      </c>
+      <c r="G82" s="17">
+        <f>E82*F82</f>
+        <v/>
+      </c>
+      <c r="H82" s="22" t="n"/>
+      <c r="I82" s="22" t="n"/>
+      <c r="J82" s="17" t="n"/>
+      <c r="K82" s="17">
+        <f>IF(ISNUMBER(J82),J82*F82,"")</f>
+        <v/>
+      </c>
+      <c r="L82" s="23">
+        <f>IF(ISNUMBER(J82),K82-G82,"")</f>
+        <v/>
+      </c>
+      <c r="M82" s="24">
+        <f>IF(ISNUMBER(J82),L82/G82,"")</f>
+        <v/>
+      </c>
+      <c r="N82" s="25">
+        <f>IF(ISNUMBER(H82),H82-C82,"")</f>
+        <v/>
+      </c>
+      <c r="O82" s="6" t="n"/>
+      <c r="P82" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>Avantor, Inc.</t>
+        </is>
+      </c>
+      <c r="C83" s="22" t="n">
+        <v>46325.60703703704</v>
+      </c>
+      <c r="D83" s="22" t="n">
+        <v>46325.3987037037</v>
+      </c>
+      <c r="E83" s="17" t="n">
+        <v>16.368458</v>
+      </c>
+      <c r="F83" s="16" t="n">
+        <v>506</v>
+      </c>
+      <c r="G83" s="17">
+        <f>E83*F83</f>
+        <v/>
+      </c>
+      <c r="H83" s="22" t="n"/>
+      <c r="I83" s="22" t="n"/>
+      <c r="J83" s="17" t="n"/>
+      <c r="K83" s="17">
+        <f>IF(ISNUMBER(J83),J83*F83,"")</f>
+        <v/>
+      </c>
+      <c r="L83" s="23">
+        <f>IF(ISNUMBER(J83),K83-G83,"")</f>
+        <v/>
+      </c>
+      <c r="M83" s="24">
+        <f>IF(ISNUMBER(J83),L83/G83,"")</f>
+        <v/>
+      </c>
+      <c r="N83" s="25">
+        <f>IF(ISNUMBER(H83),H83-C83,"")</f>
+        <v/>
+      </c>
+      <c r="O83" s="6" t="n"/>
+      <c r="P83" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Willis Towers Watson Public Limited Company Ordinary Shares</t>
+        </is>
+      </c>
+      <c r="C84" s="22" t="n">
+        <v>46325.60714120371</v>
+      </c>
+      <c r="D84" s="22" t="n">
+        <v>46325.39880787037</v>
+      </c>
+      <c r="E84" s="17" t="n">
+        <v>325.993415</v>
+      </c>
+      <c r="F84" s="16" t="n">
+        <v>25.40677088</v>
+      </c>
+      <c r="G84" s="17">
+        <f>E84*F84</f>
+        <v/>
+      </c>
+      <c r="H84" s="22" t="n"/>
+      <c r="I84" s="22" t="n"/>
+      <c r="J84" s="17" t="n"/>
+      <c r="K84" s="17">
+        <f>IF(ISNUMBER(J84),J84*F84,"")</f>
+        <v/>
+      </c>
+      <c r="L84" s="23">
+        <f>IF(ISNUMBER(J84),K84-G84,"")</f>
+        <v/>
+      </c>
+      <c r="M84" s="24">
+        <f>IF(ISNUMBER(J84),L84/G84,"")</f>
+        <v/>
+      </c>
+      <c r="N84" s="25">
+        <f>IF(ISNUMBER(H84),H84-C84,"")</f>
+        <v/>
+      </c>
+      <c r="O84" s="6" t="n"/>
+      <c r="P84" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>Veeva Systems Inc.</t>
+        </is>
+      </c>
+      <c r="C85" s="22" t="n">
+        <v>46325.60730324074</v>
+      </c>
+      <c r="D85" s="22" t="n">
+        <v>46325.39896990741</v>
+      </c>
+      <c r="E85" s="17" t="n">
+        <v>313.499635</v>
+      </c>
+      <c r="F85" s="16" t="n">
+        <v>26.419297124</v>
+      </c>
+      <c r="G85" s="17">
+        <f>E85*F85</f>
+        <v/>
+      </c>
+      <c r="H85" s="22" t="n"/>
+      <c r="I85" s="22" t="n"/>
+      <c r="J85" s="17" t="n"/>
+      <c r="K85" s="17">
+        <f>IF(ISNUMBER(J85),J85*F85,"")</f>
+        <v/>
+      </c>
+      <c r="L85" s="23">
+        <f>IF(ISNUMBER(J85),K85-G85,"")</f>
+        <v/>
+      </c>
+      <c r="M85" s="24">
+        <f>IF(ISNUMBER(J85),L85/G85,"")</f>
+        <v/>
+      </c>
+      <c r="N85" s="25">
+        <f>IF(ISNUMBER(H85),H85-C85,"")</f>
+        <v/>
+      </c>
+      <c r="O85" s="6" t="n"/>
+      <c r="P85" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>Analog Devices, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C86" s="22" t="n">
+        <v>46325.60908564815</v>
+      </c>
+      <c r="D86" s="22" t="n">
+        <v>46325.40075231482</v>
+      </c>
+      <c r="E86" s="17" t="n">
+        <v>423.37</v>
+      </c>
+      <c r="F86" s="16" t="n">
+        <v>1.637432978</v>
+      </c>
+      <c r="G86" s="17">
+        <f>E86*F86</f>
+        <v/>
+      </c>
+      <c r="H86" s="22" t="n"/>
+      <c r="I86" s="22" t="n"/>
+      <c r="J86" s="17" t="n"/>
+      <c r="K86" s="17">
+        <f>IF(ISNUMBER(J86),J86*F86,"")</f>
+        <v/>
+      </c>
+      <c r="L86" s="23">
+        <f>IF(ISNUMBER(J86),K86-G86,"")</f>
+        <v/>
+      </c>
+      <c r="M86" s="24">
+        <f>IF(ISNUMBER(J86),L86/G86,"")</f>
+        <v/>
+      </c>
+      <c r="N86" s="25">
+        <f>IF(ISNUMBER(H86),H86-C86,"")</f>
+        <v/>
+      </c>
+      <c r="O86" s="6" t="n"/>
+      <c r="P86" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>ABBVIE INC.</t>
+        </is>
+      </c>
+      <c r="C87" s="22" t="n">
+        <v>46325.60912037037</v>
+      </c>
+      <c r="D87" s="22" t="n">
+        <v>46325.40078703704</v>
+      </c>
+      <c r="E87" s="17" t="n">
+        <v>295.99</v>
+      </c>
+      <c r="F87" s="16" t="n">
+        <v>2.342106152</v>
+      </c>
+      <c r="G87" s="17">
+        <f>E87*F87</f>
+        <v/>
+      </c>
+      <c r="H87" s="22" t="n"/>
+      <c r="I87" s="22" t="n"/>
+      <c r="J87" s="17" t="n"/>
+      <c r="K87" s="17">
+        <f>IF(ISNUMBER(J87),J87*F87,"")</f>
+        <v/>
+      </c>
+      <c r="L87" s="23">
+        <f>IF(ISNUMBER(J87),K87-G87,"")</f>
+        <v/>
+      </c>
+      <c r="M87" s="24">
+        <f>IF(ISNUMBER(J87),L87/G87,"")</f>
+        <v/>
+      </c>
+      <c r="N87" s="25">
+        <f>IF(ISNUMBER(H87),H87-C87,"")</f>
+        <v/>
+      </c>
+      <c r="O87" s="6" t="n"/>
+      <c r="P87" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>Occidental Petroleum Corporation</t>
+        </is>
+      </c>
+      <c r="C88" s="22" t="n">
+        <v>46325.60914351852</v>
+      </c>
+      <c r="D88" s="22" t="n">
+        <v>46325.40081018519</v>
+      </c>
+      <c r="E88" s="17" t="n">
+        <v>63.76</v>
+      </c>
+      <c r="F88" s="16" t="n">
+        <v>10.872647427</v>
+      </c>
+      <c r="G88" s="17">
+        <f>E88*F88</f>
+        <v/>
+      </c>
+      <c r="H88" s="22" t="n"/>
+      <c r="I88" s="22" t="n"/>
+      <c r="J88" s="17" t="n"/>
+      <c r="K88" s="17">
+        <f>IF(ISNUMBER(J88),J88*F88,"")</f>
+        <v/>
+      </c>
+      <c r="L88" s="23">
+        <f>IF(ISNUMBER(J88),K88-G88,"")</f>
+        <v/>
+      </c>
+      <c r="M88" s="24">
+        <f>IF(ISNUMBER(J88),L88/G88,"")</f>
+        <v/>
+      </c>
+      <c r="N88" s="25">
+        <f>IF(ISNUMBER(H88),H88-C88,"")</f>
+        <v/>
+      </c>
+      <c r="O88" s="6" t="n"/>
+      <c r="P88" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>Intercontinental Exchange  Inc.</t>
+        </is>
+      </c>
+      <c r="C89" s="22" t="n">
+        <v>46325.60914351852</v>
+      </c>
+      <c r="D89" s="22" t="n">
+        <v>46325.40081018519</v>
+      </c>
+      <c r="E89" s="17" t="n">
+        <v>167.21</v>
+      </c>
+      <c r="F89" s="16" t="n">
+        <v>4.145924286</v>
+      </c>
+      <c r="G89" s="17">
+        <f>E89*F89</f>
+        <v/>
+      </c>
+      <c r="H89" s="22" t="n"/>
+      <c r="I89" s="22" t="n"/>
+      <c r="J89" s="17" t="n"/>
+      <c r="K89" s="17">
+        <f>IF(ISNUMBER(J89),J89*F89,"")</f>
+        <v/>
+      </c>
+      <c r="L89" s="23">
+        <f>IF(ISNUMBER(J89),K89-G89,"")</f>
+        <v/>
+      </c>
+      <c r="M89" s="24">
+        <f>IF(ISNUMBER(J89),L89/G89,"")</f>
+        <v/>
+      </c>
+      <c r="N89" s="25">
+        <f>IF(ISNUMBER(H89),H89-C89,"")</f>
+        <v/>
+      </c>
+      <c r="O89" s="6" t="n"/>
+      <c r="P89" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>Automatic Data Processing, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C90" s="22" t="n">
+        <v>46325.60915509259</v>
+      </c>
+      <c r="D90" s="22" t="n">
+        <v>46325.40082175926</v>
+      </c>
+      <c r="E90" s="17" t="n">
+        <v>293.43</v>
+      </c>
+      <c r="F90" s="16" t="n">
+        <v>2.362539617</v>
+      </c>
+      <c r="G90" s="17">
+        <f>E90*F90</f>
+        <v/>
+      </c>
+      <c r="H90" s="22" t="n"/>
+      <c r="I90" s="22" t="n"/>
+      <c r="J90" s="17" t="n"/>
+      <c r="K90" s="17">
+        <f>IF(ISNUMBER(J90),J90*F90,"")</f>
+        <v/>
+      </c>
+      <c r="L90" s="23">
+        <f>IF(ISNUMBER(J90),K90-G90,"")</f>
+        <v/>
+      </c>
+      <c r="M90" s="24">
+        <f>IF(ISNUMBER(J90),L90/G90,"")</f>
+        <v/>
+      </c>
+      <c r="N90" s="25">
+        <f>IF(ISNUMBER(H90),H90-C90,"")</f>
+        <v/>
+      </c>
+      <c r="O90" s="6" t="n"/>
+      <c r="P90" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>Equinor ASA American Depositary Shares (Each Representing One Ordinary Share, nominal value NOK 2.50 per share)</t>
+        </is>
+      </c>
+      <c r="C91" s="22" t="n">
+        <v>46325.60915509259</v>
+      </c>
+      <c r="D91" s="22" t="n">
+        <v>46325.40082175926</v>
+      </c>
+      <c r="E91" s="17" t="n">
+        <v>48.717028</v>
+      </c>
+      <c r="F91" s="16" t="n">
+        <v>14.229932252</v>
+      </c>
+      <c r="G91" s="17">
+        <f>E91*F91</f>
+        <v/>
+      </c>
+      <c r="H91" s="22" t="n"/>
+      <c r="I91" s="22" t="n"/>
+      <c r="J91" s="17" t="n"/>
+      <c r="K91" s="17">
+        <f>IF(ISNUMBER(J91),J91*F91,"")</f>
+        <v/>
+      </c>
+      <c r="L91" s="23">
+        <f>IF(ISNUMBER(J91),K91-G91,"")</f>
+        <v/>
+      </c>
+      <c r="M91" s="24">
+        <f>IF(ISNUMBER(J91),L91/G91,"")</f>
+        <v/>
+      </c>
+      <c r="N91" s="25">
+        <f>IF(ISNUMBER(H91),H91-C91,"")</f>
+        <v/>
+      </c>
+      <c r="O91" s="6" t="n"/>
+      <c r="P91" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>SharkNinja, Inc.</t>
+        </is>
+      </c>
+      <c r="C92" s="22" t="n">
+        <v>46325.60915509259</v>
+      </c>
+      <c r="D92" s="22" t="n">
+        <v>46325.40082175926</v>
+      </c>
+      <c r="E92" s="17" t="n">
+        <v>209.77</v>
+      </c>
+      <c r="F92" s="16" t="n">
+        <v>3.304762358</v>
+      </c>
+      <c r="G92" s="17">
+        <f>E92*F92</f>
+        <v/>
+      </c>
+      <c r="H92" s="22" t="n"/>
+      <c r="I92" s="22" t="n"/>
+      <c r="J92" s="17" t="n"/>
+      <c r="K92" s="17">
+        <f>IF(ISNUMBER(J92),J92*F92,"")</f>
+        <v/>
+      </c>
+      <c r="L92" s="23">
+        <f>IF(ISNUMBER(J92),K92-G92,"")</f>
+        <v/>
+      </c>
+      <c r="M92" s="24">
+        <f>IF(ISNUMBER(J92),L92/G92,"")</f>
+        <v/>
+      </c>
+      <c r="N92" s="25">
+        <f>IF(ISNUMBER(H92),H92-C92,"")</f>
+        <v/>
+      </c>
+      <c r="O92" s="6" t="n"/>
+      <c r="P92" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>Monster Beverage Corporation</t>
+        </is>
+      </c>
+      <c r="C93" s="22" t="n">
+        <v>46325.60915509259</v>
+      </c>
+      <c r="D93" s="22" t="n">
+        <v>46325.40082175926</v>
+      </c>
+      <c r="E93" s="17" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="F93" s="16" t="n">
+        <v>14.687288135</v>
+      </c>
+      <c r="G93" s="17">
+        <f>E93*F93</f>
+        <v/>
+      </c>
+      <c r="H93" s="22" t="n"/>
+      <c r="I93" s="22" t="n"/>
+      <c r="J93" s="17" t="n"/>
+      <c r="K93" s="17">
+        <f>IF(ISNUMBER(J93),J93*F93,"")</f>
+        <v/>
+      </c>
+      <c r="L93" s="23">
+        <f>IF(ISNUMBER(J93),K93-G93,"")</f>
+        <v/>
+      </c>
+      <c r="M93" s="24">
+        <f>IF(ISNUMBER(J93),L93/G93,"")</f>
+        <v/>
+      </c>
+      <c r="N93" s="25">
+        <f>IF(ISNUMBER(H93),H93-C93,"")</f>
+        <v/>
+      </c>
+      <c r="O93" s="6" t="n"/>
+      <c r="P93" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>CBOE</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>Cboe Global Markets, Inc.</t>
+        </is>
+      </c>
+      <c r="C94" s="22" t="n">
+        <v>46325.60916666667</v>
+      </c>
+      <c r="D94" s="22" t="n">
+        <v>46325.40083333333</v>
+      </c>
+      <c r="E94" s="17" t="n">
+        <v>330.64</v>
+      </c>
+      <c r="F94" s="16" t="n">
+        <v>2.096661021</v>
+      </c>
+      <c r="G94" s="17">
+        <f>E94*F94</f>
+        <v/>
+      </c>
+      <c r="H94" s="22" t="n"/>
+      <c r="I94" s="22" t="n"/>
+      <c r="J94" s="17" t="n"/>
+      <c r="K94" s="17">
+        <f>IF(ISNUMBER(J94),J94*F94,"")</f>
+        <v/>
+      </c>
+      <c r="L94" s="23">
+        <f>IF(ISNUMBER(J94),K94-G94,"")</f>
+        <v/>
+      </c>
+      <c r="M94" s="24">
+        <f>IF(ISNUMBER(J94),L94/G94,"")</f>
+        <v/>
+      </c>
+      <c r="N94" s="25">
+        <f>IF(ISNUMBER(H94),H94-C94,"")</f>
+        <v/>
+      </c>
+      <c r="O94" s="6" t="n"/>
+      <c r="P94" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>Cognizant Technology Solutions Corporation Class A Common Stock</t>
+        </is>
+      </c>
+      <c r="C95" s="22" t="n">
+        <v>46325.60917824074</v>
+      </c>
+      <c r="D95" s="22" t="n">
+        <v>46325.40084490741</v>
+      </c>
+      <c r="E95" s="17" t="n">
+        <v>64.13</v>
+      </c>
+      <c r="F95" s="16" t="n">
+        <v>10.809917355</v>
+      </c>
+      <c r="G95" s="17">
+        <f>E95*F95</f>
+        <v/>
+      </c>
+      <c r="H95" s="22" t="n"/>
+      <c r="I95" s="22" t="n"/>
+      <c r="J95" s="17" t="n"/>
+      <c r="K95" s="17">
+        <f>IF(ISNUMBER(J95),J95*F95,"")</f>
+        <v/>
+      </c>
+      <c r="L95" s="23">
+        <f>IF(ISNUMBER(J95),K95-G95,"")</f>
+        <v/>
+      </c>
+      <c r="M95" s="24">
+        <f>IF(ISNUMBER(J95),L95/G95,"")</f>
+        <v/>
+      </c>
+      <c r="N95" s="25">
+        <f>IF(ISNUMBER(H95),H95-C95,"")</f>
+        <v/>
+      </c>
+      <c r="O95" s="6" t="n"/>
+      <c r="P95" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>Zscaler, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C96" s="22" t="n">
+        <v>46325.60917824074</v>
+      </c>
+      <c r="D96" s="22" t="n">
+        <v>46325.40084490741</v>
+      </c>
+      <c r="E96" s="17" t="n">
+        <v>245.5</v>
+      </c>
+      <c r="F96" s="16" t="n">
+        <v>2.823788187</v>
+      </c>
+      <c r="G96" s="17">
+        <f>E96*F96</f>
+        <v/>
+      </c>
+      <c r="H96" s="22" t="n"/>
+      <c r="I96" s="22" t="n"/>
+      <c r="J96" s="17" t="n"/>
+      <c r="K96" s="17">
+        <f>IF(ISNUMBER(J96),J96*F96,"")</f>
+        <v/>
+      </c>
+      <c r="L96" s="23">
+        <f>IF(ISNUMBER(J96),K96-G96,"")</f>
+        <v/>
+      </c>
+      <c r="M96" s="24">
+        <f>IF(ISNUMBER(J96),L96/G96,"")</f>
+        <v/>
+      </c>
+      <c r="N96" s="25">
+        <f>IF(ISNUMBER(H96),H96-C96,"")</f>
+        <v/>
+      </c>
+      <c r="O96" s="6" t="n"/>
+      <c r="P96" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>The Kroger Co.</t>
+        </is>
+      </c>
+      <c r="C97" s="22" t="n">
+        <v>46325.60918981482</v>
+      </c>
+      <c r="D97" s="22" t="n">
+        <v>46325.40085648148</v>
+      </c>
+      <c r="E97" s="17" t="n">
+        <v>67.65000000000001</v>
+      </c>
+      <c r="F97" s="16" t="n">
+        <v>10.24745011</v>
+      </c>
+      <c r="G97" s="17">
+        <f>E97*F97</f>
+        <v/>
+      </c>
+      <c r="H97" s="22" t="n"/>
+      <c r="I97" s="22" t="n"/>
+      <c r="J97" s="17" t="n"/>
+      <c r="K97" s="17">
+        <f>IF(ISNUMBER(J97),J97*F97,"")</f>
+        <v/>
+      </c>
+      <c r="L97" s="23">
+        <f>IF(ISNUMBER(J97),K97-G97,"")</f>
+        <v/>
+      </c>
+      <c r="M97" s="24">
+        <f>IF(ISNUMBER(J97),L97/G97,"")</f>
+        <v/>
+      </c>
+      <c r="N97" s="25">
+        <f>IF(ISNUMBER(H97),H97-C97,"")</f>
+        <v/>
+      </c>
+      <c r="O97" s="6" t="n"/>
+      <c r="P97" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M74">
+  <conditionalFormatting sqref="L2:M97">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-30 13:43 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA160" headerRowCount="1">
-  <autoFilter ref="A1:BA160"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA165" headerRowCount="1">
+  <autoFilter ref="A1:BA165"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P97" headerRowCount="1">
-  <autoFilter ref="A1:P97"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P101" headerRowCount="1">
+  <autoFilter ref="A1:P101"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.60930555555</v>
+        <v>46325.6135300926</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.40097222223</v>
+        <v>46325.40519675926</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$160,"BUY")+COUNTIF(Orders!$E$2:$E$160,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$165,"BUY")+COUNTIF(Orders!$E$2:$E$165,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$160,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$165,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$160,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$165,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$160,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$165,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$160,Orders!$E$2:$E$160,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$165,Orders!$E$2:$E$165,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$160,Orders!$E$2:$E$160,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$165,Orders!$E$2:$E$165,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$97,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$101,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$97,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$101,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$97)</f>
+        <f>SUM('Round trips'!$L$2:$L$101)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$97,"Closed",'Round trips'!$L$2:$L$97,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$101,"Closed",'Round trips'!$L$2:$L$101,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA160"/>
+  <dimension ref="A1:BA165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -26488,6 +26488,854 @@
       </c>
       <c r="BA160" s="6" t="n"/>
     </row>
+    <row r="161">
+      <c r="A161" s="12" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" s="13" t="n">
+        <v>46325.61028935185</v>
+      </c>
+      <c r="C161" s="13" t="n">
+        <v>46325.40195601852</v>
+      </c>
+      <c r="D161" s="13" t="n">
+        <v>46325.56862268518</v>
+      </c>
+      <c r="E161" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F161" s="6" t="inlineStr">
+        <is>
+          <t>EBAY</t>
+        </is>
+      </c>
+      <c r="G161" s="15" t="n"/>
+      <c r="H161" s="6" t="n"/>
+      <c r="I161" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J161" s="16" t="n">
+        <v>68.49520344</v>
+      </c>
+      <c r="K161" s="17" t="n">
+        <v>120.92</v>
+      </c>
+      <c r="L161" s="17">
+        <f>IF(AND(ISNUMBER(J161),ISNUMBER(K161)),J161*K161,"")</f>
+        <v/>
+      </c>
+      <c r="M161" s="17" t="n"/>
+      <c r="N161" s="16" t="n">
+        <v>68.49520344</v>
+      </c>
+      <c r="O161" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
+      <c r="P161" s="15" t="inlineStr">
+        <is>
+          <t>Alpaca stop order triggered at 121.14 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q161" s="12" t="n"/>
+      <c r="R161" s="6" t="n"/>
+      <c r="S161" s="18" t="n"/>
+      <c r="T161" s="12" t="n"/>
+      <c r="U161" s="19" t="n"/>
+      <c r="V161" s="19" t="n"/>
+      <c r="W161" s="12" t="n"/>
+      <c r="X161" s="6" t="n"/>
+      <c r="Y161" s="19" t="n"/>
+      <c r="Z161" s="6" t="n"/>
+      <c r="AA161" s="12" t="n"/>
+      <c r="AB161" s="15" t="n"/>
+      <c r="AC161" s="6" t="n"/>
+      <c r="AD161" s="6" t="n"/>
+      <c r="AE161" s="17" t="n"/>
+      <c r="AF161" s="17" t="n"/>
+      <c r="AG161" s="17" t="n"/>
+      <c r="AH161" s="20" t="n"/>
+      <c r="AI161" s="18" t="n"/>
+      <c r="AJ161" s="6" t="n"/>
+      <c r="AK161" s="12" t="n"/>
+      <c r="AL161" s="15" t="n"/>
+      <c r="AM161" s="17" t="n"/>
+      <c r="AN161" s="19" t="n"/>
+      <c r="AO161" s="17" t="n"/>
+      <c r="AP161" s="17" t="n"/>
+      <c r="AQ161" s="19" t="n"/>
+      <c r="AR161" s="16" t="n"/>
+      <c r="AS161" s="17" t="n"/>
+      <c r="AT161" s="19" t="n"/>
+      <c r="AU161" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV161" s="6" t="inlineStr">
+        <is>
+          <t>1a7d613e-91b1-48a1-ad9d-10ee85cfb79e</t>
+        </is>
+      </c>
+      <c r="AW161" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-stop-EBAY-1793367435131</t>
+        </is>
+      </c>
+      <c r="AX161" s="13" t="n">
+        <v>46325.56755787037</v>
+      </c>
+      <c r="AY161" s="13" t="n">
+        <v>46325.56862268518</v>
+      </c>
+      <c r="AZ161" s="13" t="n"/>
+      <c r="BA161" s="6" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="12" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" s="13" t="n">
+        <v>46325.61344907407</v>
+      </c>
+      <c r="C162" s="13" t="n">
+        <v>46325.40511574074</v>
+      </c>
+      <c r="D162" s="13" t="n">
+        <v>46325.57178240741</v>
+      </c>
+      <c r="E162" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F162" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="G162" s="15" t="inlineStr">
+        <is>
+          <t>Natera, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H162" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I162" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J162" s="16" t="n">
+        <v>3.215063542</v>
+      </c>
+      <c r="K162" s="17" t="n">
+        <v>428.85</v>
+      </c>
+      <c r="L162" s="17">
+        <f>IF(AND(ISNUMBER(J162),ISNUMBER(K162)),J162*K162,"")</f>
+        <v/>
+      </c>
+      <c r="M162" s="17" t="n">
+        <v>1378.79</v>
+      </c>
+      <c r="N162" s="16" t="n"/>
+      <c r="O162" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P162" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #3, 8.33% of the $16,552.14 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q162" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R162" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S162" s="18" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="T162" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="U162" s="19" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="V162" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W162" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X162" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y162" s="19" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="Z162" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA162" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB162" s="15" t="n"/>
+      <c r="AC162" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD162" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE162" s="17" t="n">
+        <v>439.9452</v>
+      </c>
+      <c r="AF162" s="17" t="n">
+        <v>406.9572</v>
+      </c>
+      <c r="AG162" s="17" t="n">
+        <v>472.9331</v>
+      </c>
+      <c r="AH162" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI162" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ162" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK162" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL162" s="15" t="inlineStr">
+        <is>
+          <t>Natera CEO Steven Leonard Chapman Sells Shares Worth $2.38 Million</t>
+        </is>
+      </c>
+      <c r="AM162" s="17" t="n">
+        <v>426.75</v>
+      </c>
+      <c r="AN162" s="19" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="AO162" s="17" t="n">
+        <v>99363.8</v>
+      </c>
+      <c r="AP162" s="17" t="n">
+        <v>16552.14</v>
+      </c>
+      <c r="AQ162" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR162" s="16" t="n"/>
+      <c r="AS162" s="17" t="n"/>
+      <c r="AT162" s="19" t="n"/>
+      <c r="AU162" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV162" s="6" t="inlineStr">
+        <is>
+          <t>40902560-306e-49ae-90c4-eb2047e0fa0f</t>
+        </is>
+      </c>
+      <c r="AW162" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-NTRA-1793367801313</t>
+        </is>
+      </c>
+      <c r="AX162" s="13" t="n">
+        <v>46325.57177083333</v>
+      </c>
+      <c r="AY162" s="13" t="n">
+        <v>46325.57178240741</v>
+      </c>
+      <c r="AZ162" s="13" t="n">
+        <v>46325.57155092592</v>
+      </c>
+      <c r="BA162" s="6" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="12" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" s="13" t="n">
+        <v>46325.61347222222</v>
+      </c>
+      <c r="C163" s="13" t="n">
+        <v>46325.40513888889</v>
+      </c>
+      <c r="D163" s="13" t="n">
+        <v>46325.57180555556</v>
+      </c>
+      <c r="E163" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F163" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="G163" s="15" t="inlineStr">
+        <is>
+          <t>The Southern Company</t>
+        </is>
+      </c>
+      <c r="H163" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I163" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J163" s="16" t="n">
+        <v>14.649320305</v>
+      </c>
+      <c r="K163" s="17" t="n">
+        <v>94.119043</v>
+      </c>
+      <c r="L163" s="17">
+        <f>IF(AND(ISNUMBER(J163),ISNUMBER(K163)),J163*K163,"")</f>
+        <v/>
+      </c>
+      <c r="M163" s="17" t="n">
+        <v>1378.79</v>
+      </c>
+      <c r="N163" s="16" t="n"/>
+      <c r="O163" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P163" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #4, 8.33% of the $16,552.14 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q163" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R163" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S163" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T163" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="U163" s="19" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="V163" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W163" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X163" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y163" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z163" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA163" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB163" s="15" t="n"/>
+      <c r="AC163" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD163" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE163" s="17" t="n">
+        <v>94.9336</v>
+      </c>
+      <c r="AF163" s="17" t="n">
+        <v>92.64960000000001</v>
+      </c>
+      <c r="AG163" s="17" t="n">
+        <v>97.2176</v>
+      </c>
+      <c r="AH163" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI163" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ163" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK163" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL163" s="15" t="n"/>
+      <c r="AM163" s="17" t="n">
+        <v>94.02</v>
+      </c>
+      <c r="AN163" s="19" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AO163" s="17" t="n">
+        <v>99363.8</v>
+      </c>
+      <c r="AP163" s="17" t="n">
+        <v>16552.14</v>
+      </c>
+      <c r="AQ163" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR163" s="16" t="n"/>
+      <c r="AS163" s="17" t="n"/>
+      <c r="AT163" s="19" t="n"/>
+      <c r="AU163" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV163" s="6" t="inlineStr">
+        <is>
+          <t>5942b9ae-a31c-4788-bf1e-0e0baaf5d8b4</t>
+        </is>
+      </c>
+      <c r="AW163" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-SO-1793367801409</t>
+        </is>
+      </c>
+      <c r="AX163" s="13" t="n">
+        <v>46325.57177083333</v>
+      </c>
+      <c r="AY163" s="13" t="n">
+        <v>46325.57180555556</v>
+      </c>
+      <c r="AZ163" s="13" t="n">
+        <v>46325.57155092592</v>
+      </c>
+      <c r="BA163" s="6" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="12" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" s="13" t="n">
+        <v>46325.61346064815</v>
+      </c>
+      <c r="C164" s="13" t="n">
+        <v>46325.40512731481</v>
+      </c>
+      <c r="D164" s="13" t="n">
+        <v>46325.57179398148</v>
+      </c>
+      <c r="E164" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F164" s="6" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="G164" s="15" t="inlineStr">
+        <is>
+          <t>Altria Group, Inc.</t>
+        </is>
+      </c>
+      <c r="H164" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I164" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J164" s="16" t="n">
+        <v>17.501650165</v>
+      </c>
+      <c r="K164" s="17" t="n">
+        <v>78.78</v>
+      </c>
+      <c r="L164" s="17">
+        <f>IF(AND(ISNUMBER(J164),ISNUMBER(K164)),J164*K164,"")</f>
+        <v/>
+      </c>
+      <c r="M164" s="17" t="n">
+        <v>1378.79</v>
+      </c>
+      <c r="N164" s="16" t="n"/>
+      <c r="O164" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P164" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #6, 8.33% of the $16,552.14 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q164" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R164" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S164" s="18" t="n">
+        <v>0.644</v>
+      </c>
+      <c r="T164" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="U164" s="19" t="n">
+        <v>0.0097</v>
+      </c>
+      <c r="V164" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W164" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="X164" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y164" s="19" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="Z164" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA164" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB164" s="15" t="inlineStr">
+        <is>
+          <t>One day (+5.1%) did 106% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC164" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD164" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE164" s="17" t="n">
+        <v>79.84520000000001</v>
+      </c>
+      <c r="AF164" s="17" t="n">
+        <v>77.0822</v>
+      </c>
+      <c r="AG164" s="17" t="n">
+        <v>82.6082</v>
+      </c>
+      <c r="AH164" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI164" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ164" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK164" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL164" s="15" t="inlineStr">
+        <is>
+          <t>Altria Reports Q3 2026 Results, Raises Full-Year Earnings Guidance, and Expands Share Repurchase Program</t>
+        </is>
+      </c>
+      <c r="AM164" s="17" t="n">
+        <v>78.73999999999999</v>
+      </c>
+      <c r="AN164" s="19" t="n">
+        <v>0.0262</v>
+      </c>
+      <c r="AO164" s="17" t="n">
+        <v>99363.8</v>
+      </c>
+      <c r="AP164" s="17" t="n">
+        <v>16552.14</v>
+      </c>
+      <c r="AQ164" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR164" s="16" t="n"/>
+      <c r="AS164" s="17" t="n"/>
+      <c r="AT164" s="19" t="n"/>
+      <c r="AU164" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV164" s="6" t="inlineStr">
+        <is>
+          <t>1fe138dd-1cb7-4b50-8cd5-29fe5a7ae381</t>
+        </is>
+      </c>
+      <c r="AW164" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MO-1793367801462</t>
+        </is>
+      </c>
+      <c r="AX164" s="13" t="n">
+        <v>46325.57177083333</v>
+      </c>
+      <c r="AY164" s="13" t="n">
+        <v>46325.57179398148</v>
+      </c>
+      <c r="AZ164" s="13" t="n">
+        <v>46325.57155092592</v>
+      </c>
+      <c r="BA164" s="6" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="12" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" s="13" t="n">
+        <v>46325.61344907407</v>
+      </c>
+      <c r="C165" s="13" t="n">
+        <v>46325.40511574074</v>
+      </c>
+      <c r="D165" s="13" t="n">
+        <v>46325.57178240741</v>
+      </c>
+      <c r="E165" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F165" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G165" s="15" t="inlineStr">
+        <is>
+          <t>Dominion Energy, Inc Common Stock</t>
+        </is>
+      </c>
+      <c r="H165" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I165" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J165" s="16" t="n">
+        <v>20.821202053</v>
+      </c>
+      <c r="K165" s="17" t="n">
+        <v>66.22</v>
+      </c>
+      <c r="L165" s="17">
+        <f>IF(AND(ISNUMBER(J165),ISNUMBER(K165)),J165*K165,"")</f>
+        <v/>
+      </c>
+      <c r="M165" s="17" t="n">
+        <v>1378.79</v>
+      </c>
+      <c r="N165" s="16" t="n"/>
+      <c r="O165" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P165" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #7, 8.33% of the $16,552.14 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q165" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R165" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S165" s="18" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="T165" s="12" t="n">
+        <v>46</v>
+      </c>
+      <c r="U165" s="19" t="n">
+        <v>0.0083</v>
+      </c>
+      <c r="V165" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W165" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="X165" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y165" s="19" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="Z165" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA165" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB165" s="15" t="inlineStr">
+        <is>
+          <t>One day (+4.9%) did 128% of the 10-day move. The trend rests on a single jump.</t>
+        </is>
+      </c>
+      <c r="AC165" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD165" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE165" s="17" t="n">
+        <v>66.6319</v>
+      </c>
+      <c r="AF165" s="17" t="n">
+        <v>65.0022</v>
+      </c>
+      <c r="AG165" s="17" t="n">
+        <v>68.2615</v>
+      </c>
+      <c r="AH165" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI165" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ165" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK165" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL165" s="15" t="inlineStr">
+        <is>
+          <t>Dominion Energy Reports Q3 2026 Earnings and Updates Full-Year Guidance</t>
+        </is>
+      </c>
+      <c r="AM165" s="17" t="n">
+        <v>65.98</v>
+      </c>
+      <c r="AN165" s="19" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="AO165" s="17" t="n">
+        <v>99363.8</v>
+      </c>
+      <c r="AP165" s="17" t="n">
+        <v>16552.14</v>
+      </c>
+      <c r="AQ165" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR165" s="16" t="n"/>
+      <c r="AS165" s="17" t="n"/>
+      <c r="AT165" s="19" t="n"/>
+      <c r="AU165" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV165" s="6" t="inlineStr">
+        <is>
+          <t>7e2f1442-f2c8-460f-8f69-9e4275ea5ed3</t>
+        </is>
+      </c>
+      <c r="AW165" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-D-1793367801510</t>
+        </is>
+      </c>
+      <c r="AX165" s="13" t="n">
+        <v>46325.57177083333</v>
+      </c>
+      <c r="AY165" s="13" t="n">
+        <v>46325.57178240741</v>
+      </c>
+      <c r="AZ165" s="13" t="n">
+        <v>46325.57155092592</v>
+      </c>
+      <c r="BA165" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -26503,7 +27351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P97"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -31338,9 +32186,15 @@
         <f>E77*F77</f>
         <v/>
       </c>
-      <c r="H77" s="22" t="n"/>
-      <c r="I77" s="22" t="n"/>
-      <c r="J77" s="17" t="n"/>
+      <c r="H77" s="22" t="n">
+        <v>46325.61028935185</v>
+      </c>
+      <c r="I77" s="22" t="n">
+        <v>46325.40195601852</v>
+      </c>
+      <c r="J77" s="17" t="n">
+        <v>120.92</v>
+      </c>
       <c r="K77" s="17">
         <f>IF(ISNUMBER(J77),J77*F77,"")</f>
         <v/>
@@ -31357,10 +32211,14 @@
         <f>IF(ISNUMBER(H77),H77-C77,"")</f>
         <v/>
       </c>
-      <c r="O77" s="6" t="n"/>
+      <c r="O77" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P77" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -32434,8 +33292,220 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Natera, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C98" s="22" t="n">
+        <v>46325.61344907407</v>
+      </c>
+      <c r="D98" s="22" t="n">
+        <v>46325.40511574074</v>
+      </c>
+      <c r="E98" s="17" t="n">
+        <v>428.85</v>
+      </c>
+      <c r="F98" s="16" t="n">
+        <v>3.215063542</v>
+      </c>
+      <c r="G98" s="17">
+        <f>E98*F98</f>
+        <v/>
+      </c>
+      <c r="H98" s="22" t="n"/>
+      <c r="I98" s="22" t="n"/>
+      <c r="J98" s="17" t="n"/>
+      <c r="K98" s="17">
+        <f>IF(ISNUMBER(J98),J98*F98,"")</f>
+        <v/>
+      </c>
+      <c r="L98" s="23">
+        <f>IF(ISNUMBER(J98),K98-G98,"")</f>
+        <v/>
+      </c>
+      <c r="M98" s="24">
+        <f>IF(ISNUMBER(J98),L98/G98,"")</f>
+        <v/>
+      </c>
+      <c r="N98" s="25">
+        <f>IF(ISNUMBER(H98),H98-C98,"")</f>
+        <v/>
+      </c>
+      <c r="O98" s="6" t="n"/>
+      <c r="P98" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>Dominion Energy, Inc Common Stock</t>
+        </is>
+      </c>
+      <c r="C99" s="22" t="n">
+        <v>46325.61344907407</v>
+      </c>
+      <c r="D99" s="22" t="n">
+        <v>46325.40511574074</v>
+      </c>
+      <c r="E99" s="17" t="n">
+        <v>66.22</v>
+      </c>
+      <c r="F99" s="16" t="n">
+        <v>20.821202053</v>
+      </c>
+      <c r="G99" s="17">
+        <f>E99*F99</f>
+        <v/>
+      </c>
+      <c r="H99" s="22" t="n"/>
+      <c r="I99" s="22" t="n"/>
+      <c r="J99" s="17" t="n"/>
+      <c r="K99" s="17">
+        <f>IF(ISNUMBER(J99),J99*F99,"")</f>
+        <v/>
+      </c>
+      <c r="L99" s="23">
+        <f>IF(ISNUMBER(J99),K99-G99,"")</f>
+        <v/>
+      </c>
+      <c r="M99" s="24">
+        <f>IF(ISNUMBER(J99),L99/G99,"")</f>
+        <v/>
+      </c>
+      <c r="N99" s="25">
+        <f>IF(ISNUMBER(H99),H99-C99,"")</f>
+        <v/>
+      </c>
+      <c r="O99" s="6" t="n"/>
+      <c r="P99" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>Altria Group, Inc.</t>
+        </is>
+      </c>
+      <c r="C100" s="22" t="n">
+        <v>46325.61346064815</v>
+      </c>
+      <c r="D100" s="22" t="n">
+        <v>46325.40512731481</v>
+      </c>
+      <c r="E100" s="17" t="n">
+        <v>78.78</v>
+      </c>
+      <c r="F100" s="16" t="n">
+        <v>17.501650165</v>
+      </c>
+      <c r="G100" s="17">
+        <f>E100*F100</f>
+        <v/>
+      </c>
+      <c r="H100" s="22" t="n"/>
+      <c r="I100" s="22" t="n"/>
+      <c r="J100" s="17" t="n"/>
+      <c r="K100" s="17">
+        <f>IF(ISNUMBER(J100),J100*F100,"")</f>
+        <v/>
+      </c>
+      <c r="L100" s="23">
+        <f>IF(ISNUMBER(J100),K100-G100,"")</f>
+        <v/>
+      </c>
+      <c r="M100" s="24">
+        <f>IF(ISNUMBER(J100),L100/G100,"")</f>
+        <v/>
+      </c>
+      <c r="N100" s="25">
+        <f>IF(ISNUMBER(H100),H100-C100,"")</f>
+        <v/>
+      </c>
+      <c r="O100" s="6" t="n"/>
+      <c r="P100" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>The Southern Company</t>
+        </is>
+      </c>
+      <c r="C101" s="22" t="n">
+        <v>46325.61347222222</v>
+      </c>
+      <c r="D101" s="22" t="n">
+        <v>46325.40513888889</v>
+      </c>
+      <c r="E101" s="17" t="n">
+        <v>94.119043</v>
+      </c>
+      <c r="F101" s="16" t="n">
+        <v>14.649320305</v>
+      </c>
+      <c r="G101" s="17">
+        <f>E101*F101</f>
+        <v/>
+      </c>
+      <c r="H101" s="22" t="n"/>
+      <c r="I101" s="22" t="n"/>
+      <c r="J101" s="17" t="n"/>
+      <c r="K101" s="17">
+        <f>IF(ISNUMBER(J101),J101*F101,"")</f>
+        <v/>
+      </c>
+      <c r="L101" s="23">
+        <f>IF(ISNUMBER(J101),K101-G101,"")</f>
+        <v/>
+      </c>
+      <c r="M101" s="24">
+        <f>IF(ISNUMBER(J101),L101/G101,"")</f>
+        <v/>
+      </c>
+      <c r="N101" s="25">
+        <f>IF(ISNUMBER(H101),H101-C101,"")</f>
+        <v/>
+      </c>
+      <c r="O101" s="6" t="n"/>
+      <c r="P101" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M97">
+  <conditionalFormatting sqref="L2:M101">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-30 13:48 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA165" headerRowCount="1">
-  <autoFilter ref="A1:BA165"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA167" headerRowCount="1">
+  <autoFilter ref="A1:BA167"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P101" headerRowCount="1">
-  <autoFilter ref="A1:P101"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P102" headerRowCount="1">
+  <autoFilter ref="A1:P102"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.6135300926</v>
+        <v>46325.6172337963</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.40519675926</v>
+        <v>46325.40890046296</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$165,"BUY")+COUNTIF(Orders!$E$2:$E$165,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$167,"BUY")+COUNTIF(Orders!$E$2:$E$167,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$165,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$167,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$165,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$167,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$165,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$167,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$165,Orders!$E$2:$E$165,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$167,Orders!$E$2:$E$167,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$165,Orders!$E$2:$E$165,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$167,Orders!$E$2:$E$167,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$101,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$102,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$101,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$102,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$101)</f>
+        <f>SUM('Round trips'!$L$2:$L$102)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$101,"Closed",'Round trips'!$L$2:$L$101,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$102,"Closed",'Round trips'!$L$2:$L$102,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA165"/>
+  <dimension ref="A1:BA167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -27336,6 +27336,374 @@
       </c>
       <c r="BA165" s="6" t="n"/>
     </row>
+    <row r="166">
+      <c r="A166" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" s="13" t="n">
+        <v>46325.61717592592</v>
+      </c>
+      <c r="C166" s="13" t="n">
+        <v>46325.40884259259</v>
+      </c>
+      <c r="D166" s="13" t="n">
+        <v>46325.57550925926</v>
+      </c>
+      <c r="E166" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F166" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="G166" s="15" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="H166" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I166" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J166" s="16" t="n">
+        <v>3.215063542</v>
+      </c>
+      <c r="K166" s="17" t="n">
+        <v>421.1</v>
+      </c>
+      <c r="L166" s="17">
+        <f>IF(AND(ISNUMBER(J166),ISNUMBER(K166)),J166*K166,"")</f>
+        <v/>
+      </c>
+      <c r="M166" s="17" t="n"/>
+      <c r="N166" s="16" t="n">
+        <v>3.215063542</v>
+      </c>
+      <c r="O166" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P166" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 3.1% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q166" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R166" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S166" s="18" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="T166" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="U166" s="19" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="V166" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W166" s="12" t="n"/>
+      <c r="X166" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y166" s="19" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="Z166" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA166" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB166" s="15" t="n"/>
+      <c r="AC166" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD166" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE166" s="17" t="n">
+        <v>435.9801</v>
+      </c>
+      <c r="AF166" s="17" t="n">
+        <v>403.1548</v>
+      </c>
+      <c r="AG166" s="17" t="n">
+        <v>468.8054</v>
+      </c>
+      <c r="AH166" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI166" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ166" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AK166" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL166" s="15" t="inlineStr">
+        <is>
+          <t>Natera CEO Steven Leonard Chapman Sells Shares Worth $2.38 Million</t>
+        </is>
+      </c>
+      <c r="AM166" s="17" t="n">
+        <v>422.85</v>
+      </c>
+      <c r="AN166" s="19" t="n">
+        <v>-0.0302</v>
+      </c>
+      <c r="AO166" s="17" t="n">
+        <v>99252.42</v>
+      </c>
+      <c r="AP166" s="17" t="n">
+        <v>11037.02</v>
+      </c>
+      <c r="AQ166" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR166" s="16" t="n">
+        <v>3.215063542</v>
+      </c>
+      <c r="AS166" s="17" t="n">
+        <v>428.85</v>
+      </c>
+      <c r="AT166" s="19" t="n">
+        <v>-0.0147</v>
+      </c>
+      <c r="AU166" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV166" s="6" t="inlineStr">
+        <is>
+          <t>ac6a8cbc-e6a8-42b8-91e3-d185ec717ce6</t>
+        </is>
+      </c>
+      <c r="AW166" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-NTRA-1793368122275</t>
+        </is>
+      </c>
+      <c r="AX166" s="13" t="n">
+        <v>46325.57548611111</v>
+      </c>
+      <c r="AY166" s="13" t="n">
+        <v>46325.57550925926</v>
+      </c>
+      <c r="AZ166" s="13" t="n">
+        <v>46325.57515046297</v>
+      </c>
+      <c r="BA166" s="6" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="12" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" s="13" t="n">
+        <v>46325.61721064815</v>
+      </c>
+      <c r="C167" s="13" t="n">
+        <v>46325.40887731482</v>
+      </c>
+      <c r="D167" s="13" t="n">
+        <v>46325.57554398148</v>
+      </c>
+      <c r="E167" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F167" s="6" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="G167" s="15" t="inlineStr">
+        <is>
+          <t>Netskope, Inc. Class A Common Stock</t>
+        </is>
+      </c>
+      <c r="H167" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I167" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J167" s="16" t="n">
+        <v>36.050548589</v>
+      </c>
+      <c r="K167" s="17" t="n">
+        <v>25.502247</v>
+      </c>
+      <c r="L167" s="17">
+        <f>IF(AND(ISNUMBER(J167),ISNUMBER(K167)),J167*K167,"")</f>
+        <v/>
+      </c>
+      <c r="M167" s="17" t="n">
+        <v>919.38</v>
+      </c>
+      <c r="N167" s="16" t="n"/>
+      <c r="O167" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P167" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $11,037.02 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q167" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R167" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S167" s="18" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="T167" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="U167" s="19" t="n">
+        <v>0.0316</v>
+      </c>
+      <c r="V167" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W167" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X167" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y167" s="19" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="Z167" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA167" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB167" s="15" t="n"/>
+      <c r="AC167" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD167" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE167" s="17" t="n">
+        <v>26.5923</v>
+      </c>
+      <c r="AF167" s="17" t="n">
+        <v>24.0616</v>
+      </c>
+      <c r="AG167" s="17" t="n">
+        <v>29.123</v>
+      </c>
+      <c r="AH167" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI167" s="18" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AJ167" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK167" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL167" s="15" t="n"/>
+      <c r="AM167" s="17" t="n">
+        <v>25.58</v>
+      </c>
+      <c r="AN167" s="19" t="n">
+        <v>-0.0233</v>
+      </c>
+      <c r="AO167" s="17" t="n">
+        <v>99252.42</v>
+      </c>
+      <c r="AP167" s="17" t="n">
+        <v>11037.02</v>
+      </c>
+      <c r="AQ167" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR167" s="16" t="n"/>
+      <c r="AS167" s="17" t="n"/>
+      <c r="AT167" s="19" t="n"/>
+      <c r="AU167" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV167" s="6" t="inlineStr">
+        <is>
+          <t>ca38c263-e885-4d83-bc75-f4be21270219</t>
+        </is>
+      </c>
+      <c r="AW167" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-NTSK-1793368122524</t>
+        </is>
+      </c>
+      <c r="AX167" s="13" t="n">
+        <v>46325.57548611111</v>
+      </c>
+      <c r="AY167" s="13" t="n">
+        <v>46325.57554398148</v>
+      </c>
+      <c r="AZ167" s="13" t="n">
+        <v>46325.57515046297</v>
+      </c>
+      <c r="BA167" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -27351,7 +27719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:P102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -33319,9 +33687,15 @@
         <f>E98*F98</f>
         <v/>
       </c>
-      <c r="H98" s="22" t="n"/>
-      <c r="I98" s="22" t="n"/>
-      <c r="J98" s="17" t="n"/>
+      <c r="H98" s="22" t="n">
+        <v>46325.61717592592</v>
+      </c>
+      <c r="I98" s="22" t="n">
+        <v>46325.40884259259</v>
+      </c>
+      <c r="J98" s="17" t="n">
+        <v>421.1</v>
+      </c>
       <c r="K98" s="17">
         <f>IF(ISNUMBER(J98),J98*F98,"")</f>
         <v/>
@@ -33338,10 +33712,14 @@
         <f>IF(ISNUMBER(H98),H98-C98,"")</f>
         <v/>
       </c>
-      <c r="O98" s="6" t="n"/>
+      <c r="O98" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P98" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -33504,8 +33882,61 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>Netskope, Inc. Class A Common Stock</t>
+        </is>
+      </c>
+      <c r="C102" s="22" t="n">
+        <v>46325.61721064815</v>
+      </c>
+      <c r="D102" s="22" t="n">
+        <v>46325.40887731482</v>
+      </c>
+      <c r="E102" s="17" t="n">
+        <v>25.502247</v>
+      </c>
+      <c r="F102" s="16" t="n">
+        <v>36.050548589</v>
+      </c>
+      <c r="G102" s="17">
+        <f>E102*F102</f>
+        <v/>
+      </c>
+      <c r="H102" s="22" t="n"/>
+      <c r="I102" s="22" t="n"/>
+      <c r="J102" s="17" t="n"/>
+      <c r="K102" s="17">
+        <f>IF(ISNUMBER(J102),J102*F102,"")</f>
+        <v/>
+      </c>
+      <c r="L102" s="23">
+        <f>IF(ISNUMBER(J102),K102-G102,"")</f>
+        <v/>
+      </c>
+      <c r="M102" s="24">
+        <f>IF(ISNUMBER(J102),L102/G102,"")</f>
+        <v/>
+      </c>
+      <c r="N102" s="25">
+        <f>IF(ISNUMBER(H102),H102-C102,"")</f>
+        <v/>
+      </c>
+      <c r="O102" s="6" t="n"/>
+      <c r="P102" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M101">
+  <conditionalFormatting sqref="L2:M102">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-30 13:54 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA167" headerRowCount="1">
-  <autoFilter ref="A1:BA167"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA170" headerRowCount="1">
+  <autoFilter ref="A1:BA170"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.6172337963</v>
+        <v>46325.62128472222</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.40890046296</v>
+        <v>46325.41295138889</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$167,"BUY")+COUNTIF(Orders!$E$2:$E$167,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$170,"BUY")+COUNTIF(Orders!$E$2:$E$170,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$167,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$170,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$167,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$170,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$167,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$170,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$167,Orders!$E$2:$E$167,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$170,Orders!$E$2:$E$170,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$167,Orders!$E$2:$E$167,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$170,Orders!$E$2:$E$170,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA167"/>
+  <dimension ref="A1:BA170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -27341,13 +27341,13 @@
         <v>165</v>
       </c>
       <c r="B166" s="13" t="n">
-        <v>46325.61717592592</v>
+        <v>46325.62011574074</v>
       </c>
       <c r="C166" s="13" t="n">
-        <v>46325.40884259259</v>
+        <v>46325.41178240741</v>
       </c>
       <c r="D166" s="13" t="n">
-        <v>46325.57550925926</v>
+        <v>46325.57844907408</v>
       </c>
       <c r="E166" s="21" t="inlineStr">
         <is>
@@ -27356,29 +27356,21 @@
       </c>
       <c r="F166" s="6" t="inlineStr">
         <is>
-          <t>NTRA</t>
-        </is>
-      </c>
-      <c r="G166" s="15" t="inlineStr">
-        <is>
-          <t>NTRA</t>
-        </is>
-      </c>
-      <c r="H166" s="6" t="inlineStr">
-        <is>
-          <t>NASDAQ</t>
-        </is>
-      </c>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="G166" s="15" t="n"/>
+      <c r="H166" s="6" t="n"/>
       <c r="I166" s="6" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
       <c r="J166" s="16" t="n">
-        <v>3.215063542</v>
+        <v>10.809917355</v>
       </c>
       <c r="K166" s="17" t="n">
-        <v>421.1</v>
+        <v>64.54000000000001</v>
       </c>
       <c r="L166" s="17">
         <f>IF(AND(ISNUMBER(J166),ISNUMBER(K166)),J166*K166,"")</f>
@@ -27386,118 +27378,48 @@
       </c>
       <c r="M166" s="17" t="n"/>
       <c r="N166" s="16" t="n">
-        <v>3.215063542</v>
+        <v>10.809917355</v>
       </c>
       <c r="O166" s="6" t="inlineStr">
         <is>
-          <t>bad day</t>
+          <t>stop-loss (Alpaca order)</t>
         </is>
       </c>
       <c r="P166" s="15" t="inlineStr">
         <is>
-          <t>Bad day: down 3.1% today and only 4 of 5 green</t>
-        </is>
-      </c>
-      <c r="Q166" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="R166" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="S166" s="18" t="n">
-        <v>0.701</v>
-      </c>
-      <c r="T166" s="12" t="n">
-        <v>67</v>
-      </c>
-      <c r="U166" s="19" t="n">
-        <v>0.0292</v>
-      </c>
-      <c r="V166" s="19" t="n">
-        <v>0.2893</v>
-      </c>
+          <t>Alpaca stop order triggered at 64.6 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q166" s="12" t="n"/>
+      <c r="R166" s="6" t="n"/>
+      <c r="S166" s="18" t="n"/>
+      <c r="T166" s="12" t="n"/>
+      <c r="U166" s="19" t="n"/>
+      <c r="V166" s="19" t="n"/>
       <c r="W166" s="12" t="n"/>
-      <c r="X166" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y166" s="19" t="n">
-        <v>0.0007000000000000001</v>
-      </c>
-      <c r="Z166" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AA166" s="12" t="n">
-        <v>100</v>
-      </c>
+      <c r="X166" s="6" t="n"/>
+      <c r="Y166" s="19" t="n"/>
+      <c r="Z166" s="6" t="n"/>
+      <c r="AA166" s="12" t="n"/>
       <c r="AB166" s="15" t="n"/>
-      <c r="AC166" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AD166" s="6" t="inlineStr">
-        <is>
-          <t>up</t>
-        </is>
-      </c>
-      <c r="AE166" s="17" t="n">
-        <v>435.9801</v>
-      </c>
-      <c r="AF166" s="17" t="n">
-        <v>403.1548</v>
-      </c>
-      <c r="AG166" s="17" t="n">
-        <v>468.8054</v>
-      </c>
-      <c r="AH166" s="20" t="n">
-        <v>46332</v>
-      </c>
-      <c r="AI166" s="18" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="AJ166" s="6" t="inlineStr">
-        <is>
-          <t>alert</t>
-        </is>
-      </c>
-      <c r="AK166" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL166" s="15" t="inlineStr">
-        <is>
-          <t>Natera CEO Steven Leonard Chapman Sells Shares Worth $2.38 Million</t>
-        </is>
-      </c>
-      <c r="AM166" s="17" t="n">
-        <v>422.85</v>
-      </c>
-      <c r="AN166" s="19" t="n">
-        <v>-0.0302</v>
-      </c>
-      <c r="AO166" s="17" t="n">
-        <v>99252.42</v>
-      </c>
-      <c r="AP166" s="17" t="n">
-        <v>11037.02</v>
-      </c>
-      <c r="AQ166" s="19" t="n">
-        <v>0.0833</v>
-      </c>
-      <c r="AR166" s="16" t="n">
-        <v>3.215063542</v>
-      </c>
-      <c r="AS166" s="17" t="n">
-        <v>428.85</v>
-      </c>
-      <c r="AT166" s="19" t="n">
-        <v>-0.0147</v>
-      </c>
+      <c r="AC166" s="6" t="n"/>
+      <c r="AD166" s="6" t="n"/>
+      <c r="AE166" s="17" t="n"/>
+      <c r="AF166" s="17" t="n"/>
+      <c r="AG166" s="17" t="n"/>
+      <c r="AH166" s="20" t="n"/>
+      <c r="AI166" s="18" t="n"/>
+      <c r="AJ166" s="6" t="n"/>
+      <c r="AK166" s="12" t="n"/>
+      <c r="AL166" s="15" t="n"/>
+      <c r="AM166" s="17" t="n"/>
+      <c r="AN166" s="19" t="n"/>
+      <c r="AO166" s="17" t="n"/>
+      <c r="AP166" s="17" t="n"/>
+      <c r="AQ166" s="19" t="n"/>
+      <c r="AR166" s="16" t="n"/>
+      <c r="AS166" s="17" t="n"/>
+      <c r="AT166" s="19" t="n"/>
       <c r="AU166" s="6" t="inlineStr">
         <is>
           <t>paper</t>
@@ -27505,23 +27427,21 @@
       </c>
       <c r="AV166" s="6" t="inlineStr">
         <is>
-          <t>ac6a8cbc-e6a8-42b8-91e3-d185ec717ce6</t>
+          <t>1ed4d5c6-13bc-4722-92dd-a9fe2f2cf5eb</t>
         </is>
       </c>
       <c r="AW166" s="6" t="inlineStr">
         <is>
-          <t>tdagent-sell-NTRA-1793368122275</t>
+          <t>tdagent-stop-CTSH-1793367804635</t>
         </is>
       </c>
       <c r="AX166" s="13" t="n">
-        <v>46325.57548611111</v>
+        <v>46325.57180555556</v>
       </c>
       <c r="AY166" s="13" t="n">
-        <v>46325.57550925926</v>
-      </c>
-      <c r="AZ166" s="13" t="n">
-        <v>46325.57515046297</v>
-      </c>
+        <v>46325.57844907408</v>
+      </c>
+      <c r="AZ166" s="13" t="n"/>
       <c r="BA166" s="6" t="n"/>
     </row>
     <row r="167">
@@ -27529,152 +27449,82 @@
         <v>166</v>
       </c>
       <c r="B167" s="13" t="n">
-        <v>46325.61721064815</v>
+        <v>46325.61847222222</v>
       </c>
       <c r="C167" s="13" t="n">
-        <v>46325.40887731482</v>
+        <v>46325.41013888889</v>
       </c>
       <c r="D167" s="13" t="n">
-        <v>46325.57554398148</v>
-      </c>
-      <c r="E167" s="14" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>46325.57680555555</v>
+      </c>
+      <c r="E167" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F167" s="6" t="inlineStr">
         <is>
-          <t>NTSK</t>
-        </is>
-      </c>
-      <c r="G167" s="15" t="inlineStr">
-        <is>
-          <t>Netskope, Inc. Class A Common Stock</t>
-        </is>
-      </c>
-      <c r="H167" s="6" t="inlineStr">
-        <is>
-          <t>NASDAQ</t>
-        </is>
-      </c>
+          <t>CBOE</t>
+        </is>
+      </c>
+      <c r="G167" s="15" t="n"/>
+      <c r="H167" s="6" t="n"/>
       <c r="I167" s="6" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
       <c r="J167" s="16" t="n">
-        <v>36.050548589</v>
+        <v>2.096661021</v>
       </c>
       <c r="K167" s="17" t="n">
-        <v>25.502247</v>
+        <v>331.63</v>
       </c>
       <c r="L167" s="17">
         <f>IF(AND(ISNUMBER(J167),ISNUMBER(K167)),J167*K167,"")</f>
         <v/>
       </c>
-      <c r="M167" s="17" t="n">
-        <v>919.38</v>
-      </c>
-      <c r="N167" s="16" t="n"/>
+      <c r="M167" s="17" t="n"/>
+      <c r="N167" s="16" t="n">
+        <v>2.096661021</v>
+      </c>
       <c r="O167" s="6" t="inlineStr">
         <is>
-          <t>4+/5 green</t>
+          <t>stop-loss (Alpaca order)</t>
         </is>
       </c>
       <c r="P167" s="15" t="inlineStr">
         <is>
-          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $11,037.02 free cash split 12 ways</t>
-        </is>
-      </c>
-      <c r="Q167" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="R167" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="S167" s="18" t="n">
-        <v>0.643</v>
-      </c>
-      <c r="T167" s="12" t="n">
-        <v>42</v>
-      </c>
-      <c r="U167" s="19" t="n">
-        <v>0.0316</v>
-      </c>
-      <c r="V167" s="19" t="n">
-        <v>0.2893</v>
-      </c>
-      <c r="W167" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="X167" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y167" s="19" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="Z167" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AA167" s="12" t="n">
-        <v>100</v>
-      </c>
+          <t>Alpaca stop order triggered at 332.16 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q167" s="12" t="n"/>
+      <c r="R167" s="6" t="n"/>
+      <c r="S167" s="18" t="n"/>
+      <c r="T167" s="12" t="n"/>
+      <c r="U167" s="19" t="n"/>
+      <c r="V167" s="19" t="n"/>
+      <c r="W167" s="12" t="n"/>
+      <c r="X167" s="6" t="n"/>
+      <c r="Y167" s="19" t="n"/>
+      <c r="Z167" s="6" t="n"/>
+      <c r="AA167" s="12" t="n"/>
       <c r="AB167" s="15" t="n"/>
-      <c r="AC167" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AD167" s="6" t="inlineStr">
-        <is>
-          <t>up</t>
-        </is>
-      </c>
-      <c r="AE167" s="17" t="n">
-        <v>26.5923</v>
-      </c>
-      <c r="AF167" s="17" t="n">
-        <v>24.0616</v>
-      </c>
-      <c r="AG167" s="17" t="n">
-        <v>29.123</v>
-      </c>
-      <c r="AH167" s="20" t="n">
-        <v>46332</v>
-      </c>
-      <c r="AI167" s="18" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="AJ167" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AK167" s="12" t="n">
-        <v>0</v>
-      </c>
+      <c r="AC167" s="6" t="n"/>
+      <c r="AD167" s="6" t="n"/>
+      <c r="AE167" s="17" t="n"/>
+      <c r="AF167" s="17" t="n"/>
+      <c r="AG167" s="17" t="n"/>
+      <c r="AH167" s="20" t="n"/>
+      <c r="AI167" s="18" t="n"/>
+      <c r="AJ167" s="6" t="n"/>
+      <c r="AK167" s="12" t="n"/>
       <c r="AL167" s="15" t="n"/>
-      <c r="AM167" s="17" t="n">
-        <v>25.58</v>
-      </c>
-      <c r="AN167" s="19" t="n">
-        <v>-0.0233</v>
-      </c>
-      <c r="AO167" s="17" t="n">
-        <v>99252.42</v>
-      </c>
-      <c r="AP167" s="17" t="n">
-        <v>11037.02</v>
-      </c>
-      <c r="AQ167" s="19" t="n">
-        <v>0.0833</v>
-      </c>
+      <c r="AM167" s="17" t="n"/>
+      <c r="AN167" s="19" t="n"/>
+      <c r="AO167" s="17" t="n"/>
+      <c r="AP167" s="17" t="n"/>
+      <c r="AQ167" s="19" t="n"/>
       <c r="AR167" s="16" t="n"/>
       <c r="AS167" s="17" t="n"/>
       <c r="AT167" s="19" t="n"/>
@@ -27685,24 +27535,578 @@
       </c>
       <c r="AV167" s="6" t="inlineStr">
         <is>
+          <t>c460c6de-6c52-49a0-b1fb-549025e69b46</t>
+        </is>
+      </c>
+      <c r="AW167" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-stop-CBOE-1793368021815</t>
+        </is>
+      </c>
+      <c r="AX167" s="13" t="n">
+        <v>46325.5743287037</v>
+      </c>
+      <c r="AY167" s="13" t="n">
+        <v>46325.57680555555</v>
+      </c>
+      <c r="AZ167" s="13" t="n"/>
+      <c r="BA167" s="6" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="12" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" s="13" t="n">
+        <v>46325.61717592592</v>
+      </c>
+      <c r="C168" s="13" t="n">
+        <v>46325.40884259259</v>
+      </c>
+      <c r="D168" s="13" t="n">
+        <v>46325.57550925926</v>
+      </c>
+      <c r="E168" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F168" s="6" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="G168" s="15" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="H168" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I168" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J168" s="16" t="n">
+        <v>3.215063542</v>
+      </c>
+      <c r="K168" s="17" t="n">
+        <v>421.1</v>
+      </c>
+      <c r="L168" s="17">
+        <f>IF(AND(ISNUMBER(J168),ISNUMBER(K168)),J168*K168,"")</f>
+        <v/>
+      </c>
+      <c r="M168" s="17" t="n"/>
+      <c r="N168" s="16" t="n">
+        <v>3.215063542</v>
+      </c>
+      <c r="O168" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P168" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 3.1% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q168" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R168" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S168" s="18" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="T168" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="U168" s="19" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="V168" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W168" s="12" t="n"/>
+      <c r="X168" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y168" s="19" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
+      <c r="Z168" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA168" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB168" s="15" t="n"/>
+      <c r="AC168" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD168" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE168" s="17" t="n">
+        <v>435.9801</v>
+      </c>
+      <c r="AF168" s="17" t="n">
+        <v>403.1548</v>
+      </c>
+      <c r="AG168" s="17" t="n">
+        <v>468.8054</v>
+      </c>
+      <c r="AH168" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI168" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ168" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AK168" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL168" s="15" t="inlineStr">
+        <is>
+          <t>Natera CEO Steven Leonard Chapman Sells Shares Worth $2.38 Million</t>
+        </is>
+      </c>
+      <c r="AM168" s="17" t="n">
+        <v>422.85</v>
+      </c>
+      <c r="AN168" s="19" t="n">
+        <v>-0.0302</v>
+      </c>
+      <c r="AO168" s="17" t="n">
+        <v>99252.42</v>
+      </c>
+      <c r="AP168" s="17" t="n">
+        <v>11037.02</v>
+      </c>
+      <c r="AQ168" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR168" s="16" t="n">
+        <v>3.215063542</v>
+      </c>
+      <c r="AS168" s="17" t="n">
+        <v>428.85</v>
+      </c>
+      <c r="AT168" s="19" t="n">
+        <v>-0.0147</v>
+      </c>
+      <c r="AU168" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV168" s="6" t="inlineStr">
+        <is>
+          <t>ac6a8cbc-e6a8-42b8-91e3-d185ec717ce6</t>
+        </is>
+      </c>
+      <c r="AW168" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-NTRA-1793368122275</t>
+        </is>
+      </c>
+      <c r="AX168" s="13" t="n">
+        <v>46325.57548611111</v>
+      </c>
+      <c r="AY168" s="13" t="n">
+        <v>46325.57550925926</v>
+      </c>
+      <c r="AZ168" s="13" t="n">
+        <v>46325.57515046297</v>
+      </c>
+      <c r="BA168" s="6" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="12" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" s="13" t="n">
+        <v>46325.61721064815</v>
+      </c>
+      <c r="C169" s="13" t="n">
+        <v>46325.40887731482</v>
+      </c>
+      <c r="D169" s="13" t="n">
+        <v>46325.57554398148</v>
+      </c>
+      <c r="E169" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F169" s="6" t="inlineStr">
+        <is>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="G169" s="15" t="inlineStr">
+        <is>
+          <t>Netskope, Inc. Class A Common Stock</t>
+        </is>
+      </c>
+      <c r="H169" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I169" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J169" s="16" t="n">
+        <v>36.050548589</v>
+      </c>
+      <c r="K169" s="17" t="n">
+        <v>25.502247</v>
+      </c>
+      <c r="L169" s="17">
+        <f>IF(AND(ISNUMBER(J169),ISNUMBER(K169)),J169*K169,"")</f>
+        <v/>
+      </c>
+      <c r="M169" s="17" t="n">
+        <v>919.38</v>
+      </c>
+      <c r="N169" s="16" t="n"/>
+      <c r="O169" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P169" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $11,037.02 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q169" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R169" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S169" s="18" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="T169" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="U169" s="19" t="n">
+        <v>0.0316</v>
+      </c>
+      <c r="V169" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W169" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X169" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y169" s="19" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="Z169" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA169" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB169" s="15" t="n"/>
+      <c r="AC169" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD169" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE169" s="17" t="n">
+        <v>26.5923</v>
+      </c>
+      <c r="AF169" s="17" t="n">
+        <v>24.0616</v>
+      </c>
+      <c r="AG169" s="17" t="n">
+        <v>29.123</v>
+      </c>
+      <c r="AH169" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI169" s="18" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AJ169" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK169" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL169" s="15" t="n"/>
+      <c r="AM169" s="17" t="n">
+        <v>25.58</v>
+      </c>
+      <c r="AN169" s="19" t="n">
+        <v>-0.0233</v>
+      </c>
+      <c r="AO169" s="17" t="n">
+        <v>99252.42</v>
+      </c>
+      <c r="AP169" s="17" t="n">
+        <v>11037.02</v>
+      </c>
+      <c r="AQ169" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR169" s="16" t="n"/>
+      <c r="AS169" s="17" t="n"/>
+      <c r="AT169" s="19" t="n"/>
+      <c r="AU169" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV169" s="6" t="inlineStr">
+        <is>
           <t>ca38c263-e885-4d83-bc75-f4be21270219</t>
         </is>
       </c>
-      <c r="AW167" s="6" t="inlineStr">
+      <c r="AW169" s="6" t="inlineStr">
         <is>
           <t>tdagent-buy-NTSK-1793368122524</t>
         </is>
       </c>
-      <c r="AX167" s="13" t="n">
+      <c r="AX169" s="13" t="n">
         <v>46325.57548611111</v>
       </c>
-      <c r="AY167" s="13" t="n">
+      <c r="AY169" s="13" t="n">
         <v>46325.57554398148</v>
       </c>
-      <c r="AZ167" s="13" t="n">
+      <c r="AZ169" s="13" t="n">
         <v>46325.57515046297</v>
       </c>
-      <c r="BA167" s="6" t="n"/>
+      <c r="BA169" s="6" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="12" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" s="13" t="n">
+        <v>46325.6212037037</v>
+      </c>
+      <c r="C170" s="13" t="n">
+        <v>46325.41287037037</v>
+      </c>
+      <c r="D170" s="13" t="n">
+        <v>46325.57953703704</v>
+      </c>
+      <c r="E170" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F170" s="6" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="G170" s="15" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="H170" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I170" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J170" s="16" t="n">
+        <v>506</v>
+      </c>
+      <c r="K170" s="17" t="n">
+        <v>16.09581</v>
+      </c>
+      <c r="L170" s="17">
+        <f>IF(AND(ISNUMBER(J170),ISNUMBER(K170)),J170*K170,"")</f>
+        <v/>
+      </c>
+      <c r="M170" s="17" t="n"/>
+      <c r="N170" s="16" t="n">
+        <v>506</v>
+      </c>
+      <c r="O170" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P170" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 3.6% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q170" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R170" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S170" s="18" t="n">
+        <v>0.823</v>
+      </c>
+      <c r="T170" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="U170" s="19" t="n">
+        <v>0.0453</v>
+      </c>
+      <c r="V170" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W170" s="12" t="n"/>
+      <c r="X170" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y170" s="19" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Z170" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA170" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB170" s="15" t="n"/>
+      <c r="AC170" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD170" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE170" s="17" t="n">
+        <v>16.4138</v>
+      </c>
+      <c r="AF170" s="17" t="n">
+        <v>15.7543</v>
+      </c>
+      <c r="AG170" s="17" t="n">
+        <v>17.0734</v>
+      </c>
+      <c r="AH170" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI170" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ170" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AK170" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL170" s="15" t="inlineStr">
+        <is>
+          <t>Avantor Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM170" s="17" t="n">
+        <v>16.155</v>
+      </c>
+      <c r="AN170" s="19" t="n">
+        <v>-0.0315</v>
+      </c>
+      <c r="AO170" s="17" t="n">
+        <v>99175.84</v>
+      </c>
+      <c r="AP170" s="17" t="n">
+        <v>12864.5</v>
+      </c>
+      <c r="AQ170" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR170" s="16" t="n">
+        <v>506</v>
+      </c>
+      <c r="AS170" s="17" t="n">
+        <v>16.368458</v>
+      </c>
+      <c r="AT170" s="19" t="n">
+        <v>-0.0176</v>
+      </c>
+      <c r="AU170" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV170" s="6" t="inlineStr">
+        <is>
+          <t>5a2aff3f-e025-4347-b4bc-5b807d79a3dd</t>
+        </is>
+      </c>
+      <c r="AW170" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-AVTR-1793368471561</t>
+        </is>
+      </c>
+      <c r="AX170" s="13" t="n">
+        <v>46325.57952546296</v>
+      </c>
+      <c r="AY170" s="13" t="n">
+        <v>46325.57953703704</v>
+      </c>
+      <c r="AZ170" s="13" t="n">
+        <v>46325.57931712963</v>
+      </c>
+      <c r="BA170" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -32892,9 +33296,15 @@
         <f>E83*F83</f>
         <v/>
       </c>
-      <c r="H83" s="22" t="n"/>
-      <c r="I83" s="22" t="n"/>
-      <c r="J83" s="17" t="n"/>
+      <c r="H83" s="22" t="n">
+        <v>46325.6212037037</v>
+      </c>
+      <c r="I83" s="22" t="n">
+        <v>46325.41287037037</v>
+      </c>
+      <c r="J83" s="17" t="n">
+        <v>16.09581</v>
+      </c>
       <c r="K83" s="17">
         <f>IF(ISNUMBER(J83),J83*F83,"")</f>
         <v/>
@@ -32911,10 +33321,14 @@
         <f>IF(ISNUMBER(H83),H83-C83,"")</f>
         <v/>
       </c>
-      <c r="O83" s="6" t="n"/>
+      <c r="O83" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P83" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -33475,9 +33889,15 @@
         <f>E94*F94</f>
         <v/>
       </c>
-      <c r="H94" s="22" t="n"/>
-      <c r="I94" s="22" t="n"/>
-      <c r="J94" s="17" t="n"/>
+      <c r="H94" s="22" t="n">
+        <v>46325.61847222222</v>
+      </c>
+      <c r="I94" s="22" t="n">
+        <v>46325.41013888889</v>
+      </c>
+      <c r="J94" s="17" t="n">
+        <v>331.63</v>
+      </c>
       <c r="K94" s="17">
         <f>IF(ISNUMBER(J94),J94*F94,"")</f>
         <v/>
@@ -33494,10 +33914,14 @@
         <f>IF(ISNUMBER(H94),H94-C94,"")</f>
         <v/>
       </c>
-      <c r="O94" s="6" t="n"/>
+      <c r="O94" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P94" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -33528,9 +33952,15 @@
         <f>E95*F95</f>
         <v/>
       </c>
-      <c r="H95" s="22" t="n"/>
-      <c r="I95" s="22" t="n"/>
-      <c r="J95" s="17" t="n"/>
+      <c r="H95" s="22" t="n">
+        <v>46325.62011574074</v>
+      </c>
+      <c r="I95" s="22" t="n">
+        <v>46325.41178240741</v>
+      </c>
+      <c r="J95" s="17" t="n">
+        <v>64.54000000000001</v>
+      </c>
       <c r="K95" s="17">
         <f>IF(ISNUMBER(J95),J95*F95,"")</f>
         <v/>
@@ -33547,10 +33977,14 @@
         <f>IF(ISNUMBER(H95),H95-C95,"")</f>
         <v/>
       </c>
-      <c r="O95" s="6" t="n"/>
+      <c r="O95" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P95" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-30 14:01 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA170" headerRowCount="1">
-  <autoFilter ref="A1:BA170"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA171" headerRowCount="1">
+  <autoFilter ref="A1:BA171"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P102" headerRowCount="1">
-  <autoFilter ref="A1:P102"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P103" headerRowCount="1">
+  <autoFilter ref="A1:P103"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.62128472222</v>
+        <v>46325.62583333333</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.41295138889</v>
+        <v>46325.4175</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$170,"BUY")+COUNTIF(Orders!$E$2:$E$170,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$171,"BUY")+COUNTIF(Orders!$E$2:$E$171,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$170,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$171,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$170,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$171,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$170,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$171,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$170,Orders!$E$2:$E$170,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$171,Orders!$E$2:$E$171,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$170,Orders!$E$2:$E$170,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$171,Orders!$E$2:$E$171,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$102,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$103,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$102,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$103,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$102)</f>
+        <f>SUM('Round trips'!$L$2:$L$103)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$102,"Closed",'Round trips'!$L$2:$L$102,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$103,"Closed",'Round trips'!$L$2:$L$103,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA170"/>
+  <dimension ref="A1:BA171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -28108,6 +28108,190 @@
       </c>
       <c r="BA170" s="6" t="n"/>
     </row>
+    <row r="171">
+      <c r="A171" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" s="13" t="n">
+        <v>46325.62579861111</v>
+      </c>
+      <c r="C171" s="13" t="n">
+        <v>46325.41746527778</v>
+      </c>
+      <c r="D171" s="13" t="n">
+        <v>46325.58413194444</v>
+      </c>
+      <c r="E171" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F171" s="6" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="G171" s="15" t="inlineStr">
+        <is>
+          <t>Tenable Holdings, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H171" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I171" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J171" s="16" t="n">
+        <v>34.46297755</v>
+      </c>
+      <c r="K171" s="17" t="n">
+        <v>50.78</v>
+      </c>
+      <c r="L171" s="17">
+        <f>IF(AND(ISNUMBER(J171),ISNUMBER(K171)),J171*K171,"")</f>
+        <v/>
+      </c>
+      <c r="M171" s="17" t="n">
+        <v>1750.04</v>
+      </c>
+      <c r="N171" s="16" t="n"/>
+      <c r="O171" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P171" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #4, 8.33% of the $21,008.98 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q171" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R171" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S171" s="18" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="T171" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="U171" s="19" t="n">
+        <v>0.0703</v>
+      </c>
+      <c r="V171" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W171" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X171" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y171" s="19" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="Z171" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA171" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB171" s="15" t="n"/>
+      <c r="AC171" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD171" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE171" s="17" t="n">
+        <v>52.721</v>
+      </c>
+      <c r="AF171" s="17" t="n">
+        <v>47.506</v>
+      </c>
+      <c r="AG171" s="17" t="n">
+        <v>57.9361</v>
+      </c>
+      <c r="AH171" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI171" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ171" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK171" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL171" s="15" t="inlineStr">
+        <is>
+          <t>Canaccord Genuity Maintains Buy on Tenable Holdings, Raises Price Target to $54</t>
+        </is>
+      </c>
+      <c r="AM171" s="17" t="n">
+        <v>50.83</v>
+      </c>
+      <c r="AN171" s="19" t="n">
+        <v>-0.0219</v>
+      </c>
+      <c r="AO171" s="17" t="n">
+        <v>99162.94</v>
+      </c>
+      <c r="AP171" s="17" t="n">
+        <v>21008.98</v>
+      </c>
+      <c r="AQ171" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR171" s="16" t="n"/>
+      <c r="AS171" s="17" t="n"/>
+      <c r="AT171" s="19" t="n"/>
+      <c r="AU171" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV171" s="6" t="inlineStr">
+        <is>
+          <t>df26cb82-ab44-4a98-98a5-5d4ad6ebca75</t>
+        </is>
+      </c>
+      <c r="AW171" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-TENB-1793368866439</t>
+        </is>
+      </c>
+      <c r="AX171" s="13" t="n">
+        <v>46325.58409722222</v>
+      </c>
+      <c r="AY171" s="13" t="n">
+        <v>46325.58413194444</v>
+      </c>
+      <c r="AZ171" s="13" t="n">
+        <v>46325.58353009259</v>
+      </c>
+      <c r="BA171" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -28123,7 +28307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P102"/>
+  <dimension ref="A1:P103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -34369,8 +34553,61 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>Tenable Holdings, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C103" s="22" t="n">
+        <v>46325.62579861111</v>
+      </c>
+      <c r="D103" s="22" t="n">
+        <v>46325.41746527778</v>
+      </c>
+      <c r="E103" s="17" t="n">
+        <v>50.78</v>
+      </c>
+      <c r="F103" s="16" t="n">
+        <v>34.46297755</v>
+      </c>
+      <c r="G103" s="17">
+        <f>E103*F103</f>
+        <v/>
+      </c>
+      <c r="H103" s="22" t="n"/>
+      <c r="I103" s="22" t="n"/>
+      <c r="J103" s="17" t="n"/>
+      <c r="K103" s="17">
+        <f>IF(ISNUMBER(J103),J103*F103,"")</f>
+        <v/>
+      </c>
+      <c r="L103" s="23">
+        <f>IF(ISNUMBER(J103),K103-G103,"")</f>
+        <v/>
+      </c>
+      <c r="M103" s="24">
+        <f>IF(ISNUMBER(J103),L103/G103,"")</f>
+        <v/>
+      </c>
+      <c r="N103" s="25">
+        <f>IF(ISNUMBER(H103),H103-C103,"")</f>
+        <v/>
+      </c>
+      <c r="O103" s="6" t="n"/>
+      <c r="P103" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M102">
+  <conditionalFormatting sqref="L2:M103">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-30 14:07 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA171" headerRowCount="1">
-  <autoFilter ref="A1:BA171"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA172" headerRowCount="1">
+  <autoFilter ref="A1:BA172"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P103" headerRowCount="1">
-  <autoFilter ref="A1:P103"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P104" headerRowCount="1">
+  <autoFilter ref="A1:P104"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.62583333333</v>
+        <v>46325.6299074074</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.4175</v>
+        <v>46325.42157407408</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$171,"BUY")+COUNTIF(Orders!$E$2:$E$171,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$172,"BUY")+COUNTIF(Orders!$E$2:$E$172,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$171,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$172,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$171,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$172,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$171,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$172,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$171,Orders!$E$2:$E$171,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$172,Orders!$E$2:$E$172,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$171,Orders!$E$2:$E$171,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$172,Orders!$E$2:$E$172,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$103,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$104,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$103,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$104,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$103)</f>
+        <f>SUM('Round trips'!$L$2:$L$104)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$103,"Closed",'Round trips'!$L$2:$L$103,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$104,"Closed",'Round trips'!$L$2:$L$104,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA171"/>
+  <dimension ref="A1:BA172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -28292,6 +28292,190 @@
       </c>
       <c r="BA171" s="6" t="n"/>
     </row>
+    <row r="172">
+      <c r="A172" s="12" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" s="13" t="n">
+        <v>46325.62979166667</v>
+      </c>
+      <c r="C172" s="13" t="n">
+        <v>46325.42145833333</v>
+      </c>
+      <c r="D172" s="13" t="n">
+        <v>46325.588125</v>
+      </c>
+      <c r="E172" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F172" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="G172" s="15" t="inlineStr">
+        <is>
+          <t>Dynatrace, Inc.</t>
+        </is>
+      </c>
+      <c r="H172" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I172" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J172" s="16" t="n">
+        <v>27.311201906</v>
+      </c>
+      <c r="K172" s="17" t="n">
+        <v>58.74</v>
+      </c>
+      <c r="L172" s="17">
+        <f>IF(AND(ISNUMBER(J172),ISNUMBER(K172)),J172*K172,"")</f>
+        <v/>
+      </c>
+      <c r="M172" s="17" t="n">
+        <v>1604.27</v>
+      </c>
+      <c r="N172" s="16" t="n"/>
+      <c r="O172" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P172" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $19,258.95 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q172" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R172" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S172" s="18" t="n">
+        <v>0.623</v>
+      </c>
+      <c r="T172" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="U172" s="19" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="V172" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W172" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X172" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y172" s="19" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="Z172" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA172" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB172" s="15" t="n"/>
+      <c r="AC172" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD172" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE172" s="17" t="n">
+        <v>59.837</v>
+      </c>
+      <c r="AF172" s="17" t="n">
+        <v>56.957</v>
+      </c>
+      <c r="AG172" s="17" t="n">
+        <v>62.7169</v>
+      </c>
+      <c r="AH172" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI172" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ172" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK172" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL172" s="15" t="inlineStr">
+        <is>
+          <t>Cantor Fitzgerald Maintains Neutral on Dynatrace, Raises Price Target to $65</t>
+        </is>
+      </c>
+      <c r="AM172" s="17" t="n">
+        <v>58.64</v>
+      </c>
+      <c r="AN172" s="19" t="n">
+        <v>-0.0375</v>
+      </c>
+      <c r="AO172" s="17" t="n">
+        <v>98992.64</v>
+      </c>
+      <c r="AP172" s="17" t="n">
+        <v>19258.95</v>
+      </c>
+      <c r="AQ172" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR172" s="16" t="n"/>
+      <c r="AS172" s="17" t="n"/>
+      <c r="AT172" s="19" t="n"/>
+      <c r="AU172" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV172" s="6" t="inlineStr">
+        <is>
+          <t>6f7f923d-4a6d-435f-8adf-d0b1a958b583</t>
+        </is>
+      </c>
+      <c r="AW172" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-DT-1793369214139</t>
+        </is>
+      </c>
+      <c r="AX172" s="13" t="n">
+        <v>46325.588125</v>
+      </c>
+      <c r="AY172" s="13" t="n">
+        <v>46325.588125</v>
+      </c>
+      <c r="AZ172" s="13" t="n">
+        <v>46325.58769675926</v>
+      </c>
+      <c r="BA172" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -28307,7 +28491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P103"/>
+  <dimension ref="A1:P104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -34606,8 +34790,61 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>Dynatrace, Inc.</t>
+        </is>
+      </c>
+      <c r="C104" s="22" t="n">
+        <v>46325.62979166667</v>
+      </c>
+      <c r="D104" s="22" t="n">
+        <v>46325.42145833333</v>
+      </c>
+      <c r="E104" s="17" t="n">
+        <v>58.74</v>
+      </c>
+      <c r="F104" s="16" t="n">
+        <v>27.311201906</v>
+      </c>
+      <c r="G104" s="17">
+        <f>E104*F104</f>
+        <v/>
+      </c>
+      <c r="H104" s="22" t="n"/>
+      <c r="I104" s="22" t="n"/>
+      <c r="J104" s="17" t="n"/>
+      <c r="K104" s="17">
+        <f>IF(ISNUMBER(J104),J104*F104,"")</f>
+        <v/>
+      </c>
+      <c r="L104" s="23">
+        <f>IF(ISNUMBER(J104),K104-G104,"")</f>
+        <v/>
+      </c>
+      <c r="M104" s="24">
+        <f>IF(ISNUMBER(J104),L104/G104,"")</f>
+        <v/>
+      </c>
+      <c r="N104" s="25">
+        <f>IF(ISNUMBER(H104),H104-C104,"")</f>
+        <v/>
+      </c>
+      <c r="O104" s="6" t="n"/>
+      <c r="P104" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M103">
+  <conditionalFormatting sqref="L2:M104">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-30 14:12 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA172" headerRowCount="1">
-  <autoFilter ref="A1:BA172"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA176" headerRowCount="1">
+  <autoFilter ref="A1:BA176"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P104" headerRowCount="1">
-  <autoFilter ref="A1:P104"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P105" headerRowCount="1">
+  <autoFilter ref="A1:P105"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.6299074074</v>
+        <v>46325.63386574074</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.42157407408</v>
+        <v>46325.4255324074</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$172,"BUY")+COUNTIF(Orders!$E$2:$E$172,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$176,"BUY")+COUNTIF(Orders!$E$2:$E$176,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$172,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$176,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$172,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$176,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$172,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$176,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$172,Orders!$E$2:$E$172,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$176,Orders!$E$2:$E$176,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$172,Orders!$E$2:$E$172,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$176,Orders!$E$2:$E$176,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$104,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$105,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$104,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$105,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$104)</f>
+        <f>SUM('Round trips'!$L$2:$L$105)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$104,"Closed",'Round trips'!$L$2:$L$104,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$105,"Closed",'Round trips'!$L$2:$L$105,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA172"/>
+  <dimension ref="A1:BA176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -28476,6 +28476,754 @@
       </c>
       <c r="BA172" s="6" t="n"/>
     </row>
+    <row r="173">
+      <c r="A173" s="12" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" s="13" t="n">
+        <v>46325.63380787037</v>
+      </c>
+      <c r="C173" s="13" t="n">
+        <v>46325.42547453703</v>
+      </c>
+      <c r="D173" s="13" t="n">
+        <v>46325.59214120371</v>
+      </c>
+      <c r="E173" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F173" s="6" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="G173" s="15" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="H173" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I173" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J173" s="16" t="n">
+        <v>27.311201906</v>
+      </c>
+      <c r="K173" s="17" t="n">
+        <v>58.09293</v>
+      </c>
+      <c r="L173" s="17">
+        <f>IF(AND(ISNUMBER(J173),ISNUMBER(K173)),J173*K173,"")</f>
+        <v/>
+      </c>
+      <c r="M173" s="17" t="n"/>
+      <c r="N173" s="16" t="n">
+        <v>27.311201906</v>
+      </c>
+      <c r="O173" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P173" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 4.7% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q173" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R173" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S173" s="18" t="n">
+        <v>0.623</v>
+      </c>
+      <c r="T173" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="U173" s="19" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="V173" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W173" s="12" t="n"/>
+      <c r="X173" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y173" s="19" t="n">
+        <v>0.009899999999999999</v>
+      </c>
+      <c r="Z173" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA173" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB173" s="15" t="n"/>
+      <c r="AC173" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD173" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE173" s="17" t="n">
+        <v>59.3861</v>
+      </c>
+      <c r="AF173" s="17" t="n">
+        <v>56.4959</v>
+      </c>
+      <c r="AG173" s="17" t="n">
+        <v>62.2763</v>
+      </c>
+      <c r="AH173" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI173" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ173" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK173" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL173" s="15" t="inlineStr">
+        <is>
+          <t>Cantor Fitzgerald Maintains Neutral on Dynatrace, Raises Price Target to $65</t>
+        </is>
+      </c>
+      <c r="AM173" s="17" t="n">
+        <v>58.23</v>
+      </c>
+      <c r="AN173" s="19" t="n">
+        <v>-0.0449</v>
+      </c>
+      <c r="AO173" s="17" t="n">
+        <v>98829.39</v>
+      </c>
+      <c r="AP173" s="17" t="n">
+        <v>17654.69</v>
+      </c>
+      <c r="AQ173" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR173" s="16" t="n">
+        <v>27.311201906</v>
+      </c>
+      <c r="AS173" s="17" t="n">
+        <v>58.74</v>
+      </c>
+      <c r="AT173" s="19" t="n">
+        <v>-0.0104</v>
+      </c>
+      <c r="AU173" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV173" s="6" t="inlineStr">
+        <is>
+          <t>3aba86b3-800e-4454-825b-262acadd79a0</t>
+        </is>
+      </c>
+      <c r="AW173" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-DT-1793369558035</t>
+        </is>
+      </c>
+      <c r="AX173" s="13" t="n">
+        <v>46325.59210648148</v>
+      </c>
+      <c r="AY173" s="13" t="n">
+        <v>46325.59214120371</v>
+      </c>
+      <c r="AZ173" s="13" t="n">
+        <v>46325.59181712963</v>
+      </c>
+      <c r="BA173" s="6" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="12" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" s="13" t="n">
+        <v>46325.63377314815</v>
+      </c>
+      <c r="C174" s="13" t="n">
+        <v>46325.42543981481</v>
+      </c>
+      <c r="D174" s="13" t="n">
+        <v>46325.59210648148</v>
+      </c>
+      <c r="E174" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F174" s="6" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="G174" s="15" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="H174" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I174" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J174" s="16" t="n">
+        <v>34.46297755</v>
+      </c>
+      <c r="K174" s="17" t="n">
+        <v>49.54</v>
+      </c>
+      <c r="L174" s="17">
+        <f>IF(AND(ISNUMBER(J174),ISNUMBER(K174)),J174*K174,"")</f>
+        <v/>
+      </c>
+      <c r="M174" s="17" t="n"/>
+      <c r="N174" s="16" t="n">
+        <v>34.46297755</v>
+      </c>
+      <c r="O174" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P174" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 4.0% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q174" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R174" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S174" s="18" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="T174" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="U174" s="19" t="n">
+        <v>0.0703</v>
+      </c>
+      <c r="V174" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W174" s="12" t="n"/>
+      <c r="X174" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y174" s="19" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="Z174" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA174" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB174" s="15" t="n"/>
+      <c r="AC174" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD174" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE174" s="17" t="n">
+        <v>51.9228</v>
+      </c>
+      <c r="AF174" s="17" t="n">
+        <v>46.7659</v>
+      </c>
+      <c r="AG174" s="17" t="n">
+        <v>57.0797</v>
+      </c>
+      <c r="AH174" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI174" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ174" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK174" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL174" s="15" t="inlineStr">
+        <is>
+          <t>Canaccord Genuity Maintains Buy on Tenable Holdings, Raises Price Target to $54</t>
+        </is>
+      </c>
+      <c r="AM174" s="17" t="n">
+        <v>49.815</v>
+      </c>
+      <c r="AN174" s="19" t="n">
+        <v>-0.0369</v>
+      </c>
+      <c r="AO174" s="17" t="n">
+        <v>98829.39</v>
+      </c>
+      <c r="AP174" s="17" t="n">
+        <v>17654.69</v>
+      </c>
+      <c r="AQ174" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR174" s="16" t="n">
+        <v>34.46297755</v>
+      </c>
+      <c r="AS174" s="17" t="n">
+        <v>50.78</v>
+      </c>
+      <c r="AT174" s="19" t="n">
+        <v>-0.0209</v>
+      </c>
+      <c r="AU174" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV174" s="6" t="inlineStr">
+        <is>
+          <t>984f46f9-0553-4a10-aeff-3f4ecae19aab</t>
+        </is>
+      </c>
+      <c r="AW174" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-TENB-1793369558105</t>
+        </is>
+      </c>
+      <c r="AX174" s="13" t="n">
+        <v>46325.59210648148</v>
+      </c>
+      <c r="AY174" s="13" t="n">
+        <v>46325.59210648148</v>
+      </c>
+      <c r="AZ174" s="13" t="n">
+        <v>46325.59181712963</v>
+      </c>
+      <c r="BA174" s="6" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="12" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" s="13" t="n">
+        <v>46325.63378472222</v>
+      </c>
+      <c r="C175" s="13" t="n">
+        <v>46325.42545138889</v>
+      </c>
+      <c r="D175" s="13" t="n">
+        <v>46325.59211805555</v>
+      </c>
+      <c r="E175" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F175" s="6" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="G175" s="15" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="H175" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I175" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J175" s="16" t="n">
+        <v>2.823788187</v>
+      </c>
+      <c r="K175" s="17" t="n">
+        <v>238.21</v>
+      </c>
+      <c r="L175" s="17">
+        <f>IF(AND(ISNUMBER(J175),ISNUMBER(K175)),J175*K175,"")</f>
+        <v/>
+      </c>
+      <c r="M175" s="17" t="n"/>
+      <c r="N175" s="16" t="n">
+        <v>2.823788187</v>
+      </c>
+      <c r="O175" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P175" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 3.7% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q175" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R175" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S175" s="18" t="n">
+        <v>0.5580000000000001</v>
+      </c>
+      <c r="T175" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="U175" s="19" t="n">
+        <v>0.0164</v>
+      </c>
+      <c r="V175" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W175" s="12" t="n"/>
+      <c r="X175" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y175" s="19" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="Z175" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA175" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB175" s="15" t="n"/>
+      <c r="AC175" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD175" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE175" s="17" t="n">
+        <v>248.2477</v>
+      </c>
+      <c r="AF175" s="17" t="n">
+        <v>225.5784</v>
+      </c>
+      <c r="AG175" s="17" t="n">
+        <v>270.9171</v>
+      </c>
+      <c r="AH175" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI175" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ175" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AK175" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL175" s="15" t="inlineStr">
+        <is>
+          <t>ServiceNow Posts Downbeat Q3 Earnings, Joins Sprouts Farmers Market, Alphabet And Other Big Stocks Moving Lower In Thursday’s Pre-Market Session</t>
+        </is>
+      </c>
+      <c r="AM175" s="17" t="n">
+        <v>239.18</v>
+      </c>
+      <c r="AN175" s="19" t="n">
+        <v>-0.0345</v>
+      </c>
+      <c r="AO175" s="17" t="n">
+        <v>98829.39</v>
+      </c>
+      <c r="AP175" s="17" t="n">
+        <v>17654.69</v>
+      </c>
+      <c r="AQ175" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR175" s="16" t="n">
+        <v>2.823788187</v>
+      </c>
+      <c r="AS175" s="17" t="n">
+        <v>245.5</v>
+      </c>
+      <c r="AT175" s="19" t="n">
+        <v>-0.0284</v>
+      </c>
+      <c r="AU175" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV175" s="6" t="inlineStr">
+        <is>
+          <t>d4bb7f01-efee-40c4-8955-ac340b823f15</t>
+        </is>
+      </c>
+      <c r="AW175" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-ZS-1793369558209</t>
+        </is>
+      </c>
+      <c r="AX175" s="13" t="n">
+        <v>46325.59210648148</v>
+      </c>
+      <c r="AY175" s="13" t="n">
+        <v>46325.59211805555</v>
+      </c>
+      <c r="AZ175" s="13" t="n">
+        <v>46325.59181712963</v>
+      </c>
+      <c r="BA175" s="6" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="12" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" s="13" t="n">
+        <v>46325.63377314815</v>
+      </c>
+      <c r="C176" s="13" t="n">
+        <v>46325.42543981481</v>
+      </c>
+      <c r="D176" s="13" t="n">
+        <v>46325.59210648148</v>
+      </c>
+      <c r="E176" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F176" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G176" s="15" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="H176" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I176" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J176" s="16" t="n">
+        <v>2.314697642</v>
+      </c>
+      <c r="K176" s="17" t="n">
+        <v>635.34</v>
+      </c>
+      <c r="L176" s="17">
+        <f>IF(AND(ISNUMBER(J176),ISNUMBER(K176)),J176*K176,"")</f>
+        <v/>
+      </c>
+      <c r="M176" s="17" t="n">
+        <v>1470.63</v>
+      </c>
+      <c r="N176" s="16" t="n"/>
+      <c r="O176" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P176" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #3, 8.33% of the $17,654.69 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q176" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R176" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S176" s="18" t="n">
+        <v>0.553</v>
+      </c>
+      <c r="T176" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="U176" s="19" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="V176" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W176" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="X176" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y176" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z176" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA176" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB176" s="15" t="n"/>
+      <c r="AC176" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD176" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE176" s="17" t="n">
+        <v>642.7337</v>
+      </c>
+      <c r="AF176" s="17" t="n">
+        <v>624.9244</v>
+      </c>
+      <c r="AG176" s="17" t="n">
+        <v>660.543</v>
+      </c>
+      <c r="AH176" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI176" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ176" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK176" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL176" s="15" t="inlineStr">
+        <is>
+          <t>Mastercard CEO Says Consumers Keep Spending Despite Economic Uncertainty</t>
+        </is>
+      </c>
+      <c r="AM176" s="17" t="n">
+        <v>635.79</v>
+      </c>
+      <c r="AN176" s="19" t="n">
+        <v>-0.0003</v>
+      </c>
+      <c r="AO176" s="17" t="n">
+        <v>98829.39</v>
+      </c>
+      <c r="AP176" s="17" t="n">
+        <v>17654.69</v>
+      </c>
+      <c r="AQ176" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR176" s="16" t="n"/>
+      <c r="AS176" s="17" t="n"/>
+      <c r="AT176" s="19" t="n"/>
+      <c r="AU176" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV176" s="6" t="inlineStr">
+        <is>
+          <t>4ca2815e-a09a-46bc-87fa-e5e8ec48e277</t>
+        </is>
+      </c>
+      <c r="AW176" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-MA-1793369558286</t>
+        </is>
+      </c>
+      <c r="AX176" s="13" t="n">
+        <v>46325.59210648148</v>
+      </c>
+      <c r="AY176" s="13" t="n">
+        <v>46325.59210648148</v>
+      </c>
+      <c r="AZ176" s="13" t="n">
+        <v>46325.59181712963</v>
+      </c>
+      <c r="BA176" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -28491,7 +29239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P104"/>
+  <dimension ref="A1:P105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -34383,9 +35131,15 @@
         <f>E96*F96</f>
         <v/>
       </c>
-      <c r="H96" s="22" t="n"/>
-      <c r="I96" s="22" t="n"/>
-      <c r="J96" s="17" t="n"/>
+      <c r="H96" s="22" t="n">
+        <v>46325.63378472222</v>
+      </c>
+      <c r="I96" s="22" t="n">
+        <v>46325.42545138889</v>
+      </c>
+      <c r="J96" s="17" t="n">
+        <v>238.21</v>
+      </c>
       <c r="K96" s="17">
         <f>IF(ISNUMBER(J96),J96*F96,"")</f>
         <v/>
@@ -34402,10 +35156,14 @@
         <f>IF(ISNUMBER(H96),H96-C96,"")</f>
         <v/>
       </c>
-      <c r="O96" s="6" t="n"/>
+      <c r="O96" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P96" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -34764,9 +35522,15 @@
         <f>E103*F103</f>
         <v/>
       </c>
-      <c r="H103" s="22" t="n"/>
-      <c r="I103" s="22" t="n"/>
-      <c r="J103" s="17" t="n"/>
+      <c r="H103" s="22" t="n">
+        <v>46325.63377314815</v>
+      </c>
+      <c r="I103" s="22" t="n">
+        <v>46325.42543981481</v>
+      </c>
+      <c r="J103" s="17" t="n">
+        <v>49.54</v>
+      </c>
       <c r="K103" s="17">
         <f>IF(ISNUMBER(J103),J103*F103,"")</f>
         <v/>
@@ -34783,10 +35547,14 @@
         <f>IF(ISNUMBER(H103),H103-C103,"")</f>
         <v/>
       </c>
-      <c r="O103" s="6" t="n"/>
+      <c r="O103" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P103" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -34817,9 +35585,15 @@
         <f>E104*F104</f>
         <v/>
       </c>
-      <c r="H104" s="22" t="n"/>
-      <c r="I104" s="22" t="n"/>
-      <c r="J104" s="17" t="n"/>
+      <c r="H104" s="22" t="n">
+        <v>46325.63380787037</v>
+      </c>
+      <c r="I104" s="22" t="n">
+        <v>46325.42547453703</v>
+      </c>
+      <c r="J104" s="17" t="n">
+        <v>58.09293</v>
+      </c>
       <c r="K104" s="17">
         <f>IF(ISNUMBER(J104),J104*F104,"")</f>
         <v/>
@@ -34836,15 +35610,72 @@
         <f>IF(ISNUMBER(H104),H104-C104,"")</f>
         <v/>
       </c>
-      <c r="O104" s="6" t="n"/>
+      <c r="O104" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P104" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="C105" s="22" t="n">
+        <v>46325.63377314815</v>
+      </c>
+      <c r="D105" s="22" t="n">
+        <v>46325.42543981481</v>
+      </c>
+      <c r="E105" s="17" t="n">
+        <v>635.34</v>
+      </c>
+      <c r="F105" s="16" t="n">
+        <v>2.314697642</v>
+      </c>
+      <c r="G105" s="17">
+        <f>E105*F105</f>
+        <v/>
+      </c>
+      <c r="H105" s="22" t="n"/>
+      <c r="I105" s="22" t="n"/>
+      <c r="J105" s="17" t="n"/>
+      <c r="K105" s="17">
+        <f>IF(ISNUMBER(J105),J105*F105,"")</f>
+        <v/>
+      </c>
+      <c r="L105" s="23">
+        <f>IF(ISNUMBER(J105),K105-G105,"")</f>
+        <v/>
+      </c>
+      <c r="M105" s="24">
+        <f>IF(ISNUMBER(J105),L105/G105,"")</f>
+        <v/>
+      </c>
+      <c r="N105" s="25">
+        <f>IF(ISNUMBER(H105),H105-C105,"")</f>
+        <v/>
+      </c>
+      <c r="O105" s="6" t="n"/>
+      <c r="P105" s="6" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M104">
+  <conditionalFormatting sqref="L2:M105">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-30 14:31 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA176" headerRowCount="1">
-  <autoFilter ref="A1:BA176"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA177" headerRowCount="1">
+  <autoFilter ref="A1:BA177"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P105" headerRowCount="1">
-  <autoFilter ref="A1:P105"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P106" headerRowCount="1">
+  <autoFilter ref="A1:P106"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.63386574074</v>
+        <v>46325.6465625</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.4255324074</v>
+        <v>46325.43822916667</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$176,"BUY")+COUNTIF(Orders!$E$2:$E$176,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$177,"BUY")+COUNTIF(Orders!$E$2:$E$177,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$176,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$177,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$176,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$177,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$176,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$177,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$176,Orders!$E$2:$E$176,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$177,Orders!$E$2:$E$177,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$176,Orders!$E$2:$E$176,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$177,Orders!$E$2:$E$177,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$105,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$106,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$105,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$106,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$105)</f>
+        <f>SUM('Round trips'!$L$2:$L$106)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$105,"Closed",'Round trips'!$L$2:$L$105,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$106,"Closed",'Round trips'!$L$2:$L$106,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA176"/>
+  <dimension ref="A1:BA177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -29224,6 +29224,186 @@
       </c>
       <c r="BA176" s="6" t="n"/>
     </row>
+    <row r="177">
+      <c r="A177" s="12" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" s="13" t="n">
+        <v>46325.64648148148</v>
+      </c>
+      <c r="C177" s="13" t="n">
+        <v>46325.43814814815</v>
+      </c>
+      <c r="D177" s="13" t="n">
+        <v>46325.60481481482</v>
+      </c>
+      <c r="E177" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F177" s="6" t="inlineStr">
+        <is>
+          <t>ULTA</t>
+        </is>
+      </c>
+      <c r="G177" s="15" t="inlineStr">
+        <is>
+          <t>Ulta Beauty, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="H177" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I177" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J177" s="16" t="n">
+        <v>2.62602669</v>
+      </c>
+      <c r="K177" s="17" t="n">
+        <v>639.1900000000001</v>
+      </c>
+      <c r="L177" s="17">
+        <f>IF(AND(ISNUMBER(J177),ISNUMBER(K177)),J177*K177,"")</f>
+        <v/>
+      </c>
+      <c r="M177" s="17" t="n">
+        <v>1678.54</v>
+      </c>
+      <c r="N177" s="16" t="n"/>
+      <c r="O177" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P177" s="15" t="inlineStr">
+        <is>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $20,150.61 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q177" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="R177" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S177" s="18" t="n">
+        <v>0.696</v>
+      </c>
+      <c r="T177" s="12" t="n">
+        <v>46</v>
+      </c>
+      <c r="U177" s="19" t="n">
+        <v>0.0202</v>
+      </c>
+      <c r="V177" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W177" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="X177" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y177" s="19" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="Z177" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA177" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB177" s="15" t="n"/>
+      <c r="AC177" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD177" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE177" s="17" t="n">
+        <v>649.3541</v>
+      </c>
+      <c r="AF177" s="17" t="n">
+        <v>618.4689</v>
+      </c>
+      <c r="AG177" s="17" t="n">
+        <v>680.2393</v>
+      </c>
+      <c r="AH177" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI177" s="18" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AJ177" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK177" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL177" s="15" t="n"/>
+      <c r="AM177" s="17" t="n">
+        <v>637</v>
+      </c>
+      <c r="AN177" s="19" t="n">
+        <v>-0.0173</v>
+      </c>
+      <c r="AO177" s="17" t="n">
+        <v>98693.97</v>
+      </c>
+      <c r="AP177" s="17" t="n">
+        <v>20150.61</v>
+      </c>
+      <c r="AQ177" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR177" s="16" t="n"/>
+      <c r="AS177" s="17" t="n"/>
+      <c r="AT177" s="19" t="n"/>
+      <c r="AU177" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV177" s="6" t="inlineStr">
+        <is>
+          <t>36e3edb5-18f6-40c6-a7ff-26e9431c1d43</t>
+        </is>
+      </c>
+      <c r="AW177" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-ULTA-1793370656122</t>
+        </is>
+      </c>
+      <c r="AX177" s="13" t="n">
+        <v>46325.60481481482</v>
+      </c>
+      <c r="AY177" s="13" t="n">
+        <v>46325.60481481482</v>
+      </c>
+      <c r="AZ177" s="13" t="n">
+        <v>46325.60434027778</v>
+      </c>
+      <c r="BA177" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -29239,7 +29419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P105"/>
+  <dimension ref="A1:P106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -35674,8 +35854,61 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>ULTA</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>Ulta Beauty, Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="C106" s="22" t="n">
+        <v>46325.64648148148</v>
+      </c>
+      <c r="D106" s="22" t="n">
+        <v>46325.43814814815</v>
+      </c>
+      <c r="E106" s="17" t="n">
+        <v>639.1900000000001</v>
+      </c>
+      <c r="F106" s="16" t="n">
+        <v>2.62602669</v>
+      </c>
+      <c r="G106" s="17">
+        <f>E106*F106</f>
+        <v/>
+      </c>
+      <c r="H106" s="22" t="n"/>
+      <c r="I106" s="22" t="n"/>
+      <c r="J106" s="17" t="n"/>
+      <c r="K106" s="17">
+        <f>IF(ISNUMBER(J106),J106*F106,"")</f>
+        <v/>
+      </c>
+      <c r="L106" s="23">
+        <f>IF(ISNUMBER(J106),K106-G106,"")</f>
+        <v/>
+      </c>
+      <c r="M106" s="24">
+        <f>IF(ISNUMBER(J106),L106/G106,"")</f>
+        <v/>
+      </c>
+      <c r="N106" s="25">
+        <f>IF(ISNUMBER(H106),H106-C106,"")</f>
+        <v/>
+      </c>
+      <c r="O106" s="6" t="n"/>
+      <c r="P106" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M105">
+  <conditionalFormatting sqref="L2:M106">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-30 15:01 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA177" headerRowCount="1">
-  <autoFilter ref="A1:BA177"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA178" headerRowCount="1">
+  <autoFilter ref="A1:BA178"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -291,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P106" headerRowCount="1">
-  <autoFilter ref="A1:P106"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoundTrips" displayName="RoundTrips" ref="A1:P107" headerRowCount="1">
+  <autoFilter ref="A1:P107"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="Company"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.6465625</v>
+        <v>46325.66758101852</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.43822916667</v>
+        <v>46325.45924768518</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$177,"BUY")+COUNTIF(Orders!$E$2:$E$177,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$178,"BUY")+COUNTIF(Orders!$E$2:$E$178,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$177,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$178,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$177,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$178,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$177,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$178,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$177,Orders!$E$2:$E$177,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$178,Orders!$E$2:$E$178,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$177,Orders!$E$2:$E$177,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$178,Orders!$E$2:$E$178,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$106,"Closed")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$107,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>COUNTIF('Round trips'!$P$2:$P$106,"Open")</f>
+        <f>COUNTIF('Round trips'!$P$2:$P$107,"Open")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Round trips'!$L$2:$L$106)</f>
+        <f>SUM('Round trips'!$L$2:$L$107)</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>COUNTIFS('Round trips'!$P$2:$P$106,"Closed",'Round trips'!$L$2:$L$106,"&gt;0")</f>
+        <f>COUNTIFS('Round trips'!$P$2:$P$107,"Closed",'Round trips'!$L$2:$L$107,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA177"/>
+  <dimension ref="A1:BA178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -29404,6 +29404,190 @@
       </c>
       <c r="BA177" s="6" t="n"/>
     </row>
+    <row r="178">
+      <c r="A178" s="12" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" s="13" t="n">
+        <v>46325.6675</v>
+      </c>
+      <c r="C178" s="13" t="n">
+        <v>46325.45916666667</v>
+      </c>
+      <c r="D178" s="13" t="n">
+        <v>46325.62583333333</v>
+      </c>
+      <c r="E178" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F178" s="6" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="G178" s="15" t="inlineStr">
+        <is>
+          <t>ExxonMobil Holdings Corporation</t>
+        </is>
+      </c>
+      <c r="H178" s="6" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="I178" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J178" s="16" t="n">
+        <v>8.322299745</v>
+      </c>
+      <c r="K178" s="17" t="n">
+        <v>184.89</v>
+      </c>
+      <c r="L178" s="17">
+        <f>IF(AND(ISNUMBER(J178),ISNUMBER(K178)),J178*K178,"")</f>
+        <v/>
+      </c>
+      <c r="M178" s="17" t="n">
+        <v>1538.72</v>
+      </c>
+      <c r="N178" s="16" t="n"/>
+      <c r="O178" s="6" t="inlineStr">
+        <is>
+          <t>4+/5 green</t>
+        </is>
+      </c>
+      <c r="P178" s="15" t="inlineStr">
+        <is>
+          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $18,472.08 free cash split 12 ways</t>
+        </is>
+      </c>
+      <c r="Q178" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R178" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S178" s="18" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="T178" s="12" t="n">
+        <v>93</v>
+      </c>
+      <c r="U178" s="19" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="V178" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W178" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="X178" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y178" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z178" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA178" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB178" s="15" t="n"/>
+      <c r="AC178" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD178" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE178" s="17" t="n">
+        <v>187.3</v>
+      </c>
+      <c r="AF178" s="17" t="n">
+        <v>181.1249</v>
+      </c>
+      <c r="AG178" s="17" t="n">
+        <v>193.4751</v>
+      </c>
+      <c r="AH178" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI178" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AJ178" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AK178" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL178" s="15" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AM178" s="17" t="n">
+        <v>184.77</v>
+      </c>
+      <c r="AN178" s="19" t="n">
+        <v>0.0091</v>
+      </c>
+      <c r="AO178" s="17" t="n">
+        <v>98639.38</v>
+      </c>
+      <c r="AP178" s="17" t="n">
+        <v>18472.08</v>
+      </c>
+      <c r="AQ178" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR178" s="16" t="n"/>
+      <c r="AS178" s="17" t="n"/>
+      <c r="AT178" s="19" t="n"/>
+      <c r="AU178" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV178" s="6" t="inlineStr">
+        <is>
+          <t>ec6e58b3-03d4-46ad-a5b7-e1b3da62dda8</t>
+        </is>
+      </c>
+      <c r="AW178" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-XOM-1793372471119</t>
+        </is>
+      </c>
+      <c r="AX178" s="13" t="n">
+        <v>46325.62582175926</v>
+      </c>
+      <c r="AY178" s="13" t="n">
+        <v>46325.62583333333</v>
+      </c>
+      <c r="AZ178" s="13" t="n">
+        <v>46325.62520833333</v>
+      </c>
+      <c r="BA178" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -29419,7 +29603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P106"/>
+  <dimension ref="A1:P107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -35907,8 +36091,61 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>ExxonMobil Holdings Corporation</t>
+        </is>
+      </c>
+      <c r="C107" s="22" t="n">
+        <v>46325.6675</v>
+      </c>
+      <c r="D107" s="22" t="n">
+        <v>46325.45916666667</v>
+      </c>
+      <c r="E107" s="17" t="n">
+        <v>184.89</v>
+      </c>
+      <c r="F107" s="16" t="n">
+        <v>8.322299745</v>
+      </c>
+      <c r="G107" s="17">
+        <f>E107*F107</f>
+        <v/>
+      </c>
+      <c r="H107" s="22" t="n"/>
+      <c r="I107" s="22" t="n"/>
+      <c r="J107" s="17" t="n"/>
+      <c r="K107" s="17">
+        <f>IF(ISNUMBER(J107),J107*F107,"")</f>
+        <v/>
+      </c>
+      <c r="L107" s="23">
+        <f>IF(ISNUMBER(J107),K107-G107,"")</f>
+        <v/>
+      </c>
+      <c r="M107" s="24">
+        <f>IF(ISNUMBER(J107),L107/G107,"")</f>
+        <v/>
+      </c>
+      <c r="N107" s="25">
+        <f>IF(ISNUMBER(H107),H107-C107,"")</f>
+        <v/>
+      </c>
+      <c r="O107" s="6" t="n"/>
+      <c r="P107" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M106">
+  <conditionalFormatting sqref="L2:M107">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
records: 2026-10-30 15:07 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA178" headerRowCount="1">
-  <autoFilter ref="A1:BA178"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA179" headerRowCount="1">
+  <autoFilter ref="A1:BA179"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.66758101852</v>
+        <v>46325.67158564815</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.45924768518</v>
+        <v>46325.46325231482</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$178,"BUY")+COUNTIF(Orders!$E$2:$E$178,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$179,"BUY")+COUNTIF(Orders!$E$2:$E$179,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$178,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$179,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$178,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$179,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$178,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$179,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$178,Orders!$E$2:$E$178,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$179,Orders!$E$2:$E$179,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$178,Orders!$E$2:$E$178,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$179,Orders!$E$2:$E$179,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA178"/>
+  <dimension ref="A1:BA179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -29588,6 +29588,198 @@
       </c>
       <c r="BA178" s="6" t="n"/>
     </row>
+    <row r="179">
+      <c r="A179" s="12" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" s="13" t="n">
+        <v>46325.67149305555</v>
+      </c>
+      <c r="C179" s="13" t="n">
+        <v>46325.46315972223</v>
+      </c>
+      <c r="D179" s="13" t="n">
+        <v>46325.62982638889</v>
+      </c>
+      <c r="E179" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F179" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="G179" s="15" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="H179" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I179" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J179" s="16" t="n">
+        <v>1.637432978</v>
+      </c>
+      <c r="K179" s="17" t="n">
+        <v>414.8</v>
+      </c>
+      <c r="L179" s="17">
+        <f>IF(AND(ISNUMBER(J179),ISNUMBER(K179)),J179*K179,"")</f>
+        <v/>
+      </c>
+      <c r="M179" s="17" t="n"/>
+      <c r="N179" s="16" t="n">
+        <v>1.637432978</v>
+      </c>
+      <c r="O179" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P179" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 4.2% today and only 3 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q179" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R179" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S179" s="18" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="T179" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="U179" s="19" t="n">
+        <v>0.0147</v>
+      </c>
+      <c r="V179" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W179" s="12" t="n"/>
+      <c r="X179" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y179" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z179" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AA179" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="AB179" s="15" t="inlineStr">
+        <is>
+          <t>Rose 4.2% then gave back most of it within hours. Looks like pump-and-fade.</t>
+        </is>
+      </c>
+      <c r="AC179" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD179" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE179" s="17" t="n">
+        <v>422.5446</v>
+      </c>
+      <c r="AF179" s="17" t="n">
+        <v>403.3831</v>
+      </c>
+      <c r="AG179" s="17" t="n">
+        <v>441.706</v>
+      </c>
+      <c r="AH179" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI179" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ179" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK179" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL179" s="15" t="inlineStr">
+        <is>
+          <t>If You Invested $1000 In Analog Devices Stock 5 Years Ago, You Would Have This Much Today</t>
+        </is>
+      </c>
+      <c r="AM179" s="17" t="n">
+        <v>414.88</v>
+      </c>
+      <c r="AN179" s="19" t="n">
+        <v>-0.0423</v>
+      </c>
+      <c r="AO179" s="17" t="n">
+        <v>98617.39</v>
+      </c>
+      <c r="AP179" s="17" t="n">
+        <v>16933.37</v>
+      </c>
+      <c r="AQ179" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR179" s="16" t="n">
+        <v>1.637432978</v>
+      </c>
+      <c r="AS179" s="17" t="n">
+        <v>423.37</v>
+      </c>
+      <c r="AT179" s="19" t="n">
+        <v>-0.0194</v>
+      </c>
+      <c r="AU179" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV179" s="6" t="inlineStr">
+        <is>
+          <t>7d07c064-98ce-48f2-bacd-1e7bf00c735b</t>
+        </is>
+      </c>
+      <c r="AW179" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-ADI-1793372817147</t>
+        </is>
+      </c>
+      <c r="AX179" s="13" t="n">
+        <v>46325.62982638889</v>
+      </c>
+      <c r="AY179" s="13" t="n">
+        <v>46325.62982638889</v>
+      </c>
+      <c r="AZ179" s="13" t="n">
+        <v>46325.629375</v>
+      </c>
+      <c r="BA179" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -34945,9 +35137,15 @@
         <f>E86*F86</f>
         <v/>
       </c>
-      <c r="H86" s="22" t="n"/>
-      <c r="I86" s="22" t="n"/>
-      <c r="J86" s="17" t="n"/>
+      <c r="H86" s="22" t="n">
+        <v>46325.67149305555</v>
+      </c>
+      <c r="I86" s="22" t="n">
+        <v>46325.46315972223</v>
+      </c>
+      <c r="J86" s="17" t="n">
+        <v>414.8</v>
+      </c>
       <c r="K86" s="17">
         <f>IF(ISNUMBER(J86),J86*F86,"")</f>
         <v/>
@@ -34964,10 +35162,14 @@
         <f>IF(ISNUMBER(H86),H86-C86,"")</f>
         <v/>
       </c>
-      <c r="O86" s="6" t="n"/>
+      <c r="O86" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P86" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-30 16:06 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA179" headerRowCount="1">
-  <autoFilter ref="A1:BA179"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA180" headerRowCount="1">
+  <autoFilter ref="A1:BA180"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.67158564815</v>
+        <v>46325.71313657407</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.46325231482</v>
+        <v>46325.50480324074</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$179,"BUY")+COUNTIF(Orders!$E$2:$E$179,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$180,"BUY")+COUNTIF(Orders!$E$2:$E$180,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$179,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$180,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$179,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$180,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$179,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$180,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$179,Orders!$E$2:$E$179,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$180,Orders!$E$2:$E$180,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$179,Orders!$E$2:$E$179,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$180,Orders!$E$2:$E$180,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA179"/>
+  <dimension ref="A1:BA180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -27925,13 +27925,13 @@
         <v>169</v>
       </c>
       <c r="B170" s="13" t="n">
-        <v>46325.6212037037</v>
+        <v>46325.7096875</v>
       </c>
       <c r="C170" s="13" t="n">
-        <v>46325.41287037037</v>
+        <v>46325.50135416666</v>
       </c>
       <c r="D170" s="13" t="n">
-        <v>46325.57953703704</v>
+        <v>46325.66802083333</v>
       </c>
       <c r="E170" s="21" t="inlineStr">
         <is>
@@ -27940,29 +27940,21 @@
       </c>
       <c r="F170" s="6" t="inlineStr">
         <is>
-          <t>AVTR</t>
-        </is>
-      </c>
-      <c r="G170" s="15" t="inlineStr">
-        <is>
-          <t>AVTR</t>
-        </is>
-      </c>
-      <c r="H170" s="6" t="inlineStr">
-        <is>
-          <t>NYSE</t>
-        </is>
-      </c>
+          <t>NTSK</t>
+        </is>
+      </c>
+      <c r="G170" s="15" t="n"/>
+      <c r="H170" s="6" t="n"/>
       <c r="I170" s="6" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
       <c r="J170" s="16" t="n">
-        <v>506</v>
+        <v>36.050548589</v>
       </c>
       <c r="K170" s="17" t="n">
-        <v>16.09581</v>
+        <v>24.21</v>
       </c>
       <c r="L170" s="17">
         <f>IF(AND(ISNUMBER(J170),ISNUMBER(K170)),J170*K170,"")</f>
@@ -27970,118 +27962,48 @@
       </c>
       <c r="M170" s="17" t="n"/>
       <c r="N170" s="16" t="n">
-        <v>506</v>
+        <v>36.050548589</v>
       </c>
       <c r="O170" s="6" t="inlineStr">
         <is>
-          <t>bad day</t>
+          <t>stop-loss (Alpaca order)</t>
         </is>
       </c>
       <c r="P170" s="15" t="inlineStr">
         <is>
-          <t>Bad day: down 3.6% today and only 4 of 5 green</t>
-        </is>
-      </c>
-      <c r="Q170" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="R170" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="S170" s="18" t="n">
-        <v>0.823</v>
-      </c>
-      <c r="T170" s="12" t="n">
-        <v>62</v>
-      </c>
-      <c r="U170" s="19" t="n">
-        <v>0.0453</v>
-      </c>
-      <c r="V170" s="19" t="n">
-        <v>0.2893</v>
-      </c>
+          <t>Alpaca stop order triggered at 24.23 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q170" s="12" t="n"/>
+      <c r="R170" s="6" t="n"/>
+      <c r="S170" s="18" t="n"/>
+      <c r="T170" s="12" t="n"/>
+      <c r="U170" s="19" t="n"/>
+      <c r="V170" s="19" t="n"/>
       <c r="W170" s="12" t="n"/>
-      <c r="X170" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y170" s="19" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="Z170" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AA170" s="12" t="n">
-        <v>100</v>
-      </c>
+      <c r="X170" s="6" t="n"/>
+      <c r="Y170" s="19" t="n"/>
+      <c r="Z170" s="6" t="n"/>
+      <c r="AA170" s="12" t="n"/>
       <c r="AB170" s="15" t="n"/>
-      <c r="AC170" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AD170" s="6" t="inlineStr">
-        <is>
-          <t>up</t>
-        </is>
-      </c>
-      <c r="AE170" s="17" t="n">
-        <v>16.4138</v>
-      </c>
-      <c r="AF170" s="17" t="n">
-        <v>15.7543</v>
-      </c>
-      <c r="AG170" s="17" t="n">
-        <v>17.0734</v>
-      </c>
-      <c r="AH170" s="20" t="n">
-        <v>46332</v>
-      </c>
-      <c r="AI170" s="18" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="AJ170" s="6" t="inlineStr">
-        <is>
-          <t>alert</t>
-        </is>
-      </c>
-      <c r="AK170" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="AL170" s="15" t="inlineStr">
-        <is>
-          <t>Avantor Q3 2026 Earnings Call Transcript</t>
-        </is>
-      </c>
-      <c r="AM170" s="17" t="n">
-        <v>16.155</v>
-      </c>
-      <c r="AN170" s="19" t="n">
-        <v>-0.0315</v>
-      </c>
-      <c r="AO170" s="17" t="n">
-        <v>99175.84</v>
-      </c>
-      <c r="AP170" s="17" t="n">
-        <v>12864.5</v>
-      </c>
-      <c r="AQ170" s="19" t="n">
-        <v>0.0833</v>
-      </c>
-      <c r="AR170" s="16" t="n">
-        <v>506</v>
-      </c>
-      <c r="AS170" s="17" t="n">
-        <v>16.368458</v>
-      </c>
-      <c r="AT170" s="19" t="n">
-        <v>-0.0176</v>
-      </c>
+      <c r="AC170" s="6" t="n"/>
+      <c r="AD170" s="6" t="n"/>
+      <c r="AE170" s="17" t="n"/>
+      <c r="AF170" s="17" t="n"/>
+      <c r="AG170" s="17" t="n"/>
+      <c r="AH170" s="20" t="n"/>
+      <c r="AI170" s="18" t="n"/>
+      <c r="AJ170" s="6" t="n"/>
+      <c r="AK170" s="12" t="n"/>
+      <c r="AL170" s="15" t="n"/>
+      <c r="AM170" s="17" t="n"/>
+      <c r="AN170" s="19" t="n"/>
+      <c r="AO170" s="17" t="n"/>
+      <c r="AP170" s="17" t="n"/>
+      <c r="AQ170" s="19" t="n"/>
+      <c r="AR170" s="16" t="n"/>
+      <c r="AS170" s="17" t="n"/>
+      <c r="AT170" s="19" t="n"/>
       <c r="AU170" s="6" t="inlineStr">
         <is>
           <t>paper</t>
@@ -28089,23 +28011,21 @@
       </c>
       <c r="AV170" s="6" t="inlineStr">
         <is>
-          <t>5a2aff3f-e025-4347-b4bc-5b807d79a3dd</t>
+          <t>e9456b6d-cb33-4648-a824-8d5159883aa8</t>
         </is>
       </c>
       <c r="AW170" s="6" t="inlineStr">
         <is>
-          <t>tdagent-sell-AVTR-1793368471561</t>
+          <t>tdagent-stop-NTSK-1793368321507</t>
         </is>
       </c>
       <c r="AX170" s="13" t="n">
-        <v>46325.57952546296</v>
+        <v>46325.57778935185</v>
       </c>
       <c r="AY170" s="13" t="n">
-        <v>46325.57953703704</v>
-      </c>
-      <c r="AZ170" s="13" t="n">
-        <v>46325.57931712963</v>
-      </c>
+        <v>46325.66802083333</v>
+      </c>
+      <c r="AZ170" s="13" t="n"/>
       <c r="BA170" s="6" t="n"/>
     </row>
     <row r="171">
@@ -28113,32 +28033,32 @@
         <v>170</v>
       </c>
       <c r="B171" s="13" t="n">
-        <v>46325.62579861111</v>
+        <v>46325.6212037037</v>
       </c>
       <c r="C171" s="13" t="n">
-        <v>46325.41746527778</v>
+        <v>46325.41287037037</v>
       </c>
       <c r="D171" s="13" t="n">
-        <v>46325.58413194444</v>
-      </c>
-      <c r="E171" s="14" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>46325.57953703704</v>
+      </c>
+      <c r="E171" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F171" s="6" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>AVTR</t>
         </is>
       </c>
       <c r="G171" s="15" t="inlineStr">
         <is>
-          <t>Tenable Holdings, Inc. Common Stock</t>
+          <t>AVTR</t>
         </is>
       </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="I171" s="6" t="inlineStr">
@@ -28147,27 +28067,27 @@
         </is>
       </c>
       <c r="J171" s="16" t="n">
-        <v>34.46297755</v>
+        <v>506</v>
       </c>
       <c r="K171" s="17" t="n">
-        <v>50.78</v>
+        <v>16.09581</v>
       </c>
       <c r="L171" s="17">
         <f>IF(AND(ISNUMBER(J171),ISNUMBER(K171)),J171*K171,"")</f>
         <v/>
       </c>
-      <c r="M171" s="17" t="n">
-        <v>1750.04</v>
-      </c>
-      <c r="N171" s="16" t="n"/>
+      <c r="M171" s="17" t="n"/>
+      <c r="N171" s="16" t="n">
+        <v>506</v>
+      </c>
       <c r="O171" s="6" t="inlineStr">
         <is>
-          <t>4+/5 green</t>
+          <t>bad day</t>
         </is>
       </c>
       <c r="P171" s="15" t="inlineStr">
         <is>
-          <t>4 of 5 green, time machine green, rank #4, 8.33% of the $21,008.98 free cash split 12 ways</t>
+          <t>Bad day: down 3.6% today and only 4 of 5 green</t>
         </is>
       </c>
       <c r="Q171" s="12" t="n">
@@ -28179,27 +28099,25 @@
         </is>
       </c>
       <c r="S171" s="18" t="n">
-        <v>0.625</v>
+        <v>0.823</v>
       </c>
       <c r="T171" s="12" t="n">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="U171" s="19" t="n">
-        <v>0.0703</v>
+        <v>0.0453</v>
       </c>
       <c r="V171" s="19" t="n">
         <v>0.2893</v>
       </c>
-      <c r="W171" s="12" t="n">
-        <v>4</v>
-      </c>
+      <c r="W171" s="12" t="n"/>
       <c r="X171" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
       <c r="Y171" s="19" t="n">
-        <v>0.0038</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="Z171" s="6" t="inlineStr">
         <is>
@@ -28221,23 +28139,23 @@
         </is>
       </c>
       <c r="AE171" s="17" t="n">
-        <v>52.721</v>
+        <v>16.4138</v>
       </c>
       <c r="AF171" s="17" t="n">
-        <v>47.506</v>
+        <v>15.7543</v>
       </c>
       <c r="AG171" s="17" t="n">
-        <v>57.9361</v>
+        <v>17.0734</v>
       </c>
       <c r="AH171" s="20" t="n">
         <v>46332</v>
       </c>
       <c r="AI171" s="18" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="AJ171" s="6" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>alert</t>
         </is>
       </c>
       <c r="AK171" s="12" t="n">
@@ -28245,27 +28163,33 @@
       </c>
       <c r="AL171" s="15" t="inlineStr">
         <is>
-          <t>Canaccord Genuity Maintains Buy on Tenable Holdings, Raises Price Target to $54</t>
+          <t>Avantor Q3 2026 Earnings Call Transcript</t>
         </is>
       </c>
       <c r="AM171" s="17" t="n">
-        <v>50.83</v>
+        <v>16.155</v>
       </c>
       <c r="AN171" s="19" t="n">
-        <v>-0.0219</v>
+        <v>-0.0315</v>
       </c>
       <c r="AO171" s="17" t="n">
-        <v>99162.94</v>
+        <v>99175.84</v>
       </c>
       <c r="AP171" s="17" t="n">
-        <v>21008.98</v>
+        <v>12864.5</v>
       </c>
       <c r="AQ171" s="19" t="n">
         <v>0.0833</v>
       </c>
-      <c r="AR171" s="16" t="n"/>
-      <c r="AS171" s="17" t="n"/>
-      <c r="AT171" s="19" t="n"/>
+      <c r="AR171" s="16" t="n">
+        <v>506</v>
+      </c>
+      <c r="AS171" s="17" t="n">
+        <v>16.368458</v>
+      </c>
+      <c r="AT171" s="19" t="n">
+        <v>-0.0176</v>
+      </c>
       <c r="AU171" s="6" t="inlineStr">
         <is>
           <t>paper</t>
@@ -28273,22 +28197,22 @@
       </c>
       <c r="AV171" s="6" t="inlineStr">
         <is>
-          <t>df26cb82-ab44-4a98-98a5-5d4ad6ebca75</t>
+          <t>5a2aff3f-e025-4347-b4bc-5b807d79a3dd</t>
         </is>
       </c>
       <c r="AW171" s="6" t="inlineStr">
         <is>
-          <t>tdagent-buy-TENB-1793368866439</t>
+          <t>tdagent-sell-AVTR-1793368471561</t>
         </is>
       </c>
       <c r="AX171" s="13" t="n">
-        <v>46325.58409722222</v>
+        <v>46325.57952546296</v>
       </c>
       <c r="AY171" s="13" t="n">
-        <v>46325.58413194444</v>
+        <v>46325.57953703704</v>
       </c>
       <c r="AZ171" s="13" t="n">
-        <v>46325.58353009259</v>
+        <v>46325.57931712963</v>
       </c>
       <c r="BA171" s="6" t="n"/>
     </row>
@@ -28297,13 +28221,13 @@
         <v>171</v>
       </c>
       <c r="B172" s="13" t="n">
-        <v>46325.62979166667</v>
+        <v>46325.62579861111</v>
       </c>
       <c r="C172" s="13" t="n">
-        <v>46325.42145833333</v>
+        <v>46325.41746527778</v>
       </c>
       <c r="D172" s="13" t="n">
-        <v>46325.588125</v>
+        <v>46325.58413194444</v>
       </c>
       <c r="E172" s="14" t="inlineStr">
         <is>
@@ -28312,17 +28236,17 @@
       </c>
       <c r="F172" s="6" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>TENB</t>
         </is>
       </c>
       <c r="G172" s="15" t="inlineStr">
         <is>
-          <t>Dynatrace, Inc.</t>
+          <t>Tenable Holdings, Inc. Common Stock</t>
         </is>
       </c>
       <c r="H172" s="6" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="I172" s="6" t="inlineStr">
@@ -28331,17 +28255,17 @@
         </is>
       </c>
       <c r="J172" s="16" t="n">
-        <v>27.311201906</v>
+        <v>34.46297755</v>
       </c>
       <c r="K172" s="17" t="n">
-        <v>58.74</v>
+        <v>50.78</v>
       </c>
       <c r="L172" s="17">
         <f>IF(AND(ISNUMBER(J172),ISNUMBER(K172)),J172*K172,"")</f>
         <v/>
       </c>
       <c r="M172" s="17" t="n">
-        <v>1604.27</v>
+        <v>1750.04</v>
       </c>
       <c r="N172" s="16" t="n"/>
       <c r="O172" s="6" t="inlineStr">
@@ -28351,11 +28275,11 @@
       </c>
       <c r="P172" s="15" t="inlineStr">
         <is>
-          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $19,258.95 free cash split 12 ways</t>
+          <t>4 of 5 green, time machine green, rank #4, 8.33% of the $21,008.98 free cash split 12 ways</t>
         </is>
       </c>
       <c r="Q172" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R172" s="6" t="inlineStr">
         <is>
@@ -28363,19 +28287,19 @@
         </is>
       </c>
       <c r="S172" s="18" t="n">
-        <v>0.623</v>
+        <v>0.625</v>
       </c>
       <c r="T172" s="12" t="n">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="U172" s="19" t="n">
-        <v>0.0115</v>
+        <v>0.0703</v>
       </c>
       <c r="V172" s="19" t="n">
         <v>0.2893</v>
       </c>
       <c r="W172" s="12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="X172" s="6" t="inlineStr">
         <is>
@@ -28383,7 +28307,7 @@
         </is>
       </c>
       <c r="Y172" s="19" t="n">
-        <v>0.0008</v>
+        <v>0.0038</v>
       </c>
       <c r="Z172" s="6" t="inlineStr">
         <is>
@@ -28405,44 +28329,44 @@
         </is>
       </c>
       <c r="AE172" s="17" t="n">
-        <v>59.837</v>
+        <v>52.721</v>
       </c>
       <c r="AF172" s="17" t="n">
-        <v>56.957</v>
+        <v>47.506</v>
       </c>
       <c r="AG172" s="17" t="n">
-        <v>62.7169</v>
+        <v>57.9361</v>
       </c>
       <c r="AH172" s="20" t="n">
         <v>46332</v>
       </c>
       <c r="AI172" s="18" t="n">
-        <v>0.53</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ172" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>watch</t>
         </is>
       </c>
       <c r="AK172" s="12" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="AL172" s="15" t="inlineStr">
         <is>
-          <t>Cantor Fitzgerald Maintains Neutral on Dynatrace, Raises Price Target to $65</t>
+          <t>Canaccord Genuity Maintains Buy on Tenable Holdings, Raises Price Target to $54</t>
         </is>
       </c>
       <c r="AM172" s="17" t="n">
-        <v>58.64</v>
+        <v>50.83</v>
       </c>
       <c r="AN172" s="19" t="n">
-        <v>-0.0375</v>
+        <v>-0.0219</v>
       </c>
       <c r="AO172" s="17" t="n">
-        <v>98992.64</v>
+        <v>99162.94</v>
       </c>
       <c r="AP172" s="17" t="n">
-        <v>19258.95</v>
+        <v>21008.98</v>
       </c>
       <c r="AQ172" s="19" t="n">
         <v>0.0833</v>
@@ -28457,22 +28381,22 @@
       </c>
       <c r="AV172" s="6" t="inlineStr">
         <is>
-          <t>6f7f923d-4a6d-435f-8adf-d0b1a958b583</t>
+          <t>df26cb82-ab44-4a98-98a5-5d4ad6ebca75</t>
         </is>
       </c>
       <c r="AW172" s="6" t="inlineStr">
         <is>
-          <t>tdagent-buy-DT-1793369214139</t>
+          <t>tdagent-buy-TENB-1793368866439</t>
         </is>
       </c>
       <c r="AX172" s="13" t="n">
-        <v>46325.588125</v>
+        <v>46325.58409722222</v>
       </c>
       <c r="AY172" s="13" t="n">
-        <v>46325.588125</v>
+        <v>46325.58413194444</v>
       </c>
       <c r="AZ172" s="13" t="n">
-        <v>46325.58769675926</v>
+        <v>46325.58353009259</v>
       </c>
       <c r="BA172" s="6" t="n"/>
     </row>
@@ -28481,17 +28405,17 @@
         <v>172</v>
       </c>
       <c r="B173" s="13" t="n">
-        <v>46325.63380787037</v>
+        <v>46325.62979166667</v>
       </c>
       <c r="C173" s="13" t="n">
-        <v>46325.42547453703</v>
+        <v>46325.42145833333</v>
       </c>
       <c r="D173" s="13" t="n">
-        <v>46325.59214120371</v>
-      </c>
-      <c r="E173" s="21" t="inlineStr">
-        <is>
-          <t>SELL</t>
+        <v>46325.588125</v>
+      </c>
+      <c r="E173" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F173" s="6" t="inlineStr">
@@ -28501,7 +28425,7 @@
       </c>
       <c r="G173" s="15" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>Dynatrace, Inc.</t>
         </is>
       </c>
       <c r="H173" s="6" t="inlineStr">
@@ -28518,28 +28442,28 @@
         <v>27.311201906</v>
       </c>
       <c r="K173" s="17" t="n">
-        <v>58.09293</v>
+        <v>58.74</v>
       </c>
       <c r="L173" s="17">
         <f>IF(AND(ISNUMBER(J173),ISNUMBER(K173)),J173*K173,"")</f>
         <v/>
       </c>
-      <c r="M173" s="17" t="n"/>
-      <c r="N173" s="16" t="n">
-        <v>27.311201906</v>
-      </c>
+      <c r="M173" s="17" t="n">
+        <v>1604.27</v>
+      </c>
+      <c r="N173" s="16" t="n"/>
       <c r="O173" s="6" t="inlineStr">
         <is>
-          <t>bad day</t>
+          <t>4+/5 green</t>
         </is>
       </c>
       <c r="P173" s="15" t="inlineStr">
         <is>
-          <t>Bad day: down 4.7% today and only 4 of 5 green</t>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $19,258.95 free cash split 12 ways</t>
         </is>
       </c>
       <c r="Q173" s="12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R173" s="6" t="inlineStr">
         <is>
@@ -28558,14 +28482,16 @@
       <c r="V173" s="19" t="n">
         <v>0.2893</v>
       </c>
-      <c r="W173" s="12" t="n"/>
+      <c r="W173" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="X173" s="6" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="Y173" s="19" t="n">
-        <v>0.009899999999999999</v>
+        <v>0.0008</v>
       </c>
       <c r="Z173" s="6" t="inlineStr">
         <is>
@@ -28587,13 +28513,13 @@
         </is>
       </c>
       <c r="AE173" s="17" t="n">
-        <v>59.3861</v>
+        <v>59.837</v>
       </c>
       <c r="AF173" s="17" t="n">
-        <v>56.4959</v>
+        <v>56.957</v>
       </c>
       <c r="AG173" s="17" t="n">
-        <v>62.2763</v>
+        <v>62.7169</v>
       </c>
       <c r="AH173" s="20" t="n">
         <v>46332</v>
@@ -28615,29 +28541,23 @@
         </is>
       </c>
       <c r="AM173" s="17" t="n">
-        <v>58.23</v>
+        <v>58.64</v>
       </c>
       <c r="AN173" s="19" t="n">
-        <v>-0.0449</v>
+        <v>-0.0375</v>
       </c>
       <c r="AO173" s="17" t="n">
-        <v>98829.39</v>
+        <v>98992.64</v>
       </c>
       <c r="AP173" s="17" t="n">
-        <v>17654.69</v>
+        <v>19258.95</v>
       </c>
       <c r="AQ173" s="19" t="n">
         <v>0.0833</v>
       </c>
-      <c r="AR173" s="16" t="n">
-        <v>27.311201906</v>
-      </c>
-      <c r="AS173" s="17" t="n">
-        <v>58.74</v>
-      </c>
-      <c r="AT173" s="19" t="n">
-        <v>-0.0104</v>
-      </c>
+      <c r="AR173" s="16" t="n"/>
+      <c r="AS173" s="17" t="n"/>
+      <c r="AT173" s="19" t="n"/>
       <c r="AU173" s="6" t="inlineStr">
         <is>
           <t>paper</t>
@@ -28645,22 +28565,22 @@
       </c>
       <c r="AV173" s="6" t="inlineStr">
         <is>
-          <t>3aba86b3-800e-4454-825b-262acadd79a0</t>
+          <t>6f7f923d-4a6d-435f-8adf-d0b1a958b583</t>
         </is>
       </c>
       <c r="AW173" s="6" t="inlineStr">
         <is>
-          <t>tdagent-sell-DT-1793369558035</t>
+          <t>tdagent-buy-DT-1793369214139</t>
         </is>
       </c>
       <c r="AX173" s="13" t="n">
-        <v>46325.59210648148</v>
+        <v>46325.588125</v>
       </c>
       <c r="AY173" s="13" t="n">
-        <v>46325.59214120371</v>
+        <v>46325.588125</v>
       </c>
       <c r="AZ173" s="13" t="n">
-        <v>46325.59181712963</v>
+        <v>46325.58769675926</v>
       </c>
       <c r="BA173" s="6" t="n"/>
     </row>
@@ -28669,13 +28589,13 @@
         <v>173</v>
       </c>
       <c r="B174" s="13" t="n">
-        <v>46325.63377314815</v>
+        <v>46325.63380787037</v>
       </c>
       <c r="C174" s="13" t="n">
-        <v>46325.42543981481</v>
+        <v>46325.42547453703</v>
       </c>
       <c r="D174" s="13" t="n">
-        <v>46325.59210648148</v>
+        <v>46325.59214120371</v>
       </c>
       <c r="E174" s="21" t="inlineStr">
         <is>
@@ -28684,17 +28604,17 @@
       </c>
       <c r="F174" s="6" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="G174" s="15" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="H174" s="6" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="I174" s="6" t="inlineStr">
@@ -28703,10 +28623,10 @@
         </is>
       </c>
       <c r="J174" s="16" t="n">
-        <v>34.46297755</v>
+        <v>27.311201906</v>
       </c>
       <c r="K174" s="17" t="n">
-        <v>49.54</v>
+        <v>58.09293</v>
       </c>
       <c r="L174" s="17">
         <f>IF(AND(ISNUMBER(J174),ISNUMBER(K174)),J174*K174,"")</f>
@@ -28714,7 +28634,7 @@
       </c>
       <c r="M174" s="17" t="n"/>
       <c r="N174" s="16" t="n">
-        <v>34.46297755</v>
+        <v>27.311201906</v>
       </c>
       <c r="O174" s="6" t="inlineStr">
         <is>
@@ -28723,7 +28643,7 @@
       </c>
       <c r="P174" s="15" t="inlineStr">
         <is>
-          <t>Bad day: down 4.0% today and only 4 of 5 green</t>
+          <t>Bad day: down 4.7% today and only 4 of 5 green</t>
         </is>
       </c>
       <c r="Q174" s="12" t="n">
@@ -28735,13 +28655,13 @@
         </is>
       </c>
       <c r="S174" s="18" t="n">
-        <v>0.625</v>
+        <v>0.623</v>
       </c>
       <c r="T174" s="12" t="n">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="U174" s="19" t="n">
-        <v>0.0703</v>
+        <v>0.0115</v>
       </c>
       <c r="V174" s="19" t="n">
         <v>0.2893</v>
@@ -28749,11 +28669,11 @@
       <c r="W174" s="12" t="n"/>
       <c r="X174" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>watch</t>
         </is>
       </c>
       <c r="Y174" s="19" t="n">
-        <v>0.0012</v>
+        <v>0.009899999999999999</v>
       </c>
       <c r="Z174" s="6" t="inlineStr">
         <is>
@@ -28775,38 +28695,38 @@
         </is>
       </c>
       <c r="AE174" s="17" t="n">
-        <v>51.9228</v>
+        <v>59.3861</v>
       </c>
       <c r="AF174" s="17" t="n">
-        <v>46.7659</v>
+        <v>56.4959</v>
       </c>
       <c r="AG174" s="17" t="n">
-        <v>57.0797</v>
+        <v>62.2763</v>
       </c>
       <c r="AH174" s="20" t="n">
         <v>46332</v>
       </c>
       <c r="AI174" s="18" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.53</v>
       </c>
       <c r="AJ174" s="6" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AK174" s="12" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AL174" s="15" t="inlineStr">
         <is>
-          <t>Canaccord Genuity Maintains Buy on Tenable Holdings, Raises Price Target to $54</t>
+          <t>Cantor Fitzgerald Maintains Neutral on Dynatrace, Raises Price Target to $65</t>
         </is>
       </c>
       <c r="AM174" s="17" t="n">
-        <v>49.815</v>
+        <v>58.23</v>
       </c>
       <c r="AN174" s="19" t="n">
-        <v>-0.0369</v>
+        <v>-0.0449</v>
       </c>
       <c r="AO174" s="17" t="n">
         <v>98829.39</v>
@@ -28818,13 +28738,13 @@
         <v>0.0833</v>
       </c>
       <c r="AR174" s="16" t="n">
-        <v>34.46297755</v>
+        <v>27.311201906</v>
       </c>
       <c r="AS174" s="17" t="n">
-        <v>50.78</v>
+        <v>58.74</v>
       </c>
       <c r="AT174" s="19" t="n">
-        <v>-0.0209</v>
+        <v>-0.0104</v>
       </c>
       <c r="AU174" s="6" t="inlineStr">
         <is>
@@ -28833,19 +28753,19 @@
       </c>
       <c r="AV174" s="6" t="inlineStr">
         <is>
-          <t>984f46f9-0553-4a10-aeff-3f4ecae19aab</t>
+          <t>3aba86b3-800e-4454-825b-262acadd79a0</t>
         </is>
       </c>
       <c r="AW174" s="6" t="inlineStr">
         <is>
-          <t>tdagent-sell-TENB-1793369558105</t>
+          <t>tdagent-sell-DT-1793369558035</t>
         </is>
       </c>
       <c r="AX174" s="13" t="n">
         <v>46325.59210648148</v>
       </c>
       <c r="AY174" s="13" t="n">
-        <v>46325.59210648148</v>
+        <v>46325.59214120371</v>
       </c>
       <c r="AZ174" s="13" t="n">
         <v>46325.59181712963</v>
@@ -28857,13 +28777,13 @@
         <v>174</v>
       </c>
       <c r="B175" s="13" t="n">
-        <v>46325.63378472222</v>
+        <v>46325.63377314815</v>
       </c>
       <c r="C175" s="13" t="n">
-        <v>46325.42545138889</v>
+        <v>46325.42543981481</v>
       </c>
       <c r="D175" s="13" t="n">
-        <v>46325.59211805555</v>
+        <v>46325.59210648148</v>
       </c>
       <c r="E175" s="21" t="inlineStr">
         <is>
@@ -28872,12 +28792,12 @@
       </c>
       <c r="F175" s="6" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>TENB</t>
         </is>
       </c>
       <c r="G175" s="15" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>TENB</t>
         </is>
       </c>
       <c r="H175" s="6" t="inlineStr">
@@ -28891,10 +28811,10 @@
         </is>
       </c>
       <c r="J175" s="16" t="n">
-        <v>2.823788187</v>
+        <v>34.46297755</v>
       </c>
       <c r="K175" s="17" t="n">
-        <v>238.21</v>
+        <v>49.54</v>
       </c>
       <c r="L175" s="17">
         <f>IF(AND(ISNUMBER(J175),ISNUMBER(K175)),J175*K175,"")</f>
@@ -28902,7 +28822,7 @@
       </c>
       <c r="M175" s="17" t="n"/>
       <c r="N175" s="16" t="n">
-        <v>2.823788187</v>
+        <v>34.46297755</v>
       </c>
       <c r="O175" s="6" t="inlineStr">
         <is>
@@ -28911,7 +28831,7 @@
       </c>
       <c r="P175" s="15" t="inlineStr">
         <is>
-          <t>Bad day: down 3.7% today and only 4 of 5 green</t>
+          <t>Bad day: down 4.0% today and only 4 of 5 green</t>
         </is>
       </c>
       <c r="Q175" s="12" t="n">
@@ -28923,13 +28843,13 @@
         </is>
       </c>
       <c r="S175" s="18" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.625</v>
       </c>
       <c r="T175" s="12" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="U175" s="19" t="n">
-        <v>0.0164</v>
+        <v>0.0703</v>
       </c>
       <c r="V175" s="19" t="n">
         <v>0.2893</v>
@@ -28941,7 +28861,7 @@
         </is>
       </c>
       <c r="Y175" s="19" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="Z175" s="6" t="inlineStr">
         <is>
@@ -28963,38 +28883,38 @@
         </is>
       </c>
       <c r="AE175" s="17" t="n">
-        <v>248.2477</v>
+        <v>51.9228</v>
       </c>
       <c r="AF175" s="17" t="n">
-        <v>225.5784</v>
+        <v>46.7659</v>
       </c>
       <c r="AG175" s="17" t="n">
-        <v>270.9171</v>
+        <v>57.0797</v>
       </c>
       <c r="AH175" s="20" t="n">
         <v>46332</v>
       </c>
       <c r="AI175" s="18" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ175" s="6" t="inlineStr">
         <is>
-          <t>alert</t>
+          <t>watch</t>
         </is>
       </c>
       <c r="AK175" s="12" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="AL175" s="15" t="inlineStr">
         <is>
-          <t>ServiceNow Posts Downbeat Q3 Earnings, Joins Sprouts Farmers Market, Alphabet And Other Big Stocks Moving Lower In Thursday’s Pre-Market Session</t>
+          <t>Canaccord Genuity Maintains Buy on Tenable Holdings, Raises Price Target to $54</t>
         </is>
       </c>
       <c r="AM175" s="17" t="n">
-        <v>239.18</v>
+        <v>49.815</v>
       </c>
       <c r="AN175" s="19" t="n">
-        <v>-0.0345</v>
+        <v>-0.0369</v>
       </c>
       <c r="AO175" s="17" t="n">
         <v>98829.39</v>
@@ -29006,13 +28926,13 @@
         <v>0.0833</v>
       </c>
       <c r="AR175" s="16" t="n">
-        <v>2.823788187</v>
+        <v>34.46297755</v>
       </c>
       <c r="AS175" s="17" t="n">
-        <v>245.5</v>
+        <v>50.78</v>
       </c>
       <c r="AT175" s="19" t="n">
-        <v>-0.0284</v>
+        <v>-0.0209</v>
       </c>
       <c r="AU175" s="6" t="inlineStr">
         <is>
@@ -29021,19 +28941,19 @@
       </c>
       <c r="AV175" s="6" t="inlineStr">
         <is>
-          <t>d4bb7f01-efee-40c4-8955-ac340b823f15</t>
+          <t>984f46f9-0553-4a10-aeff-3f4ecae19aab</t>
         </is>
       </c>
       <c r="AW175" s="6" t="inlineStr">
         <is>
-          <t>tdagent-sell-ZS-1793369558209</t>
+          <t>tdagent-sell-TENB-1793369558105</t>
         </is>
       </c>
       <c r="AX175" s="13" t="n">
         <v>46325.59210648148</v>
       </c>
       <c r="AY175" s="13" t="n">
-        <v>46325.59211805555</v>
+        <v>46325.59210648148</v>
       </c>
       <c r="AZ175" s="13" t="n">
         <v>46325.59181712963</v>
@@ -29045,32 +28965,32 @@
         <v>175</v>
       </c>
       <c r="B176" s="13" t="n">
-        <v>46325.63377314815</v>
+        <v>46325.63378472222</v>
       </c>
       <c r="C176" s="13" t="n">
-        <v>46325.42543981481</v>
+        <v>46325.42545138889</v>
       </c>
       <c r="D176" s="13" t="n">
-        <v>46325.59210648148</v>
-      </c>
-      <c r="E176" s="14" t="inlineStr">
-        <is>
-          <t>BUY</t>
+        <v>46325.59211805555</v>
+      </c>
+      <c r="E176" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
         </is>
       </c>
       <c r="F176" s="6" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="G176" s="15" t="inlineStr">
         <is>
-          <t>Mastercard Incorporated</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="H176" s="6" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="I176" s="6" t="inlineStr">
@@ -29079,27 +28999,27 @@
         </is>
       </c>
       <c r="J176" s="16" t="n">
-        <v>2.314697642</v>
+        <v>2.823788187</v>
       </c>
       <c r="K176" s="17" t="n">
-        <v>635.34</v>
+        <v>238.21</v>
       </c>
       <c r="L176" s="17">
         <f>IF(AND(ISNUMBER(J176),ISNUMBER(K176)),J176*K176,"")</f>
         <v/>
       </c>
-      <c r="M176" s="17" t="n">
-        <v>1470.63</v>
-      </c>
-      <c r="N176" s="16" t="n"/>
+      <c r="M176" s="17" t="n"/>
+      <c r="N176" s="16" t="n">
+        <v>2.823788187</v>
+      </c>
       <c r="O176" s="6" t="inlineStr">
         <is>
-          <t>4+/5 green</t>
+          <t>bad day</t>
         </is>
       </c>
       <c r="P176" s="15" t="inlineStr">
         <is>
-          <t>4 of 5 green, time machine green, rank #3, 8.33% of the $17,654.69 free cash split 12 ways</t>
+          <t>Bad day: down 3.7% today and only 4 of 5 green</t>
         </is>
       </c>
       <c r="Q176" s="12" t="n">
@@ -29111,27 +29031,25 @@
         </is>
       </c>
       <c r="S176" s="18" t="n">
-        <v>0.553</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="T176" s="12" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="U176" s="19" t="n">
-        <v>0.006500000000000001</v>
+        <v>0.0164</v>
       </c>
       <c r="V176" s="19" t="n">
         <v>0.2893</v>
       </c>
-      <c r="W176" s="12" t="n">
-        <v>3</v>
-      </c>
+      <c r="W176" s="12" t="n"/>
       <c r="X176" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
       <c r="Y176" s="19" t="n">
-        <v>0.0003</v>
+        <v>0.0009</v>
       </c>
       <c r="Z176" s="6" t="inlineStr">
         <is>
@@ -29153,38 +29071,38 @@
         </is>
       </c>
       <c r="AE176" s="17" t="n">
-        <v>642.7337</v>
+        <v>248.2477</v>
       </c>
       <c r="AF176" s="17" t="n">
-        <v>624.9244</v>
+        <v>225.5784</v>
       </c>
       <c r="AG176" s="17" t="n">
-        <v>660.543</v>
+        <v>270.9171</v>
       </c>
       <c r="AH176" s="20" t="n">
         <v>46332</v>
       </c>
       <c r="AI176" s="18" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="AJ176" s="6" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>alert</t>
         </is>
       </c>
       <c r="AK176" s="12" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AL176" s="15" t="inlineStr">
         <is>
-          <t>Mastercard CEO Says Consumers Keep Spending Despite Economic Uncertainty</t>
+          <t>ServiceNow Posts Downbeat Q3 Earnings, Joins Sprouts Farmers Market, Alphabet And Other Big Stocks Moving Lower In Thursday’s Pre-Market Session</t>
         </is>
       </c>
       <c r="AM176" s="17" t="n">
-        <v>635.79</v>
+        <v>239.18</v>
       </c>
       <c r="AN176" s="19" t="n">
-        <v>-0.0003</v>
+        <v>-0.0345</v>
       </c>
       <c r="AO176" s="17" t="n">
         <v>98829.39</v>
@@ -29195,9 +29113,15 @@
       <c r="AQ176" s="19" t="n">
         <v>0.0833</v>
       </c>
-      <c r="AR176" s="16" t="n"/>
-      <c r="AS176" s="17" t="n"/>
-      <c r="AT176" s="19" t="n"/>
+      <c r="AR176" s="16" t="n">
+        <v>2.823788187</v>
+      </c>
+      <c r="AS176" s="17" t="n">
+        <v>245.5</v>
+      </c>
+      <c r="AT176" s="19" t="n">
+        <v>-0.0284</v>
+      </c>
       <c r="AU176" s="6" t="inlineStr">
         <is>
           <t>paper</t>
@@ -29205,19 +29129,19 @@
       </c>
       <c r="AV176" s="6" t="inlineStr">
         <is>
-          <t>4ca2815e-a09a-46bc-87fa-e5e8ec48e277</t>
+          <t>d4bb7f01-efee-40c4-8955-ac340b823f15</t>
         </is>
       </c>
       <c r="AW176" s="6" t="inlineStr">
         <is>
-          <t>tdagent-buy-MA-1793369558286</t>
+          <t>tdagent-sell-ZS-1793369558209</t>
         </is>
       </c>
       <c r="AX176" s="13" t="n">
         <v>46325.59210648148</v>
       </c>
       <c r="AY176" s="13" t="n">
-        <v>46325.59210648148</v>
+        <v>46325.59211805555</v>
       </c>
       <c r="AZ176" s="13" t="n">
         <v>46325.59181712963</v>
@@ -29229,13 +29153,13 @@
         <v>176</v>
       </c>
       <c r="B177" s="13" t="n">
-        <v>46325.64648148148</v>
+        <v>46325.63377314815</v>
       </c>
       <c r="C177" s="13" t="n">
-        <v>46325.43814814815</v>
+        <v>46325.42543981481</v>
       </c>
       <c r="D177" s="13" t="n">
-        <v>46325.60481481482</v>
+        <v>46325.59210648148</v>
       </c>
       <c r="E177" s="14" t="inlineStr">
         <is>
@@ -29244,17 +29168,17 @@
       </c>
       <c r="F177" s="6" t="inlineStr">
         <is>
-          <t>ULTA</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="G177" s="15" t="inlineStr">
         <is>
-          <t>Ulta Beauty, Inc. Common Stock</t>
+          <t>Mastercard Incorporated</t>
         </is>
       </c>
       <c r="H177" s="6" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="I177" s="6" t="inlineStr">
@@ -29263,17 +29187,17 @@
         </is>
       </c>
       <c r="J177" s="16" t="n">
-        <v>2.62602669</v>
+        <v>2.314697642</v>
       </c>
       <c r="K177" s="17" t="n">
-        <v>639.1900000000001</v>
+        <v>635.34</v>
       </c>
       <c r="L177" s="17">
         <f>IF(AND(ISNUMBER(J177),ISNUMBER(K177)),J177*K177,"")</f>
         <v/>
       </c>
       <c r="M177" s="17" t="n">
-        <v>1678.54</v>
+        <v>1470.63</v>
       </c>
       <c r="N177" s="16" t="n"/>
       <c r="O177" s="6" t="inlineStr">
@@ -29283,11 +29207,11 @@
       </c>
       <c r="P177" s="15" t="inlineStr">
         <is>
-          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $20,150.61 free cash split 12 ways</t>
+          <t>4 of 5 green, time machine green, rank #3, 8.33% of the $17,654.69 free cash split 12 ways</t>
         </is>
       </c>
       <c r="Q177" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R177" s="6" t="inlineStr">
         <is>
@@ -29295,19 +29219,19 @@
         </is>
       </c>
       <c r="S177" s="18" t="n">
-        <v>0.696</v>
+        <v>0.553</v>
       </c>
       <c r="T177" s="12" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="U177" s="19" t="n">
-        <v>0.0202</v>
+        <v>0.006500000000000001</v>
       </c>
       <c r="V177" s="19" t="n">
         <v>0.2893</v>
       </c>
       <c r="W177" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X177" s="6" t="inlineStr">
         <is>
@@ -29315,7 +29239,7 @@
         </is>
       </c>
       <c r="Y177" s="19" t="n">
-        <v>0.0013</v>
+        <v>0.0003</v>
       </c>
       <c r="Z177" s="6" t="inlineStr">
         <is>
@@ -29337,40 +29261,44 @@
         </is>
       </c>
       <c r="AE177" s="17" t="n">
-        <v>649.3541</v>
+        <v>642.7337</v>
       </c>
       <c r="AF177" s="17" t="n">
-        <v>618.4689</v>
+        <v>624.9244</v>
       </c>
       <c r="AG177" s="17" t="n">
-        <v>680.2393</v>
+        <v>660.543</v>
       </c>
       <c r="AH177" s="20" t="n">
         <v>46332</v>
       </c>
       <c r="AI177" s="18" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="AJ177" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>watch</t>
         </is>
       </c>
       <c r="AK177" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL177" s="15" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="AL177" s="15" t="inlineStr">
+        <is>
+          <t>Mastercard CEO Says Consumers Keep Spending Despite Economic Uncertainty</t>
+        </is>
+      </c>
       <c r="AM177" s="17" t="n">
-        <v>637</v>
+        <v>635.79</v>
       </c>
       <c r="AN177" s="19" t="n">
-        <v>-0.0173</v>
+        <v>-0.0003</v>
       </c>
       <c r="AO177" s="17" t="n">
-        <v>98693.97</v>
+        <v>98829.39</v>
       </c>
       <c r="AP177" s="17" t="n">
-        <v>20150.61</v>
+        <v>17654.69</v>
       </c>
       <c r="AQ177" s="19" t="n">
         <v>0.0833</v>
@@ -29385,22 +29313,22 @@
       </c>
       <c r="AV177" s="6" t="inlineStr">
         <is>
-          <t>36e3edb5-18f6-40c6-a7ff-26e9431c1d43</t>
+          <t>4ca2815e-a09a-46bc-87fa-e5e8ec48e277</t>
         </is>
       </c>
       <c r="AW177" s="6" t="inlineStr">
         <is>
-          <t>tdagent-buy-ULTA-1793370656122</t>
+          <t>tdagent-buy-MA-1793369558286</t>
         </is>
       </c>
       <c r="AX177" s="13" t="n">
-        <v>46325.60481481482</v>
+        <v>46325.59210648148</v>
       </c>
       <c r="AY177" s="13" t="n">
-        <v>46325.60481481482</v>
+        <v>46325.59210648148</v>
       </c>
       <c r="AZ177" s="13" t="n">
-        <v>46325.60434027778</v>
+        <v>46325.59181712963</v>
       </c>
       <c r="BA177" s="6" t="n"/>
     </row>
@@ -29409,13 +29337,13 @@
         <v>177</v>
       </c>
       <c r="B178" s="13" t="n">
-        <v>46325.6675</v>
+        <v>46325.64648148148</v>
       </c>
       <c r="C178" s="13" t="n">
-        <v>46325.45916666667</v>
+        <v>46325.43814814815</v>
       </c>
       <c r="D178" s="13" t="n">
-        <v>46325.62583333333</v>
+        <v>46325.60481481482</v>
       </c>
       <c r="E178" s="14" t="inlineStr">
         <is>
@@ -29424,17 +29352,17 @@
       </c>
       <c r="F178" s="6" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>ULTA</t>
         </is>
       </c>
       <c r="G178" s="15" t="inlineStr">
         <is>
-          <t>ExxonMobil Holdings Corporation</t>
+          <t>Ulta Beauty, Inc. Common Stock</t>
         </is>
       </c>
       <c r="H178" s="6" t="inlineStr">
         <is>
-          <t>NYSE</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="I178" s="6" t="inlineStr">
@@ -29443,17 +29371,17 @@
         </is>
       </c>
       <c r="J178" s="16" t="n">
-        <v>8.322299745</v>
+        <v>2.62602669</v>
       </c>
       <c r="K178" s="17" t="n">
-        <v>184.89</v>
+        <v>639.1900000000001</v>
       </c>
       <c r="L178" s="17">
         <f>IF(AND(ISNUMBER(J178),ISNUMBER(K178)),J178*K178,"")</f>
         <v/>
       </c>
       <c r="M178" s="17" t="n">
-        <v>1538.72</v>
+        <v>1678.54</v>
       </c>
       <c r="N178" s="16" t="n"/>
       <c r="O178" s="6" t="inlineStr">
@@ -29463,11 +29391,11 @@
       </c>
       <c r="P178" s="15" t="inlineStr">
         <is>
-          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $18,472.08 free cash split 12 ways</t>
+          <t>5 of 5 green, time machine green, rank #1, 8.33% of the $20,150.61 free cash split 12 ways</t>
         </is>
       </c>
       <c r="Q178" s="12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R178" s="6" t="inlineStr">
         <is>
@@ -29475,19 +29403,19 @@
         </is>
       </c>
       <c r="S178" s="18" t="n">
-        <v>0.624</v>
+        <v>0.696</v>
       </c>
       <c r="T178" s="12" t="n">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="U178" s="19" t="n">
-        <v>0.0119</v>
+        <v>0.0202</v>
       </c>
       <c r="V178" s="19" t="n">
         <v>0.2893</v>
       </c>
       <c r="W178" s="12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="X178" s="6" t="inlineStr">
         <is>
@@ -29495,7 +29423,7 @@
         </is>
       </c>
       <c r="Y178" s="19" t="n">
-        <v>0.0003</v>
+        <v>0.0013</v>
       </c>
       <c r="Z178" s="6" t="inlineStr">
         <is>
@@ -29517,44 +29445,40 @@
         </is>
       </c>
       <c r="AE178" s="17" t="n">
-        <v>187.3</v>
+        <v>649.3541</v>
       </c>
       <c r="AF178" s="17" t="n">
-        <v>181.1249</v>
+        <v>618.4689</v>
       </c>
       <c r="AG178" s="17" t="n">
-        <v>193.4751</v>
+        <v>680.2393</v>
       </c>
       <c r="AH178" s="20" t="n">
         <v>46332</v>
       </c>
       <c r="AI178" s="18" t="n">
-        <v>0.57</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AJ178" s="6" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AK178" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="AL178" s="15" t="inlineStr">
-        <is>
-          <t>Exxon Mobil Q3 2026 Earnings Call Transcript</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AL178" s="15" t="n"/>
       <c r="AM178" s="17" t="n">
-        <v>184.77</v>
+        <v>637</v>
       </c>
       <c r="AN178" s="19" t="n">
-        <v>0.0091</v>
+        <v>-0.0173</v>
       </c>
       <c r="AO178" s="17" t="n">
-        <v>98639.38</v>
+        <v>98693.97</v>
       </c>
       <c r="AP178" s="17" t="n">
-        <v>18472.08</v>
+        <v>20150.61</v>
       </c>
       <c r="AQ178" s="19" t="n">
         <v>0.0833</v>
@@ -29569,22 +29493,22 @@
       </c>
       <c r="AV178" s="6" t="inlineStr">
         <is>
-          <t>ec6e58b3-03d4-46ad-a5b7-e1b3da62dda8</t>
+          <t>36e3edb5-18f6-40c6-a7ff-26e9431c1d43</t>
         </is>
       </c>
       <c r="AW178" s="6" t="inlineStr">
         <is>
-          <t>tdagent-buy-XOM-1793372471119</t>
+          <t>tdagent-buy-ULTA-1793370656122</t>
         </is>
       </c>
       <c r="AX178" s="13" t="n">
-        <v>46325.62582175926</v>
+        <v>46325.60481481482</v>
       </c>
       <c r="AY178" s="13" t="n">
-        <v>46325.62583333333</v>
+        <v>46325.60481481482</v>
       </c>
       <c r="AZ178" s="13" t="n">
-        <v>46325.62520833333</v>
+        <v>46325.60434027778</v>
       </c>
       <c r="BA178" s="6" t="n"/>
     </row>
@@ -29593,32 +29517,32 @@
         <v>178</v>
       </c>
       <c r="B179" s="13" t="n">
-        <v>46325.67149305555</v>
+        <v>46325.6675</v>
       </c>
       <c r="C179" s="13" t="n">
-        <v>46325.46315972223</v>
+        <v>46325.45916666667</v>
       </c>
       <c r="D179" s="13" t="n">
-        <v>46325.62982638889</v>
-      </c>
-      <c r="E179" s="21" t="inlineStr">
-        <is>
-          <t>SELL</t>
+        <v>46325.62583333333</v>
+      </c>
+      <c r="E179" s="14" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="F179" s="6" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="G179" s="15" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ExxonMobil Holdings Corporation</t>
         </is>
       </c>
       <c r="H179" s="6" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>NYSE</t>
         </is>
       </c>
       <c r="I179" s="6" t="inlineStr">
@@ -29627,31 +29551,31 @@
         </is>
       </c>
       <c r="J179" s="16" t="n">
-        <v>1.637432978</v>
+        <v>8.322299745</v>
       </c>
       <c r="K179" s="17" t="n">
-        <v>414.8</v>
+        <v>184.89</v>
       </c>
       <c r="L179" s="17">
         <f>IF(AND(ISNUMBER(J179),ISNUMBER(K179)),J179*K179,"")</f>
         <v/>
       </c>
-      <c r="M179" s="17" t="n"/>
-      <c r="N179" s="16" t="n">
-        <v>1.637432978</v>
-      </c>
+      <c r="M179" s="17" t="n">
+        <v>1538.72</v>
+      </c>
+      <c r="N179" s="16" t="n"/>
       <c r="O179" s="6" t="inlineStr">
         <is>
-          <t>bad day</t>
+          <t>4+/5 green</t>
         </is>
       </c>
       <c r="P179" s="15" t="inlineStr">
         <is>
-          <t>Bad day: down 4.2% today and only 3 of 5 green</t>
+          <t>4 of 5 green, time machine green, rank #5, 8.33% of the $18,472.08 free cash split 12 ways</t>
         </is>
       </c>
       <c r="Q179" s="12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R179" s="6" t="inlineStr">
         <is>
@@ -29659,18 +29583,20 @@
         </is>
       </c>
       <c r="S179" s="18" t="n">
-        <v>0.707</v>
+        <v>0.624</v>
       </c>
       <c r="T179" s="12" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="U179" s="19" t="n">
-        <v>0.0147</v>
+        <v>0.0119</v>
       </c>
       <c r="V179" s="19" t="n">
         <v>0.2893</v>
       </c>
-      <c r="W179" s="12" t="n"/>
+      <c r="W179" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="X179" s="6" t="inlineStr">
         <is>
           <t>ok</t>
@@ -29681,20 +29607,16 @@
       </c>
       <c r="Z179" s="6" t="inlineStr">
         <is>
-          <t>alert</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AA179" s="12" t="n">
-        <v>70</v>
-      </c>
-      <c r="AB179" s="15" t="inlineStr">
-        <is>
-          <t>Rose 4.2% then gave back most of it within hours. Looks like pump-and-fade.</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="AB179" s="15" t="n"/>
       <c r="AC179" s="6" t="inlineStr">
         <is>
-          <t>watch</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="AD179" s="6" t="inlineStr">
@@ -29703,82 +29625,268 @@
         </is>
       </c>
       <c r="AE179" s="17" t="n">
-        <v>422.5446</v>
+        <v>187.3</v>
       </c>
       <c r="AF179" s="17" t="n">
-        <v>403.3831</v>
+        <v>181.1249</v>
       </c>
       <c r="AG179" s="17" t="n">
-        <v>441.706</v>
+        <v>193.4751</v>
       </c>
       <c r="AH179" s="20" t="n">
         <v>46332</v>
       </c>
       <c r="AI179" s="18" t="n">
-        <v>0.53</v>
+        <v>0.57</v>
       </c>
       <c r="AJ179" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>watch</t>
         </is>
       </c>
       <c r="AK179" s="12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="AL179" s="15" t="inlineStr">
         <is>
-          <t>If You Invested $1000 In Analog Devices Stock 5 Years Ago, You Would Have This Much Today</t>
+          <t>Exxon Mobil Q3 2026 Earnings Call Transcript</t>
         </is>
       </c>
       <c r="AM179" s="17" t="n">
-        <v>414.88</v>
+        <v>184.77</v>
       </c>
       <c r="AN179" s="19" t="n">
-        <v>-0.0423</v>
+        <v>0.0091</v>
       </c>
       <c r="AO179" s="17" t="n">
-        <v>98617.39</v>
+        <v>98639.38</v>
       </c>
       <c r="AP179" s="17" t="n">
-        <v>16933.37</v>
+        <v>18472.08</v>
       </c>
       <c r="AQ179" s="19" t="n">
         <v>0.0833</v>
       </c>
-      <c r="AR179" s="16" t="n">
+      <c r="AR179" s="16" t="n"/>
+      <c r="AS179" s="17" t="n"/>
+      <c r="AT179" s="19" t="n"/>
+      <c r="AU179" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV179" s="6" t="inlineStr">
+        <is>
+          <t>ec6e58b3-03d4-46ad-a5b7-e1b3da62dda8</t>
+        </is>
+      </c>
+      <c r="AW179" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-buy-XOM-1793372471119</t>
+        </is>
+      </c>
+      <c r="AX179" s="13" t="n">
+        <v>46325.62582175926</v>
+      </c>
+      <c r="AY179" s="13" t="n">
+        <v>46325.62583333333</v>
+      </c>
+      <c r="AZ179" s="13" t="n">
+        <v>46325.62520833333</v>
+      </c>
+      <c r="BA179" s="6" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="12" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" s="13" t="n">
+        <v>46325.67149305555</v>
+      </c>
+      <c r="C180" s="13" t="n">
+        <v>46325.46315972223</v>
+      </c>
+      <c r="D180" s="13" t="n">
+        <v>46325.62982638889</v>
+      </c>
+      <c r="E180" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F180" s="6" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="G180" s="15" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="H180" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I180" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J180" s="16" t="n">
         <v>1.637432978</v>
       </c>
-      <c r="AS179" s="17" t="n">
+      <c r="K180" s="17" t="n">
+        <v>414.8</v>
+      </c>
+      <c r="L180" s="17">
+        <f>IF(AND(ISNUMBER(J180),ISNUMBER(K180)),J180*K180,"")</f>
+        <v/>
+      </c>
+      <c r="M180" s="17" t="n"/>
+      <c r="N180" s="16" t="n">
+        <v>1.637432978</v>
+      </c>
+      <c r="O180" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P180" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 4.2% today and only 3 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q180" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R180" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S180" s="18" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="T180" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="U180" s="19" t="n">
+        <v>0.0147</v>
+      </c>
+      <c r="V180" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W180" s="12" t="n"/>
+      <c r="X180" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y180" s="19" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="Z180" s="6" t="inlineStr">
+        <is>
+          <t>alert</t>
+        </is>
+      </c>
+      <c r="AA180" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="AB180" s="15" t="inlineStr">
+        <is>
+          <t>Rose 4.2% then gave back most of it within hours. Looks like pump-and-fade.</t>
+        </is>
+      </c>
+      <c r="AC180" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="AD180" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE180" s="17" t="n">
+        <v>422.5446</v>
+      </c>
+      <c r="AF180" s="17" t="n">
+        <v>403.3831</v>
+      </c>
+      <c r="AG180" s="17" t="n">
+        <v>441.706</v>
+      </c>
+      <c r="AH180" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI180" s="18" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AJ180" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK180" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL180" s="15" t="inlineStr">
+        <is>
+          <t>If You Invested $1000 In Analog Devices Stock 5 Years Ago, You Would Have This Much Today</t>
+        </is>
+      </c>
+      <c r="AM180" s="17" t="n">
+        <v>414.88</v>
+      </c>
+      <c r="AN180" s="19" t="n">
+        <v>-0.0423</v>
+      </c>
+      <c r="AO180" s="17" t="n">
+        <v>98617.39</v>
+      </c>
+      <c r="AP180" s="17" t="n">
+        <v>16933.37</v>
+      </c>
+      <c r="AQ180" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR180" s="16" t="n">
+        <v>1.637432978</v>
+      </c>
+      <c r="AS180" s="17" t="n">
         <v>423.37</v>
       </c>
-      <c r="AT179" s="19" t="n">
+      <c r="AT180" s="19" t="n">
         <v>-0.0194</v>
       </c>
-      <c r="AU179" s="6" t="inlineStr">
+      <c r="AU180" s="6" t="inlineStr">
         <is>
           <t>paper</t>
         </is>
       </c>
-      <c r="AV179" s="6" t="inlineStr">
+      <c r="AV180" s="6" t="inlineStr">
         <is>
           <t>7d07c064-98ce-48f2-bacd-1e7bf00c735b</t>
         </is>
       </c>
-      <c r="AW179" s="6" t="inlineStr">
+      <c r="AW180" s="6" t="inlineStr">
         <is>
           <t>tdagent-sell-ADI-1793372817147</t>
         </is>
       </c>
-      <c r="AX179" s="13" t="n">
+      <c r="AX180" s="13" t="n">
         <v>46325.62982638889</v>
       </c>
-      <c r="AY179" s="13" t="n">
+      <c r="AY180" s="13" t="n">
         <v>46325.62982638889</v>
       </c>
-      <c r="AZ179" s="13" t="n">
+      <c r="AZ180" s="13" t="n">
         <v>46325.629375</v>
       </c>
-      <c r="BA179" s="6" t="n"/>
+      <c r="BA180" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -36035,9 +36143,15 @@
         <f>E102*F102</f>
         <v/>
       </c>
-      <c r="H102" s="22" t="n"/>
-      <c r="I102" s="22" t="n"/>
-      <c r="J102" s="17" t="n"/>
+      <c r="H102" s="22" t="n">
+        <v>46325.7096875</v>
+      </c>
+      <c r="I102" s="22" t="n">
+        <v>46325.50135416666</v>
+      </c>
+      <c r="J102" s="17" t="n">
+        <v>24.21</v>
+      </c>
       <c r="K102" s="17">
         <f>IF(ISNUMBER(J102),J102*F102,"")</f>
         <v/>
@@ -36054,10 +36168,14 @@
         <f>IF(ISNUMBER(H102),H102-C102,"")</f>
         <v/>
       </c>
-      <c r="O102" s="6" t="n"/>
+      <c r="O102" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P102" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-30 17:57 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA180" headerRowCount="1">
-  <autoFilter ref="A1:BA180"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA181" headerRowCount="1">
+  <autoFilter ref="A1:BA181"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.71313657407</v>
+        <v>46325.78987268519</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.50480324074</v>
+        <v>46325.58153935185</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$180,"BUY")+COUNTIF(Orders!$E$2:$E$180,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$181,"BUY")+COUNTIF(Orders!$E$2:$E$181,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$180,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$181,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$180,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$181,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$180,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$181,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$180,Orders!$E$2:$E$180,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$181,Orders!$E$2:$E$181,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$180,Orders!$E$2:$E$180,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$181,Orders!$E$2:$E$181,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA180"/>
+  <dimension ref="A1:BA181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -29888,6 +29888,114 @@
       </c>
       <c r="BA180" s="6" t="n"/>
     </row>
+    <row r="181">
+      <c r="A181" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" s="13" t="n">
+        <v>46325.78715277778</v>
+      </c>
+      <c r="C181" s="13" t="n">
+        <v>46325.57881944445</v>
+      </c>
+      <c r="D181" s="13" t="n">
+        <v>46325.74548611111</v>
+      </c>
+      <c r="E181" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F181" s="6" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="G181" s="15" t="n"/>
+      <c r="H181" s="6" t="n"/>
+      <c r="I181" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J181" s="16" t="n">
+        <v>150.343801052</v>
+      </c>
+      <c r="K181" s="17" t="n">
+        <v>55.37</v>
+      </c>
+      <c r="L181" s="17">
+        <f>IF(AND(ISNUMBER(J181),ISNUMBER(K181)),J181*K181,"")</f>
+        <v/>
+      </c>
+      <c r="M181" s="17" t="n"/>
+      <c r="N181" s="16" t="n">
+        <v>150.343801052</v>
+      </c>
+      <c r="O181" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
+      <c r="P181" s="15" t="inlineStr">
+        <is>
+          <t>Alpaca stop order triggered at 55.38 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q181" s="12" t="n"/>
+      <c r="R181" s="6" t="n"/>
+      <c r="S181" s="18" t="n"/>
+      <c r="T181" s="12" t="n"/>
+      <c r="U181" s="19" t="n"/>
+      <c r="V181" s="19" t="n"/>
+      <c r="W181" s="12" t="n"/>
+      <c r="X181" s="6" t="n"/>
+      <c r="Y181" s="19" t="n"/>
+      <c r="Z181" s="6" t="n"/>
+      <c r="AA181" s="12" t="n"/>
+      <c r="AB181" s="15" t="n"/>
+      <c r="AC181" s="6" t="n"/>
+      <c r="AD181" s="6" t="n"/>
+      <c r="AE181" s="17" t="n"/>
+      <c r="AF181" s="17" t="n"/>
+      <c r="AG181" s="17" t="n"/>
+      <c r="AH181" s="20" t="n"/>
+      <c r="AI181" s="18" t="n"/>
+      <c r="AJ181" s="6" t="n"/>
+      <c r="AK181" s="12" t="n"/>
+      <c r="AL181" s="15" t="n"/>
+      <c r="AM181" s="17" t="n"/>
+      <c r="AN181" s="19" t="n"/>
+      <c r="AO181" s="17" t="n"/>
+      <c r="AP181" s="17" t="n"/>
+      <c r="AQ181" s="19" t="n"/>
+      <c r="AR181" s="16" t="n"/>
+      <c r="AS181" s="17" t="n"/>
+      <c r="AT181" s="19" t="n"/>
+      <c r="AU181" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV181" s="6" t="inlineStr">
+        <is>
+          <t>3eb0bec5-6e74-4375-a7c3-ee4412ce6ae7</t>
+        </is>
+      </c>
+      <c r="AW181" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-stop-EQT-1793379721807</t>
+        </is>
+      </c>
+      <c r="AX181" s="13" t="n">
+        <v>46325.7097337963</v>
+      </c>
+      <c r="AY181" s="13" t="n">
+        <v>46325.74548611111</v>
+      </c>
+      <c r="AZ181" s="13" t="n"/>
+      <c r="BA181" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -34801,9 +34909,15 @@
         <f>E78*F78</f>
         <v/>
       </c>
-      <c r="H78" s="22" t="n"/>
-      <c r="I78" s="22" t="n"/>
-      <c r="J78" s="17" t="n"/>
+      <c r="H78" s="22" t="n">
+        <v>46325.78715277778</v>
+      </c>
+      <c r="I78" s="22" t="n">
+        <v>46325.57881944445</v>
+      </c>
+      <c r="J78" s="17" t="n">
+        <v>55.37</v>
+      </c>
       <c r="K78" s="17">
         <f>IF(ISNUMBER(J78),J78*F78,"")</f>
         <v/>
@@ -34820,10 +34934,14 @@
         <f>IF(ISNUMBER(H78),H78-C78,"")</f>
         <v/>
       </c>
-      <c r="O78" s="6" t="n"/>
+      <c r="O78" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P78" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-30 18:52 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA181" headerRowCount="1">
-  <autoFilter ref="A1:BA181"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA182" headerRowCount="1">
+  <autoFilter ref="A1:BA182"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.78987268519</v>
+        <v>46325.82835648148</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.58153935185</v>
+        <v>46325.62002314815</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$181,"BUY")+COUNTIF(Orders!$E$2:$E$181,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$182,"BUY")+COUNTIF(Orders!$E$2:$E$182,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$181,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$182,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$181,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$182,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$181,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$182,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$181,Orders!$E$2:$E$181,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$182,Orders!$E$2:$E$182,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$181,Orders!$E$2:$E$181,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$182,Orders!$E$2:$E$182,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA181"/>
+  <dimension ref="A1:BA182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -29996,6 +29996,194 @@
       <c r="AZ181" s="13" t="n"/>
       <c r="BA181" s="6" t="n"/>
     </row>
+    <row r="182">
+      <c r="A182" s="12" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" s="13" t="n">
+        <v>46325.82831018518</v>
+      </c>
+      <c r="C182" s="13" t="n">
+        <v>46325.61997685185</v>
+      </c>
+      <c r="D182" s="13" t="n">
+        <v>46325.78664351852</v>
+      </c>
+      <c r="E182" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F182" s="6" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="G182" s="15" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="H182" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I182" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J182" s="16" t="n">
+        <v>18.497085557</v>
+      </c>
+      <c r="K182" s="17" t="n">
+        <v>433.29</v>
+      </c>
+      <c r="L182" s="17">
+        <f>IF(AND(ISNUMBER(J182),ISNUMBER(K182)),J182*K182,"")</f>
+        <v/>
+      </c>
+      <c r="M182" s="17" t="n"/>
+      <c r="N182" s="16" t="n">
+        <v>18.497085557</v>
+      </c>
+      <c r="O182" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
+      <c r="P182" s="15" t="inlineStr">
+        <is>
+          <t>Bad day: down 3.4% today and only 4 of 5 green</t>
+        </is>
+      </c>
+      <c r="Q182" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R182" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S182" s="18" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="T182" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="U182" s="19" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="V182" s="19" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="W182" s="12" t="n"/>
+      <c r="X182" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="Y182" s="19" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="Z182" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA182" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB182" s="15" t="n"/>
+      <c r="AC182" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD182" s="6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="AE182" s="17" t="n">
+        <v>441.1307</v>
+      </c>
+      <c r="AF182" s="17" t="n">
+        <v>423.079</v>
+      </c>
+      <c r="AG182" s="17" t="n">
+        <v>459.1824</v>
+      </c>
+      <c r="AH182" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="AI182" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AJ182" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK182" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL182" s="15" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals Adopts Intuitive's Da Vinci 5 Surgical System</t>
+        </is>
+      </c>
+      <c r="AM182" s="17" t="n">
+        <v>434.06</v>
+      </c>
+      <c r="AN182" s="19" t="n">
+        <v>-0.0331</v>
+      </c>
+      <c r="AO182" s="17" t="n">
+        <v>98407.46000000001</v>
+      </c>
+      <c r="AP182" s="17" t="n">
+        <v>26809.9</v>
+      </c>
+      <c r="AQ182" s="19" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="AR182" s="16" t="n">
+        <v>18.497085557</v>
+      </c>
+      <c r="AS182" s="17" t="n">
+        <v>447.77</v>
+      </c>
+      <c r="AT182" s="19" t="n">
+        <v>-0.0315</v>
+      </c>
+      <c r="AU182" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV182" s="6" t="inlineStr">
+        <is>
+          <t>7d8948d7-4093-47c2-9729-f5016a871893</t>
+        </is>
+      </c>
+      <c r="AW182" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-sell-ISRG-1793386363557</t>
+        </is>
+      </c>
+      <c r="AX182" s="13" t="n">
+        <v>46325.7866087963</v>
+      </c>
+      <c r="AY182" s="13" t="n">
+        <v>46325.78664351852</v>
+      </c>
+      <c r="AZ182" s="13" t="n">
+        <v>46325.78628472222</v>
+      </c>
+      <c r="BA182" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -34740,9 +34928,15 @@
         <f>E75*F75</f>
         <v/>
       </c>
-      <c r="H75" s="22" t="n"/>
-      <c r="I75" s="22" t="n"/>
-      <c r="J75" s="17" t="n"/>
+      <c r="H75" s="22" t="n">
+        <v>46325.82831018518</v>
+      </c>
+      <c r="I75" s="22" t="n">
+        <v>46325.61997685185</v>
+      </c>
+      <c r="J75" s="17" t="n">
+        <v>433.29</v>
+      </c>
       <c r="K75" s="17">
         <f>IF(ISNUMBER(J75),J75*F75,"")</f>
         <v/>
@@ -34759,10 +34953,14 @@
         <f>IF(ISNUMBER(H75),H75-C75,"")</f>
         <v/>
       </c>
-      <c r="O75" s="6" t="n"/>
+      <c r="O75" s="6" t="inlineStr">
+        <is>
+          <t>bad day</t>
+        </is>
+      </c>
       <c r="P75" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-30 19:20 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA182" headerRowCount="1">
-  <autoFilter ref="A1:BA182"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA183" headerRowCount="1">
+  <autoFilter ref="A1:BA183"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.82835648148</v>
+        <v>46325.84726851852</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.62002314815</v>
+        <v>46325.63893518518</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$182,"BUY")+COUNTIF(Orders!$E$2:$E$182,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$183,"BUY")+COUNTIF(Orders!$E$2:$E$183,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$182,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$183,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$182,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$183,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$182,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$183,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$182,Orders!$E$2:$E$182,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$183,Orders!$E$2:$E$183,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$182,Orders!$E$2:$E$182,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$183,Orders!$E$2:$E$183,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA182"/>
+  <dimension ref="A1:BA183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -30001,13 +30001,13 @@
         <v>181</v>
       </c>
       <c r="B182" s="13" t="n">
-        <v>46325.82831018518</v>
+        <v>46325.84675925926</v>
       </c>
       <c r="C182" s="13" t="n">
-        <v>46325.61997685185</v>
+        <v>46325.63842592593</v>
       </c>
       <c r="D182" s="13" t="n">
-        <v>46325.78664351852</v>
+        <v>46325.80509259259</v>
       </c>
       <c r="E182" s="21" t="inlineStr">
         <is>
@@ -30016,29 +30016,21 @@
       </c>
       <c r="F182" s="6" t="inlineStr">
         <is>
-          <t>ISRG</t>
-        </is>
-      </c>
-      <c r="G182" s="15" t="inlineStr">
-        <is>
-          <t>ISRG</t>
-        </is>
-      </c>
-      <c r="H182" s="6" t="inlineStr">
-        <is>
-          <t>NASDAQ</t>
-        </is>
-      </c>
+          <t>ADP</t>
+        </is>
+      </c>
+      <c r="G182" s="15" t="n"/>
+      <c r="H182" s="6" t="n"/>
       <c r="I182" s="6" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
       <c r="J182" s="16" t="n">
-        <v>18.497085557</v>
+        <v>2.362539617</v>
       </c>
       <c r="K182" s="17" t="n">
-        <v>433.29</v>
+        <v>294.43</v>
       </c>
       <c r="L182" s="17">
         <f>IF(AND(ISNUMBER(J182),ISNUMBER(K182)),J182*K182,"")</f>
@@ -30046,143 +30038,259 @@
       </c>
       <c r="M182" s="17" t="n"/>
       <c r="N182" s="16" t="n">
+        <v>2.362539617</v>
+      </c>
+      <c r="O182" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
+      <c r="P182" s="15" t="inlineStr">
+        <is>
+          <t>Alpaca stop order triggered at 294.52 (the stock's sell line)</t>
+        </is>
+      </c>
+      <c r="Q182" s="12" t="n"/>
+      <c r="R182" s="6" t="n"/>
+      <c r="S182" s="18" t="n"/>
+      <c r="T182" s="12" t="n"/>
+      <c r="U182" s="19" t="n"/>
+      <c r="V182" s="19" t="n"/>
+      <c r="W182" s="12" t="n"/>
+      <c r="X182" s="6" t="n"/>
+      <c r="Y182" s="19" t="n"/>
+      <c r="Z182" s="6" t="n"/>
+      <c r="AA182" s="12" t="n"/>
+      <c r="AB182" s="15" t="n"/>
+      <c r="AC182" s="6" t="n"/>
+      <c r="AD182" s="6" t="n"/>
+      <c r="AE182" s="17" t="n"/>
+      <c r="AF182" s="17" t="n"/>
+      <c r="AG182" s="17" t="n"/>
+      <c r="AH182" s="20" t="n"/>
+      <c r="AI182" s="18" t="n"/>
+      <c r="AJ182" s="6" t="n"/>
+      <c r="AK182" s="12" t="n"/>
+      <c r="AL182" s="15" t="n"/>
+      <c r="AM182" s="17" t="n"/>
+      <c r="AN182" s="19" t="n"/>
+      <c r="AO182" s="17" t="n"/>
+      <c r="AP182" s="17" t="n"/>
+      <c r="AQ182" s="19" t="n"/>
+      <c r="AR182" s="16" t="n"/>
+      <c r="AS182" s="17" t="n"/>
+      <c r="AT182" s="19" t="n"/>
+      <c r="AU182" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV182" s="6" t="inlineStr">
+        <is>
+          <t>697d701f-be53-4826-b775-f3c204ac68c1</t>
+        </is>
+      </c>
+      <c r="AW182" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-stop-ADP-1793381581848</t>
+        </is>
+      </c>
+      <c r="AX182" s="13" t="n">
+        <v>46325.73126157407</v>
+      </c>
+      <c r="AY182" s="13" t="n">
+        <v>46325.80509259259</v>
+      </c>
+      <c r="AZ182" s="13" t="n"/>
+      <c r="BA182" s="6" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="12" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" s="13" t="n">
+        <v>46325.82831018518</v>
+      </c>
+      <c r="C183" s="13" t="n">
+        <v>46325.61997685185</v>
+      </c>
+      <c r="D183" s="13" t="n">
+        <v>46325.78664351852</v>
+      </c>
+      <c r="E183" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F183" s="6" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="G183" s="15" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="H183" s="6" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="I183" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J183" s="16" t="n">
         <v>18.497085557</v>
       </c>
-      <c r="O182" s="6" t="inlineStr">
+      <c r="K183" s="17" t="n">
+        <v>433.29</v>
+      </c>
+      <c r="L183" s="17">
+        <f>IF(AND(ISNUMBER(J183),ISNUMBER(K183)),J183*K183,"")</f>
+        <v/>
+      </c>
+      <c r="M183" s="17" t="n"/>
+      <c r="N183" s="16" t="n">
+        <v>18.497085557</v>
+      </c>
+      <c r="O183" s="6" t="inlineStr">
         <is>
           <t>bad day</t>
         </is>
       </c>
-      <c r="P182" s="15" t="inlineStr">
+      <c r="P183" s="15" t="inlineStr">
         <is>
           <t>Bad day: down 3.4% today and only 4 of 5 green</t>
         </is>
       </c>
-      <c r="Q182" s="12" t="n">
+      <c r="Q183" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="R182" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="S182" s="18" t="n">
+      <c r="R183" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="S183" s="18" t="n">
         <v>0.552</v>
       </c>
-      <c r="T182" s="12" t="n">
+      <c r="T183" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="U182" s="19" t="n">
+      <c r="U183" s="19" t="n">
         <v>0.0068</v>
       </c>
-      <c r="V182" s="19" t="n">
+      <c r="V183" s="19" t="n">
         <v>0.2893</v>
       </c>
-      <c r="W182" s="12" t="n"/>
-      <c r="X182" s="6" t="inlineStr">
+      <c r="W183" s="12" t="n"/>
+      <c r="X183" s="6" t="inlineStr">
         <is>
           <t>watch</t>
         </is>
       </c>
-      <c r="Y182" s="19" t="n">
+      <c r="Y183" s="19" t="n">
         <v>0.0077</v>
       </c>
-      <c r="Z182" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AA182" s="12" t="n">
+      <c r="Z183" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AA183" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="AB182" s="15" t="n"/>
-      <c r="AC182" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AD182" s="6" t="inlineStr">
+      <c r="AB183" s="15" t="n"/>
+      <c r="AC183" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AD183" s="6" t="inlineStr">
         <is>
           <t>up</t>
         </is>
       </c>
-      <c r="AE182" s="17" t="n">
+      <c r="AE183" s="17" t="n">
         <v>441.1307</v>
       </c>
-      <c r="AF182" s="17" t="n">
+      <c r="AF183" s="17" t="n">
         <v>423.079</v>
       </c>
-      <c r="AG182" s="17" t="n">
+      <c r="AG183" s="17" t="n">
         <v>459.1824</v>
       </c>
-      <c r="AH182" s="20" t="n">
+      <c r="AH183" s="20" t="n">
         <v>46332</v>
       </c>
-      <c r="AI182" s="18" t="n">
+      <c r="AI183" s="18" t="n">
         <v>0.55</v>
       </c>
-      <c r="AJ182" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="AK182" s="12" t="n">
+      <c r="AJ183" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AK183" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="AL182" s="15" t="inlineStr">
+      <c r="AL183" s="15" t="inlineStr">
         <is>
           <t>Apollo Hospitals Adopts Intuitive's Da Vinci 5 Surgical System</t>
         </is>
       </c>
-      <c r="AM182" s="17" t="n">
+      <c r="AM183" s="17" t="n">
         <v>434.06</v>
       </c>
-      <c r="AN182" s="19" t="n">
+      <c r="AN183" s="19" t="n">
         <v>-0.0331</v>
       </c>
-      <c r="AO182" s="17" t="n">
+      <c r="AO183" s="17" t="n">
         <v>98407.46000000001</v>
       </c>
-      <c r="AP182" s="17" t="n">
+      <c r="AP183" s="17" t="n">
         <v>26809.9</v>
       </c>
-      <c r="AQ182" s="19" t="n">
+      <c r="AQ183" s="19" t="n">
         <v>0.0833</v>
       </c>
-      <c r="AR182" s="16" t="n">
+      <c r="AR183" s="16" t="n">
         <v>18.497085557</v>
       </c>
-      <c r="AS182" s="17" t="n">
+      <c r="AS183" s="17" t="n">
         <v>447.77</v>
       </c>
-      <c r="AT182" s="19" t="n">
+      <c r="AT183" s="19" t="n">
         <v>-0.0315</v>
       </c>
-      <c r="AU182" s="6" t="inlineStr">
+      <c r="AU183" s="6" t="inlineStr">
         <is>
           <t>paper</t>
         </is>
       </c>
-      <c r="AV182" s="6" t="inlineStr">
+      <c r="AV183" s="6" t="inlineStr">
         <is>
           <t>7d8948d7-4093-47c2-9729-f5016a871893</t>
         </is>
       </c>
-      <c r="AW182" s="6" t="inlineStr">
+      <c r="AW183" s="6" t="inlineStr">
         <is>
           <t>tdagent-sell-ISRG-1793386363557</t>
         </is>
       </c>
-      <c r="AX182" s="13" t="n">
+      <c r="AX183" s="13" t="n">
         <v>46325.7866087963</v>
       </c>
-      <c r="AY182" s="13" t="n">
+      <c r="AY183" s="13" t="n">
         <v>46325.78664351852</v>
       </c>
-      <c r="AZ182" s="13" t="n">
+      <c r="AZ183" s="13" t="n">
         <v>46325.78628472222</v>
       </c>
-      <c r="BA182" s="6" t="n"/>
+      <c r="BA183" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -35783,9 +35891,15 @@
         <f>E90*F90</f>
         <v/>
       </c>
-      <c r="H90" s="22" t="n"/>
-      <c r="I90" s="22" t="n"/>
-      <c r="J90" s="17" t="n"/>
+      <c r="H90" s="22" t="n">
+        <v>46325.84675925926</v>
+      </c>
+      <c r="I90" s="22" t="n">
+        <v>46325.63842592593</v>
+      </c>
+      <c r="J90" s="17" t="n">
+        <v>294.43</v>
+      </c>
       <c r="K90" s="17">
         <f>IF(ISNUMBER(J90),J90*F90,"")</f>
         <v/>
@@ -35802,10 +35916,14 @@
         <f>IF(ISNUMBER(H90),H90-C90,"")</f>
         <v/>
       </c>
-      <c r="O90" s="6" t="n"/>
+      <c r="O90" s="6" t="inlineStr">
+        <is>
+          <t>stop-loss (Alpaca order)</t>
+        </is>
+      </c>
       <c r="P90" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
records: 2026-10-30 19:31 UTC
</commit_message>
<xml_diff>
--- a/trade-records/excel/2026-W44_2026-10-26.xlsx
+++ b/trade-records/excel/2026-W44_2026-10-26.xlsx
@@ -229,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA183" headerRowCount="1">
-  <autoFilter ref="A1:BA183"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Orders" displayName="Orders" ref="A1:BA202" headerRowCount="1">
+  <autoFilter ref="A1:BA202"/>
   <tableColumns count="53">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Time Berlin"/>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46325.84726851852</v>
+        <v>46325.85541666667</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46325.63893518518</v>
+        <v>46325.64708333334</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$183,"BUY")+COUNTIF(Orders!$E$2:$E$183,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$202,"BUY")+COUNTIF(Orders!$E$2:$E$202,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$183,"BUY")</f>
+        <f>COUNTIF(Orders!$E$2:$E$202,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Orders!$E$2:$E$183,"SELL")</f>
+        <f>COUNTIF(Orders!$E$2:$E$202,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Orders!$I$2:$I$183,"filled")</f>
+        <f>COUNTIF(Orders!$I$2:$I$202,"filled")</f>
         <v/>
       </c>
     </row>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$183,Orders!$E$2:$E$183,"BUY")</f>
+        <f>SUMIFS(Orders!$L$2:$L$202,Orders!$E$2:$E$202,"BUY")</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Orders!$L$2:$L$183,Orders!$E$2:$E$183,"SELL")</f>
+        <f>SUMIFS(Orders!$L$2:$L$202,Orders!$E$2:$E$202,"SELL")</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA183"/>
+  <dimension ref="A1:BA202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -30292,6 +30292,2058 @@
       </c>
       <c r="BA183" s="6" t="n"/>
     </row>
+    <row r="184">
+      <c r="A184" s="12" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" s="13" t="n">
+        <v>46325.85440972223</v>
+      </c>
+      <c r="C184" s="13" t="n">
+        <v>46325.64607638889</v>
+      </c>
+      <c r="D184" s="13" t="n">
+        <v>46325.81274305555</v>
+      </c>
+      <c r="E184" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F184" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G184" s="15" t="n"/>
+      <c r="H184" s="6" t="n"/>
+      <c r="I184" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J184" s="16" t="n">
+        <v>20.821202053</v>
+      </c>
+      <c r="K184" s="17" t="n">
+        <v>66.65000000000001</v>
+      </c>
+      <c r="L184" s="17">
+        <f>IF(AND(ISNUMBER(J184),ISNUMBER(K184)),J184*K184,"")</f>
+        <v/>
+      </c>
+      <c r="M184" s="17" t="n"/>
+      <c r="N184" s="16" t="n">
+        <v>20.821202053</v>
+      </c>
+      <c r="O184" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P184" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q184" s="12" t="n"/>
+      <c r="R184" s="6" t="n"/>
+      <c r="S184" s="18" t="n"/>
+      <c r="T184" s="12" t="n"/>
+      <c r="U184" s="19" t="n"/>
+      <c r="V184" s="19" t="n"/>
+      <c r="W184" s="12" t="n"/>
+      <c r="X184" s="6" t="n"/>
+      <c r="Y184" s="19" t="n"/>
+      <c r="Z184" s="6" t="n"/>
+      <c r="AA184" s="12" t="n"/>
+      <c r="AB184" s="15" t="n"/>
+      <c r="AC184" s="6" t="n"/>
+      <c r="AD184" s="6" t="n"/>
+      <c r="AE184" s="17" t="n"/>
+      <c r="AF184" s="17" t="n"/>
+      <c r="AG184" s="17" t="n"/>
+      <c r="AH184" s="20" t="n"/>
+      <c r="AI184" s="18" t="n"/>
+      <c r="AJ184" s="6" t="n"/>
+      <c r="AK184" s="12" t="n"/>
+      <c r="AL184" s="15" t="n"/>
+      <c r="AM184" s="17" t="n"/>
+      <c r="AN184" s="19" t="n"/>
+      <c r="AO184" s="17" t="n"/>
+      <c r="AP184" s="17" t="n"/>
+      <c r="AQ184" s="19" t="n"/>
+      <c r="AR184" s="16" t="n"/>
+      <c r="AS184" s="17" t="n"/>
+      <c r="AT184" s="19" t="n"/>
+      <c r="AU184" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV184" s="6" t="inlineStr">
+        <is>
+          <t>22fdbd3d-1777-4b88-9ab8-999dd48424af</t>
+        </is>
+      </c>
+      <c r="AW184" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-D-1793388616483</t>
+        </is>
+      </c>
+      <c r="AX184" s="13" t="n">
+        <v>46325.81269675926</v>
+      </c>
+      <c r="AY184" s="13" t="n">
+        <v>46325.81274305555</v>
+      </c>
+      <c r="AZ184" s="13" t="n"/>
+      <c r="BA184" s="6" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="12" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" s="13" t="n">
+        <v>46325.854375</v>
+      </c>
+      <c r="C185" s="13" t="n">
+        <v>46325.64604166667</v>
+      </c>
+      <c r="D185" s="13" t="n">
+        <v>46325.81270833333</v>
+      </c>
+      <c r="E185" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F185" s="6" t="inlineStr">
+        <is>
+          <t>EQNR</t>
+        </is>
+      </c>
+      <c r="G185" s="15" t="n"/>
+      <c r="H185" s="6" t="n"/>
+      <c r="I185" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J185" s="16" t="n">
+        <v>14.229932252</v>
+      </c>
+      <c r="K185" s="17" t="n">
+        <v>48.57</v>
+      </c>
+      <c r="L185" s="17">
+        <f>IF(AND(ISNUMBER(J185),ISNUMBER(K185)),J185*K185,"")</f>
+        <v/>
+      </c>
+      <c r="M185" s="17" t="n"/>
+      <c r="N185" s="16" t="n">
+        <v>14.229932252</v>
+      </c>
+      <c r="O185" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P185" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q185" s="12" t="n"/>
+      <c r="R185" s="6" t="n"/>
+      <c r="S185" s="18" t="n"/>
+      <c r="T185" s="12" t="n"/>
+      <c r="U185" s="19" t="n"/>
+      <c r="V185" s="19" t="n"/>
+      <c r="W185" s="12" t="n"/>
+      <c r="X185" s="6" t="n"/>
+      <c r="Y185" s="19" t="n"/>
+      <c r="Z185" s="6" t="n"/>
+      <c r="AA185" s="12" t="n"/>
+      <c r="AB185" s="15" t="n"/>
+      <c r="AC185" s="6" t="n"/>
+      <c r="AD185" s="6" t="n"/>
+      <c r="AE185" s="17" t="n"/>
+      <c r="AF185" s="17" t="n"/>
+      <c r="AG185" s="17" t="n"/>
+      <c r="AH185" s="20" t="n"/>
+      <c r="AI185" s="18" t="n"/>
+      <c r="AJ185" s="6" t="n"/>
+      <c r="AK185" s="12" t="n"/>
+      <c r="AL185" s="15" t="n"/>
+      <c r="AM185" s="17" t="n"/>
+      <c r="AN185" s="19" t="n"/>
+      <c r="AO185" s="17" t="n"/>
+      <c r="AP185" s="17" t="n"/>
+      <c r="AQ185" s="19" t="n"/>
+      <c r="AR185" s="16" t="n"/>
+      <c r="AS185" s="17" t="n"/>
+      <c r="AT185" s="19" t="n"/>
+      <c r="AU185" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV185" s="6" t="inlineStr">
+        <is>
+          <t>a3028d15-4981-4852-b375-defe6d904fa3</t>
+        </is>
+      </c>
+      <c r="AW185" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-EQNR-1793388617887</t>
+        </is>
+      </c>
+      <c r="AX185" s="13" t="n">
+        <v>46325.81270833333</v>
+      </c>
+      <c r="AY185" s="13" t="n">
+        <v>46325.81270833333</v>
+      </c>
+      <c r="AZ185" s="13" t="n"/>
+      <c r="BA185" s="6" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="12" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" s="13" t="n">
+        <v>46325.85440972223</v>
+      </c>
+      <c r="C186" s="13" t="n">
+        <v>46325.64607638889</v>
+      </c>
+      <c r="D186" s="13" t="n">
+        <v>46325.81274305555</v>
+      </c>
+      <c r="E186" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F186" s="6" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="G186" s="15" t="n"/>
+      <c r="H186" s="6" t="n"/>
+      <c r="I186" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J186" s="16" t="n">
+        <v>4.145924286</v>
+      </c>
+      <c r="K186" s="17" t="n">
+        <v>169.31</v>
+      </c>
+      <c r="L186" s="17">
+        <f>IF(AND(ISNUMBER(J186),ISNUMBER(K186)),J186*K186,"")</f>
+        <v/>
+      </c>
+      <c r="M186" s="17" t="n"/>
+      <c r="N186" s="16" t="n">
+        <v>4.145924286</v>
+      </c>
+      <c r="O186" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P186" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q186" s="12" t="n"/>
+      <c r="R186" s="6" t="n"/>
+      <c r="S186" s="18" t="n"/>
+      <c r="T186" s="12" t="n"/>
+      <c r="U186" s="19" t="n"/>
+      <c r="V186" s="19" t="n"/>
+      <c r="W186" s="12" t="n"/>
+      <c r="X186" s="6" t="n"/>
+      <c r="Y186" s="19" t="n"/>
+      <c r="Z186" s="6" t="n"/>
+      <c r="AA186" s="12" t="n"/>
+      <c r="AB186" s="15" t="n"/>
+      <c r="AC186" s="6" t="n"/>
+      <c r="AD186" s="6" t="n"/>
+      <c r="AE186" s="17" t="n"/>
+      <c r="AF186" s="17" t="n"/>
+      <c r="AG186" s="17" t="n"/>
+      <c r="AH186" s="20" t="n"/>
+      <c r="AI186" s="18" t="n"/>
+      <c r="AJ186" s="6" t="n"/>
+      <c r="AK186" s="12" t="n"/>
+      <c r="AL186" s="15" t="n"/>
+      <c r="AM186" s="17" t="n"/>
+      <c r="AN186" s="19" t="n"/>
+      <c r="AO186" s="17" t="n"/>
+      <c r="AP186" s="17" t="n"/>
+      <c r="AQ186" s="19" t="n"/>
+      <c r="AR186" s="16" t="n"/>
+      <c r="AS186" s="17" t="n"/>
+      <c r="AT186" s="19" t="n"/>
+      <c r="AU186" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV186" s="6" t="inlineStr">
+        <is>
+          <t>5a75eb60-575f-4110-9843-0b047d6e11d5</t>
+        </is>
+      </c>
+      <c r="AW186" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ICE-1793388619304</t>
+        </is>
+      </c>
+      <c r="AX186" s="13" t="n">
+        <v>46325.81271990741</v>
+      </c>
+      <c r="AY186" s="13" t="n">
+        <v>46325.81274305555</v>
+      </c>
+      <c r="AZ186" s="13" t="n"/>
+      <c r="BA186" s="6" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="12" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" s="13" t="n">
+        <v>46325.85440972223</v>
+      </c>
+      <c r="C187" s="13" t="n">
+        <v>46325.64607638889</v>
+      </c>
+      <c r="D187" s="13" t="n">
+        <v>46325.81274305555</v>
+      </c>
+      <c r="E187" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F187" s="6" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="G187" s="15" t="n"/>
+      <c r="H187" s="6" t="n"/>
+      <c r="I187" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J187" s="16" t="n">
+        <v>10.24745011</v>
+      </c>
+      <c r="K187" s="17" t="n">
+        <v>66.72</v>
+      </c>
+      <c r="L187" s="17">
+        <f>IF(AND(ISNUMBER(J187),ISNUMBER(K187)),J187*K187,"")</f>
+        <v/>
+      </c>
+      <c r="M187" s="17" t="n"/>
+      <c r="N187" s="16" t="n">
+        <v>10.24745011</v>
+      </c>
+      <c r="O187" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P187" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q187" s="12" t="n"/>
+      <c r="R187" s="6" t="n"/>
+      <c r="S187" s="18" t="n"/>
+      <c r="T187" s="12" t="n"/>
+      <c r="U187" s="19" t="n"/>
+      <c r="V187" s="19" t="n"/>
+      <c r="W187" s="12" t="n"/>
+      <c r="X187" s="6" t="n"/>
+      <c r="Y187" s="19" t="n"/>
+      <c r="Z187" s="6" t="n"/>
+      <c r="AA187" s="12" t="n"/>
+      <c r="AB187" s="15" t="n"/>
+      <c r="AC187" s="6" t="n"/>
+      <c r="AD187" s="6" t="n"/>
+      <c r="AE187" s="17" t="n"/>
+      <c r="AF187" s="17" t="n"/>
+      <c r="AG187" s="17" t="n"/>
+      <c r="AH187" s="20" t="n"/>
+      <c r="AI187" s="18" t="n"/>
+      <c r="AJ187" s="6" t="n"/>
+      <c r="AK187" s="12" t="n"/>
+      <c r="AL187" s="15" t="n"/>
+      <c r="AM187" s="17" t="n"/>
+      <c r="AN187" s="19" t="n"/>
+      <c r="AO187" s="17" t="n"/>
+      <c r="AP187" s="17" t="n"/>
+      <c r="AQ187" s="19" t="n"/>
+      <c r="AR187" s="16" t="n"/>
+      <c r="AS187" s="17" t="n"/>
+      <c r="AT187" s="19" t="n"/>
+      <c r="AU187" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV187" s="6" t="inlineStr">
+        <is>
+          <t>b26155fb-6157-48da-bcac-62ed2f1d8b7a</t>
+        </is>
+      </c>
+      <c r="AW187" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-KR-1793388620720</t>
+        </is>
+      </c>
+      <c r="AX187" s="13" t="n">
+        <v>46325.81273148148</v>
+      </c>
+      <c r="AY187" s="13" t="n">
+        <v>46325.81274305555</v>
+      </c>
+      <c r="AZ187" s="13" t="n"/>
+      <c r="BA187" s="6" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="12" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="13" t="n">
+        <v>46325.85443287037</v>
+      </c>
+      <c r="C188" s="13" t="n">
+        <v>46325.64609953704</v>
+      </c>
+      <c r="D188" s="13" t="n">
+        <v>46325.8127662037</v>
+      </c>
+      <c r="E188" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F188" s="6" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G188" s="15" t="n"/>
+      <c r="H188" s="6" t="n"/>
+      <c r="I188" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J188" s="16" t="n">
+        <v>2.314697642</v>
+      </c>
+      <c r="K188" s="17" t="n">
+        <v>638.50568</v>
+      </c>
+      <c r="L188" s="17">
+        <f>IF(AND(ISNUMBER(J188),ISNUMBER(K188)),J188*K188,"")</f>
+        <v/>
+      </c>
+      <c r="M188" s="17" t="n"/>
+      <c r="N188" s="16" t="n">
+        <v>2.314697642</v>
+      </c>
+      <c r="O188" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P188" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q188" s="12" t="n"/>
+      <c r="R188" s="6" t="n"/>
+      <c r="S188" s="18" t="n"/>
+      <c r="T188" s="12" t="n"/>
+      <c r="U188" s="19" t="n"/>
+      <c r="V188" s="19" t="n"/>
+      <c r="W188" s="12" t="n"/>
+      <c r="X188" s="6" t="n"/>
+      <c r="Y188" s="19" t="n"/>
+      <c r="Z188" s="6" t="n"/>
+      <c r="AA188" s="12" t="n"/>
+      <c r="AB188" s="15" t="n"/>
+      <c r="AC188" s="6" t="n"/>
+      <c r="AD188" s="6" t="n"/>
+      <c r="AE188" s="17" t="n"/>
+      <c r="AF188" s="17" t="n"/>
+      <c r="AG188" s="17" t="n"/>
+      <c r="AH188" s="20" t="n"/>
+      <c r="AI188" s="18" t="n"/>
+      <c r="AJ188" s="6" t="n"/>
+      <c r="AK188" s="12" t="n"/>
+      <c r="AL188" s="15" t="n"/>
+      <c r="AM188" s="17" t="n"/>
+      <c r="AN188" s="19" t="n"/>
+      <c r="AO188" s="17" t="n"/>
+      <c r="AP188" s="17" t="n"/>
+      <c r="AQ188" s="19" t="n"/>
+      <c r="AR188" s="16" t="n"/>
+      <c r="AS188" s="17" t="n"/>
+      <c r="AT188" s="19" t="n"/>
+      <c r="AU188" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV188" s="6" t="inlineStr">
+        <is>
+          <t>75c356ce-b92a-49a4-9e74-700f02e39644</t>
+        </is>
+      </c>
+      <c r="AW188" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MA-1793388622173</t>
+        </is>
+      </c>
+      <c r="AX188" s="13" t="n">
+        <v>46325.81275462963</v>
+      </c>
+      <c r="AY188" s="13" t="n">
+        <v>46325.8127662037</v>
+      </c>
+      <c r="AZ188" s="13" t="n"/>
+      <c r="BA188" s="6" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="12" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" s="13" t="n">
+        <v>46325.8544675926</v>
+      </c>
+      <c r="C189" s="13" t="n">
+        <v>46325.64613425926</v>
+      </c>
+      <c r="D189" s="13" t="n">
+        <v>46325.81280092592</v>
+      </c>
+      <c r="E189" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F189" s="6" t="inlineStr">
+        <is>
+          <t>MCK</t>
+        </is>
+      </c>
+      <c r="G189" s="15" t="n"/>
+      <c r="H189" s="6" t="n"/>
+      <c r="I189" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J189" s="16" t="n">
+        <v>8.201734928</v>
+      </c>
+      <c r="K189" s="17" t="n">
+        <v>990.22</v>
+      </c>
+      <c r="L189" s="17">
+        <f>IF(AND(ISNUMBER(J189),ISNUMBER(K189)),J189*K189,"")</f>
+        <v/>
+      </c>
+      <c r="M189" s="17" t="n"/>
+      <c r="N189" s="16" t="n">
+        <v>8.201734928</v>
+      </c>
+      <c r="O189" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P189" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q189" s="12" t="n"/>
+      <c r="R189" s="6" t="n"/>
+      <c r="S189" s="18" t="n"/>
+      <c r="T189" s="12" t="n"/>
+      <c r="U189" s="19" t="n"/>
+      <c r="V189" s="19" t="n"/>
+      <c r="W189" s="12" t="n"/>
+      <c r="X189" s="6" t="n"/>
+      <c r="Y189" s="19" t="n"/>
+      <c r="Z189" s="6" t="n"/>
+      <c r="AA189" s="12" t="n"/>
+      <c r="AB189" s="15" t="n"/>
+      <c r="AC189" s="6" t="n"/>
+      <c r="AD189" s="6" t="n"/>
+      <c r="AE189" s="17" t="n"/>
+      <c r="AF189" s="17" t="n"/>
+      <c r="AG189" s="17" t="n"/>
+      <c r="AH189" s="20" t="n"/>
+      <c r="AI189" s="18" t="n"/>
+      <c r="AJ189" s="6" t="n"/>
+      <c r="AK189" s="12" t="n"/>
+      <c r="AL189" s="15" t="n"/>
+      <c r="AM189" s="17" t="n"/>
+      <c r="AN189" s="19" t="n"/>
+      <c r="AO189" s="17" t="n"/>
+      <c r="AP189" s="17" t="n"/>
+      <c r="AQ189" s="19" t="n"/>
+      <c r="AR189" s="16" t="n"/>
+      <c r="AS189" s="17" t="n"/>
+      <c r="AT189" s="19" t="n"/>
+      <c r="AU189" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV189" s="6" t="inlineStr">
+        <is>
+          <t>15f869ca-1ee7-4c23-9040-20a51523155d</t>
+        </is>
+      </c>
+      <c r="AW189" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MCK-1793388623591</t>
+        </is>
+      </c>
+      <c r="AX189" s="13" t="n">
+        <v>46325.8127662037</v>
+      </c>
+      <c r="AY189" s="13" t="n">
+        <v>46325.81280092592</v>
+      </c>
+      <c r="AZ189" s="13" t="n"/>
+      <c r="BA189" s="6" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="12" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" s="13" t="n">
+        <v>46325.8544675926</v>
+      </c>
+      <c r="C190" s="13" t="n">
+        <v>46325.64613425926</v>
+      </c>
+      <c r="D190" s="13" t="n">
+        <v>46325.81280092592</v>
+      </c>
+      <c r="E190" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F190" s="6" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="G190" s="15" t="n"/>
+      <c r="H190" s="6" t="n"/>
+      <c r="I190" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J190" s="16" t="n">
+        <v>14.687288135</v>
+      </c>
+      <c r="K190" s="17" t="n">
+        <v>47.12</v>
+      </c>
+      <c r="L190" s="17">
+        <f>IF(AND(ISNUMBER(J190),ISNUMBER(K190)),J190*K190,"")</f>
+        <v/>
+      </c>
+      <c r="M190" s="17" t="n"/>
+      <c r="N190" s="16" t="n">
+        <v>14.687288135</v>
+      </c>
+      <c r="O190" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P190" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q190" s="12" t="n"/>
+      <c r="R190" s="6" t="n"/>
+      <c r="S190" s="18" t="n"/>
+      <c r="T190" s="12" t="n"/>
+      <c r="U190" s="19" t="n"/>
+      <c r="V190" s="19" t="n"/>
+      <c r="W190" s="12" t="n"/>
+      <c r="X190" s="6" t="n"/>
+      <c r="Y190" s="19" t="n"/>
+      <c r="Z190" s="6" t="n"/>
+      <c r="AA190" s="12" t="n"/>
+      <c r="AB190" s="15" t="n"/>
+      <c r="AC190" s="6" t="n"/>
+      <c r="AD190" s="6" t="n"/>
+      <c r="AE190" s="17" t="n"/>
+      <c r="AF190" s="17" t="n"/>
+      <c r="AG190" s="17" t="n"/>
+      <c r="AH190" s="20" t="n"/>
+      <c r="AI190" s="18" t="n"/>
+      <c r="AJ190" s="6" t="n"/>
+      <c r="AK190" s="12" t="n"/>
+      <c r="AL190" s="15" t="n"/>
+      <c r="AM190" s="17" t="n"/>
+      <c r="AN190" s="19" t="n"/>
+      <c r="AO190" s="17" t="n"/>
+      <c r="AP190" s="17" t="n"/>
+      <c r="AQ190" s="19" t="n"/>
+      <c r="AR190" s="16" t="n"/>
+      <c r="AS190" s="17" t="n"/>
+      <c r="AT190" s="19" t="n"/>
+      <c r="AU190" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV190" s="6" t="inlineStr">
+        <is>
+          <t>cdf9f9e7-c95f-4ed7-9bfe-fa2704da28c8</t>
+        </is>
+      </c>
+      <c r="AW190" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MNST-1793388625019</t>
+        </is>
+      </c>
+      <c r="AX190" s="13" t="n">
+        <v>46325.81278935185</v>
+      </c>
+      <c r="AY190" s="13" t="n">
+        <v>46325.81280092592</v>
+      </c>
+      <c r="AZ190" s="13" t="n"/>
+      <c r="BA190" s="6" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="12" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" s="13" t="n">
+        <v>46325.85449074074</v>
+      </c>
+      <c r="C191" s="13" t="n">
+        <v>46325.64615740741</v>
+      </c>
+      <c r="D191" s="13" t="n">
+        <v>46325.81282407408</v>
+      </c>
+      <c r="E191" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F191" s="6" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="G191" s="15" t="n"/>
+      <c r="H191" s="6" t="n"/>
+      <c r="I191" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J191" s="16" t="n">
+        <v>17.501650165</v>
+      </c>
+      <c r="K191" s="17" t="n">
+        <v>78.04000000000001</v>
+      </c>
+      <c r="L191" s="17">
+        <f>IF(AND(ISNUMBER(J191),ISNUMBER(K191)),J191*K191,"")</f>
+        <v/>
+      </c>
+      <c r="M191" s="17" t="n"/>
+      <c r="N191" s="16" t="n">
+        <v>17.501650165</v>
+      </c>
+      <c r="O191" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P191" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q191" s="12" t="n"/>
+      <c r="R191" s="6" t="n"/>
+      <c r="S191" s="18" t="n"/>
+      <c r="T191" s="12" t="n"/>
+      <c r="U191" s="19" t="n"/>
+      <c r="V191" s="19" t="n"/>
+      <c r="W191" s="12" t="n"/>
+      <c r="X191" s="6" t="n"/>
+      <c r="Y191" s="19" t="n"/>
+      <c r="Z191" s="6" t="n"/>
+      <c r="AA191" s="12" t="n"/>
+      <c r="AB191" s="15" t="n"/>
+      <c r="AC191" s="6" t="n"/>
+      <c r="AD191" s="6" t="n"/>
+      <c r="AE191" s="17" t="n"/>
+      <c r="AF191" s="17" t="n"/>
+      <c r="AG191" s="17" t="n"/>
+      <c r="AH191" s="20" t="n"/>
+      <c r="AI191" s="18" t="n"/>
+      <c r="AJ191" s="6" t="n"/>
+      <c r="AK191" s="12" t="n"/>
+      <c r="AL191" s="15" t="n"/>
+      <c r="AM191" s="17" t="n"/>
+      <c r="AN191" s="19" t="n"/>
+      <c r="AO191" s="17" t="n"/>
+      <c r="AP191" s="17" t="n"/>
+      <c r="AQ191" s="19" t="n"/>
+      <c r="AR191" s="16" t="n"/>
+      <c r="AS191" s="17" t="n"/>
+      <c r="AT191" s="19" t="n"/>
+      <c r="AU191" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV191" s="6" t="inlineStr">
+        <is>
+          <t>37bab048-6691-4e34-96b5-3528c3c5e5ca</t>
+        </is>
+      </c>
+      <c r="AW191" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MO-1793388626434</t>
+        </is>
+      </c>
+      <c r="AX191" s="13" t="n">
+        <v>46325.81280092592</v>
+      </c>
+      <c r="AY191" s="13" t="n">
+        <v>46325.81282407408</v>
+      </c>
+      <c r="AZ191" s="13" t="n"/>
+      <c r="BA191" s="6" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="12" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" s="13" t="n">
+        <v>46325.85451388889</v>
+      </c>
+      <c r="C192" s="13" t="n">
+        <v>46325.64618055556</v>
+      </c>
+      <c r="D192" s="13" t="n">
+        <v>46325.81284722222</v>
+      </c>
+      <c r="E192" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F192" s="6" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="G192" s="15" t="n"/>
+      <c r="H192" s="6" t="n"/>
+      <c r="I192" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J192" s="16" t="n">
+        <v>18.738552036</v>
+      </c>
+      <c r="K192" s="17" t="n">
+        <v>441.048933</v>
+      </c>
+      <c r="L192" s="17">
+        <f>IF(AND(ISNUMBER(J192),ISNUMBER(K192)),J192*K192,"")</f>
+        <v/>
+      </c>
+      <c r="M192" s="17" t="n"/>
+      <c r="N192" s="16" t="n">
+        <v>18.738552036</v>
+      </c>
+      <c r="O192" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P192" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q192" s="12" t="n"/>
+      <c r="R192" s="6" t="n"/>
+      <c r="S192" s="18" t="n"/>
+      <c r="T192" s="12" t="n"/>
+      <c r="U192" s="19" t="n"/>
+      <c r="V192" s="19" t="n"/>
+      <c r="W192" s="12" t="n"/>
+      <c r="X192" s="6" t="n"/>
+      <c r="Y192" s="19" t="n"/>
+      <c r="Z192" s="6" t="n"/>
+      <c r="AA192" s="12" t="n"/>
+      <c r="AB192" s="15" t="n"/>
+      <c r="AC192" s="6" t="n"/>
+      <c r="AD192" s="6" t="n"/>
+      <c r="AE192" s="17" t="n"/>
+      <c r="AF192" s="17" t="n"/>
+      <c r="AG192" s="17" t="n"/>
+      <c r="AH192" s="20" t="n"/>
+      <c r="AI192" s="18" t="n"/>
+      <c r="AJ192" s="6" t="n"/>
+      <c r="AK192" s="12" t="n"/>
+      <c r="AL192" s="15" t="n"/>
+      <c r="AM192" s="17" t="n"/>
+      <c r="AN192" s="19" t="n"/>
+      <c r="AO192" s="17" t="n"/>
+      <c r="AP192" s="17" t="n"/>
+      <c r="AQ192" s="19" t="n"/>
+      <c r="AR192" s="16" t="n"/>
+      <c r="AS192" s="17" t="n"/>
+      <c r="AT192" s="19" t="n"/>
+      <c r="AU192" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV192" s="6" t="inlineStr">
+        <is>
+          <t>511f4b94-0909-4f42-9ab2-d768bc3b0cce</t>
+        </is>
+      </c>
+      <c r="AW192" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-MPC-1793388627846</t>
+        </is>
+      </c>
+      <c r="AX192" s="13" t="n">
+        <v>46325.81282407408</v>
+      </c>
+      <c r="AY192" s="13" t="n">
+        <v>46325.81284722222</v>
+      </c>
+      <c r="AZ192" s="13" t="n"/>
+      <c r="BA192" s="6" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="12" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" s="13" t="n">
+        <v>46325.85453703703</v>
+      </c>
+      <c r="C193" s="13" t="n">
+        <v>46325.64620370371</v>
+      </c>
+      <c r="D193" s="13" t="n">
+        <v>46325.81287037037</v>
+      </c>
+      <c r="E193" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F193" s="6" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="G193" s="15" t="n"/>
+      <c r="H193" s="6" t="n"/>
+      <c r="I193" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J193" s="16" t="n">
+        <v>10.872647427</v>
+      </c>
+      <c r="K193" s="17" t="n">
+        <v>63.638278</v>
+      </c>
+      <c r="L193" s="17">
+        <f>IF(AND(ISNUMBER(J193),ISNUMBER(K193)),J193*K193,"")</f>
+        <v/>
+      </c>
+      <c r="M193" s="17" t="n"/>
+      <c r="N193" s="16" t="n">
+        <v>10.872647427</v>
+      </c>
+      <c r="O193" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P193" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q193" s="12" t="n"/>
+      <c r="R193" s="6" t="n"/>
+      <c r="S193" s="18" t="n"/>
+      <c r="T193" s="12" t="n"/>
+      <c r="U193" s="19" t="n"/>
+      <c r="V193" s="19" t="n"/>
+      <c r="W193" s="12" t="n"/>
+      <c r="X193" s="6" t="n"/>
+      <c r="Y193" s="19" t="n"/>
+      <c r="Z193" s="6" t="n"/>
+      <c r="AA193" s="12" t="n"/>
+      <c r="AB193" s="15" t="n"/>
+      <c r="AC193" s="6" t="n"/>
+      <c r="AD193" s="6" t="n"/>
+      <c r="AE193" s="17" t="n"/>
+      <c r="AF193" s="17" t="n"/>
+      <c r="AG193" s="17" t="n"/>
+      <c r="AH193" s="20" t="n"/>
+      <c r="AI193" s="18" t="n"/>
+      <c r="AJ193" s="6" t="n"/>
+      <c r="AK193" s="12" t="n"/>
+      <c r="AL193" s="15" t="n"/>
+      <c r="AM193" s="17" t="n"/>
+      <c r="AN193" s="19" t="n"/>
+      <c r="AO193" s="17" t="n"/>
+      <c r="AP193" s="17" t="n"/>
+      <c r="AQ193" s="19" t="n"/>
+      <c r="AR193" s="16" t="n"/>
+      <c r="AS193" s="17" t="n"/>
+      <c r="AT193" s="19" t="n"/>
+      <c r="AU193" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV193" s="6" t="inlineStr">
+        <is>
+          <t>1e32889a-2018-4c3b-a2d3-1dcd1edc7cae</t>
+        </is>
+      </c>
+      <c r="AW193" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-OXY-1793388629252</t>
+        </is>
+      </c>
+      <c r="AX193" s="13" t="n">
+        <v>46325.81283564815</v>
+      </c>
+      <c r="AY193" s="13" t="n">
+        <v>46325.81287037037</v>
+      </c>
+      <c r="AZ193" s="13" t="n"/>
+      <c r="BA193" s="6" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="12" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" s="13" t="n">
+        <v>46325.85453703703</v>
+      </c>
+      <c r="C194" s="13" t="n">
+        <v>46325.64620370371</v>
+      </c>
+      <c r="D194" s="13" t="n">
+        <v>46325.81287037037</v>
+      </c>
+      <c r="E194" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F194" s="6" t="inlineStr">
+        <is>
+          <t>SHEL</t>
+        </is>
+      </c>
+      <c r="G194" s="15" t="n"/>
+      <c r="H194" s="6" t="n"/>
+      <c r="I194" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J194" s="16" t="n">
+        <v>76.12460944599999</v>
+      </c>
+      <c r="K194" s="17" t="n">
+        <v>108.39</v>
+      </c>
+      <c r="L194" s="17">
+        <f>IF(AND(ISNUMBER(J194),ISNUMBER(K194)),J194*K194,"")</f>
+        <v/>
+      </c>
+      <c r="M194" s="17" t="n"/>
+      <c r="N194" s="16" t="n">
+        <v>76.12460944599999</v>
+      </c>
+      <c r="O194" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P194" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q194" s="12" t="n"/>
+      <c r="R194" s="6" t="n"/>
+      <c r="S194" s="18" t="n"/>
+      <c r="T194" s="12" t="n"/>
+      <c r="U194" s="19" t="n"/>
+      <c r="V194" s="19" t="n"/>
+      <c r="W194" s="12" t="n"/>
+      <c r="X194" s="6" t="n"/>
+      <c r="Y194" s="19" t="n"/>
+      <c r="Z194" s="6" t="n"/>
+      <c r="AA194" s="12" t="n"/>
+      <c r="AB194" s="15" t="n"/>
+      <c r="AC194" s="6" t="n"/>
+      <c r="AD194" s="6" t="n"/>
+      <c r="AE194" s="17" t="n"/>
+      <c r="AF194" s="17" t="n"/>
+      <c r="AG194" s="17" t="n"/>
+      <c r="AH194" s="20" t="n"/>
+      <c r="AI194" s="18" t="n"/>
+      <c r="AJ194" s="6" t="n"/>
+      <c r="AK194" s="12" t="n"/>
+      <c r="AL194" s="15" t="n"/>
+      <c r="AM194" s="17" t="n"/>
+      <c r="AN194" s="19" t="n"/>
+      <c r="AO194" s="17" t="n"/>
+      <c r="AP194" s="17" t="n"/>
+      <c r="AQ194" s="19" t="n"/>
+      <c r="AR194" s="16" t="n"/>
+      <c r="AS194" s="17" t="n"/>
+      <c r="AT194" s="19" t="n"/>
+      <c r="AU194" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV194" s="6" t="inlineStr">
+        <is>
+          <t>9ca2b76c-83dc-45a2-82b0-927b98ae2f2d</t>
+        </is>
+      </c>
+      <c r="AW194" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-SHEL-1793388630663</t>
+        </is>
+      </c>
+      <c r="AX194" s="13" t="n">
+        <v>46325.81284722222</v>
+      </c>
+      <c r="AY194" s="13" t="n">
+        <v>46325.81287037037</v>
+      </c>
+      <c r="AZ194" s="13" t="n"/>
+      <c r="BA194" s="6" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="12" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" s="13" t="n">
+        <v>46325.85453703703</v>
+      </c>
+      <c r="C195" s="13" t="n">
+        <v>46325.64620370371</v>
+      </c>
+      <c r="D195" s="13" t="n">
+        <v>46325.81287037037</v>
+      </c>
+      <c r="E195" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F195" s="6" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="G195" s="15" t="n"/>
+      <c r="H195" s="6" t="n"/>
+      <c r="I195" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J195" s="16" t="n">
+        <v>3.304762358</v>
+      </c>
+      <c r="K195" s="17" t="n">
+        <v>207.56</v>
+      </c>
+      <c r="L195" s="17">
+        <f>IF(AND(ISNUMBER(J195),ISNUMBER(K195)),J195*K195,"")</f>
+        <v/>
+      </c>
+      <c r="M195" s="17" t="n"/>
+      <c r="N195" s="16" t="n">
+        <v>3.304762358</v>
+      </c>
+      <c r="O195" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P195" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q195" s="12" t="n"/>
+      <c r="R195" s="6" t="n"/>
+      <c r="S195" s="18" t="n"/>
+      <c r="T195" s="12" t="n"/>
+      <c r="U195" s="19" t="n"/>
+      <c r="V195" s="19" t="n"/>
+      <c r="W195" s="12" t="n"/>
+      <c r="X195" s="6" t="n"/>
+      <c r="Y195" s="19" t="n"/>
+      <c r="Z195" s="6" t="n"/>
+      <c r="AA195" s="12" t="n"/>
+      <c r="AB195" s="15" t="n"/>
+      <c r="AC195" s="6" t="n"/>
+      <c r="AD195" s="6" t="n"/>
+      <c r="AE195" s="17" t="n"/>
+      <c r="AF195" s="17" t="n"/>
+      <c r="AG195" s="17" t="n"/>
+      <c r="AH195" s="20" t="n"/>
+      <c r="AI195" s="18" t="n"/>
+      <c r="AJ195" s="6" t="n"/>
+      <c r="AK195" s="12" t="n"/>
+      <c r="AL195" s="15" t="n"/>
+      <c r="AM195" s="17" t="n"/>
+      <c r="AN195" s="19" t="n"/>
+      <c r="AO195" s="17" t="n"/>
+      <c r="AP195" s="17" t="n"/>
+      <c r="AQ195" s="19" t="n"/>
+      <c r="AR195" s="16" t="n"/>
+      <c r="AS195" s="17" t="n"/>
+      <c r="AT195" s="19" t="n"/>
+      <c r="AU195" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV195" s="6" t="inlineStr">
+        <is>
+          <t>c21c693d-93c1-419c-a093-337c942af7de</t>
+        </is>
+      </c>
+      <c r="AW195" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-SN-1793388632074</t>
+        </is>
+      </c>
+      <c r="AX195" s="13" t="n">
+        <v>46325.81287037037</v>
+      </c>
+      <c r="AY195" s="13" t="n">
+        <v>46325.81287037037</v>
+      </c>
+      <c r="AZ195" s="13" t="n"/>
+      <c r="BA195" s="6" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="12" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" s="13" t="n">
+        <v>46325.85456018519</v>
+      </c>
+      <c r="C196" s="13" t="n">
+        <v>46325.64622685185</v>
+      </c>
+      <c r="D196" s="13" t="n">
+        <v>46325.81289351852</v>
+      </c>
+      <c r="E196" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F196" s="6" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="G196" s="15" t="n"/>
+      <c r="H196" s="6" t="n"/>
+      <c r="I196" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J196" s="16" t="n">
+        <v>14.649320305</v>
+      </c>
+      <c r="K196" s="17" t="n">
+        <v>93.91</v>
+      </c>
+      <c r="L196" s="17">
+        <f>IF(AND(ISNUMBER(J196),ISNUMBER(K196)),J196*K196,"")</f>
+        <v/>
+      </c>
+      <c r="M196" s="17" t="n"/>
+      <c r="N196" s="16" t="n">
+        <v>14.649320305</v>
+      </c>
+      <c r="O196" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P196" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q196" s="12" t="n"/>
+      <c r="R196" s="6" t="n"/>
+      <c r="S196" s="18" t="n"/>
+      <c r="T196" s="12" t="n"/>
+      <c r="U196" s="19" t="n"/>
+      <c r="V196" s="19" t="n"/>
+      <c r="W196" s="12" t="n"/>
+      <c r="X196" s="6" t="n"/>
+      <c r="Y196" s="19" t="n"/>
+      <c r="Z196" s="6" t="n"/>
+      <c r="AA196" s="12" t="n"/>
+      <c r="AB196" s="15" t="n"/>
+      <c r="AC196" s="6" t="n"/>
+      <c r="AD196" s="6" t="n"/>
+      <c r="AE196" s="17" t="n"/>
+      <c r="AF196" s="17" t="n"/>
+      <c r="AG196" s="17" t="n"/>
+      <c r="AH196" s="20" t="n"/>
+      <c r="AI196" s="18" t="n"/>
+      <c r="AJ196" s="6" t="n"/>
+      <c r="AK196" s="12" t="n"/>
+      <c r="AL196" s="15" t="n"/>
+      <c r="AM196" s="17" t="n"/>
+      <c r="AN196" s="19" t="n"/>
+      <c r="AO196" s="17" t="n"/>
+      <c r="AP196" s="17" t="n"/>
+      <c r="AQ196" s="19" t="n"/>
+      <c r="AR196" s="16" t="n"/>
+      <c r="AS196" s="17" t="n"/>
+      <c r="AT196" s="19" t="n"/>
+      <c r="AU196" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV196" s="6" t="inlineStr">
+        <is>
+          <t>631bd2cf-f6db-4916-8289-f9201dbabdfe</t>
+        </is>
+      </c>
+      <c r="AW196" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-SO-1793388633599</t>
+        </is>
+      </c>
+      <c r="AX196" s="13" t="n">
+        <v>46325.81288194445</v>
+      </c>
+      <c r="AY196" s="13" t="n">
+        <v>46325.81289351852</v>
+      </c>
+      <c r="AZ196" s="13" t="n"/>
+      <c r="BA196" s="6" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="12" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" s="13" t="n">
+        <v>46325.85459490741</v>
+      </c>
+      <c r="C197" s="13" t="n">
+        <v>46325.64626157407</v>
+      </c>
+      <c r="D197" s="13" t="n">
+        <v>46325.81292824074</v>
+      </c>
+      <c r="E197" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F197" s="6" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="G197" s="15" t="n"/>
+      <c r="H197" s="6" t="n"/>
+      <c r="I197" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J197" s="16" t="n">
+        <v>11.642778824</v>
+      </c>
+      <c r="K197" s="17" t="n">
+        <v>693.1</v>
+      </c>
+      <c r="L197" s="17">
+        <f>IF(AND(ISNUMBER(J197),ISNUMBER(K197)),J197*K197,"")</f>
+        <v/>
+      </c>
+      <c r="M197" s="17" t="n"/>
+      <c r="N197" s="16" t="n">
+        <v>11.642778824</v>
+      </c>
+      <c r="O197" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P197" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q197" s="12" t="n"/>
+      <c r="R197" s="6" t="n"/>
+      <c r="S197" s="18" t="n"/>
+      <c r="T197" s="12" t="n"/>
+      <c r="U197" s="19" t="n"/>
+      <c r="V197" s="19" t="n"/>
+      <c r="W197" s="12" t="n"/>
+      <c r="X197" s="6" t="n"/>
+      <c r="Y197" s="19" t="n"/>
+      <c r="Z197" s="6" t="n"/>
+      <c r="AA197" s="12" t="n"/>
+      <c r="AB197" s="15" t="n"/>
+      <c r="AC197" s="6" t="n"/>
+      <c r="AD197" s="6" t="n"/>
+      <c r="AE197" s="17" t="n"/>
+      <c r="AF197" s="17" t="n"/>
+      <c r="AG197" s="17" t="n"/>
+      <c r="AH197" s="20" t="n"/>
+      <c r="AI197" s="18" t="n"/>
+      <c r="AJ197" s="6" t="n"/>
+      <c r="AK197" s="12" t="n"/>
+      <c r="AL197" s="15" t="n"/>
+      <c r="AM197" s="17" t="n"/>
+      <c r="AN197" s="19" t="n"/>
+      <c r="AO197" s="17" t="n"/>
+      <c r="AP197" s="17" t="n"/>
+      <c r="AQ197" s="19" t="n"/>
+      <c r="AR197" s="16" t="n"/>
+      <c r="AS197" s="17" t="n"/>
+      <c r="AT197" s="19" t="n"/>
+      <c r="AU197" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV197" s="6" t="inlineStr">
+        <is>
+          <t>d0fa34b9-e830-4357-9942-3da91e899834</t>
+        </is>
+      </c>
+      <c r="AW197" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-TMO-1793388635016</t>
+        </is>
+      </c>
+      <c r="AX197" s="13" t="n">
+        <v>46325.81290509259</v>
+      </c>
+      <c r="AY197" s="13" t="n">
+        <v>46325.81292824074</v>
+      </c>
+      <c r="AZ197" s="13" t="n"/>
+      <c r="BA197" s="6" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="12" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" s="13" t="n">
+        <v>46325.85459490741</v>
+      </c>
+      <c r="C198" s="13" t="n">
+        <v>46325.64626157407</v>
+      </c>
+      <c r="D198" s="13" t="n">
+        <v>46325.81292824074</v>
+      </c>
+      <c r="E198" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F198" s="6" t="inlineStr">
+        <is>
+          <t>ULTA</t>
+        </is>
+      </c>
+      <c r="G198" s="15" t="n"/>
+      <c r="H198" s="6" t="n"/>
+      <c r="I198" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J198" s="16" t="n">
+        <v>2.62602669</v>
+      </c>
+      <c r="K198" s="17" t="n">
+        <v>635.78</v>
+      </c>
+      <c r="L198" s="17">
+        <f>IF(AND(ISNUMBER(J198),ISNUMBER(K198)),J198*K198,"")</f>
+        <v/>
+      </c>
+      <c r="M198" s="17" t="n"/>
+      <c r="N198" s="16" t="n">
+        <v>2.62602669</v>
+      </c>
+      <c r="O198" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P198" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q198" s="12" t="n"/>
+      <c r="R198" s="6" t="n"/>
+      <c r="S198" s="18" t="n"/>
+      <c r="T198" s="12" t="n"/>
+      <c r="U198" s="19" t="n"/>
+      <c r="V198" s="19" t="n"/>
+      <c r="W198" s="12" t="n"/>
+      <c r="X198" s="6" t="n"/>
+      <c r="Y198" s="19" t="n"/>
+      <c r="Z198" s="6" t="n"/>
+      <c r="AA198" s="12" t="n"/>
+      <c r="AB198" s="15" t="n"/>
+      <c r="AC198" s="6" t="n"/>
+      <c r="AD198" s="6" t="n"/>
+      <c r="AE198" s="17" t="n"/>
+      <c r="AF198" s="17" t="n"/>
+      <c r="AG198" s="17" t="n"/>
+      <c r="AH198" s="20" t="n"/>
+      <c r="AI198" s="18" t="n"/>
+      <c r="AJ198" s="6" t="n"/>
+      <c r="AK198" s="12" t="n"/>
+      <c r="AL198" s="15" t="n"/>
+      <c r="AM198" s="17" t="n"/>
+      <c r="AN198" s="19" t="n"/>
+      <c r="AO198" s="17" t="n"/>
+      <c r="AP198" s="17" t="n"/>
+      <c r="AQ198" s="19" t="n"/>
+      <c r="AR198" s="16" t="n"/>
+      <c r="AS198" s="17" t="n"/>
+      <c r="AT198" s="19" t="n"/>
+      <c r="AU198" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV198" s="6" t="inlineStr">
+        <is>
+          <t>e688b9de-5376-4b0c-b34b-e69a6aee7269</t>
+        </is>
+      </c>
+      <c r="AW198" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ULTA-1793388636443</t>
+        </is>
+      </c>
+      <c r="AX198" s="13" t="n">
+        <v>46325.81291666667</v>
+      </c>
+      <c r="AY198" s="13" t="n">
+        <v>46325.81292824074</v>
+      </c>
+      <c r="AZ198" s="13" t="n"/>
+      <c r="BA198" s="6" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="12" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" s="13" t="n">
+        <v>46325.85461805556</v>
+      </c>
+      <c r="C199" s="13" t="n">
+        <v>46325.64628472222</v>
+      </c>
+      <c r="D199" s="13" t="n">
+        <v>46325.81295138889</v>
+      </c>
+      <c r="E199" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F199" s="6" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="G199" s="15" t="n"/>
+      <c r="H199" s="6" t="n"/>
+      <c r="I199" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J199" s="16" t="n">
+        <v>26.419297124</v>
+      </c>
+      <c r="K199" s="17" t="n">
+        <v>311.88</v>
+      </c>
+      <c r="L199" s="17">
+        <f>IF(AND(ISNUMBER(J199),ISNUMBER(K199)),J199*K199,"")</f>
+        <v/>
+      </c>
+      <c r="M199" s="17" t="n"/>
+      <c r="N199" s="16" t="n">
+        <v>26.419297124</v>
+      </c>
+      <c r="O199" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P199" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q199" s="12" t="n"/>
+      <c r="R199" s="6" t="n"/>
+      <c r="S199" s="18" t="n"/>
+      <c r="T199" s="12" t="n"/>
+      <c r="U199" s="19" t="n"/>
+      <c r="V199" s="19" t="n"/>
+      <c r="W199" s="12" t="n"/>
+      <c r="X199" s="6" t="n"/>
+      <c r="Y199" s="19" t="n"/>
+      <c r="Z199" s="6" t="n"/>
+      <c r="AA199" s="12" t="n"/>
+      <c r="AB199" s="15" t="n"/>
+      <c r="AC199" s="6" t="n"/>
+      <c r="AD199" s="6" t="n"/>
+      <c r="AE199" s="17" t="n"/>
+      <c r="AF199" s="17" t="n"/>
+      <c r="AG199" s="17" t="n"/>
+      <c r="AH199" s="20" t="n"/>
+      <c r="AI199" s="18" t="n"/>
+      <c r="AJ199" s="6" t="n"/>
+      <c r="AK199" s="12" t="n"/>
+      <c r="AL199" s="15" t="n"/>
+      <c r="AM199" s="17" t="n"/>
+      <c r="AN199" s="19" t="n"/>
+      <c r="AO199" s="17" t="n"/>
+      <c r="AP199" s="17" t="n"/>
+      <c r="AQ199" s="19" t="n"/>
+      <c r="AR199" s="16" t="n"/>
+      <c r="AS199" s="17" t="n"/>
+      <c r="AT199" s="19" t="n"/>
+      <c r="AU199" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV199" s="6" t="inlineStr">
+        <is>
+          <t>9f9698fb-da0f-4762-a616-80f4387f11bb</t>
+        </is>
+      </c>
+      <c r="AW199" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-VEEV-1793388637859</t>
+        </is>
+      </c>
+      <c r="AX199" s="13" t="n">
+        <v>46325.81293981482</v>
+      </c>
+      <c r="AY199" s="13" t="n">
+        <v>46325.81295138889</v>
+      </c>
+      <c r="AZ199" s="13" t="n"/>
+      <c r="BA199" s="6" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="12" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" s="13" t="n">
+        <v>46325.85462962963</v>
+      </c>
+      <c r="C200" s="13" t="n">
+        <v>46325.6462962963</v>
+      </c>
+      <c r="D200" s="13" t="n">
+        <v>46325.81296296296</v>
+      </c>
+      <c r="E200" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F200" s="6" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="G200" s="15" t="n"/>
+      <c r="H200" s="6" t="n"/>
+      <c r="I200" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J200" s="16" t="n">
+        <v>25.40677088</v>
+      </c>
+      <c r="K200" s="17" t="n">
+        <v>323.02</v>
+      </c>
+      <c r="L200" s="17">
+        <f>IF(AND(ISNUMBER(J200),ISNUMBER(K200)),J200*K200,"")</f>
+        <v/>
+      </c>
+      <c r="M200" s="17" t="n"/>
+      <c r="N200" s="16" t="n">
+        <v>25.40677088</v>
+      </c>
+      <c r="O200" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P200" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q200" s="12" t="n"/>
+      <c r="R200" s="6" t="n"/>
+      <c r="S200" s="18" t="n"/>
+      <c r="T200" s="12" t="n"/>
+      <c r="U200" s="19" t="n"/>
+      <c r="V200" s="19" t="n"/>
+      <c r="W200" s="12" t="n"/>
+      <c r="X200" s="6" t="n"/>
+      <c r="Y200" s="19" t="n"/>
+      <c r="Z200" s="6" t="n"/>
+      <c r="AA200" s="12" t="n"/>
+      <c r="AB200" s="15" t="n"/>
+      <c r="AC200" s="6" t="n"/>
+      <c r="AD200" s="6" t="n"/>
+      <c r="AE200" s="17" t="n"/>
+      <c r="AF200" s="17" t="n"/>
+      <c r="AG200" s="17" t="n"/>
+      <c r="AH200" s="20" t="n"/>
+      <c r="AI200" s="18" t="n"/>
+      <c r="AJ200" s="6" t="n"/>
+      <c r="AK200" s="12" t="n"/>
+      <c r="AL200" s="15" t="n"/>
+      <c r="AM200" s="17" t="n"/>
+      <c r="AN200" s="19" t="n"/>
+      <c r="AO200" s="17" t="n"/>
+      <c r="AP200" s="17" t="n"/>
+      <c r="AQ200" s="19" t="n"/>
+      <c r="AR200" s="16" t="n"/>
+      <c r="AS200" s="17" t="n"/>
+      <c r="AT200" s="19" t="n"/>
+      <c r="AU200" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV200" s="6" t="inlineStr">
+        <is>
+          <t>a478c2f3-ecc3-4aaf-8790-f62c332ee010</t>
+        </is>
+      </c>
+      <c r="AW200" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-WTW-1793388639265</t>
+        </is>
+      </c>
+      <c r="AX200" s="13" t="n">
+        <v>46325.81295138889</v>
+      </c>
+      <c r="AY200" s="13" t="n">
+        <v>46325.81296296296</v>
+      </c>
+      <c r="AZ200" s="13" t="n"/>
+      <c r="BA200" s="6" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" s="13" t="n">
+        <v>46325.85467592593</v>
+      </c>
+      <c r="C201" s="13" t="n">
+        <v>46325.64634259259</v>
+      </c>
+      <c r="D201" s="13" t="n">
+        <v>46325.81300925926</v>
+      </c>
+      <c r="E201" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F201" s="6" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="G201" s="15" t="n"/>
+      <c r="H201" s="6" t="n"/>
+      <c r="I201" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J201" s="16" t="n">
+        <v>8.322299745</v>
+      </c>
+      <c r="K201" s="17" t="n">
+        <v>186.346008</v>
+      </c>
+      <c r="L201" s="17">
+        <f>IF(AND(ISNUMBER(J201),ISNUMBER(K201)),J201*K201,"")</f>
+        <v/>
+      </c>
+      <c r="M201" s="17" t="n"/>
+      <c r="N201" s="16" t="n">
+        <v>8.322299745</v>
+      </c>
+      <c r="O201" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P201" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q201" s="12" t="n"/>
+      <c r="R201" s="6" t="n"/>
+      <c r="S201" s="18" t="n"/>
+      <c r="T201" s="12" t="n"/>
+      <c r="U201" s="19" t="n"/>
+      <c r="V201" s="19" t="n"/>
+      <c r="W201" s="12" t="n"/>
+      <c r="X201" s="6" t="n"/>
+      <c r="Y201" s="19" t="n"/>
+      <c r="Z201" s="6" t="n"/>
+      <c r="AA201" s="12" t="n"/>
+      <c r="AB201" s="15" t="n"/>
+      <c r="AC201" s="6" t="n"/>
+      <c r="AD201" s="6" t="n"/>
+      <c r="AE201" s="17" t="n"/>
+      <c r="AF201" s="17" t="n"/>
+      <c r="AG201" s="17" t="n"/>
+      <c r="AH201" s="20" t="n"/>
+      <c r="AI201" s="18" t="n"/>
+      <c r="AJ201" s="6" t="n"/>
+      <c r="AK201" s="12" t="n"/>
+      <c r="AL201" s="15" t="n"/>
+      <c r="AM201" s="17" t="n"/>
+      <c r="AN201" s="19" t="n"/>
+      <c r="AO201" s="17" t="n"/>
+      <c r="AP201" s="17" t="n"/>
+      <c r="AQ201" s="19" t="n"/>
+      <c r="AR201" s="16" t="n"/>
+      <c r="AS201" s="17" t="n"/>
+      <c r="AT201" s="19" t="n"/>
+      <c r="AU201" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV201" s="6" t="inlineStr">
+        <is>
+          <t>7bcca843-824b-4eb8-9b37-aa9b433877f0</t>
+        </is>
+      </c>
+      <c r="AW201" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-XOM-1793388640667</t>
+        </is>
+      </c>
+      <c r="AX201" s="13" t="n">
+        <v>46325.81296296296</v>
+      </c>
+      <c r="AY201" s="13" t="n">
+        <v>46325.81300925926</v>
+      </c>
+      <c r="AZ201" s="13" t="n"/>
+      <c r="BA201" s="6" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="12" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" s="13" t="n">
+        <v>46325.8550462963</v>
+      </c>
+      <c r="C202" s="13" t="n">
+        <v>46325.64671296296</v>
+      </c>
+      <c r="D202" s="13" t="n">
+        <v>46325.81337962963</v>
+      </c>
+      <c r="E202" s="21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F202" s="6" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="G202" s="15" t="n"/>
+      <c r="H202" s="6" t="n"/>
+      <c r="I202" s="6" t="inlineStr">
+        <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="J202" s="16" t="n">
+        <v>2.342106152</v>
+      </c>
+      <c r="K202" s="17" t="n">
+        <v>293.72</v>
+      </c>
+      <c r="L202" s="17">
+        <f>IF(AND(ISNUMBER(J202),ISNUMBER(K202)),J202*K202,"")</f>
+        <v/>
+      </c>
+      <c r="M202" s="17" t="n"/>
+      <c r="N202" s="16" t="n">
+        <v>2.342106152</v>
+      </c>
+      <c r="O202" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
+      <c r="P202" s="15" t="inlineStr">
+        <is>
+          <t>Every-minute watchdog: evening rule, under +5% before the close</t>
+        </is>
+      </c>
+      <c r="Q202" s="12" t="n"/>
+      <c r="R202" s="6" t="n"/>
+      <c r="S202" s="18" t="n"/>
+      <c r="T202" s="12" t="n"/>
+      <c r="U202" s="19" t="n"/>
+      <c r="V202" s="19" t="n"/>
+      <c r="W202" s="12" t="n"/>
+      <c r="X202" s="6" t="n"/>
+      <c r="Y202" s="19" t="n"/>
+      <c r="Z202" s="6" t="n"/>
+      <c r="AA202" s="12" t="n"/>
+      <c r="AB202" s="15" t="n"/>
+      <c r="AC202" s="6" t="n"/>
+      <c r="AD202" s="6" t="n"/>
+      <c r="AE202" s="17" t="n"/>
+      <c r="AF202" s="17" t="n"/>
+      <c r="AG202" s="17" t="n"/>
+      <c r="AH202" s="20" t="n"/>
+      <c r="AI202" s="18" t="n"/>
+      <c r="AJ202" s="6" t="n"/>
+      <c r="AK202" s="12" t="n"/>
+      <c r="AL202" s="15" t="n"/>
+      <c r="AM202" s="17" t="n"/>
+      <c r="AN202" s="19" t="n"/>
+      <c r="AO202" s="17" t="n"/>
+      <c r="AP202" s="17" t="n"/>
+      <c r="AQ202" s="19" t="n"/>
+      <c r="AR202" s="16" t="n"/>
+      <c r="AS202" s="17" t="n"/>
+      <c r="AT202" s="19" t="n"/>
+      <c r="AU202" s="6" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="AV202" s="6" t="inlineStr">
+        <is>
+          <t>1a0d49bb-27f6-4526-afdf-8cca67b0a0b4</t>
+        </is>
+      </c>
+      <c r="AW202" s="6" t="inlineStr">
+        <is>
+          <t>tdagent-wd-evening-ABBV-1793388674708</t>
+        </is>
+      </c>
+      <c r="AX202" s="13" t="n">
+        <v>46325.81335648148</v>
+      </c>
+      <c r="AY202" s="13" t="n">
+        <v>46325.81337962963</v>
+      </c>
+      <c r="AZ202" s="13" t="n"/>
+      <c r="BA202" s="6" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
@@ -35099,9 +37151,15 @@
         <f>E76*F76</f>
         <v/>
       </c>
-      <c r="H76" s="22" t="n"/>
-      <c r="I76" s="22" t="n"/>
-      <c r="J76" s="17" t="n"/>
+      <c r="H76" s="22" t="n">
+        <v>46325.8544675926</v>
+      </c>
+      <c r="I76" s="22" t="n">
+        <v>46325.64613425926</v>
+      </c>
+      <c r="J76" s="17" t="n">
+        <v>990.22</v>
+      </c>
       <c r="K76" s="17">
         <f>IF(ISNUMBER(J76),J76*F76,"")</f>
         <v/>
@@ -35118,10 +37176,14 @@
         <f>IF(ISNUMBER(H76),H76-C76,"")</f>
         <v/>
       </c>
-      <c r="O76" s="6" t="n"/>
+      <c r="O76" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P76" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35341,9 +37403,15 @@
         <f>E80*F80</f>
         <v/>
       </c>
-      <c r="H80" s="22" t="n"/>
-      <c r="I80" s="22" t="n"/>
-      <c r="J80" s="17" t="n"/>
+      <c r="H80" s="22" t="n">
+        <v>46325.85459490741</v>
+      </c>
+      <c r="I80" s="22" t="n">
+        <v>46325.64626157407</v>
+      </c>
+      <c r="J80" s="17" t="n">
+        <v>693.1</v>
+      </c>
       <c r="K80" s="17">
         <f>IF(ISNUMBER(J80),J80*F80,"")</f>
         <v/>
@@ -35360,10 +37428,14 @@
         <f>IF(ISNUMBER(H80),H80-C80,"")</f>
         <v/>
       </c>
-      <c r="O80" s="6" t="n"/>
+      <c r="O80" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P80" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35394,9 +37466,15 @@
         <f>E81*F81</f>
         <v/>
       </c>
-      <c r="H81" s="22" t="n"/>
-      <c r="I81" s="22" t="n"/>
-      <c r="J81" s="17" t="n"/>
+      <c r="H81" s="22" t="n">
+        <v>46325.85453703703</v>
+      </c>
+      <c r="I81" s="22" t="n">
+        <v>46325.64620370371</v>
+      </c>
+      <c r="J81" s="17" t="n">
+        <v>108.39</v>
+      </c>
       <c r="K81" s="17">
         <f>IF(ISNUMBER(J81),J81*F81,"")</f>
         <v/>
@@ -35413,10 +37491,14 @@
         <f>IF(ISNUMBER(H81),H81-C81,"")</f>
         <v/>
       </c>
-      <c r="O81" s="6" t="n"/>
+      <c r="O81" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P81" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35447,9 +37529,15 @@
         <f>E82*F82</f>
         <v/>
       </c>
-      <c r="H82" s="22" t="n"/>
-      <c r="I82" s="22" t="n"/>
-      <c r="J82" s="17" t="n"/>
+      <c r="H82" s="22" t="n">
+        <v>46325.85451388889</v>
+      </c>
+      <c r="I82" s="22" t="n">
+        <v>46325.64618055556</v>
+      </c>
+      <c r="J82" s="17" t="n">
+        <v>441.048933</v>
+      </c>
       <c r="K82" s="17">
         <f>IF(ISNUMBER(J82),J82*F82,"")</f>
         <v/>
@@ -35466,10 +37554,14 @@
         <f>IF(ISNUMBER(H82),H82-C82,"")</f>
         <v/>
       </c>
-      <c r="O82" s="6" t="n"/>
+      <c r="O82" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P82" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35563,9 +37655,15 @@
         <f>E84*F84</f>
         <v/>
       </c>
-      <c r="H84" s="22" t="n"/>
-      <c r="I84" s="22" t="n"/>
-      <c r="J84" s="17" t="n"/>
+      <c r="H84" s="22" t="n">
+        <v>46325.85462962963</v>
+      </c>
+      <c r="I84" s="22" t="n">
+        <v>46325.6462962963</v>
+      </c>
+      <c r="J84" s="17" t="n">
+        <v>323.02</v>
+      </c>
       <c r="K84" s="17">
         <f>IF(ISNUMBER(J84),J84*F84,"")</f>
         <v/>
@@ -35582,10 +37680,14 @@
         <f>IF(ISNUMBER(H84),H84-C84,"")</f>
         <v/>
       </c>
-      <c r="O84" s="6" t="n"/>
+      <c r="O84" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P84" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35616,9 +37718,15 @@
         <f>E85*F85</f>
         <v/>
       </c>
-      <c r="H85" s="22" t="n"/>
-      <c r="I85" s="22" t="n"/>
-      <c r="J85" s="17" t="n"/>
+      <c r="H85" s="22" t="n">
+        <v>46325.85461805556</v>
+      </c>
+      <c r="I85" s="22" t="n">
+        <v>46325.64628472222</v>
+      </c>
+      <c r="J85" s="17" t="n">
+        <v>311.88</v>
+      </c>
       <c r="K85" s="17">
         <f>IF(ISNUMBER(J85),J85*F85,"")</f>
         <v/>
@@ -35635,10 +37743,14 @@
         <f>IF(ISNUMBER(H85),H85-C85,"")</f>
         <v/>
       </c>
-      <c r="O85" s="6" t="n"/>
+      <c r="O85" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P85" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35732,9 +37844,15 @@
         <f>E87*F87</f>
         <v/>
       </c>
-      <c r="H87" s="22" t="n"/>
-      <c r="I87" s="22" t="n"/>
-      <c r="J87" s="17" t="n"/>
+      <c r="H87" s="22" t="n">
+        <v>46325.8550462963</v>
+      </c>
+      <c r="I87" s="22" t="n">
+        <v>46325.64671296296</v>
+      </c>
+      <c r="J87" s="17" t="n">
+        <v>293.72</v>
+      </c>
       <c r="K87" s="17">
         <f>IF(ISNUMBER(J87),J87*F87,"")</f>
         <v/>
@@ -35751,10 +37869,14 @@
         <f>IF(ISNUMBER(H87),H87-C87,"")</f>
         <v/>
       </c>
-      <c r="O87" s="6" t="n"/>
+      <c r="O87" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P87" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35785,9 +37907,15 @@
         <f>E88*F88</f>
         <v/>
       </c>
-      <c r="H88" s="22" t="n"/>
-      <c r="I88" s="22" t="n"/>
-      <c r="J88" s="17" t="n"/>
+      <c r="H88" s="22" t="n">
+        <v>46325.85453703703</v>
+      </c>
+      <c r="I88" s="22" t="n">
+        <v>46325.64620370371</v>
+      </c>
+      <c r="J88" s="17" t="n">
+        <v>63.638278</v>
+      </c>
       <c r="K88" s="17">
         <f>IF(ISNUMBER(J88),J88*F88,"")</f>
         <v/>
@@ -35804,10 +37932,14 @@
         <f>IF(ISNUMBER(H88),H88-C88,"")</f>
         <v/>
       </c>
-      <c r="O88" s="6" t="n"/>
+      <c r="O88" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P88" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35838,9 +37970,15 @@
         <f>E89*F89</f>
         <v/>
       </c>
-      <c r="H89" s="22" t="n"/>
-      <c r="I89" s="22" t="n"/>
-      <c r="J89" s="17" t="n"/>
+      <c r="H89" s="22" t="n">
+        <v>46325.85440972223</v>
+      </c>
+      <c r="I89" s="22" t="n">
+        <v>46325.64607638889</v>
+      </c>
+      <c r="J89" s="17" t="n">
+        <v>169.31</v>
+      </c>
       <c r="K89" s="17">
         <f>IF(ISNUMBER(J89),J89*F89,"")</f>
         <v/>
@@ -35857,10 +37995,14 @@
         <f>IF(ISNUMBER(H89),H89-C89,"")</f>
         <v/>
       </c>
-      <c r="O89" s="6" t="n"/>
+      <c r="O89" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P89" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -35954,9 +38096,15 @@
         <f>E91*F91</f>
         <v/>
       </c>
-      <c r="H91" s="22" t="n"/>
-      <c r="I91" s="22" t="n"/>
-      <c r="J91" s="17" t="n"/>
+      <c r="H91" s="22" t="n">
+        <v>46325.854375</v>
+      </c>
+      <c r="I91" s="22" t="n">
+        <v>46325.64604166667</v>
+      </c>
+      <c r="J91" s="17" t="n">
+        <v>48.57</v>
+      </c>
       <c r="K91" s="17">
         <f>IF(ISNUMBER(J91),J91*F91,"")</f>
         <v/>
@@ -35973,10 +38121,14 @@
         <f>IF(ISNUMBER(H91),H91-C91,"")</f>
         <v/>
       </c>
-      <c r="O91" s="6" t="n"/>
+      <c r="O91" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P91" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36007,9 +38159,15 @@
         <f>E92*F92</f>
         <v/>
       </c>
-      <c r="H92" s="22" t="n"/>
-      <c r="I92" s="22" t="n"/>
-      <c r="J92" s="17" t="n"/>
+      <c r="H92" s="22" t="n">
+        <v>46325.85453703703</v>
+      </c>
+      <c r="I92" s="22" t="n">
+        <v>46325.64620370371</v>
+      </c>
+      <c r="J92" s="17" t="n">
+        <v>207.56</v>
+      </c>
       <c r="K92" s="17">
         <f>IF(ISNUMBER(J92),J92*F92,"")</f>
         <v/>
@@ -36026,10 +38184,14 @@
         <f>IF(ISNUMBER(H92),H92-C92,"")</f>
         <v/>
       </c>
-      <c r="O92" s="6" t="n"/>
+      <c r="O92" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P92" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36060,9 +38222,15 @@
         <f>E93*F93</f>
         <v/>
       </c>
-      <c r="H93" s="22" t="n"/>
-      <c r="I93" s="22" t="n"/>
-      <c r="J93" s="17" t="n"/>
+      <c r="H93" s="22" t="n">
+        <v>46325.8544675926</v>
+      </c>
+      <c r="I93" s="22" t="n">
+        <v>46325.64613425926</v>
+      </c>
+      <c r="J93" s="17" t="n">
+        <v>47.12</v>
+      </c>
       <c r="K93" s="17">
         <f>IF(ISNUMBER(J93),J93*F93,"")</f>
         <v/>
@@ -36079,10 +38247,14 @@
         <f>IF(ISNUMBER(H93),H93-C93,"")</f>
         <v/>
       </c>
-      <c r="O93" s="6" t="n"/>
+      <c r="O93" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P93" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36302,9 +38474,15 @@
         <f>E97*F97</f>
         <v/>
       </c>
-      <c r="H97" s="22" t="n"/>
-      <c r="I97" s="22" t="n"/>
-      <c r="J97" s="17" t="n"/>
+      <c r="H97" s="22" t="n">
+        <v>46325.85440972223</v>
+      </c>
+      <c r="I97" s="22" t="n">
+        <v>46325.64607638889</v>
+      </c>
+      <c r="J97" s="17" t="n">
+        <v>66.72</v>
+      </c>
       <c r="K97" s="17">
         <f>IF(ISNUMBER(J97),J97*F97,"")</f>
         <v/>
@@ -36321,10 +38499,14 @@
         <f>IF(ISNUMBER(H97),H97-C97,"")</f>
         <v/>
       </c>
-      <c r="O97" s="6" t="n"/>
+      <c r="O97" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P97" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36418,9 +38600,15 @@
         <f>E99*F99</f>
         <v/>
       </c>
-      <c r="H99" s="22" t="n"/>
-      <c r="I99" s="22" t="n"/>
-      <c r="J99" s="17" t="n"/>
+      <c r="H99" s="22" t="n">
+        <v>46325.85440972223</v>
+      </c>
+      <c r="I99" s="22" t="n">
+        <v>46325.64607638889</v>
+      </c>
+      <c r="J99" s="17" t="n">
+        <v>66.65000000000001</v>
+      </c>
       <c r="K99" s="17">
         <f>IF(ISNUMBER(J99),J99*F99,"")</f>
         <v/>
@@ -36437,10 +38625,14 @@
         <f>IF(ISNUMBER(H99),H99-C99,"")</f>
         <v/>
       </c>
-      <c r="O99" s="6" t="n"/>
+      <c r="O99" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P99" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36471,9 +38663,15 @@
         <f>E100*F100</f>
         <v/>
       </c>
-      <c r="H100" s="22" t="n"/>
-      <c r="I100" s="22" t="n"/>
-      <c r="J100" s="17" t="n"/>
+      <c r="H100" s="22" t="n">
+        <v>46325.85449074074</v>
+      </c>
+      <c r="I100" s="22" t="n">
+        <v>46325.64615740741</v>
+      </c>
+      <c r="J100" s="17" t="n">
+        <v>78.04000000000001</v>
+      </c>
       <c r="K100" s="17">
         <f>IF(ISNUMBER(J100),J100*F100,"")</f>
         <v/>
@@ -36490,10 +38688,14 @@
         <f>IF(ISNUMBER(H100),H100-C100,"")</f>
         <v/>
       </c>
-      <c r="O100" s="6" t="n"/>
+      <c r="O100" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P100" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36524,9 +38726,15 @@
         <f>E101*F101</f>
         <v/>
       </c>
-      <c r="H101" s="22" t="n"/>
-      <c r="I101" s="22" t="n"/>
-      <c r="J101" s="17" t="n"/>
+      <c r="H101" s="22" t="n">
+        <v>46325.85456018519</v>
+      </c>
+      <c r="I101" s="22" t="n">
+        <v>46325.64622685185</v>
+      </c>
+      <c r="J101" s="17" t="n">
+        <v>93.91</v>
+      </c>
       <c r="K101" s="17">
         <f>IF(ISNUMBER(J101),J101*F101,"")</f>
         <v/>
@@ -36543,10 +38751,14 @@
         <f>IF(ISNUMBER(H101),H101-C101,"")</f>
         <v/>
       </c>
-      <c r="O101" s="6" t="n"/>
+      <c r="O101" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P101" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36766,9 +38978,15 @@
         <f>E105*F105</f>
         <v/>
       </c>
-      <c r="H105" s="22" t="n"/>
-      <c r="I105" s="22" t="n"/>
-      <c r="J105" s="17" t="n"/>
+      <c r="H105" s="22" t="n">
+        <v>46325.85443287037</v>
+      </c>
+      <c r="I105" s="22" t="n">
+        <v>46325.64609953704</v>
+      </c>
+      <c r="J105" s="17" t="n">
+        <v>638.50568</v>
+      </c>
       <c r="K105" s="17">
         <f>IF(ISNUMBER(J105),J105*F105,"")</f>
         <v/>
@@ -36785,10 +39003,14 @@
         <f>IF(ISNUMBER(H105),H105-C105,"")</f>
         <v/>
       </c>
-      <c r="O105" s="6" t="n"/>
+      <c r="O105" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P105" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36819,9 +39041,15 @@
         <f>E106*F106</f>
         <v/>
       </c>
-      <c r="H106" s="22" t="n"/>
-      <c r="I106" s="22" t="n"/>
-      <c r="J106" s="17" t="n"/>
+      <c r="H106" s="22" t="n">
+        <v>46325.85459490741</v>
+      </c>
+      <c r="I106" s="22" t="n">
+        <v>46325.64626157407</v>
+      </c>
+      <c r="J106" s="17" t="n">
+        <v>635.78</v>
+      </c>
       <c r="K106" s="17">
         <f>IF(ISNUMBER(J106),J106*F106,"")</f>
         <v/>
@@ -36838,10 +39066,14 @@
         <f>IF(ISNUMBER(H106),H106-C106,"")</f>
         <v/>
       </c>
-      <c r="O106" s="6" t="n"/>
+      <c r="O106" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P106" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -36872,9 +39104,15 @@
         <f>E107*F107</f>
         <v/>
       </c>
-      <c r="H107" s="22" t="n"/>
-      <c r="I107" s="22" t="n"/>
-      <c r="J107" s="17" t="n"/>
+      <c r="H107" s="22" t="n">
+        <v>46325.85467592593</v>
+      </c>
+      <c r="I107" s="22" t="n">
+        <v>46325.64634259259</v>
+      </c>
+      <c r="J107" s="17" t="n">
+        <v>186.346008</v>
+      </c>
       <c r="K107" s="17">
         <f>IF(ISNUMBER(J107),J107*F107,"")</f>
         <v/>
@@ -36891,10 +39129,14 @@
         <f>IF(ISNUMBER(H107),H107-C107,"")</f>
         <v/>
       </c>
-      <c r="O107" s="6" t="n"/>
+      <c r="O107" s="6" t="inlineStr">
+        <is>
+          <t>evening under 5% (watchdog)</t>
+        </is>
+      </c>
       <c r="P107" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>